<commit_message>
14/07/2023 - Arun Removed Target from Git
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1721" uniqueCount="614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1844" uniqueCount="675">
   <si>
     <t>Scenario</t>
   </si>
@@ -1908,6 +1908,189 @@
   </si>
   <si>
     <t>2302181955125</t>
+  </si>
+  <si>
+    <t>BKPAAC</t>
+  </si>
+  <si>
+    <t>BKPAIQ</t>
+  </si>
+  <si>
+    <t>BKPAME</t>
+  </si>
+  <si>
+    <t>BKPAO5</t>
+  </si>
+  <si>
+    <t>BKPAU4</t>
+  </si>
+  <si>
+    <t>2023-07-14T06:11:10</t>
+  </si>
+  <si>
+    <t>BKPA4Y</t>
+  </si>
+  <si>
+    <t>2023-07-14T06:11:18</t>
+  </si>
+  <si>
+    <t>BKPB2R</t>
+  </si>
+  <si>
+    <t>BKPB5B</t>
+  </si>
+  <si>
+    <t>BKPCA2</t>
+  </si>
+  <si>
+    <t>2302182476441</t>
+  </si>
+  <si>
+    <t>BKPCXW</t>
+  </si>
+  <si>
+    <t>2302182476442</t>
+  </si>
+  <si>
+    <t>BKPDLD</t>
+  </si>
+  <si>
+    <t>2302182476443</t>
+  </si>
+  <si>
+    <t>BKPEPN</t>
+  </si>
+  <si>
+    <t>2302182476444</t>
+  </si>
+  <si>
+    <t>BKPETM</t>
+  </si>
+  <si>
+    <t>2302182476445</t>
+  </si>
+  <si>
+    <t>BKPE5K</t>
+  </si>
+  <si>
+    <t>BKPFHW</t>
+  </si>
+  <si>
+    <t>BKPFK2</t>
+  </si>
+  <si>
+    <t>BKPFNZ</t>
+  </si>
+  <si>
+    <t>BKPFZ4</t>
+  </si>
+  <si>
+    <t>2302182476446</t>
+  </si>
+  <si>
+    <t>2302182476447</t>
+  </si>
+  <si>
+    <t>BKPF25</t>
+  </si>
+  <si>
+    <t>2302182476448</t>
+  </si>
+  <si>
+    <t>2302182476449</t>
+  </si>
+  <si>
+    <t>BKPGBF</t>
+  </si>
+  <si>
+    <t>3703101DCMCMRPCT08267CAF51</t>
+  </si>
+  <si>
+    <t>B1085BD4CMCMRPCT05D527ED98</t>
+  </si>
+  <si>
+    <t>CBBFCA1ECMCMRPCT07C358FC56</t>
+  </si>
+  <si>
+    <t>BKPK4O</t>
+  </si>
+  <si>
+    <t>2023-07-17T07:59:00</t>
+  </si>
+  <si>
+    <t>2023-07-17T12:07:00</t>
+  </si>
+  <si>
+    <t>BKPLOU</t>
+  </si>
+  <si>
+    <t>BKPW1B</t>
+  </si>
+  <si>
+    <t>BKPW2B</t>
+  </si>
+  <si>
+    <t>BKPW20</t>
+  </si>
+  <si>
+    <t>BKPW3E</t>
+  </si>
+  <si>
+    <t>BKPW4K</t>
+  </si>
+  <si>
+    <t>2023-07-14T06:25:26</t>
+  </si>
+  <si>
+    <t>BKPXAH</t>
+  </si>
+  <si>
+    <t>2023-07-14T06:25:34</t>
+  </si>
+  <si>
+    <t>BKPXGF</t>
+  </si>
+  <si>
+    <t>BKPXHF</t>
+  </si>
+  <si>
+    <t>BKPXWJ</t>
+  </si>
+  <si>
+    <t>BKPXYY</t>
+  </si>
+  <si>
+    <t>2302182476464</t>
+  </si>
+  <si>
+    <t>2302182476465</t>
+  </si>
+  <si>
+    <t>BKPXZN</t>
+  </si>
+  <si>
+    <t>2302182476466</t>
+  </si>
+  <si>
+    <t>2302182476467</t>
+  </si>
+  <si>
+    <t>BKPX0J</t>
+  </si>
+  <si>
+    <t>852B3E82CMCMRPCT0547B6E4F8</t>
+  </si>
+  <si>
+    <t>A2CB4E0ACMCMRPCT0633F7CA6D</t>
+  </si>
+  <si>
+    <t>AFA405E6CMCMRPCT0580BBCD97</t>
+  </si>
+  <si>
+    <t>BKPZKG</t>
+  </si>
+  <si>
+    <t>BKPZPD</t>
   </si>
 </sst>
 </file>
@@ -2597,7 +2780,7 @@
         <v>16</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>473</v>
+        <v>654</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>274</v>
@@ -2614,7 +2797,7 @@
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3" t="s">
-        <v>474</v>
+        <v>655</v>
       </c>
       <c r="P2" s="24"/>
     </row>
@@ -3152,10 +3335,10 @@
       <c r="I11" s="48"/>
       <c r="J11" s="48"/>
       <c r="K11" s="48" t="s">
-        <v>573</v>
+        <v>628</v>
       </c>
       <c r="L11" s="48" t="s">
-        <v>574</v>
+        <v>629</v>
       </c>
       <c r="M11" s="48"/>
       <c r="N11" s="48"/>
@@ -3234,10 +3417,10 @@
       <c r="I13" s="48"/>
       <c r="J13" s="48"/>
       <c r="K13" s="48" t="s">
-        <v>577</v>
+        <v>630</v>
       </c>
       <c r="L13" s="48" t="s">
-        <v>578</v>
+        <v>631</v>
       </c>
       <c r="M13" s="48"/>
       <c r="N13" s="48" t="s">
@@ -3312,10 +3495,10 @@
       <c r="I15" s="48"/>
       <c r="J15" s="48"/>
       <c r="K15" s="48" t="s">
-        <v>579</v>
+        <v>632</v>
       </c>
       <c r="L15" s="48" t="s">
-        <v>580</v>
+        <v>633</v>
       </c>
       <c r="M15" s="48"/>
       <c r="N15" s="48" t="s">
@@ -3355,7 +3538,7 @@
       <c r="I16" s="48"/>
       <c r="J16" s="48"/>
       <c r="K16" s="48" t="s">
-        <v>581</v>
+        <v>634</v>
       </c>
       <c r="L16" s="48"/>
       <c r="M16" s="48"/>
@@ -3437,7 +3620,7 @@
       </c>
       <c r="J18" s="48"/>
       <c r="K18" s="48" t="s">
-        <v>583</v>
+        <v>635</v>
       </c>
       <c r="L18" s="48"/>
       <c r="M18" s="48"/>
@@ -3515,7 +3698,7 @@
       <c r="I20" s="48"/>
       <c r="J20" s="48"/>
       <c r="K20" s="48" t="s">
-        <v>585</v>
+        <v>636</v>
       </c>
       <c r="L20" s="48"/>
       <c r="M20" s="48"/>
@@ -3554,7 +3737,7 @@
       <c r="I21" s="48"/>
       <c r="J21" s="48"/>
       <c r="K21" s="48" t="s">
-        <v>588</v>
+        <v>662</v>
       </c>
       <c r="L21" s="48"/>
       <c r="M21" s="48"/>
@@ -3654,10 +3837,10 @@
         <v>2</v>
       </c>
       <c r="D2" s="62" t="s">
-        <v>396</v>
+        <v>670</v>
       </c>
       <c r="E2" s="62" t="s">
-        <v>395</v>
+        <v>669</v>
       </c>
       <c r="F2" s="60"/>
       <c r="G2" s="63"/>
@@ -3673,7 +3856,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="62" t="s">
-        <v>602</v>
+        <v>671</v>
       </c>
       <c r="E3" s="62" t="s">
         <v>331</v>
@@ -3694,7 +3877,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="62" t="s">
-        <v>603</v>
+        <v>672</v>
       </c>
       <c r="E4" s="60"/>
       <c r="F4" s="60" t="s">
@@ -3822,13 +4005,13 @@
       <c r="G5" s="60"/>
       <c r="H5" s="60"/>
       <c r="I5" s="60" t="s">
-        <v>379</v>
+        <v>666</v>
       </c>
       <c r="J5" s="60" t="s">
-        <v>380</v>
+        <v>667</v>
       </c>
       <c r="K5" s="60" t="s">
-        <v>381</v>
+        <v>668</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4276,16 +4459,16 @@
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3" t="s">
-        <v>604</v>
+        <v>673</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>605</v>
+        <v>649</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>19</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>606</v>
+        <v>650</v>
       </c>
       <c r="N5" s="3" t="s">
         <v>13</v>
@@ -5363,7 +5546,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>607</v>
+        <v>674</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>387</v>
@@ -7276,10 +7459,10 @@
         <v>65</v>
       </c>
       <c r="H2" s="26" t="s">
-        <v>406</v>
+        <v>658</v>
       </c>
       <c r="I2" s="26" t="s">
-        <v>407</v>
+        <v>659</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -7925,7 +8108,7 @@
       <c r="M2" s="48"/>
       <c r="N2" s="48"/>
       <c r="O2" s="48" t="s">
-        <v>408</v>
+        <v>661</v>
       </c>
       <c r="P2" s="48"/>
     </row>
@@ -8526,10 +8709,10 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3" t="s">
-        <v>529</v>
+        <v>624</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>530</v>
+        <v>625</v>
       </c>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
@@ -8788,10 +8971,10 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3" t="s">
-        <v>531</v>
+        <v>626</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>532</v>
+        <v>627</v>
       </c>
       <c r="T8" s="3">
         <v>0</v>

</xml_diff>

<commit_message>
14/07/2023 - Command line execution is implemented
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1844" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1888" uniqueCount="696">
   <si>
     <t>Scenario</t>
   </si>
@@ -2091,6 +2091,69 @@
   </si>
   <si>
     <t>BKPZPD</t>
+  </si>
+  <si>
+    <t>BKSL1S</t>
+  </si>
+  <si>
+    <t>BKSMTH</t>
+  </si>
+  <si>
+    <t>BKSNAA</t>
+  </si>
+  <si>
+    <t>BKSNK3</t>
+  </si>
+  <si>
+    <t>BKSOQM</t>
+  </si>
+  <si>
+    <t>2023-07-14T07:36:46</t>
+  </si>
+  <si>
+    <t>BKSO3R</t>
+  </si>
+  <si>
+    <t>2023-07-14T07:36:55</t>
+  </si>
+  <si>
+    <t>BKSTSP</t>
+  </si>
+  <si>
+    <t>BKSUQJ</t>
+  </si>
+  <si>
+    <t>2302182476517</t>
+  </si>
+  <si>
+    <t>2302182476518</t>
+  </si>
+  <si>
+    <t>BKSUWK</t>
+  </si>
+  <si>
+    <t>2302182476519</t>
+  </si>
+  <si>
+    <t>2302182476520</t>
+  </si>
+  <si>
+    <t>BKSU3W</t>
+  </si>
+  <si>
+    <t>438C0373CMCMRPCT05C8D23EE3</t>
+  </si>
+  <si>
+    <t>3A9DD03ACMCMRPCT06CEC75A1A</t>
+  </si>
+  <si>
+    <t>87FF72DDCMCMRPCT05F085B079</t>
+  </si>
+  <si>
+    <t>BKS5ZE</t>
+  </si>
+  <si>
+    <t>BKTAYM</t>
   </si>
 </sst>
 </file>
@@ -2780,7 +2843,7 @@
         <v>16</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>654</v>
+        <v>677</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>274</v>
@@ -2797,7 +2860,7 @@
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3" t="s">
-        <v>655</v>
+        <v>678</v>
       </c>
       <c r="P2" s="24"/>
     </row>
@@ -3737,7 +3800,7 @@
       <c r="I21" s="48"/>
       <c r="J21" s="48"/>
       <c r="K21" s="48" t="s">
-        <v>662</v>
+        <v>683</v>
       </c>
       <c r="L21" s="48"/>
       <c r="M21" s="48"/>
@@ -3837,10 +3900,10 @@
         <v>2</v>
       </c>
       <c r="D2" s="62" t="s">
-        <v>670</v>
+        <v>691</v>
       </c>
       <c r="E2" s="62" t="s">
-        <v>669</v>
+        <v>690</v>
       </c>
       <c r="F2" s="60"/>
       <c r="G2" s="63"/>
@@ -3856,7 +3919,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="62" t="s">
-        <v>671</v>
+        <v>692</v>
       </c>
       <c r="E3" s="62" t="s">
         <v>331</v>
@@ -3877,7 +3940,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="62" t="s">
-        <v>672</v>
+        <v>693</v>
       </c>
       <c r="E4" s="60"/>
       <c r="F4" s="60" t="s">
@@ -4005,13 +4068,13 @@
       <c r="G5" s="60"/>
       <c r="H5" s="60"/>
       <c r="I5" s="60" t="s">
-        <v>666</v>
+        <v>687</v>
       </c>
       <c r="J5" s="60" t="s">
-        <v>667</v>
+        <v>688</v>
       </c>
       <c r="K5" s="60" t="s">
-        <v>668</v>
+        <v>689</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4459,7 +4522,7 @@
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3" t="s">
-        <v>673</v>
+        <v>694</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>649</v>
@@ -5546,7 +5609,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>674</v>
+        <v>695</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>387</v>
@@ -7459,10 +7522,10 @@
         <v>65</v>
       </c>
       <c r="H2" s="26" t="s">
-        <v>658</v>
+        <v>681</v>
       </c>
       <c r="I2" s="26" t="s">
-        <v>659</v>
+        <v>682</v>
       </c>
     </row>
     <row r="3" spans="1:9">

</xml_diff>

<commit_message>
20/07/2023 - Cleanup Completed - Implemented failTest(e) in catch block
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\COPA Automation Final\Copa_API_WebServices\src\test\java\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ArunJK\Arun\Copa_SHDWebservices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{819B26A9-F34C-4039-A732-7E8C24DC73EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82EFF842-C683-47FF-ACC8-4B571910F53C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="27" activeTab="30" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1888" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1532" uniqueCount="544">
   <si>
     <t>Scenario</t>
   </si>
@@ -1205,15 +1205,6 @@
     <t>Booking_multiple_tickets</t>
   </si>
   <si>
-    <t>BPHLTF</t>
-  </si>
-  <si>
-    <t>2302181199430</t>
-  </si>
-  <si>
-    <t>2302181199431</t>
-  </si>
-  <si>
     <t>Bulk_Ticket</t>
   </si>
   <si>
@@ -1235,201 +1226,15 @@
     <t>2024-03-10T06:42:00</t>
   </si>
   <si>
-    <t>2023-05-19T07:56:00</t>
-  </si>
-  <si>
-    <t>2023-05-19T12:35:00</t>
-  </si>
-  <si>
-    <t>2023-05-19T14:06:00</t>
-  </si>
-  <si>
-    <t>2023-05-19T15:40:00</t>
-  </si>
-  <si>
     <t>BODK0Y</t>
   </si>
   <si>
     <t>2302181834307</t>
   </si>
   <si>
-    <t>BODL51</t>
-  </si>
-  <si>
-    <t>22EE7770CMCMRPCT05339998DA</t>
-  </si>
-  <si>
     <t>BODNR1</t>
   </si>
   <si>
-    <t>BODOEH</t>
-  </si>
-  <si>
-    <t>2302181834330</t>
-  </si>
-  <si>
-    <t>AEE00K</t>
-  </si>
-  <si>
-    <t>2302181859853</t>
-  </si>
-  <si>
-    <t>AEE00Z</t>
-  </si>
-  <si>
-    <t>2302181859854</t>
-  </si>
-  <si>
-    <t>AE40MU</t>
-  </si>
-  <si>
-    <t>AE40NF</t>
-  </si>
-  <si>
-    <t>AE40OY</t>
-  </si>
-  <si>
-    <t>2023-06-02T06:21:30</t>
-  </si>
-  <si>
-    <t>AE40UK</t>
-  </si>
-  <si>
-    <t>AE40UZ</t>
-  </si>
-  <si>
-    <t>2302181862749</t>
-  </si>
-  <si>
-    <t>AE40XX</t>
-  </si>
-  <si>
-    <t>2302181862750</t>
-  </si>
-  <si>
-    <t>AE401F</t>
-  </si>
-  <si>
-    <t>2302181862753</t>
-  </si>
-  <si>
-    <t>AE404A</t>
-  </si>
-  <si>
-    <t>2302181862756</t>
-  </si>
-  <si>
-    <t>AE41CN</t>
-  </si>
-  <si>
-    <t>2302181862757</t>
-  </si>
-  <si>
-    <t>AE41D5</t>
-  </si>
-  <si>
-    <t>2302181862758</t>
-  </si>
-  <si>
-    <t>AE41EM</t>
-  </si>
-  <si>
-    <t>AE41FG</t>
-  </si>
-  <si>
-    <t>AE41FS</t>
-  </si>
-  <si>
-    <t>AE41II</t>
-  </si>
-  <si>
-    <t>AE41KD</t>
-  </si>
-  <si>
-    <t>AE41KP</t>
-  </si>
-  <si>
-    <t>2302181862759</t>
-  </si>
-  <si>
-    <t>AE41LH</t>
-  </si>
-  <si>
-    <t>AE41MP</t>
-  </si>
-  <si>
-    <t>2302181862760</t>
-  </si>
-  <si>
-    <t>AE41NE</t>
-  </si>
-  <si>
-    <t>AE41NJ</t>
-  </si>
-  <si>
-    <t>AE41T0</t>
-  </si>
-  <si>
-    <t>2302181862761</t>
-  </si>
-  <si>
-    <t>AE41UT</t>
-  </si>
-  <si>
-    <t>AE41WE</t>
-  </si>
-  <si>
-    <t>2302181862762</t>
-  </si>
-  <si>
-    <t>C7D87262CMCMRPCT061B0D311A</t>
-  </si>
-  <si>
-    <t>5966EED0CMCMRPCT05BA05D4AF</t>
-  </si>
-  <si>
-    <t>AE42NH</t>
-  </si>
-  <si>
-    <t>2023-06-05T07:53:00</t>
-  </si>
-  <si>
-    <t>2023-06-05T11:56:00</t>
-  </si>
-  <si>
-    <t>AE42PG</t>
-  </si>
-  <si>
-    <t>2023-06-03T07:55:00</t>
-  </si>
-  <si>
-    <t>2023-06-03T09:29:00</t>
-  </si>
-  <si>
-    <t>AE42PU</t>
-  </si>
-  <si>
-    <t>AE42P3</t>
-  </si>
-  <si>
-    <t>2302181862768</t>
-  </si>
-  <si>
-    <t>AE42RO</t>
-  </si>
-  <si>
-    <t>AE42SV</t>
-  </si>
-  <si>
-    <t>2302181862776</t>
-  </si>
-  <si>
-    <t>AE42TI</t>
-  </si>
-  <si>
-    <t>2302181862777</t>
-  </si>
-  <si>
     <t>Carrier Code</t>
   </si>
   <si>
@@ -1451,15 +1256,9 @@
     <t>Add Flight</t>
   </si>
   <si>
-    <t>AGY2HS</t>
-  </si>
-  <si>
     <t>Add Name</t>
   </si>
   <si>
-    <t>AGY2JA</t>
-  </si>
-  <si>
     <t>FOX</t>
   </si>
   <si>
@@ -1469,9 +1268,6 @@
     <t>Add Class</t>
   </si>
   <si>
-    <t>AGY2KG</t>
-  </si>
-  <si>
     <t>AGY3OI</t>
   </si>
   <si>
@@ -1481,123 +1277,6 @@
     <t>AGY3RY</t>
   </si>
   <si>
-    <t>AG3ZTC</t>
-  </si>
-  <si>
-    <t>AG3ZTN</t>
-  </si>
-  <si>
-    <t>AG3ZTO</t>
-  </si>
-  <si>
-    <t>AG3ZTP</t>
-  </si>
-  <si>
-    <t>AIOGZH</t>
-  </si>
-  <si>
-    <t>2302181869630</t>
-  </si>
-  <si>
-    <t>AIOG2P</t>
-  </si>
-  <si>
-    <t>2302181869631</t>
-  </si>
-  <si>
-    <t>AIOHAQ</t>
-  </si>
-  <si>
-    <t>2302181869632</t>
-  </si>
-  <si>
-    <t>AIOHBA</t>
-  </si>
-  <si>
-    <t>2302181869633</t>
-  </si>
-  <si>
-    <t>AIOHB3</t>
-  </si>
-  <si>
-    <t>2302181869634</t>
-  </si>
-  <si>
-    <t>AIOHDQ</t>
-  </si>
-  <si>
-    <t>2302181869635</t>
-  </si>
-  <si>
-    <t>AIOHEY</t>
-  </si>
-  <si>
-    <t>AIOHGT</t>
-  </si>
-  <si>
-    <t>AIOHHI</t>
-  </si>
-  <si>
-    <t>AIOHH5</t>
-  </si>
-  <si>
-    <t>AIOHKI</t>
-  </si>
-  <si>
-    <t>AIOHKX</t>
-  </si>
-  <si>
-    <t>2302181869636</t>
-  </si>
-  <si>
-    <t>AIOHL5</t>
-  </si>
-  <si>
-    <t>AIOHMU</t>
-  </si>
-  <si>
-    <t>2302181869637</t>
-  </si>
-  <si>
-    <t>AIOHNA</t>
-  </si>
-  <si>
-    <t>AIOHND</t>
-  </si>
-  <si>
-    <t>AIOHOA</t>
-  </si>
-  <si>
-    <t>2302181869638</t>
-  </si>
-  <si>
-    <t>AIOHOQ</t>
-  </si>
-  <si>
-    <t>2302181869639</t>
-  </si>
-  <si>
-    <t>AIOHPG</t>
-  </si>
-  <si>
-    <t>2302181869640</t>
-  </si>
-  <si>
-    <t>AIOHQS</t>
-  </si>
-  <si>
-    <t>AIOHRU</t>
-  </si>
-  <si>
-    <t>2302181869641</t>
-  </si>
-  <si>
-    <t>8AD54668CMCMRPCT0543C365BD</t>
-  </si>
-  <si>
-    <t>E2190C22CMCMRPCT0609952907</t>
-  </si>
-  <si>
     <t>AIOIXA</t>
   </si>
   <si>
@@ -1607,168 +1286,15 @@
     <t>2023-06-08T09:29:00</t>
   </si>
   <si>
-    <t>AIOIYA</t>
-  </si>
-  <si>
     <t>AIOIYZ</t>
   </si>
   <si>
     <t>2302181869645</t>
   </si>
   <si>
-    <t>AIOI0F</t>
-  </si>
-  <si>
-    <t>AIOI02</t>
-  </si>
-  <si>
     <t>AIOI1L</t>
   </si>
   <si>
-    <t>AIOI24</t>
-  </si>
-  <si>
-    <t>2302181869651</t>
-  </si>
-  <si>
-    <t>AIOI3U</t>
-  </si>
-  <si>
-    <t>2302181869652</t>
-  </si>
-  <si>
-    <t>AIOJAN</t>
-  </si>
-  <si>
-    <t>2023-06-08T07:38:00</t>
-  </si>
-  <si>
-    <t>2023-06-08T12:03:00</t>
-  </si>
-  <si>
-    <t>2023-06-08T14:09:00</t>
-  </si>
-  <si>
-    <t>2023-06-08T15:40:00</t>
-  </si>
-  <si>
-    <t>2302181869653</t>
-  </si>
-  <si>
-    <t>AISCAS</t>
-  </si>
-  <si>
-    <t>2302181869713</t>
-  </si>
-  <si>
-    <t>AISCFT</t>
-  </si>
-  <si>
-    <t>2302181869714</t>
-  </si>
-  <si>
-    <t>AISCG0</t>
-  </si>
-  <si>
-    <t>2302181869715</t>
-  </si>
-  <si>
-    <t>AISCHD</t>
-  </si>
-  <si>
-    <t>2302181869716</t>
-  </si>
-  <si>
-    <t>AISCKP</t>
-  </si>
-  <si>
-    <t>2302181869717</t>
-  </si>
-  <si>
-    <t>AISCQA</t>
-  </si>
-  <si>
-    <t>2302181869718</t>
-  </si>
-  <si>
-    <t>AISCUB</t>
-  </si>
-  <si>
-    <t>AISCVB</t>
-  </si>
-  <si>
-    <t>AISCY0</t>
-  </si>
-  <si>
-    <t>AISCZL</t>
-  </si>
-  <si>
-    <t>AISCZQ</t>
-  </si>
-  <si>
-    <t>AISCZ0</t>
-  </si>
-  <si>
-    <t>2302181869719</t>
-  </si>
-  <si>
-    <t>AISCZ4</t>
-  </si>
-  <si>
-    <t>AISC0X</t>
-  </si>
-  <si>
-    <t>2302181869720</t>
-  </si>
-  <si>
-    <t>AISC15</t>
-  </si>
-  <si>
-    <t>AISC2A</t>
-  </si>
-  <si>
-    <t>AISC2B</t>
-  </si>
-  <si>
-    <t>2302181869721</t>
-  </si>
-  <si>
-    <t>AISC2H</t>
-  </si>
-  <si>
-    <t>2302181869722</t>
-  </si>
-  <si>
-    <t>AISC3D</t>
-  </si>
-  <si>
-    <t>2302181869723</t>
-  </si>
-  <si>
-    <t>AISC3T</t>
-  </si>
-  <si>
-    <t>AISC3Z</t>
-  </si>
-  <si>
-    <t>2302181869724</t>
-  </si>
-  <si>
-    <t>9C754478CMCMRPCT073803E992</t>
-  </si>
-  <si>
-    <t>F87B0BF4CMCMRPCT07FAAA301D</t>
-  </si>
-  <si>
-    <t>AISDCT</t>
-  </si>
-  <si>
-    <t>AISDC1</t>
-  </si>
-  <si>
-    <t>2302181869727</t>
-  </si>
-  <si>
     <t>AWMGIE</t>
   </si>
   <si>
@@ -1787,54 +1313,24 @@
     <t>2302181931005</t>
   </si>
   <si>
-    <t>ACR3YZ</t>
-  </si>
-  <si>
-    <t>2302181955113</t>
-  </si>
-  <si>
     <t>ACR3ZE</t>
   </si>
   <si>
     <t>2302181955114</t>
   </si>
   <si>
-    <t>ACR4MQ</t>
-  </si>
-  <si>
-    <t>2302181955115</t>
-  </si>
-  <si>
-    <t>ACR4WT</t>
-  </si>
-  <si>
-    <t>2302181955116</t>
-  </si>
-  <si>
-    <t>ACR5AG</t>
-  </si>
-  <si>
     <t>ACR5AJ</t>
   </si>
   <si>
-    <t>ACR5AK</t>
-  </si>
-  <si>
     <t>ACR5AM</t>
   </si>
   <si>
-    <t>ACR5CF</t>
-  </si>
-  <si>
     <t>ACR5CL</t>
   </si>
   <si>
     <t>2302181955117</t>
   </si>
   <si>
-    <t>ACR5C4</t>
-  </si>
-  <si>
     <t>ACR5EH</t>
   </si>
   <si>
@@ -1874,24 +1370,6 @@
     <t>2302181955122</t>
   </si>
   <si>
-    <t>F2D74284CMCMRPCT05A93C421D</t>
-  </si>
-  <si>
-    <t>64CDDA06CMCMRPCT0807F2389E</t>
-  </si>
-  <si>
-    <t>ACSDT4</t>
-  </si>
-  <si>
-    <t>2023-07-10T07:53:00</t>
-  </si>
-  <si>
-    <t>2023-07-10T11:56:00</t>
-  </si>
-  <si>
-    <t>ACSDVL</t>
-  </si>
-  <si>
     <t>ACSFKM</t>
   </si>
   <si>
@@ -1910,36 +1388,6 @@
     <t>2302181955125</t>
   </si>
   <si>
-    <t>BKPAAC</t>
-  </si>
-  <si>
-    <t>BKPAIQ</t>
-  </si>
-  <si>
-    <t>BKPAME</t>
-  </si>
-  <si>
-    <t>BKPAO5</t>
-  </si>
-  <si>
-    <t>BKPAU4</t>
-  </si>
-  <si>
-    <t>2023-07-14T06:11:10</t>
-  </si>
-  <si>
-    <t>BKPA4Y</t>
-  </si>
-  <si>
-    <t>2023-07-14T06:11:18</t>
-  </si>
-  <si>
-    <t>BKPB2R</t>
-  </si>
-  <si>
-    <t>BKPB5B</t>
-  </si>
-  <si>
     <t>BKPCA2</t>
   </si>
   <si>
@@ -1979,138 +1427,15 @@
     <t>BKPFK2</t>
   </si>
   <si>
-    <t>BKPFNZ</t>
-  </si>
-  <si>
-    <t>BKPFZ4</t>
-  </si>
-  <si>
-    <t>2302182476446</t>
-  </si>
-  <si>
-    <t>2302182476447</t>
-  </si>
-  <si>
-    <t>BKPF25</t>
-  </si>
-  <si>
-    <t>2302182476448</t>
-  </si>
-  <si>
-    <t>2302182476449</t>
-  </si>
-  <si>
-    <t>BKPGBF</t>
-  </si>
-  <si>
-    <t>3703101DCMCMRPCT08267CAF51</t>
-  </si>
-  <si>
-    <t>B1085BD4CMCMRPCT05D527ED98</t>
-  </si>
-  <si>
-    <t>CBBFCA1ECMCMRPCT07C358FC56</t>
-  </si>
-  <si>
-    <t>BKPK4O</t>
-  </si>
-  <si>
     <t>2023-07-17T07:59:00</t>
   </si>
   <si>
     <t>2023-07-17T12:07:00</t>
   </si>
   <si>
-    <t>BKPLOU</t>
-  </si>
-  <si>
-    <t>BKPW1B</t>
-  </si>
-  <si>
-    <t>BKPW2B</t>
-  </si>
-  <si>
-    <t>BKPW20</t>
-  </si>
-  <si>
-    <t>BKPW3E</t>
-  </si>
-  <si>
-    <t>BKPW4K</t>
-  </si>
-  <si>
-    <t>2023-07-14T06:25:26</t>
-  </si>
-  <si>
-    <t>BKPXAH</t>
-  </si>
-  <si>
-    <t>2023-07-14T06:25:34</t>
-  </si>
-  <si>
-    <t>BKPXGF</t>
-  </si>
-  <si>
     <t>BKPXHF</t>
   </si>
   <si>
-    <t>BKPXWJ</t>
-  </si>
-  <si>
-    <t>BKPXYY</t>
-  </si>
-  <si>
-    <t>2302182476464</t>
-  </si>
-  <si>
-    <t>2302182476465</t>
-  </si>
-  <si>
-    <t>BKPXZN</t>
-  </si>
-  <si>
-    <t>2302182476466</t>
-  </si>
-  <si>
-    <t>2302182476467</t>
-  </si>
-  <si>
-    <t>BKPX0J</t>
-  </si>
-  <si>
-    <t>852B3E82CMCMRPCT0547B6E4F8</t>
-  </si>
-  <si>
-    <t>A2CB4E0ACMCMRPCT0633F7CA6D</t>
-  </si>
-  <si>
-    <t>AFA405E6CMCMRPCT0580BBCD97</t>
-  </si>
-  <si>
-    <t>BKPZKG</t>
-  </si>
-  <si>
-    <t>BKPZPD</t>
-  </si>
-  <si>
-    <t>BKSL1S</t>
-  </si>
-  <si>
-    <t>BKSMTH</t>
-  </si>
-  <si>
-    <t>BKSNAA</t>
-  </si>
-  <si>
-    <t>BKSNK3</t>
-  </si>
-  <si>
-    <t>BKSOQM</t>
-  </si>
-  <si>
-    <t>2023-07-14T07:36:46</t>
-  </si>
-  <si>
     <t>BKSO3R</t>
   </si>
   <si>
@@ -2120,15 +1445,6 @@
     <t>BKSTSP</t>
   </si>
   <si>
-    <t>BKSUQJ</t>
-  </si>
-  <si>
-    <t>2302182476517</t>
-  </si>
-  <si>
-    <t>2302182476518</t>
-  </si>
-  <si>
     <t>BKSUWK</t>
   </si>
   <si>
@@ -2154,6 +1470,234 @@
   </si>
   <si>
     <t>BKTAYM</t>
+  </si>
+  <si>
+    <t>BOFXGU</t>
+  </si>
+  <si>
+    <t>BOFXGV</t>
+  </si>
+  <si>
+    <t>BOHBI2</t>
+  </si>
+  <si>
+    <t>BOHBYS</t>
+  </si>
+  <si>
+    <t>BOHB4D</t>
+  </si>
+  <si>
+    <t>BOHB5M</t>
+  </si>
+  <si>
+    <t>BO2Z2E</t>
+  </si>
+  <si>
+    <t>BO2Z3G</t>
+  </si>
+  <si>
+    <t>2023-07-21T07:59:00</t>
+  </si>
+  <si>
+    <t>2023-07-21T12:07:00</t>
+  </si>
+  <si>
+    <t>2023-07-25T06:22:00</t>
+  </si>
+  <si>
+    <t>2023-07-25T08:32:00</t>
+  </si>
+  <si>
+    <t>BO2Z33</t>
+  </si>
+  <si>
+    <t>BO2Z4L</t>
+  </si>
+  <si>
+    <t>BO2Z4T</t>
+  </si>
+  <si>
+    <t>BO2Z5V</t>
+  </si>
+  <si>
+    <t>2023-07-20T06:19:55</t>
+  </si>
+  <si>
+    <t>BO20EG</t>
+  </si>
+  <si>
+    <t>2023-07-20T06:20:03</t>
+  </si>
+  <si>
+    <t>BO20IH</t>
+  </si>
+  <si>
+    <t>BO20IZ</t>
+  </si>
+  <si>
+    <t>BO20JR</t>
+  </si>
+  <si>
+    <t>2302182500173</t>
+  </si>
+  <si>
+    <t>BO20OM</t>
+  </si>
+  <si>
+    <t>2302182500174</t>
+  </si>
+  <si>
+    <t>BO20PH</t>
+  </si>
+  <si>
+    <t>2302182500175</t>
+  </si>
+  <si>
+    <t>BO20VH</t>
+  </si>
+  <si>
+    <t>2302182500177</t>
+  </si>
+  <si>
+    <t>BO20XK</t>
+  </si>
+  <si>
+    <t>2302182500178</t>
+  </si>
+  <si>
+    <t>BO20YY</t>
+  </si>
+  <si>
+    <t>2302182500179</t>
+  </si>
+  <si>
+    <t>BO201E</t>
+  </si>
+  <si>
+    <t>2302182500180</t>
+  </si>
+  <si>
+    <t>BO203N</t>
+  </si>
+  <si>
+    <t>BO2042</t>
+  </si>
+  <si>
+    <t>BO205P</t>
+  </si>
+  <si>
+    <t>BO21AP</t>
+  </si>
+  <si>
+    <t>BO21B2</t>
+  </si>
+  <si>
+    <t>BO21C3</t>
+  </si>
+  <si>
+    <t>2302182500181</t>
+  </si>
+  <si>
+    <t>BO21EE</t>
+  </si>
+  <si>
+    <t>BO21E5</t>
+  </si>
+  <si>
+    <t>2302182500182</t>
+  </si>
+  <si>
+    <t>BO21F4</t>
+  </si>
+  <si>
+    <t>BO21GG</t>
+  </si>
+  <si>
+    <t>BO21G0</t>
+  </si>
+  <si>
+    <t>2302182500183</t>
+  </si>
+  <si>
+    <t>BO21IJ</t>
+  </si>
+  <si>
+    <t>2302182500184</t>
+  </si>
+  <si>
+    <t>BO21JO</t>
+  </si>
+  <si>
+    <t>2302182500185</t>
+  </si>
+  <si>
+    <t>BO21KR</t>
+  </si>
+  <si>
+    <t>BO21L4</t>
+  </si>
+  <si>
+    <t>2302182500186</t>
+  </si>
+  <si>
+    <t>BO21NY</t>
+  </si>
+  <si>
+    <t>2302182500187</t>
+  </si>
+  <si>
+    <t>2302182500188</t>
+  </si>
+  <si>
+    <t>BO21QA</t>
+  </si>
+  <si>
+    <t>2302182500189</t>
+  </si>
+  <si>
+    <t>2302182500190</t>
+  </si>
+  <si>
+    <t>BO21TA</t>
+  </si>
+  <si>
+    <t>8B3FE1E8CMCMRPCT069905EE9C</t>
+  </si>
+  <si>
+    <t>6A2E6A7ECMCMRPCT07AF12B404</t>
+  </si>
+  <si>
+    <t>96D65F1ACMCMRPCT053BF6616C</t>
+  </si>
+  <si>
+    <t>BO223M</t>
+  </si>
+  <si>
+    <t>2023-07-23T07:59:00</t>
+  </si>
+  <si>
+    <t>2023-07-23T12:07:00</t>
+  </si>
+  <si>
+    <t>BO23AW</t>
+  </si>
+  <si>
+    <t>BO23JG</t>
+  </si>
+  <si>
+    <t>2023-07-21T07:47:00</t>
+  </si>
+  <si>
+    <t>2023-07-21T12:23:00</t>
+  </si>
+  <si>
+    <t>2023-07-21T14:02:00</t>
+  </si>
+  <si>
+    <t>2023-07-21T15:33:00</t>
+  </si>
+  <si>
+    <t>2302182500195</t>
   </si>
 </sst>
 </file>
@@ -2755,22 +2299,22 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:P15"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="52.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="11.26953125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.26953125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="11.26953125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.1796875"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="52.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -2827,7 +2371,7 @@
       <c r="B2" s="3">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="62" t="s">
         <v>12</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -2843,7 +2387,7 @@
         <v>16</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>677</v>
+        <v>481</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>274</v>
@@ -2860,7 +2404,7 @@
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3" t="s">
-        <v>678</v>
+        <v>482</v>
       </c>
       <c r="P2" s="24"/>
     </row>
@@ -2871,7 +2415,7 @@
       <c r="B3" s="3">
         <v>4</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="62" t="s">
         <v>19</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -2930,10 +2474,10 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C501783-003E-43C7-BF08-448ED073E85B}">
   <dimension ref="A1:U22"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="10" max="10" style="45" width="8.7265625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="10" max="10" style="45" width="8.77734375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -3068,10 +2612,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="48" t="s">
-        <v>586</v>
+        <v>508</v>
       </c>
       <c r="L3" s="48" t="s">
-        <v>587</v>
+        <v>509</v>
       </c>
       <c r="M3" s="48"/>
       <c r="N3" s="48"/>
@@ -3132,10 +2676,10 @@
       <c r="I5" s="48"/>
       <c r="J5" s="48"/>
       <c r="K5" s="48" t="s">
-        <v>589</v>
+        <v>511</v>
       </c>
       <c r="L5" s="48" t="s">
-        <v>590</v>
+        <v>512</v>
       </c>
       <c r="M5" s="48"/>
       <c r="N5" s="48" t="s">
@@ -3179,7 +2723,7 @@
       <c r="I6" s="48"/>
       <c r="J6" s="48"/>
       <c r="K6" s="48" t="s">
-        <v>591</v>
+        <v>513</v>
       </c>
       <c r="L6" s="48"/>
       <c r="M6" s="48"/>
@@ -3190,7 +2734,7 @@
         <v>308</v>
       </c>
       <c r="P6" s="48" t="s">
-        <v>592</v>
+        <v>514</v>
       </c>
       <c r="Q6" s="37"/>
       <c r="R6" s="48"/>
@@ -3224,10 +2768,10 @@
       <c r="I7" s="48"/>
       <c r="J7" s="48"/>
       <c r="K7" s="48" t="s">
-        <v>593</v>
+        <v>515</v>
       </c>
       <c r="L7" s="48" t="s">
-        <v>594</v>
+        <v>516</v>
       </c>
       <c r="M7" s="48"/>
       <c r="N7" s="48" t="s">
@@ -3237,13 +2781,13 @@
         <v>308</v>
       </c>
       <c r="P7" s="48" t="s">
-        <v>595</v>
+        <v>517</v>
       </c>
       <c r="Q7" s="55" t="s">
         <v>121</v>
       </c>
       <c r="R7" s="48" t="s">
-        <v>596</v>
+        <v>518</v>
       </c>
       <c r="S7" s="48"/>
       <c r="T7" s="48"/>
@@ -3279,10 +2823,10 @@
       </c>
       <c r="J8" s="48"/>
       <c r="K8" s="48" t="s">
-        <v>597</v>
+        <v>519</v>
       </c>
       <c r="L8" s="48" t="s">
-        <v>598</v>
+        <v>520</v>
       </c>
       <c r="M8" s="48"/>
       <c r="N8" s="48" t="s">
@@ -3320,7 +2864,7 @@
       <c r="I9" s="48"/>
       <c r="J9" s="48"/>
       <c r="K9" s="48" t="s">
-        <v>599</v>
+        <v>521</v>
       </c>
       <c r="L9" s="48"/>
       <c r="M9" s="48"/>
@@ -3359,10 +2903,10 @@
       <c r="I10" s="48"/>
       <c r="J10" s="48"/>
       <c r="K10" s="48" t="s">
-        <v>600</v>
+        <v>522</v>
       </c>
       <c r="L10" s="48" t="s">
-        <v>601</v>
+        <v>523</v>
       </c>
       <c r="M10" s="48"/>
       <c r="N10" s="48"/>
@@ -3398,10 +2942,10 @@
       <c r="I11" s="48"/>
       <c r="J11" s="48"/>
       <c r="K11" s="48" t="s">
-        <v>628</v>
+        <v>495</v>
       </c>
       <c r="L11" s="48" t="s">
-        <v>629</v>
+        <v>496</v>
       </c>
       <c r="M11" s="48"/>
       <c r="N11" s="48"/>
@@ -3437,10 +2981,10 @@
       <c r="I12" s="48"/>
       <c r="J12" s="48"/>
       <c r="K12" s="48" t="s">
-        <v>575</v>
+        <v>497</v>
       </c>
       <c r="L12" s="48" t="s">
-        <v>576</v>
+        <v>498</v>
       </c>
       <c r="M12" s="48"/>
       <c r="N12" s="48" t="s">
@@ -3480,10 +3024,10 @@
       <c r="I13" s="48"/>
       <c r="J13" s="48"/>
       <c r="K13" s="48" t="s">
-        <v>630</v>
+        <v>499</v>
       </c>
       <c r="L13" s="48" t="s">
-        <v>631</v>
+        <v>500</v>
       </c>
       <c r="M13" s="48"/>
       <c r="N13" s="48" t="s">
@@ -3558,10 +3102,10 @@
       <c r="I15" s="48"/>
       <c r="J15" s="48"/>
       <c r="K15" s="48" t="s">
-        <v>632</v>
+        <v>501</v>
       </c>
       <c r="L15" s="48" t="s">
-        <v>633</v>
+        <v>502</v>
       </c>
       <c r="M15" s="48"/>
       <c r="N15" s="48" t="s">
@@ -3601,7 +3145,7 @@
       <c r="I16" s="48"/>
       <c r="J16" s="48"/>
       <c r="K16" s="48" t="s">
-        <v>634</v>
+        <v>503</v>
       </c>
       <c r="L16" s="48"/>
       <c r="M16" s="48"/>
@@ -3640,7 +3184,7 @@
       <c r="I17" s="48"/>
       <c r="J17" s="48"/>
       <c r="K17" s="48" t="s">
-        <v>582</v>
+        <v>504</v>
       </c>
       <c r="L17" s="48"/>
       <c r="M17" s="48"/>
@@ -3683,7 +3227,7 @@
       </c>
       <c r="J18" s="48"/>
       <c r="K18" s="48" t="s">
-        <v>635</v>
+        <v>505</v>
       </c>
       <c r="L18" s="48"/>
       <c r="M18" s="48"/>
@@ -3722,7 +3266,7 @@
       <c r="I19" s="48"/>
       <c r="J19" s="48"/>
       <c r="K19" s="48" t="s">
-        <v>584</v>
+        <v>506</v>
       </c>
       <c r="L19" s="48"/>
       <c r="M19" s="48"/>
@@ -3761,7 +3305,7 @@
       <c r="I20" s="48"/>
       <c r="J20" s="48"/>
       <c r="K20" s="48" t="s">
-        <v>636</v>
+        <v>507</v>
       </c>
       <c r="L20" s="48"/>
       <c r="M20" s="48"/>
@@ -3800,7 +3344,7 @@
       <c r="I21" s="48"/>
       <c r="J21" s="48"/>
       <c r="K21" s="48" t="s">
-        <v>683</v>
+        <v>510</v>
       </c>
       <c r="L21" s="48"/>
       <c r="M21" s="48"/>
@@ -3858,14 +3402,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2EA1F88-8B75-4AAD-A17A-063CA3659CA4}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="14.36328125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="30.36328125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.90625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="10.90625"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.88671875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="14.33203125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="30.33203125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.88671875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -3900,10 +3444,10 @@
         <v>2</v>
       </c>
       <c r="D2" s="62" t="s">
-        <v>691</v>
+        <v>531</v>
       </c>
       <c r="E2" s="62" t="s">
-        <v>690</v>
+        <v>530</v>
       </c>
       <c r="F2" s="60"/>
       <c r="G2" s="63"/>
@@ -3919,7 +3463,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="62" t="s">
-        <v>692</v>
+        <v>532</v>
       </c>
       <c r="E3" s="62" t="s">
         <v>331</v>
@@ -3940,7 +3484,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="62" t="s">
-        <v>693</v>
+        <v>533</v>
       </c>
       <c r="E4" s="60"/>
       <c r="F4" s="60" t="s">
@@ -3956,18 +3500,18 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88414653-50FA-4845-96AF-5B777BBDF907}">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="57" width="18.26953125"/>
-    <col min="2" max="2" customWidth="true" style="57" width="16.54296875"/>
-    <col min="3" max="3" customWidth="true" style="57" width="19.90625"/>
-    <col min="4" max="4" customWidth="true" style="57" width="18.81640625"/>
-    <col min="5" max="5" customWidth="true" style="57" width="12.90625"/>
+    <col min="1" max="1" customWidth="true" style="57" width="18.21875"/>
+    <col min="2" max="2" customWidth="true" style="57" width="16.5546875"/>
+    <col min="3" max="3" customWidth="true" style="57" width="19.88671875"/>
+    <col min="4" max="4" customWidth="true" style="57" width="18.77734375"/>
+    <col min="5" max="5" customWidth="true" style="57" width="12.88671875"/>
     <col min="6" max="8" customWidth="true" hidden="true" style="57" width="0.0"/>
-    <col min="9" max="9" style="57" width="8.7265625"/>
-    <col min="10" max="10" customWidth="true" style="57" width="17.90625"/>
-    <col min="11" max="11" customWidth="true" style="57" width="14.26953125"/>
-    <col min="12" max="16384" style="57" width="8.7265625"/>
+    <col min="9" max="9" style="57" width="8.77734375"/>
+    <col min="10" max="10" customWidth="true" style="57" width="17.88671875"/>
+    <col min="11" max="11" customWidth="true" style="57" width="14.21875"/>
+    <col min="12" max="16384" style="57" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -4068,18 +3612,18 @@
       <c r="G5" s="60"/>
       <c r="H5" s="60"/>
       <c r="I5" s="60" t="s">
-        <v>687</v>
+        <v>527</v>
       </c>
       <c r="J5" s="60" t="s">
-        <v>688</v>
+        <v>528</v>
       </c>
       <c r="K5" s="60" t="s">
-        <v>689</v>
+        <v>529</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="60" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B6" s="60"/>
       <c r="C6" s="60">
@@ -4106,14 +3650,14 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1F0BBC0-8387-4A2B-855A-0B1CE735F165}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="57" width="15.08984375"/>
-    <col min="2" max="2" customWidth="true" style="57" width="15.7265625"/>
-    <col min="3" max="3" customWidth="true" style="57" width="17.81640625"/>
-    <col min="4" max="4" customWidth="true" style="57" width="16.7265625"/>
-    <col min="5" max="5" customWidth="true" style="57" width="15.6328125"/>
-    <col min="6" max="16384" style="57" width="8.7265625"/>
+    <col min="1" max="1" customWidth="true" style="57" width="15.109375"/>
+    <col min="2" max="2" customWidth="true" style="57" width="15.77734375"/>
+    <col min="3" max="3" customWidth="true" style="57" width="17.77734375"/>
+    <col min="4" max="4" customWidth="true" style="57" width="16.77734375"/>
+    <col min="5" max="5" customWidth="true" style="57" width="15.6640625"/>
+    <col min="6" max="16384" style="57" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4189,22 +3733,22 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AB6"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="51.7265625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="14.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" customWidth="true" width="51.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.44140625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="12.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -4322,31 +3866,31 @@
         <v>13</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>102</v>
+        <v>475</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>103</v>
+        <v>476</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>85</v>
+        <v>19</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>104</v>
+        <v>477</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>105</v>
+        <v>478</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>101</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>106</v>
+        <v>479</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>14</v>
@@ -4392,16 +3936,16 @@
         <v>13</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>237</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>13</v>
@@ -4410,13 +3954,13 @@
         <v>14</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="Q3" s="3" t="s">
         <v>238</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>14</v>
@@ -4522,16 +4066,16 @@
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3" t="s">
-        <v>694</v>
+        <v>534</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>649</v>
+        <v>535</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>19</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>650</v>
+        <v>536</v>
       </c>
       <c r="N5" s="3" t="s">
         <v>13</v>
@@ -4621,12 +4165,12 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="76.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="76.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="13.44140625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4704,14 +4248,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEA2AF7E-AC89-4B47-B4D7-D3496E5327D5}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="57" width="18.453125"/>
-    <col min="2" max="2" customWidth="true" style="57" width="12.54296875"/>
-    <col min="3" max="3" customWidth="true" style="57" width="14.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="57" width="11.7265625"/>
-    <col min="5" max="5" customWidth="true" style="57" width="18.1796875"/>
-    <col min="6" max="16384" style="57" width="8.7265625"/>
+    <col min="1" max="1" customWidth="true" style="57" width="18.44140625"/>
+    <col min="2" max="2" customWidth="true" style="57" width="12.5546875"/>
+    <col min="3" max="3" customWidth="true" style="57" width="14.77734375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="57" width="11.77734375"/>
+    <col min="5" max="5" customWidth="true" style="57" width="18.21875"/>
+    <col min="6" max="16384" style="57" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4901,10 +4445,10 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F1569B0-3564-4B84-A0FB-9681D32A0E6D}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.54296875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.5546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -4939,13 +4483,13 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02A4FAA4-EFC6-47D3-BDEE-7F4F3353F3CD}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.5546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.44140625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4990,7 +4534,7 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA6A106B-75A4-4F54-9508-A66A4AEED06E}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="6" t="s">
@@ -5092,32 +4636,32 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AG4"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="49.7265625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="4.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.7265625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="9.7265625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="9.7265625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.7265625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="9.7265625"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="9.7265625"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="9.7265625"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="49.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="4.77734375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="5.44140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -5424,9 +4968,9 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4903F224-3652-48FB-81A7-CAF06A9D7463}">
   <dimension ref="A1:AD9"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30">
@@ -5545,16 +5089,16 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
-        <v>510</v>
+        <v>403</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>511</v>
+        <v>404</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>48</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>512</v>
+        <v>405</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>13</v>
@@ -5609,16 +5153,16 @@
         <v>2</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>695</v>
+        <v>537</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>222</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>36</v>
@@ -5733,16 +5277,16 @@
         <v>5</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>514</v>
+        <v>406</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>511</v>
+        <v>404</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>48</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>512</v>
+        <v>405</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>13</v>
@@ -5751,7 +5295,7 @@
         <v>49</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>515</v>
+        <v>407</v>
       </c>
       <c r="R5" s="18" t="s">
         <v>48</v>
@@ -5941,16 +5485,16 @@
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3" t="s">
-        <v>518</v>
+        <v>408</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>511</v>
+        <v>404</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>48</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>512</v>
+        <v>405</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>13</v>
@@ -5984,13 +5528,13 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="35.26953125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.54296875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="35.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.5546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.44140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -6069,10 +5613,10 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB53E397-0E70-4FE2-8956-CAC505C79FBA}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.5546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.44140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -6123,10 +5667,10 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71142910-3363-4189-996E-89090332A376}">
   <dimension ref="A1:AC4"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" customWidth="true" width="6.26953125"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="5" max="5" customWidth="true" width="6.21875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="13.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -6254,16 +5798,16 @@
       <c r="U2" s="3"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3" t="s">
-        <v>567</v>
+        <v>409</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>568</v>
+        <v>410</v>
       </c>
       <c r="Y2" s="3" t="s">
         <v>48</v>
       </c>
       <c r="Z2" s="3" t="s">
-        <v>569</v>
+        <v>411</v>
       </c>
       <c r="AA2" s="3" t="s">
         <v>13</v>
@@ -6272,7 +5816,7 @@
         <v>49</v>
       </c>
       <c r="AC2" s="3" t="s">
-        <v>570</v>
+        <v>412</v>
       </c>
     </row>
     <row r="3" spans="1:29">
@@ -6382,16 +5926,16 @@
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3" t="s">
-        <v>571</v>
+        <v>413</v>
       </c>
       <c r="X4" s="3" t="s">
-        <v>568</v>
+        <v>410</v>
       </c>
       <c r="Y4" s="3" t="s">
         <v>48</v>
       </c>
       <c r="Z4" s="3" t="s">
-        <v>569</v>
+        <v>411</v>
       </c>
       <c r="AA4" s="3" t="s">
         <v>13</v>
@@ -6400,7 +5944,7 @@
         <v>49</v>
       </c>
       <c r="AC4" s="3" t="s">
-        <v>572</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>
@@ -6414,16 +5958,16 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="63.7265625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="10.7265625"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="63.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="10.77734375"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="19.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="19.44140625"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="15.54296875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="15.5546875"/>
     <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="8" max="9" bestFit="true" customWidth="true" width="19.453125"/>
+    <col min="8" max="9" bestFit="true" customWidth="true" width="19.44140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -6554,25 +6098,25 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:R6"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="12.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.26953125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.81640625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="7.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="11.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.77734375"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="7.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="11.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -6836,7 +6380,7 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42BBEF64-F0EA-4EA8-9A62-F5A7DF1E4869}">
   <dimension ref="A1:U13"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" s="39" t="s">
@@ -6932,16 +6476,16 @@
         <v>208</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>608</v>
+        <v>538</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>609</v>
+        <v>539</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>278</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>610</v>
+        <v>540</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>13</v>
@@ -6950,13 +6494,13 @@
         <v>279</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>611</v>
+        <v>541</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>280</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>612</v>
+        <v>542</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>279</v>
@@ -6965,7 +6509,7 @@
         <v>208</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>613</v>
+        <v>543</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -7148,10 +6692,10 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.26953125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -7194,7 +6738,7 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A51EFA8C-67A7-4B7E-8EF6-A12213F165A5}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="6" t="s">
@@ -7247,11 +6791,11 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFCF6FDB-3B87-457C-A3CA-7B39CE849651}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="57" width="24.90625"/>
-    <col min="2" max="2" customWidth="true" style="57" width="17.453125"/>
-    <col min="3" max="16384" style="57" width="8.7265625"/>
+    <col min="1" max="1" customWidth="true" style="57" width="24.88671875"/>
+    <col min="2" max="2" customWidth="true" style="57" width="17.44140625"/>
+    <col min="3" max="16384" style="57" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -7458,16 +7002,16 @@
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="21.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="6.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.44140625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="21.77734375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="6.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="18.44140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -7522,10 +7066,10 @@
         <v>65</v>
       </c>
       <c r="H2" s="26" t="s">
-        <v>681</v>
+        <v>485</v>
       </c>
       <c r="I2" s="26" t="s">
-        <v>682</v>
+        <v>486</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -7565,17 +7109,17 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:M5"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.26953125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="4" max="4" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="4" max="4" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.5546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -7729,18 +7273,18 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C03B3B8-DBFD-430F-BAEF-858DA603C137}">
   <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="57" width="17.90625"/>
-    <col min="2" max="2" customWidth="true" style="57" width="11.81640625"/>
+    <col min="1" max="1" customWidth="true" style="57" width="17.88671875"/>
+    <col min="2" max="2" customWidth="true" style="57" width="11.77734375"/>
     <col min="3" max="3" customWidth="true" style="57" width="13.0"/>
-    <col min="4" max="4" customWidth="true" style="57" width="16.54296875"/>
-    <col min="5" max="5" customWidth="true" style="57" width="15.81640625"/>
-    <col min="6" max="6" style="57" width="8.7265625"/>
-    <col min="7" max="7" customWidth="true" style="57" width="17.81640625"/>
-    <col min="8" max="8" customWidth="true" style="57" width="15.453125"/>
-    <col min="9" max="9" customWidth="true" style="57" width="11.54296875"/>
-    <col min="10" max="16384" style="57" width="8.7265625"/>
+    <col min="4" max="4" customWidth="true" style="57" width="16.5546875"/>
+    <col min="5" max="5" customWidth="true" style="57" width="15.77734375"/>
+    <col min="6" max="6" style="57" width="8.77734375"/>
+    <col min="7" max="7" customWidth="true" style="57" width="17.77734375"/>
+    <col min="8" max="8" customWidth="true" style="57" width="15.44140625"/>
+    <col min="9" max="9" customWidth="true" style="57" width="11.5546875"/>
+    <col min="10" max="16384" style="57" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -7748,7 +7292,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="61" t="s">
-        <v>454</v>
+        <v>389</v>
       </c>
       <c r="C1" s="61" t="s">
         <v>1</v>
@@ -7763,24 +7307,24 @@
         <v>98</v>
       </c>
       <c r="G1" s="61" t="s">
-        <v>455</v>
+        <v>390</v>
       </c>
       <c r="H1" s="61" t="s">
-        <v>456</v>
+        <v>391</v>
       </c>
       <c r="I1" s="61" t="s">
-        <v>457</v>
+        <v>392</v>
       </c>
       <c r="J1" s="61" t="s">
-        <v>458</v>
+        <v>393</v>
       </c>
       <c r="K1" s="61" t="s">
-        <v>459</v>
+        <v>394</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="60" t="s">
-        <v>460</v>
+        <v>395</v>
       </c>
       <c r="B2" s="60" t="s">
         <v>194</v>
@@ -7795,7 +7339,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="60" t="s">
-        <v>468</v>
+        <v>400</v>
       </c>
       <c r="G2" s="60">
         <v>2</v>
@@ -7811,7 +7355,7 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="60" t="s">
-        <v>462</v>
+        <v>396</v>
       </c>
       <c r="B3" s="60" t="s">
         <v>194</v>
@@ -7826,21 +7370,21 @@
         <v>1</v>
       </c>
       <c r="F3" s="60" t="s">
-        <v>469</v>
+        <v>401</v>
       </c>
       <c r="G3" s="60"/>
       <c r="H3" s="60"/>
       <c r="I3" s="60"/>
       <c r="J3" s="62" t="s">
-        <v>464</v>
+        <v>397</v>
       </c>
       <c r="K3" s="60" t="s">
-        <v>465</v>
+        <v>398</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="60" t="s">
-        <v>466</v>
+        <v>399</v>
       </c>
       <c r="B4" s="60" t="s">
         <v>194</v>
@@ -7855,7 +7399,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="60" t="s">
-        <v>470</v>
+        <v>402</v>
       </c>
       <c r="G4" s="60"/>
       <c r="H4" s="60"/>
@@ -7874,13 +7418,13 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.7265625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.7265625"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.44140625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.77734375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -7946,13 +7490,12 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="57.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="15.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.7265625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="11.26953125"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="57.44140625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="15.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.77734375"/>
+    <col min="4" max="5" bestFit="true" customWidth="true" width="11.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -8067,24 +7610,24 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" style="45" width="42.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="45" width="18.36328125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="45" width="12.08984375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="45" width="15.36328125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="45" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="45" width="9.453125"/>
-    <col min="7" max="8" style="45" width="8.7265625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="45" width="10.453125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="45" width="11.26953125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="45" width="10.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="45" width="11.26953125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="45" width="10.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="45" width="8.26953125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="45" width="18.33203125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="45" width="12.109375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="45" width="15.33203125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="45" width="12.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="45" width="9.44140625"/>
+    <col min="7" max="8" style="45" width="8.77734375"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="45" width="10.44140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="45" width="11.21875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="45" width="10.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="45" width="11.21875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="45" width="10.44140625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="45" width="8.21875"/>
     <col min="15" max="15" customWidth="true" style="45" width="13.0"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="45" width="10.1796875"/>
-    <col min="17" max="16384" style="45" width="8.7265625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="45" width="10.21875"/>
+    <col min="17" max="16384" style="45" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -8171,7 +7714,7 @@
       <c r="M2" s="48"/>
       <c r="N2" s="48"/>
       <c r="O2" s="48" t="s">
-        <v>661</v>
+        <v>488</v>
       </c>
       <c r="P2" s="48"/>
     </row>
@@ -8276,31 +7819,31 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="44.7265625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.7265625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="44.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.77734375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="8.21875"/>
     <col min="4" max="4" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="11.26953125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="13.54296875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.7265625"/>
-    <col min="11" max="12" bestFit="true" customWidth="true" width="11.26953125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.1796875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="13.5546875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.77734375"/>
+    <col min="11" max="12" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.21875"/>
     <col min="16" max="16" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="7.7265625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="11.26953125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="8.26953125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="7.77734375"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="8.21875"/>
     <col min="22" max="22" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="11.26953125"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="11.21875"/>
     <col min="24" max="24" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="11.26953125"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="14.26953125"/>
-    <col min="27" max="28" bestFit="true" customWidth="true" width="12.81640625"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="14.26953125"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="12.81640625"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="14.21875"/>
+    <col min="27" max="28" bestFit="true" customWidth="true" width="12.77734375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="14.21875"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="12.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -8665,11 +8208,11 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:W17"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="54.36328125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="54.33203125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="13.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -8772,10 +8315,10 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3" t="s">
-        <v>624</v>
+        <v>489</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>625</v>
+        <v>490</v>
       </c>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
@@ -9034,10 +8577,10 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3" t="s">
-        <v>626</v>
+        <v>491</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>627</v>
+        <v>492</v>
       </c>
       <c r="T8" s="3">
         <v>0</v>
@@ -9083,10 +8626,10 @@
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
       <c r="R9" s="3" t="s">
-        <v>255</v>
+        <v>493</v>
       </c>
       <c r="S9" s="3" t="s">
-        <v>256</v>
+        <v>494</v>
       </c>
       <c r="T9" s="3"/>
       <c r="U9" s="3">
@@ -9362,10 +8905,10 @@
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
       <c r="R16" s="3" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="S16" s="3" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>
@@ -9418,18 +8961,18 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:S20"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="53.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="5" max="7" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="53.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="4" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="5" max="7" customWidth="true" width="12.21875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">

</xml_diff>

<commit_message>
Updated AdvancePassengerInfo by implementing Generic/RESTWrapper/postResponse()
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
@@ -47,7 +47,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1385" uniqueCount="470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1417" uniqueCount="482">
   <si>
     <t>Scenario</t>
   </si>
@@ -1476,12 +1476,49 @@
   </si>
   <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>ACYUM3</t>
+  </si>
+  <si>
+    <t>ACYXQA</t>
+  </si>
+  <si>
+    <t>ACYX1J</t>
+  </si>
+  <si>
+    <t>ACYZAP</t>
+  </si>
+  <si>
+    <t>ACYZCC</t>
+  </si>
+  <si>
+    <t>2023-07-28T07:59:00</t>
+  </si>
+  <si>
+    <t>2023-07-28T12:07:00</t>
+  </si>
+  <si>
+    <t>2023-08-01T06:26:00</t>
+  </si>
+  <si>
+    <t>2023-08-01T08:32:00</t>
+  </si>
+  <si>
+    <t>ACYZC4</t>
+  </si>
+  <si>
+    <t>ACYZDF</t>
+  </si>
+  <si>
+    <t>ACYZEH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="9">
     <font>
       <sz val="11"/>
@@ -2078,20 +2115,20 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="52.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="52.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -2164,7 +2201,7 @@
         <v>16</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>434</v>
+        <v>480</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>266</v>
@@ -2181,7 +2218,7 @@
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3" t="s">
-        <v>435</v>
+        <v>481</v>
       </c>
       <c r="P2" s="24"/>
     </row>
@@ -2253,8 +2290,8 @@
   <dimension ref="A1:U22"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="10" max="10" width="8.81640625" style="45"/>
-    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" style="45" width="8.81640625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -3181,12 +3218,12 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="14.36328125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="30.36328125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.90625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -3279,16 +3316,16 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="18.1796875" style="57" customWidth="1"/>
-    <col min="2" max="2" width="16.54296875" style="57" customWidth="1"/>
-    <col min="3" max="3" width="19.90625" style="57" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" style="57" customWidth="1"/>
-    <col min="5" max="5" width="12.90625" style="57" customWidth="1"/>
-    <col min="6" max="8" width="0" style="57" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="8.81640625" style="57"/>
-    <col min="10" max="10" width="17.90625" style="57" customWidth="1"/>
-    <col min="11" max="11" width="14.1796875" style="57" customWidth="1"/>
-    <col min="12" max="16384" width="8.81640625" style="57"/>
+    <col min="1" max="1" customWidth="true" style="57" width="18.1796875"/>
+    <col min="2" max="2" customWidth="true" style="57" width="16.54296875"/>
+    <col min="3" max="3" customWidth="true" style="57" width="19.90625"/>
+    <col min="4" max="4" customWidth="true" style="57" width="18.81640625"/>
+    <col min="5" max="5" customWidth="true" style="57" width="12.90625"/>
+    <col min="6" max="8" customWidth="true" hidden="true" style="57" width="0.0"/>
+    <col min="9" max="9" style="57" width="8.81640625"/>
+    <col min="10" max="10" customWidth="true" style="57" width="17.90625"/>
+    <col min="11" max="11" customWidth="true" style="57" width="14.1796875"/>
+    <col min="12" max="16384" style="57" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -3429,12 +3466,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="15.08984375" style="57" customWidth="1"/>
-    <col min="2" max="2" width="15.81640625" style="57" customWidth="1"/>
-    <col min="3" max="3" width="17.81640625" style="57" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" style="57" customWidth="1"/>
-    <col min="5" max="5" width="15.6328125" style="57" customWidth="1"/>
-    <col min="6" max="16384" width="8.81640625" style="57"/>
+    <col min="1" max="1" customWidth="true" style="57" width="15.08984375"/>
+    <col min="2" max="2" customWidth="true" style="57" width="15.81640625"/>
+    <col min="3" max="3" customWidth="true" style="57" width="17.81640625"/>
+    <col min="4" max="4" customWidth="true" style="57" width="16.81640625"/>
+    <col min="5" max="5" customWidth="true" style="57" width="15.6328125"/>
+    <col min="6" max="16384" style="57" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -3512,20 +3549,20 @@
   <dimension ref="A1:AB6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="51.81640625" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="51.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.453125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -3643,16 +3680,16 @@
         <v>13</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>407</v>
+        <v>474</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>408</v>
+        <v>475</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>19</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>409</v>
+        <v>476</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>13</v>
@@ -3661,13 +3698,13 @@
         <v>14</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>410</v>
+        <v>477</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>100</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>411</v>
+        <v>478</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>14</v>
@@ -3944,10 +3981,10 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="76.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="76.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4027,12 +4064,12 @@
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="18.453125" style="57" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" style="57" customWidth="1"/>
-    <col min="3" max="3" width="14.81640625" style="57" customWidth="1"/>
-    <col min="4" max="4" width="11.81640625" style="57" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.1796875" style="57" customWidth="1"/>
-    <col min="6" max="16384" width="8.81640625" style="57"/>
+    <col min="1" max="1" customWidth="true" style="57" width="18.453125"/>
+    <col min="2" max="2" customWidth="true" style="57" width="12.54296875"/>
+    <col min="3" max="3" customWidth="true" style="57" width="14.81640625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="57" width="11.81640625"/>
+    <col min="5" max="5" customWidth="true" style="57" width="18.1796875"/>
+    <col min="6" max="16384" style="57" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4224,8 +4261,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.54296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -4262,11 +4299,11 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4415,30 +4452,30 @@
   <dimension ref="A1:AG4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="49.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="49.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="4.81640625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="5.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -4747,7 +4784,7 @@
   <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30">
@@ -5307,11 +5344,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="35.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.54296875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5392,8 +5429,8 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -5446,8 +5483,8 @@
   <dimension ref="A1:AC4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="5" max="5" width="6.1796875" customWidth="1"/>
-    <col min="29" max="29" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" customWidth="true" width="6.1796875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="13.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -5737,14 +5774,14 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="63.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="63.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="10.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="19.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="15.54296875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="8" max="9" bestFit="true" customWidth="true" width="19.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -5877,23 +5914,23 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="7.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="11.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -6471,8 +6508,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -6570,9 +6607,9 @@
   <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="24.90625" style="57" customWidth="1"/>
-    <col min="2" max="2" width="17.453125" style="57" customWidth="1"/>
-    <col min="3" max="16384" width="8.81640625" style="57"/>
+    <col min="1" max="1" customWidth="true" style="57" width="24.90625"/>
+    <col min="2" max="2" customWidth="true" style="57" width="17.453125"/>
+    <col min="3" max="16384" style="57" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -6781,14 +6818,14 @@
   <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="21.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="6.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="18.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -6888,15 +6925,15 @@
   <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" customWidth="1"/>
-    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="4" max="4" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -7052,16 +7089,16 @@
   <dimension ref="A1:K4"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="17.90625" style="57" customWidth="1"/>
-    <col min="2" max="2" width="11.81640625" style="57" customWidth="1"/>
-    <col min="3" max="3" width="13" style="57" customWidth="1"/>
-    <col min="4" max="4" width="16.54296875" style="57" customWidth="1"/>
-    <col min="5" max="5" width="15.81640625" style="57" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" style="57"/>
-    <col min="7" max="7" width="17.81640625" style="57" customWidth="1"/>
-    <col min="8" max="8" width="15.453125" style="57" customWidth="1"/>
-    <col min="9" max="9" width="11.54296875" style="57" customWidth="1"/>
-    <col min="10" max="16384" width="8.81640625" style="57"/>
+    <col min="1" max="1" customWidth="true" style="57" width="17.90625"/>
+    <col min="2" max="2" customWidth="true" style="57" width="11.81640625"/>
+    <col min="3" max="3" customWidth="true" style="57" width="13.0"/>
+    <col min="4" max="4" customWidth="true" style="57" width="16.54296875"/>
+    <col min="5" max="5" customWidth="true" style="57" width="15.81640625"/>
+    <col min="6" max="6" style="57" width="8.81640625"/>
+    <col min="7" max="7" customWidth="true" style="57" width="17.81640625"/>
+    <col min="8" max="8" customWidth="true" style="57" width="15.453125"/>
+    <col min="9" max="9" customWidth="true" style="57" width="11.54296875"/>
+    <col min="10" max="16384" style="57" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -7197,11 +7234,11 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -7269,10 +7306,10 @@
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="57.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="57.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="15.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="4" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -7389,22 +7426,22 @@
   <dimension ref="A1:P5"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="42" style="45" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.36328125" style="45" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.08984375" style="45" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.36328125" style="45" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" style="45" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" style="45" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="8.81640625" style="45"/>
-    <col min="9" max="9" width="10.453125" style="45" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.1796875" style="45" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" style="45" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1796875" style="45" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.453125" style="45" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.1796875" style="45" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13" style="45" customWidth="1"/>
-    <col min="16" max="16" width="10.1796875" style="45" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.81640625" style="45"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="45" width="42.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="45" width="18.36328125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="45" width="12.08984375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="45" width="15.36328125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="45" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="45" width="9.453125"/>
+    <col min="7" max="8" style="45" width="8.81640625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="45" width="10.453125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="45" width="11.1796875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="45" width="10.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="45" width="11.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="45" width="10.453125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="45" width="8.1796875"/>
+    <col min="15" max="15" customWidth="true" style="45" width="13.0"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="45" width="10.1796875"/>
+    <col min="17" max="16384" style="45" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -7598,29 +7635,29 @@
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="44.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="44.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.81640625"/>
+    <col min="11" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.1796875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="27" max="28" bestFit="true" customWidth="true" width="12.81640625"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="12.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -7987,9 +8024,9 @@
   <dimension ref="A1:W17"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="54.36328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="54.36328125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="13.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -8740,16 +8777,16 @@
   <dimension ref="A1:S20"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="53.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="12.1796875" customWidth="1"/>
-    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="53.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="5" max="7" customWidth="true" width="12.1796875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">

</xml_diff>

<commit_message>
Modified ManageSessions and ModifyTicketingService
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC2E262A-8EA1-4844-A249-6BB1BE3E2E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BF7513F-D4E8-44F3-A783-34C83AC232C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="7" activeTab="9" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="8" activeTab="10" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2084" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2078" uniqueCount="626">
   <si>
     <t>Scenario</t>
   </si>
@@ -1108,9 +1108,6 @@
     <t>354</t>
   </si>
   <si>
-    <t>441</t>
-  </si>
-  <si>
     <t>SJO</t>
   </si>
   <si>
@@ -1444,12 +1441,6 @@
     <t>A0HHSI</t>
   </si>
   <si>
-    <t>2023-08-20T04:51:00</t>
-  </si>
-  <si>
-    <t>2023-08-20T08:23:00</t>
-  </si>
-  <si>
     <t>2023-08-18T04:51:00</t>
   </si>
   <si>
@@ -1477,18 +1468,6 @@
     <t>122</t>
   </si>
   <si>
-    <t>A0JOAN</t>
-  </si>
-  <si>
-    <t>2302182801309</t>
-  </si>
-  <si>
-    <t>2302182801310</t>
-  </si>
-  <si>
-    <t>380</t>
-  </si>
-  <si>
     <t>473</t>
   </si>
   <si>
@@ -1783,36 +1762,6 @@
     <t>2302182807136</t>
   </si>
   <si>
-    <t>A2MQ50</t>
-  </si>
-  <si>
-    <t>2023-08-23T16:54:00</t>
-  </si>
-  <si>
-    <t>2023-08-23T20:23:00</t>
-  </si>
-  <si>
-    <t>2302182807137</t>
-  </si>
-  <si>
-    <t>A2MRAH</t>
-  </si>
-  <si>
-    <t>2302182807138</t>
-  </si>
-  <si>
-    <t>A2MRAX</t>
-  </si>
-  <si>
-    <t>2302182807139</t>
-  </si>
-  <si>
-    <t>A2MRA2</t>
-  </si>
-  <si>
-    <t>2302182807140</t>
-  </si>
-  <si>
     <t>A2MRBG</t>
   </si>
   <si>
@@ -1867,18 +1816,6 @@
     <t>A2MRG5</t>
   </si>
   <si>
-    <t>A2PNFL</t>
-  </si>
-  <si>
-    <t>AA2DB342CMCMRPCT052F39DE70</t>
-  </si>
-  <si>
-    <t>A1929E18CMCMRPCT06DFA232A0</t>
-  </si>
-  <si>
-    <t>7914A342CMCMRPCT05FAA95C7E</t>
-  </si>
-  <si>
     <t>A3RAZZ</t>
   </si>
   <si>
@@ -1951,12 +1888,6 @@
     <t>2302182816201</t>
   </si>
   <si>
-    <t>A4CGEE</t>
-  </si>
-  <si>
-    <t>2302182816228</t>
-  </si>
-  <si>
     <t>6759649826438453</t>
   </si>
   <si>
@@ -1964,13 +1895,69 @@
   </si>
   <si>
     <t>2302182816322</t>
+  </si>
+  <si>
+    <t>A340FE</t>
+  </si>
+  <si>
+    <t>2023-08-26T07:56:00</t>
+  </si>
+  <si>
+    <t>2023-08-26T12:05:00</t>
+  </si>
+  <si>
+    <t>2302182816168</t>
+  </si>
+  <si>
+    <t>A4FFSD</t>
+  </si>
+  <si>
+    <t>2302182816568</t>
+  </si>
+  <si>
+    <t>2302182816569</t>
+  </si>
+  <si>
+    <t>A340F1</t>
+  </si>
+  <si>
+    <t>2302182816169</t>
+  </si>
+  <si>
+    <t>A340GR</t>
+  </si>
+  <si>
+    <t>2302182816170</t>
+  </si>
+  <si>
+    <t>A340G0</t>
+  </si>
+  <si>
+    <t>2302182816171</t>
+  </si>
+  <si>
+    <t>485</t>
+  </si>
+  <si>
+    <t>173</t>
+  </si>
+  <si>
+    <t>A4IDBW</t>
+  </si>
+  <si>
+    <t>7744BA30CMCMRPCT055143D316</t>
+  </si>
+  <si>
+    <t>039672F2CMCMRPCT064917885D</t>
+  </si>
+  <si>
+    <t>73ADEAF0CMCMRPCT0853AFE719</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="13">
     <font>
       <sz val="11"/>
@@ -2200,7 +2187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2300,6 +2287,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2620,20 +2608,20 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="52.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.1796875"/>
+    <col min="1" max="1" width="52.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -2706,7 +2694,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="44" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="I2" s="32" t="s">
         <v>211</v>
@@ -2723,7 +2711,7 @@
       <c r="M2" s="32"/>
       <c r="N2" s="32"/>
       <c r="O2" s="32" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="P2" s="38"/>
     </row>
@@ -2774,7 +2762,7 @@
     </row>
     <row r="4" spans="1:16">
       <c r="A4" s="37" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B4" s="44">
         <v>0</v>
@@ -2795,13 +2783,13 @@
         <v>1</v>
       </c>
       <c r="H4" s="37" t="s">
-        <v>522</v>
+        <v>515</v>
       </c>
       <c r="I4" s="37" t="s">
+        <v>351</v>
+      </c>
+      <c r="J4" s="37" t="s">
         <v>352</v>
-      </c>
-      <c r="J4" s="37" t="s">
-        <v>353</v>
       </c>
       <c r="K4" s="32"/>
       <c r="L4" s="32"/>
@@ -2811,7 +2799,7 @@
     </row>
     <row r="5" spans="1:16">
       <c r="A5" s="37" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B5" s="44">
         <v>0</v>
@@ -2832,7 +2820,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>523</v>
+        <v>516</v>
       </c>
       <c r="I5" s="32"/>
       <c r="J5" s="32"/>
@@ -2868,13 +2856,13 @@
   <dimension ref="A1:U22"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="49.0"/>
-    <col min="10" max="10" style="25" width="8.81640625"/>
-    <col min="12" max="12" customWidth="true" width="15.90625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="12.6328125"/>
+    <col min="1" max="1" width="49" customWidth="1"/>
+    <col min="10" max="10" width="8.81640625" style="25"/>
+    <col min="12" max="12" width="15.90625" customWidth="1"/>
+    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -2972,7 +2960,7 @@
       </c>
       <c r="J2" s="44"/>
       <c r="K2" s="44" t="s">
-        <v>601</v>
+        <v>580</v>
       </c>
       <c r="L2" s="44"/>
       <c r="M2" s="44"/>
@@ -3009,10 +2997,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>616</v>
+        <v>595</v>
       </c>
       <c r="L3" s="44" t="s">
-        <v>617</v>
+        <v>596</v>
       </c>
       <c r="M3" s="44"/>
       <c r="N3" s="44"/>
@@ -3081,10 +3069,10 @@
       <c r="I5" s="44"/>
       <c r="J5" s="44"/>
       <c r="K5" s="44" t="s">
-        <v>602</v>
+        <v>581</v>
       </c>
       <c r="L5" s="44" t="s">
-        <v>603</v>
+        <v>582</v>
       </c>
       <c r="M5" s="44"/>
       <c r="N5" s="44" t="s">
@@ -3128,7 +3116,7 @@
       <c r="I6" s="44"/>
       <c r="J6" s="44"/>
       <c r="K6" s="44" t="s">
-        <v>604</v>
+        <v>583</v>
       </c>
       <c r="L6" s="44"/>
       <c r="M6" s="44"/>
@@ -3139,7 +3127,7 @@
         <v>242</v>
       </c>
       <c r="P6" s="44" t="s">
-        <v>605</v>
+        <v>584</v>
       </c>
       <c r="Q6" s="44"/>
       <c r="R6" s="44"/>
@@ -3173,10 +3161,10 @@
       <c r="I7" s="44"/>
       <c r="J7" s="44"/>
       <c r="K7" s="44" t="s">
-        <v>606</v>
+        <v>585</v>
       </c>
       <c r="L7" s="44" t="s">
-        <v>607</v>
+        <v>586</v>
       </c>
       <c r="M7" s="44"/>
       <c r="N7" s="44" t="s">
@@ -3186,13 +3174,13 @@
         <v>242</v>
       </c>
       <c r="P7" s="44" t="s">
-        <v>620</v>
+        <v>599</v>
       </c>
       <c r="Q7" s="47" t="s">
         <v>87</v>
       </c>
       <c r="R7" s="44" t="s">
-        <v>621</v>
+        <v>600</v>
       </c>
       <c r="S7" s="44"/>
       <c r="T7" s="44"/>
@@ -3228,10 +3216,10 @@
       </c>
       <c r="J8" s="44"/>
       <c r="K8" s="44" t="s">
-        <v>618</v>
+        <v>597</v>
       </c>
       <c r="L8" s="44" t="s">
-        <v>619</v>
+        <v>598</v>
       </c>
       <c r="M8" s="44"/>
       <c r="N8" s="44" t="s">
@@ -3269,7 +3257,7 @@
       <c r="I9" s="44"/>
       <c r="J9" s="44"/>
       <c r="K9" s="44" t="s">
-        <v>622</v>
+        <v>601</v>
       </c>
       <c r="L9" s="44"/>
       <c r="M9" s="44"/>
@@ -3308,10 +3296,10 @@
       <c r="I10" s="44"/>
       <c r="J10" s="44"/>
       <c r="K10" s="44" t="s">
-        <v>628</v>
+        <v>605</v>
       </c>
       <c r="L10" s="44" t="s">
-        <v>629</v>
+        <v>606</v>
       </c>
       <c r="M10" s="44"/>
       <c r="N10" s="44"/>
@@ -3320,7 +3308,7 @@
       <c r="Q10" s="44"/>
       <c r="R10" s="44"/>
       <c r="S10" s="47" t="s">
-        <v>627</v>
+        <v>604</v>
       </c>
       <c r="T10" s="44"/>
       <c r="U10" s="44"/>
@@ -3347,10 +3335,10 @@
       <c r="I11" s="44"/>
       <c r="J11" s="44"/>
       <c r="K11" s="44" t="s">
-        <v>608</v>
+        <v>587</v>
       </c>
       <c r="L11" s="44" t="s">
-        <v>609</v>
+        <v>588</v>
       </c>
       <c r="M11" s="44"/>
       <c r="N11" s="44"/>
@@ -3386,10 +3374,10 @@
       <c r="I12" s="44"/>
       <c r="J12" s="44"/>
       <c r="K12" s="44" t="s">
-        <v>623</v>
+        <v>602</v>
       </c>
       <c r="L12" s="44" t="s">
-        <v>624</v>
+        <v>603</v>
       </c>
       <c r="M12" s="44"/>
       <c r="N12" s="44" t="s">
@@ -3429,10 +3417,10 @@
       <c r="I13" s="44"/>
       <c r="J13" s="44"/>
       <c r="K13" s="44" t="s">
+        <v>449</v>
+      </c>
+      <c r="L13" s="44" t="s">
         <v>450</v>
-      </c>
-      <c r="L13" s="44" t="s">
-        <v>451</v>
       </c>
       <c r="M13" s="44"/>
       <c r="N13" s="44" t="s">
@@ -3507,10 +3495,10 @@
       <c r="I15" s="44"/>
       <c r="J15" s="44"/>
       <c r="K15" s="44" t="s">
-        <v>610</v>
+        <v>589</v>
       </c>
       <c r="L15" s="44" t="s">
-        <v>611</v>
+        <v>590</v>
       </c>
       <c r="M15" s="44"/>
       <c r="N15" s="44" t="s">
@@ -3536,7 +3524,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="47" t="s">
-        <v>612</v>
+        <v>591</v>
       </c>
       <c r="D16" s="44" t="s">
         <v>12</v>
@@ -3550,7 +3538,7 @@
       <c r="I16" s="44"/>
       <c r="J16" s="44"/>
       <c r="K16" s="44" t="s">
-        <v>613</v>
+        <v>592</v>
       </c>
       <c r="L16" s="44"/>
       <c r="M16" s="44"/>
@@ -3589,7 +3577,7 @@
       <c r="I17" s="44"/>
       <c r="J17" s="44"/>
       <c r="K17" s="44" t="s">
-        <v>614</v>
+        <v>593</v>
       </c>
       <c r="L17" s="44"/>
       <c r="M17" s="44"/>
@@ -3632,7 +3620,7 @@
       </c>
       <c r="J18" s="44"/>
       <c r="K18" s="44" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="L18" s="44"/>
       <c r="M18" s="44"/>
@@ -3671,7 +3659,7 @@
       <c r="I19" s="44"/>
       <c r="J19" s="44"/>
       <c r="K19" s="44" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="L19" s="44"/>
       <c r="M19" s="44"/>
@@ -3710,7 +3698,7 @@
       <c r="I20" s="44"/>
       <c r="J20" s="44"/>
       <c r="K20" s="44" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="L20" s="44"/>
       <c r="M20" s="44"/>
@@ -3749,7 +3737,7 @@
       <c r="I21" s="44"/>
       <c r="J21" s="44"/>
       <c r="K21" s="44" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="L21" s="44"/>
       <c r="M21" s="44"/>
@@ -3774,7 +3762,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="47" t="s">
-        <v>471</v>
+        <v>464</v>
       </c>
       <c r="D22" s="44" t="s">
         <v>34</v>
@@ -3796,7 +3784,7 @@
       </c>
       <c r="J22" s="44"/>
       <c r="K22" s="44" t="s">
-        <v>615</v>
+        <v>594</v>
       </c>
       <c r="L22" s="44"/>
       <c r="M22" s="44"/>
@@ -3823,192 +3811,164 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" customWidth="true" style="29" width="17.54296875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="5" max="5" customWidth="true" width="13.81640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="14.36328125"/>
-    <col min="7" max="11" customWidth="true" style="29" width="14.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="30.36328125"/>
-    <col min="13" max="13" customWidth="true" width="8.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="10.90625"/>
+    <col min="1" max="1" width="32.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" style="29" customWidth="1"/>
+    <col min="4" max="4" width="29.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.81640625" customWidth="1"/>
+    <col min="6" max="6" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="11" width="14.36328125" style="29" customWidth="1"/>
+    <col min="12" max="12" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
-      <c r="A1" s="33" t="s">
+    <row r="1" spans="1:13">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="30" t="s">
+      <c r="B1" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="42" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1" s="43" t="s">
+        <v>260</v>
+      </c>
+      <c r="E1" s="43" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" s="42" t="s">
+        <v>261</v>
+      </c>
+      <c r="G1" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="H1" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="30" t="s">
+      <c r="I1" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="G1" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="30" t="s">
+      <c r="J1" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="30" t="s">
+      <c r="K1" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="30" t="s">
+      <c r="L1" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="L1" s="31" t="s">
-        <v>260</v>
-      </c>
-      <c r="M1" s="31" t="s">
-        <v>74</v>
-      </c>
-      <c r="N1" s="30" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2" s="35" t="s">
+      <c r="M1" s="42" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="44" t="s">
         <v>262</v>
       </c>
-      <c r="B2" s="32">
+      <c r="B2" s="44">
+        <v>2</v>
+      </c>
+      <c r="C2" s="44">
+        <v>2</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>623</v>
+      </c>
+      <c r="E2" s="47" t="s">
+        <v>622</v>
+      </c>
+      <c r="F2" s="44"/>
+      <c r="G2" s="47" t="s">
+        <v>620</v>
+      </c>
+      <c r="H2" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="44" t="s">
+        <v>263</v>
+      </c>
+      <c r="B3" s="44">
+        <v>2</v>
+      </c>
+      <c r="C3" s="44">
+        <v>2</v>
+      </c>
+      <c r="D3" s="47" t="s">
+        <v>624</v>
+      </c>
+      <c r="E3" s="47" t="s">
+        <v>264</v>
+      </c>
+      <c r="F3" s="44" t="s">
+        <v>149</v>
+      </c>
+      <c r="G3" s="47" t="s">
+        <v>620</v>
+      </c>
+      <c r="H3" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44">
         <v>0</v>
       </c>
-      <c r="C2" s="47" t="s">
-        <v>470</v>
-      </c>
-      <c r="D2" s="35" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="32" t="s">
-        <v>209</v>
-      </c>
-      <c r="F2" s="32">
-        <v>0</v>
-      </c>
-      <c r="G2" s="32">
-        <v>1</v>
-      </c>
-      <c r="H2" s="47" t="s">
-        <v>325</v>
-      </c>
-      <c r="I2" s="32" t="s">
-        <v>209</v>
-      </c>
-      <c r="J2" s="35" t="s">
-        <v>12</v>
-      </c>
-      <c r="K2" s="32">
-        <v>1</v>
-      </c>
-      <c r="L2" s="34" t="s">
-        <v>598</v>
-      </c>
-      <c r="M2" s="34" t="s">
-        <v>597</v>
-      </c>
-      <c r="N2" s="32"/>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="A3" s="32" t="s">
-        <v>263</v>
-      </c>
-      <c r="B3" s="32">
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="44" t="s">
+        <v>265</v>
+      </c>
+      <c r="B4" s="44">
         <v>2</v>
       </c>
-      <c r="C3" s="34" t="s">
-        <v>344</v>
-      </c>
-      <c r="D3" s="35" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="32" t="s">
+      <c r="C4" s="44">
+        <v>2</v>
+      </c>
+      <c r="D4" s="47" t="s">
+        <v>625</v>
+      </c>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44" t="s">
+        <v>149</v>
+      </c>
+      <c r="G4" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="32">
-        <v>2</v>
-      </c>
-      <c r="G3" s="32">
-        <v>6</v>
-      </c>
-      <c r="H3" s="34" t="s">
-        <v>194</v>
-      </c>
-      <c r="I3" s="32" t="s">
+      <c r="J4" s="47" t="s">
+        <v>621</v>
+      </c>
+      <c r="K4" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="35" t="s">
-        <v>12</v>
-      </c>
-      <c r="K3" s="32">
-        <v>6</v>
-      </c>
-      <c r="L3" s="34" t="s">
-        <v>599</v>
-      </c>
-      <c r="M3" s="34" t="s">
-        <v>264</v>
-      </c>
-      <c r="N3" s="32" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4" s="32" t="s">
-        <v>265</v>
-      </c>
-      <c r="B4" s="32">
-        <v>2</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>344</v>
-      </c>
-      <c r="D4" s="35" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="32">
-        <v>2</v>
-      </c>
-      <c r="G4" s="32">
-        <v>6</v>
-      </c>
-      <c r="H4" s="34" t="s">
-        <v>194</v>
-      </c>
-      <c r="I4" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="J4" s="35" t="s">
-        <v>12</v>
-      </c>
-      <c r="K4" s="32">
-        <v>6</v>
-      </c>
-      <c r="L4" s="34" t="s">
-        <v>600</v>
-      </c>
-      <c r="M4" s="32"/>
-      <c r="N4" s="32" t="s">
-        <v>149</v>
-      </c>
+      <c r="L4" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="M4" s="44"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4023,17 +3983,17 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="29" width="21.81640625"/>
-    <col min="2" max="2" customWidth="true" style="29" width="16.54296875"/>
-    <col min="3" max="3" customWidth="true" style="29" width="19.90625"/>
-    <col min="4" max="4" customWidth="true" style="29" width="18.81640625"/>
-    <col min="5" max="6" customWidth="true" style="29" width="12.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="11.90625"/>
-    <col min="9" max="9" style="29" width="8.81640625"/>
-    <col min="10" max="10" customWidth="true" style="29" width="17.90625"/>
-    <col min="11" max="11" customWidth="true" style="29" width="14.1796875"/>
-    <col min="12" max="16384" style="29" width="8.81640625"/>
+    <col min="1" max="1" width="21.81640625" style="29" customWidth="1"/>
+    <col min="2" max="2" width="16.54296875" style="29" customWidth="1"/>
+    <col min="3" max="3" width="19.90625" style="29" customWidth="1"/>
+    <col min="4" max="4" width="18.81640625" style="29" customWidth="1"/>
+    <col min="5" max="6" width="12.90625" style="29" customWidth="1"/>
+    <col min="7" max="7" width="15" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.81640625" style="29"/>
+    <col min="10" max="10" width="17.90625" style="29" customWidth="1"/>
+    <col min="11" max="11" width="14.1796875" style="29" customWidth="1"/>
+    <col min="12" max="16384" width="8.81640625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -4085,7 +4045,7 @@
       <c r="G2" s="44"/>
       <c r="H2" s="44"/>
       <c r="I2" s="44" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
       <c r="J2" s="44"/>
       <c r="K2" s="44"/>
@@ -4104,7 +4064,7 @@
       <c r="G3" s="44"/>
       <c r="H3" s="44"/>
       <c r="I3" s="44" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
       <c r="J3" s="44"/>
       <c r="K3" s="44"/>
@@ -4123,7 +4083,7 @@
       <c r="G4" s="44"/>
       <c r="H4" s="44"/>
       <c r="I4" s="44" t="s">
-        <v>515</v>
+        <v>508</v>
       </c>
       <c r="J4" s="44"/>
       <c r="K4" s="44"/>
@@ -4154,13 +4114,13 @@
         <v>12</v>
       </c>
       <c r="I5" s="44" t="s">
-        <v>544</v>
+        <v>537</v>
       </c>
       <c r="J5" s="44" t="s">
-        <v>545</v>
+        <v>538</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>546</v>
+        <v>539</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4189,10 +4149,10 @@
         <v>12</v>
       </c>
       <c r="I6" s="44" t="s">
-        <v>547</v>
+        <v>540</v>
       </c>
       <c r="J6" s="44" t="s">
-        <v>548</v>
+        <v>541</v>
       </c>
       <c r="K6" s="44"/>
     </row>
@@ -4209,12 +4169,12 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="29" width="42.1796875"/>
-    <col min="2" max="2" customWidth="true" style="29" width="15.81640625"/>
-    <col min="3" max="3" customWidth="true" style="29" width="17.81640625"/>
-    <col min="4" max="4" customWidth="true" style="29" width="16.81640625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.6328125"/>
-    <col min="6" max="16384" style="29" width="8.81640625"/>
+    <col min="1" max="1" width="42.1796875" style="29" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" style="29" customWidth="1"/>
+    <col min="3" max="3" width="17.81640625" style="29" customWidth="1"/>
+    <col min="4" max="4" width="16.81640625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.6328125" style="29" customWidth="1"/>
+    <col min="6" max="16384" width="8.81640625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4260,7 +4220,7 @@
         <v>149</v>
       </c>
       <c r="D3" s="44" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E3" s="44">
         <v>1</v>
@@ -4277,7 +4237,7 @@
         <v>149</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E4" s="44">
         <v>1</v>
@@ -4285,7 +4245,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="37" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B5" s="37"/>
       <c r="C5" s="37" t="s">
@@ -4296,7 +4256,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="37" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B6" s="37"/>
       <c r="C6" s="37" t="s">
@@ -4309,7 +4269,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="37" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B7" s="37"/>
       <c r="C7" s="37" t="s">
@@ -4333,28 +4293,28 @@
   <dimension ref="A1:AB6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="51.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="14.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="51.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -4472,16 +4432,16 @@
         <v>45</v>
       </c>
       <c r="J2" s="44" t="s">
-        <v>589</v>
+        <v>572</v>
       </c>
       <c r="K2" s="44" t="s">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="L2" s="44" t="s">
         <v>207</v>
       </c>
       <c r="M2" s="44" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="N2" s="44" t="s">
         <v>208</v>
@@ -4490,13 +4450,13 @@
         <v>12</v>
       </c>
       <c r="P2" s="44" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="Q2" s="44" t="s">
         <v>62</v>
       </c>
       <c r="R2" s="44" t="s">
-        <v>519</v>
+        <v>512</v>
       </c>
       <c r="S2" s="44" t="s">
         <v>12</v>
@@ -4542,16 +4502,16 @@
         <v>45</v>
       </c>
       <c r="J3" s="44" t="s">
-        <v>549</v>
+        <v>542</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="L3" s="44" t="s">
         <v>207</v>
       </c>
       <c r="M3" s="44" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="N3" s="44" t="s">
         <v>208</v>
@@ -4560,13 +4520,13 @@
         <v>12</v>
       </c>
       <c r="P3" s="44" t="s">
-        <v>550</v>
+        <v>543</v>
       </c>
       <c r="Q3" s="44" t="s">
         <v>239</v>
       </c>
       <c r="R3" s="44" t="s">
-        <v>551</v>
+        <v>544</v>
       </c>
       <c r="S3" s="44" t="s">
         <v>12</v>
@@ -4620,16 +4580,16 @@
       <c r="H4" s="44"/>
       <c r="I4" s="44"/>
       <c r="J4" s="44" t="s">
-        <v>555</v>
+        <v>548</v>
       </c>
       <c r="K4" s="44" t="s">
-        <v>556</v>
+        <v>549</v>
       </c>
       <c r="L4" s="44" t="s">
         <v>328</v>
       </c>
       <c r="M4" s="44" t="s">
-        <v>557</v>
+        <v>550</v>
       </c>
       <c r="N4" s="44" t="s">
         <v>209</v>
@@ -4672,16 +4632,16 @@
       <c r="H5" s="44"/>
       <c r="I5" s="44"/>
       <c r="J5" s="44" t="s">
-        <v>558</v>
+        <v>551</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>556</v>
+        <v>549</v>
       </c>
       <c r="L5" s="44" t="s">
         <v>328</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>557</v>
+        <v>550</v>
       </c>
       <c r="N5" s="44" t="s">
         <v>209</v>
@@ -4732,16 +4692,16 @@
         <v>45</v>
       </c>
       <c r="J6" s="44" t="s">
-        <v>552</v>
+        <v>545</v>
       </c>
       <c r="K6" s="44" t="s">
-        <v>553</v>
+        <v>546</v>
       </c>
       <c r="L6" s="44" t="s">
         <v>207</v>
       </c>
       <c r="M6" s="44" t="s">
-        <v>554</v>
+        <v>547</v>
       </c>
       <c r="N6" s="44" t="s">
         <v>208</v>
@@ -4777,10 +4737,10 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="76.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="76.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4865,12 +4825,12 @@
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="68.08984375"/>
-    <col min="2" max="2" customWidth="true" style="29" width="12.54296875"/>
-    <col min="3" max="3" customWidth="true" style="29" width="14.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="11.81640625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="18.1796875"/>
-    <col min="6" max="16384" style="29" width="8.81640625"/>
+    <col min="1" max="1" width="68.08984375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" style="29" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" style="29" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" style="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.1796875" style="29" customWidth="1"/>
+    <col min="6" max="16384" width="8.81640625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5006,7 +4966,7 @@
         <v>282</v>
       </c>
       <c r="D9" s="44" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E9" s="44"/>
     </row>
@@ -5117,8 +5077,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.54296875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -5158,11 +5118,11 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5212,7 +5172,7 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="21.81640625"/>
+    <col min="1" max="1" width="21.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -5317,31 +5277,31 @@
   <dimension ref="A1:AG4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="49.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="4.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="9.7265625"/>
+    <col min="1" max="1" width="49.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -5525,7 +5485,7 @@
         <v>0</v>
       </c>
       <c r="AA2" s="44" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="AB2" s="44" t="s">
         <v>45</v>
@@ -5537,7 +5497,7 @@
         <v>0</v>
       </c>
       <c r="AE2" s="44" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="AF2" s="44" t="s">
         <v>45</v>
@@ -5646,25 +5606,25 @@
   <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="33.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.36328125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.36328125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="14.36328125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="1" max="1" width="33" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30">
@@ -5783,16 +5743,16 @@
       <c r="I2" s="44"/>
       <c r="J2" s="44"/>
       <c r="K2" s="44" t="s">
-        <v>559</v>
+        <v>552</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>560</v>
+        <v>553</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>325</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>561</v>
+        <v>554</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>209</v>
@@ -5847,7 +5807,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>562</v>
+        <v>555</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>312</v>
@@ -5987,16 +5947,16 @@
         <v>2</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>563</v>
+        <v>556</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>560</v>
+        <v>553</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>325</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>561</v>
+        <v>554</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>209</v>
@@ -6005,7 +5965,7 @@
         <v>12</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>564</v>
+        <v>557</v>
       </c>
       <c r="R5" s="15" t="s">
         <v>44</v>
@@ -6203,16 +6163,16 @@
       <c r="I9" s="44"/>
       <c r="J9" s="44"/>
       <c r="K9" s="44" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>325</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>209</v>
@@ -6248,11 +6208,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="35.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.54296875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="1" max="1" width="35.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -6277,10 +6237,10 @@
         <v>127</v>
       </c>
       <c r="B2" s="44" t="s">
+        <v>445</v>
+      </c>
+      <c r="C2" s="44" t="s">
         <v>446</v>
-      </c>
-      <c r="C2" s="44" t="s">
-        <v>447</v>
       </c>
       <c r="D2" s="44" t="s">
         <v>128</v>
@@ -6336,9 +6296,9 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.90625"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -6394,9 +6354,9 @@
   <dimension ref="A1:AC4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="46.6328125"/>
-    <col min="5" max="5" customWidth="true" width="6.1796875"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="1" max="1" width="46.6328125" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" customWidth="1"/>
+    <col min="29" max="29" width="13.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -6524,16 +6484,16 @@
       <c r="U2" s="44"/>
       <c r="V2" s="44"/>
       <c r="W2" s="44" t="s">
-        <v>565</v>
+        <v>558</v>
       </c>
       <c r="X2" s="44" t="s">
-        <v>560</v>
+        <v>553</v>
       </c>
       <c r="Y2" s="44" t="s">
         <v>325</v>
       </c>
       <c r="Z2" s="44" t="s">
-        <v>561</v>
+        <v>554</v>
       </c>
       <c r="AA2" s="44" t="s">
         <v>209</v>
@@ -6542,7 +6502,7 @@
         <v>12</v>
       </c>
       <c r="AC2" s="44" t="s">
-        <v>566</v>
+        <v>559</v>
       </c>
     </row>
     <row r="3" spans="1:29">
@@ -6660,16 +6620,16 @@
       <c r="U4" s="44"/>
       <c r="V4" s="44"/>
       <c r="W4" s="44" t="s">
-        <v>567</v>
+        <v>560</v>
       </c>
       <c r="X4" s="44" t="s">
-        <v>560</v>
+        <v>553</v>
       </c>
       <c r="Y4" s="44" t="s">
         <v>325</v>
       </c>
       <c r="Z4" s="44" t="s">
-        <v>561</v>
+        <v>554</v>
       </c>
       <c r="AA4" s="44" t="s">
         <v>209</v>
@@ -6678,7 +6638,7 @@
         <v>12</v>
       </c>
       <c r="AC4" s="44" t="s">
-        <v>568</v>
+        <v>561</v>
       </c>
     </row>
   </sheetData>
@@ -6694,14 +6654,14 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="63.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="10.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="19.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="15.54296875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="8" max="9" bestFit="true" customWidth="true" width="19.453125"/>
+    <col min="1" max="1" width="63.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="19.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -6836,67 +6796,67 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.81640625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="7.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="17" max="17" customWidth="true" width="17.6328125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.6328125" customWidth="1"/>
+    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="42" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="42" t="s">
+      <c r="B1" s="58" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="42" t="s">
+      <c r="D1" s="58" t="s">
         <v>72</v>
       </c>
-      <c r="E1" s="42" t="s">
+      <c r="E1" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="42" t="s">
+      <c r="F1" s="65" t="s">
         <v>142</v>
       </c>
-      <c r="G1" s="42" t="s">
+      <c r="G1" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="42" t="s">
+      <c r="H1" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="42" t="s">
+      <c r="I1" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="42" t="s">
-        <v>1</v>
-      </c>
-      <c r="K1" s="43" t="s">
+      <c r="J1" s="58" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="L1" s="43" t="s">
-        <v>1</v>
-      </c>
-      <c r="M1" s="43" t="s">
+      <c r="L1" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="43" t="s">
+      <c r="N1" s="19" t="s">
         <v>75</v>
       </c>
       <c r="O1" s="19" t="s">
@@ -6916,19 +6876,19 @@
       <c r="A2" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="B2" s="44">
-        <v>1</v>
-      </c>
-      <c r="C2" s="44" t="s">
-        <v>329</v>
+      <c r="B2" s="47">
+        <v>1</v>
+      </c>
+      <c r="C2" s="47" t="s">
+        <v>18</v>
       </c>
       <c r="D2" s="44" t="s">
-        <v>209</v>
+        <v>12</v>
       </c>
       <c r="E2" s="44" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="44">
+        <v>13</v>
+      </c>
+      <c r="F2" s="47">
         <v>0</v>
       </c>
       <c r="G2" s="44"/>
@@ -6936,139 +6896,147 @@
       <c r="I2" s="44"/>
       <c r="J2" s="44"/>
       <c r="K2" s="44" t="s">
-        <v>569</v>
+        <v>607</v>
       </c>
       <c r="L2" s="44" t="s">
-        <v>570</v>
+        <v>608</v>
       </c>
       <c r="M2" s="44" t="s">
-        <v>329</v>
+        <v>18</v>
       </c>
       <c r="N2" s="44" t="s">
-        <v>571</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>572</v>
-      </c>
-      <c r="R2" s="3"/>
+        <v>609</v>
+      </c>
+      <c r="O2" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="44" t="s">
+        <v>610</v>
+      </c>
+      <c r="R2" s="44"/>
     </row>
     <row r="3" spans="1:18">
       <c r="A3" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="B3" s="44">
-        <v>2</v>
-      </c>
-      <c r="C3" s="44" t="s">
-        <v>325</v>
+      <c r="B3" s="47">
+        <v>1</v>
+      </c>
+      <c r="C3" s="47" t="s">
+        <v>18</v>
       </c>
       <c r="D3" s="44" t="s">
-        <v>209</v>
+        <v>12</v>
       </c>
       <c r="E3" s="44" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="44">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="F3" s="47">
+        <v>0</v>
       </c>
       <c r="G3" s="44"/>
       <c r="H3" s="44"/>
       <c r="I3" s="44"/>
       <c r="J3" s="44"/>
       <c r="K3" s="44" t="s">
-        <v>467</v>
+        <v>611</v>
       </c>
       <c r="L3" s="44" t="s">
-        <v>456</v>
+        <v>608</v>
       </c>
       <c r="M3" s="44" t="s">
-        <v>325</v>
+        <v>18</v>
       </c>
       <c r="N3" s="44" t="s">
-        <v>457</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>468</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>469</v>
+        <v>609</v>
+      </c>
+      <c r="O3" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="P3" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q3" s="44" t="s">
+        <v>612</v>
+      </c>
+      <c r="R3" s="44" t="s">
+        <v>613</v>
       </c>
     </row>
     <row r="4" spans="1:18">
       <c r="A4" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="B4" s="44">
-        <v>1</v>
-      </c>
-      <c r="C4" s="44" t="s">
-        <v>207</v>
+      <c r="B4" s="47">
+        <v>1</v>
+      </c>
+      <c r="C4" s="47" t="s">
+        <v>18</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>208</v>
+        <v>12</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="44">
+        <v>13</v>
+      </c>
+      <c r="F4" s="47">
         <v>0</v>
       </c>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44"/>
-      <c r="I4" s="44"/>
-      <c r="J4" s="44"/>
+      <c r="G4" s="47" t="s">
+        <v>44</v>
+      </c>
+      <c r="H4" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="J4" s="44">
+        <v>2</v>
+      </c>
       <c r="K4" s="44" t="s">
-        <v>573</v>
+        <v>614</v>
       </c>
       <c r="L4" s="44" t="s">
-        <v>516</v>
+        <v>608</v>
       </c>
       <c r="M4" s="44" t="s">
-        <v>207</v>
+        <v>18</v>
       </c>
       <c r="N4" s="44" t="s">
-        <v>517</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q4" s="3" t="s">
-        <v>574</v>
-      </c>
-      <c r="R4" s="3"/>
+        <v>609</v>
+      </c>
+      <c r="O4" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="P4" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q4" s="44" t="s">
+        <v>615</v>
+      </c>
+      <c r="R4" s="44"/>
     </row>
     <row r="5" spans="1:18">
       <c r="A5" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="B5" s="44">
-        <v>1</v>
-      </c>
-      <c r="C5" s="44" t="s">
-        <v>207</v>
+      <c r="B5" s="47">
+        <v>1</v>
+      </c>
+      <c r="C5" s="47" t="s">
+        <v>18</v>
       </c>
       <c r="D5" s="44" t="s">
-        <v>208</v>
+        <v>12</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="44">
+        <v>13</v>
+      </c>
+      <c r="F5" s="47">
         <v>0</v>
       </c>
       <c r="G5" s="44"/>
@@ -7076,45 +7044,45 @@
       <c r="I5" s="44"/>
       <c r="J5" s="44"/>
       <c r="K5" s="44" t="s">
-        <v>575</v>
+        <v>616</v>
       </c>
       <c r="L5" s="44" t="s">
-        <v>516</v>
+        <v>608</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>207</v>
+        <v>18</v>
       </c>
       <c r="N5" s="44" t="s">
-        <v>517</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q5" s="3" t="s">
-        <v>576</v>
-      </c>
-      <c r="R5" s="3"/>
+        <v>609</v>
+      </c>
+      <c r="O5" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="P5" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q5" s="44" t="s">
+        <v>617</v>
+      </c>
+      <c r="R5" s="44"/>
     </row>
     <row r="6" spans="1:18">
       <c r="A6" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="B6" s="44">
-        <v>1</v>
-      </c>
-      <c r="C6" s="44" t="s">
-        <v>207</v>
+      <c r="B6" s="47">
+        <v>1</v>
+      </c>
+      <c r="C6" s="47" t="s">
+        <v>18</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>208</v>
+        <v>12</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="44">
+        <v>13</v>
+      </c>
+      <c r="F6" s="47">
         <v>0</v>
       </c>
       <c r="G6" s="44"/>
@@ -7122,27 +7090,27 @@
       <c r="I6" s="44"/>
       <c r="J6" s="44"/>
       <c r="K6" s="44" t="s">
-        <v>577</v>
+        <v>618</v>
       </c>
       <c r="L6" s="44" t="s">
-        <v>516</v>
+        <v>608</v>
       </c>
       <c r="M6" s="44" t="s">
-        <v>207</v>
+        <v>18</v>
       </c>
       <c r="N6" s="44" t="s">
-        <v>517</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="P6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q6" s="3" t="s">
-        <v>578</v>
-      </c>
-      <c r="R6" s="3"/>
+        <v>609</v>
+      </c>
+      <c r="O6" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="P6" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q6" s="44" t="s">
+        <v>619</v>
+      </c>
+      <c r="R6" s="44"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7158,27 +7126,27 @@
   <dimension ref="A1:U13"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="44.08984375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.1796875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.1796875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="8.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="14.08984375"/>
+    <col min="1" max="1" width="44.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -7275,16 +7243,16 @@
         <v>163</v>
       </c>
       <c r="J2" s="56" t="s">
-        <v>579</v>
+        <v>562</v>
       </c>
       <c r="K2" s="44" t="s">
-        <v>580</v>
+        <v>563</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>215</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>581</v>
+        <v>564</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>12</v>
@@ -7293,13 +7261,13 @@
         <v>216</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>582</v>
+        <v>565</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>217</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>583</v>
+        <v>566</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>216</v>
@@ -7308,7 +7276,7 @@
         <v>163</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>584</v>
+        <v>567</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -7340,16 +7308,16 @@
         <v>163</v>
       </c>
       <c r="J3" s="56" t="s">
-        <v>585</v>
+        <v>568</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>580</v>
+        <v>563</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>215</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>581</v>
+        <v>564</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>12</v>
@@ -7358,13 +7326,13 @@
         <v>216</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>586</v>
+        <v>569</v>
       </c>
       <c r="Q3" s="3" t="s">
         <v>341</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>587</v>
+        <v>570</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>216</v>
@@ -7373,7 +7341,7 @@
         <v>163</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>588</v>
+        <v>571</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -7553,8 +7521,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -7578,7 +7546,7 @@
         <v>181</v>
       </c>
       <c r="B3" s="64" t="s">
-        <v>513</v>
+        <v>506</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -7602,7 +7570,7 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="18.0"/>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -7663,21 +7631,21 @@
   <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="29" width="24.90625"/>
-    <col min="2" max="2" customWidth="true" style="29" width="14.0"/>
-    <col min="3" max="3" customWidth="true" style="29" width="11.81640625"/>
-    <col min="4" max="4" customWidth="true" style="29" width="9.54296875"/>
-    <col min="5" max="5" customWidth="true" style="29" width="10.36328125"/>
-    <col min="6" max="6" customWidth="true" style="29" width="9.36328125"/>
-    <col min="7" max="7" customWidth="true" style="29" width="9.7265625"/>
-    <col min="8" max="8" customWidth="true" style="29" width="10.453125"/>
-    <col min="9" max="9" customWidth="true" style="29" width="8.81640625"/>
-    <col min="10" max="10" customWidth="true" style="41" width="8.08984375"/>
-    <col min="11" max="11" customWidth="true" style="29" width="10.0"/>
-    <col min="12" max="12" customWidth="true" style="29" width="7.81640625"/>
-    <col min="13" max="13" customWidth="true" style="29" width="9.0"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="19.453125"/>
-    <col min="15" max="16384" style="29" width="8.81640625"/>
+    <col min="1" max="1" width="24.90625" style="29" customWidth="1"/>
+    <col min="2" max="2" width="14" style="29" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" style="29" customWidth="1"/>
+    <col min="4" max="4" width="9.54296875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10.36328125" style="29" customWidth="1"/>
+    <col min="6" max="6" width="9.36328125" style="29" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" style="29" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" style="29" customWidth="1"/>
+    <col min="9" max="9" width="8.81640625" style="29" customWidth="1"/>
+    <col min="10" max="10" width="8.08984375" style="41" customWidth="1"/>
+    <col min="11" max="11" width="10" style="29" customWidth="1"/>
+    <col min="12" max="12" width="7.81640625" style="29" customWidth="1"/>
+    <col min="13" max="13" width="9" style="29" customWidth="1"/>
+    <col min="14" max="14" width="19.453125" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.81640625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -7688,40 +7656,40 @@
         <v>266</v>
       </c>
       <c r="C1" s="42" t="s">
-        <v>475</v>
+        <v>468</v>
       </c>
       <c r="D1" s="42" t="s">
-        <v>476</v>
+        <v>469</v>
       </c>
       <c r="E1" s="42" t="s">
-        <v>477</v>
+        <v>470</v>
       </c>
       <c r="F1" s="42" t="s">
-        <v>478</v>
+        <v>471</v>
       </c>
       <c r="G1" s="63" t="s">
-        <v>479</v>
+        <v>472</v>
       </c>
       <c r="H1" s="63" t="s">
-        <v>480</v>
+        <v>473</v>
       </c>
       <c r="I1" s="63" t="s">
-        <v>480</v>
+        <v>473</v>
       </c>
       <c r="J1" s="63" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
       <c r="K1" s="42" t="s">
-        <v>477</v>
+        <v>470</v>
       </c>
       <c r="L1" s="42" t="s">
-        <v>478</v>
+        <v>471</v>
       </c>
       <c r="M1" s="42" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="N1" s="42" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -7732,40 +7700,40 @@
         <v>149</v>
       </c>
       <c r="C2" s="32" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="D2" s="32" t="s">
         <v>121</v>
       </c>
       <c r="E2" s="32" t="s">
-        <v>482</v>
+        <v>475</v>
       </c>
       <c r="F2" s="44" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="G2" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H2" s="44" t="s">
-        <v>481</v>
+        <v>474</v>
       </c>
       <c r="I2" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J2" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K2" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L2" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M2" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N2" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -7776,40 +7744,40 @@
         <v>149</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="D3" s="32" t="s">
         <v>121</v>
       </c>
       <c r="E3" s="32" t="s">
-        <v>483</v>
+        <v>476</v>
       </c>
       <c r="F3" s="44" t="s">
-        <v>482</v>
+        <v>475</v>
       </c>
       <c r="G3" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H3" s="44" t="s">
-        <v>481</v>
+        <v>474</v>
       </c>
       <c r="I3" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J3" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L3" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M3" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N3" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -7820,40 +7788,40 @@
         <v>149</v>
       </c>
       <c r="C4" s="32" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="D4" s="32" t="s">
         <v>121</v>
       </c>
       <c r="E4" s="32" t="s">
-        <v>482</v>
+        <v>475</v>
       </c>
       <c r="F4" s="44" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="G4" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H4" s="44" t="s">
-        <v>481</v>
+        <v>474</v>
       </c>
       <c r="I4" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J4" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K4" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L4" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M4" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N4" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -7864,40 +7832,40 @@
         <v>149</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="D5" s="32" t="s">
         <v>121</v>
       </c>
       <c r="E5" s="32" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="F5" s="44" t="s">
-        <v>484</v>
+        <v>477</v>
       </c>
       <c r="G5" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H5" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="I5" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J5" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L5" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N5" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -7908,40 +7876,40 @@
         <v>149</v>
       </c>
       <c r="C6" s="44" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="D6" s="44" t="s">
         <v>121</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="F6" s="44" t="s">
-        <v>484</v>
+        <v>477</v>
       </c>
       <c r="G6" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H6" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="I6" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J6" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K6" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L6" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M6" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N6" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -7952,40 +7920,40 @@
         <v>149</v>
       </c>
       <c r="C7" s="44" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="D7" s="44" t="s">
         <v>121</v>
       </c>
       <c r="E7" s="44" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="F7" s="44" t="s">
-        <v>484</v>
+        <v>477</v>
       </c>
       <c r="G7" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H7" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="I7" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J7" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K7" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L7" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M7" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N7" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -7996,40 +7964,40 @@
         <v>149</v>
       </c>
       <c r="C8" s="44" t="s">
-        <v>485</v>
+        <v>478</v>
       </c>
       <c r="D8" s="44" t="s">
         <v>121</v>
       </c>
       <c r="E8" s="44" t="s">
-        <v>486</v>
+        <v>479</v>
       </c>
       <c r="F8" s="44" t="s">
-        <v>488</v>
+        <v>481</v>
       </c>
       <c r="G8" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H8" s="44" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
       <c r="I8" s="44" t="s">
-        <v>493</v>
+        <v>486</v>
       </c>
       <c r="J8" s="44" t="s">
-        <v>491</v>
+        <v>484</v>
       </c>
       <c r="K8" s="44" t="s">
-        <v>487</v>
+        <v>480</v>
       </c>
       <c r="L8" s="44" t="s">
-        <v>489</v>
+        <v>482</v>
       </c>
       <c r="M8" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N8" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -8040,40 +8008,40 @@
         <v>149</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="D9" s="32" t="s">
         <v>121</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="F9" s="44" t="s">
-        <v>483</v>
+        <v>476</v>
       </c>
       <c r="G9" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H9" s="44" t="s">
-        <v>498</v>
+        <v>491</v>
       </c>
       <c r="I9" s="44" t="s">
-        <v>499</v>
+        <v>492</v>
       </c>
       <c r="J9" s="44" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="K9" s="44" t="s">
-        <v>497</v>
+        <v>490</v>
       </c>
       <c r="L9" s="44" t="s">
+        <v>481</v>
+      </c>
+      <c r="M9" s="44" t="s">
+        <v>428</v>
+      </c>
+      <c r="N9" s="44" t="s">
         <v>488</v>
-      </c>
-      <c r="M9" s="44" t="s">
-        <v>429</v>
-      </c>
-      <c r="N9" s="44" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -8084,40 +8052,40 @@
         <v>149</v>
       </c>
       <c r="C10" s="44" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="D10" s="44" t="s">
         <v>121</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>502</v>
+        <v>495</v>
       </c>
       <c r="F10" s="44" t="s">
-        <v>504</v>
+        <v>497</v>
       </c>
       <c r="G10" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H10" s="44" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
       <c r="I10" s="44" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="J10" s="44" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
       <c r="K10" s="44" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
       <c r="L10" s="44" t="s">
+        <v>481</v>
+      </c>
+      <c r="M10" s="44" t="s">
+        <v>494</v>
+      </c>
+      <c r="N10" s="44" t="s">
         <v>488</v>
-      </c>
-      <c r="M10" s="44" t="s">
-        <v>501</v>
-      </c>
-      <c r="N10" s="44" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -8128,40 +8096,40 @@
         <v>149</v>
       </c>
       <c r="C11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="E11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="F11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="G11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="H11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="I11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N11" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -8172,40 +8140,40 @@
         <v>149</v>
       </c>
       <c r="C12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="D12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="E12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="F12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="G12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="I12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N12" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -8216,40 +8184,40 @@
         <v>149</v>
       </c>
       <c r="C13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="D13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="E13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="F13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="G13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="H13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="I13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N13" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -8260,40 +8228,40 @@
         <v>149</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="D14" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="E14" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="F14" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="G14" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="H14" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="I14" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J14" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K14" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L14" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M14" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N14" s="44" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
     </row>
     <row r="15" spans="1:14">
@@ -8304,40 +8272,40 @@
         <v>149</v>
       </c>
       <c r="C15" s="44" t="s">
-        <v>509</v>
+        <v>502</v>
       </c>
       <c r="D15" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="E15" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="F15" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="G15" s="44" t="s">
-        <v>510</v>
+        <v>503</v>
       </c>
       <c r="H15" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="I15" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J15" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K15" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L15" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M15" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N15" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="16" spans="1:14">
@@ -8345,43 +8313,43 @@
         <v>303</v>
       </c>
       <c r="B16" s="32" t="s">
-        <v>511</v>
+        <v>504</v>
       </c>
       <c r="C16" s="32" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="D16" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="E16" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="F16" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="G16" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="H16" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="I16" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J16" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K16" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L16" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M16" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N16" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -8392,45 +8360,45 @@
         <v>149</v>
       </c>
       <c r="C17" s="32" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
       <c r="D17" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="E17" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="F17" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="G17" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="H17" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="I17" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="J17" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="K17" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L17" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="M17" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="N17" s="44" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="62" t="s">
-        <v>474</v>
+        <v>467</v>
       </c>
     </row>
   </sheetData>
@@ -8447,14 +8415,14 @@
   <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="21.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="6.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -8509,10 +8477,10 @@
         <v>50</v>
       </c>
       <c r="H2" s="44" t="s">
-        <v>524</v>
+        <v>517</v>
       </c>
       <c r="I2" s="44" t="s">
-        <v>525</v>
+        <v>518</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -8538,10 +8506,10 @@
         <v>50</v>
       </c>
       <c r="H3" s="44" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="I3" s="44" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
   </sheetData>
@@ -8558,18 +8526,18 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="4" max="4" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" customWidth="true" width="15.08984375"/>
+    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" customWidth="1"/>
+    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -8723,16 +8691,16 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="35" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C6" s="35" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E6" s="35">
         <v>2</v>
@@ -8742,7 +8710,7 @@
       <c r="H6" s="44"/>
       <c r="I6" s="44"/>
       <c r="J6" s="44" t="s">
-        <v>590</v>
+        <v>573</v>
       </c>
       <c r="K6" s="44"/>
       <c r="L6" s="44"/>
@@ -8761,16 +8729,16 @@
   <dimension ref="A1:K4"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="29" width="17.90625"/>
-    <col min="2" max="2" customWidth="true" style="29" width="11.81640625"/>
-    <col min="3" max="3" customWidth="true" style="29" width="13.0"/>
-    <col min="4" max="4" customWidth="true" style="29" width="16.54296875"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.81640625"/>
-    <col min="6" max="6" style="29" width="8.81640625"/>
-    <col min="7" max="7" customWidth="true" style="29" width="17.81640625"/>
-    <col min="8" max="8" customWidth="true" style="29" width="15.453125"/>
-    <col min="9" max="9" customWidth="true" style="29" width="11.54296875"/>
-    <col min="10" max="16384" style="29" width="8.81640625"/>
+    <col min="1" max="1" width="17.90625" style="29" customWidth="1"/>
+    <col min="2" max="2" width="11.81640625" style="29" customWidth="1"/>
+    <col min="3" max="3" width="13" style="29" customWidth="1"/>
+    <col min="4" max="4" width="16.54296875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" style="29" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" style="29"/>
+    <col min="7" max="7" width="17.81640625" style="29" customWidth="1"/>
+    <col min="8" max="8" width="15.453125" style="29" customWidth="1"/>
+    <col min="9" max="9" width="11.54296875" style="29" customWidth="1"/>
+    <col min="10" max="16384" width="8.81640625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -8825,7 +8793,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="32" t="s">
-        <v>591</v>
+        <v>574</v>
       </c>
       <c r="G2" s="32">
         <v>2</v>
@@ -8856,7 +8824,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="32" t="s">
-        <v>592</v>
+        <v>575</v>
       </c>
       <c r="G3" s="32"/>
       <c r="H3" s="32"/>
@@ -8885,7 +8853,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="32" t="s">
-        <v>593</v>
+        <v>576</v>
       </c>
       <c r="G4" s="32"/>
       <c r="H4" s="32"/>
@@ -8906,19 +8874,19 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="19.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="1" max="1" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -8964,7 +8932,7 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2" s="44" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B2" s="47" t="s">
         <v>32</v>
@@ -8987,7 +8955,7 @@
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="44" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B3" s="47" t="s">
         <v>325</v>
@@ -9021,20 +8989,20 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="25.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="41" width="4.453125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="41" width="14.1796875"/>
-    <col min="14" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="25.81640625" style="41" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" style="41" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.1796875" style="41" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -9080,10 +9048,10 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2" s="44" t="s">
+        <v>394</v>
+      </c>
+      <c r="B2" s="47" t="s">
         <v>395</v>
-      </c>
-      <c r="B2" s="47" t="s">
-        <v>396</v>
       </c>
       <c r="C2" s="44" t="s">
         <v>12</v>
@@ -9103,10 +9071,10 @@
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="48" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B3" s="47" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C3" s="44" t="s">
         <v>12</v>
@@ -9126,7 +9094,7 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="44" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B4" s="47" t="s">
         <v>336</v>
@@ -9160,21 +9128,21 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="20.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="6" max="7" customWidth="true" style="41" width="17.36328125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="41" width="4.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="41" width="14.1796875"/>
-    <col min="16" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="20.1796875" style="41" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="17.36328125" style="41" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.453125" style="41" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.1796875" style="41" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -9194,7 +9162,7 @@
         <v>1</v>
       </c>
       <c r="F1" s="42" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="G1" s="42" t="s">
         <v>30</v>
@@ -9226,7 +9194,7 @@
     </row>
     <row r="2" spans="1:15">
       <c r="A2" s="44" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B2" s="47" t="s">
         <v>332</v>
@@ -9241,10 +9209,10 @@
         <v>2</v>
       </c>
       <c r="F2" s="44" t="s">
+        <v>400</v>
+      </c>
+      <c r="G2" s="44" t="s">
         <v>401</v>
-      </c>
-      <c r="G2" s="44" t="s">
-        <v>402</v>
       </c>
       <c r="H2" s="44"/>
       <c r="I2" s="44"/>
@@ -9257,7 +9225,7 @@
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="44" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B3" s="47" t="s">
         <v>332</v>
@@ -9272,10 +9240,10 @@
         <v>2</v>
       </c>
       <c r="F3" s="44" t="s">
+        <v>400</v>
+      </c>
+      <c r="G3" s="44" t="s">
         <v>401</v>
-      </c>
-      <c r="G3" s="44" t="s">
-        <v>402</v>
       </c>
       <c r="H3" s="44"/>
       <c r="I3" s="44"/>
@@ -9288,7 +9256,7 @@
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="44" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B4" s="47" t="s">
         <v>332</v>
@@ -9303,10 +9271,10 @@
         <v>2</v>
       </c>
       <c r="F4" s="44" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G4" s="44" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="H4" s="44"/>
       <c r="I4" s="44"/>
@@ -9319,7 +9287,7 @@
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="44" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B5" s="47" t="s">
         <v>332</v>
@@ -9334,10 +9302,10 @@
         <v>2</v>
       </c>
       <c r="F5" s="44" t="s">
+        <v>400</v>
+      </c>
+      <c r="G5" s="44" t="s">
         <v>401</v>
-      </c>
-      <c r="G5" s="44" t="s">
-        <v>402</v>
       </c>
       <c r="H5" s="44"/>
       <c r="I5" s="44"/>
@@ -9361,22 +9329,22 @@
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="28.36328125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="41" width="16.81640625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="41" width="11.08984375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="12" max="12" customWidth="true" style="41" width="13.08984375"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="41" width="14.1796875"/>
-    <col min="16" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="28.36328125" style="41" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.81640625" style="41" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.08984375" style="41" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.08984375" style="41" customWidth="1"/>
+    <col min="13" max="13" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.1796875" style="41" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -9396,10 +9364,10 @@
         <v>1</v>
       </c>
       <c r="F1" s="42" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="G1" s="42" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="H1" s="43" t="s">
         <v>74</v>
@@ -9408,23 +9376,23 @@
         <v>8</v>
       </c>
       <c r="J1" s="43" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="K1" s="43" t="s">
         <v>75</v>
       </c>
       <c r="L1" s="43" t="s">
+        <v>354</v>
+      </c>
+      <c r="M1" s="43" t="s">
         <v>355</v>
-      </c>
-      <c r="M1" s="43" t="s">
-        <v>356</v>
       </c>
       <c r="N1" s="40"/>
       <c r="O1" s="46"/>
     </row>
     <row r="2" spans="1:15">
       <c r="A2" s="44" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B2" s="47" t="s">
         <v>32</v>
@@ -9447,7 +9415,7 @@
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="44" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B3" s="47" t="s">
         <v>32</v>
@@ -9472,16 +9440,16 @@
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="44" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B4" s="47" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="C4" s="44" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E4" s="44">
         <v>1</v>
@@ -9491,34 +9459,34 @@
       </c>
       <c r="G4" s="44"/>
       <c r="H4" s="44" t="s">
-        <v>594</v>
+        <v>577</v>
       </c>
       <c r="I4" s="44" t="s">
+        <v>387</v>
+      </c>
+      <c r="J4" s="44" t="s">
         <v>388</v>
-      </c>
-      <c r="J4" s="44" t="s">
-        <v>389</v>
       </c>
       <c r="K4" s="44"/>
       <c r="L4" s="44" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="M4" s="44" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="44" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B5" s="47" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C5" s="44" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="44" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E5" s="44">
         <v>1</v>
@@ -9528,25 +9496,25 @@
       </c>
       <c r="G5" s="44"/>
       <c r="H5" s="44" t="s">
-        <v>595</v>
+        <v>578</v>
       </c>
       <c r="I5" s="44" t="s">
+        <v>387</v>
+      </c>
+      <c r="J5" s="44" t="s">
         <v>388</v>
-      </c>
-      <c r="J5" s="44" t="s">
-        <v>389</v>
       </c>
       <c r="K5" s="44"/>
       <c r="L5" s="44" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="44" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B6" s="47" t="s">
         <v>32</v>
@@ -9569,7 +9537,7 @@
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="44" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B7" s="47" t="s">
         <v>32</v>
@@ -9592,7 +9560,7 @@
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="44" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B8" s="47" t="s">
         <v>32</v>
@@ -9617,7 +9585,7 @@
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="44" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B9" s="47" t="s">
         <v>32</v>
@@ -9642,7 +9610,7 @@
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="44" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B10" s="47" t="s">
         <v>32</v>
@@ -9676,11 +9644,11 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="24.0"/>
-    <col min="2" max="2" customWidth="true" style="41" width="11.453125"/>
-    <col min="3" max="3" style="41" width="8.90625"/>
-    <col min="4" max="4" customWidth="true" style="41" width="19.6328125"/>
-    <col min="5" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="24" style="41" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" style="41" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" style="41"/>
+    <col min="4" max="4" width="19.6328125" style="41" customWidth="1"/>
+    <col min="5" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -9699,10 +9667,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="44" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B2" s="47" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C2" s="44" t="s">
         <v>12</v>
@@ -9724,12 +9692,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="32.1796875"/>
-    <col min="2" max="2" customWidth="true" style="41" width="14.0"/>
-    <col min="3" max="3" customWidth="true" style="41" width="16.6328125"/>
-    <col min="4" max="4" customWidth="true" style="41" width="17.6328125"/>
-    <col min="5" max="5" customWidth="true" style="41" width="11.81640625"/>
-    <col min="6" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="32.1796875" style="41" customWidth="1"/>
+    <col min="2" max="2" width="14" style="41" customWidth="1"/>
+    <col min="3" max="3" width="16.6328125" style="41" customWidth="1"/>
+    <col min="4" max="4" width="17.6328125" style="41" customWidth="1"/>
+    <col min="5" max="5" width="11.81640625" style="41" customWidth="1"/>
+    <col min="6" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -9751,7 +9719,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="44" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B2" s="47" t="s">
         <v>32</v>
@@ -9768,10 +9736,10 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="44" t="s">
+        <v>419</v>
+      </c>
+      <c r="B3" s="47" t="s">
         <v>420</v>
-      </c>
-      <c r="B3" s="47" t="s">
-        <v>421</v>
       </c>
       <c r="C3" s="44" t="s">
         <v>12</v>
@@ -9785,10 +9753,10 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="44" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B4" s="47" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C4" s="44" t="s">
         <v>12</v>
@@ -9813,11 +9781,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="38.1796875"/>
-    <col min="2" max="2" customWidth="true" style="41" width="13.54296875"/>
-    <col min="3" max="3" customWidth="true" style="41" width="15.54296875"/>
-    <col min="4" max="4" customWidth="true" style="41" width="19.0"/>
-    <col min="5" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="38.1796875" style="41" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" style="41" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" style="41" customWidth="1"/>
+    <col min="4" max="4" width="19" style="41" customWidth="1"/>
+    <col min="5" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -9825,30 +9793,30 @@
         <v>0</v>
       </c>
       <c r="B1" s="49" t="s">
+        <v>422</v>
+      </c>
+      <c r="C1" s="49" t="s">
         <v>423</v>
       </c>
-      <c r="C1" s="49" t="s">
+      <c r="D1" s="49" t="s">
         <v>424</v>
       </c>
-      <c r="D1" s="49" t="s">
+      <c r="E1" s="49" t="s">
         <v>425</v>
-      </c>
-      <c r="E1" s="49" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="44" t="s">
+        <v>426</v>
+      </c>
+      <c r="B2" s="47" t="s">
         <v>427</v>
       </c>
-      <c r="B2" s="47" t="s">
+      <c r="C2" s="44" t="s">
         <v>428</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="D2" s="44" t="s">
         <v>429</v>
-      </c>
-      <c r="D2" s="44" t="s">
-        <v>430</v>
       </c>
       <c r="E2" s="44" t="s">
         <v>12</v>
@@ -9856,16 +9824,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="44" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B3" s="47" t="s">
+        <v>427</v>
+      </c>
+      <c r="C3" s="44" t="s">
         <v>428</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="D3" s="44" t="s">
         <v>429</v>
-      </c>
-      <c r="D3" s="44" t="s">
-        <v>430</v>
       </c>
       <c r="E3" s="44" t="s">
         <v>12</v>
@@ -9873,23 +9841,23 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="44" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B4" s="44"/>
       <c r="C4" s="44"/>
       <c r="D4" s="44" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="E4" s="44"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="44" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B5" s="44"/>
       <c r="C5" s="44"/>
       <c r="D5" s="44" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>12</v>
@@ -9897,31 +9865,31 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="50" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B6" s="47" t="s">
+        <v>427</v>
+      </c>
+      <c r="C6" s="44" t="s">
         <v>428</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="D6" s="44" t="s">
         <v>429</v>
-      </c>
-      <c r="D6" s="44" t="s">
-        <v>430</v>
       </c>
       <c r="E6" s="44"/>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="51" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B7" s="47" t="s">
+        <v>427</v>
+      </c>
+      <c r="C7" s="44" t="s">
         <v>428</v>
       </c>
-      <c r="C7" s="44" t="s">
+      <c r="D7" s="44" t="s">
         <v>429</v>
-      </c>
-      <c r="D7" s="44" t="s">
-        <v>430</v>
       </c>
       <c r="E7" s="44" t="s">
         <v>12</v>
@@ -9940,21 +9908,21 @@
   <dimension ref="A1:N5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="30.90625"/>
-    <col min="2" max="2" customWidth="true" style="41" width="17.81640625"/>
-    <col min="3" max="3" customWidth="true" style="41" width="16.453125"/>
-    <col min="4" max="4" customWidth="true" style="41" width="16.08984375"/>
-    <col min="5" max="5" customWidth="true" style="41" width="12.0"/>
-    <col min="6" max="6" customWidth="true" style="41" width="18.08984375"/>
-    <col min="7" max="7" customWidth="true" style="41" width="15.08984375"/>
-    <col min="8" max="8" customWidth="true" style="41" width="10.453125"/>
-    <col min="9" max="9" customWidth="true" style="41" width="10.81640625"/>
-    <col min="10" max="10" style="41" width="8.90625"/>
-    <col min="11" max="11" customWidth="true" style="41" width="13.1796875"/>
-    <col min="12" max="12" customWidth="true" style="41" width="12.6328125"/>
-    <col min="13" max="13" customWidth="true" style="41" width="14.08984375"/>
-    <col min="14" max="14" customWidth="true" style="41" width="14.36328125"/>
-    <col min="15" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="30.90625" style="41" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" style="41" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" style="41" customWidth="1"/>
+    <col min="4" max="4" width="16.08984375" style="41" customWidth="1"/>
+    <col min="5" max="5" width="12" style="41" customWidth="1"/>
+    <col min="6" max="6" width="18.08984375" style="41" customWidth="1"/>
+    <col min="7" max="7" width="15.08984375" style="41" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" style="41" customWidth="1"/>
+    <col min="9" max="9" width="10.81640625" style="41" customWidth="1"/>
+    <col min="10" max="10" width="8.90625" style="41"/>
+    <col min="11" max="11" width="13.1796875" style="41" customWidth="1"/>
+    <col min="12" max="12" width="12.6328125" style="41" customWidth="1"/>
+    <col min="13" max="13" width="14.08984375" style="41" customWidth="1"/>
+    <col min="14" max="14" width="14.36328125" style="41" customWidth="1"/>
+    <col min="15" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -9980,7 +9948,7 @@
         <v>4</v>
       </c>
       <c r="H1" s="53" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="I1" s="53" t="s">
         <v>9</v>
@@ -9992,10 +9960,10 @@
         <v>210</v>
       </c>
       <c r="L1" s="42" t="s">
+        <v>354</v>
+      </c>
+      <c r="M1" s="42" t="s">
         <v>355</v>
-      </c>
-      <c r="M1" s="42" t="s">
-        <v>356</v>
       </c>
       <c r="N1" s="42" t="s">
         <v>75</v>
@@ -10003,13 +9971,13 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="54" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B2" s="44">
         <v>2</v>
       </c>
       <c r="C2" s="47" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D2" s="44" t="s">
         <v>12</v>
@@ -10021,7 +9989,7 @@
         <v>12</v>
       </c>
       <c r="G2" s="44" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="H2" s="44" t="s">
         <v>211</v>
@@ -10030,28 +9998,28 @@
         <v>212</v>
       </c>
       <c r="J2" s="44" t="s">
-        <v>596</v>
+        <v>579</v>
       </c>
       <c r="K2" s="44">
         <v>2</v>
       </c>
       <c r="L2" s="44" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="M2" s="44" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="N2" s="44"/>
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="44" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B3" s="44">
         <v>2</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D3" s="44" t="s">
         <v>12</v>
@@ -10069,13 +10037,13 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="55" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B4" s="44">
         <v>2</v>
       </c>
       <c r="C4" s="47" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D4" s="44" t="s">
         <v>12</v>
@@ -10087,16 +10055,16 @@
         <v>12</v>
       </c>
       <c r="G4" s="44" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="H4" s="44" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="I4" s="44" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="J4" s="44" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="K4" s="44"/>
       <c r="L4" s="44"/>
@@ -10107,13 +10075,13 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="44" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="B5" s="44">
         <v>2</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="D5" s="44" t="s">
         <v>12</v>
@@ -10125,16 +10093,16 @@
         <v>12</v>
       </c>
       <c r="G5" s="44" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="H5" s="44" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="I5" s="44" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="J5" s="44" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="K5" s="44"/>
       <c r="L5" s="44"/>
@@ -10156,11 +10124,11 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -10228,10 +10196,10 @@
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="57.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="15.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="4" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="1" max="1" width="57.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -10265,7 +10233,7 @@
         <v>209</v>
       </c>
       <c r="E2" s="44" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -10299,7 +10267,7 @@
         <v>209</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -10316,7 +10284,7 @@
         <v>209</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -10350,28 +10318,28 @@
   <dimension ref="A1:V15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="50.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="25" width="18.36328125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="25" width="12.08984375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="25" width="15.36328125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="25" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="25" width="9.453125"/>
-    <col min="7" max="8" style="25" width="8.81640625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="8.1796875"/>
-    <col min="15" max="15" customWidth="true" style="25" width="13.0"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="10.1796875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" style="25" width="9.1796875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="25" width="11.6328125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="23" max="16384" style="25" width="8.81640625"/>
+    <col min="1" max="1" width="50" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.36328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.08984375" style="25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.36328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="8.81640625" style="25"/>
+    <col min="9" max="9" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13" style="25" customWidth="1"/>
+    <col min="16" max="16" width="10.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="8.81640625" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -10430,16 +10398,16 @@
         <v>9</v>
       </c>
       <c r="S1" s="30" t="s">
+        <v>354</v>
+      </c>
+      <c r="T1" s="30" t="s">
         <v>355</v>
-      </c>
-      <c r="T1" s="30" t="s">
-        <v>356</v>
       </c>
       <c r="U1" s="30" t="s">
         <v>30</v>
       </c>
       <c r="V1" s="30" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="2" spans="1:22">
@@ -10465,7 +10433,7 @@
         <v>15</v>
       </c>
       <c r="H2" s="32" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="I2" s="32" t="s">
         <v>211</v>
@@ -10482,14 +10450,14 @@
       <c r="M2" s="32"/>
       <c r="N2" s="32"/>
       <c r="O2" s="32" t="s">
-        <v>528</v>
+        <v>521</v>
       </c>
       <c r="P2" s="32"/>
       <c r="Q2" s="32" t="s">
+        <v>357</v>
+      </c>
+      <c r="R2" s="32" t="s">
         <v>358</v>
-      </c>
-      <c r="R2" s="32" t="s">
-        <v>359</v>
       </c>
       <c r="S2" s="32"/>
       <c r="T2" s="32"/>
@@ -10606,7 +10574,7 @@
     </row>
     <row r="6" spans="1:22" s="29" customFormat="1">
       <c r="A6" s="32" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B6" s="44">
         <v>0</v>
@@ -10627,13 +10595,13 @@
         <v>15</v>
       </c>
       <c r="H6" s="32" t="s">
-        <v>529</v>
+        <v>522</v>
       </c>
       <c r="I6" s="32" t="s">
+        <v>387</v>
+      </c>
+      <c r="J6" s="32" t="s">
         <v>388</v>
-      </c>
-      <c r="J6" s="32" t="s">
-        <v>389</v>
       </c>
       <c r="K6" s="32"/>
       <c r="L6" s="32"/>
@@ -10644,17 +10612,17 @@
       <c r="Q6" s="32"/>
       <c r="R6" s="32"/>
       <c r="S6" s="32" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="T6" s="32" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="U6" s="32"/>
       <c r="V6" s="32"/>
     </row>
     <row r="7" spans="1:22">
       <c r="A7" s="39" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B7" s="44">
         <v>0</v>
@@ -10675,13 +10643,13 @@
         <v>19</v>
       </c>
       <c r="H7" s="32" t="s">
-        <v>533</v>
+        <v>526</v>
       </c>
       <c r="I7" s="32" t="s">
+        <v>360</v>
+      </c>
+      <c r="J7" s="32" t="s">
         <v>361</v>
-      </c>
-      <c r="J7" s="32" t="s">
-        <v>362</v>
       </c>
       <c r="K7" s="32"/>
       <c r="L7" s="32"/>
@@ -10698,7 +10666,7 @@
     </row>
     <row r="8" spans="1:22" s="29" customFormat="1">
       <c r="A8" s="32" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B8" s="44">
         <v>0</v>
@@ -10730,7 +10698,7 @@
     </row>
     <row r="9" spans="1:22">
       <c r="A9" s="39" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B9" s="44">
         <v>0</v>
@@ -10751,13 +10719,13 @@
         <v>15</v>
       </c>
       <c r="H9" s="32" t="s">
+        <v>363</v>
+      </c>
+      <c r="I9" s="32" t="s">
         <v>364</v>
       </c>
-      <c r="I9" s="32" t="s">
+      <c r="J9" s="32" t="s">
         <v>365</v>
-      </c>
-      <c r="J9" s="32" t="s">
-        <v>366</v>
       </c>
       <c r="K9" s="32"/>
       <c r="L9" s="32"/>
@@ -10774,7 +10742,7 @@
     </row>
     <row r="10" spans="1:22" s="29" customFormat="1">
       <c r="A10" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B10" s="44">
         <v>0</v>
@@ -10793,11 +10761,11 @@
       </c>
       <c r="G10" s="56"/>
       <c r="H10" s="32" t="s">
-        <v>530</v>
+        <v>523</v>
       </c>
       <c r="I10" s="32"/>
       <c r="J10" s="32" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="K10" s="32"/>
       <c r="L10" s="32"/>
@@ -10808,19 +10776,19 @@
       <c r="Q10" s="32"/>
       <c r="R10" s="32"/>
       <c r="S10" s="32" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="T10" s="32" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="U10" s="32"/>
       <c r="V10" s="32" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="11" spans="1:22">
       <c r="A11" s="39" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B11" s="44">
         <v>0</v>
@@ -10841,7 +10809,7 @@
         <v>15</v>
       </c>
       <c r="H11" s="32" t="s">
-        <v>527</v>
+        <v>520</v>
       </c>
       <c r="I11" s="32" t="s">
         <v>211</v>
@@ -10856,25 +10824,25 @@
       <c r="O11" s="32"/>
       <c r="P11" s="32"/>
       <c r="Q11" s="32" t="s">
+        <v>370</v>
+      </c>
+      <c r="R11" s="32" t="s">
         <v>371</v>
       </c>
-      <c r="R11" s="32" t="s">
+      <c r="S11" s="32" t="s">
         <v>372</v>
       </c>
-      <c r="S11" s="32" t="s">
+      <c r="T11" s="32" t="s">
         <v>373</v>
       </c>
-      <c r="T11" s="32" t="s">
+      <c r="U11" s="32" t="s">
         <v>374</v>
-      </c>
-      <c r="U11" s="32" t="s">
-        <v>375</v>
       </c>
       <c r="V11" s="32"/>
     </row>
     <row r="12" spans="1:22">
       <c r="A12" s="39" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B12" s="44">
         <v>2</v>
@@ -10893,19 +10861,19 @@
       </c>
       <c r="G12" s="56"/>
       <c r="H12" s="32" t="s">
-        <v>531</v>
+        <v>524</v>
       </c>
       <c r="I12" s="32" t="s">
+        <v>376</v>
+      </c>
+      <c r="J12" s="32" t="s">
         <v>377</v>
       </c>
-      <c r="J12" s="32" t="s">
+      <c r="K12" s="32" t="s">
         <v>378</v>
       </c>
-      <c r="K12" s="32" t="s">
-        <v>379</v>
-      </c>
       <c r="L12" s="32" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="M12" s="32"/>
       <c r="N12" s="32"/>
@@ -10914,25 +10882,25 @@
       <c r="Q12" s="32"/>
       <c r="R12" s="32"/>
       <c r="S12" s="32" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="T12" s="32" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="U12" s="32"/>
       <c r="V12" s="32" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="13" spans="1:22">
       <c r="A13" s="39" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B13" s="44">
         <v>3</v>
       </c>
       <c r="C13" s="47" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D13" s="44" t="s">
         <v>216</v>
@@ -10962,7 +10930,7 @@
     </row>
     <row r="14" spans="1:22">
       <c r="A14" s="39" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B14" s="44">
         <v>1</v>
@@ -10981,7 +10949,7 @@
       </c>
       <c r="G14" s="56"/>
       <c r="H14" s="32" t="s">
-        <v>532</v>
+        <v>525</v>
       </c>
       <c r="I14" s="32" t="s">
         <v>244</v>
@@ -10998,19 +10966,19 @@
       <c r="Q14" s="32"/>
       <c r="R14" s="32"/>
       <c r="S14" s="32" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="T14" s="32" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="U14" s="32"/>
       <c r="V14" s="32" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="15" spans="1:22" s="29" customFormat="1">
       <c r="A15" s="39" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B15" s="44">
         <v>0</v>
@@ -11031,13 +10999,13 @@
         <v>15</v>
       </c>
       <c r="H15" s="32" t="s">
-        <v>526</v>
+        <v>519</v>
       </c>
       <c r="I15" s="32" t="s">
+        <v>367</v>
+      </c>
+      <c r="J15" s="32" t="s">
         <v>368</v>
-      </c>
-      <c r="J15" s="32" t="s">
-        <v>369</v>
       </c>
       <c r="K15" s="32"/>
       <c r="L15" s="32"/>
@@ -11066,29 +11034,29 @@
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="44.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="8.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="13.54296875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.81640625"/>
-    <col min="11" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.1796875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="8.1796875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="14.1796875"/>
-    <col min="27" max="28" bestFit="true" customWidth="true" width="12.81640625"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="14.1796875"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="12.81640625"/>
+    <col min="1" max="1" width="44.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -11520,9 +11488,9 @@
   <dimension ref="A1:W17"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="54.36328125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="1" max="1" width="54.36328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -11625,10 +11593,10 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>535</v>
+        <v>528</v>
       </c>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
@@ -11887,10 +11855,10 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3" t="s">
-        <v>538</v>
+        <v>531</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>539</v>
+        <v>532</v>
       </c>
       <c r="T8" s="3">
         <v>0</v>
@@ -11907,7 +11875,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="47" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>12</v>
@@ -11936,10 +11904,10 @@
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
       <c r="R9" s="3" t="s">
-        <v>540</v>
+        <v>533</v>
       </c>
       <c r="S9" s="3" t="s">
-        <v>541</v>
+        <v>534</v>
       </c>
       <c r="T9" s="3"/>
       <c r="U9" s="3">
@@ -11960,7 +11928,7 @@
         <v>2</v>
       </c>
       <c r="C10" s="47" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>12</v>
@@ -11989,10 +11957,10 @@
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
       <c r="R10" s="3" t="s">
-        <v>542</v>
+        <v>535</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>543</v>
+        <v>536</v>
       </c>
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
@@ -12186,7 +12154,7 @@
         <v>2</v>
       </c>
       <c r="C16" s="47" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="D16" s="32" t="s">
         <v>12</v>
@@ -12215,10 +12183,10 @@
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
       <c r="R16" s="3" t="s">
-        <v>536</v>
+        <v>529</v>
       </c>
       <c r="S16" s="3" t="s">
-        <v>537</v>
+        <v>530</v>
       </c>
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>
@@ -12273,16 +12241,16 @@
   <dimension ref="A1:S20"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="53.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="5" max="7" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="53.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="12.1796875" customWidth="1"/>
+    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -12450,7 +12418,7 @@
         <v>264</v>
       </c>
       <c r="F5" s="44" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G5" s="44"/>
       <c r="H5" s="44"/>

</xml_diff>

<commit_message>
Modified TimaticService and XMLParser
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BF7513F-D4E8-44F3-A783-34C83AC232C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC38559A-FC4C-498F-958D-81BED35A6CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="8" activeTab="10" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="25" activeTab="28" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2124" uniqueCount="642">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2105" uniqueCount="635">
   <si>
     <t>Scenario</t>
   </si>
@@ -1507,9 +1507,6 @@
     <t>GB</t>
   </si>
   <si>
-    <t>NIL</t>
-  </si>
-  <si>
     <t>BA</t>
   </si>
   <si>
@@ -1588,9 +1585,6 @@
     <t>BKK</t>
   </si>
   <si>
-    <t>VS</t>
-  </si>
-  <si>
     <t>AG</t>
   </si>
   <si>
@@ -1897,45 +1891,12 @@
     <t>2302182816322</t>
   </si>
   <si>
-    <t>A340FE</t>
-  </si>
-  <si>
     <t>2023-08-26T07:56:00</t>
   </si>
   <si>
     <t>2023-08-26T12:05:00</t>
   </si>
   <si>
-    <t>2302182816168</t>
-  </si>
-  <si>
-    <t>A4FFSD</t>
-  </si>
-  <si>
-    <t>2302182816568</t>
-  </si>
-  <si>
-    <t>2302182816569</t>
-  </si>
-  <si>
-    <t>A340F1</t>
-  </si>
-  <si>
-    <t>2302182816169</t>
-  </si>
-  <si>
-    <t>A340GR</t>
-  </si>
-  <si>
-    <t>2302182816170</t>
-  </si>
-  <si>
-    <t>A340G0</t>
-  </si>
-  <si>
-    <t>2302182816171</t>
-  </si>
-  <si>
     <t>485</t>
   </si>
   <si>
@@ -1960,21 +1921,9 @@
     <t>2302182817362</t>
   </si>
   <si>
-    <t>A4INWJ</t>
-  </si>
-  <si>
-    <t>2302182817363</t>
-  </si>
-  <si>
-    <t>2302182817364</t>
-  </si>
-  <si>
     <t>A4INYY</t>
   </si>
   <si>
-    <t>2302182817365</t>
-  </si>
-  <si>
     <t>A4IN3U</t>
   </si>
   <si>
@@ -1996,10 +1945,40 @@
     <t>2302182817413</t>
   </si>
   <si>
-    <t>2182817427</t>
-  </si>
-  <si>
     <t>2182817428</t>
+  </si>
+  <si>
+    <t>A5Z2AP</t>
+  </si>
+  <si>
+    <t>A5Z2AV</t>
+  </si>
+  <si>
+    <t>2023-08-29T01:14:00</t>
+  </si>
+  <si>
+    <t>2023-08-29T10:38:00</t>
+  </si>
+  <si>
+    <t>2023-08-29T12:02:00</t>
+  </si>
+  <si>
+    <t>2023-08-29T13:43:00</t>
+  </si>
+  <si>
+    <t>A5Z2BO</t>
+  </si>
+  <si>
+    <t>A5Z2BW</t>
+  </si>
+  <si>
+    <t>A5Z2B0</t>
+  </si>
+  <si>
+    <t>A5Z2C3</t>
+  </si>
+  <si>
+    <t>A5Z2D2</t>
   </si>
 </sst>
 </file>
@@ -2236,7 +2215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2335,7 +2314,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2743,7 +2721,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="44" t="s">
-        <v>513</v>
+        <v>631</v>
       </c>
       <c r="I2" s="32" t="s">
         <v>211</v>
@@ -2760,7 +2738,7 @@
       <c r="M2" s="32"/>
       <c r="N2" s="32"/>
       <c r="O2" s="32" t="s">
-        <v>514</v>
+        <v>632</v>
       </c>
       <c r="P2" s="38"/>
     </row>
@@ -2832,7 +2810,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="37" t="s">
-        <v>515</v>
+        <v>633</v>
       </c>
       <c r="I4" s="37" t="s">
         <v>351</v>
@@ -2869,7 +2847,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>516</v>
+        <v>634</v>
       </c>
       <c r="I5" s="32"/>
       <c r="J5" s="32"/>
@@ -3009,7 +2987,7 @@
       </c>
       <c r="J2" s="44"/>
       <c r="K2" s="44" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="L2" s="44"/>
       <c r="M2" s="44"/>
@@ -3046,10 +3024,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="L3" s="44" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="M3" s="44"/>
       <c r="N3" s="44"/>
@@ -3118,10 +3096,10 @@
       <c r="I5" s="44"/>
       <c r="J5" s="44"/>
       <c r="K5" s="44" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="L5" s="44" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="M5" s="44"/>
       <c r="N5" s="44" t="s">
@@ -3165,7 +3143,7 @@
       <c r="I6" s="44"/>
       <c r="J6" s="44"/>
       <c r="K6" s="44" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="L6" s="44"/>
       <c r="M6" s="44"/>
@@ -3176,7 +3154,7 @@
         <v>242</v>
       </c>
       <c r="P6" s="44" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="Q6" s="44"/>
       <c r="R6" s="44"/>
@@ -3210,10 +3188,10 @@
       <c r="I7" s="44"/>
       <c r="J7" s="44"/>
       <c r="K7" s="44" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="L7" s="44" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="M7" s="44"/>
       <c r="N7" s="44" t="s">
@@ -3223,13 +3201,13 @@
         <v>242</v>
       </c>
       <c r="P7" s="44" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="Q7" s="47" t="s">
         <v>87</v>
       </c>
       <c r="R7" s="44" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="S7" s="44"/>
       <c r="T7" s="44"/>
@@ -3265,10 +3243,10 @@
       </c>
       <c r="J8" s="44"/>
       <c r="K8" s="44" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="L8" s="44" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="M8" s="44"/>
       <c r="N8" s="44" t="s">
@@ -3306,7 +3284,7 @@
       <c r="I9" s="44"/>
       <c r="J9" s="44"/>
       <c r="K9" s="44" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="L9" s="44"/>
       <c r="M9" s="44"/>
@@ -3345,10 +3323,10 @@
       <c r="I10" s="44"/>
       <c r="J10" s="44"/>
       <c r="K10" s="44" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="L10" s="44" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="M10" s="44"/>
       <c r="N10" s="44"/>
@@ -3357,7 +3335,7 @@
       <c r="Q10" s="44"/>
       <c r="R10" s="44"/>
       <c r="S10" s="47" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="T10" s="44"/>
       <c r="U10" s="44"/>
@@ -3384,10 +3362,10 @@
       <c r="I11" s="44"/>
       <c r="J11" s="44"/>
       <c r="K11" s="44" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="L11" s="44" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="M11" s="44"/>
       <c r="N11" s="44"/>
@@ -3423,10 +3401,10 @@
       <c r="I12" s="44"/>
       <c r="J12" s="44"/>
       <c r="K12" s="44" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="L12" s="44" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="M12" s="44"/>
       <c r="N12" s="44" t="s">
@@ -3544,10 +3522,10 @@
       <c r="I15" s="44"/>
       <c r="J15" s="44"/>
       <c r="K15" s="44" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="L15" s="44" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="M15" s="44"/>
       <c r="N15" s="44" t="s">
@@ -3573,7 +3551,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="47" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="D16" s="44" t="s">
         <v>12</v>
@@ -3587,7 +3565,7 @@
       <c r="I16" s="44"/>
       <c r="J16" s="44"/>
       <c r="K16" s="44" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="L16" s="44"/>
       <c r="M16" s="44"/>
@@ -3626,7 +3604,7 @@
       <c r="I17" s="44"/>
       <c r="J17" s="44"/>
       <c r="K17" s="44" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="L17" s="44"/>
       <c r="M17" s="44"/>
@@ -3833,7 +3811,7 @@
       </c>
       <c r="J22" s="44"/>
       <c r="K22" s="44" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="L22" s="44"/>
       <c r="M22" s="44"/>
@@ -3927,14 +3905,14 @@
         <v>2</v>
       </c>
       <c r="D2" s="47" t="s">
-        <v>623</v>
+        <v>610</v>
       </c>
       <c r="E2" s="47" t="s">
-        <v>622</v>
+        <v>609</v>
       </c>
       <c r="F2" s="44"/>
       <c r="G2" s="47" t="s">
-        <v>620</v>
+        <v>607</v>
       </c>
       <c r="H2" s="44" t="s">
         <v>12</v>
@@ -3958,7 +3936,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="47" t="s">
-        <v>624</v>
+        <v>611</v>
       </c>
       <c r="E3" s="47" t="s">
         <v>264</v>
@@ -3967,7 +3945,7 @@
         <v>149</v>
       </c>
       <c r="G3" s="47" t="s">
-        <v>620</v>
+        <v>607</v>
       </c>
       <c r="H3" s="44" t="s">
         <v>12</v>
@@ -3993,7 +3971,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="47" t="s">
-        <v>625</v>
+        <v>612</v>
       </c>
       <c r="E4" s="44"/>
       <c r="F4" s="44" t="s">
@@ -4009,7 +3987,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="47" t="s">
-        <v>621</v>
+        <v>608</v>
       </c>
       <c r="K4" s="44" t="s">
         <v>13</v>
@@ -4094,7 +4072,7 @@
       <c r="G2" s="44"/>
       <c r="H2" s="44"/>
       <c r="I2" s="44" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="J2" s="44"/>
       <c r="K2" s="44"/>
@@ -4113,7 +4091,7 @@
       <c r="G3" s="44"/>
       <c r="H3" s="44"/>
       <c r="I3" s="44" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="J3" s="44"/>
       <c r="K3" s="44"/>
@@ -4132,7 +4110,7 @@
       <c r="G4" s="44"/>
       <c r="H4" s="44"/>
       <c r="I4" s="44" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="J4" s="44"/>
       <c r="K4" s="44"/>
@@ -4163,13 +4141,13 @@
         <v>12</v>
       </c>
       <c r="I5" s="44" t="s">
+        <v>535</v>
+      </c>
+      <c r="J5" s="44" t="s">
+        <v>536</v>
+      </c>
+      <c r="K5" s="44" t="s">
         <v>537</v>
-      </c>
-      <c r="J5" s="44" t="s">
-        <v>538</v>
-      </c>
-      <c r="K5" s="44" t="s">
-        <v>539</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4198,10 +4176,10 @@
         <v>12</v>
       </c>
       <c r="I6" s="44" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="J6" s="44" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="K6" s="44"/>
     </row>
@@ -4481,16 +4459,16 @@
         <v>45</v>
       </c>
       <c r="J2" s="44" t="s">
-        <v>572</v>
+        <v>625</v>
       </c>
       <c r="K2" s="44" t="s">
-        <v>509</v>
+        <v>626</v>
       </c>
       <c r="L2" s="44" t="s">
         <v>207</v>
       </c>
       <c r="M2" s="44" t="s">
-        <v>510</v>
+        <v>627</v>
       </c>
       <c r="N2" s="44" t="s">
         <v>208</v>
@@ -4499,13 +4477,13 @@
         <v>12</v>
       </c>
       <c r="P2" s="44" t="s">
-        <v>511</v>
+        <v>628</v>
       </c>
       <c r="Q2" s="44" t="s">
         <v>62</v>
       </c>
       <c r="R2" s="44" t="s">
-        <v>512</v>
+        <v>629</v>
       </c>
       <c r="S2" s="44" t="s">
         <v>12</v>
@@ -4551,16 +4529,16 @@
         <v>45</v>
       </c>
       <c r="J3" s="44" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="L3" s="44" t="s">
         <v>207</v>
       </c>
       <c r="M3" s="44" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="N3" s="44" t="s">
         <v>208</v>
@@ -4569,13 +4547,13 @@
         <v>12</v>
       </c>
       <c r="P3" s="44" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="Q3" s="44" t="s">
         <v>239</v>
       </c>
       <c r="R3" s="44" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="S3" s="44" t="s">
         <v>12</v>
@@ -4629,16 +4607,16 @@
       <c r="H4" s="44"/>
       <c r="I4" s="44"/>
       <c r="J4" s="44" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="K4" s="44" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="L4" s="44" t="s">
         <v>328</v>
       </c>
       <c r="M4" s="44" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="N4" s="44" t="s">
         <v>209</v>
@@ -4681,16 +4659,16 @@
       <c r="H5" s="44"/>
       <c r="I5" s="44"/>
       <c r="J5" s="44" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="L5" s="44" t="s">
         <v>328</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="N5" s="44" t="s">
         <v>209</v>
@@ -4741,16 +4719,16 @@
         <v>45</v>
       </c>
       <c r="J6" s="44" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="K6" s="44" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="L6" s="44" t="s">
         <v>207</v>
       </c>
       <c r="M6" s="44" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="N6" s="44" t="s">
         <v>208</v>
@@ -5792,16 +5770,16 @@
       <c r="I2" s="44"/>
       <c r="J2" s="44"/>
       <c r="K2" s="44" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>325</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>209</v>
@@ -5856,7 +5834,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>312</v>
@@ -5996,16 +5974,16 @@
         <v>2</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>325</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>209</v>
@@ -6014,7 +5992,7 @@
         <v>12</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="R5" s="15" t="s">
         <v>44</v>
@@ -6533,16 +6511,16 @@
       <c r="U2" s="44"/>
       <c r="V2" s="44"/>
       <c r="W2" s="44" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="X2" s="44" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="Y2" s="44" t="s">
         <v>325</v>
       </c>
       <c r="Z2" s="44" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="AA2" s="44" t="s">
         <v>209</v>
@@ -6551,7 +6529,7 @@
         <v>12</v>
       </c>
       <c r="AC2" s="44" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
     <row r="3" spans="1:29">
@@ -6669,16 +6647,16 @@
       <c r="U4" s="44"/>
       <c r="V4" s="44"/>
       <c r="W4" s="44" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="X4" s="44" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="Y4" s="44" t="s">
         <v>325</v>
       </c>
       <c r="Z4" s="44" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="AA4" s="44" t="s">
         <v>209</v>
@@ -6687,7 +6665,7 @@
         <v>12</v>
       </c>
       <c r="AC4" s="44" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
     </row>
   </sheetData>
@@ -6881,7 +6859,7 @@
       <c r="E1" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="65" t="s">
+      <c r="F1" s="64" t="s">
         <v>142</v>
       </c>
       <c r="G1" s="58" t="s">
@@ -6945,16 +6923,16 @@
       <c r="I2" s="44"/>
       <c r="J2" s="44"/>
       <c r="K2" s="44" t="s">
-        <v>626</v>
+        <v>613</v>
       </c>
       <c r="L2" s="44" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="M2" s="44" t="s">
         <v>18</v>
       </c>
       <c r="N2" s="44" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="O2" s="44" t="s">
         <v>12</v>
@@ -6963,7 +6941,7 @@
         <v>13</v>
       </c>
       <c r="Q2" s="44" t="s">
-        <v>627</v>
+        <v>614</v>
       </c>
       <c r="R2" s="44"/>
     </row>
@@ -6991,16 +6969,16 @@
       <c r="I3" s="44"/>
       <c r="J3" s="44"/>
       <c r="K3" s="44" t="s">
-        <v>637</v>
+        <v>620</v>
       </c>
       <c r="L3" s="44" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="M3" s="44" t="s">
         <v>18</v>
       </c>
       <c r="N3" s="44" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="O3" s="44" t="s">
         <v>12</v>
@@ -7009,10 +6987,10 @@
         <v>13</v>
       </c>
       <c r="Q3" s="44" t="s">
-        <v>638</v>
+        <v>621</v>
       </c>
       <c r="R3" s="44" t="s">
-        <v>639</v>
+        <v>622</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -7047,16 +7025,16 @@
         <v>2</v>
       </c>
       <c r="K4" s="44" t="s">
-        <v>631</v>
+        <v>615</v>
       </c>
       <c r="L4" s="44" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="M4" s="44" t="s">
         <v>18</v>
       </c>
       <c r="N4" s="44" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="O4" s="44" t="s">
         <v>12</v>
@@ -7065,7 +7043,7 @@
         <v>13</v>
       </c>
       <c r="Q4" s="44" t="s">
-        <v>641</v>
+        <v>623</v>
       </c>
       <c r="R4" s="44"/>
     </row>
@@ -7093,16 +7071,16 @@
       <c r="I5" s="44"/>
       <c r="J5" s="44"/>
       <c r="K5" s="44" t="s">
-        <v>633</v>
+        <v>616</v>
       </c>
       <c r="L5" s="44" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="M5" s="44" t="s">
         <v>18</v>
       </c>
       <c r="N5" s="44" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="O5" s="44" t="s">
         <v>12</v>
@@ -7111,7 +7089,7 @@
         <v>13</v>
       </c>
       <c r="Q5" s="44" t="s">
-        <v>634</v>
+        <v>617</v>
       </c>
       <c r="R5" s="44"/>
     </row>
@@ -7139,16 +7117,16 @@
       <c r="I6" s="44"/>
       <c r="J6" s="44"/>
       <c r="K6" s="44" t="s">
-        <v>635</v>
+        <v>618</v>
       </c>
       <c r="L6" s="44" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="M6" s="44" t="s">
         <v>18</v>
       </c>
       <c r="N6" s="44" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="O6" s="44" t="s">
         <v>12</v>
@@ -7157,7 +7135,7 @@
         <v>13</v>
       </c>
       <c r="Q6" s="44" t="s">
-        <v>636</v>
+        <v>619</v>
       </c>
       <c r="R6" s="44"/>
     </row>
@@ -7292,16 +7270,16 @@
         <v>163</v>
       </c>
       <c r="J2" s="56" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="K2" s="44" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>215</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>12</v>
@@ -7310,13 +7288,13 @@
         <v>216</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>217</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>216</v>
@@ -7325,7 +7303,7 @@
         <v>163</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -7357,16 +7335,16 @@
         <v>163</v>
       </c>
       <c r="J3" s="56" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>215</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>12</v>
@@ -7375,13 +7353,13 @@
         <v>216</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="Q3" s="3" t="s">
         <v>341</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>216</v>
@@ -7390,7 +7368,7 @@
         <v>163</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -7586,7 +7564,7 @@
       <c r="A2" s="44" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="44" t="s">
         <v>87</v>
       </c>
     </row>
@@ -7594,15 +7572,15 @@
       <c r="A3" s="44" t="s">
         <v>181</v>
       </c>
-      <c r="B3" s="64" t="s">
-        <v>506</v>
+      <c r="B3" s="47" t="s">
+        <v>504</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="44" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="44" t="s">
         <v>182</v>
       </c>
     </row>
@@ -7726,7 +7704,7 @@
         <v>473</v>
       </c>
       <c r="J1" s="63" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="K1" s="42" t="s">
         <v>470</v>
@@ -7735,10 +7713,10 @@
         <v>471</v>
       </c>
       <c r="M1" s="42" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="N1" s="42" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -7767,22 +7745,22 @@
         <v>474</v>
       </c>
       <c r="I2" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J2" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K2" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L2" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M2" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N2" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -7799,7 +7777,7 @@
         <v>121</v>
       </c>
       <c r="E3" s="32" t="s">
-        <v>476</v>
+        <v>466</v>
       </c>
       <c r="F3" s="44" t="s">
         <v>475</v>
@@ -7811,22 +7789,22 @@
         <v>474</v>
       </c>
       <c r="I3" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J3" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L3" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M3" s="44" t="s">
-        <v>488</v>
+        <v>501</v>
       </c>
       <c r="N3" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -7855,22 +7833,22 @@
         <v>474</v>
       </c>
       <c r="I4" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J4" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K4" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L4" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M4" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N4" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -7887,34 +7865,34 @@
         <v>121</v>
       </c>
       <c r="E5" s="32" t="s">
+        <v>121</v>
+      </c>
+      <c r="F5" s="44" t="s">
         <v>466</v>
-      </c>
-      <c r="F5" s="44" t="s">
-        <v>477</v>
       </c>
       <c r="G5" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H5" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I5" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J5" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L5" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N5" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -7931,34 +7909,34 @@
         <v>121</v>
       </c>
       <c r="E6" s="44" t="s">
+        <v>121</v>
+      </c>
+      <c r="F6" s="44" t="s">
         <v>466</v>
-      </c>
-      <c r="F6" s="44" t="s">
-        <v>477</v>
       </c>
       <c r="G6" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H6" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I6" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J6" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K6" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L6" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M6" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N6" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -7975,34 +7953,34 @@
         <v>121</v>
       </c>
       <c r="E7" s="44" t="s">
+        <v>121</v>
+      </c>
+      <c r="F7" s="44" t="s">
         <v>466</v>
-      </c>
-      <c r="F7" s="44" t="s">
-        <v>477</v>
       </c>
       <c r="G7" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H7" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I7" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J7" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K7" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L7" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M7" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N7" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -8013,40 +7991,40 @@
         <v>149</v>
       </c>
       <c r="C8" s="44" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D8" s="44" t="s">
         <v>121</v>
       </c>
       <c r="E8" s="44" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="F8" s="44" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="G8" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H8" s="44" t="s">
+        <v>484</v>
+      </c>
+      <c r="I8" s="44" t="s">
         <v>485</v>
       </c>
-      <c r="I8" s="44" t="s">
-        <v>486</v>
-      </c>
       <c r="J8" s="44" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="K8" s="44" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L8" s="44" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="M8" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N8" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -8063,7 +8041,7 @@
         <v>121</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="F9" s="44" t="s">
         <v>476</v>
@@ -8072,25 +8050,25 @@
         <v>338</v>
       </c>
       <c r="H9" s="44" t="s">
+        <v>490</v>
+      </c>
+      <c r="I9" s="44" t="s">
         <v>491</v>
       </c>
-      <c r="I9" s="44" t="s">
+      <c r="J9" s="44" t="s">
         <v>492</v>
       </c>
-      <c r="J9" s="44" t="s">
-        <v>493</v>
-      </c>
       <c r="K9" s="44" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="L9" s="44" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="M9" s="44" t="s">
         <v>428</v>
       </c>
       <c r="N9" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -8107,34 +8085,34 @@
         <v>121</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F10" s="44" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="G10" s="44" t="s">
         <v>338</v>
       </c>
       <c r="H10" s="44" t="s">
+        <v>497</v>
+      </c>
+      <c r="I10" s="44" t="s">
         <v>498</v>
       </c>
-      <c r="I10" s="44" t="s">
+      <c r="J10" s="44" t="s">
         <v>499</v>
       </c>
-      <c r="J10" s="44" t="s">
-        <v>500</v>
-      </c>
       <c r="K10" s="44" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="L10" s="44" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="M10" s="44" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="N10" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -8145,40 +8123,40 @@
         <v>149</v>
       </c>
       <c r="C11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="G11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="H11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N11" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -8189,40 +8167,40 @@
         <v>149</v>
       </c>
       <c r="C12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="G12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N12" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -8233,40 +8211,40 @@
         <v>149</v>
       </c>
       <c r="C13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="G13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="H13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N13" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -8277,37 +8255,37 @@
         <v>149</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D14" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E14" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F14" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="G14" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="H14" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I14" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J14" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K14" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L14" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M14" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N14" s="44" t="s">
         <v>465</v>
@@ -8321,84 +8299,84 @@
         <v>149</v>
       </c>
       <c r="C15" s="44" t="s">
+        <v>501</v>
+      </c>
+      <c r="D15" s="44" t="s">
+        <v>487</v>
+      </c>
+      <c r="E15" s="44" t="s">
+        <v>487</v>
+      </c>
+      <c r="F15" s="44" t="s">
+        <v>487</v>
+      </c>
+      <c r="G15" s="44" t="s">
         <v>502</v>
       </c>
-      <c r="D15" s="44" t="s">
-        <v>488</v>
-      </c>
-      <c r="E15" s="44" t="s">
-        <v>488</v>
-      </c>
-      <c r="F15" s="44" t="s">
-        <v>488</v>
-      </c>
-      <c r="G15" s="44" t="s">
-        <v>503</v>
-      </c>
       <c r="H15" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I15" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J15" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K15" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L15" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M15" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N15" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="32" t="s">
         <v>303</v>
       </c>
-      <c r="B16" s="32" t="s">
-        <v>504</v>
+      <c r="B16" s="44" t="s">
+        <v>149</v>
       </c>
       <c r="C16" s="32" t="s">
         <v>465</v>
       </c>
       <c r="D16" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E16" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F16" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="G16" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="H16" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I16" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J16" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K16" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L16" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M16" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N16" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -8409,40 +8387,40 @@
         <v>149</v>
       </c>
       <c r="C17" s="32" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="D17" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E17" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F17" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="G17" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="H17" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I17" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J17" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K17" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L17" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="M17" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N17" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -8526,10 +8504,10 @@
         <v>50</v>
       </c>
       <c r="H2" s="44" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="I2" s="44" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -8759,7 +8737,7 @@
       <c r="H6" s="44"/>
       <c r="I6" s="44"/>
       <c r="J6" s="44" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="K6" s="44"/>
       <c r="L6" s="44"/>
@@ -8842,7 +8820,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="32" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="G2" s="32">
         <v>2</v>
@@ -8873,7 +8851,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="32" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="G3" s="32"/>
       <c r="H3" s="32"/>
@@ -8902,7 +8880,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="32" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="G4" s="32"/>
       <c r="H4" s="32"/>
@@ -9508,7 +9486,7 @@
       </c>
       <c r="G4" s="44"/>
       <c r="H4" s="44" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="I4" s="44" t="s">
         <v>387</v>
@@ -9545,7 +9523,7 @@
       </c>
       <c r="G5" s="44"/>
       <c r="H5" s="44" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="I5" s="44" t="s">
         <v>387</v>
@@ -10047,7 +10025,7 @@
         <v>212</v>
       </c>
       <c r="J2" s="44" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="K2" s="44">
         <v>2</v>
@@ -10499,7 +10477,7 @@
       <c r="M2" s="32"/>
       <c r="N2" s="32"/>
       <c r="O2" s="32" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="P2" s="32"/>
       <c r="Q2" s="32" t="s">
@@ -10644,7 +10622,7 @@
         <v>15</v>
       </c>
       <c r="H6" s="32" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="I6" s="32" t="s">
         <v>387</v>
@@ -10692,7 +10670,7 @@
         <v>19</v>
       </c>
       <c r="H7" s="32" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="I7" s="32" t="s">
         <v>360</v>
@@ -10810,7 +10788,7 @@
       </c>
       <c r="G10" s="56"/>
       <c r="H10" s="32" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="I10" s="32"/>
       <c r="J10" s="32" t="s">
@@ -10858,7 +10836,7 @@
         <v>15</v>
       </c>
       <c r="H11" s="32" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="I11" s="32" t="s">
         <v>211</v>
@@ -10910,7 +10888,7 @@
       </c>
       <c r="G12" s="56"/>
       <c r="H12" s="32" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="I12" s="32" t="s">
         <v>376</v>
@@ -10998,7 +10976,7 @@
       </c>
       <c r="G14" s="56"/>
       <c r="H14" s="32" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="I14" s="32" t="s">
         <v>244</v>
@@ -11048,7 +11026,7 @@
         <v>15</v>
       </c>
       <c r="H15" s="32" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="I15" s="32" t="s">
         <v>367</v>
@@ -11642,10 +11620,10 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
@@ -11904,10 +11882,10 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="T8" s="3">
         <v>0</v>
@@ -11953,10 +11931,10 @@
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
       <c r="R9" s="3" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="S9" s="3" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="T9" s="3"/>
       <c r="U9" s="3">
@@ -12006,10 +11984,10 @@
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
       <c r="R10" s="3" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
@@ -12232,10 +12210,10 @@
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
       <c r="R16" s="3" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="S16" s="3" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>

</xml_diff>

<commit_message>
Added Availability from Sowmya
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBF081C1-AADE-4AAB-8808-03DBC5730FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{269A1528-C109-44C0-86B6-2AE2597F7E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="27" activeTab="30" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="3" activeTab="7" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2119" uniqueCount="647">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2396" uniqueCount="741">
   <si>
     <t>Scenario</t>
   </si>
@@ -2015,13 +2015,295 @@
   </si>
   <si>
     <t>2302182825352</t>
+  </si>
+  <si>
+    <t>DepartureDate1</t>
+  </si>
+  <si>
+    <t>Origin1</t>
+  </si>
+  <si>
+    <t>Destination1</t>
+  </si>
+  <si>
+    <t>EquipType</t>
+  </si>
+  <si>
+    <t>ConnectionLocation</t>
+  </si>
+  <si>
+    <t>Availability overriding Point Of Sale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combined reward with first available flight search </t>
+  </si>
+  <si>
+    <t>JFK</t>
+  </si>
+  <si>
+    <t>Direct and Nonstop Flights is false, applied to all requests</t>
+  </si>
+  <si>
+    <t>LHR</t>
+  </si>
+  <si>
+    <t>Direct and Nonstop Flights only, applied to all requests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct and Nonstop Flights only, applied to first request </t>
+  </si>
+  <si>
+    <t>Filter by equipment type, all requests</t>
+  </si>
+  <si>
+    <t>752</t>
+  </si>
+  <si>
+    <t>First available flight search, find flights with 2 seats in Q class</t>
+  </si>
+  <si>
+    <t>Get non stop flights only on first request</t>
+  </si>
+  <si>
+    <t>SLC</t>
+  </si>
+  <si>
+    <t>Get non stop flights, all requests</t>
+  </si>
+  <si>
+    <t>Manually constructured connections</t>
+  </si>
+  <si>
+    <t>DEN</t>
+  </si>
+  <si>
+    <t>Max requests exceeded</t>
+  </si>
+  <si>
+    <t>Maximum connections of 1 on all requests</t>
+  </si>
+  <si>
+    <t>Maximum stops of 0, applied to all requests</t>
+  </si>
+  <si>
+    <t>Maximum stops of 0, applied to only to 2nd request</t>
+  </si>
+  <si>
+    <t>Maximum stops of 1, applied to all requests</t>
+  </si>
+  <si>
+    <t>Missing destination location</t>
+  </si>
+  <si>
+    <t>Missing origin location</t>
+  </si>
+  <si>
+    <t>Multiple requests</t>
+  </si>
+  <si>
+    <t>Nonstops on first request, Maximum connections of 1 on second request</t>
+  </si>
+  <si>
+    <t>Online connections only for first request</t>
+  </si>
+  <si>
+    <t>Online connections only, for all requests</t>
+  </si>
+  <si>
+    <t>Regular availability with maximum responses specified</t>
+  </si>
+  <si>
+    <t>Request specific carriers, only first request</t>
+  </si>
+  <si>
+    <t>Traffic restriction in availability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Untruncated Availability </t>
+  </si>
+  <si>
+    <t>Seg1Pax1SeatNum</t>
+  </si>
+  <si>
+    <t>Seg2Pax1SeatNum</t>
+  </si>
+  <si>
+    <t>Seg1Pax2SeatNum</t>
+  </si>
+  <si>
+    <t>Seg2Pax2SeatNum</t>
+  </si>
+  <si>
+    <t>CreateBooking with 2segm, 2pax (1 FF), stored fare, 2 phones, 1 remark and ticketing</t>
+  </si>
+  <si>
+    <t>BAYOBS</t>
+  </si>
+  <si>
+    <t>CreateBbooking with 4seg, 2pax, stored fare, 2phones,1remark, 2OSIs, 2SSRs and ticketing</t>
+  </si>
+  <si>
+    <t>478</t>
+  </si>
+  <si>
+    <t>435</t>
+  </si>
+  <si>
+    <t>BAYOBT</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CreateBooking with 4seg(OA), 2pax (1FF and 1inf), 1email, stored fare, 1OSI, 1remark, SeatAssignment and ticketing</t>
+  </si>
+  <si>
+    <t>2217</t>
+  </si>
+  <si>
+    <t>2362</t>
+  </si>
+  <si>
+    <t>ORD</t>
+  </si>
+  <si>
+    <t>2311</t>
+  </si>
+  <si>
+    <t>1916</t>
+  </si>
+  <si>
+    <t>BAYOBY</t>
+  </si>
+  <si>
+    <t>CreateBooking with 3 seg(1ARNK),2pax(1FF),stored fare,2phones,1OSI,3remarks,SeatAssignment and ticketing</t>
+  </si>
+  <si>
+    <t>BAYOCO</t>
+  </si>
+  <si>
+    <t>10A</t>
+  </si>
+  <si>
+    <t>10B</t>
+  </si>
+  <si>
+    <t>Check_for_invalid_AirItinerary_in_request</t>
+  </si>
+  <si>
+    <t>Check for invalid AirTraveler in request</t>
+  </si>
+  <si>
+    <t>CreateBooking_Failure_in_one_of_the_components_of_the_system_SDS_unavailable_or_SHARES_unreachable</t>
+  </si>
+  <si>
+    <t>BAYOCY</t>
+  </si>
+  <si>
+    <t>Invalid information specified in AirItinerary</t>
+  </si>
+  <si>
+    <t>9999</t>
+  </si>
+  <si>
+    <t>Invalid information specified in AirTraveler</t>
+  </si>
+  <si>
+    <t>12C</t>
+  </si>
+  <si>
+    <t>12D</t>
+  </si>
+  <si>
+    <t>Invalid information specified in PriceInfo</t>
+  </si>
+  <si>
+    <t>CreateBooking with 1 seg, 1 pax, stored fare (base fare, NVA date, fare calculation line, BA and tour code) and TL</t>
+  </si>
+  <si>
+    <t>BAYODL</t>
+  </si>
+  <si>
+    <t>Bundled segment - Invalid information in one segment</t>
+  </si>
+  <si>
+    <t>137</t>
+  </si>
+  <si>
+    <t>335</t>
+  </si>
+  <si>
+    <t>Stored fare - Ticketing item  Invalid tour code</t>
+  </si>
+  <si>
+    <t>BAYODT</t>
+  </si>
+  <si>
+    <t>Stored fare - Ticketing item Invalid original issued info</t>
+  </si>
+  <si>
+    <t>BAYODY</t>
+  </si>
+  <si>
+    <t>Stored fare - Ticketing item Invalid bankers rate info</t>
+  </si>
+  <si>
+    <t>BAYOEB</t>
+  </si>
+  <si>
+    <t>Stored fare - Ticketing item Invalid remark</t>
+  </si>
+  <si>
+    <t>BAYOEH</t>
+  </si>
+  <si>
+    <t>Stored fare - Ticketing item Invalid original origin destination city</t>
+  </si>
+  <si>
+    <t>BAYOEN</t>
+  </si>
+  <si>
+    <t>Stored fare - Ticketing item Invalid form of payment</t>
+  </si>
+  <si>
+    <t>BAYOEZ</t>
+  </si>
+  <si>
+    <t>Stored fare - Ticketing item No form of payment</t>
+  </si>
+  <si>
+    <t>BAYOFE</t>
+  </si>
+  <si>
+    <t>Stored fare - Ticketing item too long remark</t>
+  </si>
+  <si>
+    <t>BAYOFS</t>
+  </si>
+  <si>
+    <t>Create a booking with 1 segment, 1 passenger, stored fare, ticketing and place it on queue</t>
+  </si>
+  <si>
+    <t>BAYOFT</t>
+  </si>
+  <si>
+    <t>CreateBooking_with_1seg_1pax_storedfare_FBC_base_fare_fare_calculation_line_and_issue_in_exchange_without_coupons_and_TL</t>
+  </si>
+  <si>
+    <t>BAYOFY</t>
+  </si>
+  <si>
+    <t>82</t>
+  </si>
+  <si>
+    <t>481</t>
+  </si>
+  <si>
+    <t>333</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2106,6 +2388,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color theme="1"/>
+      <name val="JetBrains Mono"/>
     </font>
   </fonts>
   <fills count="11">
@@ -2256,7 +2543,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2358,6 +2645,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10381,7 +10678,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
@@ -10389,9 +10686,10 @@
     <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:10">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -10407,9 +10705,24 @@
       <c r="E1" s="12" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="6" t="s">
+      <c r="F1" s="45" t="s">
+        <v>647</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>648</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>649</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>650</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="67" t="s">
         <v>54</v>
       </c>
       <c r="B2" s="44">
@@ -10424,9 +10737,14 @@
       <c r="E2" s="44" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="6" t="s">
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="67" t="s">
         <v>55</v>
       </c>
       <c r="B3" s="44">
@@ -10441,6 +10759,601 @@
       <c r="E3" s="44" t="s">
         <v>12</v>
       </c>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="44" t="s">
+        <v>652</v>
+      </c>
+      <c r="B4" s="44">
+        <v>1</v>
+      </c>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="44"/>
+      <c r="G4" s="44"/>
+      <c r="H4" s="44"/>
+      <c r="I4" s="44"/>
+      <c r="J4" s="44"/>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="44" t="s">
+        <v>653</v>
+      </c>
+      <c r="B5" s="44">
+        <v>1</v>
+      </c>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="44" t="s">
+        <v>654</v>
+      </c>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="44" t="s">
+        <v>655</v>
+      </c>
+      <c r="B6" s="44">
+        <v>1</v>
+      </c>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="F6" s="44">
+        <v>2</v>
+      </c>
+      <c r="G6" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="H6" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="44"/>
+      <c r="J6" s="44"/>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="44" t="s">
+        <v>657</v>
+      </c>
+      <c r="B7" s="44">
+        <v>1</v>
+      </c>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="F7" s="44">
+        <v>2</v>
+      </c>
+      <c r="G7" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="H7" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="44" t="s">
+        <v>658</v>
+      </c>
+      <c r="B8" s="44">
+        <v>1</v>
+      </c>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="F8" s="44">
+        <v>2</v>
+      </c>
+      <c r="G8" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="H8" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="44" t="s">
+        <v>659</v>
+      </c>
+      <c r="B9" s="44">
+        <v>1</v>
+      </c>
+      <c r="C9" s="44"/>
+      <c r="D9" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="44" t="s">
+        <v>654</v>
+      </c>
+      <c r="F9" s="44">
+        <v>2</v>
+      </c>
+      <c r="G9" s="44" t="s">
+        <v>654</v>
+      </c>
+      <c r="H9" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" s="47" t="s">
+        <v>660</v>
+      </c>
+      <c r="J9" s="44"/>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="44" t="s">
+        <v>661</v>
+      </c>
+      <c r="B10" s="44">
+        <v>1</v>
+      </c>
+      <c r="C10" s="44"/>
+      <c r="D10" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="44" t="s">
+        <v>654</v>
+      </c>
+      <c r="F10" s="44"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="44"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="44" t="s">
+        <v>662</v>
+      </c>
+      <c r="B11" s="44">
+        <v>1</v>
+      </c>
+      <c r="C11" s="44"/>
+      <c r="D11" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="44" t="s">
+        <v>663</v>
+      </c>
+      <c r="F11" s="44">
+        <v>2</v>
+      </c>
+      <c r="G11" s="44" t="s">
+        <v>663</v>
+      </c>
+      <c r="H11" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="44" t="s">
+        <v>664</v>
+      </c>
+      <c r="B12" s="44">
+        <v>1</v>
+      </c>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="44" t="s">
+        <v>663</v>
+      </c>
+      <c r="F12" s="44">
+        <v>2</v>
+      </c>
+      <c r="G12" s="44" t="s">
+        <v>663</v>
+      </c>
+      <c r="H12" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I12" s="44"/>
+      <c r="J12" s="44"/>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="44" t="s">
+        <v>665</v>
+      </c>
+      <c r="B13" s="44">
+        <v>1</v>
+      </c>
+      <c r="C13" s="44"/>
+      <c r="D13" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="44" t="s">
+        <v>666</v>
+      </c>
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="44" t="s">
+        <v>667</v>
+      </c>
+      <c r="B14" s="44">
+        <v>1</v>
+      </c>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="44" t="s">
+        <v>666</v>
+      </c>
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="44" t="s">
+        <v>668</v>
+      </c>
+      <c r="B15" s="44">
+        <v>1</v>
+      </c>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="F15" s="44">
+        <v>2</v>
+      </c>
+      <c r="G15" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="H15" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" s="44" t="s">
+        <v>669</v>
+      </c>
+      <c r="B16" s="44">
+        <v>1</v>
+      </c>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="44" t="s">
+        <v>663</v>
+      </c>
+      <c r="F16" s="44">
+        <v>2</v>
+      </c>
+      <c r="G16" s="44" t="s">
+        <v>663</v>
+      </c>
+      <c r="H16" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I16" s="44"/>
+      <c r="J16" s="44"/>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="A17" s="44" t="s">
+        <v>670</v>
+      </c>
+      <c r="B17" s="44">
+        <v>1</v>
+      </c>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="44" t="s">
+        <v>663</v>
+      </c>
+      <c r="F17" s="44">
+        <v>2</v>
+      </c>
+      <c r="G17" s="44" t="s">
+        <v>663</v>
+      </c>
+      <c r="H17" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I17" s="44"/>
+      <c r="J17" s="44"/>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" s="44" t="s">
+        <v>671</v>
+      </c>
+      <c r="B18" s="44">
+        <v>1</v>
+      </c>
+      <c r="C18" s="44"/>
+      <c r="D18" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="44" t="s">
+        <v>663</v>
+      </c>
+      <c r="F18" s="44">
+        <v>2</v>
+      </c>
+      <c r="G18" s="44" t="s">
+        <v>663</v>
+      </c>
+      <c r="H18" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I18" s="44"/>
+      <c r="J18" s="44"/>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" s="44" t="s">
+        <v>672</v>
+      </c>
+      <c r="B19" s="44">
+        <v>1</v>
+      </c>
+      <c r="C19" s="44"/>
+      <c r="D19" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19" s="44"/>
+      <c r="F19" s="44"/>
+      <c r="G19" s="44"/>
+      <c r="H19" s="44"/>
+      <c r="I19" s="44"/>
+      <c r="J19" s="44"/>
+    </row>
+    <row r="20" spans="1:10">
+      <c r="A20" s="44" t="s">
+        <v>673</v>
+      </c>
+      <c r="B20" s="44">
+        <v>1</v>
+      </c>
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="44" t="s">
+        <v>666</v>
+      </c>
+      <c r="F20" s="44"/>
+      <c r="G20" s="44"/>
+      <c r="H20" s="44"/>
+      <c r="I20" s="44"/>
+      <c r="J20" s="44"/>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" s="44" t="s">
+        <v>674</v>
+      </c>
+      <c r="B21" s="44">
+        <v>1</v>
+      </c>
+      <c r="C21" s="44"/>
+      <c r="D21" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="44" t="s">
+        <v>666</v>
+      </c>
+      <c r="F21" s="44">
+        <v>2</v>
+      </c>
+      <c r="G21" s="44" t="s">
+        <v>666</v>
+      </c>
+      <c r="H21" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I21" s="44"/>
+      <c r="J21" s="44"/>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="A22" s="44" t="s">
+        <v>675</v>
+      </c>
+      <c r="B22" s="44">
+        <v>1</v>
+      </c>
+      <c r="C22" s="44"/>
+      <c r="D22" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="F22" s="44">
+        <v>2</v>
+      </c>
+      <c r="G22" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="H22" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I22" s="44"/>
+      <c r="J22" s="44"/>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" s="44" t="s">
+        <v>676</v>
+      </c>
+      <c r="B23" s="44">
+        <v>1</v>
+      </c>
+      <c r="C23" s="44"/>
+      <c r="D23" s="44" t="s">
+        <v>654</v>
+      </c>
+      <c r="E23" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="F23" s="44">
+        <v>2</v>
+      </c>
+      <c r="G23" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="H23" s="44" t="s">
+        <v>654</v>
+      </c>
+      <c r="I23" s="44"/>
+      <c r="J23" s="44"/>
+    </row>
+    <row r="24" spans="1:10">
+      <c r="A24" s="44" t="s">
+        <v>677</v>
+      </c>
+      <c r="B24" s="44">
+        <v>1</v>
+      </c>
+      <c r="C24" s="44"/>
+      <c r="D24" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="E24" s="44" t="s">
+        <v>654</v>
+      </c>
+      <c r="F24" s="44">
+        <v>2</v>
+      </c>
+      <c r="G24" s="44" t="s">
+        <v>654</v>
+      </c>
+      <c r="H24" s="44" t="s">
+        <v>656</v>
+      </c>
+      <c r="I24" s="44"/>
+      <c r="J24" s="44"/>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" s="44" t="s">
+        <v>678</v>
+      </c>
+      <c r="B25" s="44">
+        <v>1</v>
+      </c>
+      <c r="C25" s="44"/>
+      <c r="D25" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E25" s="44" t="s">
+        <v>666</v>
+      </c>
+      <c r="F25" s="44"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="44"/>
+      <c r="I25" s="44"/>
+      <c r="J25" s="44"/>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="44" t="s">
+        <v>679</v>
+      </c>
+      <c r="B26" s="44">
+        <v>1</v>
+      </c>
+      <c r="C26" s="44"/>
+      <c r="D26" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E26" s="44" t="s">
+        <v>654</v>
+      </c>
+      <c r="F26" s="44">
+        <v>2</v>
+      </c>
+      <c r="G26" s="44" t="s">
+        <v>654</v>
+      </c>
+      <c r="H26" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I26" s="44"/>
+      <c r="J26" s="44"/>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" s="44" t="s">
+        <v>680</v>
+      </c>
+      <c r="B27" s="44">
+        <v>1</v>
+      </c>
+      <c r="C27" s="44"/>
+      <c r="D27" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E27" s="44" t="s">
+        <v>208</v>
+      </c>
+      <c r="F27" s="44"/>
+      <c r="G27" s="44"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="44"/>
+      <c r="J27" s="44"/>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" s="44" t="s">
+        <v>681</v>
+      </c>
+      <c r="B28" s="44">
+        <v>1</v>
+      </c>
+      <c r="C28" s="44"/>
+      <c r="D28" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E28" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" s="44"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="44"/>
+      <c r="I28" s="44"/>
+      <c r="J28" s="44"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11745,22 +12658,23 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:W17"/>
+  <dimension ref="A1:AJ39"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="54.36328125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="13.90625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="5" t="s">
+    <row r="1" spans="1:36">
+      <c r="A1" s="45" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="45" t="s">
         <v>28</v>
       </c>
       <c r="D1" s="12" t="s">
@@ -11769,10 +12683,10 @@
       <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="5" t="s">
+      <c r="F1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="45" t="s">
         <v>28</v>
       </c>
       <c r="H1" s="12" t="s">
@@ -11781,10 +12695,10 @@
       <c r="I1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="K1" s="5" t="s">
+      <c r="J1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="45" t="s">
         <v>28</v>
       </c>
       <c r="L1" s="12" t="s">
@@ -11793,10 +12707,10 @@
       <c r="M1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="O1" s="5" t="s">
+      <c r="N1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="O1" s="45" t="s">
         <v>28</v>
       </c>
       <c r="P1" s="12" t="s">
@@ -11811,28 +12725,67 @@
       <c r="S1" s="23" t="s">
         <v>195</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="45" t="s">
         <v>142</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="45" t="s">
         <v>206</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="45" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="2" spans="1:23">
-      <c r="A2" s="6" t="s">
+      <c r="X1" s="45" t="s">
+        <v>682</v>
+      </c>
+      <c r="Y1" s="45" t="s">
+        <v>683</v>
+      </c>
+      <c r="Z1" s="45" t="s">
+        <v>684</v>
+      </c>
+      <c r="AA1" s="45" t="s">
+        <v>685</v>
+      </c>
+      <c r="AB1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC1" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE1" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="AG1" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="AH1" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI1" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="AJ1" s="12" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36">
+      <c r="A2" s="67" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="17">
+      <c r="B2" s="69">
         <v>1</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>194</v>
+        <v>739</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>13</v>
@@ -11840,38 +12793,51 @@
       <c r="E2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3" t="s">
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
+      <c r="Q2" s="44"/>
+      <c r="R2" s="44" t="s">
         <v>507</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="S2" s="44" t="s">
         <v>508</v>
       </c>
-      <c r="T2" s="3"/>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
-      <c r="W2" s="3"/>
-    </row>
-    <row r="3" spans="1:23">
-      <c r="A3" s="6" t="s">
+      <c r="T2" s="44"/>
+      <c r="U2" s="44"/>
+      <c r="V2" s="44"/>
+      <c r="W2" s="44"/>
+      <c r="X2" s="44"/>
+      <c r="Y2" s="44"/>
+      <c r="Z2" s="44"/>
+      <c r="AA2" s="44"/>
+      <c r="AB2" s="44"/>
+      <c r="AC2" s="44"/>
+      <c r="AD2" s="44"/>
+      <c r="AE2" s="44"/>
+      <c r="AF2" s="44"/>
+      <c r="AG2" s="44"/>
+      <c r="AH2" s="44"/>
+      <c r="AI2" s="44"/>
+      <c r="AJ2" s="44"/>
+    </row>
+    <row r="3" spans="1:36">
+      <c r="A3" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="17">
+      <c r="B3" s="69">
         <v>1</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>194</v>
+        <v>740</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>13</v>
@@ -11879,58 +12845,71 @@
       <c r="E3" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="44">
         <v>2</v>
       </c>
       <c r="G3" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" s="3" t="s">
+      <c r="H3" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3" s="44">
         <v>3</v>
       </c>
-      <c r="K3" s="15" t="s">
+      <c r="K3" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="M3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="N3" s="3">
+      <c r="M3" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="N3" s="44">
         <v>4</v>
       </c>
-      <c r="O3" s="15" t="s">
+      <c r="O3" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="P3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q3" s="3" t="s">
+      <c r="P3" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q3" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3"/>
-      <c r="V3" s="3"/>
-      <c r="W3" s="3"/>
-    </row>
-    <row r="4" spans="1:23">
-      <c r="A4" s="6" t="s">
+      <c r="R3" s="44"/>
+      <c r="S3" s="44"/>
+      <c r="T3" s="44"/>
+      <c r="U3" s="44"/>
+      <c r="V3" s="44"/>
+      <c r="W3" s="44"/>
+      <c r="X3" s="44"/>
+      <c r="Y3" s="44"/>
+      <c r="Z3" s="44"/>
+      <c r="AA3" s="44"/>
+      <c r="AB3" s="44"/>
+      <c r="AC3" s="44"/>
+      <c r="AD3" s="44"/>
+      <c r="AE3" s="44"/>
+      <c r="AF3" s="44"/>
+      <c r="AG3" s="44"/>
+      <c r="AH3" s="44"/>
+      <c r="AI3" s="44"/>
+      <c r="AJ3" s="44"/>
+    </row>
+    <row r="4" spans="1:36">
+      <c r="A4" s="67" t="s">
         <v>65</v>
       </c>
-      <c r="B4" s="17">
+      <c r="B4" s="69">
         <v>1</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>194</v>
+        <v>740</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>13</v>
@@ -11938,159 +12917,211 @@
       <c r="E4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="44">
         <v>2</v>
       </c>
       <c r="G4" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="3" t="s">
+      <c r="H4" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="44">
         <v>3</v>
       </c>
-      <c r="K4" s="15" t="s">
+      <c r="K4" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="M4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="N4" s="3">
+      <c r="M4" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="N4" s="44">
         <v>4</v>
       </c>
-      <c r="O4" s="15" t="s">
+      <c r="O4" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="P4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q4" s="3" t="s">
+      <c r="P4" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q4" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-    </row>
-    <row r="5" spans="1:23">
-      <c r="A5" s="24" t="s">
+      <c r="R4" s="44"/>
+      <c r="S4" s="44"/>
+      <c r="T4" s="44"/>
+      <c r="U4" s="44"/>
+      <c r="V4" s="44"/>
+      <c r="W4" s="44"/>
+      <c r="X4" s="44"/>
+      <c r="Y4" s="44"/>
+      <c r="Z4" s="44"/>
+      <c r="AA4" s="44"/>
+      <c r="AB4" s="44"/>
+      <c r="AC4" s="44"/>
+      <c r="AD4" s="44"/>
+      <c r="AE4" s="44"/>
+      <c r="AF4" s="44"/>
+      <c r="AG4" s="44"/>
+      <c r="AH4" s="44"/>
+      <c r="AI4" s="44"/>
+      <c r="AJ4" s="44"/>
+    </row>
+    <row r="5" spans="1:36">
+      <c r="A5" s="68" t="s">
         <v>191</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="70">
         <v>2</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="47" t="s">
         <v>189</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="3" t="s">
+      <c r="D5" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
-    </row>
-    <row r="6" spans="1:23">
-      <c r="A6" s="24" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="44"/>
+      <c r="M5" s="44"/>
+      <c r="N5" s="44"/>
+      <c r="O5" s="44"/>
+      <c r="P5" s="44"/>
+      <c r="Q5" s="44"/>
+      <c r="R5" s="44"/>
+      <c r="S5" s="44"/>
+      <c r="T5" s="44"/>
+      <c r="U5" s="44"/>
+      <c r="V5" s="44"/>
+      <c r="W5" s="44"/>
+      <c r="X5" s="44"/>
+      <c r="Y5" s="44"/>
+      <c r="Z5" s="44"/>
+      <c r="AA5" s="44"/>
+      <c r="AB5" s="44"/>
+      <c r="AC5" s="44"/>
+      <c r="AD5" s="44"/>
+      <c r="AE5" s="44"/>
+      <c r="AF5" s="44"/>
+      <c r="AG5" s="44"/>
+      <c r="AH5" s="44"/>
+      <c r="AI5" s="44"/>
+      <c r="AJ5" s="44"/>
+    </row>
+    <row r="6" spans="1:36">
+      <c r="A6" s="68" t="s">
         <v>192</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="70">
         <v>2</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="47" t="s">
         <v>189</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="D6" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
-      <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
-      <c r="W6" s="3"/>
-    </row>
-    <row r="7" spans="1:23">
-      <c r="A7" s="24" t="s">
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="44"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="44"/>
+      <c r="L6" s="44"/>
+      <c r="M6" s="44"/>
+      <c r="N6" s="44"/>
+      <c r="O6" s="44"/>
+      <c r="P6" s="44"/>
+      <c r="Q6" s="44"/>
+      <c r="R6" s="44"/>
+      <c r="S6" s="44"/>
+      <c r="T6" s="44"/>
+      <c r="U6" s="44"/>
+      <c r="V6" s="44"/>
+      <c r="W6" s="44"/>
+      <c r="X6" s="44"/>
+      <c r="Y6" s="44"/>
+      <c r="Z6" s="44"/>
+      <c r="AA6" s="44"/>
+      <c r="AB6" s="44"/>
+      <c r="AC6" s="44"/>
+      <c r="AD6" s="44"/>
+      <c r="AE6" s="44"/>
+      <c r="AF6" s="44"/>
+      <c r="AG6" s="44"/>
+      <c r="AH6" s="44"/>
+      <c r="AI6" s="44"/>
+      <c r="AJ6" s="44"/>
+    </row>
+    <row r="7" spans="1:36">
+      <c r="A7" s="68" t="s">
         <v>193</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="70">
         <v>2</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="47" t="s">
         <v>189</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="3" t="s">
+      <c r="D7" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="3"/>
-    </row>
-    <row r="8" spans="1:23">
-      <c r="A8" s="24" t="s">
+      <c r="F7" s="44"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="44"/>
+      <c r="M7" s="44"/>
+      <c r="N7" s="44"/>
+      <c r="O7" s="44"/>
+      <c r="P7" s="44"/>
+      <c r="Q7" s="44"/>
+      <c r="R7" s="44"/>
+      <c r="S7" s="44"/>
+      <c r="T7" s="44"/>
+      <c r="U7" s="44"/>
+      <c r="V7" s="44"/>
+      <c r="W7" s="44"/>
+      <c r="X7" s="44"/>
+      <c r="Y7" s="44"/>
+      <c r="Z7" s="44"/>
+      <c r="AA7" s="44"/>
+      <c r="AB7" s="44"/>
+      <c r="AC7" s="44"/>
+      <c r="AD7" s="44"/>
+      <c r="AE7" s="44"/>
+      <c r="AF7" s="44"/>
+      <c r="AG7" s="44"/>
+      <c r="AH7" s="44"/>
+      <c r="AI7" s="44"/>
+      <c r="AJ7" s="44"/>
+    </row>
+    <row r="8" spans="1:36">
+      <c r="A8" s="68" t="s">
         <v>196</v>
       </c>
-      <c r="B8" s="17">
+      <c r="B8" s="69">
         <v>1</v>
       </c>
       <c r="C8" s="16" t="s">
@@ -12102,136 +13133,175 @@
       <c r="E8" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="3" t="s">
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44"/>
+      <c r="M8" s="44"/>
+      <c r="N8" s="44"/>
+      <c r="O8" s="44"/>
+      <c r="P8" s="44"/>
+      <c r="Q8" s="44"/>
+      <c r="R8" s="44" t="s">
         <v>511</v>
       </c>
-      <c r="S8" s="3" t="s">
+      <c r="S8" s="44" t="s">
         <v>512</v>
       </c>
-      <c r="T8" s="3">
-        <v>0</v>
-      </c>
-      <c r="U8" s="3"/>
-      <c r="V8" s="3"/>
-      <c r="W8" s="3"/>
-    </row>
-    <row r="9" spans="1:23">
-      <c r="A9" s="24" t="s">
+      <c r="T8" s="44">
+        <v>0</v>
+      </c>
+      <c r="U8" s="44"/>
+      <c r="V8" s="44"/>
+      <c r="W8" s="44"/>
+      <c r="X8" s="44"/>
+      <c r="Y8" s="44"/>
+      <c r="Z8" s="44"/>
+      <c r="AA8" s="44"/>
+      <c r="AB8" s="44"/>
+      <c r="AC8" s="44"/>
+      <c r="AD8" s="44"/>
+      <c r="AE8" s="44"/>
+      <c r="AF8" s="44"/>
+      <c r="AG8" s="44"/>
+      <c r="AH8" s="44"/>
+      <c r="AI8" s="44"/>
+      <c r="AJ8" s="44"/>
+    </row>
+    <row r="9" spans="1:36">
+      <c r="A9" s="68" t="s">
         <v>197</v>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="69">
         <v>2</v>
       </c>
       <c r="C9" s="47" t="s">
         <v>451</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="3" t="s">
+      <c r="D9" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="44" t="s">
         <v>336</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="44">
         <v>3</v>
       </c>
-      <c r="G9" s="34" t="s">
+      <c r="G9" s="47" t="s">
         <v>337</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="44" t="s">
         <v>336</v>
       </c>
-      <c r="I9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="3" t="s">
+      <c r="I9" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="J9" s="44"/>
+      <c r="K9" s="44"/>
+      <c r="L9" s="44"/>
+      <c r="M9" s="44"/>
+      <c r="N9" s="44"/>
+      <c r="O9" s="44"/>
+      <c r="P9" s="44"/>
+      <c r="Q9" s="44"/>
+      <c r="R9" s="44" t="s">
         <v>513</v>
       </c>
-      <c r="S9" s="3" t="s">
+      <c r="S9" s="44" t="s">
         <v>514</v>
       </c>
-      <c r="T9" s="3"/>
-      <c r="U9" s="3">
-        <v>1</v>
-      </c>
-      <c r="V9" s="3">
+      <c r="T9" s="44"/>
+      <c r="U9" s="44">
+        <v>1</v>
+      </c>
+      <c r="V9" s="44">
         <v>6</v>
       </c>
-      <c r="W9" s="3">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23">
-      <c r="A10" s="24" t="s">
+      <c r="W9" s="44">
+        <v>12</v>
+      </c>
+      <c r="X9" s="44"/>
+      <c r="Y9" s="44"/>
+      <c r="Z9" s="44"/>
+      <c r="AA9" s="44"/>
+      <c r="AB9" s="44"/>
+      <c r="AC9" s="44"/>
+      <c r="AD9" s="44"/>
+      <c r="AE9" s="44"/>
+      <c r="AF9" s="44"/>
+      <c r="AG9" s="44"/>
+      <c r="AH9" s="44"/>
+      <c r="AI9" s="44"/>
+      <c r="AJ9" s="44"/>
+    </row>
+    <row r="10" spans="1:36">
+      <c r="A10" s="68" t="s">
         <v>198</v>
       </c>
-      <c r="B10" s="17">
+      <c r="B10" s="69">
         <v>2</v>
       </c>
       <c r="C10" s="47" t="s">
         <v>451</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="3" t="s">
+      <c r="D10" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="44" t="s">
         <v>336</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="44">
         <v>3</v>
       </c>
-      <c r="G10" s="34" t="s">
+      <c r="G10" s="47" t="s">
         <v>337</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="44" t="s">
         <v>336</v>
       </c>
-      <c r="I10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="3" t="s">
+      <c r="I10" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="J10" s="44"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="44"/>
+      <c r="M10" s="44"/>
+      <c r="N10" s="44"/>
+      <c r="O10" s="44"/>
+      <c r="P10" s="44"/>
+      <c r="Q10" s="44"/>
+      <c r="R10" s="44" t="s">
         <v>515</v>
       </c>
-      <c r="S10" s="3" t="s">
+      <c r="S10" s="44" t="s">
         <v>516</v>
       </c>
-      <c r="T10" s="3"/>
-      <c r="U10" s="3"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
-    </row>
-    <row r="11" spans="1:23">
-      <c r="A11" s="24" t="s">
+      <c r="T10" s="44"/>
+      <c r="U10" s="44"/>
+      <c r="V10" s="44"/>
+      <c r="W10" s="44"/>
+      <c r="X10" s="44"/>
+      <c r="Y10" s="44"/>
+      <c r="Z10" s="44"/>
+      <c r="AA10" s="44"/>
+      <c r="AB10" s="44"/>
+      <c r="AC10" s="44"/>
+      <c r="AD10" s="44"/>
+      <c r="AE10" s="44"/>
+      <c r="AF10" s="44"/>
+      <c r="AG10" s="44"/>
+      <c r="AH10" s="44"/>
+      <c r="AI10" s="44"/>
+      <c r="AJ10" s="44"/>
+    </row>
+    <row r="11" spans="1:36">
+      <c r="A11" s="68" t="s">
         <v>199</v>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="69">
         <v>1</v>
       </c>
       <c r="C11" s="16" t="s">
@@ -12243,32 +13313,45 @@
       <c r="E11" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
-      <c r="Q11" s="3"/>
-      <c r="R11" s="3"/>
-      <c r="S11" s="3"/>
-      <c r="T11" s="3">
-        <v>0</v>
-      </c>
-      <c r="U11" s="3"/>
-      <c r="V11" s="3"/>
-      <c r="W11" s="3"/>
-    </row>
-    <row r="12" spans="1:23">
-      <c r="A12" s="24" t="s">
+      <c r="F11" s="44"/>
+      <c r="G11" s="44"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+      <c r="K11" s="44"/>
+      <c r="L11" s="44"/>
+      <c r="M11" s="44"/>
+      <c r="N11" s="44"/>
+      <c r="O11" s="44"/>
+      <c r="P11" s="44"/>
+      <c r="Q11" s="44"/>
+      <c r="R11" s="44"/>
+      <c r="S11" s="44"/>
+      <c r="T11" s="44">
+        <v>0</v>
+      </c>
+      <c r="U11" s="44"/>
+      <c r="V11" s="44"/>
+      <c r="W11" s="44"/>
+      <c r="X11" s="44"/>
+      <c r="Y11" s="44"/>
+      <c r="Z11" s="44"/>
+      <c r="AA11" s="44"/>
+      <c r="AB11" s="44"/>
+      <c r="AC11" s="44"/>
+      <c r="AD11" s="44"/>
+      <c r="AE11" s="44"/>
+      <c r="AF11" s="44"/>
+      <c r="AG11" s="44"/>
+      <c r="AH11" s="44"/>
+      <c r="AI11" s="44"/>
+      <c r="AJ11" s="44"/>
+    </row>
+    <row r="12" spans="1:36">
+      <c r="A12" s="68" t="s">
         <v>200</v>
       </c>
-      <c r="B12" s="17">
+      <c r="B12" s="69">
         <v>1</v>
       </c>
       <c r="C12" s="16" t="s">
@@ -12280,30 +13363,43 @@
       <c r="E12" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="3"/>
-      <c r="R12" s="3"/>
-      <c r="S12" s="3"/>
-      <c r="T12" s="3"/>
-      <c r="U12" s="3"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="3"/>
-    </row>
-    <row r="13" spans="1:23">
-      <c r="A13" s="24" t="s">
+      <c r="F12" s="44"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="44"/>
+      <c r="L12" s="44"/>
+      <c r="M12" s="44"/>
+      <c r="N12" s="44"/>
+      <c r="O12" s="44"/>
+      <c r="P12" s="44"/>
+      <c r="Q12" s="44"/>
+      <c r="R12" s="44"/>
+      <c r="S12" s="44"/>
+      <c r="T12" s="44"/>
+      <c r="U12" s="44"/>
+      <c r="V12" s="44"/>
+      <c r="W12" s="44"/>
+      <c r="X12" s="44"/>
+      <c r="Y12" s="44"/>
+      <c r="Z12" s="44"/>
+      <c r="AA12" s="44"/>
+      <c r="AB12" s="44"/>
+      <c r="AC12" s="44"/>
+      <c r="AD12" s="44"/>
+      <c r="AE12" s="44"/>
+      <c r="AF12" s="44"/>
+      <c r="AG12" s="44"/>
+      <c r="AH12" s="44"/>
+      <c r="AI12" s="44"/>
+      <c r="AJ12" s="44"/>
+    </row>
+    <row r="13" spans="1:36">
+      <c r="A13" s="68" t="s">
         <v>201</v>
       </c>
-      <c r="B13" s="17">
+      <c r="B13" s="69">
         <v>1</v>
       </c>
       <c r="C13" s="16" t="s">
@@ -12315,32 +13411,45 @@
       <c r="E13" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="3"/>
-      <c r="S13" s="3"/>
-      <c r="T13" s="3">
-        <v>0</v>
-      </c>
-      <c r="U13" s="3"/>
-      <c r="V13" s="3"/>
-      <c r="W13" s="3"/>
-    </row>
-    <row r="14" spans="1:23">
-      <c r="A14" s="24" t="s">
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="44"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="44"/>
+      <c r="T13" s="44">
+        <v>0</v>
+      </c>
+      <c r="U13" s="44"/>
+      <c r="V13" s="44"/>
+      <c r="W13" s="44"/>
+      <c r="X13" s="44"/>
+      <c r="Y13" s="44"/>
+      <c r="Z13" s="44"/>
+      <c r="AA13" s="44"/>
+      <c r="AB13" s="44"/>
+      <c r="AC13" s="44"/>
+      <c r="AD13" s="44"/>
+      <c r="AE13" s="44"/>
+      <c r="AF13" s="44"/>
+      <c r="AG13" s="44"/>
+      <c r="AH13" s="44"/>
+      <c r="AI13" s="44"/>
+      <c r="AJ13" s="44"/>
+    </row>
+    <row r="14" spans="1:36">
+      <c r="A14" s="68" t="s">
         <v>202</v>
       </c>
-      <c r="B14" s="17">
+      <c r="B14" s="69">
         <v>1</v>
       </c>
       <c r="C14" s="16" t="s">
@@ -12352,30 +13461,43 @@
       <c r="E14" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
-      <c r="S14" s="3"/>
-      <c r="T14" s="3"/>
-      <c r="U14" s="3"/>
-      <c r="V14" s="3"/>
-      <c r="W14" s="3"/>
-    </row>
-    <row r="15" spans="1:23">
-      <c r="A15" s="24" t="s">
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
+      <c r="L14" s="44"/>
+      <c r="M14" s="44"/>
+      <c r="N14" s="44"/>
+      <c r="O14" s="44"/>
+      <c r="P14" s="44"/>
+      <c r="Q14" s="44"/>
+      <c r="R14" s="44"/>
+      <c r="S14" s="44"/>
+      <c r="T14" s="44"/>
+      <c r="U14" s="44"/>
+      <c r="V14" s="44"/>
+      <c r="W14" s="44"/>
+      <c r="X14" s="44"/>
+      <c r="Y14" s="44"/>
+      <c r="Z14" s="44"/>
+      <c r="AA14" s="44"/>
+      <c r="AB14" s="44"/>
+      <c r="AC14" s="44"/>
+      <c r="AD14" s="44"/>
+      <c r="AE14" s="44"/>
+      <c r="AF14" s="44"/>
+      <c r="AG14" s="44"/>
+      <c r="AH14" s="44"/>
+      <c r="AI14" s="44"/>
+      <c r="AJ14" s="44"/>
+    </row>
+    <row r="15" spans="1:36">
+      <c r="A15" s="68" t="s">
         <v>203</v>
       </c>
-      <c r="B15" s="17">
+      <c r="B15" s="69">
         <v>1</v>
       </c>
       <c r="C15" s="16" t="s">
@@ -12387,77 +13509,103 @@
       <c r="E15" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="3"/>
-      <c r="S15" s="3"/>
-      <c r="T15" s="3"/>
-      <c r="U15" s="3"/>
-      <c r="V15" s="3"/>
-      <c r="W15" s="3"/>
-    </row>
-    <row r="16" spans="1:23">
-      <c r="A16" s="24" t="s">
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="44"/>
+      <c r="L15" s="44"/>
+      <c r="M15" s="44"/>
+      <c r="N15" s="44"/>
+      <c r="O15" s="44"/>
+      <c r="P15" s="44"/>
+      <c r="Q15" s="44"/>
+      <c r="R15" s="44"/>
+      <c r="S15" s="44"/>
+      <c r="T15" s="44"/>
+      <c r="U15" s="44"/>
+      <c r="V15" s="44"/>
+      <c r="W15" s="44"/>
+      <c r="X15" s="44"/>
+      <c r="Y15" s="44"/>
+      <c r="Z15" s="44"/>
+      <c r="AA15" s="44"/>
+      <c r="AB15" s="44"/>
+      <c r="AC15" s="44"/>
+      <c r="AD15" s="44"/>
+      <c r="AE15" s="44"/>
+      <c r="AF15" s="44"/>
+      <c r="AG15" s="44"/>
+      <c r="AH15" s="44"/>
+      <c r="AI15" s="44"/>
+      <c r="AJ15" s="44"/>
+    </row>
+    <row r="16" spans="1:36">
+      <c r="A16" s="68" t="s">
         <v>204</v>
       </c>
-      <c r="B16" s="17">
+      <c r="B16" s="69">
         <v>2</v>
       </c>
       <c r="C16" s="47" t="s">
         <v>451</v>
       </c>
-      <c r="D16" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="E16" s="32" t="s">
+      <c r="D16" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="44" t="s">
         <v>336</v>
       </c>
-      <c r="F16" s="32">
+      <c r="F16" s="44">
         <v>3</v>
       </c>
-      <c r="G16" s="34" t="s">
+      <c r="G16" s="47" t="s">
         <v>337</v>
       </c>
-      <c r="H16" s="32" t="s">
+      <c r="H16" s="44" t="s">
         <v>336</v>
       </c>
-      <c r="I16" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3"/>
-      <c r="P16" s="3"/>
-      <c r="Q16" s="3"/>
-      <c r="R16" s="3" t="s">
+      <c r="I16" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="J16" s="44"/>
+      <c r="K16" s="44"/>
+      <c r="L16" s="44"/>
+      <c r="M16" s="44"/>
+      <c r="N16" s="44"/>
+      <c r="O16" s="44"/>
+      <c r="P16" s="44"/>
+      <c r="Q16" s="44"/>
+      <c r="R16" s="44" t="s">
         <v>509</v>
       </c>
-      <c r="S16" s="3" t="s">
+      <c r="S16" s="44" t="s">
         <v>510</v>
       </c>
-      <c r="T16" s="3"/>
-      <c r="U16" s="3"/>
-      <c r="V16" s="3"/>
-      <c r="W16" s="3"/>
-    </row>
-    <row r="17" spans="1:23">
-      <c r="A17" s="24" t="s">
+      <c r="T16" s="44"/>
+      <c r="U16" s="44"/>
+      <c r="V16" s="44"/>
+      <c r="W16" s="44"/>
+      <c r="X16" s="44"/>
+      <c r="Y16" s="44"/>
+      <c r="Z16" s="44"/>
+      <c r="AA16" s="44"/>
+      <c r="AB16" s="44"/>
+      <c r="AC16" s="44"/>
+      <c r="AD16" s="44"/>
+      <c r="AE16" s="44"/>
+      <c r="AF16" s="44"/>
+      <c r="AG16" s="44"/>
+      <c r="AH16" s="44"/>
+      <c r="AI16" s="44"/>
+      <c r="AJ16" s="44"/>
+    </row>
+    <row r="17" spans="1:36">
+      <c r="A17" s="68" t="s">
         <v>205</v>
       </c>
-      <c r="B17" s="17">
+      <c r="B17" s="69">
         <v>1</v>
       </c>
       <c r="C17" s="16" t="s">
@@ -12469,24 +13617,1325 @@
       <c r="E17" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="3"/>
-      <c r="S17" s="3"/>
-      <c r="T17" s="3"/>
-      <c r="U17" s="3"/>
-      <c r="V17" s="3"/>
-      <c r="W17" s="3"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="44"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="44"/>
+      <c r="J17" s="44"/>
+      <c r="K17" s="44"/>
+      <c r="L17" s="44"/>
+      <c r="M17" s="44"/>
+      <c r="N17" s="44"/>
+      <c r="O17" s="44"/>
+      <c r="P17" s="44"/>
+      <c r="Q17" s="44"/>
+      <c r="R17" s="44"/>
+      <c r="S17" s="44"/>
+      <c r="T17" s="44"/>
+      <c r="U17" s="44"/>
+      <c r="V17" s="44"/>
+      <c r="W17" s="44"/>
+      <c r="X17" s="44"/>
+      <c r="Y17" s="44"/>
+      <c r="Z17" s="44"/>
+      <c r="AA17" s="44"/>
+      <c r="AB17" s="44"/>
+      <c r="AC17" s="44"/>
+      <c r="AD17" s="44"/>
+      <c r="AE17" s="44"/>
+      <c r="AF17" s="44"/>
+      <c r="AG17" s="44"/>
+      <c r="AH17" s="44"/>
+      <c r="AI17" s="44"/>
+      <c r="AJ17" s="44"/>
+    </row>
+    <row r="18" spans="1:36">
+      <c r="A18" s="67" t="s">
+        <v>686</v>
+      </c>
+      <c r="B18" s="69">
+        <v>1</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>452</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="44">
+        <v>2</v>
+      </c>
+      <c r="G18" s="47" t="s">
+        <v>326</v>
+      </c>
+      <c r="H18" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I18" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="J18" s="44"/>
+      <c r="K18" s="44"/>
+      <c r="L18" s="44"/>
+      <c r="M18" s="44"/>
+      <c r="N18" s="44"/>
+      <c r="O18" s="44"/>
+      <c r="P18" s="44"/>
+      <c r="Q18" s="44"/>
+      <c r="R18" s="44" t="s">
+        <v>687</v>
+      </c>
+      <c r="S18" s="44"/>
+      <c r="T18" s="47">
+        <v>0</v>
+      </c>
+      <c r="U18" s="44"/>
+      <c r="V18" s="44"/>
+      <c r="W18" s="44"/>
+      <c r="X18" s="44"/>
+      <c r="Y18" s="44"/>
+      <c r="Z18" s="44"/>
+      <c r="AA18" s="44"/>
+      <c r="AB18" s="44"/>
+      <c r="AC18" s="44"/>
+      <c r="AD18" s="44"/>
+      <c r="AE18" s="44"/>
+      <c r="AF18" s="44"/>
+      <c r="AG18" s="44"/>
+      <c r="AH18" s="44"/>
+      <c r="AI18" s="44"/>
+      <c r="AJ18" s="44"/>
+    </row>
+    <row r="19" spans="1:36">
+      <c r="A19" s="67" t="s">
+        <v>688</v>
+      </c>
+      <c r="B19" s="69">
+        <v>1</v>
+      </c>
+      <c r="C19" s="47" t="s">
+        <v>330</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="44">
+        <v>1</v>
+      </c>
+      <c r="G19" s="47" t="s">
+        <v>689</v>
+      </c>
+      <c r="H19" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I19" s="44" t="s">
+        <v>216</v>
+      </c>
+      <c r="J19" s="44">
+        <v>2</v>
+      </c>
+      <c r="K19" s="47" t="s">
+        <v>690</v>
+      </c>
+      <c r="L19" s="44" t="s">
+        <v>216</v>
+      </c>
+      <c r="M19" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="N19" s="44">
+        <v>2</v>
+      </c>
+      <c r="O19" s="47" t="s">
+        <v>326</v>
+      </c>
+      <c r="P19" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q19" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="R19" s="44" t="s">
+        <v>691</v>
+      </c>
+      <c r="S19" s="44"/>
+      <c r="T19" s="47">
+        <v>0</v>
+      </c>
+      <c r="U19" s="44"/>
+      <c r="V19" s="44"/>
+      <c r="W19" s="44"/>
+      <c r="X19" s="44"/>
+      <c r="Y19" s="44"/>
+      <c r="Z19" s="44"/>
+      <c r="AA19" s="44"/>
+      <c r="AB19" s="44"/>
+      <c r="AC19" s="44"/>
+      <c r="AD19" s="44"/>
+      <c r="AE19" s="44"/>
+      <c r="AF19" s="44"/>
+      <c r="AG19" s="44"/>
+      <c r="AH19" s="44"/>
+      <c r="AI19" s="44"/>
+      <c r="AJ19" s="44"/>
+    </row>
+    <row r="20" spans="1:36">
+      <c r="A20" s="67" t="s">
+        <v>692</v>
+      </c>
+      <c r="B20" s="69">
+        <v>1</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>693</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="44">
+        <v>1</v>
+      </c>
+      <c r="G20" s="47" t="s">
+        <v>694</v>
+      </c>
+      <c r="H20" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="I20" s="44" t="s">
+        <v>695</v>
+      </c>
+      <c r="J20" s="44">
+        <v>2</v>
+      </c>
+      <c r="K20" s="47" t="s">
+        <v>696</v>
+      </c>
+      <c r="L20" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="M20" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="N20" s="44">
+        <v>2</v>
+      </c>
+      <c r="O20" s="47" t="s">
+        <v>697</v>
+      </c>
+      <c r="P20" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q20" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="R20" s="44" t="s">
+        <v>698</v>
+      </c>
+      <c r="S20" s="44"/>
+      <c r="T20" s="47">
+        <v>0</v>
+      </c>
+      <c r="U20" s="44"/>
+      <c r="V20" s="44"/>
+      <c r="W20" s="44"/>
+      <c r="X20" s="44"/>
+      <c r="Y20" s="44"/>
+      <c r="Z20" s="44"/>
+      <c r="AA20" s="44"/>
+      <c r="AB20" s="44"/>
+      <c r="AC20" s="44"/>
+      <c r="AD20" s="44"/>
+      <c r="AE20" s="44"/>
+      <c r="AF20" s="44"/>
+      <c r="AG20" s="44"/>
+      <c r="AH20" s="44"/>
+      <c r="AI20" s="44"/>
+      <c r="AJ20" s="44"/>
+    </row>
+    <row r="21" spans="1:36">
+      <c r="A21" s="67" t="s">
+        <v>699</v>
+      </c>
+      <c r="B21" s="69">
+        <v>1</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>330</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F21" s="44">
+        <v>3</v>
+      </c>
+      <c r="G21" s="47" t="s">
+        <v>326</v>
+      </c>
+      <c r="H21" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I21" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="J21" s="44">
+        <v>2</v>
+      </c>
+      <c r="K21" s="44"/>
+      <c r="L21" s="44"/>
+      <c r="M21" s="44"/>
+      <c r="N21" s="44"/>
+      <c r="O21" s="44"/>
+      <c r="P21" s="44"/>
+      <c r="Q21" s="44"/>
+      <c r="R21" s="44" t="s">
+        <v>700</v>
+      </c>
+      <c r="S21" s="44"/>
+      <c r="T21" s="47">
+        <v>0</v>
+      </c>
+      <c r="U21" s="44"/>
+      <c r="V21" s="44"/>
+      <c r="W21" s="44"/>
+      <c r="X21" s="44" t="s">
+        <v>701</v>
+      </c>
+      <c r="Y21" s="44" t="s">
+        <v>702</v>
+      </c>
+      <c r="Z21" s="44" t="s">
+        <v>701</v>
+      </c>
+      <c r="AA21" s="44" t="s">
+        <v>702</v>
+      </c>
+      <c r="AB21" s="44"/>
+      <c r="AC21" s="44"/>
+      <c r="AD21" s="44"/>
+      <c r="AE21" s="44"/>
+      <c r="AF21" s="44"/>
+      <c r="AG21" s="44"/>
+      <c r="AH21" s="44"/>
+      <c r="AI21" s="44"/>
+      <c r="AJ21" s="44"/>
+    </row>
+    <row r="22" spans="1:36">
+      <c r="A22" s="67" t="s">
+        <v>703</v>
+      </c>
+      <c r="B22" s="69"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="44"/>
+      <c r="H22" s="44"/>
+      <c r="I22" s="44"/>
+      <c r="J22" s="44"/>
+      <c r="K22" s="44"/>
+      <c r="L22" s="44"/>
+      <c r="M22" s="44"/>
+      <c r="N22" s="44"/>
+      <c r="O22" s="44"/>
+      <c r="P22" s="44"/>
+      <c r="Q22" s="44"/>
+      <c r="R22" s="44"/>
+      <c r="S22" s="44"/>
+      <c r="T22" s="44"/>
+      <c r="U22" s="44">
+        <v>1</v>
+      </c>
+      <c r="V22" s="44">
+        <v>6</v>
+      </c>
+      <c r="W22" s="44"/>
+      <c r="X22" s="44"/>
+      <c r="Y22" s="44"/>
+      <c r="Z22" s="44"/>
+      <c r="AA22" s="44"/>
+      <c r="AB22" s="44"/>
+      <c r="AC22" s="44"/>
+      <c r="AD22" s="44"/>
+      <c r="AE22" s="44"/>
+      <c r="AF22" s="44"/>
+      <c r="AG22" s="44"/>
+      <c r="AH22" s="44"/>
+      <c r="AI22" s="44"/>
+      <c r="AJ22" s="44"/>
+    </row>
+    <row r="23" spans="1:36">
+      <c r="A23" s="67" t="s">
+        <v>704</v>
+      </c>
+      <c r="B23" s="69">
+        <v>1</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="44"/>
+      <c r="I23" s="44"/>
+      <c r="J23" s="44"/>
+      <c r="K23" s="44"/>
+      <c r="L23" s="44"/>
+      <c r="M23" s="44"/>
+      <c r="N23" s="44"/>
+      <c r="O23" s="44"/>
+      <c r="P23" s="44"/>
+      <c r="Q23" s="44"/>
+      <c r="R23" s="44"/>
+      <c r="S23" s="44"/>
+      <c r="T23" s="44"/>
+      <c r="U23" s="44"/>
+      <c r="V23" s="44"/>
+      <c r="W23" s="44"/>
+      <c r="X23" s="44"/>
+      <c r="Y23" s="44"/>
+      <c r="Z23" s="44"/>
+      <c r="AA23" s="44"/>
+      <c r="AB23" s="44"/>
+      <c r="AC23" s="44"/>
+      <c r="AD23" s="44"/>
+      <c r="AE23" s="44"/>
+      <c r="AF23" s="44"/>
+      <c r="AG23" s="44"/>
+      <c r="AH23" s="44"/>
+      <c r="AI23" s="44"/>
+      <c r="AJ23" s="44"/>
+    </row>
+    <row r="24" spans="1:36">
+      <c r="A24" s="67" t="s">
+        <v>705</v>
+      </c>
+      <c r="B24" s="69">
+        <v>1</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24" s="44">
+        <v>2</v>
+      </c>
+      <c r="G24" s="47" t="s">
+        <v>176</v>
+      </c>
+      <c r="H24" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="I24" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="J24" s="44"/>
+      <c r="K24" s="44"/>
+      <c r="L24" s="44"/>
+      <c r="M24" s="44"/>
+      <c r="N24" s="44"/>
+      <c r="O24" s="44"/>
+      <c r="P24" s="44"/>
+      <c r="Q24" s="44"/>
+      <c r="R24" s="44" t="s">
+        <v>706</v>
+      </c>
+      <c r="S24" s="44"/>
+      <c r="T24" s="47"/>
+      <c r="U24" s="44"/>
+      <c r="V24" s="44"/>
+      <c r="W24" s="44"/>
+      <c r="X24" s="44"/>
+      <c r="Y24" s="44"/>
+      <c r="Z24" s="44"/>
+      <c r="AA24" s="44"/>
+      <c r="AB24" s="44"/>
+      <c r="AC24" s="44"/>
+      <c r="AD24" s="44"/>
+      <c r="AE24" s="44"/>
+      <c r="AF24" s="44"/>
+      <c r="AG24" s="44"/>
+      <c r="AH24" s="44"/>
+      <c r="AI24" s="44"/>
+      <c r="AJ24" s="44"/>
+    </row>
+    <row r="25" spans="1:36">
+      <c r="A25" s="67" t="s">
+        <v>707</v>
+      </c>
+      <c r="B25" s="69">
+        <v>1</v>
+      </c>
+      <c r="C25" s="47" t="s">
+        <v>708</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F25" s="44"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="44"/>
+      <c r="I25" s="44"/>
+      <c r="J25" s="44"/>
+      <c r="K25" s="44"/>
+      <c r="L25" s="44"/>
+      <c r="M25" s="44"/>
+      <c r="N25" s="44"/>
+      <c r="O25" s="44"/>
+      <c r="P25" s="44"/>
+      <c r="Q25" s="44"/>
+      <c r="R25" s="44"/>
+      <c r="S25" s="44"/>
+      <c r="T25" s="44"/>
+      <c r="U25" s="44"/>
+      <c r="V25" s="44"/>
+      <c r="W25" s="44"/>
+      <c r="X25" s="44"/>
+      <c r="Y25" s="44"/>
+      <c r="Z25" s="44"/>
+      <c r="AA25" s="44"/>
+      <c r="AB25" s="44"/>
+      <c r="AC25" s="44"/>
+      <c r="AD25" s="44"/>
+      <c r="AE25" s="44"/>
+      <c r="AF25" s="44"/>
+      <c r="AG25" s="44"/>
+      <c r="AH25" s="44"/>
+      <c r="AI25" s="44"/>
+      <c r="AJ25" s="44"/>
+    </row>
+    <row r="26" spans="1:36">
+      <c r="A26" s="67" t="s">
+        <v>709</v>
+      </c>
+      <c r="B26" s="69">
+        <v>1</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F26" s="44"/>
+      <c r="G26" s="44"/>
+      <c r="H26" s="44"/>
+      <c r="I26" s="44"/>
+      <c r="J26" s="44"/>
+      <c r="K26" s="44"/>
+      <c r="L26" s="44"/>
+      <c r="M26" s="44"/>
+      <c r="N26" s="44"/>
+      <c r="O26" s="44"/>
+      <c r="P26" s="44"/>
+      <c r="Q26" s="44"/>
+      <c r="R26" s="44"/>
+      <c r="S26" s="44"/>
+      <c r="T26" s="44"/>
+      <c r="U26" s="44"/>
+      <c r="V26" s="44"/>
+      <c r="W26" s="44"/>
+      <c r="X26" s="44" t="s">
+        <v>710</v>
+      </c>
+      <c r="Y26" s="44" t="s">
+        <v>711</v>
+      </c>
+      <c r="Z26" s="44"/>
+      <c r="AA26" s="44"/>
+      <c r="AB26" s="44"/>
+      <c r="AC26" s="44"/>
+      <c r="AD26" s="44"/>
+      <c r="AE26" s="44"/>
+      <c r="AF26" s="44"/>
+      <c r="AG26" s="44"/>
+      <c r="AH26" s="44"/>
+      <c r="AI26" s="44"/>
+      <c r="AJ26" s="44"/>
+    </row>
+    <row r="27" spans="1:36">
+      <c r="A27" s="67" t="s">
+        <v>712</v>
+      </c>
+      <c r="B27" s="69">
+        <v>1</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F27" s="44"/>
+      <c r="G27" s="44"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="44"/>
+      <c r="J27" s="44"/>
+      <c r="K27" s="44"/>
+      <c r="L27" s="44"/>
+      <c r="M27" s="44"/>
+      <c r="N27" s="44"/>
+      <c r="O27" s="44"/>
+      <c r="P27" s="44"/>
+      <c r="Q27" s="44"/>
+      <c r="R27" s="44"/>
+      <c r="S27" s="44"/>
+      <c r="T27" s="44"/>
+      <c r="U27" s="44"/>
+      <c r="V27" s="44"/>
+      <c r="W27" s="44"/>
+      <c r="X27" s="44" t="s">
+        <v>710</v>
+      </c>
+      <c r="Y27" s="44" t="s">
+        <v>711</v>
+      </c>
+      <c r="Z27" s="44"/>
+      <c r="AA27" s="44"/>
+      <c r="AB27" s="44"/>
+      <c r="AC27" s="44"/>
+      <c r="AD27" s="44"/>
+      <c r="AE27" s="44"/>
+      <c r="AF27" s="44"/>
+      <c r="AG27" s="44"/>
+      <c r="AH27" s="44"/>
+      <c r="AI27" s="44"/>
+      <c r="AJ27" s="44"/>
+    </row>
+    <row r="28" spans="1:36">
+      <c r="A28" s="67" t="s">
+        <v>713</v>
+      </c>
+      <c r="B28" s="69">
+        <v>1</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F28" s="44"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="44"/>
+      <c r="I28" s="44"/>
+      <c r="J28" s="44"/>
+      <c r="K28" s="44"/>
+      <c r="L28" s="44"/>
+      <c r="M28" s="44"/>
+      <c r="N28" s="44"/>
+      <c r="O28" s="44"/>
+      <c r="P28" s="44"/>
+      <c r="Q28" s="44"/>
+      <c r="R28" s="44" t="s">
+        <v>714</v>
+      </c>
+      <c r="S28" s="44"/>
+      <c r="T28" s="47">
+        <v>0</v>
+      </c>
+      <c r="U28" s="44"/>
+      <c r="V28" s="44">
+        <v>3</v>
+      </c>
+      <c r="W28" s="44"/>
+      <c r="X28" s="44"/>
+      <c r="Y28" s="44"/>
+      <c r="Z28" s="44"/>
+      <c r="AA28" s="44"/>
+      <c r="AB28" s="44"/>
+      <c r="AC28" s="44"/>
+      <c r="AD28" s="44"/>
+      <c r="AE28" s="44"/>
+      <c r="AF28" s="44"/>
+      <c r="AG28" s="44"/>
+      <c r="AH28" s="44"/>
+      <c r="AI28" s="44"/>
+      <c r="AJ28" s="44"/>
+    </row>
+    <row r="29" spans="1:36">
+      <c r="A29" s="39" t="s">
+        <v>715</v>
+      </c>
+      <c r="B29" s="69">
+        <v>1</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>337</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" s="44">
+        <v>1</v>
+      </c>
+      <c r="G29" s="47" t="s">
+        <v>46</v>
+      </c>
+      <c r="H29" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I29" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="J29" s="44">
+        <v>2</v>
+      </c>
+      <c r="K29" s="47" t="s">
+        <v>716</v>
+      </c>
+      <c r="L29" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="M29" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="N29" s="44">
+        <v>2</v>
+      </c>
+      <c r="O29" s="47" t="s">
+        <v>44</v>
+      </c>
+      <c r="P29" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q29" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="R29" s="44" t="s">
+        <v>378</v>
+      </c>
+      <c r="S29" s="44"/>
+      <c r="T29" s="44"/>
+      <c r="U29" s="44"/>
+      <c r="V29" s="44"/>
+      <c r="W29" s="44"/>
+      <c r="X29" s="44"/>
+      <c r="Y29" s="44"/>
+      <c r="Z29" s="44"/>
+      <c r="AA29" s="44"/>
+      <c r="AB29" s="44">
+        <v>3</v>
+      </c>
+      <c r="AC29" s="47" t="s">
+        <v>717</v>
+      </c>
+      <c r="AD29" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE29" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="AF29" s="44">
+        <v>3</v>
+      </c>
+      <c r="AG29" s="47" t="s">
+        <v>708</v>
+      </c>
+      <c r="AH29" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="AI29" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ29" s="44"/>
+    </row>
+    <row r="30" spans="1:36">
+      <c r="A30" s="67" t="s">
+        <v>718</v>
+      </c>
+      <c r="B30" s="69">
+        <v>1</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>563</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F30" s="44"/>
+      <c r="G30" s="44"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="44"/>
+      <c r="J30" s="44"/>
+      <c r="K30" s="44"/>
+      <c r="L30" s="44"/>
+      <c r="M30" s="44"/>
+      <c r="N30" s="44"/>
+      <c r="O30" s="44"/>
+      <c r="P30" s="44"/>
+      <c r="Q30" s="44"/>
+      <c r="R30" s="44" t="s">
+        <v>719</v>
+      </c>
+      <c r="S30" s="44"/>
+      <c r="T30" s="44">
+        <v>0</v>
+      </c>
+      <c r="U30" s="44">
+        <v>1</v>
+      </c>
+      <c r="V30" s="44">
+        <v>1</v>
+      </c>
+      <c r="W30" s="44"/>
+      <c r="X30" s="44"/>
+      <c r="Y30" s="44"/>
+      <c r="Z30" s="44"/>
+      <c r="AA30" s="44"/>
+      <c r="AB30" s="44"/>
+      <c r="AC30" s="44"/>
+      <c r="AD30" s="44"/>
+      <c r="AE30" s="44"/>
+      <c r="AF30" s="44"/>
+      <c r="AG30" s="44"/>
+      <c r="AH30" s="44"/>
+      <c r="AI30" s="44"/>
+      <c r="AJ30" s="44"/>
+    </row>
+    <row r="31" spans="1:36">
+      <c r="A31" s="67" t="s">
+        <v>720</v>
+      </c>
+      <c r="B31" s="69">
+        <v>1</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F31" s="44"/>
+      <c r="G31" s="44"/>
+      <c r="H31" s="44"/>
+      <c r="I31" s="44"/>
+      <c r="J31" s="44"/>
+      <c r="K31" s="44"/>
+      <c r="L31" s="44"/>
+      <c r="M31" s="44"/>
+      <c r="N31" s="44"/>
+      <c r="O31" s="44"/>
+      <c r="P31" s="44"/>
+      <c r="Q31" s="44"/>
+      <c r="R31" s="44" t="s">
+        <v>721</v>
+      </c>
+      <c r="S31" s="44"/>
+      <c r="T31" s="44">
+        <v>0</v>
+      </c>
+      <c r="U31" s="44">
+        <v>1</v>
+      </c>
+      <c r="V31" s="44">
+        <v>1</v>
+      </c>
+      <c r="W31" s="44"/>
+      <c r="X31" s="44"/>
+      <c r="Y31" s="44"/>
+      <c r="Z31" s="44"/>
+      <c r="AA31" s="44"/>
+      <c r="AB31" s="44"/>
+      <c r="AC31" s="44"/>
+      <c r="AD31" s="44"/>
+      <c r="AE31" s="44"/>
+      <c r="AF31" s="44"/>
+      <c r="AG31" s="44"/>
+      <c r="AH31" s="44"/>
+      <c r="AI31" s="44"/>
+      <c r="AJ31" s="44"/>
+    </row>
+    <row r="32" spans="1:36">
+      <c r="A32" s="67" t="s">
+        <v>722</v>
+      </c>
+      <c r="B32" s="69">
+        <v>1</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F32" s="44"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="44"/>
+      <c r="I32" s="44"/>
+      <c r="J32" s="44"/>
+      <c r="K32" s="44"/>
+      <c r="L32" s="44"/>
+      <c r="M32" s="44"/>
+      <c r="N32" s="44"/>
+      <c r="O32" s="44"/>
+      <c r="P32" s="44"/>
+      <c r="Q32" s="44"/>
+      <c r="R32" s="44" t="s">
+        <v>723</v>
+      </c>
+      <c r="S32" s="44"/>
+      <c r="T32" s="44">
+        <v>0</v>
+      </c>
+      <c r="U32" s="44">
+        <v>1</v>
+      </c>
+      <c r="V32" s="44">
+        <v>1</v>
+      </c>
+      <c r="W32" s="44"/>
+      <c r="X32" s="44"/>
+      <c r="Y32" s="44"/>
+      <c r="Z32" s="44"/>
+      <c r="AA32" s="44"/>
+      <c r="AB32" s="44"/>
+      <c r="AC32" s="44"/>
+      <c r="AD32" s="44"/>
+      <c r="AE32" s="44"/>
+      <c r="AF32" s="44"/>
+      <c r="AG32" s="44"/>
+      <c r="AH32" s="44"/>
+      <c r="AI32" s="44"/>
+      <c r="AJ32" s="44"/>
+    </row>
+    <row r="33" spans="1:36">
+      <c r="A33" s="67" t="s">
+        <v>724</v>
+      </c>
+      <c r="B33" s="69">
+        <v>1</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F33" s="44"/>
+      <c r="G33" s="44"/>
+      <c r="H33" s="44"/>
+      <c r="I33" s="44"/>
+      <c r="J33" s="44"/>
+      <c r="K33" s="44"/>
+      <c r="L33" s="44"/>
+      <c r="M33" s="44"/>
+      <c r="N33" s="44"/>
+      <c r="O33" s="44"/>
+      <c r="P33" s="44"/>
+      <c r="Q33" s="44"/>
+      <c r="R33" s="44" t="s">
+        <v>725</v>
+      </c>
+      <c r="S33" s="44"/>
+      <c r="T33" s="44">
+        <v>0</v>
+      </c>
+      <c r="U33" s="44">
+        <v>1</v>
+      </c>
+      <c r="V33" s="44">
+        <v>1</v>
+      </c>
+      <c r="W33" s="44"/>
+      <c r="X33" s="44"/>
+      <c r="Y33" s="44"/>
+      <c r="Z33" s="44"/>
+      <c r="AA33" s="44"/>
+      <c r="AB33" s="44"/>
+      <c r="AC33" s="44"/>
+      <c r="AD33" s="44"/>
+      <c r="AE33" s="44"/>
+      <c r="AF33" s="44"/>
+      <c r="AG33" s="44"/>
+      <c r="AH33" s="44"/>
+      <c r="AI33" s="44"/>
+      <c r="AJ33" s="44"/>
+    </row>
+    <row r="34" spans="1:36">
+      <c r="A34" s="67" t="s">
+        <v>726</v>
+      </c>
+      <c r="B34" s="69">
+        <v>1</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F34" s="44"/>
+      <c r="G34" s="44"/>
+      <c r="H34" s="44"/>
+      <c r="I34" s="44"/>
+      <c r="J34" s="44"/>
+      <c r="K34" s="44"/>
+      <c r="L34" s="44"/>
+      <c r="M34" s="44"/>
+      <c r="N34" s="44"/>
+      <c r="O34" s="44"/>
+      <c r="P34" s="44"/>
+      <c r="Q34" s="44"/>
+      <c r="R34" s="44" t="s">
+        <v>727</v>
+      </c>
+      <c r="S34" s="44"/>
+      <c r="T34" s="44">
+        <v>0</v>
+      </c>
+      <c r="U34" s="44">
+        <v>1</v>
+      </c>
+      <c r="V34" s="44">
+        <v>1</v>
+      </c>
+      <c r="W34" s="44"/>
+      <c r="X34" s="44"/>
+      <c r="Y34" s="44"/>
+      <c r="Z34" s="44"/>
+      <c r="AA34" s="44"/>
+      <c r="AB34" s="44"/>
+      <c r="AC34" s="44"/>
+      <c r="AD34" s="44"/>
+      <c r="AE34" s="44"/>
+      <c r="AF34" s="44"/>
+      <c r="AG34" s="44"/>
+      <c r="AH34" s="44"/>
+      <c r="AI34" s="44"/>
+      <c r="AJ34" s="44"/>
+    </row>
+    <row r="35" spans="1:36">
+      <c r="A35" s="67" t="s">
+        <v>728</v>
+      </c>
+      <c r="B35" s="69">
+        <v>1</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F35" s="44"/>
+      <c r="G35" s="44"/>
+      <c r="H35" s="44"/>
+      <c r="I35" s="44"/>
+      <c r="J35" s="44"/>
+      <c r="K35" s="44"/>
+      <c r="L35" s="44"/>
+      <c r="M35" s="44"/>
+      <c r="N35" s="44"/>
+      <c r="O35" s="44"/>
+      <c r="P35" s="44"/>
+      <c r="Q35" s="44"/>
+      <c r="R35" s="44" t="s">
+        <v>729</v>
+      </c>
+      <c r="S35" s="44"/>
+      <c r="T35" s="44">
+        <v>0</v>
+      </c>
+      <c r="U35" s="44">
+        <v>1</v>
+      </c>
+      <c r="V35" s="44">
+        <v>1</v>
+      </c>
+      <c r="W35" s="44"/>
+      <c r="X35" s="44"/>
+      <c r="Y35" s="44"/>
+      <c r="Z35" s="44"/>
+      <c r="AA35" s="44"/>
+      <c r="AB35" s="44"/>
+      <c r="AC35" s="44"/>
+      <c r="AD35" s="44"/>
+      <c r="AE35" s="44"/>
+      <c r="AF35" s="44"/>
+      <c r="AG35" s="44"/>
+      <c r="AH35" s="44"/>
+      <c r="AI35" s="44"/>
+      <c r="AJ35" s="44"/>
+    </row>
+    <row r="36" spans="1:36">
+      <c r="A36" s="67" t="s">
+        <v>730</v>
+      </c>
+      <c r="B36" s="69">
+        <v>1</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F36" s="44"/>
+      <c r="G36" s="44"/>
+      <c r="H36" s="44"/>
+      <c r="I36" s="44"/>
+      <c r="J36" s="44"/>
+      <c r="K36" s="44"/>
+      <c r="L36" s="44"/>
+      <c r="M36" s="44"/>
+      <c r="N36" s="44"/>
+      <c r="O36" s="44"/>
+      <c r="P36" s="44"/>
+      <c r="Q36" s="44"/>
+      <c r="R36" s="44" t="s">
+        <v>731</v>
+      </c>
+      <c r="S36" s="44"/>
+      <c r="T36" s="44">
+        <v>0</v>
+      </c>
+      <c r="U36" s="44">
+        <v>1</v>
+      </c>
+      <c r="V36" s="44">
+        <v>1</v>
+      </c>
+      <c r="W36" s="44"/>
+      <c r="X36" s="44"/>
+      <c r="Y36" s="44"/>
+      <c r="Z36" s="44"/>
+      <c r="AA36" s="44"/>
+      <c r="AB36" s="44"/>
+      <c r="AC36" s="44"/>
+      <c r="AD36" s="44"/>
+      <c r="AE36" s="44"/>
+      <c r="AF36" s="44"/>
+      <c r="AG36" s="44"/>
+      <c r="AH36" s="44"/>
+      <c r="AI36" s="44"/>
+      <c r="AJ36" s="44"/>
+    </row>
+    <row r="37" spans="1:36">
+      <c r="A37" s="39" t="s">
+        <v>732</v>
+      </c>
+      <c r="B37" s="69">
+        <v>1</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F37" s="44"/>
+      <c r="G37" s="44"/>
+      <c r="H37" s="44"/>
+      <c r="I37" s="44"/>
+      <c r="J37" s="44"/>
+      <c r="K37" s="44"/>
+      <c r="L37" s="44"/>
+      <c r="M37" s="44"/>
+      <c r="N37" s="44"/>
+      <c r="O37" s="44"/>
+      <c r="P37" s="44"/>
+      <c r="Q37" s="44"/>
+      <c r="R37" s="44" t="s">
+        <v>733</v>
+      </c>
+      <c r="S37" s="44"/>
+      <c r="T37" s="44">
+        <v>0</v>
+      </c>
+      <c r="U37" s="44">
+        <v>1</v>
+      </c>
+      <c r="V37" s="44">
+        <v>1</v>
+      </c>
+      <c r="W37" s="44"/>
+      <c r="X37" s="44"/>
+      <c r="Y37" s="44"/>
+      <c r="Z37" s="44"/>
+      <c r="AA37" s="44"/>
+      <c r="AB37" s="44"/>
+      <c r="AC37" s="44"/>
+      <c r="AD37" s="44"/>
+      <c r="AE37" s="44"/>
+      <c r="AF37" s="44"/>
+      <c r="AG37" s="44"/>
+      <c r="AH37" s="44"/>
+      <c r="AI37" s="44"/>
+      <c r="AJ37" s="44"/>
+    </row>
+    <row r="38" spans="1:36">
+      <c r="A38" s="67" t="s">
+        <v>734</v>
+      </c>
+      <c r="B38" s="69">
+        <v>1</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F38" s="44"/>
+      <c r="G38" s="44"/>
+      <c r="H38" s="44"/>
+      <c r="I38" s="44"/>
+      <c r="J38" s="44"/>
+      <c r="K38" s="44"/>
+      <c r="L38" s="44"/>
+      <c r="M38" s="44"/>
+      <c r="N38" s="44"/>
+      <c r="O38" s="44"/>
+      <c r="P38" s="44"/>
+      <c r="Q38" s="44"/>
+      <c r="R38" s="44" t="s">
+        <v>735</v>
+      </c>
+      <c r="S38" s="44"/>
+      <c r="T38" s="44">
+        <v>0</v>
+      </c>
+      <c r="U38" s="44">
+        <v>1</v>
+      </c>
+      <c r="V38" s="44">
+        <v>1</v>
+      </c>
+      <c r="W38" s="44"/>
+      <c r="X38" s="44"/>
+      <c r="Y38" s="44"/>
+      <c r="Z38" s="44"/>
+      <c r="AA38" s="44"/>
+      <c r="AB38" s="44"/>
+      <c r="AC38" s="44"/>
+      <c r="AD38" s="44"/>
+      <c r="AE38" s="44"/>
+      <c r="AF38" s="44"/>
+      <c r="AG38" s="44"/>
+      <c r="AH38" s="44"/>
+      <c r="AI38" s="44"/>
+      <c r="AJ38" s="47" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="39" spans="1:36">
+      <c r="A39" s="67" t="s">
+        <v>736</v>
+      </c>
+      <c r="B39" s="69">
+        <v>1</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F39" s="44"/>
+      <c r="G39" s="44"/>
+      <c r="H39" s="44"/>
+      <c r="I39" s="44"/>
+      <c r="J39" s="44"/>
+      <c r="K39" s="44"/>
+      <c r="L39" s="44"/>
+      <c r="M39" s="44"/>
+      <c r="N39" s="44"/>
+      <c r="O39" s="44"/>
+      <c r="P39" s="44"/>
+      <c r="Q39" s="44"/>
+      <c r="R39" s="44" t="s">
+        <v>737</v>
+      </c>
+      <c r="S39" s="44" t="s">
+        <v>378</v>
+      </c>
+      <c r="T39" s="44">
+        <v>0</v>
+      </c>
+      <c r="U39" s="44"/>
+      <c r="V39" s="44"/>
+      <c r="W39" s="44"/>
+      <c r="X39" s="44"/>
+      <c r="Y39" s="44"/>
+      <c r="Z39" s="44"/>
+      <c r="AA39" s="44"/>
+      <c r="AB39" s="44"/>
+      <c r="AC39" s="44"/>
+      <c r="AD39" s="44"/>
+      <c r="AE39" s="44"/>
+      <c r="AF39" s="44"/>
+      <c r="AG39" s="44"/>
+      <c r="AH39" s="44"/>
+      <c r="AI39" s="44"/>
+      <c r="AJ39" s="44"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added CreateBookingService from Sowmya
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
@@ -55,7 +55,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2396" uniqueCount="741">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2434" uniqueCount="779">
   <si>
     <t>Scenario</t>
   </si>
@@ -2297,12 +2297,127 @@
   </si>
   <si>
     <t>333</t>
+  </si>
+  <si>
+    <t>BA2MRK</t>
+  </si>
+  <si>
+    <t>2302182825478</t>
+  </si>
+  <si>
+    <t>BA2MR4</t>
+  </si>
+  <si>
+    <t>2302182825479</t>
+  </si>
+  <si>
+    <t>BA2MSL</t>
+  </si>
+  <si>
+    <t>BA2MSN</t>
+  </si>
+  <si>
+    <t>BA2MSO</t>
+  </si>
+  <si>
+    <t>BA2MSZ</t>
+  </si>
+  <si>
+    <t>BA2MUM</t>
+  </si>
+  <si>
+    <t>BA2MVE</t>
+  </si>
+  <si>
+    <t>BA2MVU</t>
+  </si>
+  <si>
+    <t>2302182825481</t>
+  </si>
+  <si>
+    <t>BA2MWU</t>
+  </si>
+  <si>
+    <t>BA2MWX</t>
+  </si>
+  <si>
+    <t>2302182825482</t>
+  </si>
+  <si>
+    <t>BA2MXM</t>
+  </si>
+  <si>
+    <t>BA2MXN</t>
+  </si>
+  <si>
+    <t>2302182825483</t>
+  </si>
+  <si>
+    <t>BA2MXX</t>
+  </si>
+  <si>
+    <t>BA2MXY</t>
+  </si>
+  <si>
+    <t>2302182825484</t>
+  </si>
+  <si>
+    <t>BA2MYC</t>
+  </si>
+  <si>
+    <t>BA2MYQ</t>
+  </si>
+  <si>
+    <t>2302182825485</t>
+  </si>
+  <si>
+    <t>BA2M0R</t>
+  </si>
+  <si>
+    <t>BA2M02</t>
+  </si>
+  <si>
+    <t>2302182825490</t>
+  </si>
+  <si>
+    <t>BA2M1O</t>
+  </si>
+  <si>
+    <t>BA2M1P</t>
+  </si>
+  <si>
+    <t>2302182825491</t>
+  </si>
+  <si>
+    <t>BA2M2D</t>
+  </si>
+  <si>
+    <t>BA2M2F</t>
+  </si>
+  <si>
+    <t>2302182825492</t>
+  </si>
+  <si>
+    <t>BA2M2Q</t>
+  </si>
+  <si>
+    <t>BA2M2R</t>
+  </si>
+  <si>
+    <t>BA2M2S</t>
+  </si>
+  <si>
+    <t>2302182825493</t>
+  </si>
+  <si>
+    <t>BA2M3C</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="14">
     <font>
       <sz val="11"/>
@@ -2975,20 +3090,20 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="52.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="52.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -3223,15 +3338,15 @@
   <dimension ref="A1:W22"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="49" customWidth="1"/>
-    <col min="10" max="10" width="8.81640625" style="25"/>
-    <col min="12" max="12" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="19.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="49.0"/>
+    <col min="10" max="10" style="25" width="8.81640625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="11.453125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="12.6328125"/>
+    <col min="22" max="23" bestFit="true" customWidth="true" width="19.26953125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -4239,16 +4354,16 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" style="29" customWidth="1"/>
-    <col min="4" max="4" width="29.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.81640625" customWidth="1"/>
-    <col min="6" max="6" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="11" width="14.36328125" style="29" customWidth="1"/>
-    <col min="12" max="12" width="30.36328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" customWidth="true" style="29" width="17.54296875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="29.7265625"/>
+    <col min="5" max="5" customWidth="true" width="13.81640625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="14.36328125"/>
+    <col min="7" max="11" customWidth="true" style="29" width="14.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="30.36328125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="10.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -4408,17 +4523,17 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="21.81640625" style="29" customWidth="1"/>
-    <col min="2" max="2" width="16.54296875" style="29" customWidth="1"/>
-    <col min="3" max="3" width="19.90625" style="29" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" style="29" customWidth="1"/>
-    <col min="5" max="6" width="12.90625" style="29" customWidth="1"/>
-    <col min="7" max="7" width="15" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="29" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.81640625" style="29"/>
-    <col min="10" max="10" width="17.90625" style="29" customWidth="1"/>
-    <col min="11" max="11" width="14.1796875" style="29" customWidth="1"/>
-    <col min="12" max="16384" width="8.81640625" style="29"/>
+    <col min="1" max="1" customWidth="true" style="29" width="21.81640625"/>
+    <col min="2" max="2" customWidth="true" style="29" width="16.54296875"/>
+    <col min="3" max="3" customWidth="true" style="29" width="19.90625"/>
+    <col min="4" max="4" customWidth="true" style="29" width="18.81640625"/>
+    <col min="5" max="6" customWidth="true" style="29" width="12.90625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="11.90625"/>
+    <col min="9" max="9" style="29" width="8.81640625"/>
+    <col min="10" max="10" customWidth="true" style="29" width="17.90625"/>
+    <col min="11" max="11" customWidth="true" style="29" width="14.1796875"/>
+    <col min="12" max="16384" style="29" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -4594,12 +4709,12 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="42.1796875" style="29" customWidth="1"/>
-    <col min="2" max="2" width="15.81640625" style="29" customWidth="1"/>
-    <col min="3" max="3" width="17.81640625" style="29" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="15.6328125" style="29" customWidth="1"/>
-    <col min="6" max="16384" width="8.81640625" style="29"/>
+    <col min="1" max="1" customWidth="true" style="29" width="42.1796875"/>
+    <col min="2" max="2" customWidth="true" style="29" width="15.81640625"/>
+    <col min="3" max="3" customWidth="true" style="29" width="17.81640625"/>
+    <col min="4" max="4" customWidth="true" style="29" width="16.81640625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="15.6328125"/>
+    <col min="6" max="16384" style="29" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4718,28 +4833,28 @@
   <dimension ref="A1:AB6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="51.81640625" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="51.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.453125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="15.36328125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="15.36328125"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -5162,10 +5277,10 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="76.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="76.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5250,12 +5365,12 @@
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="68.08984375" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" style="29" customWidth="1"/>
-    <col min="3" max="3" width="14.81640625" style="29" customWidth="1"/>
-    <col min="4" max="4" width="11.81640625" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.1796875" style="29" customWidth="1"/>
-    <col min="6" max="16384" width="8.81640625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="68.08984375"/>
+    <col min="2" max="2" customWidth="true" style="29" width="12.54296875"/>
+    <col min="3" max="3" customWidth="true" style="29" width="14.81640625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="11.81640625"/>
+    <col min="5" max="5" customWidth="true" style="29" width="18.1796875"/>
+    <col min="6" max="16384" style="29" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5502,8 +5617,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.54296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -5543,11 +5658,11 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5597,7 +5712,7 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="21.81640625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="21.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -5702,31 +5817,31 @@
   <dimension ref="A1:AG4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="49.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="49.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="4.81640625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="9.7265625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -6031,25 +6146,25 @@
   <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.36328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="33.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.36328125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.36328125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.36328125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="15.36328125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="14.36328125"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="15.36328125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="17.54296875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30">
@@ -6633,11 +6748,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="35.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.54296875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -6721,9 +6836,9 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -6779,9 +6894,9 @@
   <dimension ref="A1:AC4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="46.6328125" customWidth="1"/>
-    <col min="5" max="5" width="6.1796875" customWidth="1"/>
-    <col min="29" max="29" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="46.6328125"/>
+    <col min="5" max="5" customWidth="true" width="6.1796875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="13.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -7079,14 +7194,14 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="63.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="63.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="10.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="19.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="15.54296875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="8" max="9" bestFit="true" customWidth="true" width="19.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -7221,24 +7336,24 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.6328125" customWidth="1"/>
-    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="7.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="17" max="17" customWidth="true" width="17.6328125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -7551,27 +7666,27 @@
   <dimension ref="A1:U13"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="44.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="44.08984375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.1796875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="9.1796875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="6.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="8.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="14.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -7946,8 +8061,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -7995,7 +8110,7 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="18.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -8056,21 +8171,21 @@
   <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="24.90625" style="29" customWidth="1"/>
-    <col min="2" max="2" width="14" style="29" customWidth="1"/>
-    <col min="3" max="3" width="11.81640625" style="29" customWidth="1"/>
-    <col min="4" max="4" width="9.54296875" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10.36328125" style="29" customWidth="1"/>
-    <col min="6" max="6" width="9.36328125" style="29" customWidth="1"/>
-    <col min="7" max="7" width="9.7265625" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.453125" style="29" customWidth="1"/>
-    <col min="9" max="9" width="8.81640625" style="29" customWidth="1"/>
-    <col min="10" max="10" width="8.08984375" style="41" customWidth="1"/>
-    <col min="11" max="11" width="10" style="29" customWidth="1"/>
-    <col min="12" max="12" width="7.81640625" style="29" customWidth="1"/>
-    <col min="13" max="13" width="9" style="29" customWidth="1"/>
-    <col min="14" max="14" width="19.453125" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.81640625" style="29"/>
+    <col min="1" max="1" customWidth="true" style="29" width="24.90625"/>
+    <col min="2" max="2" customWidth="true" style="29" width="14.0"/>
+    <col min="3" max="3" customWidth="true" style="29" width="11.81640625"/>
+    <col min="4" max="4" customWidth="true" style="29" width="9.54296875"/>
+    <col min="5" max="5" customWidth="true" style="29" width="10.36328125"/>
+    <col min="6" max="6" customWidth="true" style="29" width="9.36328125"/>
+    <col min="7" max="7" customWidth="true" style="29" width="9.7265625"/>
+    <col min="8" max="8" customWidth="true" style="29" width="10.453125"/>
+    <col min="9" max="9" customWidth="true" style="29" width="8.81640625"/>
+    <col min="10" max="10" customWidth="true" style="41" width="8.08984375"/>
+    <col min="11" max="11" customWidth="true" style="29" width="10.0"/>
+    <col min="12" max="12" customWidth="true" style="29" width="7.81640625"/>
+    <col min="13" max="13" customWidth="true" style="29" width="9.0"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="19.453125"/>
+    <col min="15" max="16384" style="29" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -8840,14 +8955,14 @@
   <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="21.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="6.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="18.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -8951,18 +9066,18 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" customWidth="1"/>
-    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.08984375" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="4" max="4" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="13" max="13" customWidth="true" width="15.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -9154,30 +9269,30 @@
   <dimension ref="A1:W4"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" style="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.453125" style="41" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7265625" style="41" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" style="41" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.7265625" style="41" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="29" customWidth="1"/>
-    <col min="9" max="9" width="16.54296875" style="29" customWidth="1"/>
-    <col min="10" max="10" width="14.08984375" style="29" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.36328125" style="41" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.36328125" style="41" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" style="29"/>
-    <col min="14" max="14" width="12.54296875" style="29" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.7265625" style="29" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.26953125" style="29" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" style="41" customWidth="1"/>
-    <col min="18" max="18" width="8.7265625" style="41" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.90625" style="29" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12" style="29" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.81640625" style="29"/>
-    <col min="22" max="22" width="10.6328125" style="29" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.90625" style="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="8.81640625" style="29"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="9.54296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="41" width="10.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="41" width="9.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="41" width="7.7265625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="41" width="10.90625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="41" width="9.453125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="41" width="7.7265625"/>
+    <col min="8" max="8" customWidth="true" style="29" width="13.0"/>
+    <col min="9" max="9" customWidth="true" style="29" width="16.54296875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="14.08984375"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="41" width="10.36328125"/>
+    <col min="12" max="12" customWidth="true" style="41" width="10.36328125"/>
+    <col min="13" max="13" style="29" width="8.81640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="12.54296875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="29" width="14.7265625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="13.26953125"/>
+    <col min="17" max="17" customWidth="true" style="41" width="11.54296875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="41" width="8.7265625"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="9.90625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="12.0"/>
+    <col min="21" max="21" style="29" width="8.81640625"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.6328125"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="13.90625"/>
+    <col min="24" max="16384" style="29" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -9431,19 +9546,19 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="19.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -9546,20 +9661,20 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="25.81640625" style="41" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="41" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" style="41" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.453125" style="41" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.1796875" style="41" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.90625" style="41"/>
+    <col min="1" max="1" customWidth="true" style="41" width="25.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="41" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="41" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="41" width="4.453125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="41" width="14.1796875"/>
+    <col min="14" max="16384" style="41" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -9685,21 +9800,21 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="20.1796875" style="41" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="41" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="17.36328125" style="41" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" style="41" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.453125" style="41" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.1796875" style="41" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.90625" style="41"/>
+    <col min="1" max="1" customWidth="true" style="41" width="20.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="41" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
+    <col min="6" max="7" customWidth="true" style="41" width="17.36328125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="41" width="15.0"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="41" width="4.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="41" width="14.1796875"/>
+    <col min="16" max="16384" style="41" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -9886,22 +10001,22 @@
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="28.36328125" style="41" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="41" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.81640625" style="41" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.08984375" style="41" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" style="41" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.08984375" style="41" customWidth="1"/>
-    <col min="13" max="13" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.90625" style="41" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.1796875" style="41" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.90625" style="41"/>
+    <col min="1" max="1" customWidth="true" style="41" width="28.36328125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="41" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="41" width="16.81640625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="41" width="11.08984375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="41" width="15.0"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
+    <col min="12" max="12" customWidth="true" style="41" width="13.08984375"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="41" width="11.90625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="41" width="14.1796875"/>
+    <col min="16" max="16384" style="41" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -10201,11 +10316,11 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="24" style="41" customWidth="1"/>
-    <col min="2" max="2" width="11.453125" style="41" customWidth="1"/>
-    <col min="3" max="3" width="8.90625" style="41"/>
-    <col min="4" max="4" width="19.6328125" style="41" customWidth="1"/>
-    <col min="5" max="16384" width="8.90625" style="41"/>
+    <col min="1" max="1" customWidth="true" style="41" width="24.0"/>
+    <col min="2" max="2" customWidth="true" style="41" width="11.453125"/>
+    <col min="3" max="3" style="41" width="8.90625"/>
+    <col min="4" max="4" customWidth="true" style="41" width="19.6328125"/>
+    <col min="5" max="16384" style="41" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -10249,12 +10364,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.1796875" style="41" customWidth="1"/>
-    <col min="2" max="2" width="14" style="41" customWidth="1"/>
-    <col min="3" max="3" width="16.6328125" style="41" customWidth="1"/>
-    <col min="4" max="4" width="17.6328125" style="41" customWidth="1"/>
-    <col min="5" max="5" width="11.81640625" style="41" customWidth="1"/>
-    <col min="6" max="16384" width="8.90625" style="41"/>
+    <col min="1" max="1" customWidth="true" style="41" width="32.1796875"/>
+    <col min="2" max="2" customWidth="true" style="41" width="14.0"/>
+    <col min="3" max="3" customWidth="true" style="41" width="16.6328125"/>
+    <col min="4" max="4" customWidth="true" style="41" width="17.6328125"/>
+    <col min="5" max="5" customWidth="true" style="41" width="11.81640625"/>
+    <col min="6" max="16384" style="41" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -10338,11 +10453,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="38.1796875" style="41" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" style="41" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" style="41" customWidth="1"/>
-    <col min="4" max="4" width="19" style="41" customWidth="1"/>
-    <col min="5" max="16384" width="8.90625" style="41"/>
+    <col min="1" max="1" customWidth="true" style="41" width="38.1796875"/>
+    <col min="2" max="2" customWidth="true" style="41" width="13.54296875"/>
+    <col min="3" max="3" customWidth="true" style="41" width="15.54296875"/>
+    <col min="4" max="4" customWidth="true" style="41" width="19.0"/>
+    <col min="5" max="16384" style="41" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -10465,21 +10580,21 @@
   <dimension ref="A1:N5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="30.90625" style="41" customWidth="1"/>
-    <col min="2" max="2" width="17.81640625" style="41" customWidth="1"/>
-    <col min="3" max="3" width="16.453125" style="41" customWidth="1"/>
-    <col min="4" max="4" width="16.08984375" style="41" customWidth="1"/>
-    <col min="5" max="5" width="12" style="41" customWidth="1"/>
-    <col min="6" max="6" width="18.08984375" style="41" customWidth="1"/>
-    <col min="7" max="7" width="15.08984375" style="41" customWidth="1"/>
-    <col min="8" max="8" width="10.453125" style="41" customWidth="1"/>
-    <col min="9" max="9" width="10.81640625" style="41" customWidth="1"/>
-    <col min="10" max="10" width="8.90625" style="41"/>
-    <col min="11" max="11" width="13.1796875" style="41" customWidth="1"/>
-    <col min="12" max="12" width="12.6328125" style="41" customWidth="1"/>
-    <col min="13" max="13" width="14.08984375" style="41" customWidth="1"/>
-    <col min="14" max="14" width="14.36328125" style="41" customWidth="1"/>
-    <col min="15" max="16384" width="8.90625" style="41"/>
+    <col min="1" max="1" customWidth="true" style="41" width="30.90625"/>
+    <col min="2" max="2" customWidth="true" style="41" width="17.81640625"/>
+    <col min="3" max="3" customWidth="true" style="41" width="16.453125"/>
+    <col min="4" max="4" customWidth="true" style="41" width="16.08984375"/>
+    <col min="5" max="5" customWidth="true" style="41" width="12.0"/>
+    <col min="6" max="6" customWidth="true" style="41" width="18.08984375"/>
+    <col min="7" max="7" customWidth="true" style="41" width="15.08984375"/>
+    <col min="8" max="8" customWidth="true" style="41" width="10.453125"/>
+    <col min="9" max="9" customWidth="true" style="41" width="10.81640625"/>
+    <col min="10" max="10" style="41" width="8.90625"/>
+    <col min="11" max="11" customWidth="true" style="41" width="13.1796875"/>
+    <col min="12" max="12" customWidth="true" style="41" width="12.6328125"/>
+    <col min="13" max="13" customWidth="true" style="41" width="14.08984375"/>
+    <col min="14" max="14" customWidth="true" style="41" width="14.36328125"/>
+    <col min="15" max="16384" style="41" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -10681,12 +10796,12 @@
   <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="16.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -11369,10 +11484,10 @@
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="57.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="57.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="15.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="4" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -11491,28 +11606,28 @@
   <dimension ref="A1:V15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="50" style="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.36328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.08984375" style="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.36328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="8.81640625" style="25"/>
-    <col min="9" max="9" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13" style="25" customWidth="1"/>
-    <col min="16" max="16" width="10.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="8.81640625" style="25"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="50.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="25" width="18.36328125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="25" width="12.08984375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="25" width="15.36328125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="25" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="25" width="9.453125"/>
+    <col min="7" max="8" style="25" width="8.81640625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="8.1796875"/>
+    <col min="15" max="15" customWidth="true" style="25" width="13.0"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="10.1796875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="25" width="9.1796875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="25" width="11.6328125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
+    <col min="23" max="16384" style="25" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -12207,29 +12322,29 @@
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="44.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="44.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.81640625"/>
+    <col min="11" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.1796875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="27" max="28" bestFit="true" customWidth="true" width="12.81640625"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="12.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -12661,10 +12776,10 @@
   <dimension ref="A1:AJ39"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="54.36328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="54.36328125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="12.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36">
@@ -12806,10 +12921,10 @@
       <c r="P2" s="44"/>
       <c r="Q2" s="44"/>
       <c r="R2" s="44" t="s">
-        <v>507</v>
+        <v>776</v>
       </c>
       <c r="S2" s="44" t="s">
-        <v>508</v>
+        <v>777</v>
       </c>
       <c r="T2" s="44"/>
       <c r="U2" s="44"/>
@@ -13578,10 +13693,10 @@
       <c r="P16" s="44"/>
       <c r="Q16" s="44"/>
       <c r="R16" s="44" t="s">
-        <v>509</v>
+        <v>743</v>
       </c>
       <c r="S16" s="44" t="s">
-        <v>510</v>
+        <v>744</v>
       </c>
       <c r="T16" s="44"/>
       <c r="U16" s="44"/>
@@ -13686,7 +13801,7 @@
       <c r="P18" s="44"/>
       <c r="Q18" s="44"/>
       <c r="R18" s="44" t="s">
-        <v>687</v>
+        <v>745</v>
       </c>
       <c r="S18" s="44"/>
       <c r="T18" s="47">
@@ -13762,7 +13877,7 @@
         <v>34</v>
       </c>
       <c r="R19" s="44" t="s">
-        <v>691</v>
+        <v>746</v>
       </c>
       <c r="S19" s="44"/>
       <c r="T19" s="47">
@@ -13838,7 +13953,7 @@
         <v>12</v>
       </c>
       <c r="R20" s="44" t="s">
-        <v>698</v>
+        <v>747</v>
       </c>
       <c r="S20" s="44"/>
       <c r="T20" s="47">
@@ -13900,7 +14015,7 @@
       <c r="P21" s="44"/>
       <c r="Q21" s="44"/>
       <c r="R21" s="44" t="s">
-        <v>700</v>
+        <v>748</v>
       </c>
       <c r="S21" s="44"/>
       <c r="T21" s="47">
@@ -14060,7 +14175,7 @@
       <c r="P24" s="44"/>
       <c r="Q24" s="44"/>
       <c r="R24" s="44" t="s">
-        <v>706</v>
+        <v>749</v>
       </c>
       <c r="S24" s="44"/>
       <c r="T24" s="47"/>
@@ -14262,7 +14377,7 @@
       <c r="P28" s="44"/>
       <c r="Q28" s="44"/>
       <c r="R28" s="44" t="s">
-        <v>714</v>
+        <v>750</v>
       </c>
       <c r="S28" s="44"/>
       <c r="T28" s="47">
@@ -14406,7 +14521,7 @@
       <c r="P30" s="44"/>
       <c r="Q30" s="44"/>
       <c r="R30" s="44" t="s">
-        <v>719</v>
+        <v>753</v>
       </c>
       <c r="S30" s="44"/>
       <c r="T30" s="44">
@@ -14462,7 +14577,7 @@
       <c r="P31" s="44"/>
       <c r="Q31" s="44"/>
       <c r="R31" s="44" t="s">
-        <v>721</v>
+        <v>756</v>
       </c>
       <c r="S31" s="44"/>
       <c r="T31" s="44">
@@ -14518,7 +14633,7 @@
       <c r="P32" s="44"/>
       <c r="Q32" s="44"/>
       <c r="R32" s="44" t="s">
-        <v>723</v>
+        <v>759</v>
       </c>
       <c r="S32" s="44"/>
       <c r="T32" s="44">
@@ -14574,7 +14689,7 @@
       <c r="P33" s="44"/>
       <c r="Q33" s="44"/>
       <c r="R33" s="44" t="s">
-        <v>725</v>
+        <v>762</v>
       </c>
       <c r="S33" s="44"/>
       <c r="T33" s="44">
@@ -14630,7 +14745,7 @@
       <c r="P34" s="44"/>
       <c r="Q34" s="44"/>
       <c r="R34" s="44" t="s">
-        <v>727</v>
+        <v>765</v>
       </c>
       <c r="S34" s="44"/>
       <c r="T34" s="44">
@@ -14686,7 +14801,7 @@
       <c r="P35" s="44"/>
       <c r="Q35" s="44"/>
       <c r="R35" s="44" t="s">
-        <v>729</v>
+        <v>768</v>
       </c>
       <c r="S35" s="44"/>
       <c r="T35" s="44">
@@ -14742,7 +14857,7 @@
       <c r="P36" s="44"/>
       <c r="Q36" s="44"/>
       <c r="R36" s="44" t="s">
-        <v>731</v>
+        <v>771</v>
       </c>
       <c r="S36" s="44"/>
       <c r="T36" s="44">
@@ -14798,7 +14913,7 @@
       <c r="P37" s="44"/>
       <c r="Q37" s="44"/>
       <c r="R37" s="44" t="s">
-        <v>733</v>
+        <v>774</v>
       </c>
       <c r="S37" s="44"/>
       <c r="T37" s="44">
@@ -14854,7 +14969,7 @@
       <c r="P38" s="44"/>
       <c r="Q38" s="44"/>
       <c r="R38" s="44" t="s">
-        <v>735</v>
+        <v>775</v>
       </c>
       <c r="S38" s="44"/>
       <c r="T38" s="44">
@@ -14912,7 +15027,7 @@
       <c r="P39" s="44"/>
       <c r="Q39" s="44"/>
       <c r="R39" s="44" t="s">
-        <v>737</v>
+        <v>778</v>
       </c>
       <c r="S39" s="44" t="s">
         <v>378</v>
@@ -14950,16 +15065,16 @@
   <dimension ref="A1:S20"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="53.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="12.1796875" customWidth="1"/>
-    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="53.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="5" max="7" customWidth="true" width="12.1796875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">

</xml_diff>

<commit_message>
Added AirSchedule from Sowmya
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{269A1528-C109-44C0-86B6-2AE2597F7E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC1A36FD-7576-43C1-8C40-D775FD8E6336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="3" activeTab="7" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="16" activeTab="18" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2434" uniqueCount="779">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2440" uniqueCount="756">
   <si>
     <t>Scenario</t>
   </si>
@@ -1597,18 +1597,6 @@
     <t>A2MQRL</t>
   </si>
   <si>
-    <t>A2MQRT</t>
-  </si>
-  <si>
-    <t>2302182807110</t>
-  </si>
-  <si>
-    <t>A2MQSH</t>
-  </si>
-  <si>
-    <t>2302182807111</t>
-  </si>
-  <si>
     <t>A2MQSV</t>
   </si>
   <si>
@@ -2137,9 +2125,6 @@
     <t>CreateBooking with 2segm, 2pax (1 FF), stored fare, 2 phones, 1 remark and ticketing</t>
   </si>
   <si>
-    <t>BAYOBS</t>
-  </si>
-  <si>
     <t>CreateBbooking with 4seg, 2pax, stored fare, 2phones,1remark, 2OSIs, 2SSRs and ticketing</t>
   </si>
   <si>
@@ -2149,9 +2134,6 @@
     <t>435</t>
   </si>
   <si>
-    <t>BAYOBT</t>
-  </si>
-  <si>
     <t xml:space="preserve"> CreateBooking with 4seg(OA), 2pax (1FF and 1inf), 1email, stored fare, 1OSI, 1remark, SeatAssignment and ticketing</t>
   </si>
   <si>
@@ -2170,15 +2152,9 @@
     <t>1916</t>
   </si>
   <si>
-    <t>BAYOBY</t>
-  </si>
-  <si>
     <t>CreateBooking with 3 seg(1ARNK),2pax(1FF),stored fare,2phones,1OSI,3remarks,SeatAssignment and ticketing</t>
   </si>
   <si>
-    <t>BAYOCO</t>
-  </si>
-  <si>
     <t>10A</t>
   </si>
   <si>
@@ -2194,9 +2170,6 @@
     <t>CreateBooking_Failure_in_one_of_the_components_of_the_system_SDS_unavailable_or_SHARES_unreachable</t>
   </si>
   <si>
-    <t>BAYOCY</t>
-  </si>
-  <si>
     <t>Invalid information specified in AirItinerary</t>
   </si>
   <si>
@@ -2218,9 +2191,6 @@
     <t>CreateBooking with 1 seg, 1 pax, stored fare (base fare, NVA date, fare calculation line, BA and tour code) and TL</t>
   </si>
   <si>
-    <t>BAYODL</t>
-  </si>
-  <si>
     <t>Bundled segment - Invalid information in one segment</t>
   </si>
   <si>
@@ -2233,63 +2203,33 @@
     <t>Stored fare - Ticketing item  Invalid tour code</t>
   </si>
   <si>
-    <t>BAYODT</t>
-  </si>
-  <si>
     <t>Stored fare - Ticketing item Invalid original issued info</t>
   </si>
   <si>
-    <t>BAYODY</t>
-  </si>
-  <si>
     <t>Stored fare - Ticketing item Invalid bankers rate info</t>
   </si>
   <si>
-    <t>BAYOEB</t>
-  </si>
-  <si>
     <t>Stored fare - Ticketing item Invalid remark</t>
   </si>
   <si>
-    <t>BAYOEH</t>
-  </si>
-  <si>
     <t>Stored fare - Ticketing item Invalid original origin destination city</t>
   </si>
   <si>
-    <t>BAYOEN</t>
-  </si>
-  <si>
     <t>Stored fare - Ticketing item Invalid form of payment</t>
   </si>
   <si>
-    <t>BAYOEZ</t>
-  </si>
-  <si>
     <t>Stored fare - Ticketing item No form of payment</t>
   </si>
   <si>
-    <t>BAYOFE</t>
-  </si>
-  <si>
     <t>Stored fare - Ticketing item too long remark</t>
   </si>
   <si>
-    <t>BAYOFS</t>
-  </si>
-  <si>
     <t>Create a booking with 1 segment, 1 passenger, stored fare, ticketing and place it on queue</t>
   </si>
   <si>
-    <t>BAYOFT</t>
-  </si>
-  <si>
     <t>CreateBooking_with_1seg_1pax_storedfare_FBC_base_fare_fare_calculation_line_and_issue_in_exchange_without_coupons_and_TL</t>
   </si>
   <si>
-    <t>BAYOFY</t>
-  </si>
-  <si>
     <t>82</t>
   </si>
   <si>
@@ -2299,12 +2239,6 @@
     <t>333</t>
   </si>
   <si>
-    <t>BA2MRK</t>
-  </si>
-  <si>
-    <t>2302182825478</t>
-  </si>
-  <si>
     <t>BA2MR4</t>
   </si>
   <si>
@@ -2329,75 +2263,27 @@
     <t>BA2MVE</t>
   </si>
   <si>
-    <t>BA2MVU</t>
-  </si>
-  <si>
-    <t>2302182825481</t>
-  </si>
-  <si>
     <t>BA2MWU</t>
   </si>
   <si>
-    <t>BA2MWX</t>
-  </si>
-  <si>
-    <t>2302182825482</t>
-  </si>
-  <si>
     <t>BA2MXM</t>
   </si>
   <si>
-    <t>BA2MXN</t>
-  </si>
-  <si>
-    <t>2302182825483</t>
-  </si>
-  <si>
     <t>BA2MXX</t>
   </si>
   <si>
-    <t>BA2MXY</t>
-  </si>
-  <si>
-    <t>2302182825484</t>
-  </si>
-  <si>
     <t>BA2MYC</t>
   </si>
   <si>
-    <t>BA2MYQ</t>
-  </si>
-  <si>
-    <t>2302182825485</t>
-  </si>
-  <si>
     <t>BA2M0R</t>
   </si>
   <si>
-    <t>BA2M02</t>
-  </si>
-  <si>
-    <t>2302182825490</t>
-  </si>
-  <si>
     <t>BA2M1O</t>
   </si>
   <si>
-    <t>BA2M1P</t>
-  </si>
-  <si>
-    <t>2302182825491</t>
-  </si>
-  <si>
     <t>BA2M2D</t>
   </si>
   <si>
-    <t>BA2M2F</t>
-  </si>
-  <si>
-    <t>2302182825492</t>
-  </si>
-  <si>
     <t>BA2M2Q</t>
   </si>
   <si>
@@ -2411,13 +2297,57 @@
   </si>
   <si>
     <t>BA2M3C</t>
+  </si>
+  <si>
+    <t>LAS</t>
+  </si>
+  <si>
+    <t>391</t>
+  </si>
+  <si>
+    <t>1031</t>
+  </si>
+  <si>
+    <t>One request  with 7 vendor preferences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other airline flight </t>
+  </si>
+  <si>
+    <t>Request missing departure date</t>
+  </si>
+  <si>
+    <t>Request missing destination location and departure date</t>
+  </si>
+  <si>
+    <t>DFW</t>
+  </si>
+  <si>
+    <t>Request missing origin location</t>
+  </si>
+  <si>
+    <t>Request with vendor preferences shows traffic restrictions as comments</t>
+  </si>
+  <si>
+    <t>Get Direct Service Display - Error showing unimplemented method</t>
+  </si>
+  <si>
+    <t>Get Flight Details - Error showing unimplemented method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multiple requests, mixed host and other airline </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Host airline, 2 leg flight </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Host airline, one leg flight </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="14">
     <font>
       <sz val="11"/>
@@ -2658,7 +2588,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2770,6 +2700,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3090,20 +3024,20 @@
   <dimension ref="A1:P15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="52.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.1796875"/>
+    <col min="1" max="1" width="52.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -3176,7 +3110,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="44" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
       <c r="I2" s="32" t="s">
         <v>211</v>
@@ -3193,7 +3127,7 @@
       <c r="M2" s="32"/>
       <c r="N2" s="32"/>
       <c r="O2" s="32" t="s">
-        <v>599</v>
+        <v>595</v>
       </c>
       <c r="P2" s="38"/>
     </row>
@@ -3265,7 +3199,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="37" t="s">
-        <v>600</v>
+        <v>596</v>
       </c>
       <c r="I4" s="37" t="s">
         <v>345</v>
@@ -3302,7 +3236,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>601</v>
+        <v>597</v>
       </c>
       <c r="I5" s="32"/>
       <c r="J5" s="32"/>
@@ -3338,15 +3272,15 @@
   <dimension ref="A1:W22"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="49.0"/>
-    <col min="10" max="10" style="25" width="8.81640625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="11.453125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="12.6328125"/>
-    <col min="22" max="23" bestFit="true" customWidth="true" width="19.26953125"/>
+    <col min="1" max="1" width="49" customWidth="1"/>
+    <col min="10" max="10" width="8.81640625" style="25"/>
+    <col min="12" max="12" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="19.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -3414,10 +3348,10 @@
         <v>257</v>
       </c>
       <c r="V1" s="43" t="s">
-        <v>612</v>
+        <v>608</v>
       </c>
       <c r="W1" s="43" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
     </row>
     <row r="2" spans="1:23">
@@ -3450,7 +3384,7 @@
       </c>
       <c r="J2" s="44"/>
       <c r="K2" s="44" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="L2" s="44"/>
       <c r="M2" s="44"/>
@@ -3489,10 +3423,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>565</v>
+        <v>561</v>
       </c>
       <c r="L3" s="44" t="s">
-        <v>566</v>
+        <v>562</v>
       </c>
       <c r="M3" s="44"/>
       <c r="N3" s="44"/>
@@ -3565,10 +3499,10 @@
       <c r="I5" s="44"/>
       <c r="J5" s="44"/>
       <c r="K5" s="44" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="L5" s="44" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="M5" s="44"/>
       <c r="N5" s="44" t="s">
@@ -3614,7 +3548,7 @@
       <c r="I6" s="44"/>
       <c r="J6" s="44"/>
       <c r="K6" s="44" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="L6" s="44"/>
       <c r="M6" s="44"/>
@@ -3625,7 +3559,7 @@
         <v>242</v>
       </c>
       <c r="P6" s="44" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="Q6" s="44"/>
       <c r="R6" s="44"/>
@@ -3661,10 +3595,10 @@
       <c r="I7" s="44"/>
       <c r="J7" s="44"/>
       <c r="K7" s="44" t="s">
-        <v>559</v>
+        <v>555</v>
       </c>
       <c r="L7" s="44" t="s">
-        <v>560</v>
+        <v>556</v>
       </c>
       <c r="M7" s="44"/>
       <c r="N7" s="44" t="s">
@@ -3674,13 +3608,13 @@
         <v>242</v>
       </c>
       <c r="P7" s="44" t="s">
-        <v>569</v>
+        <v>565</v>
       </c>
       <c r="Q7" s="47" t="s">
         <v>87</v>
       </c>
       <c r="R7" s="44" t="s">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="S7" s="44"/>
       <c r="T7" s="44"/>
@@ -3718,10 +3652,10 @@
       </c>
       <c r="J8" s="44"/>
       <c r="K8" s="44" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
       <c r="L8" s="44" t="s">
-        <v>568</v>
+        <v>564</v>
       </c>
       <c r="M8" s="44"/>
       <c r="N8" s="44" t="s">
@@ -3761,7 +3695,7 @@
       <c r="I9" s="44"/>
       <c r="J9" s="44"/>
       <c r="K9" s="44" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="L9" s="44"/>
       <c r="M9" s="44"/>
@@ -3778,7 +3712,7 @@
       <c r="T9" s="44"/>
       <c r="U9" s="44"/>
       <c r="V9" s="44" t="s">
-        <v>603</v>
+        <v>599</v>
       </c>
       <c r="W9" s="44"/>
     </row>
@@ -3804,10 +3738,10 @@
       <c r="I10" s="44"/>
       <c r="J10" s="44"/>
       <c r="K10" s="44" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="L10" s="44" t="s">
-        <v>573</v>
+        <v>569</v>
       </c>
       <c r="M10" s="44"/>
       <c r="N10" s="44"/>
@@ -3816,7 +3750,7 @@
       <c r="Q10" s="44"/>
       <c r="R10" s="44"/>
       <c r="S10" s="47" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="T10" s="44"/>
       <c r="U10" s="44"/>
@@ -3845,10 +3779,10 @@
       <c r="I11" s="44"/>
       <c r="J11" s="44"/>
       <c r="K11" s="44" t="s">
-        <v>561</v>
+        <v>557</v>
       </c>
       <c r="L11" s="44" t="s">
-        <v>562</v>
+        <v>558</v>
       </c>
       <c r="M11" s="44"/>
       <c r="N11" s="44"/>
@@ -3886,10 +3820,10 @@
       <c r="I12" s="44"/>
       <c r="J12" s="44"/>
       <c r="K12" s="44" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="L12" s="44" t="s">
-        <v>605</v>
+        <v>601</v>
       </c>
       <c r="M12" s="44"/>
       <c r="N12" s="44" t="s">
@@ -3931,10 +3865,10 @@
       <c r="I13" s="44"/>
       <c r="J13" s="44"/>
       <c r="K13" s="44" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="L13" s="44" t="s">
-        <v>607</v>
+        <v>603</v>
       </c>
       <c r="M13" s="44"/>
       <c r="N13" s="44" t="s">
@@ -4013,10 +3947,10 @@
       <c r="I15" s="44"/>
       <c r="J15" s="44"/>
       <c r="K15" s="44" t="s">
-        <v>608</v>
+        <v>604</v>
       </c>
       <c r="L15" s="44" t="s">
-        <v>609</v>
+        <v>605</v>
       </c>
       <c r="M15" s="44"/>
       <c r="N15" s="44" t="s">
@@ -4044,7 +3978,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="47" t="s">
-        <v>563</v>
+        <v>559</v>
       </c>
       <c r="D16" s="44" t="s">
         <v>12</v>
@@ -4058,7 +3992,7 @@
       <c r="I16" s="44"/>
       <c r="J16" s="44"/>
       <c r="K16" s="44" t="s">
-        <v>610</v>
+        <v>606</v>
       </c>
       <c r="L16" s="44"/>
       <c r="M16" s="44"/>
@@ -4099,7 +4033,7 @@
       <c r="I17" s="44"/>
       <c r="J17" s="44"/>
       <c r="K17" s="44" t="s">
-        <v>611</v>
+        <v>607</v>
       </c>
       <c r="L17" s="44"/>
       <c r="M17" s="44"/>
@@ -4144,7 +4078,7 @@
       </c>
       <c r="J18" s="44"/>
       <c r="K18" s="44" t="s">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="L18" s="44"/>
       <c r="M18" s="44"/>
@@ -4161,10 +4095,10 @@
       <c r="T18" s="44"/>
       <c r="U18" s="44"/>
       <c r="V18" s="44" t="s">
-        <v>614</v>
+        <v>610</v>
       </c>
       <c r="W18" s="44" t="s">
-        <v>615</v>
+        <v>611</v>
       </c>
     </row>
     <row r="19" spans="1:23">
@@ -4189,7 +4123,7 @@
       <c r="I19" s="44"/>
       <c r="J19" s="44"/>
       <c r="K19" s="44" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="L19" s="44"/>
       <c r="M19" s="44"/>
@@ -4206,7 +4140,7 @@
       <c r="T19" s="44"/>
       <c r="U19" s="44"/>
       <c r="V19" s="44" t="s">
-        <v>603</v>
+        <v>599</v>
       </c>
       <c r="W19" s="44"/>
     </row>
@@ -4232,7 +4166,7 @@
       <c r="I20" s="44"/>
       <c r="J20" s="44"/>
       <c r="K20" s="44" t="s">
-        <v>618</v>
+        <v>614</v>
       </c>
       <c r="L20" s="44"/>
       <c r="M20" s="44"/>
@@ -4259,7 +4193,7 @@
         <v>0</v>
       </c>
       <c r="C21" s="47" t="s">
-        <v>619</v>
+        <v>615</v>
       </c>
       <c r="D21" s="44" t="s">
         <v>12</v>
@@ -4273,15 +4207,15 @@
       <c r="I21" s="44"/>
       <c r="J21" s="44"/>
       <c r="K21" s="44" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="L21" s="44"/>
       <c r="M21" s="44"/>
       <c r="N21" s="44" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="O21" s="44" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
       <c r="P21" s="44"/>
       <c r="Q21" s="44"/>
@@ -4322,7 +4256,7 @@
       </c>
       <c r="J22" s="44"/>
       <c r="K22" s="44" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="L22" s="44"/>
       <c r="M22" s="44"/>
@@ -4354,16 +4288,16 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" customWidth="true" style="29" width="17.54296875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="29.7265625"/>
-    <col min="5" max="5" customWidth="true" width="13.81640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="14.36328125"/>
-    <col min="7" max="11" customWidth="true" style="29" width="14.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="30.36328125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="13.81640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="10.90625"/>
+    <col min="1" max="1" width="32.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" style="29" customWidth="1"/>
+    <col min="4" max="4" width="29.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.81640625" customWidth="1"/>
+    <col min="6" max="6" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="11" width="14.36328125" style="29" customWidth="1"/>
+    <col min="12" max="12" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -4418,14 +4352,14 @@
         <v>2</v>
       </c>
       <c r="D2" s="47" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="E2" s="47" t="s">
-        <v>578</v>
+        <v>574</v>
       </c>
       <c r="F2" s="44"/>
       <c r="G2" s="47" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="H2" s="44" t="s">
         <v>12</v>
@@ -4449,7 +4383,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="47" t="s">
-        <v>580</v>
+        <v>576</v>
       </c>
       <c r="E3" s="47" t="s">
         <v>264</v>
@@ -4458,7 +4392,7 @@
         <v>149</v>
       </c>
       <c r="G3" s="47" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="H3" s="44" t="s">
         <v>12</v>
@@ -4484,7 +4418,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="47" t="s">
-        <v>581</v>
+        <v>577</v>
       </c>
       <c r="E4" s="44"/>
       <c r="F4" s="44" t="s">
@@ -4500,7 +4434,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="47" t="s">
-        <v>577</v>
+        <v>573</v>
       </c>
       <c r="K4" s="44" t="s">
         <v>13</v>
@@ -4523,17 +4457,17 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="29" width="21.81640625"/>
-    <col min="2" max="2" customWidth="true" style="29" width="16.54296875"/>
-    <col min="3" max="3" customWidth="true" style="29" width="19.90625"/>
-    <col min="4" max="4" customWidth="true" style="29" width="18.81640625"/>
-    <col min="5" max="6" customWidth="true" style="29" width="12.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="29" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="29" width="11.90625"/>
-    <col min="9" max="9" style="29" width="8.81640625"/>
-    <col min="10" max="10" customWidth="true" style="29" width="17.90625"/>
-    <col min="11" max="11" customWidth="true" style="29" width="14.1796875"/>
-    <col min="12" max="16384" style="29" width="8.81640625"/>
+    <col min="1" max="1" width="21.81640625" style="29" customWidth="1"/>
+    <col min="2" max="2" width="16.54296875" style="29" customWidth="1"/>
+    <col min="3" max="3" width="19.90625" style="29" customWidth="1"/>
+    <col min="4" max="4" width="18.81640625" style="29" customWidth="1"/>
+    <col min="5" max="6" width="12.90625" style="29" customWidth="1"/>
+    <col min="7" max="7" width="15" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="29" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.81640625" style="29"/>
+    <col min="10" max="10" width="17.90625" style="29" customWidth="1"/>
+    <col min="11" max="11" width="14.1796875" style="29" customWidth="1"/>
+    <col min="12" max="16384" width="8.81640625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -4654,13 +4588,13 @@
         <v>12</v>
       </c>
       <c r="I5" s="44" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="J5" s="44" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4689,10 +4623,10 @@
         <v>12</v>
       </c>
       <c r="I6" s="44" t="s">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="J6" s="44" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="K6" s="44"/>
     </row>
@@ -4709,12 +4643,12 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="29" width="42.1796875"/>
-    <col min="2" max="2" customWidth="true" style="29" width="15.81640625"/>
-    <col min="3" max="3" customWidth="true" style="29" width="17.81640625"/>
-    <col min="4" max="4" customWidth="true" style="29" width="16.81640625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="15.6328125"/>
-    <col min="6" max="16384" style="29" width="8.81640625"/>
+    <col min="1" max="1" width="42.1796875" style="29" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" style="29" customWidth="1"/>
+    <col min="3" max="3" width="17.81640625" style="29" customWidth="1"/>
+    <col min="4" max="4" width="16.81640625" style="29" customWidth="1"/>
+    <col min="5" max="5" width="15.6328125" style="29" customWidth="1"/>
+    <col min="6" max="16384" width="8.81640625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4833,28 +4767,28 @@
   <dimension ref="A1:AB6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="51.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="14.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="51.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -4972,16 +4906,16 @@
         <v>45</v>
       </c>
       <c r="J2" s="44" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="K2" s="44" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="L2" s="44" t="s">
         <v>207</v>
       </c>
       <c r="M2" s="44" t="s">
-        <v>595</v>
+        <v>591</v>
       </c>
       <c r="N2" s="44" t="s">
         <v>208</v>
@@ -4990,13 +4924,13 @@
         <v>12</v>
       </c>
       <c r="P2" s="44" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="Q2" s="44" t="s">
         <v>62</v>
       </c>
       <c r="R2" s="44" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="S2" s="44" t="s">
         <v>12</v>
@@ -5042,7 +4976,7 @@
         <v>45</v>
       </c>
       <c r="J3" s="44" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
       <c r="K3" s="44" t="s">
         <v>495</v>
@@ -5060,13 +4994,13 @@
         <v>12</v>
       </c>
       <c r="P3" s="44" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="Q3" s="44" t="s">
         <v>239</v>
       </c>
       <c r="R3" s="44" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
       <c r="S3" s="44" t="s">
         <v>12</v>
@@ -5120,16 +5054,16 @@
       <c r="H4" s="44"/>
       <c r="I4" s="44"/>
       <c r="J4" s="44" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="K4" s="44" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="L4" s="44" t="s">
         <v>322</v>
       </c>
       <c r="M4" s="44" t="s">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="N4" s="44" t="s">
         <v>209</v>
@@ -5172,16 +5106,16 @@
       <c r="H5" s="44"/>
       <c r="I5" s="44"/>
       <c r="J5" s="44" t="s">
-        <v>531</v>
+        <v>527</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="L5" s="44" t="s">
         <v>322</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="N5" s="44" t="s">
         <v>209</v>
@@ -5232,16 +5166,16 @@
         <v>45</v>
       </c>
       <c r="J6" s="44" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="K6" s="44" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="L6" s="44" t="s">
         <v>207</v>
       </c>
       <c r="M6" s="44" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="N6" s="44" t="s">
         <v>208</v>
@@ -5277,10 +5211,10 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="76.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="76.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5365,12 +5299,12 @@
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="68.08984375"/>
-    <col min="2" max="2" customWidth="true" style="29" width="12.54296875"/>
-    <col min="3" max="3" customWidth="true" style="29" width="14.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="29" width="11.81640625"/>
-    <col min="5" max="5" customWidth="true" style="29" width="18.1796875"/>
-    <col min="6" max="16384" style="29" width="8.81640625"/>
+    <col min="1" max="1" width="68.08984375" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" style="29" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" style="29" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" style="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.1796875" style="29" customWidth="1"/>
+    <col min="6" max="16384" width="8.81640625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5617,8 +5551,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.54296875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -5658,11 +5592,11 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5709,27 +5643,55 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="21.81640625"/>
+    <col min="1" max="1" width="61.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:13" s="72" customFormat="1">
       <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="42" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="42" t="s">
+      <c r="B1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="45" t="s">
         <v>72</v>
       </c>
-      <c r="D1" s="42" t="s">
+      <c r="D1" s="45" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="45" t="s">
+        <v>72</v>
+      </c>
+      <c r="H1" s="45" t="s">
+        <v>73</v>
+      </c>
+      <c r="I1" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="45" t="s">
+        <v>72</v>
+      </c>
+      <c r="L1" s="45" t="s">
+        <v>73</v>
+      </c>
+      <c r="M1" s="45" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="22" t="s">
         <v>184</v>
       </c>
@@ -5742,8 +5704,17 @@
       <c r="D2" s="44" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="22" t="s">
         <v>185</v>
       </c>
@@ -5756,8 +5727,17 @@
       <c r="D3" s="44" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="22" t="s">
         <v>186</v>
       </c>
@@ -5770,42 +5750,288 @@
       <c r="D4" s="44" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="B8" s="29">
-        <v>1</v>
-      </c>
-      <c r="C8" s="29" t="s">
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="44"/>
+      <c r="H4" s="44"/>
+      <c r="I4" s="44"/>
+      <c r="J4" s="44"/>
+      <c r="K4" s="44"/>
+      <c r="L4" s="44"/>
+      <c r="M4" s="44"/>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="22" t="s">
+        <v>751</v>
+      </c>
+      <c r="B5" s="44">
+        <v>1</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="44" t="s">
+        <v>741</v>
+      </c>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="44"/>
+      <c r="M5" s="44"/>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="22" t="s">
+        <v>752</v>
+      </c>
+      <c r="B6" s="44">
+        <v>1</v>
+      </c>
+      <c r="C6" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="44"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="44"/>
+      <c r="L6" s="44"/>
+      <c r="M6" s="44"/>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="22" t="s">
+        <v>754</v>
+      </c>
+      <c r="B7" s="44">
+        <v>1</v>
+      </c>
+      <c r="C7" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="44" t="s">
         <v>209</v>
       </c>
-      <c r="D8" s="29" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="B9" s="29">
-        <v>2</v>
-      </c>
-      <c r="C9" s="29" t="s">
+      <c r="E7" s="47" t="s">
+        <v>742</v>
+      </c>
+      <c r="F7" s="44"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="44"/>
+      <c r="M7" s="44"/>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="22" t="s">
+        <v>755</v>
+      </c>
+      <c r="B8" s="44">
+        <v>1</v>
+      </c>
+      <c r="C8" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="47" t="s">
+        <v>330</v>
+      </c>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44"/>
+      <c r="M8" s="44"/>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="22" t="s">
+        <v>753</v>
+      </c>
+      <c r="B9" s="44">
+        <v>1</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="44" t="s">
+        <v>338</v>
+      </c>
+      <c r="E9" s="47" t="s">
+        <v>449</v>
+      </c>
+      <c r="F9" s="44">
+        <v>1</v>
+      </c>
+      <c r="G9" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="44" t="s">
         <v>209</v>
       </c>
-      <c r="D9" s="29" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="B10" s="29">
-        <v>0</v>
-      </c>
-      <c r="C10" s="29" t="s">
-        <v>209</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>12</v>
-      </c>
+      <c r="I9" s="47" t="s">
+        <v>742</v>
+      </c>
+      <c r="J9" s="44">
+        <v>1</v>
+      </c>
+      <c r="K9" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="L9" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="M9" s="47" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="22" t="s">
+        <v>744</v>
+      </c>
+      <c r="B10" s="44">
+        <v>1</v>
+      </c>
+      <c r="C10" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="44" t="s">
+        <v>741</v>
+      </c>
+      <c r="E10" s="44"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="44"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="44"/>
+      <c r="M10" s="44"/>
+    </row>
+    <row r="11" spans="1:13">
+      <c r="A11" s="22" t="s">
+        <v>745</v>
+      </c>
+      <c r="B11" s="44">
+        <v>1</v>
+      </c>
+      <c r="C11" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="E11" s="47" t="s">
+        <v>615</v>
+      </c>
+      <c r="F11" s="44"/>
+      <c r="G11" s="44"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+      <c r="K11" s="44"/>
+      <c r="L11" s="44"/>
+      <c r="M11" s="44"/>
+    </row>
+    <row r="12" spans="1:13">
+      <c r="A12" s="22" t="s">
+        <v>746</v>
+      </c>
+      <c r="B12" s="44"/>
+      <c r="C12" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="44"/>
+      <c r="L12" s="44"/>
+      <c r="M12" s="44"/>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="A13" s="22" t="s">
+        <v>747</v>
+      </c>
+      <c r="B13" s="44"/>
+      <c r="C13" s="44" t="s">
+        <v>748</v>
+      </c>
+      <c r="D13" s="44"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" s="71" t="s">
+        <v>749</v>
+      </c>
+      <c r="B14" s="44">
+        <v>1</v>
+      </c>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
+      <c r="L14" s="44"/>
+      <c r="M14" s="44"/>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15" s="22" t="s">
+        <v>750</v>
+      </c>
+      <c r="B15" s="44">
+        <v>1</v>
+      </c>
+      <c r="C15" s="44" t="s">
+        <v>652</v>
+      </c>
+      <c r="D15" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="44"/>
+      <c r="L15" s="44"/>
+      <c r="M15" s="44"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5817,31 +6043,31 @@
   <dimension ref="A1:AG4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="49.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="4.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="9.7265625"/>
+    <col min="1" max="1" width="49.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -6146,25 +6372,25 @@
   <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="33.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.36328125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.36328125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="14.36328125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="1" max="1" width="33" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30">
@@ -6283,16 +6509,16 @@
       <c r="I2" s="44"/>
       <c r="J2" s="44"/>
       <c r="K2" s="44" t="s">
-        <v>532</v>
+        <v>528</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>319</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>209</v>
@@ -6347,7 +6573,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>535</v>
+        <v>531</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>312</v>
@@ -6487,16 +6713,16 @@
         <v>2</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>319</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>209</v>
@@ -6505,7 +6731,7 @@
         <v>12</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
       <c r="R5" s="15" t="s">
         <v>44</v>
@@ -6748,11 +6974,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="35.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.54296875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="1" max="1" width="35.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -6836,9 +7062,9 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.90625"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -6894,9 +7120,9 @@
   <dimension ref="A1:AC4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="46.6328125"/>
-    <col min="5" max="5" customWidth="true" width="6.1796875"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="1" max="1" width="46.6328125" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" customWidth="1"/>
+    <col min="29" max="29" width="13.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -7024,16 +7250,16 @@
       <c r="U2" s="44"/>
       <c r="V2" s="44"/>
       <c r="W2" s="44" t="s">
-        <v>538</v>
+        <v>534</v>
       </c>
       <c r="X2" s="44" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="Y2" s="44" t="s">
         <v>319</v>
       </c>
       <c r="Z2" s="44" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="AA2" s="44" t="s">
         <v>209</v>
@@ -7042,7 +7268,7 @@
         <v>12</v>
       </c>
       <c r="AC2" s="44" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
     </row>
     <row r="3" spans="1:29">
@@ -7160,16 +7386,16 @@
       <c r="U4" s="44"/>
       <c r="V4" s="44"/>
       <c r="W4" s="44" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
       <c r="X4" s="44" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="Y4" s="44" t="s">
         <v>319</v>
       </c>
       <c r="Z4" s="44" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="AA4" s="44" t="s">
         <v>209</v>
@@ -7178,7 +7404,7 @@
         <v>12</v>
       </c>
       <c r="AC4" s="44" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
     </row>
   </sheetData>
@@ -7194,14 +7420,14 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="63.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="10.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="19.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="15.54296875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="8" max="9" bestFit="true" customWidth="true" width="19.453125"/>
+    <col min="1" max="1" width="63.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="19.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -7336,24 +7562,24 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.81640625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="7.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="17" max="17" customWidth="true" width="17.6328125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.6328125" customWidth="1"/>
+    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -7436,16 +7662,16 @@
       <c r="I2" s="44"/>
       <c r="J2" s="44"/>
       <c r="K2" s="44" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="L2" s="44" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="M2" s="44" t="s">
         <v>18</v>
       </c>
       <c r="N2" s="44" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="O2" s="44" t="s">
         <v>12</v>
@@ -7454,7 +7680,7 @@
         <v>13</v>
       </c>
       <c r="Q2" s="44" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="R2" s="44"/>
     </row>
@@ -7482,16 +7708,16 @@
       <c r="I3" s="44"/>
       <c r="J3" s="44"/>
       <c r="K3" s="44" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="L3" s="44" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="M3" s="44" t="s">
         <v>18</v>
       </c>
       <c r="N3" s="44" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="O3" s="44" t="s">
         <v>12</v>
@@ -7500,10 +7726,10 @@
         <v>13</v>
       </c>
       <c r="Q3" s="44" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="R3" s="44" t="s">
-        <v>591</v>
+        <v>587</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -7538,16 +7764,16 @@
         <v>2</v>
       </c>
       <c r="K4" s="44" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="L4" s="44" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="M4" s="44" t="s">
         <v>18</v>
       </c>
       <c r="N4" s="44" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="O4" s="44" t="s">
         <v>12</v>
@@ -7556,7 +7782,7 @@
         <v>13</v>
       </c>
       <c r="Q4" s="44" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="R4" s="44"/>
     </row>
@@ -7584,16 +7810,16 @@
       <c r="I5" s="44"/>
       <c r="J5" s="44"/>
       <c r="K5" s="44" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="L5" s="44" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="M5" s="44" t="s">
         <v>18</v>
       </c>
       <c r="N5" s="44" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="O5" s="44" t="s">
         <v>12</v>
@@ -7602,7 +7828,7 @@
         <v>13</v>
       </c>
       <c r="Q5" s="44" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="R5" s="44"/>
     </row>
@@ -7630,16 +7856,16 @@
       <c r="I6" s="44"/>
       <c r="J6" s="44"/>
       <c r="K6" s="44" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="L6" s="44" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="M6" s="44" t="s">
         <v>18</v>
       </c>
       <c r="N6" s="44" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="O6" s="44" t="s">
         <v>12</v>
@@ -7648,7 +7874,7 @@
         <v>13</v>
       </c>
       <c r="Q6" s="44" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="R6" s="44"/>
     </row>
@@ -7666,27 +7892,27 @@
   <dimension ref="A1:U13"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="44.08984375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.1796875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.1796875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="8.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="14.08984375"/>
+    <col min="1" max="1" width="44.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -7783,16 +8009,16 @@
         <v>163</v>
       </c>
       <c r="J2" s="56" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="K2" s="44" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>215</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>12</v>
@@ -7801,13 +8027,13 @@
         <v>216</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>217</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>216</v>
@@ -7816,7 +8042,7 @@
         <v>163</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -7848,16 +8074,16 @@
         <v>163</v>
       </c>
       <c r="J3" s="56" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>215</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>12</v>
@@ -7866,13 +8092,13 @@
         <v>216</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
       <c r="Q3" s="3" t="s">
         <v>335</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>550</v>
+        <v>546</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>216</v>
@@ -7881,7 +8107,7 @@
         <v>163</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -8061,8 +8287,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -8110,7 +8336,7 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="18.0"/>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -8171,21 +8397,21 @@
   <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="29" width="24.90625"/>
-    <col min="2" max="2" customWidth="true" style="29" width="14.0"/>
-    <col min="3" max="3" customWidth="true" style="29" width="11.81640625"/>
-    <col min="4" max="4" customWidth="true" style="29" width="9.54296875"/>
-    <col min="5" max="5" customWidth="true" style="29" width="10.36328125"/>
-    <col min="6" max="6" customWidth="true" style="29" width="9.36328125"/>
-    <col min="7" max="7" customWidth="true" style="29" width="9.7265625"/>
-    <col min="8" max="8" customWidth="true" style="29" width="10.453125"/>
-    <col min="9" max="9" customWidth="true" style="29" width="8.81640625"/>
-    <col min="10" max="10" customWidth="true" style="41" width="8.08984375"/>
-    <col min="11" max="11" customWidth="true" style="29" width="10.0"/>
-    <col min="12" max="12" customWidth="true" style="29" width="7.81640625"/>
-    <col min="13" max="13" customWidth="true" style="29" width="9.0"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="19.453125"/>
-    <col min="15" max="16384" style="29" width="8.81640625"/>
+    <col min="1" max="1" width="24.90625" style="29" customWidth="1"/>
+    <col min="2" max="2" width="14" style="29" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" style="29" customWidth="1"/>
+    <col min="4" max="4" width="9.54296875" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10.36328125" style="29" customWidth="1"/>
+    <col min="6" max="6" width="9.36328125" style="29" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" style="29" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" style="29" customWidth="1"/>
+    <col min="9" max="9" width="8.81640625" style="29" customWidth="1"/>
+    <col min="10" max="10" width="8.08984375" style="41" customWidth="1"/>
+    <col min="11" max="11" width="10" style="29" customWidth="1"/>
+    <col min="12" max="12" width="7.81640625" style="29" customWidth="1"/>
+    <col min="13" max="13" width="9" style="29" customWidth="1"/>
+    <col min="14" max="14" width="19.453125" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.81640625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -8955,14 +9181,14 @@
   <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="21.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="6.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -9066,18 +9292,18 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="4" max="4" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" customWidth="true" width="15.08984375"/>
+    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" customWidth="1"/>
+    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -9250,7 +9476,7 @@
       <c r="H6" s="44"/>
       <c r="I6" s="44"/>
       <c r="J6" s="44" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="K6" s="44"/>
       <c r="L6" s="44"/>
@@ -9269,30 +9495,30 @@
   <dimension ref="A1:W4"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="29" width="9.54296875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="41" width="10.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="41" width="9.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="41" width="7.7265625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="41" width="10.90625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="41" width="9.453125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="41" width="7.7265625"/>
-    <col min="8" max="8" customWidth="true" style="29" width="13.0"/>
-    <col min="9" max="9" customWidth="true" style="29" width="16.54296875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="29" width="14.08984375"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="41" width="10.36328125"/>
-    <col min="12" max="12" customWidth="true" style="41" width="10.36328125"/>
-    <col min="13" max="13" style="29" width="8.81640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="29" width="12.54296875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="29" width="14.7265625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="29" width="13.26953125"/>
-    <col min="17" max="17" customWidth="true" style="41" width="11.54296875"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" style="41" width="8.7265625"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="29" width="9.90625"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="29" width="12.0"/>
-    <col min="21" max="21" style="29" width="8.81640625"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="29" width="10.6328125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="29" width="13.90625"/>
-    <col min="24" max="16384" style="29" width="8.81640625"/>
+    <col min="1" max="1" width="9.54296875" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.453125" style="41" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7265625" style="41" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" style="41" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.7265625" style="41" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" style="29" customWidth="1"/>
+    <col min="9" max="9" width="16.54296875" style="29" customWidth="1"/>
+    <col min="10" max="10" width="14.08984375" style="29" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.36328125" style="41" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" style="29"/>
+    <col min="14" max="14" width="12.54296875" style="29" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.7265625" style="29" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.26953125" style="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" style="41" customWidth="1"/>
+    <col min="18" max="18" width="8.7265625" style="41" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.90625" style="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12" style="29" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.81640625" style="29"/>
+    <col min="22" max="22" width="10.6328125" style="29" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.90625" style="29" bestFit="1" customWidth="1"/>
+    <col min="24" max="16384" width="8.81640625" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -9303,7 +9529,7 @@
         <v>56</v>
       </c>
       <c r="C1" s="45" t="s">
-        <v>628</v>
+        <v>624</v>
       </c>
       <c r="D1" s="45" t="s">
         <v>28</v>
@@ -9312,55 +9538,55 @@
         <v>56</v>
       </c>
       <c r="F1" s="45" t="s">
-        <v>628</v>
+        <v>624</v>
       </c>
       <c r="G1" s="45" t="s">
         <v>28</v>
       </c>
       <c r="H1" s="33" t="s">
-        <v>626</v>
+        <v>622</v>
       </c>
       <c r="I1" s="33" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="J1" s="33" t="s">
         <v>142</v>
       </c>
       <c r="K1" s="45" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="L1" s="45" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="M1" s="65" t="s">
         <v>74</v>
       </c>
       <c r="N1" s="66" t="s">
+        <v>627</v>
+      </c>
+      <c r="O1" s="66" t="s">
+        <v>628</v>
+      </c>
+      <c r="P1" s="66" t="s">
+        <v>629</v>
+      </c>
+      <c r="Q1" s="66" t="s">
+        <v>630</v>
+      </c>
+      <c r="R1" s="66" t="s">
         <v>631</v>
       </c>
-      <c r="O1" s="66" t="s">
+      <c r="S1" s="33" t="s">
+        <v>637</v>
+      </c>
+      <c r="T1" s="33" t="s">
+        <v>638</v>
+      </c>
+      <c r="U1" s="65" t="s">
         <v>632</v>
       </c>
-      <c r="P1" s="66" t="s">
+      <c r="V1" s="65" t="s">
         <v>633</v>
-      </c>
-      <c r="Q1" s="66" t="s">
-        <v>634</v>
-      </c>
-      <c r="R1" s="66" t="s">
-        <v>635</v>
-      </c>
-      <c r="S1" s="33" t="s">
-        <v>641</v>
-      </c>
-      <c r="T1" s="33" t="s">
-        <v>642</v>
-      </c>
-      <c r="U1" s="65" t="s">
-        <v>636</v>
-      </c>
-      <c r="V1" s="65" t="s">
-        <v>637</v>
       </c>
       <c r="W1" s="43" t="s">
         <v>195</v>
@@ -9404,7 +9630,7 @@
         <v>14</v>
       </c>
       <c r="M2" s="32" t="s">
-        <v>640</v>
+        <v>636</v>
       </c>
       <c r="N2" s="32">
         <v>2</v>
@@ -9424,10 +9650,10 @@
       <c r="S2" s="32"/>
       <c r="T2" s="32"/>
       <c r="U2" s="44" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="V2" s="44" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="W2" s="44" t="s">
         <v>378</v>
@@ -9471,7 +9697,7 @@
         <v>14</v>
       </c>
       <c r="M3" s="32" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="N3" s="32"/>
       <c r="O3" s="32"/>
@@ -9485,13 +9711,13 @@
         <v>317</v>
       </c>
       <c r="U3" s="44" t="s">
-        <v>643</v>
+        <v>639</v>
       </c>
       <c r="V3" s="44" t="s">
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="W3" s="44" t="s">
-        <v>646</v>
+        <v>642</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -9520,7 +9746,7 @@
         <v>14</v>
       </c>
       <c r="M4" s="32" t="s">
-        <v>625</v>
+        <v>621</v>
       </c>
       <c r="N4" s="32"/>
       <c r="O4" s="32"/>
@@ -9546,19 +9772,19 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="19.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="1" max="1" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -9661,20 +9887,20 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="25.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="41" width="4.453125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="41" width="14.1796875"/>
-    <col min="14" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="25.81640625" style="41" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" style="41" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.1796875" style="41" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -9800,21 +10026,21 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="20.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="6" max="7" customWidth="true" style="41" width="17.36328125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="41" width="4.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="41" width="14.1796875"/>
-    <col min="16" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="20.1796875" style="41" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="17.36328125" style="41" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.453125" style="41" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.1796875" style="41" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -10001,22 +10227,22 @@
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="28.36328125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="41" width="16.81640625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="41" width="11.08984375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="41" width="15.0"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="12" max="12" customWidth="true" style="41" width="13.08984375"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="41" width="17.36328125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="41" width="11.90625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="41" width="14.1796875"/>
-    <col min="16" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="28.36328125" style="41" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.81640625" style="41" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.08984375" style="41" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="41" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.08984375" style="41" customWidth="1"/>
+    <col min="13" max="13" width="17.36328125" style="41" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.90625" style="41" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.1796875" style="41" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -10131,7 +10357,7 @@
       </c>
       <c r="G4" s="44"/>
       <c r="H4" s="44" t="s">
-        <v>623</v>
+        <v>619</v>
       </c>
       <c r="I4" s="44" t="s">
         <v>381</v>
@@ -10168,7 +10394,7 @@
       </c>
       <c r="G5" s="44"/>
       <c r="H5" s="44" t="s">
-        <v>624</v>
+        <v>620</v>
       </c>
       <c r="I5" s="44" t="s">
         <v>381</v>
@@ -10316,11 +10542,11 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="24.0"/>
-    <col min="2" max="2" customWidth="true" style="41" width="11.453125"/>
-    <col min="3" max="3" style="41" width="8.90625"/>
-    <col min="4" max="4" customWidth="true" style="41" width="19.6328125"/>
-    <col min="5" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="24" style="41" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" style="41" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" style="41"/>
+    <col min="4" max="4" width="19.6328125" style="41" customWidth="1"/>
+    <col min="5" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -10364,12 +10590,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="32.1796875"/>
-    <col min="2" max="2" customWidth="true" style="41" width="14.0"/>
-    <col min="3" max="3" customWidth="true" style="41" width="16.6328125"/>
-    <col min="4" max="4" customWidth="true" style="41" width="17.6328125"/>
-    <col min="5" max="5" customWidth="true" style="41" width="11.81640625"/>
-    <col min="6" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="32.1796875" style="41" customWidth="1"/>
+    <col min="2" max="2" width="14" style="41" customWidth="1"/>
+    <col min="3" max="3" width="16.6328125" style="41" customWidth="1"/>
+    <col min="4" max="4" width="17.6328125" style="41" customWidth="1"/>
+    <col min="5" max="5" width="11.81640625" style="41" customWidth="1"/>
+    <col min="6" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -10453,11 +10679,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="38.1796875"/>
-    <col min="2" max="2" customWidth="true" style="41" width="13.54296875"/>
-    <col min="3" max="3" customWidth="true" style="41" width="15.54296875"/>
-    <col min="4" max="4" customWidth="true" style="41" width="19.0"/>
-    <col min="5" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="38.1796875" style="41" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" style="41" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" style="41" customWidth="1"/>
+    <col min="4" max="4" width="19" style="41" customWidth="1"/>
+    <col min="5" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -10580,21 +10806,21 @@
   <dimension ref="A1:N5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="41" width="30.90625"/>
-    <col min="2" max="2" customWidth="true" style="41" width="17.81640625"/>
-    <col min="3" max="3" customWidth="true" style="41" width="16.453125"/>
-    <col min="4" max="4" customWidth="true" style="41" width="16.08984375"/>
-    <col min="5" max="5" customWidth="true" style="41" width="12.0"/>
-    <col min="6" max="6" customWidth="true" style="41" width="18.08984375"/>
-    <col min="7" max="7" customWidth="true" style="41" width="15.08984375"/>
-    <col min="8" max="8" customWidth="true" style="41" width="10.453125"/>
-    <col min="9" max="9" customWidth="true" style="41" width="10.81640625"/>
-    <col min="10" max="10" style="41" width="8.90625"/>
-    <col min="11" max="11" customWidth="true" style="41" width="13.1796875"/>
-    <col min="12" max="12" customWidth="true" style="41" width="12.6328125"/>
-    <col min="13" max="13" customWidth="true" style="41" width="14.08984375"/>
-    <col min="14" max="14" customWidth="true" style="41" width="14.36328125"/>
-    <col min="15" max="16384" style="41" width="8.90625"/>
+    <col min="1" max="1" width="30.90625" style="41" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" style="41" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" style="41" customWidth="1"/>
+    <col min="4" max="4" width="16.08984375" style="41" customWidth="1"/>
+    <col min="5" max="5" width="12" style="41" customWidth="1"/>
+    <col min="6" max="6" width="18.08984375" style="41" customWidth="1"/>
+    <col min="7" max="7" width="15.08984375" style="41" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" style="41" customWidth="1"/>
+    <col min="9" max="9" width="10.81640625" style="41" customWidth="1"/>
+    <col min="10" max="10" width="8.90625" style="41"/>
+    <col min="11" max="11" width="13.1796875" style="41" customWidth="1"/>
+    <col min="12" max="12" width="12.6328125" style="41" customWidth="1"/>
+    <col min="13" max="13" width="14.08984375" style="41" customWidth="1"/>
+    <col min="14" max="14" width="14.36328125" style="41" customWidth="1"/>
+    <col min="15" max="16384" width="8.90625" style="41"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -10670,7 +10896,7 @@
         <v>212</v>
       </c>
       <c r="J2" s="44" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="K2" s="44">
         <v>2</v>
@@ -10796,12 +11022,12 @@
   <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="16.08984375"/>
+    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -10821,19 +11047,19 @@
         <v>40</v>
       </c>
       <c r="F1" s="45" t="s">
+        <v>643</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>644</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>645</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>646</v>
+      </c>
+      <c r="J1" s="12" t="s">
         <v>647</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>648</v>
-      </c>
-      <c r="H1" s="12" t="s">
-        <v>649</v>
-      </c>
-      <c r="I1" s="12" t="s">
-        <v>650</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>651</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -10882,7 +11108,7 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="44" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
       <c r="B4" s="44">
         <v>1</v>
@@ -10902,7 +11128,7 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="44" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="B5" s="44">
         <v>1</v>
@@ -10912,7 +11138,7 @@
         <v>34</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="F5" s="44"/>
       <c r="G5" s="44"/>
@@ -10922,7 +11148,7 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="44" t="s">
-        <v>655</v>
+        <v>651</v>
       </c>
       <c r="B6" s="44">
         <v>1</v>
@@ -10932,13 +11158,13 @@
         <v>34</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="F6" s="44">
         <v>2</v>
       </c>
       <c r="G6" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="H6" s="44" t="s">
         <v>34</v>
@@ -10948,7 +11174,7 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="44" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="B7" s="44">
         <v>1</v>
@@ -10958,13 +11184,13 @@
         <v>34</v>
       </c>
       <c r="E7" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="F7" s="44">
         <v>2</v>
       </c>
       <c r="G7" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="H7" s="44" t="s">
         <v>34</v>
@@ -10974,7 +11200,7 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="44" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="B8" s="44">
         <v>1</v>
@@ -10984,13 +11210,13 @@
         <v>34</v>
       </c>
       <c r="E8" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="F8" s="44">
         <v>2</v>
       </c>
       <c r="G8" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="H8" s="44" t="s">
         <v>34</v>
@@ -11000,7 +11226,7 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="44" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="B9" s="44">
         <v>1</v>
@@ -11010,25 +11236,25 @@
         <v>34</v>
       </c>
       <c r="E9" s="44" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="F9" s="44">
         <v>2</v>
       </c>
       <c r="G9" s="44" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="H9" s="44" t="s">
         <v>34</v>
       </c>
       <c r="I9" s="47" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="J9" s="44"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="44" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="B10" s="44">
         <v>1</v>
@@ -11038,7 +11264,7 @@
         <v>34</v>
       </c>
       <c r="E10" s="44" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="F10" s="44"/>
       <c r="G10" s="44"/>
@@ -11048,7 +11274,7 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="44" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="B11" s="44">
         <v>1</v>
@@ -11058,13 +11284,13 @@
         <v>34</v>
       </c>
       <c r="E11" s="44" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="F11" s="44">
         <v>2</v>
       </c>
       <c r="G11" s="44" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="H11" s="44" t="s">
         <v>34</v>
@@ -11074,7 +11300,7 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="44" t="s">
-        <v>664</v>
+        <v>660</v>
       </c>
       <c r="B12" s="44">
         <v>1</v>
@@ -11084,13 +11310,13 @@
         <v>34</v>
       </c>
       <c r="E12" s="44" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="F12" s="44">
         <v>2</v>
       </c>
       <c r="G12" s="44" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="H12" s="44" t="s">
         <v>34</v>
@@ -11100,7 +11326,7 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="44" t="s">
-        <v>665</v>
+        <v>661</v>
       </c>
       <c r="B13" s="44">
         <v>1</v>
@@ -11110,19 +11336,19 @@
         <v>34</v>
       </c>
       <c r="E13" s="44" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="F13" s="44"/>
       <c r="G13" s="44"/>
       <c r="H13" s="44"/>
       <c r="I13" s="44"/>
       <c r="J13" s="44" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="44" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="B14" s="44">
         <v>1</v>
@@ -11132,7 +11358,7 @@
         <v>34</v>
       </c>
       <c r="E14" s="44" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="F14" s="44"/>
       <c r="G14" s="44"/>
@@ -11142,7 +11368,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="44" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="B15" s="44">
         <v>1</v>
@@ -11152,13 +11378,13 @@
         <v>34</v>
       </c>
       <c r="E15" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="F15" s="44">
         <v>2</v>
       </c>
       <c r="G15" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="H15" s="44" t="s">
         <v>34</v>
@@ -11168,7 +11394,7 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="44" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="B16" s="44">
         <v>1</v>
@@ -11178,13 +11404,13 @@
         <v>34</v>
       </c>
       <c r="E16" s="44" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="F16" s="44">
         <v>2</v>
       </c>
       <c r="G16" s="44" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="H16" s="44" t="s">
         <v>34</v>
@@ -11194,7 +11420,7 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="44" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="B17" s="44">
         <v>1</v>
@@ -11204,13 +11430,13 @@
         <v>34</v>
       </c>
       <c r="E17" s="44" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="F17" s="44">
         <v>2</v>
       </c>
       <c r="G17" s="44" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="H17" s="44" t="s">
         <v>34</v>
@@ -11220,7 +11446,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="44" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
       <c r="B18" s="44">
         <v>1</v>
@@ -11230,13 +11456,13 @@
         <v>34</v>
       </c>
       <c r="E18" s="44" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="F18" s="44">
         <v>2</v>
       </c>
       <c r="G18" s="44" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="H18" s="44" t="s">
         <v>34</v>
@@ -11246,7 +11472,7 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="44" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="B19" s="44">
         <v>1</v>
@@ -11264,7 +11490,7 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="44" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="B20" s="44">
         <v>1</v>
@@ -11272,7 +11498,7 @@
       <c r="C20" s="44"/>
       <c r="D20" s="44"/>
       <c r="E20" s="44" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="F20" s="44"/>
       <c r="G20" s="44"/>
@@ -11282,7 +11508,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="44" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="B21" s="44">
         <v>1</v>
@@ -11292,13 +11518,13 @@
         <v>34</v>
       </c>
       <c r="E21" s="44" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="F21" s="44">
         <v>2</v>
       </c>
       <c r="G21" s="44" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="H21" s="44" t="s">
         <v>34</v>
@@ -11308,7 +11534,7 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="44" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="B22" s="44">
         <v>1</v>
@@ -11334,59 +11560,59 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="44" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="B23" s="44">
         <v>1</v>
       </c>
       <c r="C23" s="44"/>
       <c r="D23" s="44" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="E23" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="F23" s="44">
         <v>2</v>
       </c>
       <c r="G23" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="H23" s="44" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="I23" s="44"/>
       <c r="J23" s="44"/>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="44" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
       <c r="B24" s="44">
         <v>1</v>
       </c>
       <c r="C24" s="44"/>
       <c r="D24" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="E24" s="44" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="F24" s="44">
         <v>2</v>
       </c>
       <c r="G24" s="44" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="H24" s="44" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="I24" s="44"/>
       <c r="J24" s="44"/>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="44" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="B25" s="44">
         <v>1</v>
@@ -11396,7 +11622,7 @@
         <v>34</v>
       </c>
       <c r="E25" s="44" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="F25" s="44"/>
       <c r="G25" s="44"/>
@@ -11406,7 +11632,7 @@
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="44" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="B26" s="44">
         <v>1</v>
@@ -11416,13 +11642,13 @@
         <v>34</v>
       </c>
       <c r="E26" s="44" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="F26" s="44">
         <v>2</v>
       </c>
       <c r="G26" s="44" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="H26" s="44" t="s">
         <v>34</v>
@@ -11432,7 +11658,7 @@
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="44" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="B27" s="44">
         <v>1</v>
@@ -11452,7 +11678,7 @@
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="44" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="B28" s="44">
         <v>1</v>
@@ -11484,10 +11710,10 @@
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="57.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="15.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="4" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="1" max="1" width="57.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -11606,28 +11832,28 @@
   <dimension ref="A1:V15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="50.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="25" width="18.36328125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="25" width="12.08984375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="25" width="15.36328125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="25" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="25" width="9.453125"/>
-    <col min="7" max="8" style="25" width="8.81640625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="8.1796875"/>
-    <col min="15" max="15" customWidth="true" style="25" width="13.0"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="10.1796875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" style="25" width="9.1796875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="25" width="11.6328125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="23" max="16384" style="25" width="8.81640625"/>
+    <col min="1" max="1" width="50" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.36328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.08984375" style="25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.36328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="8.81640625" style="25"/>
+    <col min="9" max="9" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13" style="25" customWidth="1"/>
+    <col min="16" max="16" width="10.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="8.81640625" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -12322,29 +12548,29 @@
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="44.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="8.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="13.54296875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.81640625"/>
-    <col min="11" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.1796875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="8.1796875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="14.1796875"/>
-    <col min="27" max="28" bestFit="true" customWidth="true" width="12.81640625"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="14.1796875"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="12.81640625"/>
+    <col min="1" max="1" width="44.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -12776,10 +13002,10 @@
   <dimension ref="A1:AJ39"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="54.36328125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="13.81640625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="1" max="1" width="54.36328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36">
@@ -12853,16 +13079,16 @@
         <v>58</v>
       </c>
       <c r="X1" s="45" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="Y1" s="45" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
       <c r="Z1" s="45" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
       <c r="AA1" s="45" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="AB1" s="45" t="s">
         <v>1</v>
@@ -12900,7 +13126,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>739</v>
+        <v>719</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>13</v>
@@ -12921,10 +13147,10 @@
       <c r="P2" s="44"/>
       <c r="Q2" s="44"/>
       <c r="R2" s="44" t="s">
-        <v>776</v>
+        <v>738</v>
       </c>
       <c r="S2" s="44" t="s">
-        <v>777</v>
+        <v>739</v>
       </c>
       <c r="T2" s="44"/>
       <c r="U2" s="44"/>
@@ -12952,7 +13178,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>740</v>
+        <v>720</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>13</v>
@@ -13024,7 +13250,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>740</v>
+        <v>720</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>13</v>
@@ -13261,10 +13487,10 @@
       <c r="P8" s="44"/>
       <c r="Q8" s="44"/>
       <c r="R8" s="44" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="S8" s="44" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="T8" s="44">
         <v>0</v>
@@ -13323,10 +13549,10 @@
       <c r="P9" s="44"/>
       <c r="Q9" s="44"/>
       <c r="R9" s="44" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="S9" s="44" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="T9" s="44"/>
       <c r="U9" s="44">
@@ -13389,10 +13615,10 @@
       <c r="P10" s="44"/>
       <c r="Q10" s="44"/>
       <c r="R10" s="44" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="S10" s="44" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="T10" s="44"/>
       <c r="U10" s="44"/>
@@ -13693,10 +13919,10 @@
       <c r="P16" s="44"/>
       <c r="Q16" s="44"/>
       <c r="R16" s="44" t="s">
-        <v>743</v>
+        <v>721</v>
       </c>
       <c r="S16" s="44" t="s">
-        <v>744</v>
+        <v>722</v>
       </c>
       <c r="T16" s="44"/>
       <c r="U16" s="44"/>
@@ -13766,7 +13992,7 @@
     </row>
     <row r="18" spans="1:36">
       <c r="A18" s="67" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
       <c r="B18" s="69">
         <v>1</v>
@@ -13801,7 +14027,7 @@
       <c r="P18" s="44"/>
       <c r="Q18" s="44"/>
       <c r="R18" s="44" t="s">
-        <v>745</v>
+        <v>723</v>
       </c>
       <c r="S18" s="44"/>
       <c r="T18" s="47">
@@ -13826,7 +14052,7 @@
     </row>
     <row r="19" spans="1:36">
       <c r="A19" s="67" t="s">
-        <v>688</v>
+        <v>683</v>
       </c>
       <c r="B19" s="69">
         <v>1</v>
@@ -13844,7 +14070,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="47" t="s">
-        <v>689</v>
+        <v>684</v>
       </c>
       <c r="H19" s="44" t="s">
         <v>12</v>
@@ -13856,7 +14082,7 @@
         <v>2</v>
       </c>
       <c r="K19" s="47" t="s">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="L19" s="44" t="s">
         <v>216</v>
@@ -13877,7 +14103,7 @@
         <v>34</v>
       </c>
       <c r="R19" s="44" t="s">
-        <v>746</v>
+        <v>724</v>
       </c>
       <c r="S19" s="44"/>
       <c r="T19" s="47">
@@ -13902,13 +14128,13 @@
     </row>
     <row r="20" spans="1:36">
       <c r="A20" s="67" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
       <c r="B20" s="69">
         <v>1</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>693</v>
+        <v>687</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>163</v>
@@ -13920,19 +14146,19 @@
         <v>1</v>
       </c>
       <c r="G20" s="47" t="s">
-        <v>694</v>
+        <v>688</v>
       </c>
       <c r="H20" s="44" t="s">
         <v>13</v>
       </c>
       <c r="I20" s="44" t="s">
-        <v>695</v>
+        <v>689</v>
       </c>
       <c r="J20" s="44">
         <v>2</v>
       </c>
       <c r="K20" s="47" t="s">
-        <v>696</v>
+        <v>690</v>
       </c>
       <c r="L20" s="44" t="s">
         <v>13</v>
@@ -13944,7 +14170,7 @@
         <v>2</v>
       </c>
       <c r="O20" s="47" t="s">
-        <v>697</v>
+        <v>691</v>
       </c>
       <c r="P20" s="44" t="s">
         <v>163</v>
@@ -13953,7 +14179,7 @@
         <v>12</v>
       </c>
       <c r="R20" s="44" t="s">
-        <v>747</v>
+        <v>725</v>
       </c>
       <c r="S20" s="44"/>
       <c r="T20" s="47">
@@ -13978,7 +14204,7 @@
     </row>
     <row r="21" spans="1:36">
       <c r="A21" s="67" t="s">
-        <v>699</v>
+        <v>692</v>
       </c>
       <c r="B21" s="69">
         <v>1</v>
@@ -14015,7 +14241,7 @@
       <c r="P21" s="44"/>
       <c r="Q21" s="44"/>
       <c r="R21" s="44" t="s">
-        <v>748</v>
+        <v>726</v>
       </c>
       <c r="S21" s="44"/>
       <c r="T21" s="47">
@@ -14025,16 +14251,16 @@
       <c r="V21" s="44"/>
       <c r="W21" s="44"/>
       <c r="X21" s="44" t="s">
-        <v>701</v>
+        <v>693</v>
       </c>
       <c r="Y21" s="44" t="s">
-        <v>702</v>
+        <v>694</v>
       </c>
       <c r="Z21" s="44" t="s">
-        <v>701</v>
+        <v>693</v>
       </c>
       <c r="AA21" s="44" t="s">
-        <v>702</v>
+        <v>694</v>
       </c>
       <c r="AB21" s="44"/>
       <c r="AC21" s="44"/>
@@ -14048,7 +14274,7 @@
     </row>
     <row r="22" spans="1:36">
       <c r="A22" s="67" t="s">
-        <v>703</v>
+        <v>695</v>
       </c>
       <c r="B22" s="69"/>
       <c r="C22" s="16"/>
@@ -14092,7 +14318,7 @@
     </row>
     <row r="23" spans="1:36">
       <c r="A23" s="67" t="s">
-        <v>704</v>
+        <v>696</v>
       </c>
       <c r="B23" s="69">
         <v>1</v>
@@ -14140,7 +14366,7 @@
     </row>
     <row r="24" spans="1:36">
       <c r="A24" s="67" t="s">
-        <v>705</v>
+        <v>697</v>
       </c>
       <c r="B24" s="69">
         <v>1</v>
@@ -14175,7 +14401,7 @@
       <c r="P24" s="44"/>
       <c r="Q24" s="44"/>
       <c r="R24" s="44" t="s">
-        <v>749</v>
+        <v>727</v>
       </c>
       <c r="S24" s="44"/>
       <c r="T24" s="47"/>
@@ -14198,13 +14424,13 @@
     </row>
     <row r="25" spans="1:36">
       <c r="A25" s="67" t="s">
-        <v>707</v>
+        <v>698</v>
       </c>
       <c r="B25" s="69">
         <v>1</v>
       </c>
       <c r="C25" s="47" t="s">
-        <v>708</v>
+        <v>699</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>12</v>
@@ -14246,7 +14472,7 @@
     </row>
     <row r="26" spans="1:36">
       <c r="A26" s="67" t="s">
-        <v>709</v>
+        <v>700</v>
       </c>
       <c r="B26" s="69">
         <v>1</v>
@@ -14279,10 +14505,10 @@
       <c r="V26" s="44"/>
       <c r="W26" s="44"/>
       <c r="X26" s="44" t="s">
-        <v>710</v>
+        <v>701</v>
       </c>
       <c r="Y26" s="44" t="s">
-        <v>711</v>
+        <v>702</v>
       </c>
       <c r="Z26" s="44"/>
       <c r="AA26" s="44"/>
@@ -14298,7 +14524,7 @@
     </row>
     <row r="27" spans="1:36">
       <c r="A27" s="67" t="s">
-        <v>712</v>
+        <v>703</v>
       </c>
       <c r="B27" s="69">
         <v>1</v>
@@ -14331,10 +14557,10 @@
       <c r="V27" s="44"/>
       <c r="W27" s="44"/>
       <c r="X27" s="44" t="s">
-        <v>710</v>
+        <v>701</v>
       </c>
       <c r="Y27" s="44" t="s">
-        <v>711</v>
+        <v>702</v>
       </c>
       <c r="Z27" s="44"/>
       <c r="AA27" s="44"/>
@@ -14350,7 +14576,7 @@
     </row>
     <row r="28" spans="1:36">
       <c r="A28" s="67" t="s">
-        <v>713</v>
+        <v>704</v>
       </c>
       <c r="B28" s="69">
         <v>1</v>
@@ -14377,7 +14603,7 @@
       <c r="P28" s="44"/>
       <c r="Q28" s="44"/>
       <c r="R28" s="44" t="s">
-        <v>750</v>
+        <v>728</v>
       </c>
       <c r="S28" s="44"/>
       <c r="T28" s="47">
@@ -14404,7 +14630,7 @@
     </row>
     <row r="29" spans="1:36">
       <c r="A29" s="39" t="s">
-        <v>715</v>
+        <v>705</v>
       </c>
       <c r="B29" s="69">
         <v>1</v>
@@ -14434,7 +14660,7 @@
         <v>2</v>
       </c>
       <c r="K29" s="47" t="s">
-        <v>716</v>
+        <v>706</v>
       </c>
       <c r="L29" s="44" t="s">
         <v>47</v>
@@ -14470,7 +14696,7 @@
         <v>3</v>
       </c>
       <c r="AC29" s="47" t="s">
-        <v>717</v>
+        <v>707</v>
       </c>
       <c r="AD29" s="44" t="s">
         <v>45</v>
@@ -14482,7 +14708,7 @@
         <v>3</v>
       </c>
       <c r="AG29" s="47" t="s">
-        <v>708</v>
+        <v>699</v>
       </c>
       <c r="AH29" s="44" t="s">
         <v>12</v>
@@ -14494,13 +14720,13 @@
     </row>
     <row r="30" spans="1:36">
       <c r="A30" s="67" t="s">
-        <v>718</v>
+        <v>708</v>
       </c>
       <c r="B30" s="69">
         <v>1</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>563</v>
+        <v>559</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>12</v>
@@ -14521,7 +14747,7 @@
       <c r="P30" s="44"/>
       <c r="Q30" s="44"/>
       <c r="R30" s="44" t="s">
-        <v>753</v>
+        <v>729</v>
       </c>
       <c r="S30" s="44"/>
       <c r="T30" s="44">
@@ -14550,7 +14776,7 @@
     </row>
     <row r="31" spans="1:36">
       <c r="A31" s="67" t="s">
-        <v>720</v>
+        <v>709</v>
       </c>
       <c r="B31" s="69">
         <v>1</v>
@@ -14577,7 +14803,7 @@
       <c r="P31" s="44"/>
       <c r="Q31" s="44"/>
       <c r="R31" s="44" t="s">
-        <v>756</v>
+        <v>730</v>
       </c>
       <c r="S31" s="44"/>
       <c r="T31" s="44">
@@ -14606,7 +14832,7 @@
     </row>
     <row r="32" spans="1:36">
       <c r="A32" s="67" t="s">
-        <v>722</v>
+        <v>710</v>
       </c>
       <c r="B32" s="69">
         <v>1</v>
@@ -14633,7 +14859,7 @@
       <c r="P32" s="44"/>
       <c r="Q32" s="44"/>
       <c r="R32" s="44" t="s">
-        <v>759</v>
+        <v>731</v>
       </c>
       <c r="S32" s="44"/>
       <c r="T32" s="44">
@@ -14662,7 +14888,7 @@
     </row>
     <row r="33" spans="1:36">
       <c r="A33" s="67" t="s">
-        <v>724</v>
+        <v>711</v>
       </c>
       <c r="B33" s="69">
         <v>1</v>
@@ -14689,7 +14915,7 @@
       <c r="P33" s="44"/>
       <c r="Q33" s="44"/>
       <c r="R33" s="44" t="s">
-        <v>762</v>
+        <v>732</v>
       </c>
       <c r="S33" s="44"/>
       <c r="T33" s="44">
@@ -14718,7 +14944,7 @@
     </row>
     <row r="34" spans="1:36">
       <c r="A34" s="67" t="s">
-        <v>726</v>
+        <v>712</v>
       </c>
       <c r="B34" s="69">
         <v>1</v>
@@ -14745,7 +14971,7 @@
       <c r="P34" s="44"/>
       <c r="Q34" s="44"/>
       <c r="R34" s="44" t="s">
-        <v>765</v>
+        <v>733</v>
       </c>
       <c r="S34" s="44"/>
       <c r="T34" s="44">
@@ -14774,7 +15000,7 @@
     </row>
     <row r="35" spans="1:36">
       <c r="A35" s="67" t="s">
-        <v>728</v>
+        <v>713</v>
       </c>
       <c r="B35" s="69">
         <v>1</v>
@@ -14801,7 +15027,7 @@
       <c r="P35" s="44"/>
       <c r="Q35" s="44"/>
       <c r="R35" s="44" t="s">
-        <v>768</v>
+        <v>734</v>
       </c>
       <c r="S35" s="44"/>
       <c r="T35" s="44">
@@ -14830,7 +15056,7 @@
     </row>
     <row r="36" spans="1:36">
       <c r="A36" s="67" t="s">
-        <v>730</v>
+        <v>714</v>
       </c>
       <c r="B36" s="69">
         <v>1</v>
@@ -14857,7 +15083,7 @@
       <c r="P36" s="44"/>
       <c r="Q36" s="44"/>
       <c r="R36" s="44" t="s">
-        <v>771</v>
+        <v>735</v>
       </c>
       <c r="S36" s="44"/>
       <c r="T36" s="44">
@@ -14886,7 +15112,7 @@
     </row>
     <row r="37" spans="1:36">
       <c r="A37" s="39" t="s">
-        <v>732</v>
+        <v>715</v>
       </c>
       <c r="B37" s="69">
         <v>1</v>
@@ -14913,7 +15139,7 @@
       <c r="P37" s="44"/>
       <c r="Q37" s="44"/>
       <c r="R37" s="44" t="s">
-        <v>774</v>
+        <v>736</v>
       </c>
       <c r="S37" s="44"/>
       <c r="T37" s="44">
@@ -14942,7 +15168,7 @@
     </row>
     <row r="38" spans="1:36">
       <c r="A38" s="67" t="s">
-        <v>734</v>
+        <v>716</v>
       </c>
       <c r="B38" s="69">
         <v>1</v>
@@ -14969,7 +15195,7 @@
       <c r="P38" s="44"/>
       <c r="Q38" s="44"/>
       <c r="R38" s="44" t="s">
-        <v>775</v>
+        <v>737</v>
       </c>
       <c r="S38" s="44"/>
       <c r="T38" s="44">
@@ -14995,12 +15221,12 @@
       <c r="AH38" s="44"/>
       <c r="AI38" s="44"/>
       <c r="AJ38" s="47" t="s">
-        <v>738</v>
+        <v>718</v>
       </c>
     </row>
     <row r="39" spans="1:36">
       <c r="A39" s="67" t="s">
-        <v>736</v>
+        <v>717</v>
       </c>
       <c r="B39" s="69">
         <v>1</v>
@@ -15027,7 +15253,7 @@
       <c r="P39" s="44"/>
       <c r="Q39" s="44"/>
       <c r="R39" s="44" t="s">
-        <v>778</v>
+        <v>740</v>
       </c>
       <c r="S39" s="44" t="s">
         <v>378</v>
@@ -15065,16 +15291,16 @@
   <dimension ref="A1:S20"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="53.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="5" max="7" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="53.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="12.1796875" customWidth="1"/>
+    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">

</xml_diff>

<commit_message>
AirportPassengerList given by Rohin
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E2DEE8B-1475-406C-9471-FC4991C5F158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{875C6E14-BEB5-438C-A3E3-64B06211B37E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="14" activeTab="14" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2717" uniqueCount="879">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2822" uniqueCount="922">
   <si>
     <t>Scenario</t>
   </si>
@@ -1543,12 +1543,6 @@
     <t>2023-08-23T10:38:00</t>
   </si>
   <si>
-    <t>A2MQN5</t>
-  </si>
-  <si>
-    <t>2023-08-22T05:24:50</t>
-  </si>
-  <si>
     <t>A2MQPD</t>
   </si>
   <si>
@@ -2711,6 +2705,141 @@
   </si>
   <si>
     <t>12</t>
+  </si>
+  <si>
+    <t>List type</t>
+  </si>
+  <si>
+    <t>FilterValues</t>
+  </si>
+  <si>
+    <t>Standard list - Code 0 - All Passengers</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Standard_list_Code_30_passengers_with_no_meals</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Standard_list_Code_44_passengers_with_elite_frequent_traveler_numbers</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>Custom_list_Filter_Value_0</t>
+  </si>
+  <si>
+    <t>Standard_list_Code_6_Out_of_synch_electronic_tickets</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Custom_list_Filter_Value_1_Surname</t>
+  </si>
+  <si>
+    <t>Find passengers with passcode SA3R09</t>
+  </si>
+  <si>
+    <t>DCS_reference_number</t>
+  </si>
+  <si>
+    <t>Standard_list_Code_26_passengers_with_inbound_connections</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>Large_Parties</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>Passengers_with_outbound_connections</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>Code_33_Specific_passengers</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>Code_34_specific_party</t>
+  </si>
+  <si>
+    <t>Code_36_requiring_seats</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>BCHVBD</t>
+  </si>
+  <si>
+    <t>2023-09-01T13:07:46</t>
+  </si>
+  <si>
+    <t>BCHVCX</t>
+  </si>
+  <si>
+    <t>2023-09-01T13:07:52</t>
+  </si>
+  <si>
+    <t>BCHVD3</t>
+  </si>
+  <si>
+    <t>2023-09-01T13:07:57</t>
+  </si>
+  <si>
+    <t>BCHVGW</t>
+  </si>
+  <si>
+    <t>2023-09-01T13:08:00</t>
+  </si>
+  <si>
+    <t>BCHVHV</t>
+  </si>
+  <si>
+    <t>2023-09-01T13:08:05</t>
+  </si>
+  <si>
+    <t>BCHVJI</t>
+  </si>
+  <si>
+    <t>2023-09-01T13:08:09</t>
+  </si>
+  <si>
+    <t>BCHVLZ</t>
+  </si>
+  <si>
+    <t>2023-09-01T13:08:17</t>
+  </si>
+  <si>
+    <t>BCHVNP</t>
+  </si>
+  <si>
+    <t>2023-09-01T13:08:21</t>
+  </si>
+  <si>
+    <t>BCHVUB</t>
+  </si>
+  <si>
+    <t>2023-09-01T13:08:26</t>
+  </si>
+  <si>
+    <t>BCHVWQ</t>
+  </si>
+  <si>
+    <t>2023-09-01T13:08:29</t>
   </si>
 </sst>
 </file>
@@ -3584,7 +3713,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="43" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="I2" s="43" t="s">
         <v>210</v>
@@ -3601,7 +3730,7 @@
       <c r="M2" s="43"/>
       <c r="N2" s="43"/>
       <c r="O2" s="43" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="P2" s="43"/>
       <c r="Q2" s="43"/>
@@ -3696,7 +3825,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="37" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="I4" s="37" t="s">
         <v>341</v>
@@ -3745,13 +3874,13 @@
         <v>1</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="I5" s="43" t="s">
         <v>211</v>
       </c>
       <c r="J5" s="43" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="K5" s="43"/>
       <c r="L5" s="43"/>
@@ -3777,13 +3906,13 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6" s="43" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="B6" s="43">
         <v>0</v>
       </c>
       <c r="C6" s="46" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="D6" s="43" t="s">
         <v>47</v>
@@ -3796,10 +3925,10 @@
       </c>
       <c r="G6" s="43"/>
       <c r="H6" s="43" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="I6" s="43" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="J6" s="43" t="s">
         <v>241</v>
@@ -3810,7 +3939,7 @@
       <c r="N6" s="43"/>
       <c r="O6" s="43"/>
       <c r="P6" s="43" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="Q6" s="43" t="s">
         <v>442</v>
@@ -3828,13 +3957,13 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7" s="43" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="B7" s="43">
         <v>0</v>
       </c>
       <c r="C7" s="46" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="D7" s="43" t="s">
         <v>47</v>
@@ -3847,13 +3976,13 @@
       </c>
       <c r="G7" s="43"/>
       <c r="H7" s="43" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="I7" s="43" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="J7" s="43" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="K7" s="43"/>
       <c r="L7" s="43"/>
@@ -3875,13 +4004,13 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8" s="72" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="B8" s="43">
         <v>0</v>
       </c>
       <c r="C8" s="46" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="D8" s="43" t="s">
         <v>47</v>
@@ -3894,13 +4023,13 @@
       </c>
       <c r="G8" s="43"/>
       <c r="H8" s="43" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="I8" s="43" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="J8" s="43" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="K8" s="43"/>
       <c r="L8" s="43"/>
@@ -3908,7 +4037,7 @@
       <c r="N8" s="43"/>
       <c r="O8" s="43"/>
       <c r="P8" s="43" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="Q8" s="43" t="s">
         <v>442</v>
@@ -3926,13 +4055,13 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9" s="73" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="B9" s="43">
         <v>1</v>
       </c>
       <c r="C9" s="46" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="D9" s="43" t="s">
         <v>47</v>
@@ -3945,13 +4074,13 @@
       </c>
       <c r="G9" s="43"/>
       <c r="H9" s="43" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="I9" s="43" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="J9" s="43" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="K9" s="43"/>
       <c r="L9" s="43"/>
@@ -3959,7 +4088,7 @@
       <c r="N9" s="43"/>
       <c r="O9" s="43"/>
       <c r="P9" s="43" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="Q9" s="43" t="s">
         <v>442</v>
@@ -3977,13 +4106,13 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10" s="43" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="B10" s="43">
         <v>1</v>
       </c>
       <c r="C10" s="46" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="D10" s="43" t="s">
         <v>47</v>
@@ -3996,27 +4125,27 @@
       </c>
       <c r="G10" s="43"/>
       <c r="H10" s="43" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="I10" s="43" t="s">
+        <v>710</v>
+      </c>
+      <c r="J10" s="43" t="s">
+        <v>711</v>
+      </c>
+      <c r="K10" s="43" t="s">
         <v>712</v>
       </c>
-      <c r="J10" s="43" t="s">
+      <c r="L10" s="43" t="s">
         <v>713</v>
-      </c>
-      <c r="K10" s="43" t="s">
-        <v>714</v>
-      </c>
-      <c r="L10" s="43" t="s">
-        <v>715</v>
       </c>
       <c r="M10" s="43"/>
       <c r="N10" s="43"/>
       <c r="O10" s="43" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="P10" s="43" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="Q10" s="43" t="s">
         <v>442</v>
@@ -4034,13 +4163,13 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11" s="43" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="B11" s="43">
         <v>1</v>
       </c>
       <c r="C11" s="46" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="D11" s="43" t="s">
         <v>47</v>
@@ -4053,13 +4182,13 @@
       </c>
       <c r="G11" s="43"/>
       <c r="H11" s="43" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="I11" s="43" t="s">
         <v>347</v>
       </c>
       <c r="J11" s="43" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="K11" s="43"/>
       <c r="L11" s="43"/>
@@ -4067,7 +4196,7 @@
       <c r="N11" s="43"/>
       <c r="O11" s="43"/>
       <c r="P11" s="43" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="Q11" s="43" t="s">
         <v>442</v>
@@ -4085,7 +4214,7 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12" s="43" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="B12" s="43">
         <v>0</v>
@@ -4104,7 +4233,7 @@
       </c>
       <c r="G12" s="43"/>
       <c r="H12" s="43" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="I12" s="43" t="s">
         <v>21</v>
@@ -4121,7 +4250,7 @@
       <c r="M12" s="43"/>
       <c r="N12" s="43"/>
       <c r="O12" s="43" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="P12" s="43"/>
       <c r="Q12" s="43"/>
@@ -4138,13 +4267,13 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13" s="43" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="B13" s="43">
         <v>0</v>
       </c>
       <c r="C13" s="46" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="D13" s="43" t="s">
         <v>47</v>
@@ -4157,16 +4286,16 @@
       </c>
       <c r="G13" s="43"/>
       <c r="H13" s="43" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="I13" s="43" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="J13" s="43" t="s">
         <v>16</v>
       </c>
       <c r="K13" s="43" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="L13" s="43" t="s">
         <v>16</v>
@@ -4174,7 +4303,7 @@
       <c r="M13" s="43"/>
       <c r="N13" s="43"/>
       <c r="O13" s="43" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="P13" s="43"/>
       <c r="Q13" s="43"/>
@@ -4191,43 +4320,43 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14" s="43" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="B14" s="43">
         <v>0</v>
       </c>
       <c r="C14" s="46" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="D14" s="43" t="s">
         <v>12</v>
       </c>
       <c r="E14" s="43" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="F14" s="43" t="s">
         <v>14</v>
       </c>
       <c r="G14" s="43"/>
       <c r="H14" s="43" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="I14" s="43" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="J14" s="43" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="K14" s="43" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="L14" s="43" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="M14" s="43"/>
       <c r="N14" s="43"/>
       <c r="O14" s="43" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="P14" s="43"/>
       <c r="Q14" s="43"/>
@@ -4244,13 +4373,13 @@
     </row>
     <row r="15" spans="1:27">
       <c r="A15" s="53" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="B15" s="43">
         <v>0</v>
       </c>
       <c r="C15" s="46" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="D15" s="43" t="s">
         <v>47</v>
@@ -4263,13 +4392,13 @@
       </c>
       <c r="G15" s="43"/>
       <c r="H15" s="43" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="I15" s="43" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="J15" s="43" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="K15" s="43"/>
       <c r="L15" s="43"/>
@@ -4277,7 +4406,7 @@
       <c r="N15" s="43"/>
       <c r="O15" s="43"/>
       <c r="P15" s="43" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="Q15" s="43" t="s">
         <v>442</v>
@@ -4295,7 +4424,7 @@
     </row>
     <row r="16" spans="1:27">
       <c r="A16" s="43" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="B16" s="43">
         <v>1</v>
@@ -4314,13 +4443,13 @@
       </c>
       <c r="G16" s="43"/>
       <c r="H16" s="43" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="I16" s="43" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="J16" s="43" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="K16" s="43"/>
       <c r="L16" s="43"/>
@@ -4342,7 +4471,7 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17" s="53" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="B17" s="43">
         <v>1</v>
@@ -4361,7 +4490,7 @@
       </c>
       <c r="G17" s="43"/>
       <c r="H17" s="43" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="I17" s="43"/>
       <c r="J17" s="43"/>
@@ -4385,7 +4514,7 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18" s="53" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="B18" s="43">
         <v>1</v>
@@ -4404,7 +4533,7 @@
       </c>
       <c r="G18" s="43"/>
       <c r="H18" s="43" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="I18" s="43" t="s">
         <v>21</v>
@@ -4432,13 +4561,13 @@
     </row>
     <row r="19" spans="1:27">
       <c r="A19" s="53" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="B19" s="43">
         <v>1</v>
       </c>
       <c r="C19" s="46" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="D19" s="43" t="s">
         <v>12</v>
@@ -4464,7 +4593,7 @@
         <v>2</v>
       </c>
       <c r="S19" s="46" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="T19" s="43" t="s">
         <v>334</v>
@@ -4479,7 +4608,7 @@
         <v>3</v>
       </c>
       <c r="X19" s="46" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="Y19" s="43" t="s">
         <v>12</v>
@@ -4493,26 +4622,26 @@
     </row>
     <row r="20" spans="1:27">
       <c r="A20" s="43" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="B20" s="43">
         <v>0</v>
       </c>
       <c r="C20" s="46" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="D20" s="43" t="s">
         <v>12</v>
       </c>
       <c r="E20" s="43" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="F20" s="43" t="s">
         <v>14</v>
       </c>
       <c r="G20" s="43"/>
       <c r="H20" s="43" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="I20" s="43"/>
       <c r="J20" s="43"/>
@@ -4527,10 +4656,10 @@
         <v>1</v>
       </c>
       <c r="S20" s="46" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="T20" s="43" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="U20" s="43" t="s">
         <v>12</v>
@@ -4542,13 +4671,13 @@
         <v>2</v>
       </c>
       <c r="X20" s="46" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="Y20" s="43" t="s">
         <v>12</v>
       </c>
       <c r="Z20" s="43" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="AA20" s="43" t="s">
         <v>14</v>
@@ -4656,10 +4785,10 @@
         <v>256</v>
       </c>
       <c r="V1" s="42" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="W1" s="42" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
     </row>
     <row r="2" spans="1:23">
@@ -4692,7 +4821,7 @@
       </c>
       <c r="J2" s="43"/>
       <c r="K2" s="43" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="L2" s="43"/>
       <c r="M2" s="43"/>
@@ -4731,10 +4860,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="43" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="L3" s="43" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="M3" s="43"/>
       <c r="N3" s="43"/>
@@ -4807,10 +4936,10 @@
       <c r="I5" s="43"/>
       <c r="J5" s="43"/>
       <c r="K5" s="43" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="L5" s="43" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="M5" s="43"/>
       <c r="N5" s="43" t="s">
@@ -4856,7 +4985,7 @@
       <c r="I6" s="43"/>
       <c r="J6" s="43"/>
       <c r="K6" s="43" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="L6" s="43"/>
       <c r="M6" s="43"/>
@@ -4867,7 +4996,7 @@
         <v>241</v>
       </c>
       <c r="P6" s="43" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="Q6" s="43"/>
       <c r="R6" s="43"/>
@@ -4903,10 +5032,10 @@
       <c r="I7" s="43"/>
       <c r="J7" s="43"/>
       <c r="K7" s="43" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="L7" s="43" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="M7" s="43"/>
       <c r="N7" s="43" t="s">
@@ -4916,13 +5045,13 @@
         <v>241</v>
       </c>
       <c r="P7" s="43" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="Q7" s="46" t="s">
         <v>87</v>
       </c>
       <c r="R7" s="43" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="S7" s="43"/>
       <c r="T7" s="43"/>
@@ -4960,10 +5089,10 @@
       </c>
       <c r="J8" s="43"/>
       <c r="K8" s="43" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="L8" s="43" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="M8" s="43"/>
       <c r="N8" s="43" t="s">
@@ -5003,7 +5132,7 @@
       <c r="I9" s="43"/>
       <c r="J9" s="43"/>
       <c r="K9" s="43" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="L9" s="43"/>
       <c r="M9" s="43"/>
@@ -5020,7 +5149,7 @@
       <c r="T9" s="43"/>
       <c r="U9" s="43"/>
       <c r="V9" s="43" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="W9" s="43"/>
     </row>
@@ -5046,10 +5175,10 @@
       <c r="I10" s="43"/>
       <c r="J10" s="43"/>
       <c r="K10" s="43" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="L10" s="43" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="M10" s="43"/>
       <c r="N10" s="43"/>
@@ -5058,7 +5187,7 @@
       <c r="Q10" s="43"/>
       <c r="R10" s="43"/>
       <c r="S10" s="46" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="T10" s="43"/>
       <c r="U10" s="43"/>
@@ -5087,10 +5216,10 @@
       <c r="I11" s="43"/>
       <c r="J11" s="43"/>
       <c r="K11" s="43" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="L11" s="43" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="M11" s="43"/>
       <c r="N11" s="43"/>
@@ -5128,10 +5257,10 @@
       <c r="I12" s="43"/>
       <c r="J12" s="43"/>
       <c r="K12" s="43" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="L12" s="43" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="M12" s="43"/>
       <c r="N12" s="43" t="s">
@@ -5173,10 +5302,10 @@
       <c r="I13" s="43"/>
       <c r="J13" s="43"/>
       <c r="K13" s="43" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="L13" s="43" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="M13" s="43"/>
       <c r="N13" s="43" t="s">
@@ -5255,10 +5384,10 @@
       <c r="I15" s="43"/>
       <c r="J15" s="43"/>
       <c r="K15" s="43" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="L15" s="43" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="M15" s="43"/>
       <c r="N15" s="43" t="s">
@@ -5286,7 +5415,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="46" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="D16" s="43" t="s">
         <v>12</v>
@@ -5300,7 +5429,7 @@
       <c r="I16" s="43"/>
       <c r="J16" s="43"/>
       <c r="K16" s="43" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="43"/>
@@ -5341,7 +5470,7 @@
       <c r="I17" s="43"/>
       <c r="J17" s="43"/>
       <c r="K17" s="43" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="43"/>
@@ -5386,7 +5515,7 @@
       </c>
       <c r="J18" s="43"/>
       <c r="K18" s="43" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="L18" s="43"/>
       <c r="M18" s="43"/>
@@ -5403,10 +5532,10 @@
       <c r="T18" s="43"/>
       <c r="U18" s="43"/>
       <c r="V18" s="43" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="W18" s="43" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
     </row>
     <row r="19" spans="1:23">
@@ -5431,7 +5560,7 @@
       <c r="I19" s="43"/>
       <c r="J19" s="43"/>
       <c r="K19" s="43" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="43"/>
@@ -5448,7 +5577,7 @@
       <c r="T19" s="43"/>
       <c r="U19" s="43"/>
       <c r="V19" s="43" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="W19" s="43"/>
     </row>
@@ -5474,7 +5603,7 @@
       <c r="I20" s="43"/>
       <c r="J20" s="43"/>
       <c r="K20" s="43" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="43"/>
@@ -5501,7 +5630,7 @@
         <v>0</v>
       </c>
       <c r="C21" s="46" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="D21" s="43" t="s">
         <v>12</v>
@@ -5515,15 +5644,15 @@
       <c r="I21" s="43"/>
       <c r="J21" s="43"/>
       <c r="K21" s="43" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="L21" s="43"/>
       <c r="M21" s="43"/>
       <c r="N21" s="43" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="O21" s="43" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="P21" s="43"/>
       <c r="Q21" s="43"/>
@@ -5542,7 +5671,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="46" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="D22" s="43" t="s">
         <v>12</v>
@@ -5557,14 +5686,14 @@
         <v>62</v>
       </c>
       <c r="H22" s="43" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="I22" s="43" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="J22" s="43"/>
       <c r="K22" s="43" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="L22" s="43"/>
       <c r="M22" s="43"/>
@@ -5660,14 +5789,14 @@
         <v>2</v>
       </c>
       <c r="D2" s="46" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="E2" s="46" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="F2" s="43"/>
       <c r="G2" s="46" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="H2" s="43" t="s">
         <v>12</v>
@@ -5691,7 +5820,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="46" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="E3" s="46" t="s">
         <v>263</v>
@@ -5700,7 +5829,7 @@
         <v>149</v>
       </c>
       <c r="G3" s="46" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="H3" s="43" t="s">
         <v>12</v>
@@ -5726,7 +5855,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="46" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="E4" s="43"/>
       <c r="F4" s="43" t="s">
@@ -5742,7 +5871,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="46" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="K4" s="43" t="s">
         <v>13</v>
@@ -5896,13 +6025,13 @@
         <v>12</v>
       </c>
       <c r="I5" s="43" t="s">
+        <v>503</v>
+      </c>
+      <c r="J5" s="43" t="s">
+        <v>504</v>
+      </c>
+      <c r="K5" s="43" t="s">
         <v>505</v>
-      </c>
-      <c r="J5" s="43" t="s">
-        <v>506</v>
-      </c>
-      <c r="K5" s="43" t="s">
-        <v>507</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -5931,10 +6060,10 @@
         <v>12</v>
       </c>
       <c r="I6" s="43" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="J6" s="43" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="K6" s="43"/>
     </row>
@@ -6214,16 +6343,16 @@
         <v>45</v>
       </c>
       <c r="J2" s="43" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="K2" s="43" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="L2" s="43" t="s">
         <v>206</v>
       </c>
       <c r="M2" s="43" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="N2" s="43" t="s">
         <v>207</v>
@@ -6232,13 +6361,13 @@
         <v>12</v>
       </c>
       <c r="P2" s="43" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="Q2" s="43" t="s">
         <v>62</v>
       </c>
       <c r="R2" s="43" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="S2" s="43" t="s">
         <v>12</v>
@@ -6284,7 +6413,7 @@
         <v>45</v>
       </c>
       <c r="J3" s="43" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="K3" s="43" t="s">
         <v>487</v>
@@ -6302,13 +6431,13 @@
         <v>12</v>
       </c>
       <c r="P3" s="43" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="Q3" s="43" t="s">
         <v>238</v>
       </c>
       <c r="R3" s="43" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="S3" s="43" t="s">
         <v>12</v>
@@ -6362,16 +6491,16 @@
       <c r="H4" s="43"/>
       <c r="I4" s="43"/>
       <c r="J4" s="43" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="K4" s="43" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="L4" s="43" t="s">
         <v>319</v>
       </c>
       <c r="M4" s="43" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="N4" s="43" t="s">
         <v>208</v>
@@ -6414,16 +6543,16 @@
       <c r="H5" s="43"/>
       <c r="I5" s="43"/>
       <c r="J5" s="43" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="K5" s="43" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="L5" s="43" t="s">
         <v>319</v>
       </c>
       <c r="M5" s="43" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="N5" s="43" t="s">
         <v>208</v>
@@ -6474,16 +6603,16 @@
         <v>45</v>
       </c>
       <c r="J6" s="43" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="K6" s="43" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="L6" s="43" t="s">
         <v>206</v>
       </c>
       <c r="M6" s="43" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="N6" s="43" t="s">
         <v>207</v>
@@ -6544,16 +6673,16 @@
         <v>68</v>
       </c>
       <c r="F1" s="44" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="G1" s="44" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="H1" s="44" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="I1" s="44" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -6577,7 +6706,7 @@
       </c>
       <c r="G2" s="38"/>
       <c r="H2" s="46" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="I2" s="43"/>
     </row>
@@ -6598,10 +6727,10 @@
         <v>34</v>
       </c>
       <c r="F3" s="38" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="G3" s="69" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="H3" s="43"/>
       <c r="I3" s="43"/>
@@ -6611,7 +6740,7 @@
         <v>71</v>
       </c>
       <c r="B4" s="69" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="C4" s="38">
         <v>0</v>
@@ -6626,13 +6755,13 @@
         <v>50</v>
       </c>
       <c r="G4" s="69" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="H4" s="46" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
       <c r="I4" s="43" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
     </row>
   </sheetData>
@@ -6679,7 +6808,7 @@
         <v>1</v>
       </c>
       <c r="F1" s="41" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="G1" s="41" t="s">
         <v>56</v>
@@ -6688,19 +6817,19 @@
         <v>4</v>
       </c>
       <c r="I1" s="41" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="J1" s="42" t="s">
         <v>74</v>
       </c>
       <c r="K1" s="41" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="L1" s="41" t="s">
+        <v>864</v>
+      </c>
+      <c r="M1" s="41" t="s">
         <v>866</v>
-      </c>
-      <c r="M1" s="41" t="s">
-        <v>868</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -6711,7 +6840,7 @@
         <v>149</v>
       </c>
       <c r="C2" s="46" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="D2" s="43" t="s">
         <v>263</v>
@@ -6736,7 +6865,7 @@
         <v>149</v>
       </c>
       <c r="C3" s="46" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="D3" s="43" t="s">
         <v>263</v>
@@ -6761,7 +6890,7 @@
         <v>149</v>
       </c>
       <c r="C4" s="46" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="D4" s="43" t="s">
         <v>263</v>
@@ -6779,10 +6908,10 @@
         <v>34</v>
       </c>
       <c r="I4" s="46" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="J4" s="43" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="K4" s="43"/>
       <c r="L4" s="43"/>
@@ -6851,7 +6980,7 @@
       </c>
       <c r="E7" s="43"/>
       <c r="F7" s="43" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="G7" s="43"/>
       <c r="H7" s="43"/>
@@ -6904,10 +7033,10 @@
       <c r="I9" s="43"/>
       <c r="J9" s="43"/>
       <c r="K9" s="46" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="L9" s="46" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="M9" s="43"/>
     </row>
@@ -6990,7 +7119,7 @@
         <v>149</v>
       </c>
       <c r="C13" s="46" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="D13" s="43" t="s">
         <v>263</v>
@@ -7006,7 +7135,7 @@
       <c r="K13" s="43"/>
       <c r="L13" s="43"/>
       <c r="M13" s="43" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -7017,7 +7146,7 @@
         <v>149</v>
       </c>
       <c r="C14" s="46" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="D14" s="43" t="s">
         <v>263</v>
@@ -7048,7 +7177,7 @@
         <v>149</v>
       </c>
       <c r="C15" s="46" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="D15" s="43" t="s">
         <v>263</v>
@@ -7296,7 +7425,7 @@
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="22" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="B5" s="43">
         <v>1</v>
@@ -7305,7 +7434,7 @@
         <v>34</v>
       </c>
       <c r="D5" s="43" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="E5" s="43"/>
       <c r="F5" s="43"/>
@@ -7319,7 +7448,7 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="22" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="B6" s="43">
         <v>1</v>
@@ -7342,7 +7471,7 @@
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="22" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="B7" s="43">
         <v>1</v>
@@ -7354,7 +7483,7 @@
         <v>208</v>
       </c>
       <c r="E7" s="46" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="F7" s="43"/>
       <c r="G7" s="43"/>
@@ -7367,7 +7496,7 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="22" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="B8" s="43">
         <v>1</v>
@@ -7392,7 +7521,7 @@
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="22" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="B9" s="43">
         <v>1</v>
@@ -7416,7 +7545,7 @@
         <v>208</v>
       </c>
       <c r="I9" s="46" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="J9" s="43">
         <v>1</v>
@@ -7428,12 +7557,12 @@
         <v>163</v>
       </c>
       <c r="M9" s="46" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="22" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="B10" s="43">
         <v>1</v>
@@ -7442,7 +7571,7 @@
         <v>34</v>
       </c>
       <c r="D10" s="43" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="E10" s="43"/>
       <c r="F10" s="43"/>
@@ -7456,7 +7585,7 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="22" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B11" s="43">
         <v>1</v>
@@ -7468,7 +7597,7 @@
         <v>163</v>
       </c>
       <c r="E11" s="46" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -7481,7 +7610,7 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="22" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B12" s="43"/>
       <c r="C12" s="43" t="s">
@@ -7502,11 +7631,11 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="22" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="B13" s="43"/>
       <c r="C13" s="43" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="D13" s="43"/>
       <c r="E13" s="43"/>
@@ -7521,7 +7650,7 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="70" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="B14" s="43">
         <v>1</v>
@@ -7542,13 +7671,13 @@
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="22" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="B15" s="43">
         <v>1</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="D15" s="43" t="s">
         <v>34</v>
@@ -7894,7 +8023,7 @@
     </row>
     <row r="5" spans="1:33">
       <c r="A5" s="66" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="B5" s="75">
         <v>1</v>
@@ -7939,7 +8068,7 @@
     </row>
     <row r="6" spans="1:33">
       <c r="A6" s="66" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="B6" s="75">
         <v>1</v>
@@ -7984,14 +8113,14 @@
     </row>
     <row r="7" spans="1:33">
       <c r="A7" s="66" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="B7" s="75"/>
       <c r="C7" s="76" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="D7" s="77" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="E7" s="77" t="s">
         <v>34</v>
@@ -8027,16 +8156,16 @@
     </row>
     <row r="8" spans="1:33">
       <c r="A8" s="66" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="B8" s="75">
         <v>3</v>
       </c>
       <c r="C8" s="76" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="D8" s="77" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="E8" s="77" t="s">
         <v>34</v>
@@ -8072,16 +8201,16 @@
     </row>
     <row r="9" spans="1:33">
       <c r="A9" s="66" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="B9" s="75">
         <v>1</v>
       </c>
       <c r="C9" s="76" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="D9" s="77" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="E9" s="77" t="s">
         <v>34</v>
@@ -8117,13 +8246,13 @@
     </row>
     <row r="10" spans="1:33">
       <c r="A10" s="66" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="B10" s="75">
         <v>1</v>
       </c>
       <c r="C10" s="76" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="D10" s="76"/>
       <c r="E10" s="76"/>
@@ -8158,13 +8287,13 @@
     </row>
     <row r="11" spans="1:33">
       <c r="A11" s="66" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="B11" s="75">
         <v>1</v>
       </c>
       <c r="C11" s="76" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
       <c r="D11" s="77" t="s">
         <v>34</v>
@@ -8203,13 +8332,13 @@
     </row>
     <row r="12" spans="1:33">
       <c r="A12" s="66" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="B12" s="75">
         <v>1</v>
       </c>
       <c r="C12" s="76" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="D12" s="77" t="s">
         <v>12</v>
@@ -8248,25 +8377,25 @@
     </row>
     <row r="13" spans="1:33">
       <c r="A13" s="66" t="s">
+        <v>823</v>
+      </c>
+      <c r="B13" s="75">
+        <v>1</v>
+      </c>
+      <c r="C13" s="74" t="s">
+        <v>824</v>
+      </c>
+      <c r="D13" s="77" t="s">
         <v>825</v>
       </c>
-      <c r="B13" s="75">
-        <v>1</v>
-      </c>
-      <c r="C13" s="74" t="s">
+      <c r="E13" s="77" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="79">
+        <v>1</v>
+      </c>
+      <c r="G13" s="79" t="s">
         <v>826</v>
-      </c>
-      <c r="D13" s="77" t="s">
-        <v>827</v>
-      </c>
-      <c r="E13" s="77" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="79">
-        <v>1</v>
-      </c>
-      <c r="G13" s="79" t="s">
-        <v>828</v>
       </c>
       <c r="H13" s="79" t="s">
         <v>34</v>
@@ -8301,13 +8430,13 @@
     </row>
     <row r="14" spans="1:33">
       <c r="A14" s="66" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="B14" s="75">
         <v>1</v>
       </c>
       <c r="C14" s="74" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="D14" s="77" t="s">
         <v>12</v>
@@ -8320,10 +8449,10 @@
         <v>1</v>
       </c>
       <c r="G14" s="79" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="H14" s="78" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="I14" s="78" t="s">
         <v>12</v>
@@ -8333,7 +8462,7 @@
         <v>1</v>
       </c>
       <c r="K14" s="76" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="L14" s="77" t="s">
         <v>334</v>
@@ -8526,14 +8655,14 @@
       <c r="I2" s="43"/>
       <c r="J2" s="43"/>
       <c r="K2" s="43" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="L2" s="3"/>
       <c r="M2" s="3" t="s">
         <v>316</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>208</v>
@@ -8592,7 +8721,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="43" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
@@ -8646,7 +8775,7 @@
         <v>4</v>
       </c>
       <c r="AE3" s="46" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="AF3" s="43" t="s">
         <v>12</v>
@@ -8746,7 +8875,7 @@
         <v>1</v>
       </c>
       <c r="K5" s="43" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="L5" s="3"/>
       <c r="M5" s="3" t="s">
@@ -8756,7 +8885,7 @@
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="46" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="R5" s="15" t="s">
         <v>44</v>
@@ -8826,7 +8955,7 @@
       <c r="I6" s="43"/>
       <c r="J6" s="43"/>
       <c r="K6" s="43" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
@@ -8876,12 +9005,12 @@
       <c r="I7" s="43"/>
       <c r="J7" s="43"/>
       <c r="K7" s="43" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
       <c r="N7" s="3" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="O7" s="3"/>
       <c r="P7" s="3"/>
@@ -8976,7 +9105,7 @@
       <c r="I9" s="43"/>
       <c r="J9" s="43"/>
       <c r="K9" s="43" t="s">
-        <v>843</v>
+        <v>841</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>438</v>
@@ -8985,7 +9114,7 @@
         <v>316</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>208</v>
@@ -9014,37 +9143,37 @@
     </row>
     <row r="10" spans="1:34">
       <c r="B10" s="84" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="C10" s="84"/>
       <c r="D10" s="84"/>
       <c r="E10" s="84"/>
       <c r="G10" s="84" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="H10" s="84"/>
       <c r="I10" s="84"/>
       <c r="J10" s="84"/>
       <c r="R10" s="84" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="S10" s="84"/>
       <c r="T10" s="84"/>
       <c r="U10" s="84"/>
       <c r="W10" s="84" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="X10" s="84"/>
       <c r="Y10" s="84"/>
       <c r="Z10" s="84"/>
       <c r="AA10" s="84" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="AB10" s="84"/>
       <c r="AC10" s="84"/>
       <c r="AD10" s="84"/>
       <c r="AE10" s="81" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="AF10" s="82"/>
       <c r="AG10" s="82"/>
@@ -9052,7 +9181,7 @@
     </row>
     <row r="11" spans="1:34">
       <c r="G11" s="80" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="H11" s="80"/>
       <c r="I11" s="80"/>
@@ -9220,10 +9349,10 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="43" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="B3" s="46" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
       <c r="C3" s="43" t="s">
         <v>138</v>
@@ -9232,16 +9361,16 @@
         <v>139</v>
       </c>
       <c r="E3" s="46" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="F3" s="46" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="G3" s="43"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="43" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="B4" s="43"/>
       <c r="C4" s="43"/>
@@ -9395,16 +9524,16 @@
       <c r="U2" s="43"/>
       <c r="V2" s="43"/>
       <c r="W2" s="43" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="X2" s="43" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="Y2" s="43" t="s">
         <v>316</v>
       </c>
       <c r="Z2" s="43" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="AA2" s="43" t="s">
         <v>208</v>
@@ -9413,7 +9542,7 @@
         <v>12</v>
       </c>
       <c r="AC2" s="43" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="3" spans="1:29">
@@ -9531,16 +9660,16 @@
       <c r="U4" s="43"/>
       <c r="V4" s="43"/>
       <c r="W4" s="43" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="X4" s="43" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="Y4" s="43" t="s">
         <v>316</v>
       </c>
       <c r="Z4" s="43" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="AA4" s="43" t="s">
         <v>208</v>
@@ -9549,7 +9678,7 @@
         <v>12</v>
       </c>
       <c r="AC4" s="43" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
   </sheetData>
@@ -9807,16 +9936,16 @@
       <c r="I2" s="43"/>
       <c r="J2" s="43"/>
       <c r="K2" s="43" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="L2" s="43" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="M2" s="43" t="s">
         <v>18</v>
       </c>
       <c r="N2" s="43" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="O2" s="43" t="s">
         <v>12</v>
@@ -9825,7 +9954,7 @@
         <v>13</v>
       </c>
       <c r="Q2" s="43" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="R2" s="43"/>
     </row>
@@ -9853,16 +9982,16 @@
       <c r="I3" s="43"/>
       <c r="J3" s="43"/>
       <c r="K3" s="43" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="L3" s="43" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="M3" s="43" t="s">
         <v>18</v>
       </c>
       <c r="N3" s="43" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="O3" s="43" t="s">
         <v>12</v>
@@ -9871,10 +10000,10 @@
         <v>13</v>
       </c>
       <c r="Q3" s="43" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="R3" s="43" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -9909,16 +10038,16 @@
         <v>2</v>
       </c>
       <c r="K4" s="43" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="L4" s="43" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="M4" s="43" t="s">
         <v>18</v>
       </c>
       <c r="N4" s="43" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="O4" s="43" t="s">
         <v>12</v>
@@ -9927,7 +10056,7 @@
         <v>13</v>
       </c>
       <c r="Q4" s="43" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="R4" s="43"/>
     </row>
@@ -9955,16 +10084,16 @@
       <c r="I5" s="43"/>
       <c r="J5" s="43"/>
       <c r="K5" s="43" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="L5" s="43" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="M5" s="43" t="s">
         <v>18</v>
       </c>
       <c r="N5" s="43" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="O5" s="43" t="s">
         <v>12</v>
@@ -9973,7 +10102,7 @@
         <v>13</v>
       </c>
       <c r="Q5" s="43" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="R5" s="43"/>
     </row>
@@ -10001,16 +10130,16 @@
       <c r="I6" s="43"/>
       <c r="J6" s="43"/>
       <c r="K6" s="43" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="L6" s="43" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="M6" s="43" t="s">
         <v>18</v>
       </c>
       <c r="N6" s="43" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="O6" s="43" t="s">
         <v>12</v>
@@ -10019,7 +10148,7 @@
         <v>13</v>
       </c>
       <c r="Q6" s="43" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="R6" s="43"/>
     </row>
@@ -10145,7 +10274,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="46" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="H2" s="43" t="s">
         <v>162</v>
@@ -10154,16 +10283,16 @@
         <v>163</v>
       </c>
       <c r="J2" s="55" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
       <c r="K2" s="43" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>214</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>12</v>
@@ -10172,13 +10301,13 @@
         <v>215</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>216</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>215</v>
@@ -10187,7 +10316,7 @@
         <v>163</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -10210,7 +10339,7 @@
         <v>1</v>
       </c>
       <c r="G3" s="46" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="H3" s="43" t="s">
         <v>162</v>
@@ -10219,16 +10348,16 @@
         <v>163</v>
       </c>
       <c r="J3" s="55" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="K3" s="43" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>161</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>12</v>
@@ -10237,13 +10366,13 @@
         <v>162</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>162</v>
@@ -10252,18 +10381,18 @@
         <v>163</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
     </row>
     <row r="4" spans="1:21">
       <c r="B4" s="85" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
       <c r="C4" s="86"/>
       <c r="D4" s="86"/>
       <c r="E4" s="87"/>
       <c r="F4" s="85" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="G4" s="86"/>
       <c r="H4" s="86"/>
@@ -10356,7 +10485,7 @@
         <v>147</v>
       </c>
       <c r="F1" s="41" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -10388,7 +10517,7 @@
         <v>153</v>
       </c>
       <c r="F3" s="43" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
   </sheetData>
@@ -11185,7 +11314,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
@@ -11198,7 +11327,7 @@
     <col min="9" max="9" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:16">
       <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
@@ -11226,9 +11355,30 @@
       <c r="I1" s="42" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="6" t="s">
+      <c r="J1" s="41" t="s">
+        <v>877</v>
+      </c>
+      <c r="K1" s="41" t="s">
+        <v>878</v>
+      </c>
+      <c r="L1" s="41" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" s="41" t="s">
+        <v>2</v>
+      </c>
+      <c r="N1" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="O1" s="41" t="s">
+        <v>4</v>
+      </c>
+      <c r="P1" s="41" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16">
+      <c r="A2" s="66" t="s">
         <v>49</v>
       </c>
       <c r="B2" s="43">
@@ -11250,14 +11400,21 @@
         <v>50</v>
       </c>
       <c r="H2" s="43" t="s">
-        <v>489</v>
+        <v>916</v>
       </c>
       <c r="I2" s="43" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="18" t="s">
+        <v>917</v>
+      </c>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
+    </row>
+    <row r="3" spans="1:16">
+      <c r="A3" s="38" t="s">
         <v>51</v>
       </c>
       <c r="B3" s="43">
@@ -11284,6 +11441,491 @@
       <c r="I3" s="43" t="s">
         <v>374</v>
       </c>
+      <c r="J3" s="43"/>
+      <c r="K3" s="43"/>
+      <c r="L3" s="43"/>
+      <c r="M3" s="43"/>
+      <c r="N3" s="43"/>
+      <c r="O3" s="43"/>
+      <c r="P3" s="43"/>
+    </row>
+    <row r="4" spans="1:16">
+      <c r="A4" s="43" t="s">
+        <v>879</v>
+      </c>
+      <c r="B4" s="43">
+        <v>1</v>
+      </c>
+      <c r="C4" s="46" t="s">
+        <v>327</v>
+      </c>
+      <c r="D4" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="43"/>
+      <c r="I4" s="43"/>
+      <c r="J4" s="46" t="s">
+        <v>880</v>
+      </c>
+      <c r="K4" s="43"/>
+      <c r="L4" s="43"/>
+      <c r="M4" s="43"/>
+      <c r="N4" s="43"/>
+      <c r="O4" s="43"/>
+      <c r="P4" s="43"/>
+    </row>
+    <row r="5" spans="1:16">
+      <c r="A5" s="43" t="s">
+        <v>881</v>
+      </c>
+      <c r="B5" s="43">
+        <v>1</v>
+      </c>
+      <c r="C5" s="46" t="s">
+        <v>327</v>
+      </c>
+      <c r="D5" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
+      <c r="I5" s="43"/>
+      <c r="J5" s="46" t="s">
+        <v>882</v>
+      </c>
+      <c r="K5" s="43"/>
+      <c r="L5" s="43"/>
+      <c r="M5" s="43"/>
+      <c r="N5" s="43"/>
+      <c r="O5" s="43"/>
+      <c r="P5" s="43"/>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="A6" s="43" t="s">
+        <v>883</v>
+      </c>
+      <c r="B6" s="43">
+        <v>1</v>
+      </c>
+      <c r="C6" s="46" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="43"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="46" t="s">
+        <v>884</v>
+      </c>
+      <c r="K6" s="43"/>
+      <c r="L6" s="43"/>
+      <c r="M6" s="43"/>
+      <c r="N6" s="43"/>
+      <c r="O6" s="43"/>
+      <c r="P6" s="43"/>
+    </row>
+    <row r="7" spans="1:16">
+      <c r="A7" s="43" t="s">
+        <v>885</v>
+      </c>
+      <c r="B7" s="43">
+        <v>1</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>327</v>
+      </c>
+      <c r="D7" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
+      <c r="K7" s="43"/>
+      <c r="L7" s="43"/>
+      <c r="M7" s="43"/>
+      <c r="N7" s="43"/>
+      <c r="O7" s="43"/>
+      <c r="P7" s="43"/>
+    </row>
+    <row r="8" spans="1:16">
+      <c r="A8" s="43" t="s">
+        <v>886</v>
+      </c>
+      <c r="B8" s="43">
+        <v>1</v>
+      </c>
+      <c r="C8" s="46" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="43"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="43"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="46" t="s">
+        <v>887</v>
+      </c>
+      <c r="K8" s="43"/>
+      <c r="L8" s="43"/>
+      <c r="M8" s="43"/>
+      <c r="N8" s="43"/>
+      <c r="O8" s="43"/>
+      <c r="P8" s="43"/>
+    </row>
+    <row r="9" spans="1:16">
+      <c r="A9" s="43" t="s">
+        <v>888</v>
+      </c>
+      <c r="B9" s="43">
+        <v>1</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>327</v>
+      </c>
+      <c r="D9" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="43"/>
+      <c r="H9" s="43" t="s">
+        <v>902</v>
+      </c>
+      <c r="I9" s="43" t="s">
+        <v>903</v>
+      </c>
+      <c r="J9" s="43"/>
+      <c r="K9" s="43"/>
+      <c r="L9" s="43"/>
+      <c r="M9" s="43"/>
+      <c r="N9" s="43"/>
+      <c r="O9" s="43"/>
+      <c r="P9" s="43"/>
+    </row>
+    <row r="10" spans="1:16">
+      <c r="A10" s="43" t="s">
+        <v>889</v>
+      </c>
+      <c r="B10" s="43">
+        <v>1</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>327</v>
+      </c>
+      <c r="D10" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="43"/>
+      <c r="H10" s="43" t="s">
+        <v>904</v>
+      </c>
+      <c r="I10" s="43" t="s">
+        <v>905</v>
+      </c>
+      <c r="J10" s="43"/>
+      <c r="K10" s="43"/>
+      <c r="L10" s="43"/>
+      <c r="M10" s="43"/>
+      <c r="N10" s="43"/>
+      <c r="O10" s="43"/>
+      <c r="P10" s="43"/>
+    </row>
+    <row r="11" spans="1:16">
+      <c r="A11" s="53" t="s">
+        <v>890</v>
+      </c>
+      <c r="B11" s="43">
+        <v>1</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>327</v>
+      </c>
+      <c r="D11" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="43"/>
+      <c r="H11" s="43" t="s">
+        <v>906</v>
+      </c>
+      <c r="I11" s="43" t="s">
+        <v>907</v>
+      </c>
+      <c r="J11" s="43"/>
+      <c r="K11" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="L11" s="43"/>
+      <c r="M11" s="43"/>
+      <c r="N11" s="43"/>
+      <c r="O11" s="43"/>
+      <c r="P11" s="43"/>
+    </row>
+    <row r="12" spans="1:16">
+      <c r="A12" s="53" t="s">
+        <v>891</v>
+      </c>
+      <c r="B12" s="43">
+        <v>1</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>327</v>
+      </c>
+      <c r="D12" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="43"/>
+      <c r="H12" s="43" t="s">
+        <v>908</v>
+      </c>
+      <c r="I12" s="43" t="s">
+        <v>909</v>
+      </c>
+      <c r="J12" s="46" t="s">
+        <v>892</v>
+      </c>
+      <c r="K12" s="43"/>
+      <c r="L12" s="43">
+        <v>1</v>
+      </c>
+      <c r="M12" s="46" t="s">
+        <v>439</v>
+      </c>
+      <c r="N12" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="O12" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="P12" s="43" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16">
+      <c r="A13" s="53" t="s">
+        <v>893</v>
+      </c>
+      <c r="B13" s="43">
+        <v>1</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>175</v>
+      </c>
+      <c r="D13" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="43"/>
+      <c r="H13" s="43" t="s">
+        <v>910</v>
+      </c>
+      <c r="I13" s="43" t="s">
+        <v>911</v>
+      </c>
+      <c r="J13" s="46" t="s">
+        <v>894</v>
+      </c>
+      <c r="K13" s="43"/>
+      <c r="L13" s="43"/>
+      <c r="M13" s="43"/>
+      <c r="N13" s="43"/>
+      <c r="O13" s="43"/>
+      <c r="P13" s="43"/>
+    </row>
+    <row r="14" spans="1:16">
+      <c r="A14" s="53" t="s">
+        <v>895</v>
+      </c>
+      <c r="B14" s="43">
+        <v>1</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>175</v>
+      </c>
+      <c r="D14" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="43"/>
+      <c r="H14" s="43" t="s">
+        <v>912</v>
+      </c>
+      <c r="I14" s="43" t="s">
+        <v>913</v>
+      </c>
+      <c r="J14" s="46" t="s">
+        <v>896</v>
+      </c>
+      <c r="K14" s="43"/>
+      <c r="L14" s="43">
+        <v>1</v>
+      </c>
+      <c r="M14" s="46" t="s">
+        <v>439</v>
+      </c>
+      <c r="N14" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="O14" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="P14" s="43" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16">
+      <c r="A15" s="53" t="s">
+        <v>897</v>
+      </c>
+      <c r="B15" s="43">
+        <v>1</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>439</v>
+      </c>
+      <c r="D15" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="43" t="s">
+        <v>334</v>
+      </c>
+      <c r="F15" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="43"/>
+      <c r="H15" s="43" t="s">
+        <v>914</v>
+      </c>
+      <c r="I15" s="43" t="s">
+        <v>915</v>
+      </c>
+      <c r="J15" s="46" t="s">
+        <v>898</v>
+      </c>
+      <c r="K15" s="43"/>
+      <c r="L15" s="43"/>
+      <c r="M15" s="43"/>
+      <c r="N15" s="43"/>
+      <c r="O15" s="43"/>
+      <c r="P15" s="43"/>
+    </row>
+    <row r="16" spans="1:16">
+      <c r="A16" s="53" t="s">
+        <v>899</v>
+      </c>
+      <c r="B16" s="43">
+        <v>1</v>
+      </c>
+      <c r="C16" s="46" t="s">
+        <v>175</v>
+      </c>
+      <c r="D16" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="43"/>
+      <c r="H16" s="43" t="s">
+        <v>918</v>
+      </c>
+      <c r="I16" s="43" t="s">
+        <v>919</v>
+      </c>
+      <c r="J16" s="46" t="s">
+        <v>865</v>
+      </c>
+      <c r="K16" s="43"/>
+      <c r="L16" s="43"/>
+      <c r="M16" s="43"/>
+      <c r="N16" s="43"/>
+      <c r="O16" s="43"/>
+      <c r="P16" s="43"/>
+    </row>
+    <row r="17" spans="1:16">
+      <c r="A17" s="53" t="s">
+        <v>900</v>
+      </c>
+      <c r="B17" s="43">
+        <v>1</v>
+      </c>
+      <c r="C17" s="46" t="s">
+        <v>175</v>
+      </c>
+      <c r="D17" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="43"/>
+      <c r="H17" s="43" t="s">
+        <v>920</v>
+      </c>
+      <c r="I17" s="43" t="s">
+        <v>921</v>
+      </c>
+      <c r="J17" s="46" t="s">
+        <v>901</v>
+      </c>
+      <c r="K17" s="43"/>
+      <c r="L17" s="43"/>
+      <c r="M17" s="43"/>
+      <c r="N17" s="43"/>
+      <c r="O17" s="43"/>
+      <c r="P17" s="43"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11483,7 +12125,7 @@
       <c r="H6" s="43"/>
       <c r="I6" s="43"/>
       <c r="J6" s="43" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="K6" s="43"/>
       <c r="L6" s="43"/>
@@ -11536,7 +12178,7 @@
         <v>56</v>
       </c>
       <c r="C1" s="44" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="D1" s="44" t="s">
         <v>28</v>
@@ -11545,55 +12187,55 @@
         <v>56</v>
       </c>
       <c r="F1" s="44" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="G1" s="44" t="s">
         <v>28</v>
       </c>
       <c r="H1" s="33" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="I1" s="33" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="J1" s="33" t="s">
         <v>142</v>
       </c>
       <c r="K1" s="44" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="L1" s="44" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="M1" s="64" t="s">
         <v>74</v>
       </c>
       <c r="N1" s="65" t="s">
+        <v>567</v>
+      </c>
+      <c r="O1" s="65" t="s">
+        <v>568</v>
+      </c>
+      <c r="P1" s="65" t="s">
         <v>569</v>
       </c>
-      <c r="O1" s="65" t="s">
+      <c r="Q1" s="65" t="s">
         <v>570</v>
       </c>
-      <c r="P1" s="65" t="s">
+      <c r="R1" s="65" t="s">
         <v>571</v>
       </c>
-      <c r="Q1" s="65" t="s">
+      <c r="S1" s="33" t="s">
+        <v>577</v>
+      </c>
+      <c r="T1" s="33" t="s">
+        <v>578</v>
+      </c>
+      <c r="U1" s="64" t="s">
         <v>572</v>
       </c>
-      <c r="R1" s="65" t="s">
+      <c r="V1" s="64" t="s">
         <v>573</v>
-      </c>
-      <c r="S1" s="33" t="s">
-        <v>579</v>
-      </c>
-      <c r="T1" s="33" t="s">
-        <v>580</v>
-      </c>
-      <c r="U1" s="64" t="s">
-        <v>574</v>
-      </c>
-      <c r="V1" s="64" t="s">
-        <v>575</v>
       </c>
       <c r="W1" s="42" t="s">
         <v>194</v>
@@ -11637,7 +12279,7 @@
         <v>14</v>
       </c>
       <c r="M2" s="32" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="N2" s="32">
         <v>2</v>
@@ -11657,10 +12299,10 @@
       <c r="S2" s="32"/>
       <c r="T2" s="32"/>
       <c r="U2" s="43" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="V2" s="43" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="W2" s="43" t="s">
         <v>374</v>
@@ -11704,7 +12346,7 @@
         <v>14</v>
       </c>
       <c r="M3" s="32" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="N3" s="32"/>
       <c r="O3" s="32"/>
@@ -11718,13 +12360,13 @@
         <v>314</v>
       </c>
       <c r="U3" s="43" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="V3" s="43" t="s">
+        <v>580</v>
+      </c>
+      <c r="W3" s="43" t="s">
         <v>582</v>
-      </c>
-      <c r="W3" s="43" t="s">
-        <v>584</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -11765,7 +12407,7 @@
         <v>14</v>
       </c>
       <c r="M4" s="32" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="N4" s="32"/>
       <c r="O4" s="32"/>
@@ -11779,10 +12421,10 @@
       <c r="S4" s="32"/>
       <c r="T4" s="32"/>
       <c r="U4" s="43" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="V4" s="43" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="W4" s="43" t="s">
         <v>374</v>
@@ -12386,7 +13028,7 @@
       </c>
       <c r="G4" s="43"/>
       <c r="H4" s="43" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="I4" s="43" t="s">
         <v>377</v>
@@ -12423,7 +13065,7 @@
       </c>
       <c r="G5" s="43"/>
       <c r="H5" s="43" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="I5" s="43" t="s">
         <v>377</v>
@@ -12616,7 +13258,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="32.1796875" style="40" customWidth="1"/>
@@ -12624,10 +13266,11 @@
     <col min="3" max="3" width="16.6328125" style="40" customWidth="1"/>
     <col min="4" max="4" width="17.6328125" style="40" customWidth="1"/>
     <col min="5" max="5" width="11.81640625" style="40" customWidth="1"/>
-    <col min="6" max="16384" width="8.90625" style="40"/>
+    <col min="6" max="6" width="12.08984375" style="40" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.90625" style="40"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="41" t="s">
         <v>0</v>
       </c>
@@ -12643,8 +13286,11 @@
       <c r="E1" s="41" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" s="41" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" s="43" t="s">
         <v>408</v>
       </c>
@@ -12660,8 +13306,9 @@
       <c r="E2" s="43" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="F2" s="43"/>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" s="43" t="s">
         <v>409</v>
       </c>
@@ -12677,8 +13324,9 @@
       <c r="E3" s="43" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F3" s="43"/>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" s="43" t="s">
         <v>411</v>
       </c>
@@ -12694,6 +13342,7 @@
       <c r="E4" s="43" t="s">
         <v>14</v>
       </c>
+      <c r="F4" s="43"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12925,7 +13574,7 @@
         <v>211</v>
       </c>
       <c r="J2" s="43" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="K2" s="43">
         <v>2</v>
@@ -13076,19 +13725,19 @@
         <v>40</v>
       </c>
       <c r="F1" s="44" t="s">
+        <v>583</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>584</v>
+      </c>
+      <c r="H1" s="12" t="s">
         <v>585</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="I1" s="12" t="s">
         <v>586</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="J1" s="12" t="s">
         <v>587</v>
-      </c>
-      <c r="I1" s="12" t="s">
-        <v>588</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>589</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -13137,7 +13786,7 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="43" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="B4" s="43">
         <v>1</v>
@@ -13157,7 +13806,7 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="43" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="B5" s="43">
         <v>1</v>
@@ -13167,7 +13816,7 @@
         <v>34</v>
       </c>
       <c r="E5" s="43" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="F5" s="43"/>
       <c r="G5" s="43"/>
@@ -13177,7 +13826,7 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="43" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B6" s="43">
         <v>1</v>
@@ -13187,13 +13836,13 @@
         <v>34</v>
       </c>
       <c r="E6" s="43" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="F6" s="43">
         <v>2</v>
       </c>
       <c r="G6" s="43" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="H6" s="43" t="s">
         <v>34</v>
@@ -13203,7 +13852,7 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="43" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="B7" s="43">
         <v>1</v>
@@ -13213,13 +13862,13 @@
         <v>34</v>
       </c>
       <c r="E7" s="43" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="F7" s="43">
         <v>2</v>
       </c>
       <c r="G7" s="43" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="H7" s="43" t="s">
         <v>34</v>
@@ -13229,7 +13878,7 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="43" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="B8" s="43">
         <v>1</v>
@@ -13239,13 +13888,13 @@
         <v>34</v>
       </c>
       <c r="E8" s="43" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="F8" s="43">
         <v>2</v>
       </c>
       <c r="G8" s="43" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="H8" s="43" t="s">
         <v>34</v>
@@ -13255,7 +13904,7 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="43" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B9" s="43">
         <v>1</v>
@@ -13265,25 +13914,25 @@
         <v>34</v>
       </c>
       <c r="E9" s="43" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="F9" s="43">
         <v>2</v>
       </c>
       <c r="G9" s="43" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="H9" s="43" t="s">
         <v>34</v>
       </c>
       <c r="I9" s="46" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="J9" s="43"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="43" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="B10" s="43">
         <v>1</v>
@@ -13293,7 +13942,7 @@
         <v>34</v>
       </c>
       <c r="E10" s="43" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="F10" s="43"/>
       <c r="G10" s="43"/>
@@ -13303,7 +13952,7 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="43" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="B11" s="43">
         <v>1</v>
@@ -13313,13 +13962,13 @@
         <v>34</v>
       </c>
       <c r="E11" s="43" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="F11" s="43">
         <v>2</v>
       </c>
       <c r="G11" s="43" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="H11" s="43" t="s">
         <v>34</v>
@@ -13329,7 +13978,7 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="43" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="B12" s="43">
         <v>1</v>
@@ -13339,13 +13988,13 @@
         <v>34</v>
       </c>
       <c r="E12" s="43" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="F12" s="43">
         <v>2</v>
       </c>
       <c r="G12" s="43" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="H12" s="43" t="s">
         <v>34</v>
@@ -13355,7 +14004,7 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="43" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B13" s="43">
         <v>1</v>
@@ -13365,19 +14014,19 @@
         <v>34</v>
       </c>
       <c r="E13" s="43" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
       <c r="H13" s="43"/>
       <c r="I13" s="43"/>
       <c r="J13" s="43" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="43" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="B14" s="43">
         <v>1</v>
@@ -13387,7 +14036,7 @@
         <v>34</v>
       </c>
       <c r="E14" s="43" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="F14" s="43"/>
       <c r="G14" s="43"/>
@@ -13397,7 +14046,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="43" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B15" s="43">
         <v>1</v>
@@ -13407,13 +14056,13 @@
         <v>34</v>
       </c>
       <c r="E15" s="43" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="F15" s="43">
         <v>2</v>
       </c>
       <c r="G15" s="43" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="H15" s="43" t="s">
         <v>34</v>
@@ -13423,7 +14072,7 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="43" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B16" s="43">
         <v>1</v>
@@ -13433,13 +14082,13 @@
         <v>34</v>
       </c>
       <c r="E16" s="43" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="F16" s="43">
         <v>2</v>
       </c>
       <c r="G16" s="43" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="H16" s="43" t="s">
         <v>34</v>
@@ -13449,7 +14098,7 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="43" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="B17" s="43">
         <v>1</v>
@@ -13459,13 +14108,13 @@
         <v>34</v>
       </c>
       <c r="E17" s="43" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="F17" s="43">
         <v>2</v>
       </c>
       <c r="G17" s="43" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="H17" s="43" t="s">
         <v>34</v>
@@ -13475,7 +14124,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="43" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="B18" s="43">
         <v>1</v>
@@ -13485,13 +14134,13 @@
         <v>34</v>
       </c>
       <c r="E18" s="43" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="F18" s="43">
         <v>2</v>
       </c>
       <c r="G18" s="43" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="H18" s="43" t="s">
         <v>34</v>
@@ -13501,7 +14150,7 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="43" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="B19" s="43">
         <v>1</v>
@@ -13519,7 +14168,7 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="43" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="B20" s="43">
         <v>1</v>
@@ -13527,7 +14176,7 @@
       <c r="C20" s="43"/>
       <c r="D20" s="43"/>
       <c r="E20" s="43" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="F20" s="43"/>
       <c r="G20" s="43"/>
@@ -13537,7 +14186,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="43" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="B21" s="43">
         <v>1</v>
@@ -13547,13 +14196,13 @@
         <v>34</v>
       </c>
       <c r="E21" s="43" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="F21" s="43">
         <v>2</v>
       </c>
       <c r="G21" s="43" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="H21" s="43" t="s">
         <v>34</v>
@@ -13563,7 +14212,7 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="43" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="B22" s="43">
         <v>1</v>
@@ -13589,59 +14238,59 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="43" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="B23" s="43">
         <v>1</v>
       </c>
       <c r="C23" s="43"/>
       <c r="D23" s="43" t="s">
+        <v>590</v>
+      </c>
+      <c r="E23" s="43" t="s">
         <v>592</v>
-      </c>
-      <c r="E23" s="43" t="s">
-        <v>594</v>
       </c>
       <c r="F23" s="43">
         <v>2</v>
       </c>
       <c r="G23" s="43" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="H23" s="43" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="I23" s="43"/>
       <c r="J23" s="43"/>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="43" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="B24" s="43">
         <v>1</v>
       </c>
       <c r="C24" s="43"/>
       <c r="D24" s="43" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E24" s="43" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="F24" s="43">
         <v>2</v>
       </c>
       <c r="G24" s="43" t="s">
+        <v>590</v>
+      </c>
+      <c r="H24" s="43" t="s">
         <v>592</v>
-      </c>
-      <c r="H24" s="43" t="s">
-        <v>594</v>
       </c>
       <c r="I24" s="43"/>
       <c r="J24" s="43"/>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="43" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="B25" s="43">
         <v>1</v>
@@ -13651,7 +14300,7 @@
         <v>34</v>
       </c>
       <c r="E25" s="43" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="F25" s="43"/>
       <c r="G25" s="43"/>
@@ -13661,7 +14310,7 @@
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="43" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="B26" s="43">
         <v>1</v>
@@ -13671,13 +14320,13 @@
         <v>34</v>
       </c>
       <c r="E26" s="43" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="F26" s="43">
         <v>2</v>
       </c>
       <c r="G26" s="43" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="H26" s="43" t="s">
         <v>34</v>
@@ -13687,7 +14336,7 @@
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="43" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="B27" s="43">
         <v>1</v>
@@ -13707,7 +14356,7 @@
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="43" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B28" s="43">
         <v>1</v>
@@ -13763,7 +14412,7 @@
         <v>30</v>
       </c>
       <c r="F1" s="44" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -13858,7 +14507,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="13" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="B7" s="13">
         <v>1</v>
@@ -13874,7 +14523,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="13" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="B8" s="13">
         <v>1</v>
@@ -13890,13 +14539,13 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="13" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="B9" s="43">
         <v>2</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
       <c r="D9" s="45" t="s">
         <v>12</v>
@@ -14052,7 +14701,7 @@
       <c r="M2" s="32"/>
       <c r="N2" s="32"/>
       <c r="O2" s="32" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="P2" s="32"/>
       <c r="Q2" s="32" t="s">
@@ -14197,7 +14846,7 @@
         <v>15</v>
       </c>
       <c r="H6" s="32" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="I6" s="32" t="s">
         <v>377</v>
@@ -14245,7 +14894,7 @@
         <v>19</v>
       </c>
       <c r="H7" s="32" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="I7" s="32" t="s">
         <v>350</v>
@@ -14363,7 +15012,7 @@
       </c>
       <c r="G10" s="55"/>
       <c r="H10" s="32" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="I10" s="32"/>
       <c r="J10" s="32" t="s">
@@ -14411,7 +15060,7 @@
         <v>15</v>
       </c>
       <c r="H11" s="32" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="I11" s="32" t="s">
         <v>210</v>
@@ -14463,7 +15112,7 @@
       </c>
       <c r="G12" s="55"/>
       <c r="H12" s="32" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="I12" s="32" t="s">
         <v>366</v>
@@ -14551,7 +15200,7 @@
       </c>
       <c r="G14" s="55"/>
       <c r="H14" s="32" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="I14" s="32" t="s">
         <v>243</v>
@@ -14601,7 +15250,7 @@
         <v>15</v>
       </c>
       <c r="H15" s="32" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="I15" s="32" t="s">
         <v>357</v>
@@ -15167,16 +15816,16 @@
         <v>58</v>
       </c>
       <c r="X1" s="44" t="s">
+        <v>618</v>
+      </c>
+      <c r="Y1" s="44" t="s">
+        <v>619</v>
+      </c>
+      <c r="Z1" s="44" t="s">
         <v>620</v>
       </c>
-      <c r="Y1" s="44" t="s">
+      <c r="AA1" s="44" t="s">
         <v>621</v>
-      </c>
-      <c r="Z1" s="44" t="s">
-        <v>622</v>
-      </c>
-      <c r="AA1" s="44" t="s">
-        <v>623</v>
       </c>
       <c r="AB1" s="44" t="s">
         <v>1</v>
@@ -15214,7 +15863,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>13</v>
@@ -15235,10 +15884,10 @@
       <c r="P2" s="43"/>
       <c r="Q2" s="43"/>
       <c r="R2" s="43" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="S2" s="43" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="T2" s="43"/>
       <c r="U2" s="43"/>
@@ -15266,7 +15915,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>13</v>
@@ -15338,7 +15987,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>13</v>
@@ -15575,10 +16224,10 @@
       <c r="P8" s="43"/>
       <c r="Q8" s="43"/>
       <c r="R8" s="43" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="S8" s="43" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="T8" s="43">
         <v>0</v>
@@ -15637,10 +16286,10 @@
       <c r="P9" s="43"/>
       <c r="Q9" s="43"/>
       <c r="R9" s="43" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="S9" s="43" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="T9" s="43"/>
       <c r="U9" s="43">
@@ -15703,10 +16352,10 @@
       <c r="P10" s="43"/>
       <c r="Q10" s="43"/>
       <c r="R10" s="43" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="S10" s="43" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="T10" s="43"/>
       <c r="U10" s="43"/>
@@ -16007,10 +16656,10 @@
       <c r="P16" s="43"/>
       <c r="Q16" s="43"/>
       <c r="R16" s="43" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="S16" s="43" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="T16" s="43"/>
       <c r="U16" s="43"/>
@@ -16080,7 +16729,7 @@
     </row>
     <row r="18" spans="1:36">
       <c r="A18" s="66" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="B18" s="68">
         <v>1</v>
@@ -16115,7 +16764,7 @@
       <c r="P18" s="43"/>
       <c r="Q18" s="43"/>
       <c r="R18" s="43" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="S18" s="43"/>
       <c r="T18" s="46">
@@ -16140,7 +16789,7 @@
     </row>
     <row r="19" spans="1:36">
       <c r="A19" s="66" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B19" s="68">
         <v>1</v>
@@ -16158,7 +16807,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="46" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="H19" s="43" t="s">
         <v>12</v>
@@ -16170,7 +16819,7 @@
         <v>2</v>
       </c>
       <c r="K19" s="46" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="L19" s="43" t="s">
         <v>215</v>
@@ -16191,7 +16840,7 @@
         <v>34</v>
       </c>
       <c r="R19" s="43" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="S19" s="43"/>
       <c r="T19" s="46">
@@ -16216,13 +16865,13 @@
     </row>
     <row r="20" spans="1:36">
       <c r="A20" s="66" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B20" s="68">
         <v>1</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>163</v>
@@ -16234,19 +16883,19 @@
         <v>1</v>
       </c>
       <c r="G20" s="46" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="H20" s="43" t="s">
         <v>13</v>
       </c>
       <c r="I20" s="43" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="J20" s="43">
         <v>2</v>
       </c>
       <c r="K20" s="46" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="L20" s="43" t="s">
         <v>13</v>
@@ -16258,7 +16907,7 @@
         <v>2</v>
       </c>
       <c r="O20" s="46" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="P20" s="43" t="s">
         <v>163</v>
@@ -16267,7 +16916,7 @@
         <v>12</v>
       </c>
       <c r="R20" s="43" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="S20" s="43"/>
       <c r="T20" s="46">
@@ -16292,7 +16941,7 @@
     </row>
     <row r="21" spans="1:36">
       <c r="A21" s="66" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="B21" s="68">
         <v>1</v>
@@ -16329,7 +16978,7 @@
       <c r="P21" s="43"/>
       <c r="Q21" s="43"/>
       <c r="R21" s="43" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="S21" s="43"/>
       <c r="T21" s="46">
@@ -16339,16 +16988,16 @@
       <c r="V21" s="43"/>
       <c r="W21" s="43"/>
       <c r="X21" s="43" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="Y21" s="43" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="Z21" s="43" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="AA21" s="43" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="AB21" s="43"/>
       <c r="AC21" s="43"/>
@@ -16362,7 +17011,7 @@
     </row>
     <row r="22" spans="1:36">
       <c r="A22" s="66" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B22" s="68"/>
       <c r="C22" s="16"/>
@@ -16406,7 +17055,7 @@
     </row>
     <row r="23" spans="1:36">
       <c r="A23" s="66" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="B23" s="68">
         <v>1</v>
@@ -16454,7 +17103,7 @@
     </row>
     <row r="24" spans="1:36">
       <c r="A24" s="66" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="B24" s="68">
         <v>1</v>
@@ -16489,7 +17138,7 @@
       <c r="P24" s="43"/>
       <c r="Q24" s="43"/>
       <c r="R24" s="43" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="S24" s="43"/>
       <c r="T24" s="46"/>
@@ -16512,13 +17161,13 @@
     </row>
     <row r="25" spans="1:36">
       <c r="A25" s="66" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B25" s="68">
         <v>1</v>
       </c>
       <c r="C25" s="46" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>12</v>
@@ -16560,7 +17209,7 @@
     </row>
     <row r="26" spans="1:36">
       <c r="A26" s="66" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="B26" s="68">
         <v>1</v>
@@ -16593,10 +17242,10 @@
       <c r="V26" s="43"/>
       <c r="W26" s="43"/>
       <c r="X26" s="43" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="Y26" s="43" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="Z26" s="43"/>
       <c r="AA26" s="43"/>
@@ -16612,7 +17261,7 @@
     </row>
     <row r="27" spans="1:36">
       <c r="A27" s="66" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B27" s="68">
         <v>1</v>
@@ -16645,10 +17294,10 @@
       <c r="V27" s="43"/>
       <c r="W27" s="43"/>
       <c r="X27" s="43" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="Y27" s="43" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="Z27" s="43"/>
       <c r="AA27" s="43"/>
@@ -16664,7 +17313,7 @@
     </row>
     <row r="28" spans="1:36">
       <c r="A28" s="66" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="B28" s="68">
         <v>1</v>
@@ -16691,7 +17340,7 @@
       <c r="P28" s="43"/>
       <c r="Q28" s="43"/>
       <c r="R28" s="43" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="S28" s="43"/>
       <c r="T28" s="46">
@@ -16718,7 +17367,7 @@
     </row>
     <row r="29" spans="1:36">
       <c r="A29" s="38" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="B29" s="68">
         <v>1</v>
@@ -16748,7 +17397,7 @@
         <v>2</v>
       </c>
       <c r="K29" s="46" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="L29" s="43" t="s">
         <v>47</v>
@@ -16784,7 +17433,7 @@
         <v>3</v>
       </c>
       <c r="AC29" s="46" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="AD29" s="43" t="s">
         <v>45</v>
@@ -16796,7 +17445,7 @@
         <v>3</v>
       </c>
       <c r="AG29" s="46" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="AH29" s="43" t="s">
         <v>12</v>
@@ -16808,13 +17457,13 @@
     </row>
     <row r="30" spans="1:36">
       <c r="A30" s="66" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="B30" s="68">
         <v>1</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>12</v>
@@ -16835,7 +17484,7 @@
       <c r="P30" s="43"/>
       <c r="Q30" s="43"/>
       <c r="R30" s="43" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="S30" s="43"/>
       <c r="T30" s="43">
@@ -16864,7 +17513,7 @@
     </row>
     <row r="31" spans="1:36">
       <c r="A31" s="66" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B31" s="68">
         <v>1</v>
@@ -16891,7 +17540,7 @@
       <c r="P31" s="43"/>
       <c r="Q31" s="43"/>
       <c r="R31" s="43" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="S31" s="43"/>
       <c r="T31" s="43">
@@ -16920,7 +17569,7 @@
     </row>
     <row r="32" spans="1:36">
       <c r="A32" s="66" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="B32" s="68">
         <v>1</v>
@@ -16947,7 +17596,7 @@
       <c r="P32" s="43"/>
       <c r="Q32" s="43"/>
       <c r="R32" s="43" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="S32" s="43"/>
       <c r="T32" s="43">
@@ -16976,7 +17625,7 @@
     </row>
     <row r="33" spans="1:36">
       <c r="A33" s="66" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="B33" s="68">
         <v>1</v>
@@ -17003,7 +17652,7 @@
       <c r="P33" s="43"/>
       <c r="Q33" s="43"/>
       <c r="R33" s="43" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="S33" s="43"/>
       <c r="T33" s="43">
@@ -17032,7 +17681,7 @@
     </row>
     <row r="34" spans="1:36">
       <c r="A34" s="66" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="B34" s="68">
         <v>1</v>
@@ -17059,7 +17708,7 @@
       <c r="P34" s="43"/>
       <c r="Q34" s="43"/>
       <c r="R34" s="43" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="S34" s="43"/>
       <c r="T34" s="43">
@@ -17088,7 +17737,7 @@
     </row>
     <row r="35" spans="1:36">
       <c r="A35" s="66" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="B35" s="68">
         <v>1</v>
@@ -17115,7 +17764,7 @@
       <c r="P35" s="43"/>
       <c r="Q35" s="43"/>
       <c r="R35" s="43" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="S35" s="43"/>
       <c r="T35" s="43">
@@ -17144,7 +17793,7 @@
     </row>
     <row r="36" spans="1:36">
       <c r="A36" s="66" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="B36" s="68">
         <v>1</v>
@@ -17171,7 +17820,7 @@
       <c r="P36" s="43"/>
       <c r="Q36" s="43"/>
       <c r="R36" s="43" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="S36" s="43"/>
       <c r="T36" s="43">
@@ -17200,7 +17849,7 @@
     </row>
     <row r="37" spans="1:36">
       <c r="A37" s="38" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B37" s="68">
         <v>1</v>
@@ -17227,7 +17876,7 @@
       <c r="P37" s="43"/>
       <c r="Q37" s="43"/>
       <c r="R37" s="43" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="S37" s="43"/>
       <c r="T37" s="43">
@@ -17256,7 +17905,7 @@
     </row>
     <row r="38" spans="1:36">
       <c r="A38" s="66" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="B38" s="68">
         <v>1</v>
@@ -17283,7 +17932,7 @@
       <c r="P38" s="43"/>
       <c r="Q38" s="43"/>
       <c r="R38" s="43" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="S38" s="43"/>
       <c r="T38" s="43">
@@ -17309,12 +17958,12 @@
       <c r="AH38" s="43"/>
       <c r="AI38" s="43"/>
       <c r="AJ38" s="46" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="39" spans="1:36">
       <c r="A39" s="66" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="B39" s="68">
         <v>1</v>
@@ -17341,7 +17990,7 @@
       <c r="P39" s="43"/>
       <c r="Q39" s="43"/>
       <c r="R39" s="43" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="S39" s="43" t="s">
         <v>374</v>

</xml_diff>

<commit_message>
ModifySeatMap and CrewReportService updated
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3C71EAE-F6ED-454E-8A16-4B68590B79E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8226D3C0-7880-4B38-B281-00377BA3475F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="32" activeTab="35" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2854" uniqueCount="948">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2853" uniqueCount="945">
   <si>
     <t>Scenario</t>
   </si>
@@ -2719,18 +2719,6 @@
     <t>36</t>
   </si>
   <si>
-    <t>BCHVUB</t>
-  </si>
-  <si>
-    <t>2023-09-01T13:08:26</t>
-  </si>
-  <si>
-    <t>BCHVWQ</t>
-  </si>
-  <si>
-    <t>2023-09-01T13:08:29</t>
-  </si>
-  <si>
     <t>2nd Seg</t>
   </si>
   <si>
@@ -2918,13 +2906,15 @@
   </si>
   <si>
     <t>2023-09-03T20:15:46</t>
+  </si>
+  <si>
+    <t>Crew_Report_Services_PR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="15">
     <font>
       <sz val="11"/>
@@ -3690,23 +3680,23 @@
   <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="52.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="8.1796875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.1796875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="11.6328125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="12.6328125"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="1" max="1" width="52.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27">
@@ -3815,7 +3805,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="42" t="s">
-        <v>893</v>
+        <v>889</v>
       </c>
       <c r="I2" s="42" t="s">
         <v>206</v>
@@ -3832,7 +3822,7 @@
       <c r="M2" s="42"/>
       <c r="N2" s="42"/>
       <c r="O2" s="42" t="s">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="P2" s="42"/>
       <c r="Q2" s="42"/>
@@ -3870,7 +3860,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="42" t="s">
-        <v>892</v>
+        <v>888</v>
       </c>
       <c r="I3" s="42" t="s">
         <v>207</v>
@@ -3879,13 +3869,13 @@
         <v>206</v>
       </c>
       <c r="K3" s="42" t="s">
-        <v>890</v>
+        <v>886</v>
       </c>
       <c r="L3" s="42" t="s">
         <v>206</v>
       </c>
       <c r="M3" s="42" t="s">
-        <v>891</v>
+        <v>887</v>
       </c>
       <c r="N3" s="42" t="s">
         <v>206</v>
@@ -3912,7 +3902,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="D4" s="42" t="s">
         <v>12</v>
@@ -3927,7 +3917,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="36" t="s">
-        <v>899</v>
+        <v>895</v>
       </c>
       <c r="I4" s="36" t="s">
         <v>337</v>
@@ -3944,7 +3934,7 @@
         <v>358</v>
       </c>
       <c r="Q4" s="42" t="s">
-        <v>895</v>
+        <v>891</v>
       </c>
       <c r="R4" s="42"/>
       <c r="S4" s="42"/>
@@ -3965,7 +3955,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="45" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="D5" s="42" t="s">
         <v>12</v>
@@ -3980,7 +3970,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="36" t="s">
-        <v>900</v>
+        <v>896</v>
       </c>
       <c r="I5" s="42" t="s">
         <v>207</v>
@@ -3989,7 +3979,7 @@
         <v>741</v>
       </c>
       <c r="K5" s="42" t="s">
-        <v>890</v>
+        <v>886</v>
       </c>
       <c r="L5" s="42" t="s">
         <v>741</v>
@@ -4001,7 +3991,7 @@
         <v>358</v>
       </c>
       <c r="Q5" s="42" t="s">
-        <v>895</v>
+        <v>891</v>
       </c>
       <c r="R5" s="42"/>
       <c r="S5" s="42"/>
@@ -4022,7 +4012,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="D6" s="42" t="s">
         <v>12</v>
@@ -4035,7 +4025,7 @@
       </c>
       <c r="G6" s="42"/>
       <c r="H6" s="42" t="s">
-        <v>909</v>
+        <v>905</v>
       </c>
       <c r="I6" s="42" t="s">
         <v>692</v>
@@ -4052,7 +4042,7 @@
         <v>358</v>
       </c>
       <c r="Q6" s="42" t="s">
-        <v>895</v>
+        <v>891</v>
       </c>
       <c r="R6" s="42"/>
       <c r="S6" s="42"/>
@@ -4073,7 +4063,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="D7" s="42" t="s">
         <v>12</v>
@@ -4086,7 +4076,7 @@
       </c>
       <c r="G7" s="42"/>
       <c r="H7" s="42" t="s">
-        <v>896</v>
+        <v>892</v>
       </c>
       <c r="I7" s="42" t="s">
         <v>695</v>
@@ -4120,7 +4110,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="45" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="D8" s="42" t="s">
         <v>12</v>
@@ -4133,7 +4123,7 @@
       </c>
       <c r="G8" s="42"/>
       <c r="H8" s="42" t="s">
-        <v>898</v>
+        <v>894</v>
       </c>
       <c r="I8" s="42" t="s">
         <v>698</v>
@@ -4150,7 +4140,7 @@
         <v>358</v>
       </c>
       <c r="Q8" s="42" t="s">
-        <v>895</v>
+        <v>891</v>
       </c>
       <c r="R8" s="42"/>
       <c r="S8" s="42"/>
@@ -4171,7 +4161,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="D9" s="42" t="s">
         <v>12</v>
@@ -4184,7 +4174,7 @@
       </c>
       <c r="G9" s="42"/>
       <c r="H9" s="42" t="s">
-        <v>901</v>
+        <v>897</v>
       </c>
       <c r="I9" s="42" t="s">
         <v>701</v>
@@ -4201,7 +4191,7 @@
         <v>358</v>
       </c>
       <c r="Q9" s="42" t="s">
-        <v>895</v>
+        <v>891</v>
       </c>
       <c r="R9" s="42"/>
       <c r="S9" s="42"/>
@@ -4292,7 +4282,7 @@
       </c>
       <c r="G11" s="42"/>
       <c r="H11" s="42" t="s">
-        <v>908</v>
+        <v>904</v>
       </c>
       <c r="I11" s="42" t="s">
         <v>343</v>
@@ -4489,7 +4479,7 @@
         <v>0</v>
       </c>
       <c r="C15" s="45" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="D15" s="42" t="s">
         <v>43</v>
@@ -4502,7 +4492,7 @@
       </c>
       <c r="G15" s="42"/>
       <c r="H15" s="42" t="s">
-        <v>905</v>
+        <v>901</v>
       </c>
       <c r="I15" s="42" t="s">
         <v>723</v>
@@ -4553,7 +4543,7 @@
       </c>
       <c r="G16" s="42"/>
       <c r="H16" s="42" t="s">
-        <v>907</v>
+        <v>903</v>
       </c>
       <c r="I16" s="42" t="s">
         <v>726</v>
@@ -4600,7 +4590,7 @@
       </c>
       <c r="G17" s="42"/>
       <c r="H17" s="42" t="s">
-        <v>906</v>
+        <v>902</v>
       </c>
       <c r="I17" s="42"/>
       <c r="J17" s="42"/>
@@ -4643,7 +4633,7 @@
       </c>
       <c r="G18" s="42"/>
       <c r="H18" s="42" t="s">
-        <v>904</v>
+        <v>900</v>
       </c>
       <c r="I18" s="42" t="s">
         <v>20</v>
@@ -4690,7 +4680,7 @@
       </c>
       <c r="G19" s="42"/>
       <c r="H19" s="42" t="s">
-        <v>903</v>
+        <v>899</v>
       </c>
       <c r="I19" s="42"/>
       <c r="J19" s="42"/>
@@ -4753,7 +4743,7 @@
       </c>
       <c r="G20" s="42"/>
       <c r="H20" s="42" t="s">
-        <v>902</v>
+        <v>898</v>
       </c>
       <c r="I20" s="42"/>
       <c r="J20" s="42"/>
@@ -4797,7 +4787,7 @@
     </row>
     <row r="21" spans="1:27" ht="14.5" customHeight="1">
       <c r="P21" s="80" t="s">
-        <v>918</v>
+        <v>914</v>
       </c>
       <c r="Q21" s="80"/>
     </row>
@@ -4838,15 +4828,15 @@
   <dimension ref="A1:W22"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="49.0"/>
-    <col min="10" max="10" style="25" width="8.81640625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="11.453125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="12.6328125"/>
-    <col min="22" max="23" bestFit="true" customWidth="true" width="19.26953125"/>
+    <col min="1" max="1" width="49" customWidth="1"/>
+    <col min="10" max="10" width="8.81640625" style="25"/>
+    <col min="12" max="12" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="19.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -5854,16 +5844,16 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" customWidth="true" style="28" width="17.54296875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="29.7265625"/>
-    <col min="5" max="5" customWidth="true" width="13.81640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="14.36328125"/>
-    <col min="7" max="11" customWidth="true" style="28" width="14.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="30.36328125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="13.81640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="10.90625"/>
+    <col min="1" max="1" width="32.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" style="28" customWidth="1"/>
+    <col min="4" max="4" width="29.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.81640625" customWidth="1"/>
+    <col min="6" max="6" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="11" width="14.36328125" style="28" customWidth="1"/>
+    <col min="12" max="12" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -6023,17 +6013,17 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="28" width="21.81640625"/>
-    <col min="2" max="2" customWidth="true" style="28" width="16.54296875"/>
-    <col min="3" max="3" customWidth="true" style="28" width="19.90625"/>
-    <col min="4" max="4" customWidth="true" style="28" width="18.81640625"/>
-    <col min="5" max="6" customWidth="true" style="28" width="12.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="28" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="28" width="11.90625"/>
-    <col min="9" max="9" style="28" width="8.81640625"/>
-    <col min="10" max="10" customWidth="true" style="28" width="17.90625"/>
-    <col min="11" max="11" customWidth="true" style="28" width="14.1796875"/>
-    <col min="12" max="16384" style="28" width="8.81640625"/>
+    <col min="1" max="1" width="21.81640625" style="28" customWidth="1"/>
+    <col min="2" max="2" width="16.54296875" style="28" customWidth="1"/>
+    <col min="3" max="3" width="19.90625" style="28" customWidth="1"/>
+    <col min="4" max="4" width="18.81640625" style="28" customWidth="1"/>
+    <col min="5" max="6" width="12.90625" style="28" customWidth="1"/>
+    <col min="7" max="7" width="15" style="28" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="28" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.81640625" style="28"/>
+    <col min="10" max="10" width="17.90625" style="28" customWidth="1"/>
+    <col min="11" max="11" width="14.1796875" style="28" customWidth="1"/>
+    <col min="12" max="16384" width="8.81640625" style="28"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -6209,12 +6199,12 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="28" width="42.1796875"/>
-    <col min="2" max="2" customWidth="true" style="28" width="15.81640625"/>
-    <col min="3" max="3" customWidth="true" style="28" width="17.81640625"/>
-    <col min="4" max="4" customWidth="true" style="28" width="16.81640625"/>
-    <col min="5" max="5" customWidth="true" style="28" width="15.6328125"/>
-    <col min="6" max="16384" style="28" width="8.81640625"/>
+    <col min="1" max="1" width="42.1796875" style="28" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" style="28" customWidth="1"/>
+    <col min="3" max="3" width="17.81640625" style="28" customWidth="1"/>
+    <col min="4" max="4" width="16.81640625" style="28" customWidth="1"/>
+    <col min="5" max="5" width="15.6328125" style="28" customWidth="1"/>
+    <col min="6" max="16384" width="8.81640625" style="28"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -6333,28 +6323,28 @@
   <dimension ref="A1:AB6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="51.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="14.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="51.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -6777,12 +6767,12 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="76.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="16.6328125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="1" max="1" width="76.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -6907,17 +6897,17 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="28" width="68.08984375"/>
-    <col min="2" max="2" customWidth="true" style="28" width="12.54296875"/>
-    <col min="3" max="3" customWidth="true" style="28" width="12.36328125"/>
-    <col min="4" max="4" customWidth="true" style="28" width="9.6328125"/>
-    <col min="5" max="5" customWidth="true" style="28" width="17.26953125"/>
-    <col min="6" max="6" customWidth="true" style="28" width="12.54296875"/>
-    <col min="7" max="10" style="28" width="8.81640625"/>
-    <col min="11" max="11" customWidth="true" style="28" width="10.6328125"/>
-    <col min="12" max="12" customWidth="true" style="28" width="12.26953125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="28" width="15.36328125"/>
-    <col min="14" max="16384" style="28" width="8.81640625"/>
+    <col min="1" max="1" width="68.08984375" style="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" style="28" customWidth="1"/>
+    <col min="3" max="3" width="12.36328125" style="28" customWidth="1"/>
+    <col min="4" max="4" width="9.6328125" style="28" customWidth="1"/>
+    <col min="5" max="5" width="17.26953125" style="28" customWidth="1"/>
+    <col min="6" max="6" width="12.54296875" style="28" customWidth="1"/>
+    <col min="7" max="10" width="8.81640625" style="28"/>
+    <col min="11" max="11" width="10.6328125" style="28" customWidth="1"/>
+    <col min="12" max="12" width="12.26953125" style="28" customWidth="1"/>
+    <col min="13" max="13" width="15.36328125" style="28" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.81640625" style="28"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -7343,8 +7333,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.54296875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -7384,11 +7374,11 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -7438,8 +7428,8 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="61.7265625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="1" max="1" width="61.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="70" customFormat="1">
@@ -7835,31 +7825,31 @@
   <dimension ref="A1:AG14"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="49.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="4.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="9.7265625"/>
+    <col min="1" max="1" width="49.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -8085,7 +8075,7 @@
         <v>0</v>
       </c>
       <c r="K4" s="68" t="s">
-        <v>911</v>
+        <v>907</v>
       </c>
       <c r="L4" s="37" t="s">
         <v>12</v>
@@ -8103,7 +8093,7 @@
         <v>12</v>
       </c>
       <c r="Q4" s="37" t="s">
-        <v>910</v>
+        <v>906</v>
       </c>
       <c r="R4" s="37">
         <v>0</v>
@@ -8121,37 +8111,37 @@
         <v>0</v>
       </c>
       <c r="W4" s="68" t="s">
-        <v>913</v>
+        <v>909</v>
       </c>
       <c r="X4" s="37" t="s">
         <v>12</v>
       </c>
       <c r="Y4" s="37" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
       <c r="Z4" s="37">
         <v>0</v>
       </c>
       <c r="AA4" s="68" t="s">
-        <v>915</v>
+        <v>911</v>
       </c>
       <c r="AB4" s="37" t="s">
         <v>12</v>
       </c>
       <c r="AC4" s="37" t="s">
-        <v>914</v>
+        <v>910</v>
       </c>
       <c r="AD4" s="37">
         <v>0</v>
       </c>
       <c r="AE4" s="68" t="s">
-        <v>917</v>
+        <v>913</v>
       </c>
       <c r="AF4" s="37" t="s">
         <v>12</v>
       </c>
       <c r="AG4" s="37" t="s">
-        <v>916</v>
+        <v>912</v>
       </c>
     </row>
     <row r="5" spans="1:33">
@@ -8638,27 +8628,27 @@
   <dimension ref="A1:AH11"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="33.0"/>
-    <col min="2" max="2" customWidth="true" width="10.453125"/>
-    <col min="6" max="6" customWidth="true" width="10.90625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.36328125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.36328125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="19" max="19" customWidth="true" width="8.81640625"/>
-    <col min="20" max="20" customWidth="true" width="9.453125"/>
-    <col min="21" max="21" customWidth="true" width="11.08984375"/>
-    <col min="22" max="22" customWidth="true" width="9.36328125"/>
-    <col min="23" max="23" customWidth="true" width="9.453125"/>
-    <col min="24" max="24" customWidth="true" width="10.7265625"/>
-    <col min="25" max="25" customWidth="true" width="11.36328125"/>
-    <col min="26" max="26" customWidth="true" width="12.0"/>
-    <col min="27" max="27" customWidth="true" width="10.1796875"/>
-    <col min="30" max="30" customWidth="true" width="9.0"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="1" max="1" width="33" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" customWidth="1"/>
+    <col min="6" max="6" width="10.90625" customWidth="1"/>
+    <col min="12" max="12" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.81640625" customWidth="1"/>
+    <col min="20" max="20" width="9.453125" customWidth="1"/>
+    <col min="21" max="21" width="11.08984375" customWidth="1"/>
+    <col min="22" max="22" width="9.36328125" customWidth="1"/>
+    <col min="23" max="23" width="9.453125" customWidth="1"/>
+    <col min="24" max="24" width="10.7265625" customWidth="1"/>
+    <col min="25" max="25" width="11.36328125" customWidth="1"/>
+    <col min="26" max="26" width="12" customWidth="1"/>
+    <col min="27" max="27" width="10.1796875" customWidth="1"/>
+    <col min="30" max="30" width="9" customWidth="1"/>
+    <col min="34" max="34" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -9343,11 +9333,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="35.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.54296875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="1" max="1" width="35.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -9431,10 +9421,10 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -9528,9 +9518,9 @@
   <dimension ref="A1:AC4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="46.6328125"/>
-    <col min="5" max="5" customWidth="true" width="6.1796875"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="1" max="1" width="46.6328125" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" customWidth="1"/>
+    <col min="29" max="29" width="13.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -9828,14 +9818,14 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="63.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="10.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="19.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="15.54296875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="8" max="9" bestFit="true" customWidth="true" width="19.453125"/>
+    <col min="1" max="1" width="63.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="19.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -9970,24 +9960,24 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.81640625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="7.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="17" max="17" customWidth="true" width="17.6328125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.6328125" customWidth="1"/>
+    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -10300,27 +10290,27 @@
   <dimension ref="A1:U4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="44.08984375"/>
-    <col min="2" max="2" customWidth="true" width="13.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.1796875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="6" max="6" customWidth="true" width="11.6328125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.1796875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="8.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="14.08984375"/>
+    <col min="1" max="1" width="44.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.1796875" customWidth="1"/>
+    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6328125" customWidth="1"/>
+    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -10549,8 +10539,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -10598,8 +10588,8 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="18.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="11.453125"/>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -10667,21 +10657,21 @@
   <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="28" width="24.90625"/>
-    <col min="2" max="2" customWidth="true" style="28" width="14.0"/>
-    <col min="3" max="3" customWidth="true" style="28" width="11.81640625"/>
-    <col min="4" max="4" customWidth="true" style="28" width="9.54296875"/>
-    <col min="5" max="5" customWidth="true" style="28" width="10.36328125"/>
-    <col min="6" max="6" customWidth="true" style="28" width="9.36328125"/>
-    <col min="7" max="7" customWidth="true" style="28" width="9.7265625"/>
-    <col min="8" max="8" customWidth="true" style="28" width="10.453125"/>
-    <col min="9" max="9" customWidth="true" style="28" width="8.81640625"/>
-    <col min="10" max="10" customWidth="true" style="39" width="8.08984375"/>
-    <col min="11" max="11" customWidth="true" style="28" width="10.0"/>
-    <col min="12" max="12" customWidth="true" style="28" width="7.81640625"/>
-    <col min="13" max="13" customWidth="true" style="28" width="9.0"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="28" width="19.453125"/>
-    <col min="15" max="16384" style="28" width="8.81640625"/>
+    <col min="1" max="1" width="24.90625" style="28" customWidth="1"/>
+    <col min="2" max="2" width="14" style="28" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" style="28" customWidth="1"/>
+    <col min="4" max="4" width="9.54296875" style="28" customWidth="1"/>
+    <col min="5" max="5" width="10.36328125" style="28" customWidth="1"/>
+    <col min="6" max="6" width="9.36328125" style="28" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" style="28" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" style="28" customWidth="1"/>
+    <col min="9" max="9" width="8.81640625" style="28" customWidth="1"/>
+    <col min="10" max="10" width="8.08984375" style="39" customWidth="1"/>
+    <col min="11" max="11" width="10" style="28" customWidth="1"/>
+    <col min="12" max="12" width="7.81640625" style="28" customWidth="1"/>
+    <col min="13" max="13" width="9" style="28" customWidth="1"/>
+    <col min="14" max="14" width="19.453125" style="28" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.81640625" style="28"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -11451,15 +11441,15 @@
   <dimension ref="A1:P19"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="21.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="6.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -11535,10 +11525,10 @@
         <v>46</v>
       </c>
       <c r="H2" s="42" t="s">
-        <v>920</v>
+        <v>916</v>
       </c>
       <c r="I2" s="42" t="s">
-        <v>921</v>
+        <v>917</v>
       </c>
       <c r="J2" s="42"/>
       <c r="K2" s="42"/>
@@ -11571,7 +11561,7 @@
         <v>46</v>
       </c>
       <c r="H3" s="42" t="s">
-        <v>919</v>
+        <v>915</v>
       </c>
       <c r="I3" s="42" t="s">
         <v>370</v>
@@ -11743,14 +11733,14 @@
       </c>
       <c r="G9" s="42"/>
       <c r="H9" s="42" t="s">
-        <v>930</v>
+        <v>926</v>
       </c>
       <c r="I9" s="42" t="s">
-        <v>931</v>
+        <v>927</v>
       </c>
       <c r="J9" s="42"/>
       <c r="K9" s="42" t="s">
-        <v>928</v>
+        <v>924</v>
       </c>
       <c r="L9" s="42"/>
       <c r="M9" s="42"/>
@@ -11779,14 +11769,14 @@
       </c>
       <c r="G10" s="42"/>
       <c r="H10" s="42" t="s">
-        <v>932</v>
+        <v>928</v>
       </c>
       <c r="I10" s="42" t="s">
-        <v>933</v>
+        <v>929</v>
       </c>
       <c r="J10" s="42"/>
       <c r="K10" s="42" t="s">
-        <v>929</v>
+        <v>925</v>
       </c>
       <c r="L10" s="42"/>
       <c r="M10" s="42"/>
@@ -11815,10 +11805,10 @@
       </c>
       <c r="G11" s="42"/>
       <c r="H11" s="42" t="s">
-        <v>934</v>
+        <v>930</v>
       </c>
       <c r="I11" s="42" t="s">
-        <v>935</v>
+        <v>931</v>
       </c>
       <c r="J11" s="42"/>
       <c r="K11" s="45" t="s">
@@ -11851,10 +11841,10 @@
       </c>
       <c r="G12" s="42"/>
       <c r="H12" s="42" t="s">
-        <v>936</v>
+        <v>932</v>
       </c>
       <c r="I12" s="42" t="s">
-        <v>937</v>
+        <v>933</v>
       </c>
       <c r="J12" s="45" t="s">
         <v>871</v>
@@ -11897,10 +11887,10 @@
       </c>
       <c r="G13" s="42"/>
       <c r="H13" s="42" t="s">
-        <v>938</v>
+        <v>934</v>
       </c>
       <c r="I13" s="42" t="s">
-        <v>939</v>
+        <v>935</v>
       </c>
       <c r="J13" s="45" t="s">
         <v>873</v>
@@ -11933,10 +11923,10 @@
       </c>
       <c r="G14" s="42"/>
       <c r="H14" s="42" t="s">
-        <v>940</v>
+        <v>936</v>
       </c>
       <c r="I14" s="42" t="s">
-        <v>941</v>
+        <v>937</v>
       </c>
       <c r="J14" s="45" t="s">
         <v>875</v>
@@ -11979,10 +11969,10 @@
       </c>
       <c r="G15" s="42"/>
       <c r="H15" s="42" t="s">
-        <v>942</v>
+        <v>938</v>
       </c>
       <c r="I15" s="42" t="s">
-        <v>943</v>
+        <v>939</v>
       </c>
       <c r="J15" s="45" t="s">
         <v>877</v>
@@ -12015,16 +12005,16 @@
       </c>
       <c r="G16" s="42"/>
       <c r="H16" s="42" t="s">
-        <v>944</v>
+        <v>940</v>
       </c>
       <c r="I16" s="42" t="s">
-        <v>945</v>
+        <v>941</v>
       </c>
       <c r="J16" s="45" t="s">
         <v>844</v>
       </c>
       <c r="K16" s="42" t="s">
-        <v>928</v>
+        <v>924</v>
       </c>
       <c r="L16" s="42"/>
       <c r="M16" s="42"/>
@@ -12053,10 +12043,10 @@
       </c>
       <c r="G17" s="42"/>
       <c r="H17" s="42" t="s">
-        <v>946</v>
+        <v>942</v>
       </c>
       <c r="I17" s="42" t="s">
-        <v>947</v>
+        <v>943</v>
       </c>
       <c r="J17" s="45" t="s">
         <v>880</v>
@@ -12070,7 +12060,7 @@
     </row>
     <row r="18" spans="1:16">
       <c r="A18" s="79" t="s">
-        <v>922</v>
+        <v>918</v>
       </c>
       <c r="B18" s="42">
         <v>0</v>
@@ -12091,10 +12081,10 @@
         <v>46</v>
       </c>
       <c r="H18" s="42" t="s">
-        <v>923</v>
+        <v>919</v>
       </c>
       <c r="I18" s="42" t="s">
-        <v>924</v>
+        <v>920</v>
       </c>
       <c r="J18" s="42"/>
       <c r="K18" s="42"/>
@@ -12106,7 +12096,7 @@
     </row>
     <row r="19" spans="1:16">
       <c r="A19" s="79" t="s">
-        <v>925</v>
+        <v>921</v>
       </c>
       <c r="B19" s="42">
         <v>0</v>
@@ -12127,10 +12117,10 @@
         <v>46</v>
       </c>
       <c r="H19" s="42" t="s">
-        <v>926</v>
+        <v>922</v>
       </c>
       <c r="I19" s="42" t="s">
-        <v>927</v>
+        <v>923</v>
       </c>
       <c r="J19" s="42"/>
       <c r="K19" s="42"/>
@@ -12154,18 +12144,18 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="4" max="4" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" customWidth="true" width="15.08984375"/>
+    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" customWidth="1"/>
+    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -12357,30 +12347,30 @@
   <dimension ref="A1:W5"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="28" width="19.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="39" width="10.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="39" width="9.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="39" width="7.7265625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="39" width="10.90625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="39" width="9.453125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="39" width="7.7265625"/>
-    <col min="8" max="8" customWidth="true" style="28" width="13.0"/>
-    <col min="9" max="9" customWidth="true" style="28" width="16.54296875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="28" width="14.08984375"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="39" width="10.36328125"/>
-    <col min="12" max="12" customWidth="true" style="39" width="10.36328125"/>
-    <col min="13" max="13" style="28" width="8.81640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="28" width="12.54296875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="28" width="14.7265625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="28" width="13.26953125"/>
-    <col min="17" max="17" customWidth="true" style="39" width="11.54296875"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" style="39" width="8.7265625"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="28" width="9.90625"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="28" width="12.0"/>
-    <col min="21" max="21" style="28" width="8.81640625"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="28" width="10.6328125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="28" width="13.90625"/>
-    <col min="24" max="16384" style="28" width="8.81640625"/>
+    <col min="1" max="1" width="19.90625" style="28" customWidth="1"/>
+    <col min="2" max="2" width="10.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" style="28" customWidth="1"/>
+    <col min="9" max="9" width="16.54296875" style="28" customWidth="1"/>
+    <col min="10" max="10" width="14.08984375" style="28" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.36328125" style="39" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.36328125" style="39" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" style="28"/>
+    <col min="14" max="14" width="12.54296875" style="28" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.7265625" style="28" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.26953125" style="28" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" style="39" customWidth="1"/>
+    <col min="18" max="18" width="8.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.90625" style="28" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12" style="28" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.81640625" style="28"/>
+    <col min="22" max="22" width="10.6328125" style="28" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.90625" style="28" bestFit="1" customWidth="1"/>
+    <col min="24" max="16384" width="8.81640625" style="28"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -12620,7 +12610,7 @@
         <v>14</v>
       </c>
       <c r="M4" s="31" t="s">
-        <v>887</v>
+        <v>883</v>
       </c>
       <c r="N4" s="31"/>
       <c r="O4" s="31"/>
@@ -12629,15 +12619,15 @@
         <v>42</v>
       </c>
       <c r="R4" s="42" t="s">
-        <v>886</v>
+        <v>882</v>
       </c>
       <c r="S4" s="31"/>
       <c r="T4" s="31"/>
       <c r="U4" s="42" t="s">
-        <v>888</v>
+        <v>884</v>
       </c>
       <c r="V4" s="42" t="s">
-        <v>889</v>
+        <v>885</v>
       </c>
       <c r="W4" s="42" t="s">
         <v>370</v>
@@ -12650,7 +12640,7 @@
       <c r="C5" s="89"/>
       <c r="D5" s="89"/>
       <c r="E5" s="90" t="s">
-        <v>885</v>
+        <v>881</v>
       </c>
       <c r="F5" s="90"/>
       <c r="G5" s="90"/>
@@ -12672,19 +12662,19 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="19.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="1" max="1" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -12787,20 +12777,20 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="39" width="25.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="39" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="39" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="39" width="4.453125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="39" width="14.1796875"/>
-    <col min="14" max="16384" style="39" width="8.90625"/>
+    <col min="1" max="1" width="25.81640625" style="39" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="39" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" style="39" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.1796875" style="39" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.90625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -12926,21 +12916,21 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="39" width="20.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="39" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
-    <col min="6" max="7" customWidth="true" style="39" width="17.36328125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="39" width="15.0"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="39" width="4.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="39" width="14.1796875"/>
-    <col min="16" max="16384" style="39" width="8.90625"/>
+    <col min="1" max="1" width="20.1796875" style="39" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="39" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="17.36328125" style="39" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="39" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.1796875" style="39" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.90625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -13127,22 +13117,22 @@
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="39" width="28.36328125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="3" max="3" customWidth="true" style="39" width="10.36328125"/>
-    <col min="4" max="4" customWidth="true" style="39" width="11.1796875"/>
-    <col min="5" max="5" customWidth="true" style="39" width="12.81640625"/>
-    <col min="6" max="6" customWidth="true" style="39" width="12.453125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="39" width="11.08984375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="9" max="9" customWidth="true" style="39" width="9.08984375"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="11" max="11" customWidth="true" style="39" width="11.54296875"/>
-    <col min="12" max="12" customWidth="true" style="39" width="10.81640625"/>
-    <col min="13" max="13" customWidth="true" style="39" width="12.1796875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="39" width="11.90625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="39" width="14.1796875"/>
-    <col min="16" max="16384" style="39" width="8.90625"/>
+    <col min="1" max="1" width="28.36328125" style="39" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.36328125" style="39" customWidth="1"/>
+    <col min="4" max="4" width="11.1796875" style="39" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" style="39" customWidth="1"/>
+    <col min="6" max="6" width="12.453125" style="39" customWidth="1"/>
+    <col min="7" max="7" width="11.08984375" style="39" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" style="39" customWidth="1"/>
+    <col min="10" max="10" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.54296875" style="39" customWidth="1"/>
+    <col min="12" max="12" width="10.81640625" style="39" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" style="39" customWidth="1"/>
+    <col min="14" max="14" width="11.90625" style="39" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.1796875" style="39" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.90625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -13439,14 +13429,14 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="39" width="24.0"/>
-    <col min="2" max="2" customWidth="true" style="39" width="11.453125"/>
-    <col min="3" max="3" style="39" width="8.90625"/>
-    <col min="4" max="4" customWidth="true" style="39" width="19.6328125"/>
-    <col min="5" max="16384" style="39" width="8.90625"/>
+    <col min="1" max="1" width="24" style="39" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" style="39" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" style="39"/>
+    <col min="4" max="4" width="19.6328125" style="39" customWidth="1"/>
+    <col min="5" max="16384" width="8.90625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -13474,6 +13464,20 @@
         <v>12</v>
       </c>
       <c r="D2" s="42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="42" t="s">
+        <v>944</v>
+      </c>
+      <c r="B3" s="45" t="s">
+        <v>339</v>
+      </c>
+      <c r="C3" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="42">
         <v>1</v>
       </c>
     </row>
@@ -13490,12 +13494,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="39" width="32.1796875"/>
-    <col min="2" max="2" customWidth="true" style="39" width="14.0"/>
-    <col min="3" max="3" customWidth="true" style="39" width="16.6328125"/>
-    <col min="4" max="4" customWidth="true" style="39" width="17.6328125"/>
-    <col min="5" max="5" customWidth="true" style="39" width="11.81640625"/>
-    <col min="6" max="16384" style="39" width="8.90625"/>
+    <col min="1" max="1" width="32.1796875" style="39" customWidth="1"/>
+    <col min="2" max="2" width="14" style="39" customWidth="1"/>
+    <col min="3" max="3" width="16.6328125" style="39" customWidth="1"/>
+    <col min="4" max="4" width="17.6328125" style="39" customWidth="1"/>
+    <col min="5" max="5" width="11.81640625" style="39" customWidth="1"/>
+    <col min="6" max="16384" width="8.90625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -13579,11 +13583,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="39" width="38.1796875"/>
-    <col min="2" max="2" customWidth="true" style="39" width="13.54296875"/>
-    <col min="3" max="3" customWidth="true" style="39" width="15.54296875"/>
-    <col min="4" max="4" customWidth="true" style="39" width="19.0"/>
-    <col min="5" max="16384" style="39" width="8.90625"/>
+    <col min="1" max="1" width="38.1796875" style="39" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" style="39" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" style="39" customWidth="1"/>
+    <col min="4" max="4" width="19" style="39" customWidth="1"/>
+    <col min="5" max="16384" width="8.90625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -13706,21 +13710,21 @@
   <dimension ref="A1:N5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="39" width="30.90625"/>
-    <col min="2" max="2" customWidth="true" style="39" width="17.81640625"/>
-    <col min="3" max="3" customWidth="true" style="39" width="16.453125"/>
-    <col min="4" max="4" customWidth="true" style="39" width="16.08984375"/>
-    <col min="5" max="5" customWidth="true" style="39" width="12.0"/>
-    <col min="6" max="6" customWidth="true" style="39" width="18.08984375"/>
-    <col min="7" max="7" customWidth="true" style="39" width="15.08984375"/>
-    <col min="8" max="8" customWidth="true" style="39" width="10.453125"/>
-    <col min="9" max="9" customWidth="true" style="39" width="10.81640625"/>
-    <col min="10" max="10" style="39" width="8.90625"/>
-    <col min="11" max="11" customWidth="true" style="39" width="13.1796875"/>
-    <col min="12" max="12" customWidth="true" style="39" width="12.6328125"/>
-    <col min="13" max="13" customWidth="true" style="39" width="14.08984375"/>
-    <col min="14" max="14" customWidth="true" style="39" width="14.36328125"/>
-    <col min="15" max="16384" style="39" width="8.90625"/>
+    <col min="1" max="1" width="30.90625" style="39" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" style="39" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" style="39" customWidth="1"/>
+    <col min="4" max="4" width="16.08984375" style="39" customWidth="1"/>
+    <col min="5" max="5" width="12" style="39" customWidth="1"/>
+    <col min="6" max="6" width="18.08984375" style="39" customWidth="1"/>
+    <col min="7" max="7" width="15.08984375" style="39" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" style="39" customWidth="1"/>
+    <col min="9" max="9" width="10.81640625" style="39" customWidth="1"/>
+    <col min="10" max="10" width="8.90625" style="39"/>
+    <col min="11" max="11" width="13.1796875" style="39" customWidth="1"/>
+    <col min="12" max="12" width="12.6328125" style="39" customWidth="1"/>
+    <col min="13" max="13" width="14.08984375" style="39" customWidth="1"/>
+    <col min="14" max="14" width="14.36328125" style="39" customWidth="1"/>
+    <col min="15" max="16384" width="8.90625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -13922,12 +13926,12 @@
   <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="16.08984375"/>
+    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -14610,11 +14614,11 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="57.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="15.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="4" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="20.08984375"/>
+    <col min="1" max="1" width="57.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -14791,28 +14795,28 @@
   <dimension ref="A1:V15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="50.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="25" width="18.36328125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="25" width="12.08984375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="25" width="15.36328125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="25" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="25" width="9.453125"/>
-    <col min="7" max="8" style="25" width="8.81640625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="8.1796875"/>
-    <col min="15" max="15" customWidth="true" style="25" width="13.0"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="10.1796875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" style="25" width="9.1796875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="25" width="11.6328125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="23" max="16384" style="25" width="8.81640625"/>
+    <col min="1" max="1" width="50" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.36328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.08984375" style="25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.36328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="8.81640625" style="25"/>
+    <col min="9" max="9" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13" style="25" customWidth="1"/>
+    <col min="16" max="16" width="10.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="8.81640625" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -15507,29 +15511,29 @@
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="44.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="8.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="13.54296875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.81640625"/>
-    <col min="11" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.1796875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="8.1796875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="14.1796875"/>
-    <col min="27" max="28" bestFit="true" customWidth="true" width="12.81640625"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="14.1796875"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="12.81640625"/>
+    <col min="1" max="1" width="44.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -15961,10 +15965,10 @@
   <dimension ref="A1:AJ39"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="54.36328125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="13.81640625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="1" max="1" width="54.36328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36">
@@ -18250,16 +18254,16 @@
   <dimension ref="A1:S20"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="53.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="5" max="7" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="53.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="12.1796875" customWidth="1"/>
+    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">

</xml_diff>

<commit_message>
DisplayBookingService taken from Harshitha
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8226D3C0-7880-4B38-B281-00377BA3475F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BE403E-4F9C-40B6-8A4D-497F364F6CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="32" activeTab="35" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="7" activeTab="9" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2853" uniqueCount="945">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2934" uniqueCount="987">
   <si>
     <t>Scenario</t>
   </si>
@@ -2386,12 +2386,6 @@
     <t>2302182828215</t>
   </si>
   <si>
-    <t>BBO43F</t>
-  </si>
-  <si>
-    <t>BBO5D5</t>
-  </si>
-  <si>
     <t>BBO5YO</t>
   </si>
   <si>
@@ -2909,13 +2903,146 @@
   </si>
   <si>
     <t>Crew_Report_Services_PR</t>
+  </si>
+  <si>
+    <t>BDRLQX</t>
+  </si>
+  <si>
+    <t>FEMALE</t>
+  </si>
+  <si>
+    <t>THOMPSON</t>
+  </si>
+  <si>
+    <t>BDRLWJ</t>
+  </si>
+  <si>
+    <t>HUSBAND</t>
+  </si>
+  <si>
+    <t>Error display booking</t>
+  </si>
+  <si>
+    <t>ABC123</t>
+  </si>
+  <si>
+    <t>DM1Z3Y</t>
+  </si>
+  <si>
+    <t>Display booking by e-ticket number</t>
+  </si>
+  <si>
+    <t>BBMW5F</t>
+  </si>
+  <si>
+    <t>2302182828135</t>
+  </si>
+  <si>
+    <t>2312182793885</t>
+  </si>
+  <si>
+    <t>Display_confirmed_booking</t>
+  </si>
+  <si>
+    <t>BBM0K0</t>
+  </si>
+  <si>
+    <t>Display_waitlist_booking</t>
+  </si>
+  <si>
+    <t>BB4TGN</t>
+  </si>
+  <si>
+    <t>EMILY</t>
+  </si>
+  <si>
+    <t>WATSON</t>
+  </si>
+  <si>
+    <t>Display waitlist booking list (including multiple name entries in list on same booking)</t>
+  </si>
+  <si>
+    <t>BCAY5D</t>
+  </si>
+  <si>
+    <t>195</t>
+  </si>
+  <si>
+    <t>Display confirmed and waitlist booking (same passenger name in both lists)</t>
+  </si>
+  <si>
+    <t>Missing required data (flight number, flight date or passenger surname)</t>
+  </si>
+  <si>
+    <t>BCETSF</t>
+  </si>
+  <si>
+    <t>Display_booking_No_bookings_found</t>
+  </si>
+  <si>
+    <t>395</t>
+  </si>
+  <si>
+    <t>Display an Other Airline booking</t>
+  </si>
+  <si>
+    <t>BCEGNP</t>
+  </si>
+  <si>
+    <t>FERRELL</t>
+  </si>
+  <si>
+    <t>Error display booking for no Eticket Number and no Record locator</t>
+  </si>
+  <si>
+    <t>Error displaying a booking from a specific address LNIATA</t>
+  </si>
+  <si>
+    <t>Error display booking for Incorrect Eticket Number</t>
+  </si>
+  <si>
+    <t>Display confirmed booking list 1st flt in one booking and 2nd flt in another booking</t>
+  </si>
+  <si>
+    <t>Display confirmed and waitlist booking list Multiple name entries in list on same booking</t>
+  </si>
+  <si>
+    <t>BDRUEN</t>
+  </si>
+  <si>
+    <t>BDRXJR</t>
+  </si>
+  <si>
+    <t>2302182834559</t>
+  </si>
+  <si>
+    <t>BDRZ55</t>
+  </si>
+  <si>
+    <t>BDR0CT</t>
+  </si>
+  <si>
+    <t>BDR0V5</t>
+  </si>
+  <si>
+    <t>BDR0WB</t>
+  </si>
+  <si>
+    <t>BDR03Q</t>
+  </si>
+  <si>
+    <t>BDR033</t>
+  </si>
+  <si>
+    <t>BDR1AJ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <numFmts count="0"/>
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3012,6 +3139,15 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="17">
@@ -3112,7 +3248,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -3196,11 +3332,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -3325,6 +3474,25 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3680,23 +3848,23 @@
   <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="52.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="52.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.1796875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="11.6328125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="12.6328125"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="9.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27">
@@ -3805,7 +3973,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="42" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="I2" s="42" t="s">
         <v>206</v>
@@ -3822,7 +3990,7 @@
       <c r="M2" s="42"/>
       <c r="N2" s="42"/>
       <c r="O2" s="42" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="P2" s="42"/>
       <c r="Q2" s="42"/>
@@ -3860,7 +4028,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="42" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="I3" s="42" t="s">
         <v>207</v>
@@ -3869,13 +4037,13 @@
         <v>206</v>
       </c>
       <c r="K3" s="42" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="L3" s="42" t="s">
         <v>206</v>
       </c>
       <c r="M3" s="42" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="N3" s="42" t="s">
         <v>206</v>
@@ -3902,7 +4070,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="D4" s="42" t="s">
         <v>12</v>
@@ -3917,7 +4085,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="36" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
       <c r="I4" s="36" t="s">
         <v>337</v>
@@ -3934,7 +4102,7 @@
         <v>358</v>
       </c>
       <c r="Q4" s="42" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="R4" s="42"/>
       <c r="S4" s="42"/>
@@ -3955,7 +4123,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="45" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="D5" s="42" t="s">
         <v>12</v>
@@ -3970,7 +4138,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="36" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="I5" s="42" t="s">
         <v>207</v>
@@ -3979,7 +4147,7 @@
         <v>741</v>
       </c>
       <c r="K5" s="42" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="L5" s="42" t="s">
         <v>741</v>
@@ -3991,7 +4159,7 @@
         <v>358</v>
       </c>
       <c r="Q5" s="42" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="R5" s="42"/>
       <c r="S5" s="42"/>
@@ -4012,7 +4180,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="D6" s="42" t="s">
         <v>12</v>
@@ -4025,7 +4193,7 @@
       </c>
       <c r="G6" s="42"/>
       <c r="H6" s="42" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="I6" s="42" t="s">
         <v>692</v>
@@ -4042,7 +4210,7 @@
         <v>358</v>
       </c>
       <c r="Q6" s="42" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="R6" s="42"/>
       <c r="S6" s="42"/>
@@ -4063,7 +4231,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="D7" s="42" t="s">
         <v>12</v>
@@ -4076,7 +4244,7 @@
       </c>
       <c r="G7" s="42"/>
       <c r="H7" s="42" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="I7" s="42" t="s">
         <v>695</v>
@@ -4110,7 +4278,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="45" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="D8" s="42" t="s">
         <v>12</v>
@@ -4123,7 +4291,7 @@
       </c>
       <c r="G8" s="42"/>
       <c r="H8" s="42" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="I8" s="42" t="s">
         <v>698</v>
@@ -4140,7 +4308,7 @@
         <v>358</v>
       </c>
       <c r="Q8" s="42" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="R8" s="42"/>
       <c r="S8" s="42"/>
@@ -4161,7 +4329,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="D9" s="42" t="s">
         <v>12</v>
@@ -4174,7 +4342,7 @@
       </c>
       <c r="G9" s="42"/>
       <c r="H9" s="42" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="I9" s="42" t="s">
         <v>701</v>
@@ -4191,7 +4359,7 @@
         <v>358</v>
       </c>
       <c r="Q9" s="42" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="R9" s="42"/>
       <c r="S9" s="42"/>
@@ -4282,7 +4450,7 @@
       </c>
       <c r="G11" s="42"/>
       <c r="H11" s="42" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
       <c r="I11" s="42" t="s">
         <v>343</v>
@@ -4479,7 +4647,7 @@
         <v>0</v>
       </c>
       <c r="C15" s="45" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="D15" s="42" t="s">
         <v>43</v>
@@ -4492,7 +4660,7 @@
       </c>
       <c r="G15" s="42"/>
       <c r="H15" s="42" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="I15" s="42" t="s">
         <v>723</v>
@@ -4543,7 +4711,7 @@
       </c>
       <c r="G16" s="42"/>
       <c r="H16" s="42" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="I16" s="42" t="s">
         <v>726</v>
@@ -4590,7 +4758,7 @@
       </c>
       <c r="G17" s="42"/>
       <c r="H17" s="42" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="I17" s="42"/>
       <c r="J17" s="42"/>
@@ -4633,7 +4801,7 @@
       </c>
       <c r="G18" s="42"/>
       <c r="H18" s="42" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="I18" s="42" t="s">
         <v>20</v>
@@ -4680,7 +4848,7 @@
       </c>
       <c r="G19" s="42"/>
       <c r="H19" s="42" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="I19" s="42"/>
       <c r="J19" s="42"/>
@@ -4743,7 +4911,7 @@
       </c>
       <c r="G20" s="42"/>
       <c r="H20" s="42" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="I20" s="42"/>
       <c r="J20" s="42"/>
@@ -4786,18 +4954,18 @@
       </c>
     </row>
     <row r="21" spans="1:27" ht="14.5" customHeight="1">
-      <c r="P21" s="80" t="s">
-        <v>914</v>
-      </c>
-      <c r="Q21" s="80"/>
+      <c r="P21" s="87" t="s">
+        <v>912</v>
+      </c>
+      <c r="Q21" s="87"/>
     </row>
     <row r="22" spans="1:27">
-      <c r="P22" s="80"/>
-      <c r="Q22" s="80"/>
+      <c r="P22" s="87"/>
+      <c r="Q22" s="87"/>
     </row>
     <row r="23" spans="1:27">
-      <c r="P23" s="80"/>
-      <c r="Q23" s="80"/>
+      <c r="P23" s="87"/>
+      <c r="Q23" s="87"/>
     </row>
     <row r="24" spans="1:27">
       <c r="H24" s="1"/>
@@ -4825,18 +4993,18 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:W22"/>
+  <dimension ref="A1:W36"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="49" customWidth="1"/>
-    <col min="10" max="10" width="8.81640625" style="25"/>
-    <col min="12" max="12" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="19.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="54.7265625"/>
+    <col min="10" max="10" style="25" width="8.81640625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="11.453125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="12.6328125"/>
+    <col min="22" max="23" bestFit="true" customWidth="true" width="19.26953125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -5104,27 +5272,27 @@
       <c r="I6" s="42"/>
       <c r="J6" s="42"/>
       <c r="K6" s="42" t="s">
-        <v>770</v>
+        <v>943</v>
       </c>
       <c r="L6" s="42"/>
       <c r="M6" s="42"/>
       <c r="N6" s="42" t="s">
-        <v>20</v>
+        <v>944</v>
       </c>
       <c r="O6" s="42" t="s">
-        <v>237</v>
+        <v>945</v>
       </c>
       <c r="P6" s="42" t="s">
-        <v>771</v>
+        <v>946</v>
       </c>
       <c r="Q6" s="42"/>
       <c r="R6" s="42"/>
       <c r="S6" s="42"/>
       <c r="T6" s="42" t="s">
-        <v>253</v>
+        <v>947</v>
       </c>
       <c r="U6" s="42" t="s">
-        <v>237</v>
+        <v>945</v>
       </c>
       <c r="V6" s="42"/>
       <c r="W6" s="42"/>
@@ -5208,10 +5376,10 @@
       </c>
       <c r="J8" s="42"/>
       <c r="K8" s="42" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="L8" s="42" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="M8" s="42"/>
       <c r="N8" s="42" t="s">
@@ -5294,10 +5462,10 @@
       <c r="I10" s="42"/>
       <c r="J10" s="42"/>
       <c r="K10" s="42" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="L10" s="42" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="M10" s="42"/>
       <c r="N10" s="42"/>
@@ -5831,6 +5999,510 @@
       <c r="V22" s="42"/>
       <c r="W22" s="42"/>
     </row>
+    <row r="23" spans="1:23">
+      <c r="A23" s="27" t="s">
+        <v>948</v>
+      </c>
+      <c r="B23" s="42"/>
+      <c r="C23" s="42"/>
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="42"/>
+      <c r="I23" s="42"/>
+      <c r="J23" s="42"/>
+      <c r="K23" s="42" t="s">
+        <v>949</v>
+      </c>
+      <c r="L23" s="42"/>
+      <c r="M23" s="42"/>
+      <c r="N23" s="42"/>
+      <c r="O23" s="42"/>
+      <c r="P23" s="42"/>
+      <c r="Q23" s="42"/>
+      <c r="R23" s="42"/>
+      <c r="S23" s="42"/>
+      <c r="T23" s="42"/>
+      <c r="U23" s="42"/>
+      <c r="V23" s="42"/>
+      <c r="W23" s="42"/>
+    </row>
+    <row r="24" spans="1:23">
+      <c r="A24" s="80" t="s">
+        <v>973</v>
+      </c>
+      <c r="B24" s="42"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="42"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="42"/>
+      <c r="H24" s="42"/>
+      <c r="I24" s="42"/>
+      <c r="J24" s="42"/>
+      <c r="K24" s="81" t="s">
+        <v>950</v>
+      </c>
+      <c r="L24" s="42"/>
+      <c r="M24" s="42"/>
+      <c r="N24" s="42"/>
+      <c r="O24" s="42"/>
+      <c r="P24" s="42"/>
+      <c r="Q24" s="42"/>
+      <c r="R24" s="42"/>
+      <c r="S24" s="42"/>
+      <c r="T24" s="42"/>
+      <c r="U24" s="42"/>
+      <c r="V24" s="42"/>
+      <c r="W24" s="42"/>
+    </row>
+    <row r="25" spans="1:23">
+      <c r="A25" s="42" t="s">
+        <v>951</v>
+      </c>
+      <c r="B25" s="42">
+        <v>0</v>
+      </c>
+      <c r="C25" s="45" t="s">
+        <v>438</v>
+      </c>
+      <c r="D25" s="42" t="s">
+        <v>30</v>
+      </c>
+      <c r="E25" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" s="42"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="42"/>
+      <c r="I25" s="42"/>
+      <c r="J25" s="42"/>
+      <c r="K25" s="42" t="s">
+        <v>978</v>
+      </c>
+      <c r="L25" s="42" t="s">
+        <v>979</v>
+      </c>
+      <c r="M25" s="42"/>
+      <c r="N25" s="42" t="s">
+        <v>692</v>
+      </c>
+      <c r="O25" s="42" t="s">
+        <v>237</v>
+      </c>
+      <c r="P25" s="42"/>
+      <c r="Q25" s="42"/>
+      <c r="R25" s="42"/>
+      <c r="S25" s="42"/>
+      <c r="T25" s="42"/>
+      <c r="U25" s="42"/>
+      <c r="V25" s="42"/>
+      <c r="W25" s="42"/>
+    </row>
+    <row r="26" spans="1:23">
+      <c r="A26" s="82" t="s">
+        <v>974</v>
+      </c>
+      <c r="B26" s="54"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="42"/>
+      <c r="F26" s="42"/>
+      <c r="G26" s="42"/>
+      <c r="H26" s="42"/>
+      <c r="I26" s="42"/>
+      <c r="J26" s="42"/>
+      <c r="K26" s="42"/>
+      <c r="L26" s="83" t="s">
+        <v>954</v>
+      </c>
+      <c r="M26" s="42"/>
+      <c r="N26" s="42"/>
+      <c r="O26" s="42"/>
+      <c r="P26" s="42"/>
+      <c r="Q26" s="42"/>
+      <c r="R26" s="42"/>
+      <c r="S26" s="42"/>
+      <c r="T26" s="42"/>
+      <c r="U26" s="42"/>
+      <c r="V26" s="42"/>
+      <c r="W26" s="42"/>
+    </row>
+    <row r="27" spans="1:23">
+      <c r="A27" s="82" t="s">
+        <v>972</v>
+      </c>
+      <c r="B27" s="54"/>
+      <c r="C27" s="42"/>
+      <c r="D27" s="42"/>
+      <c r="E27" s="42"/>
+      <c r="F27" s="42"/>
+      <c r="G27" s="42"/>
+      <c r="H27" s="42"/>
+      <c r="I27" s="42"/>
+      <c r="J27" s="42"/>
+      <c r="K27" s="42"/>
+      <c r="L27" s="42"/>
+      <c r="M27" s="42"/>
+      <c r="N27" s="42"/>
+      <c r="O27" s="42"/>
+      <c r="P27" s="42"/>
+      <c r="Q27" s="42"/>
+      <c r="R27" s="42"/>
+      <c r="S27" s="42"/>
+      <c r="T27" s="42"/>
+      <c r="U27" s="42"/>
+      <c r="V27" s="42"/>
+      <c r="W27" s="42"/>
+    </row>
+    <row r="28" spans="1:23">
+      <c r="A28" s="52" t="s">
+        <v>955</v>
+      </c>
+      <c r="B28" s="54">
+        <v>0</v>
+      </c>
+      <c r="C28" s="45" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="F28" s="42"/>
+      <c r="G28" s="42"/>
+      <c r="H28" s="42"/>
+      <c r="I28" s="42"/>
+      <c r="J28" s="42"/>
+      <c r="K28" s="42" t="s">
+        <v>980</v>
+      </c>
+      <c r="L28" s="42"/>
+      <c r="M28" s="42"/>
+      <c r="N28" s="42"/>
+      <c r="O28" s="42"/>
+      <c r="P28" s="42"/>
+      <c r="Q28" s="42"/>
+      <c r="R28" s="42"/>
+      <c r="S28" s="42"/>
+      <c r="T28" s="42"/>
+      <c r="U28" s="42"/>
+      <c r="V28" s="42"/>
+      <c r="W28" s="42"/>
+    </row>
+    <row r="29" spans="1:23">
+      <c r="A29" s="52" t="s">
+        <v>957</v>
+      </c>
+      <c r="B29" s="54">
+        <v>0</v>
+      </c>
+      <c r="C29" s="45" t="s">
+        <v>62</v>
+      </c>
+      <c r="D29" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="E29" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" s="42"/>
+      <c r="G29" s="42"/>
+      <c r="H29" s="42"/>
+      <c r="I29" s="42"/>
+      <c r="J29" s="42"/>
+      <c r="K29" s="42" t="s">
+        <v>981</v>
+      </c>
+      <c r="L29" s="42"/>
+      <c r="M29" s="42"/>
+      <c r="N29" s="42" t="s">
+        <v>959</v>
+      </c>
+      <c r="O29" s="42" t="s">
+        <v>960</v>
+      </c>
+      <c r="P29" s="42"/>
+      <c r="Q29" s="42"/>
+      <c r="R29" s="42"/>
+      <c r="S29" s="42"/>
+      <c r="T29" s="42"/>
+      <c r="U29" s="42"/>
+      <c r="V29" s="42"/>
+      <c r="W29" s="42"/>
+    </row>
+    <row r="30" spans="1:23">
+      <c r="A30" s="20" t="s">
+        <v>961</v>
+      </c>
+      <c r="B30" s="42">
+        <v>0</v>
+      </c>
+      <c r="C30" s="45" t="s">
+        <v>62</v>
+      </c>
+      <c r="D30" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="E30" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" s="42"/>
+      <c r="G30" s="42"/>
+      <c r="H30" s="42"/>
+      <c r="I30" s="42"/>
+      <c r="J30" s="42"/>
+      <c r="K30" s="42" t="s">
+        <v>962</v>
+      </c>
+      <c r="L30" s="42"/>
+      <c r="M30" s="42"/>
+      <c r="N30" s="42"/>
+      <c r="O30" s="42"/>
+      <c r="P30" s="42"/>
+      <c r="Q30" s="42"/>
+      <c r="R30" s="42"/>
+      <c r="S30" s="42"/>
+      <c r="T30" s="42"/>
+      <c r="U30" s="42"/>
+      <c r="V30" s="42"/>
+      <c r="W30" s="42"/>
+    </row>
+    <row r="31" spans="1:23">
+      <c r="A31" s="52" t="s">
+        <v>976</v>
+      </c>
+      <c r="B31" s="54">
+        <v>1</v>
+      </c>
+      <c r="C31" s="45" t="s">
+        <v>963</v>
+      </c>
+      <c r="D31" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="E31" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" s="42"/>
+      <c r="G31" s="42"/>
+      <c r="H31" s="42"/>
+      <c r="I31" s="42"/>
+      <c r="J31" s="42"/>
+      <c r="K31" s="42"/>
+      <c r="L31" s="42"/>
+      <c r="M31" s="42"/>
+      <c r="N31" s="42"/>
+      <c r="O31" s="42"/>
+      <c r="P31" s="42"/>
+      <c r="Q31" s="42"/>
+      <c r="R31" s="42"/>
+      <c r="S31" s="42"/>
+      <c r="T31" s="42"/>
+      <c r="U31" s="42"/>
+      <c r="V31" s="42"/>
+      <c r="W31" s="42"/>
+    </row>
+    <row r="32" spans="1:23">
+      <c r="A32" s="52" t="s">
+        <v>964</v>
+      </c>
+      <c r="B32" s="54">
+        <v>0</v>
+      </c>
+      <c r="C32" s="45" t="s">
+        <v>891</v>
+      </c>
+      <c r="D32" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E32" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="F32" s="42"/>
+      <c r="G32" s="42"/>
+      <c r="H32" s="42"/>
+      <c r="I32" s="42"/>
+      <c r="J32" s="42"/>
+      <c r="K32" s="42" t="s">
+        <v>984</v>
+      </c>
+      <c r="L32" s="42"/>
+      <c r="M32" s="42"/>
+      <c r="N32" s="42"/>
+      <c r="O32" s="42"/>
+      <c r="P32" s="42" t="s">
+        <v>985</v>
+      </c>
+      <c r="Q32" s="42"/>
+      <c r="R32" s="42"/>
+      <c r="S32" s="42"/>
+      <c r="T32" s="42"/>
+      <c r="U32" s="42"/>
+      <c r="V32" s="42"/>
+      <c r="W32" s="42"/>
+    </row>
+    <row r="33" spans="1:23">
+      <c r="A33" s="84" t="s">
+        <v>965</v>
+      </c>
+      <c r="B33" s="54">
+        <v>0</v>
+      </c>
+      <c r="C33" s="45" t="s">
+        <v>891</v>
+      </c>
+      <c r="D33" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="F33" s="42"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="42" t="s">
+        <v>986</v>
+      </c>
+      <c r="L33" s="42"/>
+      <c r="M33" s="42"/>
+      <c r="N33" s="42" t="s">
+        <v>239</v>
+      </c>
+      <c r="O33" s="42" t="s">
+        <v>244</v>
+      </c>
+      <c r="P33" s="42"/>
+      <c r="Q33" s="83" t="s">
+        <v>83</v>
+      </c>
+      <c r="R33" s="42"/>
+      <c r="S33" s="42"/>
+      <c r="T33" s="42"/>
+      <c r="U33" s="42"/>
+      <c r="V33" s="42"/>
+      <c r="W33" s="42"/>
+    </row>
+    <row r="34" spans="1:23">
+      <c r="A34" s="85" t="s">
+        <v>967</v>
+      </c>
+      <c r="B34" s="54">
+        <v>0</v>
+      </c>
+      <c r="C34" s="45" t="s">
+        <v>968</v>
+      </c>
+      <c r="D34" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" s="42"/>
+      <c r="F34" s="42"/>
+      <c r="G34" s="42"/>
+      <c r="H34" s="42"/>
+      <c r="I34" s="42"/>
+      <c r="J34" s="42"/>
+      <c r="K34" s="42"/>
+      <c r="L34" s="42"/>
+      <c r="M34" s="42"/>
+      <c r="N34" s="42"/>
+      <c r="O34" s="42"/>
+      <c r="P34" s="42"/>
+      <c r="Q34" s="42"/>
+      <c r="R34" s="42"/>
+      <c r="S34" s="42"/>
+      <c r="T34" s="42"/>
+      <c r="U34" s="42"/>
+      <c r="V34" s="42"/>
+      <c r="W34" s="42"/>
+    </row>
+    <row r="35" spans="1:23">
+      <c r="A35" s="86" t="s">
+        <v>969</v>
+      </c>
+      <c r="B35" s="54">
+        <v>0</v>
+      </c>
+      <c r="C35" s="45" t="s">
+        <v>532</v>
+      </c>
+      <c r="D35" s="42" t="s">
+        <v>159</v>
+      </c>
+      <c r="E35" s="42" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35" s="42"/>
+      <c r="G35" s="42"/>
+      <c r="H35" s="42"/>
+      <c r="I35" s="42"/>
+      <c r="J35" s="42"/>
+      <c r="K35" s="42" t="s">
+        <v>977</v>
+      </c>
+      <c r="L35" s="42"/>
+      <c r="M35" s="42"/>
+      <c r="N35" s="42"/>
+      <c r="O35" s="42"/>
+      <c r="P35" s="42"/>
+      <c r="Q35" s="42"/>
+      <c r="R35" s="42"/>
+      <c r="S35" s="42"/>
+      <c r="T35" s="42"/>
+      <c r="U35" s="42"/>
+      <c r="V35" s="42"/>
+      <c r="W35" s="42"/>
+    </row>
+    <row r="36" spans="1:23">
+      <c r="A36" s="52" t="s">
+        <v>975</v>
+      </c>
+      <c r="B36" s="42">
+        <v>1</v>
+      </c>
+      <c r="C36" s="45" t="s">
+        <v>533</v>
+      </c>
+      <c r="D36" s="42" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="F36" s="42">
+        <v>1</v>
+      </c>
+      <c r="G36" s="45" t="s">
+        <v>968</v>
+      </c>
+      <c r="H36" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="I36" s="42" t="s">
+        <v>733</v>
+      </c>
+      <c r="J36" s="42"/>
+      <c r="K36" s="42"/>
+      <c r="L36" s="42"/>
+      <c r="M36" s="42"/>
+      <c r="N36" s="42"/>
+      <c r="O36" s="42" t="s">
+        <v>971</v>
+      </c>
+      <c r="P36" s="42"/>
+      <c r="Q36" s="42"/>
+      <c r="R36" s="42"/>
+      <c r="S36" s="42"/>
+      <c r="T36" s="42"/>
+      <c r="U36" s="42"/>
+      <c r="V36" s="42"/>
+      <c r="W36" s="42"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5844,16 +6516,16 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" style="28" customWidth="1"/>
-    <col min="4" max="4" width="29.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.81640625" customWidth="1"/>
-    <col min="6" max="6" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="11" width="14.36328125" style="28" customWidth="1"/>
-    <col min="12" max="12" width="30.36328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" customWidth="true" style="28" width="17.54296875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="29.7265625"/>
+    <col min="5" max="5" customWidth="true" width="13.81640625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="14.36328125"/>
+    <col min="7" max="11" customWidth="true" style="28" width="14.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="30.36328125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="10.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -6013,17 +6685,17 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="21.81640625" style="28" customWidth="1"/>
-    <col min="2" max="2" width="16.54296875" style="28" customWidth="1"/>
-    <col min="3" max="3" width="19.90625" style="28" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" style="28" customWidth="1"/>
-    <col min="5" max="6" width="12.90625" style="28" customWidth="1"/>
-    <col min="7" max="7" width="15" style="28" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="28" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.81640625" style="28"/>
-    <col min="10" max="10" width="17.90625" style="28" customWidth="1"/>
-    <col min="11" max="11" width="14.1796875" style="28" customWidth="1"/>
-    <col min="12" max="16384" width="8.81640625" style="28"/>
+    <col min="1" max="1" customWidth="true" style="28" width="21.81640625"/>
+    <col min="2" max="2" customWidth="true" style="28" width="16.54296875"/>
+    <col min="3" max="3" customWidth="true" style="28" width="19.90625"/>
+    <col min="4" max="4" customWidth="true" style="28" width="18.81640625"/>
+    <col min="5" max="6" customWidth="true" style="28" width="12.90625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="28" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="28" width="11.90625"/>
+    <col min="9" max="9" style="28" width="8.81640625"/>
+    <col min="10" max="10" customWidth="true" style="28" width="17.90625"/>
+    <col min="11" max="11" customWidth="true" style="28" width="14.1796875"/>
+    <col min="12" max="16384" style="28" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -6199,12 +6871,12 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="42.1796875" style="28" customWidth="1"/>
-    <col min="2" max="2" width="15.81640625" style="28" customWidth="1"/>
-    <col min="3" max="3" width="17.81640625" style="28" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" style="28" customWidth="1"/>
-    <col min="5" max="5" width="15.6328125" style="28" customWidth="1"/>
-    <col min="6" max="16384" width="8.81640625" style="28"/>
+    <col min="1" max="1" customWidth="true" style="28" width="42.1796875"/>
+    <col min="2" max="2" customWidth="true" style="28" width="15.81640625"/>
+    <col min="3" max="3" customWidth="true" style="28" width="17.81640625"/>
+    <col min="4" max="4" customWidth="true" style="28" width="16.81640625"/>
+    <col min="5" max="5" customWidth="true" style="28" width="15.6328125"/>
+    <col min="6" max="16384" style="28" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -6323,28 +6995,28 @@
   <dimension ref="A1:AB6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="51.81640625" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="51.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.453125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="15.36328125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="15.36328125"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -6767,12 +7439,12 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="76.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="76.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="16.6328125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="19.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -6792,16 +7464,16 @@
         <v>64</v>
       </c>
       <c r="F1" s="43" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="G1" s="43" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
       <c r="H1" s="43" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
       <c r="I1" s="43" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -6825,7 +7497,7 @@
       </c>
       <c r="G2" s="37"/>
       <c r="H2" s="45" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="I2" s="42"/>
     </row>
@@ -6846,10 +7518,10 @@
         <v>30</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="G3" s="68" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="H3" s="42"/>
       <c r="I3" s="42"/>
@@ -6874,13 +7546,13 @@
         <v>46</v>
       </c>
       <c r="G4" s="68" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="H4" s="45" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="I4" s="42" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
     </row>
   </sheetData>
@@ -6897,17 +7569,17 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="68.08984375" style="28" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" style="28" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" style="28" customWidth="1"/>
-    <col min="4" max="4" width="9.6328125" style="28" customWidth="1"/>
-    <col min="5" max="5" width="17.26953125" style="28" customWidth="1"/>
-    <col min="6" max="6" width="12.54296875" style="28" customWidth="1"/>
-    <col min="7" max="10" width="8.81640625" style="28"/>
-    <col min="11" max="11" width="10.6328125" style="28" customWidth="1"/>
-    <col min="12" max="12" width="12.26953125" style="28" customWidth="1"/>
-    <col min="13" max="13" width="15.36328125" style="28" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.81640625" style="28"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="28" width="68.08984375"/>
+    <col min="2" max="2" customWidth="true" style="28" width="12.54296875"/>
+    <col min="3" max="3" customWidth="true" style="28" width="12.36328125"/>
+    <col min="4" max="4" customWidth="true" style="28" width="9.6328125"/>
+    <col min="5" max="5" customWidth="true" style="28" width="17.26953125"/>
+    <col min="6" max="6" customWidth="true" style="28" width="12.54296875"/>
+    <col min="7" max="10" style="28" width="8.81640625"/>
+    <col min="11" max="11" customWidth="true" style="28" width="10.6328125"/>
+    <col min="12" max="12" customWidth="true" style="28" width="12.26953125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="28" width="15.36328125"/>
+    <col min="14" max="16384" style="28" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -6927,7 +7599,7 @@
         <v>1</v>
       </c>
       <c r="F1" s="40" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
       <c r="G1" s="40" t="s">
         <v>52</v>
@@ -6936,19 +7608,19 @@
         <v>4</v>
       </c>
       <c r="I1" s="40" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="J1" s="41" t="s">
         <v>70</v>
       </c>
       <c r="K1" s="40" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="L1" s="40" t="s">
+        <v>841</v>
+      </c>
+      <c r="M1" s="40" t="s">
         <v>843</v>
-      </c>
-      <c r="M1" s="40" t="s">
-        <v>845</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -6959,7 +7631,7 @@
         <v>145</v>
       </c>
       <c r="C2" s="45" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="D2" s="42" t="s">
         <v>259</v>
@@ -6984,7 +7656,7 @@
         <v>145</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="D3" s="42" t="s">
         <v>259</v>
@@ -7009,7 +7681,7 @@
         <v>145</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="D4" s="42" t="s">
         <v>259</v>
@@ -7030,7 +7702,7 @@
         <v>524</v>
       </c>
       <c r="J4" s="42" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="K4" s="42"/>
       <c r="L4" s="42"/>
@@ -7152,10 +7824,10 @@
       <c r="I9" s="42"/>
       <c r="J9" s="42"/>
       <c r="K9" s="45" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="L9" s="45" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="M9" s="42"/>
     </row>
@@ -7238,7 +7910,7 @@
         <v>145</v>
       </c>
       <c r="C13" s="45" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="D13" s="42" t="s">
         <v>259</v>
@@ -7265,7 +7937,7 @@
         <v>145</v>
       </c>
       <c r="C14" s="45" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="D14" s="42" t="s">
         <v>259</v>
@@ -7296,7 +7968,7 @@
         <v>145</v>
       </c>
       <c r="C15" s="45" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="D15" s="42" t="s">
         <v>259</v>
@@ -7333,8 +8005,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.54296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -7374,11 +8046,11 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -7428,8 +8100,8 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="61.7265625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="61.7265625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="70" customFormat="1">
@@ -7825,31 +8497,31 @@
   <dimension ref="A1:AG14"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="49.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="49.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="4.81640625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="9.7265625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -8075,7 +8747,7 @@
         <v>0</v>
       </c>
       <c r="K4" s="68" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
       <c r="L4" s="37" t="s">
         <v>12</v>
@@ -8093,7 +8765,7 @@
         <v>12</v>
       </c>
       <c r="Q4" s="37" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="R4" s="37">
         <v>0</v>
@@ -8111,42 +8783,42 @@
         <v>0</v>
       </c>
       <c r="W4" s="68" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="X4" s="37" t="s">
         <v>12</v>
       </c>
       <c r="Y4" s="37" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="Z4" s="37">
         <v>0</v>
       </c>
       <c r="AA4" s="68" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="AB4" s="37" t="s">
         <v>12</v>
       </c>
       <c r="AC4" s="37" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="AD4" s="37">
         <v>0</v>
       </c>
       <c r="AE4" s="68" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="AF4" s="37" t="s">
         <v>12</v>
       </c>
       <c r="AG4" s="37" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
     </row>
     <row r="5" spans="1:33">
       <c r="A5" s="65" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="B5" s="74">
         <v>1</v>
@@ -8191,7 +8863,7 @@
     </row>
     <row r="6" spans="1:33">
       <c r="A6" s="65" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="B6" s="74">
         <v>1</v>
@@ -8236,11 +8908,11 @@
     </row>
     <row r="7" spans="1:33">
       <c r="A7" s="65" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="B7" s="74"/>
       <c r="C7" s="75" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="D7" s="76" t="s">
         <v>675</v>
@@ -8279,13 +8951,13 @@
     </row>
     <row r="8" spans="1:33">
       <c r="A8" s="65" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="B8" s="74">
         <v>3</v>
       </c>
       <c r="C8" s="75" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="D8" s="76" t="s">
         <v>584</v>
@@ -8324,7 +8996,7 @@
     </row>
     <row r="9" spans="1:33">
       <c r="A9" s="65" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="B9" s="74">
         <v>1</v>
@@ -8369,13 +9041,13 @@
     </row>
     <row r="10" spans="1:33">
       <c r="A10" s="65" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="B10" s="74">
         <v>1</v>
       </c>
       <c r="C10" s="75" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="D10" s="75"/>
       <c r="E10" s="75"/>
@@ -8410,13 +9082,13 @@
     </row>
     <row r="11" spans="1:33">
       <c r="A11" s="65" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="B11" s="74">
         <v>1</v>
       </c>
       <c r="C11" s="75" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="D11" s="76" t="s">
         <v>30</v>
@@ -8455,13 +9127,13 @@
     </row>
     <row r="12" spans="1:33">
       <c r="A12" s="65" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="B12" s="74">
         <v>1</v>
       </c>
       <c r="C12" s="75" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="D12" s="76" t="s">
         <v>12</v>
@@ -8500,25 +9172,25 @@
     </row>
     <row r="13" spans="1:33">
       <c r="A13" s="65" t="s">
+        <v>800</v>
+      </c>
+      <c r="B13" s="74">
+        <v>1</v>
+      </c>
+      <c r="C13" s="73" t="s">
+        <v>801</v>
+      </c>
+      <c r="D13" s="76" t="s">
         <v>802</v>
       </c>
-      <c r="B13" s="74">
-        <v>1</v>
-      </c>
-      <c r="C13" s="73" t="s">
+      <c r="E13" s="76" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="78">
+        <v>1</v>
+      </c>
+      <c r="G13" s="78" t="s">
         <v>803</v>
-      </c>
-      <c r="D13" s="76" t="s">
-        <v>804</v>
-      </c>
-      <c r="E13" s="76" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="78">
-        <v>1</v>
-      </c>
-      <c r="G13" s="78" t="s">
-        <v>805</v>
       </c>
       <c r="H13" s="78" t="s">
         <v>30</v>
@@ -8553,7 +9225,7 @@
     </row>
     <row r="14" spans="1:33">
       <c r="A14" s="65" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="B14" s="74">
         <v>1</v>
@@ -8572,7 +9244,7 @@
         <v>1</v>
       </c>
       <c r="G14" s="78" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="H14" s="77" t="s">
         <v>596</v>
@@ -8628,27 +9300,27 @@
   <dimension ref="A1:AH11"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="10.453125" customWidth="1"/>
-    <col min="6" max="6" width="10.90625" customWidth="1"/>
-    <col min="12" max="12" width="18.36328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.81640625" customWidth="1"/>
-    <col min="20" max="20" width="9.453125" customWidth="1"/>
-    <col min="21" max="21" width="11.08984375" customWidth="1"/>
-    <col min="22" max="22" width="9.36328125" customWidth="1"/>
-    <col min="23" max="23" width="9.453125" customWidth="1"/>
-    <col min="24" max="24" width="10.7265625" customWidth="1"/>
-    <col min="25" max="25" width="11.36328125" customWidth="1"/>
-    <col min="26" max="26" width="12" customWidth="1"/>
-    <col min="27" max="27" width="10.1796875" customWidth="1"/>
-    <col min="30" max="30" width="9" customWidth="1"/>
-    <col min="34" max="34" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="33.0"/>
+    <col min="2" max="2" customWidth="true" width="10.453125"/>
+    <col min="6" max="6" customWidth="true" width="10.90625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.36328125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.36328125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.36328125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="19" max="19" customWidth="true" width="8.81640625"/>
+    <col min="20" max="20" customWidth="true" width="9.453125"/>
+    <col min="21" max="21" customWidth="true" width="11.08984375"/>
+    <col min="22" max="22" customWidth="true" width="9.36328125"/>
+    <col min="23" max="23" customWidth="true" width="9.453125"/>
+    <col min="24" max="24" customWidth="true" width="10.7265625"/>
+    <col min="25" max="25" customWidth="true" width="11.36328125"/>
+    <col min="26" max="26" customWidth="true" width="12.0"/>
+    <col min="27" max="27" customWidth="true" width="10.1796875"/>
+    <col min="30" max="30" customWidth="true" width="9.0"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="17.54296875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -8779,14 +9451,14 @@
       <c r="I2" s="42"/>
       <c r="J2" s="42"/>
       <c r="K2" s="42" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="L2" s="3"/>
       <c r="M2" s="3" t="s">
         <v>312</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>204</v>
@@ -8845,7 +9517,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="42" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
@@ -8899,7 +9571,7 @@
         <v>4</v>
       </c>
       <c r="AE3" s="45" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="AF3" s="42" t="s">
         <v>12</v>
@@ -8999,7 +9671,7 @@
         <v>1</v>
       </c>
       <c r="K5" s="42" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="L5" s="3"/>
       <c r="M5" s="3" t="s">
@@ -9009,7 +9681,7 @@
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="45" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="R5" s="15" t="s">
         <v>40</v>
@@ -9079,7 +9751,7 @@
       <c r="I6" s="42"/>
       <c r="J6" s="42"/>
       <c r="K6" s="42" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
@@ -9129,12 +9801,12 @@
       <c r="I7" s="42"/>
       <c r="J7" s="42"/>
       <c r="K7" s="42" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
       <c r="N7" s="3" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="O7" s="3"/>
       <c r="P7" s="3"/>
@@ -9229,7 +9901,7 @@
       <c r="I9" s="42"/>
       <c r="J9" s="42"/>
       <c r="K9" s="42" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>432</v>
@@ -9238,7 +9910,7 @@
         <v>312</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>204</v>
@@ -9266,50 +9938,50 @@
       <c r="AH9" s="42"/>
     </row>
     <row r="10" spans="1:34">
-      <c r="B10" s="85" t="s">
+      <c r="B10" s="92" t="s">
+        <v>776</v>
+      </c>
+      <c r="C10" s="92"/>
+      <c r="D10" s="92"/>
+      <c r="E10" s="92"/>
+      <c r="G10" s="92" t="s">
+        <v>777</v>
+      </c>
+      <c r="H10" s="92"/>
+      <c r="I10" s="92"/>
+      <c r="J10" s="92"/>
+      <c r="R10" s="92" t="s">
         <v>778</v>
       </c>
-      <c r="C10" s="85"/>
-      <c r="D10" s="85"/>
-      <c r="E10" s="85"/>
-      <c r="G10" s="85" t="s">
+      <c r="S10" s="92"/>
+      <c r="T10" s="92"/>
+      <c r="U10" s="92"/>
+      <c r="W10" s="92" t="s">
         <v>779</v>
       </c>
-      <c r="H10" s="85"/>
-      <c r="I10" s="85"/>
-      <c r="J10" s="85"/>
-      <c r="R10" s="85" t="s">
+      <c r="X10" s="92"/>
+      <c r="Y10" s="92"/>
+      <c r="Z10" s="92"/>
+      <c r="AA10" s="92" t="s">
         <v>780</v>
       </c>
-      <c r="S10" s="85"/>
-      <c r="T10" s="85"/>
-      <c r="U10" s="85"/>
-      <c r="W10" s="85" t="s">
+      <c r="AB10" s="92"/>
+      <c r="AC10" s="92"/>
+      <c r="AD10" s="92"/>
+      <c r="AE10" s="89" t="s">
         <v>781</v>
       </c>
-      <c r="X10" s="85"/>
-      <c r="Y10" s="85"/>
-      <c r="Z10" s="85"/>
-      <c r="AA10" s="85" t="s">
-        <v>782</v>
-      </c>
-      <c r="AB10" s="85"/>
-      <c r="AC10" s="85"/>
-      <c r="AD10" s="85"/>
-      <c r="AE10" s="82" t="s">
-        <v>783</v>
-      </c>
-      <c r="AF10" s="83"/>
-      <c r="AG10" s="83"/>
-      <c r="AH10" s="84"/>
+      <c r="AF10" s="90"/>
+      <c r="AG10" s="90"/>
+      <c r="AH10" s="91"/>
     </row>
     <row r="11" spans="1:34">
-      <c r="G11" s="81" t="s">
-        <v>813</v>
-      </c>
-      <c r="H11" s="81"/>
-      <c r="I11" s="81"/>
-      <c r="J11" s="81"/>
+      <c r="G11" s="88" t="s">
+        <v>811</v>
+      </c>
+      <c r="H11" s="88"/>
+      <c r="I11" s="88"/>
+      <c r="J11" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -9333,11 +10005,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="35.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.54296875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -9421,10 +10093,10 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.90625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="14.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -9473,10 +10145,10 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="42" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="B3" s="45" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="C3" s="42" t="s">
         <v>134</v>
@@ -9485,16 +10157,16 @@
         <v>135</v>
       </c>
       <c r="E3" s="45" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="F3" s="45" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
       <c r="G3" s="42"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="42" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="B4" s="42"/>
       <c r="C4" s="42"/>
@@ -9518,9 +10190,9 @@
   <dimension ref="A1:AC4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="46.6328125" customWidth="1"/>
-    <col min="5" max="5" width="6.1796875" customWidth="1"/>
-    <col min="29" max="29" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="46.6328125"/>
+    <col min="5" max="5" customWidth="true" width="6.1796875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="13.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -9818,14 +10490,14 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="63.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="63.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="10.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="19.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="15.54296875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="8" max="9" bestFit="true" customWidth="true" width="19.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -9960,24 +10632,24 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.6328125" customWidth="1"/>
-    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="7.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="17" max="17" customWidth="true" width="17.6328125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -10290,27 +10962,27 @@
   <dimension ref="A1:U4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="44.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.1796875" customWidth="1"/>
-    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6328125" customWidth="1"/>
-    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="44.08984375"/>
+    <col min="2" max="2" customWidth="true" width="13.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.1796875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
+    <col min="6" max="6" customWidth="true" width="11.6328125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="9.1796875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="6.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="8.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="14.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -10398,7 +11070,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="45" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="H2" s="42" t="s">
         <v>158</v>
@@ -10407,7 +11079,7 @@
         <v>159</v>
       </c>
       <c r="J2" s="54" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="K2" s="42" t="s">
         <v>518</v>
@@ -10416,7 +11088,7 @@
         <v>210</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>12</v>
@@ -10431,7 +11103,7 @@
         <v>212</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>211</v>
@@ -10440,7 +11112,7 @@
         <v>159</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -10463,7 +11135,7 @@
         <v>1</v>
       </c>
       <c r="G3" s="45" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="H3" s="42" t="s">
         <v>158</v>
@@ -10472,16 +11144,16 @@
         <v>159</v>
       </c>
       <c r="J3" s="54" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="K3" s="42" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>157</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>12</v>
@@ -10490,13 +11162,13 @@
         <v>158</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>158</v>
@@ -10505,22 +11177,22 @@
         <v>159</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
     </row>
     <row r="4" spans="1:21">
-      <c r="B4" s="86" t="s">
-        <v>822</v>
-      </c>
-      <c r="C4" s="87"/>
-      <c r="D4" s="87"/>
-      <c r="E4" s="88"/>
-      <c r="F4" s="86" t="s">
-        <v>832</v>
-      </c>
-      <c r="G4" s="87"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="88"/>
+      <c r="B4" s="93" t="s">
+        <v>820</v>
+      </c>
+      <c r="C4" s="94"/>
+      <c r="D4" s="94"/>
+      <c r="E4" s="95"/>
+      <c r="F4" s="93" t="s">
+        <v>830</v>
+      </c>
+      <c r="G4" s="94"/>
+      <c r="H4" s="94"/>
+      <c r="I4" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -10539,8 +11211,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -10588,8 +11260,8 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="18.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="11.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -10609,7 +11281,7 @@
         <v>143</v>
       </c>
       <c r="F1" s="40" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -10641,7 +11313,7 @@
         <v>149</v>
       </c>
       <c r="F3" s="42" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
     </row>
   </sheetData>
@@ -10657,21 +11329,21 @@
   <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="24.90625" style="28" customWidth="1"/>
-    <col min="2" max="2" width="14" style="28" customWidth="1"/>
-    <col min="3" max="3" width="11.81640625" style="28" customWidth="1"/>
-    <col min="4" max="4" width="9.54296875" style="28" customWidth="1"/>
-    <col min="5" max="5" width="10.36328125" style="28" customWidth="1"/>
-    <col min="6" max="6" width="9.36328125" style="28" customWidth="1"/>
-    <col min="7" max="7" width="9.7265625" style="28" customWidth="1"/>
-    <col min="8" max="8" width="10.453125" style="28" customWidth="1"/>
-    <col min="9" max="9" width="8.81640625" style="28" customWidth="1"/>
-    <col min="10" max="10" width="8.08984375" style="39" customWidth="1"/>
-    <col min="11" max="11" width="10" style="28" customWidth="1"/>
-    <col min="12" max="12" width="7.81640625" style="28" customWidth="1"/>
-    <col min="13" max="13" width="9" style="28" customWidth="1"/>
-    <col min="14" max="14" width="19.453125" style="28" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.81640625" style="28"/>
+    <col min="1" max="1" customWidth="true" style="28" width="24.90625"/>
+    <col min="2" max="2" customWidth="true" style="28" width="14.0"/>
+    <col min="3" max="3" customWidth="true" style="28" width="11.81640625"/>
+    <col min="4" max="4" customWidth="true" style="28" width="9.54296875"/>
+    <col min="5" max="5" customWidth="true" style="28" width="10.36328125"/>
+    <col min="6" max="6" customWidth="true" style="28" width="9.36328125"/>
+    <col min="7" max="7" customWidth="true" style="28" width="9.7265625"/>
+    <col min="8" max="8" customWidth="true" style="28" width="10.453125"/>
+    <col min="9" max="9" customWidth="true" style="28" width="8.81640625"/>
+    <col min="10" max="10" customWidth="true" style="39" width="8.08984375"/>
+    <col min="11" max="11" customWidth="true" style="28" width="10.0"/>
+    <col min="12" max="12" customWidth="true" style="28" width="7.81640625"/>
+    <col min="13" max="13" customWidth="true" style="28" width="9.0"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="28" width="19.453125"/>
+    <col min="15" max="16384" style="28" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -11441,15 +12113,15 @@
   <dimension ref="A1:P19"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="21.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="6.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -11481,10 +12153,10 @@
         <v>44</v>
       </c>
       <c r="J1" s="40" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="K1" s="40" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="L1" s="40" t="s">
         <v>1</v>
@@ -11525,10 +12197,10 @@
         <v>46</v>
       </c>
       <c r="H2" s="42" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
       <c r="I2" s="42" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="J2" s="42"/>
       <c r="K2" s="42"/>
@@ -11561,7 +12233,7 @@
         <v>46</v>
       </c>
       <c r="H3" s="42" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
       <c r="I3" s="42" t="s">
         <v>370</v>
@@ -11576,7 +12248,7 @@
     </row>
     <row r="4" spans="1:16">
       <c r="A4" s="42" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="B4" s="42">
         <v>1</v>
@@ -11593,7 +12265,7 @@
       <c r="H4" s="42"/>
       <c r="I4" s="42"/>
       <c r="J4" s="45" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="K4" s="42"/>
       <c r="L4" s="42"/>
@@ -11604,7 +12276,7 @@
     </row>
     <row r="5" spans="1:16">
       <c r="A5" s="42" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="B5" s="42">
         <v>1</v>
@@ -11621,7 +12293,7 @@
       <c r="H5" s="42"/>
       <c r="I5" s="42"/>
       <c r="J5" s="45" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="K5" s="42"/>
       <c r="L5" s="42"/>
@@ -11632,7 +12304,7 @@
     </row>
     <row r="6" spans="1:16">
       <c r="A6" s="42" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="B6" s="42">
         <v>1</v>
@@ -11649,7 +12321,7 @@
       <c r="H6" s="42"/>
       <c r="I6" s="42"/>
       <c r="J6" s="45" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="K6" s="42"/>
       <c r="L6" s="42"/>
@@ -11660,7 +12332,7 @@
     </row>
     <row r="7" spans="1:16">
       <c r="A7" s="42" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="B7" s="42">
         <v>1</v>
@@ -11686,7 +12358,7 @@
     </row>
     <row r="8" spans="1:16">
       <c r="A8" s="42" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="B8" s="42">
         <v>1</v>
@@ -11703,7 +12375,7 @@
       <c r="H8" s="42"/>
       <c r="I8" s="42"/>
       <c r="J8" s="45" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
       <c r="K8" s="42"/>
       <c r="L8" s="42"/>
@@ -11714,7 +12386,7 @@
     </row>
     <row r="9" spans="1:16">
       <c r="A9" s="42" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="B9" s="42">
         <v>1</v>
@@ -11733,14 +12405,14 @@
       </c>
       <c r="G9" s="42"/>
       <c r="H9" s="42" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="I9" s="42" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
       <c r="J9" s="42"/>
       <c r="K9" s="42" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="L9" s="42"/>
       <c r="M9" s="42"/>
@@ -11750,7 +12422,7 @@
     </row>
     <row r="10" spans="1:16">
       <c r="A10" s="42" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="B10" s="42">
         <v>1</v>
@@ -11769,14 +12441,14 @@
       </c>
       <c r="G10" s="42"/>
       <c r="H10" s="42" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
       <c r="I10" s="42" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="J10" s="42"/>
       <c r="K10" s="42" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="L10" s="42"/>
       <c r="M10" s="42"/>
@@ -11786,7 +12458,7 @@
     </row>
     <row r="11" spans="1:16">
       <c r="A11" s="52" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="B11" s="42">
         <v>1</v>
@@ -11805,10 +12477,10 @@
       </c>
       <c r="G11" s="42"/>
       <c r="H11" s="42" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="I11" s="42" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="J11" s="42"/>
       <c r="K11" s="45" t="s">
@@ -11822,7 +12494,7 @@
     </row>
     <row r="12" spans="1:16">
       <c r="A12" s="52" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="B12" s="42">
         <v>1</v>
@@ -11841,13 +12513,13 @@
       </c>
       <c r="G12" s="42"/>
       <c r="H12" s="42" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="I12" s="42" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="J12" s="45" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="K12" s="42"/>
       <c r="L12" s="42">
@@ -11868,7 +12540,7 @@
     </row>
     <row r="13" spans="1:16">
       <c r="A13" s="52" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="B13" s="42">
         <v>1</v>
@@ -11887,13 +12559,13 @@
       </c>
       <c r="G13" s="42"/>
       <c r="H13" s="42" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="I13" s="42" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="J13" s="45" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="K13" s="42"/>
       <c r="L13" s="42"/>
@@ -11904,7 +12576,7 @@
     </row>
     <row r="14" spans="1:16">
       <c r="A14" s="52" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="B14" s="42">
         <v>1</v>
@@ -11923,13 +12595,13 @@
       </c>
       <c r="G14" s="42"/>
       <c r="H14" s="42" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="I14" s="42" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="J14" s="45" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
       <c r="K14" s="42"/>
       <c r="L14" s="42">
@@ -11950,7 +12622,7 @@
     </row>
     <row r="15" spans="1:16">
       <c r="A15" s="52" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="B15" s="42">
         <v>1</v>
@@ -11969,13 +12641,13 @@
       </c>
       <c r="G15" s="42"/>
       <c r="H15" s="42" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="I15" s="42" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="J15" s="45" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
       <c r="K15" s="42"/>
       <c r="L15" s="42"/>
@@ -11986,7 +12658,7 @@
     </row>
     <row r="16" spans="1:16">
       <c r="A16" s="52" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="B16" s="42">
         <v>1</v>
@@ -12005,16 +12677,16 @@
       </c>
       <c r="G16" s="42"/>
       <c r="H16" s="42" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="I16" s="42" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="J16" s="45" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="K16" s="42" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="L16" s="42"/>
       <c r="M16" s="42"/>
@@ -12024,7 +12696,7 @@
     </row>
     <row r="17" spans="1:16">
       <c r="A17" s="52" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="B17" s="42">
         <v>1</v>
@@ -12043,13 +12715,13 @@
       </c>
       <c r="G17" s="42"/>
       <c r="H17" s="42" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="I17" s="42" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
       <c r="J17" s="45" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="K17" s="42"/>
       <c r="L17" s="42"/>
@@ -12060,7 +12732,7 @@
     </row>
     <row r="18" spans="1:16">
       <c r="A18" s="79" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
       <c r="B18" s="42">
         <v>0</v>
@@ -12081,10 +12753,10 @@
         <v>46</v>
       </c>
       <c r="H18" s="42" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
       <c r="I18" s="42" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
       <c r="J18" s="42"/>
       <c r="K18" s="42"/>
@@ -12096,7 +12768,7 @@
     </row>
     <row r="19" spans="1:16">
       <c r="A19" s="79" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
       <c r="B19" s="42">
         <v>0</v>
@@ -12117,10 +12789,10 @@
         <v>46</v>
       </c>
       <c r="H19" s="42" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="I19" s="42" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="J19" s="42"/>
       <c r="K19" s="42"/>
@@ -12144,18 +12816,18 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" customWidth="1"/>
-    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.08984375" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="4" max="4" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="13" max="13" customWidth="true" width="15.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -12347,30 +13019,30 @@
   <dimension ref="A1:W5"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.90625" style="28" customWidth="1"/>
-    <col min="2" max="2" width="10.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.453125" style="39" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7265625" style="39" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" style="39" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.7265625" style="39" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="28" customWidth="1"/>
-    <col min="9" max="9" width="16.54296875" style="28" customWidth="1"/>
-    <col min="10" max="10" width="14.08984375" style="28" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.36328125" style="39" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.36328125" style="39" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" style="28"/>
-    <col min="14" max="14" width="12.54296875" style="28" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.7265625" style="28" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.26953125" style="28" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" style="39" customWidth="1"/>
-    <col min="18" max="18" width="8.7265625" style="39" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.90625" style="28" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12" style="28" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.81640625" style="28"/>
-    <col min="22" max="22" width="10.6328125" style="28" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.90625" style="28" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="8.81640625" style="28"/>
+    <col min="1" max="1" customWidth="true" style="28" width="19.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="39" width="10.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="39" width="9.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="39" width="7.7265625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="39" width="10.90625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="39" width="9.453125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="39" width="7.7265625"/>
+    <col min="8" max="8" customWidth="true" style="28" width="13.0"/>
+    <col min="9" max="9" customWidth="true" style="28" width="16.54296875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="28" width="14.08984375"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="39" width="10.36328125"/>
+    <col min="12" max="12" customWidth="true" style="39" width="10.36328125"/>
+    <col min="13" max="13" style="28" width="8.81640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="28" width="12.54296875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="28" width="14.7265625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="28" width="13.26953125"/>
+    <col min="17" max="17" customWidth="true" style="39" width="11.54296875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="39" width="8.7265625"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="28" width="9.90625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="28" width="12.0"/>
+    <col min="21" max="21" style="28" width="8.81640625"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="28" width="10.6328125"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="28" width="13.90625"/>
+    <col min="24" max="16384" style="28" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -12610,7 +13282,7 @@
         <v>14</v>
       </c>
       <c r="M4" s="31" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="N4" s="31"/>
       <c r="O4" s="31"/>
@@ -12619,31 +13291,31 @@
         <v>42</v>
       </c>
       <c r="R4" s="42" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="S4" s="31"/>
       <c r="T4" s="31"/>
       <c r="U4" s="42" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="V4" s="42" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="W4" s="42" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="5" spans="1:23">
-      <c r="B5" s="89" t="s">
-        <v>822</v>
-      </c>
-      <c r="C5" s="89"/>
-      <c r="D5" s="89"/>
-      <c r="E5" s="90" t="s">
-        <v>881</v>
-      </c>
-      <c r="F5" s="90"/>
-      <c r="G5" s="90"/>
+      <c r="B5" s="96" t="s">
+        <v>820</v>
+      </c>
+      <c r="C5" s="96"/>
+      <c r="D5" s="96"/>
+      <c r="E5" s="97" t="s">
+        <v>879</v>
+      </c>
+      <c r="F5" s="97"/>
+      <c r="G5" s="97"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -12662,19 +13334,19 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="19.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -12777,20 +13449,20 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="25.81640625" style="39" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="39" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" style="39" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.453125" style="39" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.1796875" style="39" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.90625" style="39"/>
+    <col min="1" max="1" customWidth="true" style="39" width="25.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="39" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="39" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="39" width="4.453125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="39" width="14.1796875"/>
+    <col min="14" max="16384" style="39" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -12916,21 +13588,21 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="20.1796875" style="39" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="39" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="17.36328125" style="39" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" style="39" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.453125" style="39" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.36328125" style="39" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.1796875" style="39" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.90625" style="39"/>
+    <col min="1" max="1" customWidth="true" style="39" width="20.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="39" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
+    <col min="6" max="7" customWidth="true" style="39" width="17.36328125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="39" width="15.0"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="39" width="4.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="39" width="17.36328125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="39" width="14.1796875"/>
+    <col min="16" max="16384" style="39" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -13117,22 +13789,22 @@
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="28.36328125" style="39" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.36328125" style="39" customWidth="1"/>
-    <col min="4" max="4" width="11.1796875" style="39" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" style="39" customWidth="1"/>
-    <col min="6" max="6" width="12.453125" style="39" customWidth="1"/>
-    <col min="7" max="7" width="11.08984375" style="39" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" style="39" customWidth="1"/>
-    <col min="10" max="10" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.54296875" style="39" customWidth="1"/>
-    <col min="12" max="12" width="10.81640625" style="39" customWidth="1"/>
-    <col min="13" max="13" width="12.1796875" style="39" customWidth="1"/>
-    <col min="14" max="14" width="11.90625" style="39" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.1796875" style="39" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.90625" style="39"/>
+    <col min="1" max="1" customWidth="true" style="39" width="28.36328125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="3" max="3" customWidth="true" style="39" width="10.36328125"/>
+    <col min="4" max="4" customWidth="true" style="39" width="11.1796875"/>
+    <col min="5" max="5" customWidth="true" style="39" width="12.81640625"/>
+    <col min="6" max="6" customWidth="true" style="39" width="12.453125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="39" width="11.08984375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="9" max="9" customWidth="true" style="39" width="9.08984375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="11" max="11" customWidth="true" style="39" width="11.54296875"/>
+    <col min="12" max="12" customWidth="true" style="39" width="10.81640625"/>
+    <col min="13" max="13" customWidth="true" style="39" width="12.1796875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="39" width="11.90625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="39" width="14.1796875"/>
+    <col min="16" max="16384" style="39" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -13247,7 +13919,7 @@
       </c>
       <c r="G4" s="42"/>
       <c r="H4" s="42" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="I4" s="42" t="s">
         <v>373</v>
@@ -13284,7 +13956,7 @@
       </c>
       <c r="G5" s="42"/>
       <c r="H5" s="42" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="I5" s="42" t="s">
         <v>373</v>
@@ -13432,11 +14104,11 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="24" style="39" customWidth="1"/>
-    <col min="2" max="2" width="11.453125" style="39" customWidth="1"/>
-    <col min="3" max="3" width="8.90625" style="39"/>
-    <col min="4" max="4" width="19.6328125" style="39" customWidth="1"/>
-    <col min="5" max="16384" width="8.90625" style="39"/>
+    <col min="1" max="1" customWidth="true" style="39" width="24.0"/>
+    <col min="2" max="2" customWidth="true" style="39" width="11.453125"/>
+    <col min="3" max="3" style="39" width="8.90625"/>
+    <col min="4" max="4" customWidth="true" style="39" width="19.6328125"/>
+    <col min="5" max="16384" style="39" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -13469,7 +14141,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="42" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
       <c r="B3" s="45" t="s">
         <v>339</v>
@@ -13494,12 +14166,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.1796875" style="39" customWidth="1"/>
-    <col min="2" max="2" width="14" style="39" customWidth="1"/>
-    <col min="3" max="3" width="16.6328125" style="39" customWidth="1"/>
-    <col min="4" max="4" width="17.6328125" style="39" customWidth="1"/>
-    <col min="5" max="5" width="11.81640625" style="39" customWidth="1"/>
-    <col min="6" max="16384" width="8.90625" style="39"/>
+    <col min="1" max="1" customWidth="true" style="39" width="32.1796875"/>
+    <col min="2" max="2" customWidth="true" style="39" width="14.0"/>
+    <col min="3" max="3" customWidth="true" style="39" width="16.6328125"/>
+    <col min="4" max="4" customWidth="true" style="39" width="17.6328125"/>
+    <col min="5" max="5" customWidth="true" style="39" width="11.81640625"/>
+    <col min="6" max="16384" style="39" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -13583,11 +14255,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="38.1796875" style="39" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" style="39" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" style="39" customWidth="1"/>
-    <col min="4" max="4" width="19" style="39" customWidth="1"/>
-    <col min="5" max="16384" width="8.90625" style="39"/>
+    <col min="1" max="1" customWidth="true" style="39" width="38.1796875"/>
+    <col min="2" max="2" customWidth="true" style="39" width="13.54296875"/>
+    <col min="3" max="3" customWidth="true" style="39" width="15.54296875"/>
+    <col min="4" max="4" customWidth="true" style="39" width="19.0"/>
+    <col min="5" max="16384" style="39" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -13710,21 +14382,21 @@
   <dimension ref="A1:N5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="30.90625" style="39" customWidth="1"/>
-    <col min="2" max="2" width="17.81640625" style="39" customWidth="1"/>
-    <col min="3" max="3" width="16.453125" style="39" customWidth="1"/>
-    <col min="4" max="4" width="16.08984375" style="39" customWidth="1"/>
-    <col min="5" max="5" width="12" style="39" customWidth="1"/>
-    <col min="6" max="6" width="18.08984375" style="39" customWidth="1"/>
-    <col min="7" max="7" width="15.08984375" style="39" customWidth="1"/>
-    <col min="8" max="8" width="10.453125" style="39" customWidth="1"/>
-    <col min="9" max="9" width="10.81640625" style="39" customWidth="1"/>
-    <col min="10" max="10" width="8.90625" style="39"/>
-    <col min="11" max="11" width="13.1796875" style="39" customWidth="1"/>
-    <col min="12" max="12" width="12.6328125" style="39" customWidth="1"/>
-    <col min="13" max="13" width="14.08984375" style="39" customWidth="1"/>
-    <col min="14" max="14" width="14.36328125" style="39" customWidth="1"/>
-    <col min="15" max="16384" width="8.90625" style="39"/>
+    <col min="1" max="1" customWidth="true" style="39" width="30.90625"/>
+    <col min="2" max="2" customWidth="true" style="39" width="17.81640625"/>
+    <col min="3" max="3" customWidth="true" style="39" width="16.453125"/>
+    <col min="4" max="4" customWidth="true" style="39" width="16.08984375"/>
+    <col min="5" max="5" customWidth="true" style="39" width="12.0"/>
+    <col min="6" max="6" customWidth="true" style="39" width="18.08984375"/>
+    <col min="7" max="7" customWidth="true" style="39" width="15.08984375"/>
+    <col min="8" max="8" customWidth="true" style="39" width="10.453125"/>
+    <col min="9" max="9" customWidth="true" style="39" width="10.81640625"/>
+    <col min="10" max="10" style="39" width="8.90625"/>
+    <col min="11" max="11" customWidth="true" style="39" width="13.1796875"/>
+    <col min="12" max="12" customWidth="true" style="39" width="12.6328125"/>
+    <col min="13" max="13" customWidth="true" style="39" width="14.08984375"/>
+    <col min="14" max="14" customWidth="true" style="39" width="14.36328125"/>
+    <col min="15" max="16384" style="39" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -13926,12 +14598,12 @@
   <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="16.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -14614,11 +15286,11 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="57.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="57.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="15.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="4" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="20.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -14638,7 +15310,7 @@
         <v>26</v>
       </c>
       <c r="F1" s="43" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -14733,7 +15405,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="13" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="B7" s="13">
         <v>1</v>
@@ -14749,7 +15421,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="13" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="B8" s="13">
         <v>1</v>
@@ -14765,13 +15437,13 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="13" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="B9" s="42">
         <v>2</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="D9" s="44" t="s">
         <v>12</v>
@@ -14795,28 +15467,28 @@
   <dimension ref="A1:V15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="50" style="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.36328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.08984375" style="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.36328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="8.81640625" style="25"/>
-    <col min="9" max="9" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13" style="25" customWidth="1"/>
-    <col min="16" max="16" width="10.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="8.81640625" style="25"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="50.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="25" width="18.36328125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="25" width="12.08984375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="25" width="15.36328125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="25" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="25" width="9.453125"/>
+    <col min="7" max="8" style="25" width="8.81640625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="8.1796875"/>
+    <col min="15" max="15" customWidth="true" style="25" width="13.0"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="10.1796875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="25" width="9.1796875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="25" width="11.6328125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
+    <col min="23" max="16384" style="25" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -15511,29 +16183,29 @@
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="44.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="44.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.81640625"/>
+    <col min="11" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.1796875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="27" max="28" bestFit="true" customWidth="true" width="12.81640625"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="12.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -15965,10 +16637,10 @@
   <dimension ref="A1:AJ39"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="54.36328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="54.36328125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="12.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36">
@@ -18254,16 +18926,16 @@
   <dimension ref="A1:S20"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="53.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="12.1796875" customWidth="1"/>
-    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="53.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="5" max="7" customWidth="true" width="12.1796875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">

</xml_diff>

<commit_message>
ProcessMealReport,QueueService and DepartureControlService done by Harshitha
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9FDA1B-BA8D-4856-9CC3-8D54B59B7E2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A836B06-F27C-4EE1-8992-004B58AEF9CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="11" activeTab="12" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="13" activeTab="15" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2972" uniqueCount="1001">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2984" uniqueCount="1005">
   <si>
     <t>Scenario</t>
   </si>
@@ -2560,9 +2560,6 @@
     <t>230033217</t>
   </si>
   <si>
-    <t>303</t>
-  </si>
-  <si>
     <t>BDT3W2</t>
   </si>
   <si>
@@ -2707,12 +2704,6 @@
     <t>ABCD</t>
   </si>
   <si>
-    <t>BKCI4U</t>
-  </si>
-  <si>
-    <t>2023-09-16T00:00:00</t>
-  </si>
-  <si>
     <t>BKDND0</t>
   </si>
   <si>
@@ -2935,9 +2926,6 @@
     <t>2023-09-18T10:20:44</t>
   </si>
   <si>
-    <t>BLWG5Q</t>
-  </si>
-  <si>
     <t>2023-09-19T10:38:00</t>
   </si>
   <si>
@@ -3077,13 +3065,36 @@
   </si>
   <si>
     <t>BLXWFT</t>
+  </si>
+  <si>
+    <t>BMQL5S</t>
+  </si>
+  <si>
+    <t>2023-09-21T00:00:00</t>
+  </si>
+  <si>
+    <t>17D</t>
+  </si>
+  <si>
+    <t>BMQMQN</t>
+  </si>
+  <si>
+    <t>2023-09-21T07:54:00</t>
+  </si>
+  <si>
+    <t>2023-09-21T12:54:00</t>
+  </si>
+  <si>
+    <t>136</t>
+  </si>
+  <si>
+    <t>CTG</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="17">
     <font>
       <sz val="11"/>
@@ -3936,24 +3947,24 @@
   <dimension ref="A1:AC25"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="52.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="8.1796875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.1796875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="11.6328125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="12.6328125"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="12.6328125"/>
+    <col min="1" max="1" width="52.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="12.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -4042,7 +4053,7 @@
         <v>358</v>
       </c>
       <c r="AC1" s="60" t="s">
-        <v>894</v>
+        <v>891</v>
       </c>
     </row>
     <row r="2" spans="1:29">
@@ -4068,7 +4079,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="41" t="s">
-        <v>886</v>
+        <v>883</v>
       </c>
       <c r="I2" s="41" t="s">
         <v>199</v>
@@ -4085,7 +4096,7 @@
       <c r="M2" s="41"/>
       <c r="N2" s="41"/>
       <c r="O2" s="41" t="s">
-        <v>887</v>
+        <v>884</v>
       </c>
       <c r="P2" s="41"/>
       <c r="Q2" s="41"/>
@@ -4125,7 +4136,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="41" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="I3" s="41" t="s">
         <v>200</v>
@@ -4184,7 +4195,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="35" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="I4" s="35" t="s">
         <v>327</v>
@@ -4239,7 +4250,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="35" t="s">
-        <v>908</v>
+        <v>905</v>
       </c>
       <c r="I5" s="41" t="s">
         <v>200</v>
@@ -4296,7 +4307,7 @@
       </c>
       <c r="G6" s="41"/>
       <c r="H6" s="41" t="s">
-        <v>891</v>
+        <v>888</v>
       </c>
       <c r="I6" s="41" t="s">
         <v>606</v>
@@ -4349,7 +4360,7 @@
       </c>
       <c r="G7" s="41"/>
       <c r="H7" s="41" t="s">
-        <v>881</v>
+        <v>878</v>
       </c>
       <c r="I7" s="41" t="s">
         <v>609</v>
@@ -4398,7 +4409,7 @@
       </c>
       <c r="G8" s="41"/>
       <c r="H8" s="41" t="s">
-        <v>893</v>
+        <v>890</v>
       </c>
       <c r="I8" s="41" t="s">
         <v>612</v>
@@ -4451,7 +4462,7 @@
       </c>
       <c r="G9" s="41"/>
       <c r="H9" s="41" t="s">
-        <v>890</v>
+        <v>887</v>
       </c>
       <c r="I9" s="41" t="s">
         <v>615</v>
@@ -4504,7 +4515,7 @@
       </c>
       <c r="G10" s="41"/>
       <c r="H10" s="41" t="s">
-        <v>895</v>
+        <v>892</v>
       </c>
       <c r="I10" s="41" t="s">
         <v>618</v>
@@ -4521,7 +4532,7 @@
       <c r="M10" s="41"/>
       <c r="N10" s="41"/>
       <c r="O10" s="41" t="s">
-        <v>896</v>
+        <v>893</v>
       </c>
       <c r="P10" s="41" t="s">
         <v>345</v>
@@ -4567,7 +4578,7 @@
       </c>
       <c r="G11" s="41"/>
       <c r="H11" s="41" t="s">
-        <v>892</v>
+        <v>889</v>
       </c>
       <c r="I11" s="41" t="s">
         <v>333</v>
@@ -4675,7 +4686,7 @@
       </c>
       <c r="G13" s="41"/>
       <c r="H13" s="41" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="I13" s="41" t="s">
         <v>628</v>
@@ -4730,7 +4741,7 @@
       </c>
       <c r="G14" s="41"/>
       <c r="H14" s="41" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
       <c r="I14" s="41" t="s">
         <v>633</v>
@@ -4785,7 +4796,7 @@
       </c>
       <c r="G15" s="41"/>
       <c r="H15" s="41" t="s">
-        <v>910</v>
+        <v>907</v>
       </c>
       <c r="I15" s="41" t="s">
         <v>637</v>
@@ -4838,7 +4849,7 @@
       </c>
       <c r="G16" s="41"/>
       <c r="H16" s="41" t="s">
-        <v>882</v>
+        <v>879</v>
       </c>
       <c r="I16" s="41" t="s">
         <v>640</v>
@@ -4887,7 +4898,7 @@
       </c>
       <c r="G17" s="41"/>
       <c r="H17" s="41" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="I17" s="41"/>
       <c r="J17" s="41"/>
@@ -4932,7 +4943,7 @@
       </c>
       <c r="G18" s="41"/>
       <c r="H18" s="41" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
       <c r="I18" s="41" t="s">
         <v>20</v>
@@ -4981,7 +4992,7 @@
       </c>
       <c r="G19" s="41"/>
       <c r="H19" s="41" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="I19" s="41"/>
       <c r="J19" s="41"/>
@@ -5046,7 +5057,7 @@
       </c>
       <c r="G20" s="41"/>
       <c r="H20" s="41" t="s">
-        <v>909</v>
+        <v>906</v>
       </c>
       <c r="I20" s="41"/>
       <c r="J20" s="41"/>
@@ -5133,15 +5144,15 @@
   <dimension ref="A1:W36"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="54.81640625"/>
-    <col min="10" max="10" style="25" width="8.81640625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="11.453125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="12.6328125"/>
-    <col min="22" max="23" bestFit="true" customWidth="true" width="19.1796875"/>
+    <col min="1" max="1" width="54.81640625" customWidth="1"/>
+    <col min="10" max="10" width="8.81640625" style="25"/>
+    <col min="12" max="12" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="19.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -5245,7 +5256,7 @@
       </c>
       <c r="J2" s="41"/>
       <c r="K2" s="41" t="s">
-        <v>984</v>
+        <v>980</v>
       </c>
       <c r="L2" s="41"/>
       <c r="M2" s="41"/>
@@ -5360,10 +5371,10 @@
       <c r="I5" s="41"/>
       <c r="J5" s="41"/>
       <c r="K5" s="41" t="s">
-        <v>987</v>
+        <v>983</v>
       </c>
       <c r="L5" s="41" t="s">
-        <v>988</v>
+        <v>984</v>
       </c>
       <c r="M5" s="41"/>
       <c r="N5" s="41" t="s">
@@ -5409,7 +5420,7 @@
       <c r="I6" s="41"/>
       <c r="J6" s="41"/>
       <c r="K6" s="41" t="s">
-        <v>989</v>
+        <v>985</v>
       </c>
       <c r="L6" s="41"/>
       <c r="M6" s="41"/>
@@ -5420,7 +5431,7 @@
         <v>795</v>
       </c>
       <c r="P6" s="41" t="s">
-        <v>990</v>
+        <v>986</v>
       </c>
       <c r="Q6" s="41"/>
       <c r="R6" s="41"/>
@@ -5513,10 +5524,10 @@
       </c>
       <c r="J8" s="41"/>
       <c r="K8" s="41" t="s">
-        <v>991</v>
+        <v>987</v>
       </c>
       <c r="L8" s="41" t="s">
-        <v>992</v>
+        <v>988</v>
       </c>
       <c r="M8" s="41"/>
       <c r="N8" s="41" t="s">
@@ -5556,7 +5567,7 @@
       <c r="I9" s="41"/>
       <c r="J9" s="41"/>
       <c r="K9" s="41" t="s">
-        <v>993</v>
+        <v>989</v>
       </c>
       <c r="L9" s="41"/>
       <c r="M9" s="41"/>
@@ -5573,7 +5584,7 @@
       <c r="T9" s="41"/>
       <c r="U9" s="41"/>
       <c r="V9" s="41" t="s">
-        <v>976</v>
+        <v>972</v>
       </c>
       <c r="W9" s="41"/>
     </row>
@@ -5599,10 +5610,10 @@
       <c r="I10" s="41"/>
       <c r="J10" s="41"/>
       <c r="K10" s="41" t="s">
-        <v>994</v>
+        <v>990</v>
       </c>
       <c r="L10" s="41" t="s">
-        <v>995</v>
+        <v>991</v>
       </c>
       <c r="M10" s="41"/>
       <c r="N10" s="41"/>
@@ -5640,10 +5651,10 @@
       <c r="I11" s="41"/>
       <c r="J11" s="41"/>
       <c r="K11" s="41" t="s">
-        <v>966</v>
+        <v>962</v>
       </c>
       <c r="L11" s="41" t="s">
-        <v>967</v>
+        <v>963</v>
       </c>
       <c r="M11" s="41"/>
       <c r="N11" s="41"/>
@@ -5726,10 +5737,10 @@
       <c r="I13" s="41"/>
       <c r="J13" s="41"/>
       <c r="K13" s="41" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="L13" s="41" t="s">
-        <v>969</v>
+        <v>965</v>
       </c>
       <c r="M13" s="41"/>
       <c r="N13" s="41" t="s">
@@ -5853,7 +5864,7 @@
       <c r="I16" s="41"/>
       <c r="J16" s="41"/>
       <c r="K16" s="41" t="s">
-        <v>970</v>
+        <v>966</v>
       </c>
       <c r="L16" s="41"/>
       <c r="M16" s="41"/>
@@ -5894,7 +5905,7 @@
       <c r="I17" s="41"/>
       <c r="J17" s="41"/>
       <c r="K17" s="41" t="s">
-        <v>971</v>
+        <v>967</v>
       </c>
       <c r="L17" s="41"/>
       <c r="M17" s="41"/>
@@ -5939,7 +5950,7 @@
       </c>
       <c r="J18" s="41"/>
       <c r="K18" s="41" t="s">
-        <v>972</v>
+        <v>968</v>
       </c>
       <c r="L18" s="41"/>
       <c r="M18" s="41"/>
@@ -5956,10 +5967,10 @@
       <c r="T18" s="41"/>
       <c r="U18" s="41"/>
       <c r="V18" s="41" t="s">
-        <v>973</v>
+        <v>969</v>
       </c>
       <c r="W18" s="41" t="s">
-        <v>974</v>
+        <v>970</v>
       </c>
     </row>
     <row r="19" spans="1:23">
@@ -5984,7 +5995,7 @@
       <c r="I19" s="41"/>
       <c r="J19" s="41"/>
       <c r="K19" s="41" t="s">
-        <v>975</v>
+        <v>971</v>
       </c>
       <c r="L19" s="41"/>
       <c r="M19" s="41"/>
@@ -6001,7 +6012,7 @@
       <c r="T19" s="41"/>
       <c r="U19" s="41"/>
       <c r="V19" s="41" t="s">
-        <v>976</v>
+        <v>972</v>
       </c>
       <c r="W19" s="41"/>
     </row>
@@ -6027,7 +6038,7 @@
       <c r="I20" s="41"/>
       <c r="J20" s="41"/>
       <c r="K20" s="41" t="s">
-        <v>977</v>
+        <v>973</v>
       </c>
       <c r="L20" s="41"/>
       <c r="M20" s="41"/>
@@ -6068,7 +6079,7 @@
       <c r="I21" s="41"/>
       <c r="J21" s="41"/>
       <c r="K21" s="41" t="s">
-        <v>978</v>
+        <v>974</v>
       </c>
       <c r="L21" s="41"/>
       <c r="M21" s="41"/>
@@ -6117,7 +6128,7 @@
       </c>
       <c r="J22" s="41"/>
       <c r="K22" s="41" t="s">
-        <v>979</v>
+        <v>975</v>
       </c>
       <c r="L22" s="41"/>
       <c r="M22" s="41"/>
@@ -6216,10 +6227,10 @@
       <c r="I25" s="41"/>
       <c r="J25" s="41"/>
       <c r="K25" s="41" t="s">
-        <v>980</v>
+        <v>976</v>
       </c>
       <c r="L25" s="41" t="s">
-        <v>981</v>
+        <v>977</v>
       </c>
       <c r="M25" s="41"/>
       <c r="N25" s="41" t="s">
@@ -6315,7 +6326,7 @@
       <c r="I28" s="41"/>
       <c r="J28" s="41"/>
       <c r="K28" s="41" t="s">
-        <v>982</v>
+        <v>978</v>
       </c>
       <c r="L28" s="41"/>
       <c r="M28" s="41"/>
@@ -6352,7 +6363,7 @@
       <c r="I29" s="41"/>
       <c r="J29" s="41"/>
       <c r="K29" s="41" t="s">
-        <v>983</v>
+        <v>979</v>
       </c>
       <c r="L29" s="41"/>
       <c r="M29" s="41"/>
@@ -6465,14 +6476,14 @@
       <c r="I32" s="41"/>
       <c r="J32" s="41"/>
       <c r="K32" s="41" t="s">
-        <v>985</v>
+        <v>981</v>
       </c>
       <c r="L32" s="41"/>
       <c r="M32" s="41"/>
       <c r="N32" s="41"/>
       <c r="O32" s="41"/>
       <c r="P32" s="41" t="s">
-        <v>986</v>
+        <v>982</v>
       </c>
       <c r="Q32" s="41"/>
       <c r="R32" s="41"/>
@@ -6653,16 +6664,16 @@
   <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" customWidth="true" style="27" width="17.54296875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="29.81640625"/>
-    <col min="5" max="5" customWidth="true" width="13.81640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="14.36328125"/>
-    <col min="7" max="11" customWidth="true" style="27" width="14.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="13.81640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.54296875"/>
+    <col min="1" max="1" width="32.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" style="27" customWidth="1"/>
+    <col min="4" max="4" width="29.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.81640625" customWidth="1"/>
+    <col min="6" max="6" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="11" width="14.36328125" style="27" customWidth="1"/>
+    <col min="12" max="12" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -6670,7 +6681,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="39" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="C1" s="40" t="s">
         <v>70</v>
@@ -6706,7 +6717,7 @@
         <v>134</v>
       </c>
       <c r="N1" s="39" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -6717,13 +6728,13 @@
         <v>2</v>
       </c>
       <c r="C2" s="41" t="s">
+        <v>829</v>
+      </c>
+      <c r="D2" s="44" t="s">
         <v>830</v>
       </c>
-      <c r="D2" s="44" t="s">
-        <v>831</v>
-      </c>
       <c r="E2" s="44" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="F2" s="41"/>
       <c r="G2" s="44" t="s">
@@ -6752,7 +6763,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="44" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E3" s="44" t="s">
         <v>252</v>
@@ -6788,14 +6799,14 @@
         <v>2</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="E4" s="41"/>
       <c r="F4" s="41" t="s">
         <v>141</v>
       </c>
       <c r="G4" s="44" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="H4" s="41" t="s">
         <v>12</v>
@@ -6830,17 +6841,17 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="27" width="21.81640625"/>
-    <col min="2" max="2" customWidth="true" style="27" width="16.54296875"/>
-    <col min="3" max="3" customWidth="true" style="27" width="19.90625"/>
-    <col min="4" max="4" customWidth="true" style="27" width="18.81640625"/>
-    <col min="5" max="6" customWidth="true" style="27" width="12.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="27" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="27" width="11.90625"/>
-    <col min="9" max="9" style="27" width="8.81640625"/>
-    <col min="10" max="10" customWidth="true" style="27" width="17.90625"/>
-    <col min="11" max="11" customWidth="true" style="27" width="14.1796875"/>
-    <col min="12" max="16384" style="27" width="8.81640625"/>
+    <col min="1" max="1" width="21.81640625" style="27" customWidth="1"/>
+    <col min="2" max="2" width="16.54296875" style="27" customWidth="1"/>
+    <col min="3" max="3" width="19.90625" style="27" customWidth="1"/>
+    <col min="4" max="4" width="18.81640625" style="27" customWidth="1"/>
+    <col min="5" max="6" width="12.90625" style="27" customWidth="1"/>
+    <col min="7" max="7" width="15" style="27" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="27" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.81640625" style="27"/>
+    <col min="10" max="10" width="17.90625" style="27" customWidth="1"/>
+    <col min="11" max="11" width="14.1796875" style="27" customWidth="1"/>
+    <col min="12" max="16384" width="8.81640625" style="27"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -6967,13 +6978,13 @@
         <v>12</v>
       </c>
       <c r="I5" s="41" t="s">
-        <v>924</v>
+        <v>921</v>
       </c>
       <c r="J5" s="41" t="s">
-        <v>925</v>
+        <v>922</v>
       </c>
       <c r="K5" s="41" t="s">
-        <v>926</v>
+        <v>923</v>
       </c>
       <c r="L5" s="41"/>
     </row>
@@ -7003,10 +7014,10 @@
         <v>12</v>
       </c>
       <c r="I6" s="41" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="J6" s="41" t="s">
-        <v>928</v>
+        <v>925</v>
       </c>
       <c r="K6" s="41"/>
       <c r="L6" s="41"/>
@@ -7024,14 +7035,14 @@
   <dimension ref="A1:L7"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="27" width="42.1796875"/>
-    <col min="2" max="2" customWidth="true" style="27" width="15.81640625"/>
-    <col min="3" max="3" customWidth="true" style="27" width="17.81640625"/>
-    <col min="4" max="4" customWidth="true" style="27" width="16.81640625"/>
-    <col min="5" max="5" customWidth="true" style="27" width="15.6328125"/>
-    <col min="6" max="11" style="27" width="8.81640625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="27" width="31.0"/>
-    <col min="13" max="16384" style="27" width="8.81640625"/>
+    <col min="1" max="1" width="42.1796875" style="27" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" style="27" customWidth="1"/>
+    <col min="3" max="3" width="17.81640625" style="27" customWidth="1"/>
+    <col min="4" max="4" width="16.81640625" style="27" customWidth="1"/>
+    <col min="5" max="5" width="15.6328125" style="27" customWidth="1"/>
+    <col min="6" max="11" width="8.81640625" style="27"/>
+    <col min="12" max="12" width="31" style="27" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.81640625" style="27"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -7048,7 +7059,7 @@
         <v>255</v>
       </c>
       <c r="E1" s="39" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
       <c r="F1" s="39" t="s">
         <v>24</v>
@@ -7177,7 +7188,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="44" t="s">
-        <v>997</v>
+        <v>993</v>
       </c>
       <c r="G5" s="41"/>
       <c r="H5" s="41"/>
@@ -7185,7 +7196,7 @@
       <c r="J5" s="41"/>
       <c r="K5" s="41"/>
       <c r="L5" s="84" t="s">
-        <v>996</v>
+        <v>992</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -7201,7 +7212,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="44" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="G6" s="41"/>
       <c r="H6" s="41"/>
@@ -7209,7 +7220,7 @@
       <c r="J6" s="41"/>
       <c r="K6" s="41"/>
       <c r="L6" s="41" t="s">
-        <v>998</v>
+        <v>994</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -7225,7 +7236,7 @@
         <v>-1</v>
       </c>
       <c r="F7" s="44" t="s">
-        <v>999</v>
+        <v>995</v>
       </c>
       <c r="G7" s="41"/>
       <c r="H7" s="41"/>
@@ -7247,22 +7258,22 @@
   <dimension ref="A1:V11"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="51.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="11" max="12" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="13" max="13" customWidth="true" width="13.90625"/>
-    <col min="14" max="14" customWidth="true" width="12.6328125"/>
-    <col min="15" max="15" customWidth="true" width="11.453125"/>
-    <col min="16" max="16" customWidth="true" width="7.81640625"/>
-    <col min="17" max="18" customWidth="true" width="10.6328125"/>
-    <col min="19" max="19" customWidth="true" width="11.81640625"/>
-    <col min="20" max="20" customWidth="true" width="8.81640625"/>
-    <col min="21" max="21" customWidth="true" width="10.81640625"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="51.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.90625" customWidth="1"/>
+    <col min="14" max="14" width="12.6328125" customWidth="1"/>
+    <col min="15" max="15" width="11.453125" customWidth="1"/>
+    <col min="16" max="16" width="7.81640625" customWidth="1"/>
+    <col min="17" max="18" width="10.6328125" customWidth="1"/>
+    <col min="19" max="19" width="11.81640625" customWidth="1"/>
+    <col min="20" max="20" width="8.81640625" customWidth="1"/>
+    <col min="21" max="21" width="10.81640625" customWidth="1"/>
+    <col min="22" max="22" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -7297,16 +7308,16 @@
         <v>69</v>
       </c>
       <c r="K1" s="40" t="s">
+        <v>837</v>
+      </c>
+      <c r="L1" s="40" t="s">
         <v>838</v>
       </c>
-      <c r="L1" s="40" t="s">
-        <v>839</v>
-      </c>
       <c r="M1" s="40" t="s">
+        <v>832</v>
+      </c>
+      <c r="N1" s="40" t="s">
         <v>833</v>
-      </c>
-      <c r="N1" s="40" t="s">
-        <v>834</v>
       </c>
       <c r="O1" s="39" t="s">
         <v>1</v>
@@ -7362,13 +7373,13 @@
         <v>41</v>
       </c>
       <c r="J2" s="41" t="s">
-        <v>1000</v>
+        <v>996</v>
       </c>
       <c r="K2" s="41" t="s">
-        <v>954</v>
+        <v>950</v>
       </c>
       <c r="L2" s="41" t="s">
-        <v>955</v>
+        <v>951</v>
       </c>
       <c r="M2" s="41" t="s">
         <v>652</v>
@@ -7414,19 +7425,19 @@
         <v>12</v>
       </c>
       <c r="J3" s="41" t="s">
-        <v>963</v>
+        <v>959</v>
       </c>
       <c r="K3" s="41" t="s">
-        <v>962</v>
+        <v>958</v>
       </c>
       <c r="L3" s="41" t="s">
-        <v>964</v>
+        <v>960</v>
       </c>
       <c r="M3" s="41" t="s">
+        <v>957</v>
+      </c>
+      <c r="N3" s="41" t="s">
         <v>961</v>
-      </c>
-      <c r="N3" s="41" t="s">
-        <v>965</v>
       </c>
       <c r="O3" s="41">
         <v>30</v>
@@ -7474,16 +7485,16 @@
       <c r="H4" s="41"/>
       <c r="I4" s="41"/>
       <c r="J4" s="41" t="s">
-        <v>959</v>
+        <v>955</v>
       </c>
       <c r="K4" s="41" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
       <c r="L4" s="41" t="s">
         <v>652</v>
       </c>
       <c r="M4" s="41" t="s">
-        <v>957</v>
+        <v>953</v>
       </c>
       <c r="N4" s="41" t="s">
         <v>652</v>
@@ -7518,16 +7529,16 @@
       <c r="H5" s="41"/>
       <c r="I5" s="41"/>
       <c r="J5" s="41" t="s">
-        <v>960</v>
+        <v>956</v>
       </c>
       <c r="K5" s="41" t="s">
-        <v>962</v>
+        <v>958</v>
       </c>
       <c r="L5" s="41" t="s">
         <v>652</v>
       </c>
       <c r="M5" s="41" t="s">
-        <v>961</v>
+        <v>957</v>
       </c>
       <c r="N5" s="41" t="s">
         <v>652</v>
@@ -7570,16 +7581,16 @@
         <v>30</v>
       </c>
       <c r="J6" s="41" t="s">
-        <v>958</v>
+        <v>954</v>
       </c>
       <c r="K6" s="41" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
       <c r="L6" s="41" t="s">
         <v>652</v>
       </c>
       <c r="M6" s="41" t="s">
-        <v>957</v>
+        <v>953</v>
       </c>
       <c r="N6" s="41" t="s">
         <v>652</v>
@@ -7595,13 +7606,13 @@
     </row>
     <row r="7" spans="1:22">
       <c r="K7" s="94" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="L7" s="94"/>
       <c r="M7" s="94"/>
       <c r="N7" s="94"/>
       <c r="O7" s="91" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="P7" s="91"/>
       <c r="Q7" s="91"/>
@@ -7671,12 +7682,12 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="76.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="16.6328125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="1" max="1" width="76.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -7801,17 +7812,17 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="27" width="68.08984375"/>
-    <col min="2" max="2" customWidth="true" style="27" width="12.54296875"/>
-    <col min="3" max="3" customWidth="true" style="27" width="12.36328125"/>
-    <col min="4" max="4" customWidth="true" style="27" width="9.6328125"/>
-    <col min="5" max="5" customWidth="true" style="27" width="17.1796875"/>
-    <col min="6" max="6" customWidth="true" style="27" width="12.54296875"/>
-    <col min="7" max="10" style="27" width="8.81640625"/>
-    <col min="11" max="11" customWidth="true" style="27" width="10.6328125"/>
-    <col min="12" max="12" customWidth="true" style="27" width="12.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="27" width="15.36328125"/>
-    <col min="14" max="16384" style="27" width="8.81640625"/>
+    <col min="1" max="1" width="68.08984375" style="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" style="27" customWidth="1"/>
+    <col min="3" max="3" width="12.36328125" style="27" customWidth="1"/>
+    <col min="4" max="4" width="9.6328125" style="27" customWidth="1"/>
+    <col min="5" max="5" width="17.1796875" style="27" customWidth="1"/>
+    <col min="6" max="6" width="12.54296875" style="27" customWidth="1"/>
+    <col min="7" max="10" width="8.81640625" style="27"/>
+    <col min="11" max="11" width="10.6328125" style="27" customWidth="1"/>
+    <col min="12" max="12" width="12.1796875" style="27" customWidth="1"/>
+    <col min="13" max="13" width="15.36328125" style="27" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.81640625" style="27"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -7895,7 +7906,7 @@
       </c>
       <c r="E3" s="41"/>
       <c r="F3" s="41" t="s">
-        <v>30</v>
+        <v>1004</v>
       </c>
       <c r="G3" s="41"/>
       <c r="H3" s="41"/>
@@ -8237,8 +8248,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.54296875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -8278,11 +8289,11 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -8332,8 +8343,8 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="61.81640625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="1" max="1" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="69" customFormat="1">
@@ -8729,31 +8740,31 @@
   <dimension ref="A1:AG14"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="49.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="4.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="1" max="1" width="49.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -9532,27 +9543,27 @@
   <dimension ref="A1:AH11"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="33.0"/>
-    <col min="2" max="2" customWidth="true" width="10.453125"/>
-    <col min="6" max="6" customWidth="true" width="10.90625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.36328125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.36328125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.36328125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="19" max="19" customWidth="true" width="8.81640625"/>
-    <col min="20" max="20" customWidth="true" width="9.453125"/>
-    <col min="21" max="21" customWidth="true" width="11.08984375"/>
-    <col min="22" max="22" customWidth="true" width="9.36328125"/>
-    <col min="23" max="23" customWidth="true" width="9.453125"/>
-    <col min="24" max="24" customWidth="true" width="10.81640625"/>
-    <col min="25" max="25" customWidth="true" width="11.36328125"/>
-    <col min="26" max="26" customWidth="true" width="12.0"/>
-    <col min="27" max="27" customWidth="true" width="10.1796875"/>
-    <col min="30" max="30" customWidth="true" width="9.0"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="1" max="1" width="33" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" customWidth="1"/>
+    <col min="6" max="6" width="10.90625" customWidth="1"/>
+    <col min="12" max="12" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.81640625" customWidth="1"/>
+    <col min="20" max="20" width="9.453125" customWidth="1"/>
+    <col min="21" max="21" width="11.08984375" customWidth="1"/>
+    <col min="22" max="22" width="9.36328125" customWidth="1"/>
+    <col min="23" max="23" width="9.453125" customWidth="1"/>
+    <col min="24" max="24" width="10.81640625" customWidth="1"/>
+    <col min="25" max="25" width="11.36328125" customWidth="1"/>
+    <col min="26" max="26" width="12" customWidth="1"/>
+    <col min="27" max="27" width="10.1796875" customWidth="1"/>
+    <col min="30" max="30" width="9" customWidth="1"/>
+    <col min="34" max="34" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -10237,11 +10248,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="35.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.54296875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="1" max="1" width="35.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -10325,10 +10336,10 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -10422,10 +10433,10 @@
   <dimension ref="A1:AH5"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="46.6328125"/>
-    <col min="5" max="5" customWidth="true" width="6.1796875"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="13.36328125"/>
+    <col min="1" max="1" width="46.6328125" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" customWidth="1"/>
+    <col min="29" max="29" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="13.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -10568,16 +10579,16 @@
       <c r="U2" s="41"/>
       <c r="V2" s="41"/>
       <c r="W2" s="41" t="s">
-        <v>900</v>
+        <v>897</v>
       </c>
       <c r="X2" s="41" t="s">
-        <v>901</v>
+        <v>898</v>
       </c>
       <c r="Y2" s="41" t="s">
         <v>305</v>
       </c>
       <c r="Z2" s="41" t="s">
-        <v>902</v>
+        <v>899</v>
       </c>
       <c r="AA2" s="41" t="s">
         <v>197</v>
@@ -10586,7 +10597,7 @@
         <v>12</v>
       </c>
       <c r="AC2" s="41" t="s">
-        <v>903</v>
+        <v>900</v>
       </c>
       <c r="AD2" s="41"/>
       <c r="AE2" s="41"/>
@@ -10662,7 +10673,7 @@
         <v>5</v>
       </c>
       <c r="W3" s="41" t="s">
-        <v>911</v>
+        <v>908</v>
       </c>
       <c r="X3" s="41"/>
       <c r="Y3" s="41"/>
@@ -10670,10 +10681,10 @@
       <c r="AA3" s="41"/>
       <c r="AB3" s="41"/>
       <c r="AC3" s="41" t="s">
-        <v>912</v>
+        <v>909</v>
       </c>
       <c r="AD3" s="44" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AE3" s="41" t="s">
         <v>12</v>
@@ -10685,7 +10696,7 @@
         <v>6</v>
       </c>
       <c r="AH3" s="44" t="s">
-        <v>913</v>
+        <v>910</v>
       </c>
     </row>
     <row r="4" spans="1:34">
@@ -10724,16 +10735,16 @@
       <c r="U4" s="41"/>
       <c r="V4" s="41"/>
       <c r="W4" s="41" t="s">
-        <v>904</v>
+        <v>901</v>
       </c>
       <c r="X4" s="41" t="s">
-        <v>901</v>
+        <v>898</v>
       </c>
       <c r="Y4" s="41" t="s">
         <v>305</v>
       </c>
       <c r="Z4" s="41" t="s">
-        <v>902</v>
+        <v>899</v>
       </c>
       <c r="AA4" s="41" t="s">
         <v>197</v>
@@ -10742,7 +10753,7 @@
         <v>12</v>
       </c>
       <c r="AC4" s="41" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
       <c r="AD4" s="41"/>
       <c r="AE4" s="41"/>
@@ -10802,14 +10813,14 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="63.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="10.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="19.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="15.54296875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="8" max="9" bestFit="true" customWidth="true" width="19.453125"/>
+    <col min="1" max="1" width="63.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="19.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -10848,7 +10859,7 @@
       <c r="B2" s="41"/>
       <c r="C2" s="41"/>
       <c r="D2" s="41" t="s">
-        <v>899</v>
+        <v>896</v>
       </c>
       <c r="E2" s="41"/>
       <c r="F2" s="41"/>
@@ -10944,24 +10955,24 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.81640625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="7.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="17" max="17" customWidth="true" width="17.6328125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.6328125" customWidth="1"/>
+    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -11044,21 +11055,21 @@
       <c r="I2" s="41"/>
       <c r="J2" s="41"/>
       <c r="K2" s="41" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="L2" s="41" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="M2" s="41" t="s">
         <v>473</v>
       </c>
       <c r="N2" s="41" t="s">
-        <v>931</v>
+        <v>928</v>
       </c>
       <c r="O2" s="41"/>
       <c r="P2" s="41"/>
       <c r="Q2" s="41" t="s">
-        <v>932</v>
+        <v>929</v>
       </c>
       <c r="R2" s="41"/>
     </row>
@@ -11070,7 +11081,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="44" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D3" s="41" t="s">
         <v>12</v>
@@ -11086,16 +11097,16 @@
       <c r="I3" s="41"/>
       <c r="J3" s="41"/>
       <c r="K3" s="41" t="s">
-        <v>933</v>
+        <v>930</v>
       </c>
       <c r="L3" s="41" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
       <c r="M3" s="41" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="N3" s="41" t="s">
-        <v>935</v>
+        <v>932</v>
       </c>
       <c r="O3" s="41" t="s">
         <v>12</v>
@@ -11104,10 +11115,10 @@
         <v>13</v>
       </c>
       <c r="Q3" s="41" t="s">
-        <v>936</v>
+        <v>933</v>
       </c>
       <c r="R3" s="41" t="s">
-        <v>937</v>
+        <v>934</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -11134,16 +11145,16 @@
       <c r="I4" s="41"/>
       <c r="J4" s="41"/>
       <c r="K4" s="41" t="s">
-        <v>938</v>
+        <v>935</v>
       </c>
       <c r="L4" s="41" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="M4" s="41" t="s">
         <v>473</v>
       </c>
       <c r="N4" s="41" t="s">
-        <v>931</v>
+        <v>928</v>
       </c>
       <c r="O4" s="41" t="s">
         <v>12</v>
@@ -11152,7 +11163,7 @@
         <v>30</v>
       </c>
       <c r="Q4" s="41" t="s">
-        <v>939</v>
+        <v>936</v>
       </c>
       <c r="R4" s="41"/>
     </row>
@@ -11164,7 +11175,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="44" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D5" s="41" t="s">
         <v>12</v>
@@ -11180,16 +11191,16 @@
       <c r="I5" s="41"/>
       <c r="J5" s="41"/>
       <c r="K5" s="41" t="s">
-        <v>940</v>
+        <v>937</v>
       </c>
       <c r="L5" s="41" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
       <c r="M5" s="41" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="N5" s="41" t="s">
-        <v>935</v>
+        <v>932</v>
       </c>
       <c r="O5" s="41" t="s">
         <v>12</v>
@@ -11198,7 +11209,7 @@
         <v>13</v>
       </c>
       <c r="Q5" s="41" t="s">
-        <v>941</v>
+        <v>938</v>
       </c>
       <c r="R5" s="41"/>
     </row>
@@ -11210,7 +11221,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="44" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D6" s="41" t="s">
         <v>12</v>
@@ -11226,16 +11237,16 @@
       <c r="I6" s="41"/>
       <c r="J6" s="41"/>
       <c r="K6" s="41" t="s">
-        <v>942</v>
+        <v>939</v>
       </c>
       <c r="L6" s="41" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
       <c r="M6" s="41" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="N6" s="41" t="s">
-        <v>935</v>
+        <v>932</v>
       </c>
       <c r="O6" s="41" t="s">
         <v>12</v>
@@ -11244,7 +11255,7 @@
         <v>13</v>
       </c>
       <c r="Q6" s="41" t="s">
-        <v>943</v>
+        <v>940</v>
       </c>
       <c r="R6" s="41"/>
     </row>
@@ -11262,27 +11273,27 @@
   <dimension ref="A1:U4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="44.08984375"/>
-    <col min="2" max="2" customWidth="true" width="13.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.1796875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="6" max="6" customWidth="true" width="11.6328125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.1796875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="6.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="8.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="14.08984375"/>
+    <col min="1" max="1" width="44.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.1796875" customWidth="1"/>
+    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6328125" customWidth="1"/>
+    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -11511,8 +11522,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -11560,8 +11571,8 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="18.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="11.453125"/>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -11629,21 +11640,21 @@
   <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="27" width="24.90625"/>
-    <col min="2" max="2" customWidth="true" style="27" width="14.0"/>
-    <col min="3" max="3" customWidth="true" style="27" width="11.81640625"/>
-    <col min="4" max="4" customWidth="true" style="27" width="9.54296875"/>
-    <col min="5" max="5" customWidth="true" style="27" width="10.36328125"/>
-    <col min="6" max="6" customWidth="true" style="27" width="9.36328125"/>
-    <col min="7" max="7" customWidth="true" style="27" width="9.81640625"/>
-    <col min="8" max="8" customWidth="true" style="27" width="10.453125"/>
-    <col min="9" max="9" customWidth="true" style="27" width="8.81640625"/>
-    <col min="10" max="10" customWidth="true" style="38" width="8.08984375"/>
-    <col min="11" max="11" customWidth="true" style="27" width="10.0"/>
-    <col min="12" max="12" customWidth="true" style="27" width="7.81640625"/>
-    <col min="13" max="13" customWidth="true" style="27" width="9.0"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="27" width="19.453125"/>
-    <col min="15" max="16384" style="27" width="8.81640625"/>
+    <col min="1" max="1" width="24.90625" style="27" customWidth="1"/>
+    <col min="2" max="2" width="14" style="27" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" style="27" customWidth="1"/>
+    <col min="4" max="4" width="9.54296875" style="27" customWidth="1"/>
+    <col min="5" max="5" width="10.36328125" style="27" customWidth="1"/>
+    <col min="6" max="6" width="9.36328125" style="27" customWidth="1"/>
+    <col min="7" max="7" width="9.81640625" style="27" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" style="27" customWidth="1"/>
+    <col min="9" max="9" width="8.81640625" style="27" customWidth="1"/>
+    <col min="10" max="10" width="8.08984375" style="38" customWidth="1"/>
+    <col min="11" max="11" width="10" style="27" customWidth="1"/>
+    <col min="12" max="12" width="7.81640625" style="27" customWidth="1"/>
+    <col min="13" max="13" width="9" style="27" customWidth="1"/>
+    <col min="14" max="14" width="19.453125" style="27" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.81640625" style="27"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -12413,15 +12424,15 @@
   <dimension ref="A1:P19"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="21.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="6.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="18.453125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -12497,10 +12508,10 @@
         <v>46</v>
       </c>
       <c r="H2" s="41" t="s">
-        <v>946</v>
+        <v>943</v>
       </c>
       <c r="I2" s="41" t="s">
-        <v>947</v>
+        <v>944</v>
       </c>
       <c r="J2" s="41"/>
       <c r="K2" s="41"/>
@@ -12533,7 +12544,7 @@
         <v>46</v>
       </c>
       <c r="H3" s="41" t="s">
-        <v>950</v>
+        <v>947</v>
       </c>
       <c r="I3" s="41" t="s">
         <v>357</v>
@@ -12741,10 +12752,10 @@
       </c>
       <c r="G10" s="41"/>
       <c r="H10" s="41" t="s">
-        <v>922</v>
+        <v>919</v>
       </c>
       <c r="I10" s="41" t="s">
-        <v>923</v>
+        <v>920</v>
       </c>
       <c r="J10" s="41"/>
       <c r="K10" s="41" t="s">
@@ -12859,10 +12870,10 @@
       </c>
       <c r="G13" s="41"/>
       <c r="H13" s="41" t="s">
-        <v>914</v>
+        <v>911</v>
       </c>
       <c r="I13" s="41" t="s">
-        <v>915</v>
+        <v>912</v>
       </c>
       <c r="J13" s="44" t="s">
         <v>755</v>
@@ -12941,10 +12952,10 @@
       </c>
       <c r="G15" s="41"/>
       <c r="H15" s="41" t="s">
-        <v>916</v>
+        <v>913</v>
       </c>
       <c r="I15" s="41" t="s">
-        <v>917</v>
+        <v>914</v>
       </c>
       <c r="J15" s="44" t="s">
         <v>759</v>
@@ -12977,10 +12988,10 @@
       </c>
       <c r="G16" s="41"/>
       <c r="H16" s="41" t="s">
-        <v>918</v>
+        <v>915</v>
       </c>
       <c r="I16" s="41" t="s">
-        <v>919</v>
+        <v>916</v>
       </c>
       <c r="J16" s="44" t="s">
         <v>726</v>
@@ -13015,10 +13026,10 @@
       </c>
       <c r="G17" s="41"/>
       <c r="H17" s="41" t="s">
-        <v>920</v>
+        <v>917</v>
       </c>
       <c r="I17" s="41" t="s">
-        <v>921</v>
+        <v>918</v>
       </c>
       <c r="J17" s="44" t="s">
         <v>762</v>
@@ -13053,10 +13064,10 @@
         <v>46</v>
       </c>
       <c r="H18" s="41" t="s">
-        <v>948</v>
+        <v>945</v>
       </c>
       <c r="I18" s="41" t="s">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="J18" s="41"/>
       <c r="K18" s="41"/>
@@ -13089,10 +13100,10 @@
         <v>46</v>
       </c>
       <c r="H19" s="41" t="s">
-        <v>951</v>
+        <v>948</v>
       </c>
       <c r="I19" s="41" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
       <c r="J19" s="41"/>
       <c r="K19" s="41"/>
@@ -13116,18 +13127,18 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="4" max="4" customWidth="true" width="15.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" customWidth="true" width="15.08984375"/>
+    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" customWidth="1"/>
+    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -13319,30 +13330,30 @@
   <dimension ref="A1:W5"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="27" width="19.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="38" width="10.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="38" width="9.453125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="38" width="7.81640625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="38" width="10.90625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="38" width="9.453125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="38" width="7.81640625"/>
-    <col min="8" max="8" customWidth="true" style="27" width="13.0"/>
-    <col min="9" max="9" customWidth="true" style="27" width="16.54296875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="27" width="14.08984375"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="38" width="10.36328125"/>
-    <col min="12" max="12" customWidth="true" style="38" width="10.36328125"/>
-    <col min="13" max="13" style="27" width="8.81640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="27" width="12.54296875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="27" width="14.81640625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="27" width="13.1796875"/>
-    <col min="17" max="17" customWidth="true" style="38" width="11.54296875"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" style="38" width="8.81640625"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="27" width="9.90625"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="27" width="12.0"/>
-    <col min="21" max="21" style="27" width="8.81640625"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="27" width="10.6328125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="27" width="13.90625"/>
-    <col min="24" max="16384" style="27" width="8.81640625"/>
+    <col min="1" max="1" width="19.90625" style="27" customWidth="1"/>
+    <col min="2" max="2" width="10.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.453125" style="38" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.81640625" style="38" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" style="38" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.81640625" style="38" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" style="27" customWidth="1"/>
+    <col min="9" max="9" width="16.54296875" style="27" customWidth="1"/>
+    <col min="10" max="10" width="14.08984375" style="27" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.36328125" style="38" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.36328125" style="38" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" style="27"/>
+    <col min="14" max="14" width="12.54296875" style="27" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.81640625" style="27" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.1796875" style="27" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" style="38" customWidth="1"/>
+    <col min="18" max="18" width="8.81640625" style="38" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.90625" style="27" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12" style="27" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.81640625" style="27"/>
+    <col min="22" max="22" width="10.6328125" style="27" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.90625" style="27" bestFit="1" customWidth="1"/>
+    <col min="24" max="16384" width="8.81640625" style="27"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -13521,7 +13532,7 @@
         <v>14</v>
       </c>
       <c r="M3" s="30" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="N3" s="30"/>
       <c r="O3" s="30"/>
@@ -13535,13 +13546,13 @@
         <v>303</v>
       </c>
       <c r="U3" s="41" t="s">
+        <v>840</v>
+      </c>
+      <c r="V3" s="41" t="s">
         <v>841</v>
       </c>
-      <c r="V3" s="41" t="s">
-        <v>842</v>
-      </c>
       <c r="W3" s="41" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -13634,19 +13645,19 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="19.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="1" max="1" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -13749,20 +13760,20 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="38" width="25.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="38" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="38" width="17.36328125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="38" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="38" width="17.36328125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="38" width="4.453125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="38" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="38" width="14.1796875"/>
-    <col min="14" max="16384" style="38" width="8.90625"/>
+    <col min="1" max="1" width="25.81640625" style="38" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="38" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="38" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" style="38" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.36328125" style="38" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.453125" style="38" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="38" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.1796875" style="38" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.90625" style="38"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -13888,21 +13899,21 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="38" width="20.1796875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="38" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="38" width="17.36328125"/>
-    <col min="6" max="7" customWidth="true" style="38" width="17.36328125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="38" width="15.0"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="38" width="17.36328125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="38" width="4.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="38" width="17.36328125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="38" width="14.1796875"/>
-    <col min="16" max="16384" style="38" width="8.90625"/>
+    <col min="1" max="1" width="20.1796875" style="38" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="38" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="38" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="17.36328125" style="38" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="38" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="38" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.453125" style="38" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.36328125" style="38" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.1796875" style="38" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.90625" style="38"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -14089,22 +14100,22 @@
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="38" width="28.36328125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="3" max="3" customWidth="true" style="38" width="10.36328125"/>
-    <col min="4" max="4" customWidth="true" style="38" width="11.1796875"/>
-    <col min="5" max="5" customWidth="true" style="38" width="12.81640625"/>
-    <col min="6" max="6" customWidth="true" style="38" width="12.453125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="38" width="11.08984375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="9" max="9" customWidth="true" style="38" width="9.08984375"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="11" max="11" customWidth="true" style="38" width="11.54296875"/>
-    <col min="12" max="12" customWidth="true" style="38" width="10.81640625"/>
-    <col min="13" max="13" customWidth="true" style="38" width="12.1796875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="38" width="11.90625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="38" width="14.1796875"/>
-    <col min="16" max="16384" style="38" width="8.90625"/>
+    <col min="1" max="1" width="28.36328125" style="38" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.36328125" style="38" customWidth="1"/>
+    <col min="4" max="4" width="11.1796875" style="38" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" style="38" customWidth="1"/>
+    <col min="6" max="6" width="12.453125" style="38" customWidth="1"/>
+    <col min="7" max="7" width="11.08984375" style="38" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" style="38" customWidth="1"/>
+    <col min="10" max="10" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.54296875" style="38" customWidth="1"/>
+    <col min="12" max="12" width="10.81640625" style="38" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" style="38" customWidth="1"/>
+    <col min="14" max="14" width="11.90625" style="38" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.1796875" style="38" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.90625" style="38"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -14404,11 +14415,11 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="38" width="24.0"/>
-    <col min="2" max="2" customWidth="true" style="38" width="11.453125"/>
-    <col min="3" max="3" style="38" width="8.90625"/>
-    <col min="4" max="4" customWidth="true" style="38" width="19.6328125"/>
-    <col min="5" max="16384" style="38" width="8.90625"/>
+    <col min="1" max="1" width="24" style="38" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" style="38" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" style="38"/>
+    <col min="4" max="4" width="19.6328125" style="38" customWidth="1"/>
+    <col min="5" max="16384" width="8.90625" style="38"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -14466,12 +14477,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="38" width="32.1796875"/>
-    <col min="2" max="2" customWidth="true" style="38" width="14.0"/>
-    <col min="3" max="3" customWidth="true" style="38" width="16.6328125"/>
-    <col min="4" max="4" customWidth="true" style="38" width="17.6328125"/>
-    <col min="5" max="5" customWidth="true" style="38" width="11.81640625"/>
-    <col min="6" max="16384" style="38" width="8.90625"/>
+    <col min="1" max="1" width="32.1796875" style="38" customWidth="1"/>
+    <col min="2" max="2" width="14" style="38" customWidth="1"/>
+    <col min="3" max="3" width="16.6328125" style="38" customWidth="1"/>
+    <col min="4" max="4" width="17.6328125" style="38" customWidth="1"/>
+    <col min="5" max="5" width="11.81640625" style="38" customWidth="1"/>
+    <col min="6" max="16384" width="8.90625" style="38"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -14555,11 +14566,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="38" width="38.1796875"/>
-    <col min="2" max="2" customWidth="true" style="38" width="13.54296875"/>
-    <col min="3" max="3" customWidth="true" style="38" width="15.54296875"/>
-    <col min="4" max="4" customWidth="true" style="38" width="19.0"/>
-    <col min="5" max="16384" style="38" width="8.90625"/>
+    <col min="1" max="1" width="38.1796875" style="38" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" style="38" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" style="38" customWidth="1"/>
+    <col min="4" max="4" width="19" style="38" customWidth="1"/>
+    <col min="5" max="16384" width="8.90625" style="38"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -14682,21 +14693,21 @@
   <dimension ref="A1:N5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="38" width="30.90625"/>
-    <col min="2" max="2" customWidth="true" style="38" width="17.81640625"/>
-    <col min="3" max="3" customWidth="true" style="38" width="16.453125"/>
-    <col min="4" max="4" customWidth="true" style="38" width="16.08984375"/>
-    <col min="5" max="5" customWidth="true" style="38" width="12.0"/>
-    <col min="6" max="6" customWidth="true" style="38" width="18.08984375"/>
-    <col min="7" max="7" customWidth="true" style="38" width="15.08984375"/>
-    <col min="8" max="8" customWidth="true" style="38" width="10.453125"/>
-    <col min="9" max="9" customWidth="true" style="38" width="10.81640625"/>
-    <col min="10" max="10" style="38" width="8.90625"/>
-    <col min="11" max="11" customWidth="true" style="38" width="13.1796875"/>
-    <col min="12" max="12" customWidth="true" style="38" width="12.6328125"/>
-    <col min="13" max="13" customWidth="true" style="38" width="14.08984375"/>
-    <col min="14" max="14" customWidth="true" style="38" width="14.36328125"/>
-    <col min="15" max="16384" style="38" width="8.90625"/>
+    <col min="1" max="1" width="30.90625" style="38" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" style="38" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" style="38" customWidth="1"/>
+    <col min="4" max="4" width="16.08984375" style="38" customWidth="1"/>
+    <col min="5" max="5" width="12" style="38" customWidth="1"/>
+    <col min="6" max="6" width="18.08984375" style="38" customWidth="1"/>
+    <col min="7" max="7" width="15.08984375" style="38" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" style="38" customWidth="1"/>
+    <col min="9" max="9" width="10.81640625" style="38" customWidth="1"/>
+    <col min="10" max="10" width="8.90625" style="38"/>
+    <col min="11" max="11" width="13.1796875" style="38" customWidth="1"/>
+    <col min="12" max="12" width="12.6328125" style="38" customWidth="1"/>
+    <col min="13" max="13" width="14.08984375" style="38" customWidth="1"/>
+    <col min="14" max="14" width="14.36328125" style="38" customWidth="1"/>
+    <col min="15" max="16384" width="8.90625" style="38"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -14898,12 +14909,12 @@
   <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="16.08984375"/>
+    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -15586,11 +15597,11 @@
   <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="57.453125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="15.54296875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="4" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="20.08984375"/>
+    <col min="1" max="1" width="57.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -15621,7 +15632,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="44" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="D2" s="41" t="s">
         <v>12</v>
@@ -15779,7 +15790,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="38" t="s">
-        <v>906</v>
+        <v>903</v>
       </c>
       <c r="B13" s="38"/>
       <c r="C13" s="38"/>
@@ -15797,7 +15808,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="89" t="s">
-        <v>907</v>
+        <v>904</v>
       </c>
       <c r="B15" s="38"/>
       <c r="C15" s="38"/>
@@ -15819,28 +15830,28 @@
   <dimension ref="A1:W15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="50.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="25" width="18.36328125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="25" width="12.08984375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="25" width="15.36328125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="25" width="12.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="25" width="9.453125"/>
-    <col min="7" max="8" style="25" width="8.81640625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="8.1796875"/>
-    <col min="15" max="15" customWidth="true" style="25" width="13.0"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="10.1796875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="25" width="10.453125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" style="25" width="9.1796875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="25" width="11.6328125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
-    <col min="22" max="23" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
-    <col min="24" max="16384" style="25" width="8.81640625"/>
+    <col min="1" max="1" width="50" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.36328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.08984375" style="25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.36328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="8.81640625" style="25"/>
+    <col min="9" max="9" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13" style="25" customWidth="1"/>
+    <col min="16" max="16" width="10.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.453125" style="25" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
+    <col min="24" max="16384" width="8.81640625" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -15954,7 +15965,7 @@
       <c r="M2" s="30"/>
       <c r="N2" s="30"/>
       <c r="O2" s="30" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="P2" s="30"/>
       <c r="Q2" s="30" t="s">
@@ -16103,7 +16114,7 @@
         <v>15</v>
       </c>
       <c r="H6" s="30" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="I6" s="30" t="s">
         <v>360</v>
@@ -16152,13 +16163,13 @@
         <v>19</v>
       </c>
       <c r="H7" s="30" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="I7" s="30" t="s">
         <v>336</v>
       </c>
       <c r="J7" s="30" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="K7" s="30"/>
       <c r="L7" s="30"/>
@@ -16281,7 +16292,7 @@
       </c>
       <c r="G10" s="53"/>
       <c r="H10" s="30" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="I10" s="30"/>
       <c r="J10" s="30" t="s">
@@ -16330,7 +16341,7 @@
         <v>15</v>
       </c>
       <c r="H11" s="30" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="I11" s="30" t="s">
         <v>199</v>
@@ -16383,7 +16394,7 @@
       </c>
       <c r="G12" s="53"/>
       <c r="H12" s="30" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="I12" s="30" t="s">
         <v>349</v>
@@ -16473,7 +16484,7 @@
       </c>
       <c r="G14" s="53"/>
       <c r="H14" s="30" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="I14" s="30" t="s">
         <v>232</v>
@@ -16524,13 +16535,13 @@
         <v>15</v>
       </c>
       <c r="H15" s="30" t="s">
-        <v>944</v>
+        <v>941</v>
       </c>
       <c r="I15" s="30" t="s">
         <v>199</v>
       </c>
       <c r="J15" s="30" t="s">
-        <v>945</v>
+        <v>942</v>
       </c>
       <c r="K15" s="30"/>
       <c r="L15" s="30"/>
@@ -16560,29 +16571,29 @@
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="44.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="8.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="13.54296875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.81640625"/>
-    <col min="11" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.1796875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="8.1796875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="14.1796875"/>
-    <col min="27" max="28" bestFit="true" customWidth="true" width="12.81640625"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="14.1796875"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="12.81640625"/>
+    <col min="1" max="1" width="44.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -17014,10 +17025,10 @@
   <dimension ref="A1:AJ39"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="54.36328125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="13.81640625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="1" max="1" width="54.36328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36">
@@ -17159,10 +17170,10 @@
       <c r="P2" s="41"/>
       <c r="Q2" s="41"/>
       <c r="R2" s="41" t="s">
+        <v>864</v>
+      </c>
+      <c r="S2" s="41" t="s">
         <v>865</v>
-      </c>
-      <c r="S2" s="41" t="s">
-        <v>866</v>
       </c>
       <c r="T2" s="41"/>
       <c r="U2" s="41"/>
@@ -17226,7 +17237,7 @@
         <v>4</v>
       </c>
       <c r="O3" s="44" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="P3" s="41" t="s">
         <v>12</v>
@@ -17235,10 +17246,10 @@
         <v>13</v>
       </c>
       <c r="R3" s="41" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="S3" s="41" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="T3" s="41"/>
       <c r="U3" s="41"/>
@@ -17302,7 +17313,7 @@
         <v>4</v>
       </c>
       <c r="O4" s="44" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="P4" s="41" t="s">
         <v>12</v>
@@ -17519,10 +17530,10 @@
       <c r="P8" s="41"/>
       <c r="Q8" s="41"/>
       <c r="R8" s="41" t="s">
+        <v>866</v>
+      </c>
+      <c r="S8" s="41" t="s">
         <v>867</v>
-      </c>
-      <c r="S8" s="41" t="s">
-        <v>868</v>
       </c>
       <c r="T8" s="41">
         <v>0</v>
@@ -17581,10 +17592,10 @@
       <c r="P9" s="41"/>
       <c r="Q9" s="41"/>
       <c r="R9" s="41" t="s">
+        <v>868</v>
+      </c>
+      <c r="S9" s="41" t="s">
         <v>869</v>
-      </c>
-      <c r="S9" s="41" t="s">
-        <v>870</v>
       </c>
       <c r="T9" s="41"/>
       <c r="U9" s="41">
@@ -17647,10 +17658,10 @@
       <c r="P10" s="41"/>
       <c r="Q10" s="41"/>
       <c r="R10" s="41" t="s">
+        <v>870</v>
+      </c>
+      <c r="S10" s="41" t="s">
         <v>871</v>
-      </c>
-      <c r="S10" s="41" t="s">
-        <v>872</v>
       </c>
       <c r="T10" s="41"/>
       <c r="U10" s="41"/>
@@ -17732,7 +17743,7 @@
         <v>1</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>12</v>
@@ -17971,10 +17982,10 @@
       <c r="P16" s="41"/>
       <c r="Q16" s="41"/>
       <c r="R16" s="41" t="s">
+        <v>855</v>
+      </c>
+      <c r="S16" s="41" t="s">
         <v>856</v>
-      </c>
-      <c r="S16" s="41" t="s">
-        <v>857</v>
       </c>
       <c r="T16" s="41"/>
       <c r="U16" s="41"/>
@@ -18159,10 +18170,10 @@
         <v>30</v>
       </c>
       <c r="R19" s="41" t="s">
+        <v>872</v>
+      </c>
+      <c r="S19" s="41" t="s">
         <v>873</v>
-      </c>
-      <c r="S19" s="41" t="s">
-        <v>874</v>
       </c>
       <c r="T19" s="44">
         <v>0</v>
@@ -18192,7 +18203,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>155</v>
@@ -18237,10 +18248,10 @@
         <v>12</v>
       </c>
       <c r="R20" s="41" t="s">
+        <v>857</v>
+      </c>
+      <c r="S20" s="41" t="s">
         <v>858</v>
-      </c>
-      <c r="S20" s="41" t="s">
-        <v>859</v>
       </c>
       <c r="T20" s="44">
         <v>0</v>
@@ -18301,10 +18312,10 @@
       <c r="P21" s="41"/>
       <c r="Q21" s="41"/>
       <c r="R21" s="41" t="s">
+        <v>859</v>
+      </c>
+      <c r="S21" s="41" t="s">
         <v>860</v>
-      </c>
-      <c r="S21" s="41" t="s">
-        <v>861</v>
       </c>
       <c r="T21" s="44">
         <v>0</v>
@@ -18463,7 +18474,7 @@
       <c r="P24" s="41"/>
       <c r="Q24" s="41"/>
       <c r="R24" s="41" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="S24" s="41"/>
       <c r="T24" s="44"/>
@@ -18665,7 +18676,7 @@
       <c r="P28" s="41"/>
       <c r="Q28" s="41"/>
       <c r="R28" s="41" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="S28" s="41"/>
       <c r="T28" s="44">
@@ -18809,7 +18820,7 @@
       <c r="P30" s="41"/>
       <c r="Q30" s="41"/>
       <c r="R30" s="41" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="S30" s="41"/>
       <c r="T30" s="41">
@@ -19353,16 +19364,16 @@
   <dimension ref="A1:U17"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="53.81640625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="3" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="5" max="7" customWidth="true" width="12.1796875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="15.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="1" max="1" width="53.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="12.1796875" customWidth="1"/>
+    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -19385,7 +19396,7 @@
         <v>26</v>
       </c>
       <c r="G1" s="39" t="s">
-        <v>85</v>
+        <v>2</v>
       </c>
       <c r="H1" s="39" t="s">
         <v>3</v>
@@ -19397,7 +19408,7 @@
         <v>1</v>
       </c>
       <c r="K1" s="39" t="s">
-        <v>2</v>
+        <v>85</v>
       </c>
       <c r="L1" s="39" t="s">
         <v>3</v>
@@ -19488,27 +19499,27 @@
         <v>43</v>
       </c>
       <c r="J3" s="41"/>
-      <c r="K3" s="41" t="s">
-        <v>877</v>
-      </c>
-      <c r="L3" s="41" t="s">
-        <v>878</v>
-      </c>
-      <c r="M3" s="41" t="s">
+      <c r="K3" s="41"/>
+      <c r="L3" s="41"/>
+      <c r="M3" s="41"/>
+      <c r="N3" s="41" t="s">
+        <v>997</v>
+      </c>
+      <c r="O3" s="41" t="s">
+        <v>998</v>
+      </c>
+      <c r="P3" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="N3" s="41" t="s">
-        <v>878</v>
-      </c>
-      <c r="O3" s="41" t="s">
-        <v>12</v>
-      </c>
-      <c r="P3" s="41" t="s">
+      <c r="Q3" s="41" t="s">
+        <v>998</v>
+      </c>
+      <c r="R3" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="S3" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="Q3" s="41"/>
-      <c r="R3" s="41"/>
-      <c r="S3" s="41"/>
       <c r="T3" s="41"/>
       <c r="U3" s="41"/>
     </row>
@@ -19560,7 +19571,7 @@
         <v>252</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>823</v>
+        <v>999</v>
       </c>
       <c r="G5" s="41"/>
       <c r="H5" s="41"/>
@@ -19579,7 +19590,7 @@
         <v>14</v>
       </c>
       <c r="U5" s="44" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:21">
@@ -19630,7 +19641,7 @@
         <v>252</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>823</v>
+        <v>999</v>
       </c>
       <c r="G7" s="41"/>
       <c r="H7" s="41"/>
@@ -19727,14 +19738,10 @@
         <v>94</v>
       </c>
       <c r="B10" s="41">
-        <v>2</v>
-      </c>
-      <c r="C10" s="44" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="41" t="s">
-        <v>12</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C10" s="44"/>
+      <c r="D10" s="41"/>
       <c r="E10" s="41" t="s">
         <v>252</v>
       </c>
@@ -19742,20 +19749,44 @@
         <v>252</v>
       </c>
       <c r="G10" s="44" t="s">
-        <v>828</v>
-      </c>
-      <c r="H10" s="41"/>
-      <c r="I10" s="41"/>
-      <c r="J10" s="41"/>
-      <c r="K10" s="41"/>
-      <c r="L10" s="41"/>
-      <c r="M10" s="41"/>
-      <c r="N10" s="41"/>
-      <c r="O10" s="41"/>
-      <c r="P10" s="41"/>
-      <c r="Q10" s="41"/>
-      <c r="R10" s="41"/>
-      <c r="S10" s="41"/>
+        <v>28</v>
+      </c>
+      <c r="H10" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="J10" s="41">
+        <v>1</v>
+      </c>
+      <c r="K10" s="44" t="s">
+        <v>314</v>
+      </c>
+      <c r="L10" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="M10" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="N10" s="41" t="s">
+        <v>1000</v>
+      </c>
+      <c r="O10" s="41" t="s">
+        <v>1001</v>
+      </c>
+      <c r="P10" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q10" s="41" t="s">
+        <v>1002</v>
+      </c>
+      <c r="R10" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="S10" s="41" t="s">
+        <v>30</v>
+      </c>
       <c r="T10" s="41"/>
       <c r="U10" s="41"/>
     </row>
@@ -19764,29 +19795,37 @@
         <v>95</v>
       </c>
       <c r="B11" s="41">
-        <v>2</v>
-      </c>
-      <c r="C11" s="41" t="s">
-        <v>195</v>
-      </c>
-      <c r="D11" s="41" t="s">
-        <v>196</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C11" s="44"/>
+      <c r="D11" s="41"/>
       <c r="E11" s="41" t="s">
         <v>252</v>
       </c>
       <c r="F11" s="41" t="s">
         <v>252</v>
       </c>
-      <c r="G11" s="41" t="s">
-        <v>311</v>
-      </c>
-      <c r="H11" s="41"/>
-      <c r="I11" s="41"/>
-      <c r="J11" s="41"/>
-      <c r="K11" s="41"/>
-      <c r="L11" s="41"/>
-      <c r="M11" s="41"/>
+      <c r="G11" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="J11" s="41">
+        <v>1</v>
+      </c>
+      <c r="K11" s="44" t="s">
+        <v>314</v>
+      </c>
+      <c r="L11" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="M11" s="41" t="s">
+        <v>12</v>
+      </c>
       <c r="N11" s="41"/>
       <c r="O11" s="41"/>
       <c r="P11" s="41"/>
@@ -19803,13 +19842,15 @@
       <c r="B12" s="41">
         <v>1</v>
       </c>
-      <c r="C12" s="41" t="s">
+      <c r="C12" s="44" t="s">
         <v>307</v>
       </c>
       <c r="D12" s="41" t="s">
         <v>197</v>
       </c>
-      <c r="E12" s="41"/>
+      <c r="E12" s="44" t="s">
+        <v>822</v>
+      </c>
       <c r="F12" s="41"/>
       <c r="G12" s="41"/>
       <c r="H12" s="41"/>
@@ -19865,11 +19906,11 @@
       <c r="B14" s="41">
         <v>1</v>
       </c>
-      <c r="C14" s="41" t="s">
-        <v>307</v>
+      <c r="C14" s="44" t="s">
+        <v>1003</v>
       </c>
       <c r="D14" s="41" t="s">
-        <v>197</v>
+        <v>12</v>
       </c>
       <c r="E14" s="41"/>
       <c r="F14" s="41"/>
@@ -19896,11 +19937,11 @@
       <c r="B15" s="41">
         <v>1</v>
       </c>
-      <c r="C15" s="41" t="s">
-        <v>308</v>
+      <c r="C15" s="44" t="s">
+        <v>178</v>
       </c>
       <c r="D15" s="41" t="s">
-        <v>197</v>
+        <v>12</v>
       </c>
       <c r="E15" s="41"/>
       <c r="F15" s="41"/>
@@ -19927,13 +19968,15 @@
       <c r="B16" s="41">
         <v>1</v>
       </c>
-      <c r="C16" s="41" t="s">
-        <v>308</v>
+      <c r="C16" s="44" t="s">
+        <v>307</v>
       </c>
       <c r="D16" s="41" t="s">
         <v>197</v>
       </c>
-      <c r="E16" s="41"/>
+      <c r="E16" s="44" t="s">
+        <v>822</v>
+      </c>
       <c r="F16" s="41"/>
       <c r="G16" s="41"/>
       <c r="H16" s="41"/>
@@ -19962,13 +20005,15 @@
       <c r="B17" s="41">
         <v>1</v>
       </c>
-      <c r="C17" s="41" t="s">
-        <v>308</v>
+      <c r="C17" s="44" t="s">
+        <v>307</v>
       </c>
       <c r="D17" s="41" t="s">
         <v>197</v>
       </c>
-      <c r="E17" s="41"/>
+      <c r="E17" s="44" t="s">
+        <v>822</v>
+      </c>
       <c r="F17" s="41"/>
       <c r="G17" s="41"/>
       <c r="H17" s="41"/>

</xml_diff>

<commit_message>
Ticketing and TicketControlService updated
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4E5119-8246-4423-840E-57681BF2C7CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53CDB032-10A1-42AA-80A6-FDC132B7EF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="33" activeTab="38" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="33" activeTab="34" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3035" uniqueCount="1018">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3052" uniqueCount="1021">
   <si>
     <t>Scenario</t>
   </si>
@@ -3128,12 +3128,22 @@
   </si>
   <si>
     <t>BNZ2GN</t>
+  </si>
+  <si>
+    <t>BO3NWK</t>
+  </si>
+  <si>
+    <t>BO3NYS</t>
+  </si>
+  <si>
+    <t>BO3N0G</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="17">
     <font>
       <sz val="11"/>
@@ -3968,24 +3978,24 @@
   <dimension ref="A1:AC25"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="52.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="52.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.1796875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="11.6328125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="12.6328125"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="12.6328125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -5165,15 +5175,15 @@
   <dimension ref="A1:W36"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="54.81640625" customWidth="1"/>
-    <col min="10" max="10" width="8.81640625" style="25"/>
-    <col min="12" max="12" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="54.81640625"/>
+    <col min="10" max="10" style="25" width="8.81640625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="11.453125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="12.6328125"/>
+    <col min="22" max="23" bestFit="true" customWidth="true" width="19.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -6707,16 +6717,16 @@
   <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" style="27" customWidth="1"/>
-    <col min="4" max="4" width="29.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.81640625" customWidth="1"/>
-    <col min="6" max="6" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="11" width="14.36328125" style="27" customWidth="1"/>
-    <col min="12" max="12" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" customWidth="true" style="27" width="17.54296875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="29.81640625"/>
+    <col min="5" max="5" customWidth="true" width="13.81640625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="14.36328125"/>
+    <col min="7" max="11" customWidth="true" style="27" width="14.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.54296875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -6884,17 +6894,17 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="21.81640625" style="27" customWidth="1"/>
-    <col min="2" max="2" width="16.54296875" style="27" customWidth="1"/>
-    <col min="3" max="3" width="19.90625" style="27" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" style="27" customWidth="1"/>
-    <col min="5" max="6" width="12.90625" style="27" customWidth="1"/>
-    <col min="7" max="7" width="15" style="27" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="27" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.81640625" style="27"/>
-    <col min="10" max="10" width="17.90625" style="27" customWidth="1"/>
-    <col min="11" max="11" width="14.1796875" style="27" customWidth="1"/>
-    <col min="12" max="16384" width="8.81640625" style="27"/>
+    <col min="1" max="1" customWidth="true" style="27" width="21.81640625"/>
+    <col min="2" max="2" customWidth="true" style="27" width="16.54296875"/>
+    <col min="3" max="3" customWidth="true" style="27" width="19.90625"/>
+    <col min="4" max="4" customWidth="true" style="27" width="18.81640625"/>
+    <col min="5" max="6" customWidth="true" style="27" width="12.90625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="27" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="27" width="11.90625"/>
+    <col min="9" max="9" style="27" width="8.81640625"/>
+    <col min="10" max="10" customWidth="true" style="27" width="17.90625"/>
+    <col min="11" max="11" customWidth="true" style="27" width="14.1796875"/>
+    <col min="12" max="16384" style="27" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -7078,14 +7088,14 @@
   <dimension ref="A1:L7"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="42.1796875" style="27" customWidth="1"/>
-    <col min="2" max="2" width="15.81640625" style="27" customWidth="1"/>
-    <col min="3" max="3" width="17.81640625" style="27" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" style="27" customWidth="1"/>
-    <col min="5" max="5" width="15.6328125" style="27" customWidth="1"/>
-    <col min="6" max="11" width="8.81640625" style="27"/>
-    <col min="12" max="12" width="31" style="27" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.81640625" style="27"/>
+    <col min="1" max="1" customWidth="true" style="27" width="42.1796875"/>
+    <col min="2" max="2" customWidth="true" style="27" width="15.81640625"/>
+    <col min="3" max="3" customWidth="true" style="27" width="17.81640625"/>
+    <col min="4" max="4" customWidth="true" style="27" width="16.81640625"/>
+    <col min="5" max="5" customWidth="true" style="27" width="15.6328125"/>
+    <col min="6" max="11" style="27" width="8.81640625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="27" width="31.0"/>
+    <col min="13" max="16384" style="27" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -7301,22 +7311,22 @@
   <dimension ref="A1:V11"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="51.81640625" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.90625" customWidth="1"/>
-    <col min="14" max="14" width="12.6328125" customWidth="1"/>
-    <col min="15" max="15" width="11.453125" customWidth="1"/>
-    <col min="16" max="16" width="7.81640625" customWidth="1"/>
-    <col min="17" max="18" width="10.6328125" customWidth="1"/>
-    <col min="19" max="19" width="11.81640625" customWidth="1"/>
-    <col min="20" max="20" width="8.81640625" customWidth="1"/>
-    <col min="21" max="21" width="10.81640625" customWidth="1"/>
-    <col min="22" max="22" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="51.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="11" max="12" bestFit="true" customWidth="true" width="15.36328125"/>
+    <col min="13" max="13" customWidth="true" width="13.90625"/>
+    <col min="14" max="14" customWidth="true" width="12.6328125"/>
+    <col min="15" max="15" customWidth="true" width="11.453125"/>
+    <col min="16" max="16" customWidth="true" width="7.81640625"/>
+    <col min="17" max="18" customWidth="true" width="10.6328125"/>
+    <col min="19" max="19" customWidth="true" width="11.81640625"/>
+    <col min="20" max="20" customWidth="true" width="8.81640625"/>
+    <col min="21" max="21" customWidth="true" width="10.81640625"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -7725,12 +7735,12 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="76.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="76.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="16.6328125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="19.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -7855,17 +7865,17 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="68.08984375" style="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" style="27" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" style="27" customWidth="1"/>
-    <col min="4" max="4" width="9.6328125" style="27" customWidth="1"/>
-    <col min="5" max="5" width="17.1796875" style="27" customWidth="1"/>
-    <col min="6" max="6" width="12.54296875" style="27" customWidth="1"/>
-    <col min="7" max="10" width="8.81640625" style="27"/>
-    <col min="11" max="11" width="10.6328125" style="27" customWidth="1"/>
-    <col min="12" max="12" width="12.1796875" style="27" customWidth="1"/>
-    <col min="13" max="13" width="15.36328125" style="27" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.81640625" style="27"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="27" width="68.08984375"/>
+    <col min="2" max="2" customWidth="true" style="27" width="12.54296875"/>
+    <col min="3" max="3" customWidth="true" style="27" width="12.36328125"/>
+    <col min="4" max="4" customWidth="true" style="27" width="9.6328125"/>
+    <col min="5" max="5" customWidth="true" style="27" width="17.1796875"/>
+    <col min="6" max="6" customWidth="true" style="27" width="12.54296875"/>
+    <col min="7" max="10" style="27" width="8.81640625"/>
+    <col min="11" max="11" customWidth="true" style="27" width="10.6328125"/>
+    <col min="12" max="12" customWidth="true" style="27" width="12.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="27" width="15.36328125"/>
+    <col min="14" max="16384" style="27" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -8291,8 +8301,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.54296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -8332,11 +8342,11 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -8386,8 +8396,8 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="61.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="61.81640625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="68" customFormat="1">
@@ -8783,31 +8793,31 @@
   <dimension ref="A1:AG14"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="49.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="49.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="4.81640625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="9.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -9586,27 +9596,27 @@
   <dimension ref="A1:AH11"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="10.453125" customWidth="1"/>
-    <col min="6" max="6" width="10.90625" customWidth="1"/>
-    <col min="12" max="12" width="18.36328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.81640625" customWidth="1"/>
-    <col min="20" max="20" width="9.453125" customWidth="1"/>
-    <col min="21" max="21" width="11.08984375" customWidth="1"/>
-    <col min="22" max="22" width="9.36328125" customWidth="1"/>
-    <col min="23" max="23" width="9.453125" customWidth="1"/>
-    <col min="24" max="24" width="10.81640625" customWidth="1"/>
-    <col min="25" max="25" width="11.36328125" customWidth="1"/>
-    <col min="26" max="26" width="12" customWidth="1"/>
-    <col min="27" max="27" width="10.1796875" customWidth="1"/>
-    <col min="30" max="30" width="9" customWidth="1"/>
-    <col min="34" max="34" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="33.0"/>
+    <col min="2" max="2" customWidth="true" width="10.453125"/>
+    <col min="6" max="6" customWidth="true" width="10.90625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.36328125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.36328125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.36328125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="12.08984375"/>
+    <col min="19" max="19" customWidth="true" width="8.81640625"/>
+    <col min="20" max="20" customWidth="true" width="9.453125"/>
+    <col min="21" max="21" customWidth="true" width="11.08984375"/>
+    <col min="22" max="22" customWidth="true" width="9.36328125"/>
+    <col min="23" max="23" customWidth="true" width="9.453125"/>
+    <col min="24" max="24" customWidth="true" width="10.81640625"/>
+    <col min="25" max="25" customWidth="true" width="11.36328125"/>
+    <col min="26" max="26" customWidth="true" width="12.0"/>
+    <col min="27" max="27" customWidth="true" width="10.1796875"/>
+    <col min="30" max="30" customWidth="true" width="9.0"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="17.54296875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -10291,11 +10301,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="35.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.54296875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -10379,10 +10389,10 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.54296875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.453125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.90625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="14.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -10476,10 +10486,10 @@
   <dimension ref="A1:AH5"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="46.6328125" customWidth="1"/>
-    <col min="5" max="5" width="6.1796875" customWidth="1"/>
-    <col min="29" max="29" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="46.6328125"/>
+    <col min="5" max="5" customWidth="true" width="6.1796875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="13.36328125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -10856,14 +10866,14 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="63.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="63.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="10.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="19.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="15.54296875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="8" max="9" bestFit="true" customWidth="true" width="19.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -10998,24 +11008,24 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.6328125" customWidth="1"/>
-    <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="7.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="17" max="17" customWidth="true" width="17.6328125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="13.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -11316,27 +11326,27 @@
   <dimension ref="A1:U4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="44.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.1796875" customWidth="1"/>
-    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6328125" customWidth="1"/>
-    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="44.08984375"/>
+    <col min="2" max="2" customWidth="true" width="13.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.1796875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.1796875"/>
+    <col min="6" max="6" customWidth="true" width="11.6328125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="9.1796875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="6.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="8.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="18.6328125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="14.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -11565,8 +11575,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -11614,8 +11624,8 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="18.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="11.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -11683,21 +11693,21 @@
   <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="24.90625" style="27" customWidth="1"/>
-    <col min="2" max="2" width="14" style="27" customWidth="1"/>
-    <col min="3" max="3" width="11.81640625" style="27" customWidth="1"/>
-    <col min="4" max="4" width="9.54296875" style="27" customWidth="1"/>
-    <col min="5" max="5" width="10.36328125" style="27" customWidth="1"/>
-    <col min="6" max="6" width="9.36328125" style="27" customWidth="1"/>
-    <col min="7" max="7" width="9.81640625" style="27" customWidth="1"/>
-    <col min="8" max="8" width="10.453125" style="27" customWidth="1"/>
-    <col min="9" max="9" width="8.81640625" style="27" customWidth="1"/>
-    <col min="10" max="10" width="8.08984375" style="37" customWidth="1"/>
-    <col min="11" max="11" width="10" style="27" customWidth="1"/>
-    <col min="12" max="12" width="7.81640625" style="27" customWidth="1"/>
-    <col min="13" max="13" width="9" style="27" customWidth="1"/>
-    <col min="14" max="14" width="19.453125" style="27" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.81640625" style="27"/>
+    <col min="1" max="1" customWidth="true" style="27" width="24.90625"/>
+    <col min="2" max="2" customWidth="true" style="27" width="14.0"/>
+    <col min="3" max="3" customWidth="true" style="27" width="11.81640625"/>
+    <col min="4" max="4" customWidth="true" style="27" width="9.54296875"/>
+    <col min="5" max="5" customWidth="true" style="27" width="10.36328125"/>
+    <col min="6" max="6" customWidth="true" style="27" width="9.36328125"/>
+    <col min="7" max="7" customWidth="true" style="27" width="9.81640625"/>
+    <col min="8" max="8" customWidth="true" style="27" width="10.453125"/>
+    <col min="9" max="9" customWidth="true" style="27" width="8.81640625"/>
+    <col min="10" max="10" customWidth="true" style="37" width="8.08984375"/>
+    <col min="11" max="11" customWidth="true" style="27" width="10.0"/>
+    <col min="12" max="12" customWidth="true" style="27" width="7.81640625"/>
+    <col min="13" max="13" customWidth="true" style="27" width="9.0"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="27" width="19.453125"/>
+    <col min="15" max="16384" style="27" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -12467,15 +12477,15 @@
   <dimension ref="A1:P19"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="21.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="6.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="18.453125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -13170,18 +13180,18 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" customWidth="1"/>
-    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.08984375" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="4" max="4" customWidth="true" width="15.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="13" max="13" customWidth="true" width="15.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -13373,30 +13383,30 @@
   <dimension ref="A1:W5"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.90625" style="27" customWidth="1"/>
-    <col min="2" max="2" width="10.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.453125" style="37" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" style="37" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.81640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="27" customWidth="1"/>
-    <col min="9" max="9" width="16.54296875" style="27" customWidth="1"/>
-    <col min="10" max="10" width="14.08984375" style="27" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.36328125" style="37" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.36328125" style="37" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" style="27"/>
-    <col min="14" max="14" width="12.54296875" style="27" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.81640625" style="27" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.1796875" style="27" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" style="37" customWidth="1"/>
-    <col min="18" max="18" width="8.81640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.90625" style="27" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12" style="27" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.81640625" style="27"/>
-    <col min="22" max="22" width="10.6328125" style="27" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.90625" style="27" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="8.81640625" style="27"/>
+    <col min="1" max="1" customWidth="true" style="27" width="19.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="37" width="10.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="37" width="9.453125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="37" width="7.81640625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="37" width="10.90625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="37" width="9.453125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="37" width="7.81640625"/>
+    <col min="8" max="8" customWidth="true" style="27" width="13.0"/>
+    <col min="9" max="9" customWidth="true" style="27" width="16.54296875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="27" width="14.08984375"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="37" width="10.36328125"/>
+    <col min="12" max="12" customWidth="true" style="37" width="10.36328125"/>
+    <col min="13" max="13" style="27" width="8.81640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="27" width="12.54296875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="27" width="14.81640625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="27" width="13.1796875"/>
+    <col min="17" max="17" customWidth="true" style="37" width="11.54296875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="37" width="8.81640625"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="27" width="9.90625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="27" width="12.0"/>
+    <col min="21" max="21" style="27" width="8.81640625"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="27" width="10.6328125"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="27" width="13.90625"/>
+    <col min="24" max="16384" style="27" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -13688,19 +13698,19 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="19.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.453125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.90625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -13803,20 +13813,20 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="25.81640625" style="37" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="37" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.36328125" style="37" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" style="37" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.36328125" style="37" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.453125" style="37" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" style="37" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.1796875" style="37" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.90625" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="25.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="37" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="37" width="17.36328125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="37" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="37" width="17.36328125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="37" width="4.453125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="37" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="37" width="14.1796875"/>
+    <col min="14" max="16384" style="37" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -13942,21 +13952,21 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="20.1796875" style="37" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="37" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.36328125" style="37" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="17.36328125" style="37" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" style="37" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.36328125" style="37" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.453125" style="37" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.36328125" style="37" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.1796875" style="37" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.90625" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="20.1796875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="37" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="37" width="17.36328125"/>
+    <col min="6" max="7" customWidth="true" style="37" width="17.36328125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="37" width="15.0"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="37" width="17.36328125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="37" width="4.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="37" width="17.36328125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="37" width="14.1796875"/>
+    <col min="16" max="16384" style="37" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -14143,22 +14153,22 @@
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="28.36328125" style="37" customWidth="1"/>
-    <col min="2" max="2" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.36328125" style="37" customWidth="1"/>
-    <col min="4" max="4" width="11.1796875" style="37" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" style="37" customWidth="1"/>
-    <col min="6" max="6" width="12.453125" style="37" customWidth="1"/>
-    <col min="7" max="7" width="11.08984375" style="37" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" style="37" customWidth="1"/>
-    <col min="10" max="10" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.54296875" style="37" customWidth="1"/>
-    <col min="12" max="12" width="10.81640625" style="37" customWidth="1"/>
-    <col min="13" max="13" width="12.1796875" style="37" customWidth="1"/>
-    <col min="14" max="14" width="11.90625" style="37" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.1796875" style="37" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.90625" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="28.36328125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="3" max="3" customWidth="true" style="37" width="10.36328125"/>
+    <col min="4" max="4" customWidth="true" style="37" width="11.1796875"/>
+    <col min="5" max="5" customWidth="true" style="37" width="12.81640625"/>
+    <col min="6" max="6" customWidth="true" style="37" width="12.453125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="37" width="11.08984375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="9" max="9" customWidth="true" style="37" width="9.08984375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="37" width="11.90625"/>
+    <col min="11" max="11" customWidth="true" style="37" width="11.54296875"/>
+    <col min="12" max="12" customWidth="true" style="37" width="10.81640625"/>
+    <col min="13" max="13" customWidth="true" style="37" width="12.1796875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="37" width="12.6328125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="37" width="14.1796875"/>
+    <col min="16" max="16384" style="37" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -14277,7 +14287,7 @@
       </c>
       <c r="G4" s="40"/>
       <c r="H4" s="40" t="s">
-        <v>703</v>
+        <v>1018</v>
       </c>
       <c r="I4" s="40" t="s">
         <v>359</v>
@@ -14287,10 +14297,10 @@
       </c>
       <c r="K4" s="40"/>
       <c r="L4" s="40" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="M4" s="40" t="s">
-        <v>344</v>
+        <v>409</v>
       </c>
       <c r="N4" s="40" t="s">
         <v>352</v>
@@ -14317,7 +14327,7 @@
       </c>
       <c r="G5" s="40"/>
       <c r="H5" s="40" t="s">
-        <v>960</v>
+        <v>1019</v>
       </c>
       <c r="I5" s="40" t="s">
         <v>359</v>
@@ -14433,7 +14443,7 @@
         <v>829</v>
       </c>
       <c r="H9" s="40" t="s">
-        <v>961</v>
+        <v>1020</v>
       </c>
       <c r="I9" s="40" t="s">
         <v>359</v>
@@ -14489,11 +14499,11 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="24" style="37" customWidth="1"/>
-    <col min="2" max="2" width="11.453125" style="37" customWidth="1"/>
-    <col min="3" max="3" width="8.90625" style="37"/>
-    <col min="4" max="4" width="19.6328125" style="37" customWidth="1"/>
-    <col min="5" max="16384" width="8.90625" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="24.0"/>
+    <col min="2" max="2" customWidth="true" style="37" width="11.453125"/>
+    <col min="3" max="3" style="37" width="8.90625"/>
+    <col min="4" max="4" customWidth="true" style="37" width="19.6328125"/>
+    <col min="5" max="16384" style="37" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -14551,12 +14561,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="32.1796875" style="37" customWidth="1"/>
-    <col min="2" max="2" width="14" style="37" customWidth="1"/>
-    <col min="3" max="3" width="16.6328125" style="37" customWidth="1"/>
-    <col min="4" max="4" width="17.6328125" style="37" customWidth="1"/>
-    <col min="5" max="5" width="11.81640625" style="37" customWidth="1"/>
-    <col min="6" max="16384" width="8.90625" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="32.1796875"/>
+    <col min="2" max="2" customWidth="true" style="37" width="14.0"/>
+    <col min="3" max="3" customWidth="true" style="37" width="16.6328125"/>
+    <col min="4" max="4" customWidth="true" style="37" width="17.6328125"/>
+    <col min="5" max="5" customWidth="true" style="37" width="11.81640625"/>
+    <col min="6" max="16384" style="37" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -14640,11 +14650,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="38.1796875" style="37" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" style="37" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" style="37" customWidth="1"/>
-    <col min="4" max="4" width="19" style="37" customWidth="1"/>
-    <col min="5" max="16384" width="8.90625" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="38.1796875"/>
+    <col min="2" max="2" customWidth="true" style="37" width="13.54296875"/>
+    <col min="3" max="3" customWidth="true" style="37" width="15.54296875"/>
+    <col min="4" max="4" customWidth="true" style="37" width="19.0"/>
+    <col min="5" max="16384" style="37" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -14767,23 +14777,23 @@
   <dimension ref="A1:S5"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="30.90625" style="37" customWidth="1"/>
-    <col min="2" max="2" width="17.81640625" style="37" customWidth="1"/>
-    <col min="3" max="3" width="16.453125" style="37" customWidth="1"/>
-    <col min="4" max="4" width="16.08984375" style="37" customWidth="1"/>
-    <col min="5" max="5" width="12" style="37" customWidth="1"/>
-    <col min="6" max="6" width="18.08984375" style="37" customWidth="1"/>
-    <col min="7" max="7" width="15.08984375" style="37" customWidth="1"/>
-    <col min="8" max="8" width="10.453125" style="37" customWidth="1"/>
-    <col min="9" max="9" width="10.81640625" style="37" customWidth="1"/>
-    <col min="10" max="10" width="8.90625" style="37"/>
-    <col min="11" max="11" width="13.1796875" style="37" customWidth="1"/>
-    <col min="12" max="12" width="12.6328125" style="37" customWidth="1"/>
-    <col min="13" max="13" width="14.08984375" style="37" customWidth="1"/>
-    <col min="14" max="14" width="14.36328125" style="37" customWidth="1"/>
-    <col min="15" max="18" width="8.90625" style="37"/>
-    <col min="19" max="19" width="18.36328125" style="37" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="8.90625" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="30.90625"/>
+    <col min="2" max="2" customWidth="true" style="37" width="17.81640625"/>
+    <col min="3" max="3" customWidth="true" style="37" width="16.453125"/>
+    <col min="4" max="4" customWidth="true" style="37" width="16.08984375"/>
+    <col min="5" max="5" customWidth="true" style="37" width="12.0"/>
+    <col min="6" max="6" customWidth="true" style="37" width="18.08984375"/>
+    <col min="7" max="7" customWidth="true" style="37" width="15.08984375"/>
+    <col min="8" max="8" customWidth="true" style="37" width="10.453125"/>
+    <col min="9" max="9" customWidth="true" style="37" width="10.81640625"/>
+    <col min="10" max="10" style="37" width="8.90625"/>
+    <col min="11" max="11" customWidth="true" style="37" width="13.1796875"/>
+    <col min="12" max="12" customWidth="true" style="37" width="12.6328125"/>
+    <col min="13" max="13" customWidth="true" style="37" width="14.08984375"/>
+    <col min="14" max="14" customWidth="true" style="37" width="14.36328125"/>
+    <col min="15" max="18" style="37" width="8.90625"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="37" width="18.36328125"/>
+    <col min="20" max="16384" style="37" width="8.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -15073,12 +15083,12 @@
   <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.453125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.81640625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="16.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -15761,11 +15771,11 @@
   <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="57.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="57.453125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="15.54296875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="4" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="20.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -15994,28 +16004,28 @@
   <dimension ref="A1:W15"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="50" style="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.36328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.08984375" style="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.36328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="8.81640625" style="25"/>
-    <col min="9" max="9" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13" style="25" customWidth="1"/>
-    <col min="16" max="16" width="10.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.453125" style="25" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.1796875" style="25" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="12.6328125" style="25" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="8.81640625" style="25"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="50.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="25" width="18.36328125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="25" width="12.08984375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="25" width="15.36328125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="25" width="12.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="25" width="9.453125"/>
+    <col min="7" max="8" style="25" width="8.81640625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="8.1796875"/>
+    <col min="15" max="15" customWidth="true" style="25" width="13.0"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="10.1796875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="25" width="10.453125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="25" width="9.1796875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="25" width="11.6328125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="25" width="11.1796875"/>
+    <col min="22" max="23" bestFit="true" customWidth="true" style="25" width="12.6328125"/>
+    <col min="24" max="16384" style="25" width="8.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -16735,29 +16745,29 @@
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="44.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="44.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.453125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="13.54296875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.81640625"/>
+    <col min="11" max="12" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.1796875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="27" max="28" bestFit="true" customWidth="true" width="12.81640625"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="14.1796875"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="12.81640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -17189,10 +17199,10 @@
   <dimension ref="A1:AJ39"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="54.36328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="54.36328125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="13.90625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="13.81640625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="12.08984375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36">
@@ -19528,16 +19538,16 @@
   <dimension ref="A1:U17"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="53.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="12.1796875" customWidth="1"/>
-    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="53.81640625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="3" max="4" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="5" max="7" customWidth="true" width="12.1796875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.54296875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="12.1796875"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="15.453125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.1796875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">

</xml_diff>

<commit_message>
CreateBookingService updated by Sowmya
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B608B5E3-CC76-40A1-BC3F-9D054F7766DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B42C0889-82B7-497D-8E33-53B0B7C33811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="8" activeTab="9" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="5" activeTab="7" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3038" uniqueCount="1019">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3044" uniqueCount="1020">
   <si>
     <t>Scenario</t>
   </si>
@@ -2125,9 +2125,6 @@
     <t>382</t>
   </si>
   <si>
-    <t>BBVIQD</t>
-  </si>
-  <si>
     <t>BBVUO2</t>
   </si>
   <si>
@@ -3118,12 +3115,6 @@
     <t>BO3N0G</t>
   </si>
   <si>
-    <t>BPGSDQ</t>
-  </si>
-  <si>
-    <t>BPGSGM</t>
-  </si>
-  <si>
     <t>BPGTS5</t>
   </si>
   <si>
@@ -3131,6 +3122,18 @@
   </si>
   <si>
     <t>BPGUOF</t>
+  </si>
+  <si>
+    <t>create_booking_one_seg_telephone_ticketing_PreRequest</t>
+  </si>
+  <si>
+    <t>BPH54W</t>
+  </si>
+  <si>
+    <t>2302182903197</t>
+  </si>
+  <si>
+    <t>BPIACK</t>
   </si>
 </sst>
 </file>
@@ -4078,7 +4081,7 @@
         <v>357</v>
       </c>
       <c r="AC1" s="59" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:29">
@@ -4104,7 +4107,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="40" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="I2" s="40" t="s">
         <v>199</v>
@@ -4121,7 +4124,7 @@
       <c r="M2" s="40"/>
       <c r="N2" s="40"/>
       <c r="O2" s="40" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="P2" s="40"/>
       <c r="Q2" s="40"/>
@@ -4161,7 +4164,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="40" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="I3" s="40" t="s">
         <v>200</v>
@@ -4170,13 +4173,13 @@
         <v>199</v>
       </c>
       <c r="K3" s="40" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="L3" s="40" t="s">
         <v>199</v>
       </c>
       <c r="M3" s="40" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="N3" s="40" t="s">
         <v>199</v>
@@ -4205,7 +4208,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D4" s="40" t="s">
         <v>12</v>
@@ -4220,7 +4223,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="35" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="I4" s="35" t="s">
         <v>326</v>
@@ -4237,7 +4240,7 @@
         <v>344</v>
       </c>
       <c r="Q4" s="40" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="R4" s="40"/>
       <c r="S4" s="40"/>
@@ -4260,7 +4263,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D5" s="40" t="s">
         <v>12</v>
@@ -4275,7 +4278,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="35" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="I5" s="40" t="s">
         <v>200</v>
@@ -4284,7 +4287,7 @@
         <v>641</v>
       </c>
       <c r="K5" s="40" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="L5" s="40" t="s">
         <v>641</v>
@@ -4296,7 +4299,7 @@
         <v>344</v>
       </c>
       <c r="Q5" s="40" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="R5" s="40"/>
       <c r="S5" s="40"/>
@@ -4319,7 +4322,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D6" s="40" t="s">
         <v>12</v>
@@ -4332,7 +4335,7 @@
       </c>
       <c r="G6" s="40"/>
       <c r="H6" s="40" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="I6" s="40" t="s">
         <v>596</v>
@@ -4349,7 +4352,7 @@
         <v>344</v>
       </c>
       <c r="Q6" s="40" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="R6" s="40"/>
       <c r="S6" s="40"/>
@@ -4372,7 +4375,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D7" s="40" t="s">
         <v>12</v>
@@ -4385,7 +4388,7 @@
       </c>
       <c r="G7" s="40"/>
       <c r="H7" s="40" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="I7" s="40" t="s">
         <v>599</v>
@@ -4421,7 +4424,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D8" s="40" t="s">
         <v>12</v>
@@ -4434,7 +4437,7 @@
       </c>
       <c r="G8" s="40"/>
       <c r="H8" s="40" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="I8" s="40" t="s">
         <v>602</v>
@@ -4451,7 +4454,7 @@
         <v>344</v>
       </c>
       <c r="Q8" s="40" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="R8" s="40"/>
       <c r="S8" s="40"/>
@@ -4474,7 +4477,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D9" s="40" t="s">
         <v>12</v>
@@ -4487,7 +4490,7 @@
       </c>
       <c r="G9" s="40"/>
       <c r="H9" s="40" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="I9" s="40" t="s">
         <v>605</v>
@@ -4504,7 +4507,7 @@
         <v>344</v>
       </c>
       <c r="Q9" s="40" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="R9" s="40"/>
       <c r="S9" s="40"/>
@@ -4540,7 +4543,7 @@
       </c>
       <c r="G10" s="40"/>
       <c r="H10" s="40" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="I10" s="40" t="s">
         <v>608</v>
@@ -4557,13 +4560,13 @@
       <c r="M10" s="40"/>
       <c r="N10" s="40"/>
       <c r="O10" s="40" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="P10" s="40" t="s">
         <v>344</v>
       </c>
       <c r="Q10" s="40" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="R10" s="40"/>
       <c r="S10" s="40"/>
@@ -4579,7 +4582,7 @@
         <v>344</v>
       </c>
       <c r="AC10" s="40" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
     </row>
     <row r="11" spans="1:29">
@@ -4603,7 +4606,7 @@
       </c>
       <c r="G11" s="40"/>
       <c r="H11" s="40" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="I11" s="40" t="s">
         <v>332</v>
@@ -4711,7 +4714,7 @@
       </c>
       <c r="G13" s="40"/>
       <c r="H13" s="40" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="I13" s="40" t="s">
         <v>618</v>
@@ -4766,7 +4769,7 @@
       </c>
       <c r="G14" s="40"/>
       <c r="H14" s="40" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="I14" s="40" t="s">
         <v>623</v>
@@ -4821,7 +4824,7 @@
       </c>
       <c r="G15" s="40"/>
       <c r="H15" s="40" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="I15" s="40" t="s">
         <v>627</v>
@@ -4838,7 +4841,7 @@
         <v>344</v>
       </c>
       <c r="Q15" s="40" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="R15" s="40"/>
       <c r="S15" s="40"/>
@@ -4874,7 +4877,7 @@
       </c>
       <c r="G16" s="40"/>
       <c r="H16" s="40" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="I16" s="40" t="s">
         <v>630</v>
@@ -4923,7 +4926,7 @@
       </c>
       <c r="G17" s="40"/>
       <c r="H17" s="40" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="I17" s="40"/>
       <c r="J17" s="40"/>
@@ -4968,7 +4971,7 @@
       </c>
       <c r="G18" s="40"/>
       <c r="H18" s="40" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="I18" s="40" t="s">
         <v>20</v>
@@ -5017,7 +5020,7 @@
       </c>
       <c r="G19" s="40"/>
       <c r="H19" s="40" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="I19" s="40"/>
       <c r="J19" s="40"/>
@@ -5082,7 +5085,7 @@
       </c>
       <c r="G20" s="40"/>
       <c r="H20" s="40" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="I20" s="40"/>
       <c r="J20" s="40"/>
@@ -5128,7 +5131,7 @@
     </row>
     <row r="21" spans="1:29" ht="14.5" customHeight="1">
       <c r="P21" s="87" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="Q21" s="87"/>
     </row>
@@ -5281,7 +5284,7 @@
       </c>
       <c r="J2" s="40"/>
       <c r="K2" s="40" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="L2" s="40"/>
       <c r="M2" s="40"/>
@@ -5320,10 +5323,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="40" t="s">
+        <v>952</v>
+      </c>
+      <c r="L3" s="40" t="s">
         <v>953</v>
-      </c>
-      <c r="L3" s="40" t="s">
-        <v>954</v>
       </c>
       <c r="M3" s="40"/>
       <c r="N3" s="40"/>
@@ -5396,10 +5399,10 @@
       <c r="I5" s="40"/>
       <c r="J5" s="40"/>
       <c r="K5" s="40" t="s">
+        <v>954</v>
+      </c>
+      <c r="L5" s="40" t="s">
         <v>955</v>
-      </c>
-      <c r="L5" s="40" t="s">
-        <v>956</v>
       </c>
       <c r="M5" s="40"/>
       <c r="N5" s="40" t="s">
@@ -5445,27 +5448,27 @@
       <c r="I6" s="40"/>
       <c r="J6" s="40"/>
       <c r="K6" s="40" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="L6" s="40"/>
       <c r="M6" s="40"/>
       <c r="N6" s="40" t="s">
+        <v>777</v>
+      </c>
+      <c r="O6" s="40" t="s">
         <v>778</v>
       </c>
-      <c r="O6" s="40" t="s">
-        <v>779</v>
-      </c>
       <c r="P6" s="40" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="Q6" s="40"/>
       <c r="R6" s="40"/>
       <c r="S6" s="40"/>
       <c r="T6" s="40" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="U6" s="40" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="V6" s="40"/>
       <c r="W6" s="40"/>
@@ -5492,26 +5495,26 @@
       <c r="I7" s="40"/>
       <c r="J7" s="40"/>
       <c r="K7" s="40" t="s">
+        <v>980</v>
+      </c>
+      <c r="L7" s="40" t="s">
         <v>981</v>
-      </c>
-      <c r="L7" s="40" t="s">
-        <v>982</v>
       </c>
       <c r="M7" s="40"/>
       <c r="N7" s="40" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="O7" s="40" t="s">
         <v>237</v>
       </c>
       <c r="P7" s="40" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="Q7" s="43" t="s">
         <v>82</v>
       </c>
       <c r="R7" s="40" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="S7" s="40"/>
       <c r="T7" s="40"/>
@@ -5549,10 +5552,10 @@
       </c>
       <c r="J8" s="40"/>
       <c r="K8" s="40" t="s">
+        <v>964</v>
+      </c>
+      <c r="L8" s="40" t="s">
         <v>965</v>
-      </c>
-      <c r="L8" s="40" t="s">
-        <v>966</v>
       </c>
       <c r="M8" s="40"/>
       <c r="N8" s="40" t="s">
@@ -5592,7 +5595,7 @@
       <c r="I9" s="40"/>
       <c r="J9" s="40"/>
       <c r="K9" s="40" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="L9" s="40"/>
       <c r="M9" s="40"/>
@@ -5609,7 +5612,7 @@
       <c r="T9" s="40"/>
       <c r="U9" s="40"/>
       <c r="V9" s="40" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="W9" s="40"/>
     </row>
@@ -5635,10 +5638,10 @@
       <c r="I10" s="40"/>
       <c r="J10" s="40"/>
       <c r="K10" s="40" t="s">
+        <v>967</v>
+      </c>
+      <c r="L10" s="40" t="s">
         <v>968</v>
-      </c>
-      <c r="L10" s="40" t="s">
-        <v>969</v>
       </c>
       <c r="M10" s="40"/>
       <c r="N10" s="40"/>
@@ -5676,10 +5679,10 @@
       <c r="I11" s="40"/>
       <c r="J11" s="40"/>
       <c r="K11" s="40" t="s">
+        <v>937</v>
+      </c>
+      <c r="L11" s="40" t="s">
         <v>938</v>
-      </c>
-      <c r="L11" s="40" t="s">
-        <v>939</v>
       </c>
       <c r="M11" s="40"/>
       <c r="N11" s="40"/>
@@ -5717,10 +5720,10 @@
       <c r="I12" s="40"/>
       <c r="J12" s="40"/>
       <c r="K12" s="40" t="s">
+        <v>969</v>
+      </c>
+      <c r="L12" s="40" t="s">
         <v>970</v>
-      </c>
-      <c r="L12" s="40" t="s">
-        <v>971</v>
       </c>
       <c r="M12" s="40"/>
       <c r="N12" s="40" t="s">
@@ -5762,10 +5765,10 @@
       <c r="I13" s="40"/>
       <c r="J13" s="40"/>
       <c r="K13" s="40" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="L13" s="40" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="M13" s="40"/>
       <c r="N13" s="40" t="s">
@@ -5844,10 +5847,10 @@
       <c r="I15" s="40"/>
       <c r="J15" s="40"/>
       <c r="K15" s="40" t="s">
+        <v>973</v>
+      </c>
+      <c r="L15" s="40" t="s">
         <v>974</v>
-      </c>
-      <c r="L15" s="40" t="s">
-        <v>975</v>
       </c>
       <c r="M15" s="40"/>
       <c r="N15" s="40" t="s">
@@ -5889,7 +5892,7 @@
       <c r="I16" s="40"/>
       <c r="J16" s="40"/>
       <c r="K16" s="40" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="L16" s="40"/>
       <c r="M16" s="40"/>
@@ -5930,7 +5933,7 @@
       <c r="I17" s="40"/>
       <c r="J17" s="40"/>
       <c r="K17" s="40" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="L17" s="40"/>
       <c r="M17" s="40"/>
@@ -5975,7 +5978,7 @@
       </c>
       <c r="J18" s="40"/>
       <c r="K18" s="40" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="L18" s="40"/>
       <c r="M18" s="40"/>
@@ -5992,10 +5995,10 @@
       <c r="T18" s="40"/>
       <c r="U18" s="40"/>
       <c r="V18" s="40" t="s">
+        <v>976</v>
+      </c>
+      <c r="W18" s="40" t="s">
         <v>977</v>
-      </c>
-      <c r="W18" s="40" t="s">
-        <v>978</v>
       </c>
     </row>
     <row r="19" spans="1:23">
@@ -6020,7 +6023,7 @@
       <c r="I19" s="40"/>
       <c r="J19" s="40"/>
       <c r="K19" s="40" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="L19" s="40"/>
       <c r="M19" s="40"/>
@@ -6037,7 +6040,7 @@
       <c r="T19" s="40"/>
       <c r="U19" s="40"/>
       <c r="V19" s="40" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="W19" s="40"/>
     </row>
@@ -6063,7 +6066,7 @@
       <c r="I20" s="40"/>
       <c r="J20" s="40"/>
       <c r="K20" s="40" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="L20" s="40"/>
       <c r="M20" s="40"/>
@@ -6104,7 +6107,7 @@
       <c r="I21" s="40"/>
       <c r="J21" s="40"/>
       <c r="K21" s="40" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="L21" s="40"/>
       <c r="M21" s="40"/>
@@ -6153,7 +6156,7 @@
       </c>
       <c r="J22" s="40"/>
       <c r="K22" s="40" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="L22" s="40"/>
       <c r="M22" s="40"/>
@@ -6174,7 +6177,7 @@
     </row>
     <row r="23" spans="1:23">
       <c r="A23" s="26" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B23" s="40"/>
       <c r="C23" s="40"/>
@@ -6186,7 +6189,7 @@
       <c r="I23" s="40"/>
       <c r="J23" s="40"/>
       <c r="K23" s="40" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="L23" s="40"/>
       <c r="M23" s="40"/>
@@ -6203,7 +6206,7 @@
     </row>
     <row r="24" spans="1:23">
       <c r="A24" s="76" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B24" s="40"/>
       <c r="C24" s="40"/>
@@ -6215,7 +6218,7 @@
       <c r="I24" s="40"/>
       <c r="J24" s="40"/>
       <c r="K24" s="77" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="L24" s="40"/>
       <c r="M24" s="40"/>
@@ -6232,7 +6235,7 @@
     </row>
     <row r="25" spans="1:23">
       <c r="A25" s="40" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="B25" s="40">
         <v>2</v>
@@ -6252,10 +6255,10 @@
       <c r="I25" s="40"/>
       <c r="J25" s="40"/>
       <c r="K25" s="40" t="s">
+        <v>997</v>
+      </c>
+      <c r="L25" s="40" t="s">
         <v>998</v>
-      </c>
-      <c r="L25" s="40" t="s">
-        <v>999</v>
       </c>
       <c r="M25" s="40"/>
       <c r="N25" s="40" t="s">
@@ -6275,7 +6278,7 @@
     </row>
     <row r="26" spans="1:23">
       <c r="A26" s="78" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="B26" s="52"/>
       <c r="C26" s="40"/>
@@ -6288,7 +6291,7 @@
       <c r="J26" s="40"/>
       <c r="K26" s="40"/>
       <c r="L26" s="79" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="M26" s="40"/>
       <c r="N26" s="40"/>
@@ -6304,7 +6307,7 @@
     </row>
     <row r="27" spans="1:23">
       <c r="A27" s="78" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B27" s="52"/>
       <c r="C27" s="40"/>
@@ -6331,7 +6334,7 @@
     </row>
     <row r="28" spans="1:23">
       <c r="A28" s="50" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="B28" s="52">
         <v>2</v>
@@ -6351,7 +6354,7 @@
       <c r="I28" s="40"/>
       <c r="J28" s="40"/>
       <c r="K28" s="40" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="L28" s="40"/>
       <c r="M28" s="40"/>
@@ -6368,7 +6371,7 @@
     </row>
     <row r="29" spans="1:23">
       <c r="A29" s="50" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="B29" s="52">
         <v>0</v>
@@ -6388,15 +6391,15 @@
       <c r="I29" s="40"/>
       <c r="J29" s="40"/>
       <c r="K29" s="40" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="L29" s="40"/>
       <c r="M29" s="40"/>
       <c r="N29" s="40" t="s">
+        <v>787</v>
+      </c>
+      <c r="O29" s="40" t="s">
         <v>788</v>
-      </c>
-      <c r="O29" s="40" t="s">
-        <v>789</v>
       </c>
       <c r="P29" s="40"/>
       <c r="Q29" s="40"/>
@@ -6409,7 +6412,7 @@
     </row>
     <row r="30" spans="1:23">
       <c r="A30" s="20" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="B30" s="40">
         <v>0</v>
@@ -6429,14 +6432,14 @@
       <c r="I30" s="40"/>
       <c r="J30" s="40"/>
       <c r="K30" s="40" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="L30" s="40"/>
       <c r="M30" s="40"/>
       <c r="N30" s="40"/>
       <c r="O30" s="40"/>
       <c r="P30" s="40" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="Q30" s="40"/>
       <c r="R30" s="40"/>
@@ -6448,13 +6451,13 @@
     </row>
     <row r="31" spans="1:23">
       <c r="A31" s="86" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="B31" s="52">
         <v>1</v>
       </c>
       <c r="C31" s="43" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="D31" s="40" t="s">
         <v>43</v>
@@ -6483,13 +6486,13 @@
     </row>
     <row r="32" spans="1:23">
       <c r="A32" s="50" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B32" s="52">
         <v>0</v>
       </c>
       <c r="C32" s="43" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="D32" s="40" t="s">
         <v>12</v>
@@ -6501,7 +6504,7 @@
         <v>0</v>
       </c>
       <c r="G32" s="43" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="H32" s="40" t="s">
         <v>12</v>
@@ -6511,14 +6514,14 @@
       </c>
       <c r="J32" s="40"/>
       <c r="K32" s="40" t="s">
-        <v>1016</v>
+        <v>1013</v>
       </c>
       <c r="L32" s="40"/>
       <c r="M32" s="40"/>
       <c r="N32" s="40"/>
       <c r="O32" s="40"/>
       <c r="P32" s="40" t="s">
-        <v>1017</v>
+        <v>1014</v>
       </c>
       <c r="Q32" s="40"/>
       <c r="R32" s="40"/>
@@ -6530,13 +6533,13 @@
     </row>
     <row r="33" spans="1:23">
       <c r="A33" s="20" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="B33" s="52">
         <v>0</v>
       </c>
       <c r="C33" s="43" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D33" s="40" t="s">
         <v>12</v>
@@ -6550,7 +6553,7 @@
       <c r="I33" s="40"/>
       <c r="J33" s="40"/>
       <c r="K33" s="40" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="L33" s="40"/>
       <c r="M33" s="40"/>
@@ -6573,13 +6576,13 @@
     </row>
     <row r="34" spans="1:23">
       <c r="A34" s="50" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B34" s="52">
         <v>0</v>
       </c>
       <c r="C34" s="43" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="D34" s="40" t="s">
         <v>12</v>
@@ -6606,7 +6609,7 @@
     </row>
     <row r="35" spans="1:23">
       <c r="A35" s="50" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="B35" s="52">
         <v>1</v>
@@ -6634,7 +6637,7 @@
       </c>
       <c r="J35" s="40"/>
       <c r="K35" s="40" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="L35" s="40"/>
       <c r="M35" s="40"/>
@@ -6651,13 +6654,13 @@
     </row>
     <row r="36" spans="1:23">
       <c r="A36" s="50" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B36" s="40">
         <v>1</v>
       </c>
       <c r="C36" s="43" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D36" s="40" t="s">
         <v>13</v>
@@ -6669,7 +6672,7 @@
         <v>2</v>
       </c>
       <c r="G36" s="43" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="H36" s="40" t="s">
         <v>12</v>
@@ -6679,16 +6682,16 @@
       </c>
       <c r="J36" s="40"/>
       <c r="K36" s="40" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="L36" s="40"/>
       <c r="M36" s="40"/>
       <c r="N36" s="40"/>
       <c r="O36" s="40" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="P36" s="40" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="Q36" s="40"/>
       <c r="R36" s="40"/>
@@ -6728,7 +6731,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="38" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="C1" s="39" t="s">
         <v>70</v>
@@ -6764,7 +6767,7 @@
         <v>134</v>
       </c>
       <c r="N1" s="38" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -6775,13 +6778,13 @@
         <v>3</v>
       </c>
       <c r="C2" s="40" t="s">
+        <v>956</v>
+      </c>
+      <c r="D2" s="43" t="s">
         <v>957</v>
       </c>
-      <c r="D2" s="43" t="s">
+      <c r="E2" s="43" t="s">
         <v>958</v>
-      </c>
-      <c r="E2" s="43" t="s">
-        <v>959</v>
       </c>
       <c r="F2" s="40"/>
       <c r="G2" s="43" t="s">
@@ -6810,7 +6813,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="43" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="E3" s="43" t="s">
         <v>252</v>
@@ -6846,7 +6849,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="43" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="E4" s="40"/>
       <c r="F4" s="40" t="s">
@@ -7025,13 +7028,13 @@
         <v>12</v>
       </c>
       <c r="I5" s="40" t="s">
+        <v>896</v>
+      </c>
+      <c r="J5" s="40" t="s">
         <v>897</v>
       </c>
-      <c r="J5" s="40" t="s">
+      <c r="K5" s="40" t="s">
         <v>898</v>
-      </c>
-      <c r="K5" s="40" t="s">
-        <v>899</v>
       </c>
       <c r="L5" s="40"/>
     </row>
@@ -7061,10 +7064,10 @@
         <v>12</v>
       </c>
       <c r="I6" s="40" t="s">
+        <v>899</v>
+      </c>
+      <c r="J6" s="40" t="s">
         <v>900</v>
-      </c>
-      <c r="J6" s="40" t="s">
-        <v>901</v>
       </c>
       <c r="K6" s="40"/>
       <c r="L6" s="40"/>
@@ -7106,7 +7109,7 @@
         <v>255</v>
       </c>
       <c r="E1" s="38" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="F1" s="38" t="s">
         <v>24</v>
@@ -7235,7 +7238,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="43" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="G5" s="40"/>
       <c r="H5" s="40"/>
@@ -7243,7 +7246,7 @@
       <c r="J5" s="40"/>
       <c r="K5" s="40"/>
       <c r="L5" s="80" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -7259,7 +7262,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="43" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="G6" s="40"/>
       <c r="H6" s="40"/>
@@ -7267,7 +7270,7 @@
       <c r="J6" s="40"/>
       <c r="K6" s="40"/>
       <c r="L6" s="40" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -7283,7 +7286,7 @@
         <v>-1</v>
       </c>
       <c r="F7" s="43" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="G7" s="40"/>
       <c r="H7" s="40"/>
@@ -7355,16 +7358,16 @@
         <v>69</v>
       </c>
       <c r="K1" s="39" t="s">
+        <v>812</v>
+      </c>
+      <c r="L1" s="39" t="s">
         <v>813</v>
       </c>
-      <c r="L1" s="39" t="s">
-        <v>814</v>
-      </c>
       <c r="M1" s="39" t="s">
+        <v>808</v>
+      </c>
+      <c r="N1" s="39" t="s">
         <v>809</v>
-      </c>
-      <c r="N1" s="39" t="s">
-        <v>810</v>
       </c>
       <c r="O1" s="38" t="s">
         <v>1</v>
@@ -7420,13 +7423,13 @@
         <v>41</v>
       </c>
       <c r="J2" s="40" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="K2" s="40" t="s">
+        <v>925</v>
+      </c>
+      <c r="L2" s="40" t="s">
         <v>926</v>
-      </c>
-      <c r="L2" s="40" t="s">
-        <v>927</v>
       </c>
       <c r="M2" s="40" t="s">
         <v>642</v>
@@ -7472,19 +7475,19 @@
         <v>12</v>
       </c>
       <c r="J3" s="40" t="s">
+        <v>934</v>
+      </c>
+      <c r="K3" s="40" t="s">
+        <v>933</v>
+      </c>
+      <c r="L3" s="40" t="s">
         <v>935</v>
       </c>
-      <c r="K3" s="40" t="s">
-        <v>934</v>
-      </c>
-      <c r="L3" s="40" t="s">
+      <c r="M3" s="40" t="s">
+        <v>932</v>
+      </c>
+      <c r="N3" s="40" t="s">
         <v>936</v>
-      </c>
-      <c r="M3" s="40" t="s">
-        <v>933</v>
-      </c>
-      <c r="N3" s="40" t="s">
-        <v>937</v>
       </c>
       <c r="O3" s="40">
         <v>30</v>
@@ -7532,16 +7535,16 @@
       <c r="H4" s="40"/>
       <c r="I4" s="40"/>
       <c r="J4" s="40" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="K4" s="40" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="L4" s="40" t="s">
         <v>642</v>
       </c>
       <c r="M4" s="40" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="N4" s="40" t="s">
         <v>642</v>
@@ -7576,16 +7579,16 @@
       <c r="H5" s="40"/>
       <c r="I5" s="40"/>
       <c r="J5" s="40" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="K5" s="40" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="L5" s="40" t="s">
         <v>642</v>
       </c>
       <c r="M5" s="40" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="N5" s="40" t="s">
         <v>642</v>
@@ -7628,16 +7631,16 @@
         <v>30</v>
       </c>
       <c r="J6" s="40" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="K6" s="40" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="L6" s="40" t="s">
         <v>642</v>
       </c>
       <c r="M6" s="40" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="N6" s="40" t="s">
         <v>642</v>
@@ -7653,13 +7656,13 @@
     </row>
     <row r="7" spans="1:22">
       <c r="K7" s="91" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="L7" s="91"/>
       <c r="M7" s="91"/>
       <c r="N7" s="91"/>
       <c r="O7" s="88" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="P7" s="88"/>
       <c r="Q7" s="88"/>
@@ -7671,13 +7674,13 @@
     </row>
     <row r="8" spans="1:22">
       <c r="O8" s="89" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="P8" s="89"/>
       <c r="Q8" s="89"/>
       <c r="R8" s="89"/>
       <c r="S8" s="90" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="T8" s="90"/>
       <c r="U8" s="90"/>
@@ -7754,16 +7757,16 @@
         <v>63</v>
       </c>
       <c r="F1" s="41" t="s">
+        <v>718</v>
+      </c>
+      <c r="G1" s="41" t="s">
+        <v>712</v>
+      </c>
+      <c r="H1" s="41" t="s">
+        <v>715</v>
+      </c>
+      <c r="I1" s="41" t="s">
         <v>719</v>
-      </c>
-      <c r="G1" s="41" t="s">
-        <v>713</v>
-      </c>
-      <c r="H1" s="41" t="s">
-        <v>716</v>
-      </c>
-      <c r="I1" s="41" t="s">
-        <v>720</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -7787,7 +7790,7 @@
       </c>
       <c r="G2" s="36"/>
       <c r="H2" s="43" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="I2" s="40"/>
     </row>
@@ -7808,10 +7811,10 @@
         <v>30</v>
       </c>
       <c r="F3" s="36" t="s">
+        <v>713</v>
+      </c>
+      <c r="G3" s="66" t="s">
         <v>714</v>
-      </c>
-      <c r="G3" s="66" t="s">
-        <v>715</v>
       </c>
       <c r="H3" s="40"/>
       <c r="I3" s="40"/>
@@ -7836,13 +7839,13 @@
         <v>46</v>
       </c>
       <c r="G4" s="66" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="H4" s="43" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="I4" s="40" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
   </sheetData>
@@ -7889,7 +7892,7 @@
         <v>1</v>
       </c>
       <c r="F1" s="38" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="G1" s="38" t="s">
         <v>52</v>
@@ -7898,19 +7901,19 @@
         <v>4</v>
       </c>
       <c r="I1" s="38" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="J1" s="39" t="s">
         <v>69</v>
       </c>
       <c r="K1" s="38" t="s">
+        <v>707</v>
+      </c>
+      <c r="L1" s="38" t="s">
         <v>708</v>
       </c>
-      <c r="L1" s="38" t="s">
-        <v>709</v>
-      </c>
       <c r="M1" s="38" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -7921,7 +7924,7 @@
         <v>141</v>
       </c>
       <c r="C2" s="43" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="D2" s="40" t="s">
         <v>252</v>
@@ -7946,14 +7949,14 @@
         <v>141</v>
       </c>
       <c r="C3" s="43" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="D3" s="40" t="s">
         <v>252</v>
       </c>
       <c r="E3" s="40"/>
       <c r="F3" s="40" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="G3" s="40"/>
       <c r="H3" s="40"/>
@@ -7971,7 +7974,7 @@
         <v>141</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="D4" s="40" t="s">
         <v>252</v>
@@ -7992,7 +7995,7 @@
         <v>467</v>
       </c>
       <c r="J4" s="40" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="K4" s="40"/>
       <c r="L4" s="40"/>
@@ -8114,10 +8117,10 @@
       <c r="I9" s="40"/>
       <c r="J9" s="40"/>
       <c r="K9" s="43" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="L9" s="43" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="M9" s="40"/>
     </row>
@@ -8200,7 +8203,7 @@
         <v>141</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="D13" s="40" t="s">
         <v>252</v>
@@ -8227,7 +8230,7 @@
         <v>141</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="D14" s="40" t="s">
         <v>252</v>
@@ -8258,7 +8261,7 @@
         <v>141</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="D15" s="40" t="s">
         <v>252</v>
@@ -9037,7 +9040,7 @@
         <v>0</v>
       </c>
       <c r="K4" s="66" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="L4" s="36" t="s">
         <v>12</v>
@@ -9055,7 +9058,7 @@
         <v>12</v>
       </c>
       <c r="Q4" s="36" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="R4" s="36">
         <v>0</v>
@@ -9073,37 +9076,37 @@
         <v>0</v>
       </c>
       <c r="W4" s="66" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="X4" s="36" t="s">
         <v>12</v>
       </c>
       <c r="Y4" s="36" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="Z4" s="36">
         <v>0</v>
       </c>
       <c r="AA4" s="66" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="AB4" s="36" t="s">
         <v>12</v>
       </c>
       <c r="AC4" s="36" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="AD4" s="36">
         <v>0</v>
       </c>
       <c r="AE4" s="66" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="AF4" s="36" t="s">
         <v>12</v>
       </c>
       <c r="AG4" s="36" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="5" spans="1:33">
@@ -9807,7 +9810,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="40" t="s">
-        <v>1018</v>
+        <v>1015</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
@@ -9961,7 +9964,7 @@
         <v>1</v>
       </c>
       <c r="K5" s="40" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="L5" s="3"/>
       <c r="M5" s="3" t="s">
@@ -9971,7 +9974,7 @@
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="43" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="R5" s="15" t="s">
         <v>40</v>
@@ -10041,7 +10044,7 @@
       <c r="I6" s="40"/>
       <c r="J6" s="40"/>
       <c r="K6" s="40" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
@@ -10091,12 +10094,12 @@
       <c r="I7" s="40"/>
       <c r="J7" s="40"/>
       <c r="K7" s="40" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
       <c r="N7" s="3" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="O7" s="3"/>
       <c r="P7" s="3"/>
@@ -10191,7 +10194,7 @@
       <c r="I9" s="40"/>
       <c r="J9" s="40"/>
       <c r="K9" s="40" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>416</v>
@@ -10200,7 +10203,7 @@
         <v>304</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>197</v>
@@ -10626,16 +10629,16 @@
       <c r="U2" s="40"/>
       <c r="V2" s="40"/>
       <c r="W2" s="40" t="s">
+        <v>872</v>
+      </c>
+      <c r="X2" s="40" t="s">
         <v>873</v>
-      </c>
-      <c r="X2" s="40" t="s">
-        <v>874</v>
       </c>
       <c r="Y2" s="40" t="s">
         <v>304</v>
       </c>
       <c r="Z2" s="40" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="AA2" s="40" t="s">
         <v>197</v>
@@ -10644,7 +10647,7 @@
         <v>12</v>
       </c>
       <c r="AC2" s="40" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="AD2" s="40"/>
       <c r="AE2" s="40"/>
@@ -10720,7 +10723,7 @@
         <v>5</v>
       </c>
       <c r="W3" s="40" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="X3" s="40"/>
       <c r="Y3" s="40"/>
@@ -10728,10 +10731,10 @@
       <c r="AA3" s="40"/>
       <c r="AB3" s="40"/>
       <c r="AC3" s="40" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="AD3" s="43" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="AE3" s="40" t="s">
         <v>12</v>
@@ -10743,7 +10746,7 @@
         <v>6</v>
       </c>
       <c r="AH3" s="43" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
     </row>
     <row r="4" spans="1:34">
@@ -10782,16 +10785,16 @@
       <c r="U4" s="40"/>
       <c r="V4" s="40"/>
       <c r="W4" s="40" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="X4" s="40" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="Y4" s="40" t="s">
         <v>304</v>
       </c>
       <c r="Z4" s="40" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="AA4" s="40" t="s">
         <v>197</v>
@@ -10800,7 +10803,7 @@
         <v>12</v>
       </c>
       <c r="AC4" s="40" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="AD4" s="40"/>
       <c r="AE4" s="40"/>
@@ -10906,7 +10909,7 @@
       <c r="B2" s="40"/>
       <c r="C2" s="40"/>
       <c r="D2" s="40" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="E2" s="40"/>
       <c r="F2" s="40"/>
@@ -11102,21 +11105,21 @@
       <c r="I2" s="40"/>
       <c r="J2" s="40"/>
       <c r="K2" s="40" t="s">
+        <v>901</v>
+      </c>
+      <c r="L2" s="40" t="s">
         <v>902</v>
-      </c>
-      <c r="L2" s="40" t="s">
-        <v>903</v>
       </c>
       <c r="M2" s="40" t="s">
         <v>467</v>
       </c>
       <c r="N2" s="40" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="O2" s="40"/>
       <c r="P2" s="40"/>
       <c r="Q2" s="40" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="R2" s="40"/>
     </row>
@@ -11128,7 +11131,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="43" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="D3" s="40" t="s">
         <v>12</v>
@@ -11144,16 +11147,16 @@
       <c r="I3" s="40"/>
       <c r="J3" s="40"/>
       <c r="K3" s="40" t="s">
+        <v>905</v>
+      </c>
+      <c r="L3" s="40" t="s">
         <v>906</v>
       </c>
-      <c r="L3" s="40" t="s">
+      <c r="M3" s="40" t="s">
+        <v>810</v>
+      </c>
+      <c r="N3" s="40" t="s">
         <v>907</v>
-      </c>
-      <c r="M3" s="40" t="s">
-        <v>811</v>
-      </c>
-      <c r="N3" s="40" t="s">
-        <v>908</v>
       </c>
       <c r="O3" s="40" t="s">
         <v>12</v>
@@ -11162,10 +11165,10 @@
         <v>13</v>
       </c>
       <c r="Q3" s="40" t="s">
+        <v>908</v>
+      </c>
+      <c r="R3" s="40" t="s">
         <v>909</v>
-      </c>
-      <c r="R3" s="40" t="s">
-        <v>910</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -11192,16 +11195,16 @@
       <c r="I4" s="40"/>
       <c r="J4" s="40"/>
       <c r="K4" s="40" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="L4" s="40" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="M4" s="40" t="s">
         <v>467</v>
       </c>
       <c r="N4" s="40" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="O4" s="40" t="s">
         <v>12</v>
@@ -11210,7 +11213,7 @@
         <v>30</v>
       </c>
       <c r="Q4" s="40" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="R4" s="40"/>
     </row>
@@ -11222,7 +11225,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="D5" s="40" t="s">
         <v>12</v>
@@ -11238,16 +11241,16 @@
       <c r="I5" s="40"/>
       <c r="J5" s="40"/>
       <c r="K5" s="40" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="L5" s="40" t="s">
+        <v>906</v>
+      </c>
+      <c r="M5" s="40" t="s">
+        <v>810</v>
+      </c>
+      <c r="N5" s="40" t="s">
         <v>907</v>
-      </c>
-      <c r="M5" s="40" t="s">
-        <v>811</v>
-      </c>
-      <c r="N5" s="40" t="s">
-        <v>908</v>
       </c>
       <c r="O5" s="40" t="s">
         <v>12</v>
@@ -11256,7 +11259,7 @@
         <v>13</v>
       </c>
       <c r="Q5" s="40" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="R5" s="40"/>
     </row>
@@ -11268,7 +11271,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="D6" s="40" t="s">
         <v>12</v>
@@ -11284,16 +11287,16 @@
       <c r="I6" s="40"/>
       <c r="J6" s="40"/>
       <c r="K6" s="40" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="L6" s="40" t="s">
+        <v>906</v>
+      </c>
+      <c r="M6" s="40" t="s">
+        <v>810</v>
+      </c>
+      <c r="N6" s="40" t="s">
         <v>907</v>
-      </c>
-      <c r="M6" s="40" t="s">
-        <v>811</v>
-      </c>
-      <c r="N6" s="40" t="s">
-        <v>908</v>
       </c>
       <c r="O6" s="40" t="s">
         <v>12</v>
@@ -11302,7 +11305,7 @@
         <v>13</v>
       </c>
       <c r="Q6" s="40" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="R6" s="40"/>
     </row>
@@ -11428,7 +11431,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="43" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="H2" s="40" t="s">
         <v>154</v>
@@ -11437,7 +11440,7 @@
         <v>155</v>
       </c>
       <c r="J2" s="52" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="K2" s="40" t="s">
         <v>464</v>
@@ -11446,7 +11449,7 @@
         <v>203</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>12</v>
@@ -11461,7 +11464,7 @@
         <v>205</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>204</v>
@@ -11470,7 +11473,7 @@
         <v>155</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -11493,7 +11496,7 @@
         <v>1</v>
       </c>
       <c r="G3" s="43" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="H3" s="40" t="s">
         <v>154</v>
@@ -11502,16 +11505,16 @@
         <v>155</v>
       </c>
       <c r="J3" s="52" t="s">
+        <v>695</v>
+      </c>
+      <c r="K3" s="40" t="s">
         <v>696</v>
-      </c>
-      <c r="K3" s="40" t="s">
-        <v>697</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>153</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>12</v>
@@ -11520,13 +11523,13 @@
         <v>154</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>154</v>
@@ -11535,18 +11538,18 @@
         <v>155</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="4" spans="1:21">
       <c r="B4" s="97" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="C4" s="98"/>
       <c r="D4" s="98"/>
       <c r="E4" s="99"/>
       <c r="F4" s="97" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="G4" s="98"/>
       <c r="H4" s="98"/>
@@ -11586,7 +11589,7 @@
         <v>81</v>
       </c>
       <c r="B2" s="43" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -11594,7 +11597,7 @@
         <v>170</v>
       </c>
       <c r="B3" s="43" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -11639,7 +11642,7 @@
         <v>139</v>
       </c>
       <c r="F1" s="38" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -11671,7 +11674,7 @@
         <v>145</v>
       </c>
       <c r="F3" s="40" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
   </sheetData>
@@ -12511,10 +12514,10 @@
         <v>44</v>
       </c>
       <c r="J1" s="38" t="s">
+        <v>721</v>
+      </c>
+      <c r="K1" s="38" t="s">
         <v>722</v>
-      </c>
-      <c r="K1" s="38" t="s">
-        <v>723</v>
       </c>
       <c r="L1" s="38" t="s">
         <v>1</v>
@@ -12555,10 +12558,10 @@
         <v>46</v>
       </c>
       <c r="H2" s="40" t="s">
+        <v>918</v>
+      </c>
+      <c r="I2" s="40" t="s">
         <v>919</v>
-      </c>
-      <c r="I2" s="40" t="s">
-        <v>920</v>
       </c>
       <c r="J2" s="40"/>
       <c r="K2" s="40"/>
@@ -12591,7 +12594,7 @@
         <v>46</v>
       </c>
       <c r="H3" s="40" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="I3" s="40" t="s">
         <v>356</v>
@@ -12606,7 +12609,7 @@
     </row>
     <row r="4" spans="1:16">
       <c r="A4" s="40" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B4" s="40">
         <v>0</v>
@@ -12623,7 +12626,7 @@
       <c r="H4" s="40"/>
       <c r="I4" s="40"/>
       <c r="J4" s="43" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K4" s="40"/>
       <c r="L4" s="40"/>
@@ -12634,7 +12637,7 @@
     </row>
     <row r="5" spans="1:16">
       <c r="A5" s="40" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B5" s="40">
         <v>1</v>
@@ -12651,7 +12654,7 @@
       <c r="H5" s="40"/>
       <c r="I5" s="40"/>
       <c r="J5" s="43" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="K5" s="40"/>
       <c r="L5" s="40"/>
@@ -12662,7 +12665,7 @@
     </row>
     <row r="6" spans="1:16">
       <c r="A6" s="40" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="B6" s="40">
         <v>1</v>
@@ -12679,7 +12682,7 @@
       <c r="H6" s="40"/>
       <c r="I6" s="40"/>
       <c r="J6" s="43" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="K6" s="40"/>
       <c r="L6" s="40"/>
@@ -12690,7 +12693,7 @@
     </row>
     <row r="7" spans="1:16">
       <c r="A7" s="40" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B7" s="40">
         <v>1</v>
@@ -12716,7 +12719,7 @@
     </row>
     <row r="8" spans="1:16">
       <c r="A8" s="40" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B8" s="40">
         <v>1</v>
@@ -12733,7 +12736,7 @@
       <c r="H8" s="40"/>
       <c r="I8" s="40"/>
       <c r="J8" s="43" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="K8" s="40"/>
       <c r="L8" s="40"/>
@@ -12744,7 +12747,7 @@
     </row>
     <row r="9" spans="1:16">
       <c r="A9" s="40" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="B9" s="40">
         <v>1</v>
@@ -12763,14 +12766,14 @@
       </c>
       <c r="G9" s="40"/>
       <c r="H9" s="40" t="s">
+        <v>768</v>
+      </c>
+      <c r="I9" s="40" t="s">
         <v>769</v>
-      </c>
-      <c r="I9" s="40" t="s">
-        <v>770</v>
       </c>
       <c r="J9" s="40"/>
       <c r="K9" s="40" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="L9" s="40"/>
       <c r="M9" s="40"/>
@@ -12780,7 +12783,7 @@
     </row>
     <row r="10" spans="1:16">
       <c r="A10" s="40" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="B10" s="40">
         <v>1</v>
@@ -12799,14 +12802,14 @@
       </c>
       <c r="G10" s="40"/>
       <c r="H10" s="40" t="s">
+        <v>894</v>
+      </c>
+      <c r="I10" s="40" t="s">
         <v>895</v>
-      </c>
-      <c r="I10" s="40" t="s">
-        <v>896</v>
       </c>
       <c r="J10" s="40"/>
       <c r="K10" s="40" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="L10" s="40"/>
       <c r="M10" s="40"/>
@@ -12816,7 +12819,7 @@
     </row>
     <row r="11" spans="1:16">
       <c r="A11" s="50" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B11" s="40">
         <v>1</v>
@@ -12835,10 +12838,10 @@
       </c>
       <c r="G11" s="40"/>
       <c r="H11" s="40" t="s">
+        <v>770</v>
+      </c>
+      <c r="I11" s="40" t="s">
         <v>771</v>
-      </c>
-      <c r="I11" s="40" t="s">
-        <v>772</v>
       </c>
       <c r="J11" s="40"/>
       <c r="K11" s="43" t="s">
@@ -12852,7 +12855,7 @@
     </row>
     <row r="12" spans="1:16">
       <c r="A12" s="50" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="B12" s="40">
         <v>1</v>
@@ -12871,13 +12874,13 @@
       </c>
       <c r="G12" s="40"/>
       <c r="H12" s="40" t="s">
+        <v>772</v>
+      </c>
+      <c r="I12" s="40" t="s">
         <v>773</v>
       </c>
-      <c r="I12" s="40" t="s">
-        <v>774</v>
-      </c>
       <c r="J12" s="43" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="K12" s="40"/>
       <c r="L12" s="40">
@@ -12898,7 +12901,7 @@
     </row>
     <row r="13" spans="1:16">
       <c r="A13" s="50" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="B13" s="40">
         <v>1</v>
@@ -12917,13 +12920,13 @@
       </c>
       <c r="G13" s="40"/>
       <c r="H13" s="40" t="s">
+        <v>886</v>
+      </c>
+      <c r="I13" s="40" t="s">
         <v>887</v>
       </c>
-      <c r="I13" s="40" t="s">
-        <v>888</v>
-      </c>
       <c r="J13" s="43" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="K13" s="40"/>
       <c r="L13" s="40"/>
@@ -12934,7 +12937,7 @@
     </row>
     <row r="14" spans="1:16">
       <c r="A14" s="50" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="B14" s="40">
         <v>1</v>
@@ -12953,13 +12956,13 @@
       </c>
       <c r="G14" s="40"/>
       <c r="H14" s="40" t="s">
+        <v>774</v>
+      </c>
+      <c r="I14" s="40" t="s">
         <v>775</v>
       </c>
-      <c r="I14" s="40" t="s">
-        <v>776</v>
-      </c>
       <c r="J14" s="43" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="K14" s="40"/>
       <c r="L14" s="40">
@@ -12980,7 +12983,7 @@
     </row>
     <row r="15" spans="1:16">
       <c r="A15" s="50" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="B15" s="40">
         <v>1</v>
@@ -12999,13 +13002,13 @@
       </c>
       <c r="G15" s="40"/>
       <c r="H15" s="40" t="s">
+        <v>888</v>
+      </c>
+      <c r="I15" s="40" t="s">
         <v>889</v>
       </c>
-      <c r="I15" s="40" t="s">
-        <v>890</v>
-      </c>
       <c r="J15" s="43" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="K15" s="40"/>
       <c r="L15" s="40"/>
@@ -13016,7 +13019,7 @@
     </row>
     <row r="16" spans="1:16">
       <c r="A16" s="50" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="B16" s="40">
         <v>1</v>
@@ -13035,16 +13038,16 @@
       </c>
       <c r="G16" s="40"/>
       <c r="H16" s="40" t="s">
+        <v>890</v>
+      </c>
+      <c r="I16" s="40" t="s">
         <v>891</v>
       </c>
-      <c r="I16" s="40" t="s">
-        <v>892</v>
-      </c>
       <c r="J16" s="43" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="K16" s="40" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="L16" s="40"/>
       <c r="M16" s="40"/>
@@ -13054,7 +13057,7 @@
     </row>
     <row r="17" spans="1:16">
       <c r="A17" s="50" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B17" s="40">
         <v>1</v>
@@ -13073,13 +13076,13 @@
       </c>
       <c r="G17" s="40"/>
       <c r="H17" s="40" t="s">
+        <v>892</v>
+      </c>
+      <c r="I17" s="40" t="s">
         <v>893</v>
       </c>
-      <c r="I17" s="40" t="s">
-        <v>894</v>
-      </c>
       <c r="J17" s="43" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="K17" s="40"/>
       <c r="L17" s="40"/>
@@ -13090,7 +13093,7 @@
     </row>
     <row r="18" spans="1:16">
       <c r="A18" s="75" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="B18" s="40">
         <v>0</v>
@@ -13111,10 +13114,10 @@
         <v>46</v>
       </c>
       <c r="H18" s="40" t="s">
+        <v>920</v>
+      </c>
+      <c r="I18" s="40" t="s">
         <v>921</v>
-      </c>
-      <c r="I18" s="40" t="s">
-        <v>922</v>
       </c>
       <c r="J18" s="40"/>
       <c r="K18" s="40"/>
@@ -13126,7 +13129,7 @@
     </row>
     <row r="19" spans="1:16">
       <c r="A19" s="75" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="B19" s="40">
         <v>0</v>
@@ -13147,10 +13150,10 @@
         <v>46</v>
       </c>
       <c r="H19" s="40" t="s">
+        <v>923</v>
+      </c>
+      <c r="I19" s="40" t="s">
         <v>924</v>
-      </c>
-      <c r="I19" s="40" t="s">
-        <v>925</v>
       </c>
       <c r="J19" s="40"/>
       <c r="K19" s="40"/>
@@ -13579,7 +13582,7 @@
         <v>14</v>
       </c>
       <c r="M3" s="30" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="N3" s="30"/>
       <c r="O3" s="30"/>
@@ -13587,19 +13590,19 @@
       <c r="Q3" s="40"/>
       <c r="R3" s="40"/>
       <c r="S3" s="43" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="T3" s="30" t="s">
         <v>302</v>
       </c>
       <c r="U3" s="40" t="s">
+        <v>815</v>
+      </c>
+      <c r="V3" s="40" t="s">
         <v>816</v>
       </c>
-      <c r="V3" s="40" t="s">
-        <v>817</v>
-      </c>
       <c r="W3" s="40" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -13640,7 +13643,7 @@
         <v>14</v>
       </c>
       <c r="M4" s="30" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="N4" s="30"/>
       <c r="O4" s="30"/>
@@ -13649,15 +13652,15 @@
         <v>42</v>
       </c>
       <c r="R4" s="40" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="S4" s="30"/>
       <c r="T4" s="30"/>
       <c r="U4" s="40" t="s">
+        <v>749</v>
+      </c>
+      <c r="V4" s="40" t="s">
         <v>750</v>
-      </c>
-      <c r="V4" s="40" t="s">
-        <v>751</v>
       </c>
       <c r="W4" s="40" t="s">
         <v>356</v>
@@ -13665,12 +13668,12 @@
     </row>
     <row r="5" spans="1:23">
       <c r="B5" s="100" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="C5" s="100"/>
       <c r="D5" s="100"/>
       <c r="E5" s="101" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="F5" s="101"/>
       <c r="G5" s="101"/>
@@ -14281,7 +14284,7 @@
       </c>
       <c r="G4" s="40"/>
       <c r="H4" s="40" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="I4" s="40" t="s">
         <v>359</v>
@@ -14321,7 +14324,7 @@
       </c>
       <c r="G5" s="40"/>
       <c r="H5" s="40" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="I5" s="40" t="s">
         <v>359</v>
@@ -14434,10 +14437,10 @@
         <v>14</v>
       </c>
       <c r="G9" s="43" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="H9" s="40" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="I9" s="40" t="s">
         <v>359</v>
@@ -14530,7 +14533,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="40" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="B3" s="43" t="s">
         <v>328</v>
@@ -14878,7 +14881,7 @@
         <v>200</v>
       </c>
       <c r="J2" s="40" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="K2" s="40">
         <f>B2</f>
@@ -14924,13 +14927,13 @@
         <v>204</v>
       </c>
       <c r="H3" s="40" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="I3" s="40" t="s">
         <v>20</v>
       </c>
       <c r="J3" s="40" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="K3" s="40"/>
       <c r="L3" s="40" t="s">
@@ -14966,7 +14969,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="D4" s="40" t="s">
         <v>12</v>
@@ -14984,10 +14987,10 @@
         <v>199</v>
       </c>
       <c r="I4" s="40" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="J4" s="40" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="K4" s="40"/>
       <c r="L4" s="40" t="s">
@@ -15030,13 +15033,13 @@
         <v>204</v>
       </c>
       <c r="H5" s="40" t="s">
+        <v>1007</v>
+      </c>
+      <c r="I5" s="40" t="s">
         <v>1008</v>
       </c>
-      <c r="I5" s="40" t="s">
+      <c r="J5" s="40" t="s">
         <v>1009</v>
-      </c>
-      <c r="J5" s="40" t="s">
-        <v>1010</v>
       </c>
       <c r="K5" s="40"/>
       <c r="L5" s="40" t="s">
@@ -15800,7 +15803,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="43" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="D2" s="40" t="s">
         <v>12</v>
@@ -15958,7 +15961,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="37" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B13" s="37"/>
       <c r="C13" s="37"/>
@@ -15976,7 +15979,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="85" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B15" s="37"/>
       <c r="C15" s="37"/>
@@ -16133,7 +16136,7 @@
       <c r="M2" s="30"/>
       <c r="N2" s="30"/>
       <c r="O2" s="30" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="P2" s="30"/>
       <c r="Q2" s="30" t="s">
@@ -16282,7 +16285,7 @@
         <v>15</v>
       </c>
       <c r="H6" s="30" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="I6" s="30" t="s">
         <v>359</v>
@@ -16331,13 +16334,13 @@
         <v>19</v>
       </c>
       <c r="H7" s="30" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="I7" s="30" t="s">
         <v>335</v>
       </c>
       <c r="J7" s="30" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="K7" s="30"/>
       <c r="L7" s="30"/>
@@ -16460,7 +16463,7 @@
       </c>
       <c r="G10" s="52"/>
       <c r="H10" s="30" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="I10" s="30"/>
       <c r="J10" s="30" t="s">
@@ -16509,7 +16512,7 @@
         <v>15</v>
       </c>
       <c r="H11" s="30" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="I11" s="30" t="s">
         <v>199</v>
@@ -16562,7 +16565,7 @@
       </c>
       <c r="G12" s="52"/>
       <c r="H12" s="30" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="I12" s="30" t="s">
         <v>348</v>
@@ -16652,7 +16655,7 @@
       </c>
       <c r="G14" s="52"/>
       <c r="H14" s="30" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="I14" s="30" t="s">
         <v>232</v>
@@ -16703,13 +16706,13 @@
         <v>15</v>
       </c>
       <c r="H15" s="30" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="I15" s="30" t="s">
         <v>199</v>
       </c>
       <c r="J15" s="30" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="K15" s="30"/>
       <c r="L15" s="30"/>
@@ -17190,7 +17193,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:AJ39"/>
+  <dimension ref="A1:AJ40"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="54.36328125"/>
@@ -17338,10 +17341,10 @@
       <c r="P2" s="40"/>
       <c r="Q2" s="40"/>
       <c r="R2" s="40" t="s">
+        <v>839</v>
+      </c>
+      <c r="S2" s="40" t="s">
         <v>840</v>
-      </c>
-      <c r="S2" s="40" t="s">
-        <v>841</v>
       </c>
       <c r="T2" s="40"/>
       <c r="U2" s="40"/>
@@ -17405,7 +17408,7 @@
         <v>4</v>
       </c>
       <c r="O3" s="43" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="P3" s="40" t="s">
         <v>12</v>
@@ -17414,10 +17417,10 @@
         <v>13</v>
       </c>
       <c r="R3" s="40" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="S3" s="40" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="T3" s="40"/>
       <c r="U3" s="40"/>
@@ -17481,7 +17484,7 @@
         <v>4</v>
       </c>
       <c r="O4" s="43" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="P4" s="40" t="s">
         <v>12</v>
@@ -17698,10 +17701,10 @@
       <c r="P8" s="40"/>
       <c r="Q8" s="40"/>
       <c r="R8" s="40" t="s">
+        <v>841</v>
+      </c>
+      <c r="S8" s="40" t="s">
         <v>842</v>
-      </c>
-      <c r="S8" s="40" t="s">
-        <v>843</v>
       </c>
       <c r="T8" s="40">
         <v>0</v>
@@ -17760,10 +17763,10 @@
       <c r="P9" s="40"/>
       <c r="Q9" s="40"/>
       <c r="R9" s="40" t="s">
+        <v>843</v>
+      </c>
+      <c r="S9" s="40" t="s">
         <v>844</v>
-      </c>
-      <c r="S9" s="40" t="s">
-        <v>845</v>
       </c>
       <c r="T9" s="40"/>
       <c r="U9" s="40">
@@ -17826,10 +17829,10 @@
       <c r="P10" s="40"/>
       <c r="Q10" s="40"/>
       <c r="R10" s="40" t="s">
+        <v>845</v>
+      </c>
+      <c r="S10" s="40" t="s">
         <v>846</v>
-      </c>
-      <c r="S10" s="40" t="s">
-        <v>847</v>
       </c>
       <c r="T10" s="40"/>
       <c r="U10" s="40"/>
@@ -17911,7 +17914,7 @@
         <v>1</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>12</v>
@@ -18150,10 +18153,10 @@
       <c r="P16" s="40"/>
       <c r="Q16" s="40"/>
       <c r="R16" s="40" t="s">
+        <v>830</v>
+      </c>
+      <c r="S16" s="40" t="s">
         <v>831</v>
-      </c>
-      <c r="S16" s="40" t="s">
-        <v>832</v>
       </c>
       <c r="T16" s="40"/>
       <c r="U16" s="40"/>
@@ -18338,10 +18341,10 @@
         <v>30</v>
       </c>
       <c r="R19" s="40" t="s">
+        <v>847</v>
+      </c>
+      <c r="S19" s="40" t="s">
         <v>848</v>
-      </c>
-      <c r="S19" s="40" t="s">
-        <v>849</v>
       </c>
       <c r="T19" s="43">
         <v>0</v>
@@ -18371,7 +18374,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>155</v>
@@ -18416,10 +18419,10 @@
         <v>12</v>
       </c>
       <c r="R20" s="40" t="s">
+        <v>832</v>
+      </c>
+      <c r="S20" s="40" t="s">
         <v>833</v>
-      </c>
-      <c r="S20" s="40" t="s">
-        <v>834</v>
       </c>
       <c r="T20" s="43">
         <v>0</v>
@@ -18480,10 +18483,10 @@
       <c r="P21" s="40"/>
       <c r="Q21" s="40"/>
       <c r="R21" s="40" t="s">
+        <v>834</v>
+      </c>
+      <c r="S21" s="40" t="s">
         <v>835</v>
-      </c>
-      <c r="S21" s="40" t="s">
-        <v>836</v>
       </c>
       <c r="T21" s="43">
         <v>0</v>
@@ -18642,7 +18645,7 @@
       <c r="P24" s="40"/>
       <c r="Q24" s="40"/>
       <c r="R24" s="40" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="S24" s="40"/>
       <c r="T24" s="43"/>
@@ -18844,7 +18847,7 @@
       <c r="P28" s="40"/>
       <c r="Q28" s="40"/>
       <c r="R28" s="40" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="S28" s="40"/>
       <c r="T28" s="43">
@@ -18988,7 +18991,7 @@
       <c r="P30" s="40"/>
       <c r="Q30" s="40"/>
       <c r="R30" s="40" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="S30" s="40"/>
       <c r="T30" s="40">
@@ -19494,7 +19497,7 @@
       <c r="P39" s="40"/>
       <c r="Q39" s="40"/>
       <c r="R39" s="40" t="s">
-        <v>578</v>
+        <v>1019</v>
       </c>
       <c r="S39" s="40" t="s">
         <v>356</v>
@@ -19518,6 +19521,58 @@
       <c r="AH39" s="40"/>
       <c r="AI39" s="40"/>
       <c r="AJ39" s="40"/>
+    </row>
+    <row r="40" spans="1:36">
+      <c r="A40" s="63" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B40" s="65">
+        <v>1</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>568</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F40" s="40"/>
+      <c r="G40" s="40"/>
+      <c r="H40" s="40"/>
+      <c r="I40" s="40"/>
+      <c r="J40" s="40"/>
+      <c r="K40" s="40"/>
+      <c r="L40" s="40"/>
+      <c r="M40" s="40"/>
+      <c r="N40" s="40"/>
+      <c r="O40" s="40"/>
+      <c r="P40" s="40"/>
+      <c r="Q40" s="40"/>
+      <c r="R40" s="40" t="s">
+        <v>1017</v>
+      </c>
+      <c r="S40" s="40" t="s">
+        <v>1018</v>
+      </c>
+      <c r="T40" s="40"/>
+      <c r="U40" s="40"/>
+      <c r="V40" s="40"/>
+      <c r="W40" s="40"/>
+      <c r="X40" s="40"/>
+      <c r="Y40" s="40"/>
+      <c r="Z40" s="40"/>
+      <c r="AA40" s="40"/>
+      <c r="AB40" s="40"/>
+      <c r="AC40" s="40"/>
+      <c r="AD40" s="40"/>
+      <c r="AE40" s="40"/>
+      <c r="AF40" s="40"/>
+      <c r="AG40" s="40"/>
+      <c r="AH40" s="40"/>
+      <c r="AI40" s="40"/>
+      <c r="AJ40" s="40"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19603,10 +19658,10 @@
         <v>4</v>
       </c>
       <c r="T1" s="38" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="U1" s="38" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="2" spans="1:21">
@@ -19623,7 +19678,7 @@
         <v>12</v>
       </c>
       <c r="E2" s="43" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="F2" s="40"/>
       <c r="G2" s="40"/>
@@ -19656,7 +19711,7 @@
         <v>12</v>
       </c>
       <c r="E3" s="43" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="F3" s="40"/>
       <c r="G3" s="40"/>
@@ -19671,16 +19726,16 @@
       <c r="L3" s="40"/>
       <c r="M3" s="40"/>
       <c r="N3" s="40" t="s">
+        <v>944</v>
+      </c>
+      <c r="O3" s="40" t="s">
         <v>945</v>
-      </c>
-      <c r="O3" s="40" t="s">
-        <v>946</v>
       </c>
       <c r="P3" s="40" t="s">
         <v>42</v>
       </c>
       <c r="Q3" s="40" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="R3" s="40" t="s">
         <v>12</v>
@@ -19739,7 +19794,7 @@
         <v>252</v>
       </c>
       <c r="F5" s="40" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="G5" s="40"/>
       <c r="H5" s="40"/>
@@ -19809,7 +19864,7 @@
         <v>252</v>
       </c>
       <c r="F7" s="40" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="G7" s="40"/>
       <c r="H7" s="40"/>
@@ -19848,7 +19903,7 @@
         <v>252</v>
       </c>
       <c r="F8" s="40" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="G8" s="40"/>
       <c r="H8" s="40"/>
@@ -19883,7 +19938,7 @@
         <v>252</v>
       </c>
       <c r="F9" s="40" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="G9" s="40"/>
       <c r="H9" s="40"/>
@@ -19938,16 +19993,16 @@
         <v>12</v>
       </c>
       <c r="N10" s="40" t="s">
+        <v>947</v>
+      </c>
+      <c r="O10" s="40" t="s">
         <v>948</v>
-      </c>
-      <c r="O10" s="40" t="s">
-        <v>949</v>
       </c>
       <c r="P10" s="40" t="s">
         <v>28</v>
       </c>
       <c r="Q10" s="40" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="R10" s="40" t="s">
         <v>12</v>
@@ -20017,7 +20072,7 @@
         <v>197</v>
       </c>
       <c r="E12" s="43" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="F12" s="40"/>
       <c r="G12" s="40"/>
@@ -20075,7 +20130,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="D14" s="40" t="s">
         <v>12</v>
@@ -20143,7 +20198,7 @@
         <v>197</v>
       </c>
       <c r="E16" s="43" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="F16" s="40"/>
       <c r="G16" s="40"/>
@@ -20163,7 +20218,7 @@
         <v>14</v>
       </c>
       <c r="U16" s="43" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="17" spans="1:21">
@@ -20180,7 +20235,7 @@
         <v>197</v>
       </c>
       <c r="E17" s="43" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="F17" s="40"/>
       <c r="G17" s="40"/>
@@ -20200,7 +20255,7 @@
         <v>14</v>
       </c>
       <c r="U17" s="43" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates taken from Sowmya and Harshitha
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{689D8FB2-7816-4C30-B468-AC07E22FEDE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E4EF2BE-C2F1-471C-A590-1A91254B5F97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="26" activeTab="27" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="25" activeTab="25" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4276" uniqueCount="1236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4297" uniqueCount="1243">
   <si>
     <t>Scenario</t>
   </si>
@@ -3782,6 +3782,27 @@
   </si>
   <si>
     <t>Error - CATEGORY DOES NOT EXIST</t>
+  </si>
+  <si>
+    <t>2302183453838</t>
+  </si>
+  <si>
+    <t>BL4WAH</t>
+  </si>
+  <si>
+    <t>Missing Validating Airline code in RedirectControl request.</t>
+  </si>
+  <si>
+    <t>Missing the ticket document number in the RequestControl request.</t>
+  </si>
+  <si>
+    <t>BLZID4</t>
+  </si>
+  <si>
+    <t>434</t>
+  </si>
+  <si>
+    <t>A booking with two passengers and two tickets. Get control of one cuopon for each ticket within the same PNR</t>
   </si>
 </sst>
 </file>
@@ -4150,7 +4171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -4236,9 +4257,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -4335,6 +4353,19 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4380,19 +4411,6 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4779,10 +4797,10 @@
       <c r="O1" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="P1" s="59" t="s">
+      <c r="P1" s="56" t="s">
         <v>328</v>
       </c>
-      <c r="Q1" s="59" t="s">
+      <c r="Q1" s="56" t="s">
         <v>329</v>
       </c>
       <c r="R1" s="38" t="s">
@@ -4815,10 +4833,10 @@
       <c r="AA1" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="AB1" s="59" t="s">
+      <c r="AB1" s="56" t="s">
         <v>356</v>
       </c>
-      <c r="AC1" s="59" t="s">
+      <c r="AC1" s="56" t="s">
         <v>858</v>
       </c>
     </row>
@@ -5868,18 +5886,18 @@
       <c r="AC20" s="40"/>
     </row>
     <row r="21" spans="1:29" ht="14.5" customHeight="1">
-      <c r="P21" s="102" t="s">
+      <c r="P21" s="112" t="s">
         <v>760</v>
       </c>
-      <c r="Q21" s="102"/>
+      <c r="Q21" s="112"/>
     </row>
     <row r="22" spans="1:29">
-      <c r="P22" s="102"/>
-      <c r="Q22" s="102"/>
+      <c r="P22" s="112"/>
+      <c r="Q22" s="112"/>
     </row>
     <row r="23" spans="1:29">
-      <c r="P23" s="102"/>
-      <c r="Q23" s="102"/>
+      <c r="P23" s="112"/>
+      <c r="Q23" s="112"/>
     </row>
     <row r="24" spans="1:29">
       <c r="H24" s="1"/>
@@ -6943,7 +6961,7 @@
       <c r="W23" s="40"/>
     </row>
     <row r="24" spans="1:23">
-      <c r="A24" s="76" t="s">
+      <c r="A24" s="73" t="s">
         <v>790</v>
       </c>
       <c r="B24" s="40"/>
@@ -6955,7 +6973,7 @@
       <c r="H24" s="40"/>
       <c r="I24" s="40"/>
       <c r="J24" s="40"/>
-      <c r="K24" s="77" t="s">
+      <c r="K24" s="74" t="s">
         <v>774</v>
       </c>
       <c r="L24" s="40"/>
@@ -7015,7 +7033,7 @@
       <c r="W25" s="40"/>
     </row>
     <row r="26" spans="1:23">
-      <c r="A26" s="78" t="s">
+      <c r="A26" s="75" t="s">
         <v>791</v>
       </c>
       <c r="B26" s="52"/>
@@ -7028,7 +7046,7 @@
       <c r="I26" s="40"/>
       <c r="J26" s="40"/>
       <c r="K26" s="40"/>
-      <c r="L26" s="79" t="s">
+      <c r="L26" s="76" t="s">
         <v>776</v>
       </c>
       <c r="M26" s="40"/>
@@ -7044,7 +7062,7 @@
       <c r="W26" s="40"/>
     </row>
     <row r="27" spans="1:23">
-      <c r="A27" s="78" t="s">
+      <c r="A27" s="75" t="s">
         <v>789</v>
       </c>
       <c r="B27" s="52"/>
@@ -7188,7 +7206,7 @@
       <c r="W30" s="40"/>
     </row>
     <row r="31" spans="1:23">
-      <c r="A31" s="86" t="s">
+      <c r="A31" s="83" t="s">
         <v>793</v>
       </c>
       <c r="B31" s="52">
@@ -7302,7 +7320,7 @@
         <v>237</v>
       </c>
       <c r="P33" s="40"/>
-      <c r="Q33" s="79" t="s">
+      <c r="Q33" s="76" t="s">
         <v>82</v>
       </c>
       <c r="R33" s="40"/>
@@ -8322,7 +8340,7 @@
       <c r="G11" s="40"/>
       <c r="H11" s="40"/>
       <c r="I11" s="40"/>
-      <c r="J11" s="98"/>
+      <c r="J11" s="95"/>
       <c r="K11" s="43"/>
       <c r="L11" s="40"/>
       <c r="M11" s="40"/>
@@ -8364,7 +8382,7 @@
       <c r="G12" s="40"/>
       <c r="H12" s="40"/>
       <c r="I12" s="40"/>
-      <c r="J12" s="98" t="s">
+      <c r="J12" s="95" t="s">
         <v>1082</v>
       </c>
       <c r="K12" s="43" t="s">
@@ -8563,7 +8581,7 @@
       <c r="L1" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="M1" s="88" t="s">
+      <c r="M1" s="85" t="s">
         <v>84</v>
       </c>
     </row>
@@ -8682,7 +8700,7 @@
       <c r="I5" s="40"/>
       <c r="J5" s="40"/>
       <c r="K5" s="40"/>
-      <c r="L5" s="80" t="s">
+      <c r="L5" s="77" t="s">
         <v>923</v>
       </c>
       <c r="M5" s="40"/>
@@ -8757,7 +8775,7 @@
       <c r="M8" s="40"/>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="89" t="s">
+      <c r="A9" s="86" t="s">
         <v>1027</v>
       </c>
       <c r="B9" s="40"/>
@@ -8780,7 +8798,7 @@
       <c r="M9" s="40"/>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="90" t="s">
+      <c r="A10" s="87" t="s">
         <v>1028</v>
       </c>
       <c r="B10" s="40"/>
@@ -8807,7 +8825,7 @@
       <c r="M10" s="40"/>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="89" t="s">
+      <c r="A11" s="86" t="s">
         <v>1029</v>
       </c>
       <c r="B11" s="40"/>
@@ -8834,7 +8852,7 @@
       <c r="M11" s="40"/>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" s="89" t="s">
+      <c r="A12" s="86" t="s">
         <v>1030</v>
       </c>
       <c r="B12" s="40"/>
@@ -8903,7 +8921,7 @@
       <c r="M14" s="40"/>
     </row>
     <row r="15" spans="1:13">
-      <c r="A15" s="91" t="s">
+      <c r="A15" s="88" t="s">
         <v>1033</v>
       </c>
       <c r="B15" s="40"/>
@@ -8925,12 +8943,12 @@
       <c r="J15" s="40"/>
       <c r="K15" s="40"/>
       <c r="L15" s="40"/>
-      <c r="M15" s="92" t="s">
+      <c r="M15" s="89" t="s">
         <v>1035</v>
       </c>
     </row>
     <row r="16" spans="1:13">
-      <c r="A16" s="93" t="s">
+      <c r="A16" s="90" t="s">
         <v>1036</v>
       </c>
       <c r="B16" s="40"/>
@@ -8953,7 +8971,7 @@
       <c r="M16" s="40"/>
     </row>
     <row r="17" spans="1:13">
-      <c r="A17" s="89" t="s">
+      <c r="A17" s="86" t="s">
         <v>1037</v>
       </c>
       <c r="B17" s="40"/>
@@ -8976,13 +8994,13 @@
       <c r="I17" s="40"/>
       <c r="J17" s="40"/>
       <c r="K17" s="40"/>
-      <c r="L17" s="97" t="s">
+      <c r="L17" s="94" t="s">
         <v>1038</v>
       </c>
       <c r="M17" s="40"/>
     </row>
     <row r="18" spans="1:13">
-      <c r="A18" s="90" t="s">
+      <c r="A18" s="87" t="s">
         <v>1039</v>
       </c>
       <c r="B18" s="40"/>
@@ -8993,7 +9011,7 @@
       <c r="E18" s="40">
         <v>2</v>
       </c>
-      <c r="F18" s="94" t="s">
+      <c r="F18" s="91" t="s">
         <v>1040</v>
       </c>
       <c r="G18" s="40" t="s">
@@ -9005,13 +9023,13 @@
       <c r="I18" s="40"/>
       <c r="J18" s="40"/>
       <c r="K18" s="40"/>
-      <c r="L18" s="97" t="s">
+      <c r="L18" s="94" t="s">
         <v>1041</v>
       </c>
       <c r="M18" s="40"/>
     </row>
     <row r="19" spans="1:13">
-      <c r="A19" s="89" t="s">
+      <c r="A19" s="86" t="s">
         <v>1042</v>
       </c>
       <c r="B19" s="40"/>
@@ -9034,13 +9052,13 @@
       <c r="I19" s="40"/>
       <c r="J19" s="40"/>
       <c r="K19" s="40"/>
-      <c r="L19" s="97" t="s">
+      <c r="L19" s="94" t="s">
         <v>1044</v>
       </c>
       <c r="M19" s="40"/>
     </row>
     <row r="20" spans="1:13">
-      <c r="A20" s="93" t="s">
+      <c r="A20" s="90" t="s">
         <v>1045</v>
       </c>
       <c r="B20" s="40"/>
@@ -9051,7 +9069,7 @@
       <c r="E20" s="40">
         <v>0</v>
       </c>
-      <c r="F20" s="94" t="s">
+      <c r="F20" s="91" t="s">
         <v>579</v>
       </c>
       <c r="G20" s="40"/>
@@ -9082,13 +9100,13 @@
       <c r="I21" s="40"/>
       <c r="J21" s="40"/>
       <c r="K21" s="40"/>
-      <c r="L21" s="95" t="s">
+      <c r="L21" s="92" t="s">
         <v>1048</v>
       </c>
       <c r="M21" s="40"/>
     </row>
     <row r="22" spans="1:13">
-      <c r="A22" s="91" t="s">
+      <c r="A22" s="88" t="s">
         <v>1049</v>
       </c>
       <c r="B22" s="40"/>
@@ -9107,7 +9125,7 @@
       <c r="I22" s="40"/>
       <c r="J22" s="40"/>
       <c r="K22" s="40"/>
-      <c r="L22" s="95" t="s">
+      <c r="L22" s="92" t="s">
         <v>1051</v>
       </c>
       <c r="M22" s="40"/>
@@ -9132,7 +9150,7 @@
       <c r="I23" s="40"/>
       <c r="J23" s="40"/>
       <c r="K23" s="40"/>
-      <c r="L23" s="96" t="s">
+      <c r="L23" s="93" t="s">
         <v>1053</v>
       </c>
       <c r="M23" s="40"/>
@@ -9547,36 +9565,36 @@
       <c r="V6" s="40"/>
     </row>
     <row r="7" spans="1:22">
-      <c r="K7" s="106" t="s">
+      <c r="K7" s="116" t="s">
         <v>806</v>
       </c>
-      <c r="L7" s="106"/>
-      <c r="M7" s="106"/>
-      <c r="N7" s="106"/>
-      <c r="O7" s="103" t="s">
+      <c r="L7" s="116"/>
+      <c r="M7" s="116"/>
+      <c r="N7" s="116"/>
+      <c r="O7" s="113" t="s">
         <v>803</v>
       </c>
-      <c r="P7" s="103"/>
-      <c r="Q7" s="103"/>
-      <c r="R7" s="103"/>
-      <c r="S7" s="103"/>
-      <c r="T7" s="103"/>
-      <c r="U7" s="103"/>
-      <c r="V7" s="103"/>
+      <c r="P7" s="113"/>
+      <c r="Q7" s="113"/>
+      <c r="R7" s="113"/>
+      <c r="S7" s="113"/>
+      <c r="T7" s="113"/>
+      <c r="U7" s="113"/>
+      <c r="V7" s="113"/>
     </row>
     <row r="8" spans="1:22">
-      <c r="O8" s="104" t="s">
+      <c r="O8" s="114" t="s">
         <v>686</v>
       </c>
-      <c r="P8" s="104"/>
-      <c r="Q8" s="104"/>
-      <c r="R8" s="104"/>
-      <c r="S8" s="105" t="s">
+      <c r="P8" s="114"/>
+      <c r="Q8" s="114"/>
+      <c r="R8" s="114"/>
+      <c r="S8" s="115" t="s">
         <v>743</v>
       </c>
-      <c r="T8" s="105"/>
-      <c r="U8" s="105"/>
-      <c r="V8" s="105"/>
+      <c r="T8" s="115"/>
+      <c r="U8" s="115"/>
+      <c r="V8" s="115"/>
     </row>
     <row r="11" spans="1:22">
       <c r="O11">
@@ -9662,7 +9680,7 @@
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="60" t="s">
         <v>64</v>
       </c>
       <c r="B2" s="36" t="s">
@@ -9677,7 +9695,7 @@
       <c r="E2" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="66" t="s">
+      <c r="F2" s="63" t="s">
         <v>15</v>
       </c>
       <c r="G2" s="36"/>
@@ -9687,10 +9705,10 @@
       <c r="I2" s="40"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="60" t="s">
         <v>65</v>
       </c>
-      <c r="B3" s="66" t="s">
+      <c r="B3" s="63" t="s">
         <v>28</v>
       </c>
       <c r="C3" s="36">
@@ -9705,17 +9723,17 @@
       <c r="F3" s="36" t="s">
         <v>710</v>
       </c>
-      <c r="G3" s="66" t="s">
+      <c r="G3" s="63" t="s">
         <v>711</v>
       </c>
       <c r="H3" s="40"/>
       <c r="I3" s="40"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="60" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="66" t="s">
+      <c r="B4" s="63" t="s">
         <v>466</v>
       </c>
       <c r="C4" s="36">
@@ -9727,10 +9745,10 @@
       <c r="E4" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="66" t="s">
+      <c r="F4" s="63" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="66" t="s">
+      <c r="G4" s="63" t="s">
         <v>717</v>
       </c>
       <c r="H4" s="43" t="s">
@@ -10208,7 +10226,7 @@
       <c r="C1" s="38" t="s">
         <v>1223</v>
       </c>
-      <c r="D1" s="101" t="s">
+      <c r="D1" s="98" t="s">
         <v>1224</v>
       </c>
       <c r="E1" s="38" t="s">
@@ -10757,7 +10775,7 @@
       <c r="X9" s="40"/>
       <c r="Y9" s="40"/>
       <c r="Z9" s="40"/>
-      <c r="AA9" s="100" t="s">
+      <c r="AA9" s="97" t="s">
         <v>1216</v>
       </c>
     </row>
@@ -10778,7 +10796,7 @@
     <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="68" customFormat="1">
+    <row r="1" spans="1:13" s="65" customFormat="1">
       <c r="A1" s="41" t="s">
         <v>0</v>
       </c>
@@ -11114,7 +11132,7 @@
       <c r="M13" s="40"/>
     </row>
     <row r="14" spans="1:13">
-      <c r="A14" s="67" t="s">
+      <c r="A14" s="64" t="s">
         <v>585</v>
       </c>
       <c r="B14" s="40">
@@ -11300,25 +11318,25 @@
       </c>
     </row>
     <row r="2" spans="1:33">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="71">
+      <c r="B2" s="68">
         <v>0</v>
       </c>
-      <c r="C2" s="71" t="s">
+      <c r="C2" s="68" t="s">
         <v>305</v>
       </c>
-      <c r="D2" s="71" t="s">
+      <c r="D2" s="68" t="s">
         <v>197</v>
       </c>
-      <c r="E2" s="71" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="74"/>
-      <c r="G2" s="74"/>
-      <c r="H2" s="74"/>
-      <c r="I2" s="74"/>
+      <c r="E2" s="68" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
       <c r="J2" s="36"/>
       <c r="K2" s="36"/>
       <c r="L2" s="36"/>
@@ -11345,25 +11363,25 @@
       <c r="AG2" s="36"/>
     </row>
     <row r="3" spans="1:33">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="71">
+      <c r="B3" s="68">
         <v>-7</v>
       </c>
-      <c r="C3" s="71" t="s">
+      <c r="C3" s="68" t="s">
         <v>304</v>
       </c>
-      <c r="D3" s="71" t="s">
+      <c r="D3" s="68" t="s">
         <v>197</v>
       </c>
-      <c r="E3" s="71" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="74"/>
-      <c r="G3" s="74"/>
-      <c r="H3" s="74"/>
-      <c r="I3" s="74"/>
+      <c r="E3" s="68" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="71"/>
       <c r="J3" s="36"/>
       <c r="K3" s="36"/>
       <c r="L3" s="36"/>
@@ -11390,37 +11408,37 @@
       <c r="AG3" s="36"/>
     </row>
     <row r="4" spans="1:33">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="71">
+      <c r="B4" s="68">
         <v>0</v>
       </c>
-      <c r="C4" s="71" t="s">
+      <c r="C4" s="68" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="71" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="71" t="s">
+      <c r="D4" s="68" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="68" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="74">
+      <c r="F4" s="71">
         <v>0</v>
       </c>
-      <c r="G4" s="74" t="s">
+      <c r="G4" s="71" t="s">
         <v>42</v>
       </c>
-      <c r="H4" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="74" t="s">
+      <c r="H4" s="71" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="71" t="s">
         <v>43</v>
       </c>
       <c r="J4" s="36">
         <v>0</v>
       </c>
-      <c r="K4" s="66" t="s">
+      <c r="K4" s="63" t="s">
         <v>753</v>
       </c>
       <c r="L4" s="36" t="s">
@@ -11444,7 +11462,7 @@
       <c r="R4" s="36">
         <v>0</v>
       </c>
-      <c r="S4" s="66" t="s">
+      <c r="S4" s="63" t="s">
         <v>327</v>
       </c>
       <c r="T4" s="36" t="s">
@@ -11456,7 +11474,7 @@
       <c r="V4" s="36">
         <v>0</v>
       </c>
-      <c r="W4" s="66" t="s">
+      <c r="W4" s="63" t="s">
         <v>755</v>
       </c>
       <c r="X4" s="36" t="s">
@@ -11468,7 +11486,7 @@
       <c r="Z4" s="36">
         <v>0</v>
       </c>
-      <c r="AA4" s="66" t="s">
+      <c r="AA4" s="63" t="s">
         <v>757</v>
       </c>
       <c r="AB4" s="36" t="s">
@@ -11480,7 +11498,7 @@
       <c r="AD4" s="36">
         <v>0</v>
       </c>
-      <c r="AE4" s="66" t="s">
+      <c r="AE4" s="63" t="s">
         <v>759</v>
       </c>
       <c r="AF4" s="36" t="s">
@@ -11491,25 +11509,25 @@
       </c>
     </row>
     <row r="5" spans="1:33">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="60" t="s">
         <v>654</v>
       </c>
-      <c r="B5" s="70">
-        <v>1</v>
-      </c>
-      <c r="C5" s="71" t="s">
+      <c r="B5" s="67">
+        <v>1</v>
+      </c>
+      <c r="C5" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="72" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="72" t="s">
+      <c r="D5" s="69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="74"/>
-      <c r="G5" s="74"/>
-      <c r="H5" s="74"/>
-      <c r="I5" s="74"/>
+      <c r="F5" s="71"/>
+      <c r="G5" s="71"/>
+      <c r="H5" s="71"/>
+      <c r="I5" s="71"/>
       <c r="J5" s="36"/>
       <c r="K5" s="36"/>
       <c r="L5" s="36"/>
@@ -11536,25 +11554,25 @@
       <c r="AG5" s="36"/>
     </row>
     <row r="6" spans="1:33">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="60" t="s">
         <v>655</v>
       </c>
-      <c r="B6" s="70">
-        <v>1</v>
-      </c>
-      <c r="C6" s="71" t="s">
+      <c r="B6" s="67">
+        <v>1</v>
+      </c>
+      <c r="C6" s="68" t="s">
         <v>391</v>
       </c>
-      <c r="D6" s="72" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="72" t="s">
+      <c r="D6" s="69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="74"/>
-      <c r="G6" s="74"/>
-      <c r="H6" s="74"/>
-      <c r="I6" s="74"/>
+      <c r="F6" s="71"/>
+      <c r="G6" s="71"/>
+      <c r="H6" s="71"/>
+      <c r="I6" s="71"/>
       <c r="J6" s="36"/>
       <c r="K6" s="36"/>
       <c r="L6" s="36"/>
@@ -11581,23 +11599,23 @@
       <c r="AG6" s="36"/>
     </row>
     <row r="7" spans="1:33">
-      <c r="A7" s="63" t="s">
+      <c r="A7" s="60" t="s">
         <v>656</v>
       </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="71" t="s">
+      <c r="B7" s="67"/>
+      <c r="C7" s="68" t="s">
         <v>657</v>
       </c>
-      <c r="D7" s="72" t="s">
+      <c r="D7" s="69" t="s">
         <v>577</v>
       </c>
-      <c r="E7" s="72" t="s">
+      <c r="E7" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="74"/>
-      <c r="G7" s="74"/>
-      <c r="H7" s="74"/>
-      <c r="I7" s="74"/>
+      <c r="F7" s="71"/>
+      <c r="G7" s="71"/>
+      <c r="H7" s="71"/>
+      <c r="I7" s="71"/>
       <c r="J7" s="36"/>
       <c r="K7" s="36"/>
       <c r="L7" s="36"/>
@@ -11624,25 +11642,25 @@
       <c r="AG7" s="36"/>
     </row>
     <row r="8" spans="1:33">
-      <c r="A8" s="63" t="s">
+      <c r="A8" s="60" t="s">
         <v>658</v>
       </c>
-      <c r="B8" s="70">
+      <c r="B8" s="67">
         <v>3</v>
       </c>
-      <c r="C8" s="71" t="s">
+      <c r="C8" s="68" t="s">
         <v>659</v>
       </c>
-      <c r="D8" s="72" t="s">
+      <c r="D8" s="69" t="s">
         <v>499</v>
       </c>
-      <c r="E8" s="72" t="s">
+      <c r="E8" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="74"/>
-      <c r="G8" s="74"/>
-      <c r="H8" s="74"/>
-      <c r="I8" s="74"/>
+      <c r="F8" s="71"/>
+      <c r="G8" s="71"/>
+      <c r="H8" s="71"/>
+      <c r="I8" s="71"/>
       <c r="J8" s="36"/>
       <c r="K8" s="36"/>
       <c r="L8" s="36"/>
@@ -11669,25 +11687,25 @@
       <c r="AG8" s="36"/>
     </row>
     <row r="9" spans="1:33">
-      <c r="A9" s="63" t="s">
+      <c r="A9" s="60" t="s">
         <v>660</v>
       </c>
-      <c r="B9" s="70">
-        <v>1</v>
-      </c>
-      <c r="C9" s="71" t="s">
+      <c r="B9" s="67">
+        <v>1</v>
+      </c>
+      <c r="C9" s="68" t="s">
         <v>466</v>
       </c>
-      <c r="D9" s="72" t="s">
+      <c r="D9" s="69" t="s">
         <v>499</v>
       </c>
-      <c r="E9" s="72" t="s">
+      <c r="E9" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="F9" s="74"/>
-      <c r="G9" s="74"/>
-      <c r="H9" s="74"/>
-      <c r="I9" s="74"/>
+      <c r="F9" s="71"/>
+      <c r="G9" s="71"/>
+      <c r="H9" s="71"/>
+      <c r="I9" s="71"/>
       <c r="J9" s="36"/>
       <c r="K9" s="36"/>
       <c r="L9" s="36"/>
@@ -11714,21 +11732,21 @@
       <c r="AG9" s="36"/>
     </row>
     <row r="10" spans="1:33">
-      <c r="A10" s="63" t="s">
+      <c r="A10" s="60" t="s">
         <v>661</v>
       </c>
-      <c r="B10" s="70">
-        <v>1</v>
-      </c>
-      <c r="C10" s="71" t="s">
+      <c r="B10" s="67">
+        <v>1</v>
+      </c>
+      <c r="C10" s="68" t="s">
         <v>662</v>
       </c>
-      <c r="D10" s="71"/>
-      <c r="E10" s="71"/>
-      <c r="F10" s="74"/>
-      <c r="G10" s="74"/>
-      <c r="H10" s="74"/>
-      <c r="I10" s="74"/>
+      <c r="D10" s="68"/>
+      <c r="E10" s="68"/>
+      <c r="F10" s="71"/>
+      <c r="G10" s="71"/>
+      <c r="H10" s="71"/>
+      <c r="I10" s="71"/>
       <c r="J10" s="36"/>
       <c r="K10" s="36"/>
       <c r="L10" s="36"/>
@@ -11755,25 +11773,25 @@
       <c r="AG10" s="36"/>
     </row>
     <row r="11" spans="1:33">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="60" t="s">
         <v>663</v>
       </c>
-      <c r="B11" s="70">
-        <v>1</v>
-      </c>
-      <c r="C11" s="71" t="s">
+      <c r="B11" s="67">
+        <v>1</v>
+      </c>
+      <c r="C11" s="68" t="s">
         <v>664</v>
       </c>
-      <c r="D11" s="72" t="s">
+      <c r="D11" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="72" t="s">
+      <c r="E11" s="69" t="s">
         <v>155</v>
       </c>
-      <c r="F11" s="74"/>
-      <c r="G11" s="74"/>
-      <c r="H11" s="74"/>
-      <c r="I11" s="74"/>
+      <c r="F11" s="71"/>
+      <c r="G11" s="71"/>
+      <c r="H11" s="71"/>
+      <c r="I11" s="71"/>
       <c r="J11" s="36"/>
       <c r="K11" s="36"/>
       <c r="L11" s="36"/>
@@ -11800,25 +11818,25 @@
       <c r="AG11" s="36"/>
     </row>
     <row r="12" spans="1:33">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="60" t="s">
         <v>665</v>
       </c>
-      <c r="B12" s="70">
-        <v>1</v>
-      </c>
-      <c r="C12" s="71" t="s">
+      <c r="B12" s="67">
+        <v>1</v>
+      </c>
+      <c r="C12" s="68" t="s">
         <v>666</v>
       </c>
-      <c r="D12" s="72" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="72" t="s">
+      <c r="D12" s="69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="74"/>
-      <c r="G12" s="74"/>
-      <c r="H12" s="74"/>
-      <c r="I12" s="74"/>
+      <c r="F12" s="71"/>
+      <c r="G12" s="71"/>
+      <c r="H12" s="71"/>
+      <c r="I12" s="71"/>
       <c r="J12" s="36"/>
       <c r="K12" s="36"/>
       <c r="L12" s="36"/>
@@ -11845,31 +11863,31 @@
       <c r="AG12" s="36"/>
     </row>
     <row r="13" spans="1:33">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="60" t="s">
         <v>667</v>
       </c>
-      <c r="B13" s="70">
-        <v>1</v>
-      </c>
-      <c r="C13" s="69" t="s">
+      <c r="B13" s="67">
+        <v>1</v>
+      </c>
+      <c r="C13" s="66" t="s">
         <v>668</v>
       </c>
-      <c r="D13" s="72" t="s">
+      <c r="D13" s="69" t="s">
         <v>669</v>
       </c>
-      <c r="E13" s="72" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="74">
-        <v>1</v>
-      </c>
-      <c r="G13" s="74" t="s">
+      <c r="E13" s="69" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="71">
+        <v>1</v>
+      </c>
+      <c r="G13" s="71" t="s">
         <v>670</v>
       </c>
-      <c r="H13" s="74" t="s">
+      <c r="H13" s="71" t="s">
         <v>30</v>
       </c>
-      <c r="I13" s="74" t="s">
+      <c r="I13" s="71" t="s">
         <v>155</v>
       </c>
       <c r="J13" s="36"/>
@@ -11898,45 +11916,45 @@
       <c r="AG13" s="36"/>
     </row>
     <row r="14" spans="1:33">
-      <c r="A14" s="63" t="s">
+      <c r="A14" s="60" t="s">
         <v>671</v>
       </c>
-      <c r="B14" s="70">
-        <v>1</v>
-      </c>
-      <c r="C14" s="69" t="s">
+      <c r="B14" s="67">
+        <v>1</v>
+      </c>
+      <c r="C14" s="66" t="s">
         <v>578</v>
       </c>
-      <c r="D14" s="72" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="72" t="s">
+      <c r="D14" s="69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="69" t="s">
         <v>197</v>
       </c>
-      <c r="F14" s="73">
+      <c r="F14" s="70">
         <f>B14</f>
         <v>1</v>
       </c>
-      <c r="G14" s="74" t="s">
+      <c r="G14" s="71" t="s">
         <v>672</v>
       </c>
-      <c r="H14" s="73" t="s">
+      <c r="H14" s="70" t="s">
         <v>511</v>
       </c>
-      <c r="I14" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="J14" s="72">
+      <c r="I14" s="70" t="s">
+        <v>12</v>
+      </c>
+      <c r="J14" s="69">
         <f>B14</f>
         <v>1</v>
       </c>
-      <c r="K14" s="71" t="s">
+      <c r="K14" s="68" t="s">
         <v>578</v>
       </c>
-      <c r="L14" s="72" t="s">
+      <c r="L14" s="69" t="s">
         <v>318</v>
       </c>
-      <c r="M14" s="72" t="s">
+      <c r="M14" s="69" t="s">
         <v>197</v>
       </c>
       <c r="N14" s="36"/>
@@ -12612,50 +12630,50 @@
       <c r="AH9" s="40"/>
     </row>
     <row r="10" spans="1:34">
-      <c r="B10" s="110" t="s">
+      <c r="B10" s="120" t="s">
         <v>644</v>
       </c>
-      <c r="C10" s="110"/>
-      <c r="D10" s="110"/>
-      <c r="E10" s="110"/>
-      <c r="G10" s="110" t="s">
+      <c r="C10" s="120"/>
+      <c r="D10" s="120"/>
+      <c r="E10" s="120"/>
+      <c r="G10" s="120" t="s">
         <v>645</v>
       </c>
-      <c r="H10" s="110"/>
-      <c r="I10" s="110"/>
-      <c r="J10" s="110"/>
-      <c r="R10" s="110" t="s">
+      <c r="H10" s="120"/>
+      <c r="I10" s="120"/>
+      <c r="J10" s="120"/>
+      <c r="R10" s="120" t="s">
         <v>646</v>
       </c>
-      <c r="S10" s="110"/>
-      <c r="T10" s="110"/>
-      <c r="U10" s="110"/>
-      <c r="W10" s="110" t="s">
+      <c r="S10" s="120"/>
+      <c r="T10" s="120"/>
+      <c r="U10" s="120"/>
+      <c r="W10" s="120" t="s">
         <v>647</v>
       </c>
-      <c r="X10" s="110"/>
-      <c r="Y10" s="110"/>
-      <c r="Z10" s="110"/>
-      <c r="AA10" s="110" t="s">
+      <c r="X10" s="120"/>
+      <c r="Y10" s="120"/>
+      <c r="Z10" s="120"/>
+      <c r="AA10" s="120" t="s">
         <v>648</v>
       </c>
-      <c r="AB10" s="110"/>
-      <c r="AC10" s="110"/>
-      <c r="AD10" s="110"/>
-      <c r="AE10" s="107" t="s">
+      <c r="AB10" s="120"/>
+      <c r="AC10" s="120"/>
+      <c r="AD10" s="120"/>
+      <c r="AE10" s="117" t="s">
         <v>649</v>
       </c>
-      <c r="AF10" s="108"/>
-      <c r="AG10" s="108"/>
-      <c r="AH10" s="109"/>
+      <c r="AF10" s="118"/>
+      <c r="AG10" s="118"/>
+      <c r="AH10" s="119"/>
     </row>
     <row r="11" spans="1:34">
-      <c r="G11" s="103" t="s">
+      <c r="G11" s="113" t="s">
         <v>678</v>
       </c>
-      <c r="H11" s="103"/>
-      <c r="I11" s="103"/>
-      <c r="J11" s="103"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -13194,27 +13212,27 @@
     </row>
     <row r="5" spans="1:34">
       <c r="A5" s="37"/>
-      <c r="B5" s="111"/>
-      <c r="C5" s="111"/>
-      <c r="D5" s="111"/>
-      <c r="E5" s="111"/>
+      <c r="B5" s="121"/>
+      <c r="C5" s="121"/>
+      <c r="D5" s="121"/>
+      <c r="E5" s="121"/>
       <c r="F5" s="37"/>
-      <c r="G5" s="81"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="81"/>
-      <c r="J5" s="81"/>
-      <c r="K5" s="82"/>
-      <c r="L5" s="82"/>
-      <c r="M5" s="82"/>
-      <c r="N5" s="82"/>
-      <c r="O5" s="83"/>
-      <c r="P5" s="83"/>
-      <c r="Q5" s="83"/>
-      <c r="R5" s="83"/>
-      <c r="S5" s="84"/>
-      <c r="T5" s="84"/>
-      <c r="U5" s="84"/>
-      <c r="V5" s="84"/>
+      <c r="G5" s="78"/>
+      <c r="H5" s="78"/>
+      <c r="I5" s="78"/>
+      <c r="J5" s="78"/>
+      <c r="K5" s="79"/>
+      <c r="L5" s="79"/>
+      <c r="M5" s="79"/>
+      <c r="N5" s="79"/>
+      <c r="O5" s="80"/>
+      <c r="P5" s="80"/>
+      <c r="Q5" s="80"/>
+      <c r="R5" s="80"/>
+      <c r="S5" s="81"/>
+      <c r="T5" s="81"/>
+      <c r="U5" s="81"/>
+      <c r="V5" s="81"/>
       <c r="W5" s="37"/>
       <c r="X5" s="37"/>
       <c r="Y5" s="37"/>
@@ -13391,7 +13409,7 @@
       <c r="K6" s="40"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="67" t="s">
+      <c r="A7" s="64" t="s">
         <v>1097</v>
       </c>
       <c r="B7" s="40"/>
@@ -13429,7 +13447,7 @@
         <v>1100</v>
       </c>
       <c r="B9" s="40"/>
-      <c r="C9" s="95" t="s">
+      <c r="C9" s="92" t="s">
         <v>1098</v>
       </c>
       <c r="D9" s="40"/>
@@ -13447,8 +13465,8 @@
       </c>
       <c r="B10" s="40"/>
       <c r="C10" s="40"/>
-      <c r="D10" s="80"/>
-      <c r="E10" s="80"/>
+      <c r="D10" s="77"/>
+      <c r="E10" s="77"/>
       <c r="F10" s="40"/>
       <c r="G10" s="40"/>
       <c r="H10" s="40"/>
@@ -13462,19 +13480,19 @@
       </c>
       <c r="B11" s="40"/>
       <c r="C11" s="40"/>
-      <c r="D11" s="95" t="s">
+      <c r="D11" s="92" t="s">
         <v>1103</v>
       </c>
-      <c r="E11" s="95" t="s">
+      <c r="E11" s="92" t="s">
         <v>115</v>
       </c>
-      <c r="F11" s="95" t="s">
+      <c r="F11" s="92" t="s">
         <v>111</v>
       </c>
-      <c r="G11" s="95" t="s">
+      <c r="G11" s="92" t="s">
         <v>1104</v>
       </c>
-      <c r="H11" s="95" t="s">
+      <c r="H11" s="92" t="s">
         <v>1105</v>
       </c>
       <c r="I11" s="40"/>
@@ -13506,7 +13524,7 @@
       </c>
       <c r="B13" s="40"/>
       <c r="C13" s="40"/>
-      <c r="D13" s="95" t="s">
+      <c r="D13" s="92" t="s">
         <v>863</v>
       </c>
       <c r="E13" s="40"/>
@@ -13552,7 +13570,7 @@
       <c r="K15" s="40"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="91" t="s">
+      <c r="A16" s="88" t="s">
         <v>1111</v>
       </c>
       <c r="B16" s="40"/>
@@ -13618,7 +13636,7 @@
       <c r="E1" s="54" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="60" t="s">
+      <c r="F1" s="57" t="s">
         <v>134</v>
       </c>
       <c r="G1" s="54" t="s">
@@ -13897,10 +13915,10 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:W10"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="44.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="93.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.1796875" customWidth="1"/>
     <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.1796875" bestFit="1" customWidth="1"/>
@@ -13921,223 +13939,354 @@
     <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="11.90625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="14.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
-      <c r="A1" s="55" t="s">
+    <row r="1" spans="1:23">
+      <c r="A1" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="38" t="s">
+      <c r="B1" s="100" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="100" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="38" t="s">
+      <c r="D1" s="100" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="38" t="s">
+      <c r="E1" s="100" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="38" t="s">
+      <c r="F1" s="100" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="100" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="38" t="s">
+      <c r="H1" s="100" t="s">
         <v>67</v>
       </c>
-      <c r="I1" s="38" t="s">
+      <c r="I1" s="100" t="s">
         <v>68</v>
       </c>
-      <c r="J1" s="57" t="s">
+      <c r="J1" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="K1" s="39" t="s">
-        <v>1</v>
-      </c>
-      <c r="L1" s="19" t="s">
+      <c r="K1" s="101" t="s">
+        <v>1</v>
+      </c>
+      <c r="L1" s="101" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="19" t="s">
+      <c r="M1" s="101" t="s">
         <v>70</v>
       </c>
-      <c r="N1" s="19" t="s">
+      <c r="N1" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="19" t="s">
+      <c r="O1" s="101" t="s">
         <v>4</v>
       </c>
-      <c r="P1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q1" s="2" t="s">
+      <c r="P1" s="101" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q1" s="101" t="s">
         <v>2</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="101" t="s">
         <v>70</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="101" t="s">
         <v>4</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="101" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="2" spans="1:21">
-      <c r="A2" s="56" t="s">
+      <c r="V1" s="101" t="s">
+        <v>183</v>
+      </c>
+      <c r="W1" s="101" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23">
+      <c r="A2" s="36" t="s">
         <v>152</v>
       </c>
-      <c r="B2" s="40">
+      <c r="B2" s="108">
         <v>0</v>
       </c>
-      <c r="C2" s="43" t="s">
+      <c r="C2" s="109" t="s">
         <v>153</v>
       </c>
-      <c r="D2" s="40" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="40" t="s">
+      <c r="D2" s="108" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="108" t="s">
         <v>154</v>
       </c>
-      <c r="F2" s="40">
-        <v>1</v>
-      </c>
-      <c r="G2" s="43" t="s">
+      <c r="F2" s="108">
+        <v>1</v>
+      </c>
+      <c r="G2" s="109" t="s">
         <v>687</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="H2" s="108" t="s">
         <v>154</v>
       </c>
-      <c r="I2" s="40" t="s">
+      <c r="I2" s="108" t="s">
         <v>155</v>
       </c>
-      <c r="J2" s="52" t="s">
+      <c r="J2" s="108" t="s">
         <v>688</v>
       </c>
-      <c r="K2" s="40" t="s">
+      <c r="K2" s="108" t="s">
         <v>463</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="108" t="s">
         <v>203</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="108" t="s">
         <v>689</v>
       </c>
-      <c r="N2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="O2" s="3" t="s">
+      <c r="N2" s="108" t="s">
+        <v>12</v>
+      </c>
+      <c r="O2" s="108" t="s">
         <v>204</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="P2" s="108" t="s">
         <v>464</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="Q2" s="108" t="s">
         <v>205</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="R2" s="108" t="s">
         <v>690</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="S2" s="108" t="s">
         <v>204</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="T2" s="108" t="s">
         <v>155</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="U2" s="108" t="s">
         <v>691</v>
       </c>
-    </row>
-    <row r="3" spans="1:21">
-      <c r="A3" s="56" t="s">
+      <c r="V2" s="108"/>
+      <c r="W2" s="108"/>
+    </row>
+    <row r="3" spans="1:23">
+      <c r="A3" s="36" t="s">
         <v>172</v>
       </c>
-      <c r="B3" s="40">
+      <c r="B3" s="108">
         <v>0</v>
       </c>
-      <c r="C3" s="43" t="s">
+      <c r="C3" s="109" t="s">
         <v>153</v>
       </c>
-      <c r="D3" s="40" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="40" t="s">
+      <c r="D3" s="108" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="108" t="s">
         <v>154</v>
       </c>
-      <c r="F3" s="40">
-        <v>1</v>
-      </c>
-      <c r="G3" s="43" t="s">
+      <c r="F3" s="108">
+        <v>1</v>
+      </c>
+      <c r="G3" s="109" t="s">
         <v>687</v>
       </c>
-      <c r="H3" s="40" t="s">
+      <c r="H3" s="108" t="s">
         <v>154</v>
       </c>
-      <c r="I3" s="40" t="s">
+      <c r="I3" s="108" t="s">
         <v>155</v>
       </c>
-      <c r="J3" s="52" t="s">
+      <c r="J3" s="108" t="s">
         <v>692</v>
       </c>
-      <c r="K3" s="40" t="s">
+      <c r="K3" s="108" t="s">
         <v>693</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="108" t="s">
         <v>153</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="108" t="s">
         <v>689</v>
       </c>
-      <c r="N3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="O3" s="3" t="s">
+      <c r="N3" s="108" t="s">
+        <v>12</v>
+      </c>
+      <c r="O3" s="108" t="s">
         <v>154</v>
       </c>
-      <c r="P3" s="3" t="s">
+      <c r="P3" s="108" t="s">
         <v>694</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="Q3" s="108" t="s">
         <v>687</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="R3" s="108" t="s">
         <v>690</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="S3" s="108" t="s">
         <v>154</v>
       </c>
-      <c r="T3" s="3" t="s">
+      <c r="T3" s="108" t="s">
         <v>155</v>
       </c>
-      <c r="U3" s="3" t="s">
+      <c r="U3" s="108" t="s">
         <v>695</v>
       </c>
-    </row>
-    <row r="4" spans="1:21">
-      <c r="B4" s="112" t="s">
+      <c r="V3" s="108"/>
+      <c r="W3" s="108"/>
+    </row>
+    <row r="4" spans="1:23">
+      <c r="A4" s="108" t="s">
+        <v>1242</v>
+      </c>
+      <c r="B4" s="108">
+        <v>1</v>
+      </c>
+      <c r="C4" s="109" t="s">
+        <v>1241</v>
+      </c>
+      <c r="D4" s="108" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="108" t="s">
+        <v>204</v>
+      </c>
+      <c r="F4" s="108">
+        <v>1</v>
+      </c>
+      <c r="G4" s="109" t="s">
+        <v>353</v>
+      </c>
+      <c r="H4" s="108" t="s">
+        <v>204</v>
+      </c>
+      <c r="I4" s="108" t="s">
+        <v>155</v>
+      </c>
+      <c r="J4" s="108" t="s">
+        <v>1240</v>
+      </c>
+      <c r="K4" s="108"/>
+      <c r="L4" s="108"/>
+      <c r="M4" s="108"/>
+      <c r="N4" s="108"/>
+      <c r="O4" s="108"/>
+      <c r="P4" s="108"/>
+      <c r="Q4" s="108"/>
+      <c r="R4" s="108"/>
+      <c r="S4" s="108"/>
+      <c r="T4" s="108"/>
+      <c r="U4" s="108" t="s">
+        <v>355</v>
+      </c>
+      <c r="V4" s="108" t="s">
+        <v>355</v>
+      </c>
+      <c r="W4" s="108"/>
+    </row>
+    <row r="5" spans="1:23">
+      <c r="A5" s="108" t="s">
+        <v>1239</v>
+      </c>
+      <c r="B5" s="108"/>
+      <c r="C5" s="108"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="108"/>
+      <c r="F5" s="108"/>
+      <c r="G5" s="108"/>
+      <c r="H5" s="108"/>
+      <c r="I5" s="108"/>
+      <c r="J5" s="108"/>
+      <c r="K5" s="108"/>
+      <c r="L5" s="108"/>
+      <c r="M5" s="108"/>
+      <c r="N5" s="108"/>
+      <c r="O5" s="108"/>
+      <c r="P5" s="108"/>
+      <c r="Q5" s="108"/>
+      <c r="R5" s="108"/>
+      <c r="S5" s="108"/>
+      <c r="T5" s="108"/>
+      <c r="U5" s="108"/>
+      <c r="V5" s="108"/>
+      <c r="W5" s="108" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23">
+      <c r="A6" s="108" t="s">
+        <v>1238</v>
+      </c>
+      <c r="B6" s="108">
+        <v>1</v>
+      </c>
+      <c r="C6" s="109" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="108" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="108" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="108"/>
+      <c r="G6" s="108"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="108" t="s">
+        <v>1237</v>
+      </c>
+      <c r="K6" s="108"/>
+      <c r="L6" s="108"/>
+      <c r="M6" s="108"/>
+      <c r="N6" s="108"/>
+      <c r="O6" s="108"/>
+      <c r="P6" s="108"/>
+      <c r="Q6" s="108"/>
+      <c r="R6" s="108"/>
+      <c r="S6" s="108"/>
+      <c r="T6" s="108"/>
+      <c r="U6" s="89" t="s">
+        <v>1236</v>
+      </c>
+      <c r="V6" s="108"/>
+      <c r="W6" s="108" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23">
+      <c r="B10" s="122" t="s">
         <v>686</v>
       </c>
-      <c r="C4" s="113"/>
-      <c r="D4" s="113"/>
-      <c r="E4" s="114"/>
-      <c r="F4" s="112" t="s">
+      <c r="C10" s="123"/>
+      <c r="D10" s="123"/>
+      <c r="E10" s="124"/>
+      <c r="F10" s="122" t="s">
         <v>696</v>
       </c>
-      <c r="G4" s="113"/>
-      <c r="H4" s="113"/>
-      <c r="I4" s="114"/>
+      <c r="G10" s="123"/>
+      <c r="H10" s="123"/>
+      <c r="I10" s="124"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="F10:I10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -14255,100 +14404,100 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="126" t="s">
+      <c r="A4" s="108" t="s">
         <v>1229</v>
       </c>
-      <c r="B4" s="126" t="s">
+      <c r="B4" s="108" t="s">
         <v>141</v>
       </c>
-      <c r="C4" s="126" t="s">
+      <c r="C4" s="108" t="s">
         <v>1230</v>
       </c>
-      <c r="D4" s="126"/>
-      <c r="E4" s="126"/>
-      <c r="F4" s="126"/>
+      <c r="D4" s="108"/>
+      <c r="E4" s="108"/>
+      <c r="F4" s="108"/>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="128" t="s">
+      <c r="A5" s="110" t="s">
         <v>1231</v>
       </c>
-      <c r="B5" s="129" t="s">
+      <c r="B5" s="111" t="s">
         <v>141</v>
       </c>
-      <c r="C5" s="129" t="s">
+      <c r="C5" s="111" t="s">
         <v>1230</v>
       </c>
-      <c r="D5" s="126" t="s">
+      <c r="D5" s="108" t="s">
         <v>144</v>
       </c>
-      <c r="E5" s="126"/>
-      <c r="F5" s="126"/>
+      <c r="E5" s="108"/>
+      <c r="F5" s="108"/>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="128" t="s">
+      <c r="A6" s="110" t="s">
         <v>1232</v>
       </c>
-      <c r="B6" s="129" t="s">
+      <c r="B6" s="111" t="s">
         <v>141</v>
       </c>
-      <c r="C6" s="129" t="s">
+      <c r="C6" s="111" t="s">
         <v>1230</v>
       </c>
-      <c r="D6" s="126"/>
-      <c r="E6" s="126" t="s">
+      <c r="D6" s="108"/>
+      <c r="E6" s="108" t="s">
         <v>145</v>
       </c>
-      <c r="F6" s="126"/>
+      <c r="F6" s="108"/>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="128" t="s">
+      <c r="A7" s="110" t="s">
         <v>1233</v>
       </c>
-      <c r="B7" s="129" t="s">
+      <c r="B7" s="111" t="s">
         <v>141</v>
       </c>
-      <c r="C7" s="129" t="s">
+      <c r="C7" s="111" t="s">
         <v>1230</v>
       </c>
-      <c r="D7" s="126" t="s">
+      <c r="D7" s="108" t="s">
         <v>144</v>
       </c>
-      <c r="E7" s="127" t="s">
+      <c r="E7" s="109" t="s">
         <v>1234</v>
       </c>
-      <c r="F7" s="126"/>
+      <c r="F7" s="108"/>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="126" t="s">
+      <c r="A8" s="108" t="s">
         <v>1235</v>
       </c>
-      <c r="B8" s="129" t="s">
+      <c r="B8" s="111" t="s">
         <v>141</v>
       </c>
-      <c r="C8" s="126"/>
-      <c r="D8" s="126"/>
-      <c r="E8" s="126"/>
-      <c r="F8" s="126" t="s">
+      <c r="C8" s="108"/>
+      <c r="D8" s="108"/>
+      <c r="E8" s="108"/>
+      <c r="F8" s="108" t="s">
         <v>698</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="126" t="s">
+      <c r="A9" s="108" t="s">
         <v>142</v>
       </c>
-      <c r="B9" s="126" t="s">
+      <c r="B9" s="108" t="s">
         <v>141</v>
       </c>
-      <c r="C9" s="126" t="s">
+      <c r="C9" s="108" t="s">
         <v>1230</v>
       </c>
-      <c r="D9" s="126" t="s">
+      <c r="D9" s="108" t="s">
         <v>144</v>
       </c>
-      <c r="E9" s="126" t="s">
+      <c r="E9" s="108" t="s">
         <v>145</v>
       </c>
-      <c r="F9" s="126"/>
+      <c r="F9" s="108"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14401,16 +14550,16 @@
       <c r="F1" s="38" t="s">
         <v>428</v>
       </c>
-      <c r="G1" s="59" t="s">
+      <c r="G1" s="56" t="s">
         <v>429</v>
       </c>
-      <c r="H1" s="59" t="s">
+      <c r="H1" s="56" t="s">
         <v>430</v>
       </c>
-      <c r="I1" s="59" t="s">
+      <c r="I1" s="56" t="s">
         <v>430</v>
       </c>
-      <c r="J1" s="59" t="s">
+      <c r="J1" s="56" t="s">
         <v>439</v>
       </c>
       <c r="K1" s="38" t="s">
@@ -16817,7 +16966,7 @@
       </c>
     </row>
     <row r="51" spans="1:16">
-      <c r="A51" s="99" t="s">
+      <c r="A51" s="96" t="s">
         <v>1179</v>
       </c>
       <c r="B51" s="40" t="s">
@@ -17967,7 +18116,7 @@
       </c>
     </row>
     <row r="75" spans="1:16">
-      <c r="A75" s="58" t="s">
+      <c r="A75" s="55" t="s">
         <v>424</v>
       </c>
     </row>
@@ -18047,12 +18196,12 @@
       <c r="P1" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="Q1" s="87" t="s">
+      <c r="Q1" s="84" t="s">
         <v>1010</v>
       </c>
     </row>
     <row r="2" spans="1:17">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="60" t="s">
         <v>45</v>
       </c>
       <c r="B2" s="40">
@@ -18666,7 +18815,7 @@
       <c r="Q17" s="40"/>
     </row>
     <row r="18" spans="1:17">
-      <c r="A18" s="75" t="s">
+      <c r="A18" s="72" t="s">
         <v>761</v>
       </c>
       <c r="B18" s="40">
@@ -18703,7 +18852,7 @@
       <c r="Q18" s="40"/>
     </row>
     <row r="19" spans="1:17">
-      <c r="A19" s="75" t="s">
+      <c r="A19" s="72" t="s">
         <v>762</v>
       </c>
       <c r="B19" s="40">
@@ -18740,7 +18889,7 @@
       <c r="Q19" s="40"/>
     </row>
     <row r="20" spans="1:17">
-      <c r="A20" s="63" t="s">
+      <c r="A20" s="60" t="s">
         <v>1004</v>
       </c>
       <c r="B20" s="40">
@@ -19056,22 +19205,22 @@
       <c r="L1" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="M1" s="61" t="s">
+      <c r="M1" s="58" t="s">
         <v>69</v>
       </c>
-      <c r="N1" s="62" t="s">
+      <c r="N1" s="59" t="s">
         <v>480</v>
       </c>
-      <c r="O1" s="62" t="s">
+      <c r="O1" s="59" t="s">
         <v>481</v>
       </c>
-      <c r="P1" s="62" t="s">
+      <c r="P1" s="59" t="s">
         <v>482</v>
       </c>
-      <c r="Q1" s="62" t="s">
+      <c r="Q1" s="59" t="s">
         <v>483</v>
       </c>
-      <c r="R1" s="62" t="s">
+      <c r="R1" s="59" t="s">
         <v>484</v>
       </c>
       <c r="S1" s="31" t="s">
@@ -19080,10 +19229,10 @@
       <c r="T1" s="31" t="s">
         <v>491</v>
       </c>
-      <c r="U1" s="61" t="s">
+      <c r="U1" s="58" t="s">
         <v>485</v>
       </c>
-      <c r="V1" s="61" t="s">
+      <c r="V1" s="58" t="s">
         <v>486</v>
       </c>
       <c r="W1" s="39" t="s">
@@ -19280,16 +19429,16 @@
       </c>
     </row>
     <row r="5" spans="1:23">
-      <c r="B5" s="115" t="s">
+      <c r="B5" s="125" t="s">
         <v>686</v>
       </c>
-      <c r="C5" s="115"/>
-      <c r="D5" s="115"/>
-      <c r="E5" s="116" t="s">
+      <c r="C5" s="125"/>
+      <c r="D5" s="125"/>
+      <c r="E5" s="126" t="s">
         <v>743</v>
       </c>
-      <c r="F5" s="116"/>
-      <c r="G5" s="116"/>
+      <c r="F5" s="126"/>
+      <c r="G5" s="126"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -20734,7 +20883,7 @@
       </c>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="60" t="s">
         <v>50</v>
       </c>
       <c r="B2" s="40">
@@ -20756,7 +20905,7 @@
       <c r="J2" s="40"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="60" t="s">
         <v>51</v>
       </c>
       <c r="B3" s="40">
@@ -21613,7 +21762,7 @@
       <c r="F14" s="37"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="85" t="s">
+      <c r="A15" s="82" t="s">
         <v>871</v>
       </c>
       <c r="B15" s="37"/>
@@ -22948,10 +23097,10 @@
       </c>
     </row>
     <row r="2" spans="1:36">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="60" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="65">
+      <c r="B2" s="62">
         <v>1</v>
       </c>
       <c r="C2" s="16" t="s">
@@ -23000,10 +23149,10 @@
       <c r="AJ2" s="40"/>
     </row>
     <row r="3" spans="1:36">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="60" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="65">
+      <c r="B3" s="62">
         <v>1</v>
       </c>
       <c r="C3" s="16" t="s">
@@ -23076,10 +23225,10 @@
       <c r="AJ3" s="40"/>
     </row>
     <row r="4" spans="1:36">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="60" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="65">
+      <c r="B4" s="62">
         <v>1</v>
       </c>
       <c r="C4" s="16" t="s">
@@ -23152,10 +23301,10 @@
       <c r="AJ4" s="40"/>
     </row>
     <row r="5" spans="1:36">
-      <c r="A5" s="64" t="s">
+      <c r="A5" s="61" t="s">
         <v>179</v>
       </c>
-      <c r="B5" s="66">
+      <c r="B5" s="63">
         <v>2</v>
       </c>
       <c r="C5" s="43" t="s">
@@ -23204,10 +23353,10 @@
       <c r="AJ5" s="40"/>
     </row>
     <row r="6" spans="1:36">
-      <c r="A6" s="64" t="s">
+      <c r="A6" s="61" t="s">
         <v>180</v>
       </c>
-      <c r="B6" s="66">
+      <c r="B6" s="63">
         <v>2</v>
       </c>
       <c r="C6" s="43" t="s">
@@ -23256,10 +23405,10 @@
       <c r="AJ6" s="40"/>
     </row>
     <row r="7" spans="1:36">
-      <c r="A7" s="64" t="s">
+      <c r="A7" s="61" t="s">
         <v>181</v>
       </c>
-      <c r="B7" s="66">
+      <c r="B7" s="63">
         <v>2</v>
       </c>
       <c r="C7" s="43" t="s">
@@ -23308,10 +23457,10 @@
       <c r="AJ7" s="40"/>
     </row>
     <row r="8" spans="1:36">
-      <c r="A8" s="64" t="s">
+      <c r="A8" s="61" t="s">
         <v>184</v>
       </c>
-      <c r="B8" s="65">
+      <c r="B8" s="62">
         <v>1</v>
       </c>
       <c r="C8" s="16" t="s">
@@ -23362,10 +23511,10 @@
       <c r="AJ8" s="40"/>
     </row>
     <row r="9" spans="1:36">
-      <c r="A9" s="64" t="s">
+      <c r="A9" s="61" t="s">
         <v>185</v>
       </c>
-      <c r="B9" s="65">
+      <c r="B9" s="62">
         <v>2</v>
       </c>
       <c r="C9" s="43" t="s">
@@ -23428,10 +23577,10 @@
       <c r="AJ9" s="40"/>
     </row>
     <row r="10" spans="1:36">
-      <c r="A10" s="64" t="s">
+      <c r="A10" s="61" t="s">
         <v>186</v>
       </c>
-      <c r="B10" s="65">
+      <c r="B10" s="62">
         <v>2</v>
       </c>
       <c r="C10" s="43" t="s">
@@ -23488,10 +23637,10 @@
       <c r="AJ10" s="40"/>
     </row>
     <row r="11" spans="1:36">
-      <c r="A11" s="64" t="s">
+      <c r="A11" s="61" t="s">
         <v>187</v>
       </c>
-      <c r="B11" s="65">
+      <c r="B11" s="62">
         <v>1</v>
       </c>
       <c r="C11" s="16" t="s">
@@ -23542,10 +23691,10 @@
       <c r="AJ11" s="40"/>
     </row>
     <row r="12" spans="1:36">
-      <c r="A12" s="64" t="s">
+      <c r="A12" s="61" t="s">
         <v>188</v>
       </c>
-      <c r="B12" s="65">
+      <c r="B12" s="62">
         <v>1</v>
       </c>
       <c r="C12" s="16" t="s">
@@ -23594,10 +23743,10 @@
       <c r="AJ12" s="40"/>
     </row>
     <row r="13" spans="1:36">
-      <c r="A13" s="64" t="s">
+      <c r="A13" s="61" t="s">
         <v>189</v>
       </c>
-      <c r="B13" s="65">
+      <c r="B13" s="62">
         <v>1</v>
       </c>
       <c r="C13" s="16" t="s">
@@ -23648,10 +23797,10 @@
       <c r="AJ13" s="40"/>
     </row>
     <row r="14" spans="1:36">
-      <c r="A14" s="64" t="s">
+      <c r="A14" s="61" t="s">
         <v>190</v>
       </c>
-      <c r="B14" s="65">
+      <c r="B14" s="62">
         <v>1</v>
       </c>
       <c r="C14" s="16" t="s">
@@ -23700,10 +23849,10 @@
       <c r="AJ14" s="40"/>
     </row>
     <row r="15" spans="1:36">
-      <c r="A15" s="64" t="s">
+      <c r="A15" s="61" t="s">
         <v>191</v>
       </c>
-      <c r="B15" s="65">
+      <c r="B15" s="62">
         <v>1</v>
       </c>
       <c r="C15" s="16" t="s">
@@ -23752,10 +23901,10 @@
       <c r="AJ15" s="40"/>
     </row>
     <row r="16" spans="1:36">
-      <c r="A16" s="64" t="s">
+      <c r="A16" s="61" t="s">
         <v>192</v>
       </c>
-      <c r="B16" s="65">
+      <c r="B16" s="62">
         <v>2</v>
       </c>
       <c r="C16" s="43" t="s">
@@ -23812,10 +23961,10 @@
       <c r="AJ16" s="40"/>
     </row>
     <row r="17" spans="1:36">
-      <c r="A17" s="64" t="s">
+      <c r="A17" s="61" t="s">
         <v>193</v>
       </c>
-      <c r="B17" s="65">
+      <c r="B17" s="62">
         <v>1</v>
       </c>
       <c r="C17" s="16" t="s">
@@ -23864,10 +24013,10 @@
       <c r="AJ17" s="40"/>
     </row>
     <row r="18" spans="1:36">
-      <c r="A18" s="63" t="s">
+      <c r="A18" s="60" t="s">
         <v>531</v>
       </c>
-      <c r="B18" s="65">
+      <c r="B18" s="62">
         <v>1</v>
       </c>
       <c r="C18" s="16" t="s">
@@ -23924,10 +24073,10 @@
       <c r="AJ18" s="40"/>
     </row>
     <row r="19" spans="1:36">
-      <c r="A19" s="63" t="s">
+      <c r="A19" s="60" t="s">
         <v>532</v>
       </c>
-      <c r="B19" s="65">
+      <c r="B19" s="62">
         <v>2</v>
       </c>
       <c r="C19" s="43" t="s">
@@ -24002,10 +24151,10 @@
       <c r="AJ19" s="40"/>
     </row>
     <row r="20" spans="1:36">
-      <c r="A20" s="63" t="s">
+      <c r="A20" s="60" t="s">
         <v>535</v>
       </c>
-      <c r="B20" s="65">
+      <c r="B20" s="62">
         <v>1</v>
       </c>
       <c r="C20" s="16" t="s">
@@ -24080,10 +24229,10 @@
       <c r="AJ20" s="40"/>
     </row>
     <row r="21" spans="1:36">
-      <c r="A21" s="63" t="s">
+      <c r="A21" s="60" t="s">
         <v>540</v>
       </c>
-      <c r="B21" s="65">
+      <c r="B21" s="62">
         <v>1</v>
       </c>
       <c r="C21" s="16" t="s">
@@ -24152,10 +24301,10 @@
       <c r="AJ21" s="40"/>
     </row>
     <row r="22" spans="1:36">
-      <c r="A22" s="63" t="s">
+      <c r="A22" s="60" t="s">
         <v>543</v>
       </c>
-      <c r="B22" s="65"/>
+      <c r="B22" s="62"/>
       <c r="C22" s="16"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
@@ -24196,10 +24345,10 @@
       <c r="AJ22" s="40"/>
     </row>
     <row r="23" spans="1:36">
-      <c r="A23" s="63" t="s">
+      <c r="A23" s="60" t="s">
         <v>544</v>
       </c>
-      <c r="B23" s="65">
+      <c r="B23" s="62">
         <v>1</v>
       </c>
       <c r="C23" s="16" t="s">
@@ -24244,10 +24393,10 @@
       <c r="AJ23" s="40"/>
     </row>
     <row r="24" spans="1:36">
-      <c r="A24" s="63" t="s">
+      <c r="A24" s="60" t="s">
         <v>545</v>
       </c>
-      <c r="B24" s="65">
+      <c r="B24" s="62">
         <v>1</v>
       </c>
       <c r="C24" s="16" t="s">
@@ -24302,10 +24451,10 @@
       <c r="AJ24" s="40"/>
     </row>
     <row r="25" spans="1:36">
-      <c r="A25" s="63" t="s">
+      <c r="A25" s="60" t="s">
         <v>546</v>
       </c>
-      <c r="B25" s="65">
+      <c r="B25" s="62">
         <v>1</v>
       </c>
       <c r="C25" s="43" t="s">
@@ -24350,10 +24499,10 @@
       <c r="AJ25" s="40"/>
     </row>
     <row r="26" spans="1:36">
-      <c r="A26" s="63" t="s">
+      <c r="A26" s="60" t="s">
         <v>548</v>
       </c>
-      <c r="B26" s="65">
+      <c r="B26" s="62">
         <v>1</v>
       </c>
       <c r="C26" s="16" t="s">
@@ -24402,10 +24551,10 @@
       <c r="AJ26" s="40"/>
     </row>
     <row r="27" spans="1:36">
-      <c r="A27" s="63" t="s">
+      <c r="A27" s="60" t="s">
         <v>551</v>
       </c>
-      <c r="B27" s="65">
+      <c r="B27" s="62">
         <v>1</v>
       </c>
       <c r="C27" s="16" t="s">
@@ -24454,10 +24603,10 @@
       <c r="AJ27" s="40"/>
     </row>
     <row r="28" spans="1:36">
-      <c r="A28" s="63" t="s">
+      <c r="A28" s="60" t="s">
         <v>552</v>
       </c>
-      <c r="B28" s="65">
+      <c r="B28" s="62">
         <v>1</v>
       </c>
       <c r="C28" s="16" t="s">
@@ -24511,7 +24660,7 @@
       <c r="A29" s="36" t="s">
         <v>553</v>
       </c>
-      <c r="B29" s="65">
+      <c r="B29" s="62">
         <v>1</v>
       </c>
       <c r="C29" s="16" t="s">
@@ -24598,10 +24747,10 @@
       <c r="AJ29" s="40"/>
     </row>
     <row r="30" spans="1:36">
-      <c r="A30" s="63" t="s">
+      <c r="A30" s="60" t="s">
         <v>556</v>
       </c>
-      <c r="B30" s="65">
+      <c r="B30" s="62">
         <v>1</v>
       </c>
       <c r="C30" s="16" t="s">
@@ -24654,10 +24803,10 @@
       <c r="AJ30" s="40"/>
     </row>
     <row r="31" spans="1:36">
-      <c r="A31" s="63" t="s">
+      <c r="A31" s="60" t="s">
         <v>557</v>
       </c>
-      <c r="B31" s="65">
+      <c r="B31" s="62">
         <v>1</v>
       </c>
       <c r="C31" s="16" t="s">
@@ -24710,10 +24859,10 @@
       <c r="AJ31" s="40"/>
     </row>
     <row r="32" spans="1:36">
-      <c r="A32" s="63" t="s">
+      <c r="A32" s="60" t="s">
         <v>558</v>
       </c>
-      <c r="B32" s="65">
+      <c r="B32" s="62">
         <v>1</v>
       </c>
       <c r="C32" s="16" t="s">
@@ -24766,10 +24915,10 @@
       <c r="AJ32" s="40"/>
     </row>
     <row r="33" spans="1:36">
-      <c r="A33" s="63" t="s">
+      <c r="A33" s="60" t="s">
         <v>559</v>
       </c>
-      <c r="B33" s="65">
+      <c r="B33" s="62">
         <v>1</v>
       </c>
       <c r="C33" s="16" t="s">
@@ -24822,10 +24971,10 @@
       <c r="AJ33" s="40"/>
     </row>
     <row r="34" spans="1:36">
-      <c r="A34" s="63" t="s">
+      <c r="A34" s="60" t="s">
         <v>560</v>
       </c>
-      <c r="B34" s="65">
+      <c r="B34" s="62">
         <v>1</v>
       </c>
       <c r="C34" s="16" t="s">
@@ -24878,10 +25027,10 @@
       <c r="AJ34" s="40"/>
     </row>
     <row r="35" spans="1:36">
-      <c r="A35" s="63" t="s">
+      <c r="A35" s="60" t="s">
         <v>561</v>
       </c>
-      <c r="B35" s="65">
+      <c r="B35" s="62">
         <v>1</v>
       </c>
       <c r="C35" s="16" t="s">
@@ -24934,10 +25083,10 @@
       <c r="AJ35" s="40"/>
     </row>
     <row r="36" spans="1:36">
-      <c r="A36" s="63" t="s">
+      <c r="A36" s="60" t="s">
         <v>562</v>
       </c>
-      <c r="B36" s="65">
+      <c r="B36" s="62">
         <v>1</v>
       </c>
       <c r="C36" s="16" t="s">
@@ -24993,7 +25142,7 @@
       <c r="A37" s="36" t="s">
         <v>563</v>
       </c>
-      <c r="B37" s="65">
+      <c r="B37" s="62">
         <v>1</v>
       </c>
       <c r="C37" s="16" t="s">
@@ -25046,10 +25195,10 @@
       <c r="AJ37" s="40"/>
     </row>
     <row r="38" spans="1:36">
-      <c r="A38" s="63" t="s">
+      <c r="A38" s="60" t="s">
         <v>564</v>
       </c>
-      <c r="B38" s="65">
+      <c r="B38" s="62">
         <v>1</v>
       </c>
       <c r="C38" s="16" t="s">
@@ -25104,10 +25253,10 @@
       </c>
     </row>
     <row r="39" spans="1:36">
-      <c r="A39" s="63" t="s">
+      <c r="A39" s="60" t="s">
         <v>565</v>
       </c>
-      <c r="B39" s="65">
+      <c r="B39" s="62">
         <v>1</v>
       </c>
       <c r="C39" s="16" t="s">
@@ -25158,10 +25307,10 @@
       <c r="AJ39" s="40"/>
     </row>
     <row r="40" spans="1:36">
-      <c r="A40" s="63" t="s">
+      <c r="A40" s="60" t="s">
         <v>1000</v>
       </c>
-      <c r="B40" s="65">
+      <c r="B40" s="62">
         <v>1</v>
       </c>
       <c r="C40" s="16" t="s">
@@ -25236,718 +25385,718 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="121" t="s">
+      <c r="A1" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="118" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="118" t="s">
+      <c r="B1" s="100" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="100" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="118" t="s">
+      <c r="D1" s="100" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="118" t="s">
+      <c r="E1" s="100" t="s">
         <v>84</v>
       </c>
-      <c r="F1" s="118" t="s">
+      <c r="F1" s="100" t="s">
         <v>26</v>
       </c>
-      <c r="G1" s="118" t="s">
+      <c r="G1" s="100" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="118" t="s">
+      <c r="H1" s="100" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="118" t="s">
+      <c r="I1" s="100" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="118" t="s">
-        <v>1</v>
-      </c>
-      <c r="K1" s="118" t="s">
+      <c r="J1" s="100" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="100" t="s">
         <v>85</v>
       </c>
-      <c r="L1" s="118" t="s">
+      <c r="L1" s="100" t="s">
         <v>3</v>
       </c>
-      <c r="M1" s="118" t="s">
+      <c r="M1" s="100" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="119" t="s">
+      <c r="N1" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="O1" s="119" t="s">
-        <v>1</v>
-      </c>
-      <c r="P1" s="119" t="s">
+      <c r="O1" s="101" t="s">
+        <v>1</v>
+      </c>
+      <c r="P1" s="101" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="119" t="s">
+      <c r="Q1" s="101" t="s">
         <v>70</v>
       </c>
-      <c r="R1" s="119" t="s">
+      <c r="R1" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="S1" s="119" t="s">
+      <c r="S1" s="101" t="s">
         <v>4</v>
       </c>
-      <c r="T1" s="118" t="s">
+      <c r="T1" s="100" t="s">
         <v>797</v>
       </c>
-      <c r="U1" s="118" t="s">
+      <c r="U1" s="100" t="s">
         <v>796</v>
       </c>
-      <c r="V1" s="118" t="s">
+      <c r="V1" s="100" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="123" t="s">
+      <c r="A2" s="105" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="120">
-        <v>1</v>
-      </c>
-      <c r="C2" s="122" t="s">
+      <c r="B2" s="102">
+        <v>1</v>
+      </c>
+      <c r="C2" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="122" t="s">
+      <c r="D2" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="104" t="s">
         <v>794</v>
       </c>
-      <c r="F2" s="120"/>
-      <c r="G2" s="120"/>
-      <c r="H2" s="120"/>
-      <c r="I2" s="120"/>
-      <c r="J2" s="120"/>
-      <c r="K2" s="120"/>
-      <c r="L2" s="120"/>
-      <c r="M2" s="120"/>
-      <c r="N2" s="120"/>
-      <c r="O2" s="120"/>
-      <c r="P2" s="120"/>
-      <c r="Q2" s="120"/>
-      <c r="R2" s="120"/>
-      <c r="S2" s="120"/>
-      <c r="T2" s="120"/>
-      <c r="U2" s="120"/>
-      <c r="V2" s="120"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="102"/>
+      <c r="I2" s="102"/>
+      <c r="J2" s="102"/>
+      <c r="K2" s="102"/>
+      <c r="L2" s="102"/>
+      <c r="M2" s="102"/>
+      <c r="N2" s="102"/>
+      <c r="O2" s="102"/>
+      <c r="P2" s="102"/>
+      <c r="Q2" s="102"/>
+      <c r="R2" s="102"/>
+      <c r="S2" s="102"/>
+      <c r="T2" s="102"/>
+      <c r="U2" s="102"/>
+      <c r="V2" s="102"/>
     </row>
     <row r="3" spans="1:22">
-      <c r="A3" s="123" t="s">
+      <c r="A3" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="B3" s="120">
-        <v>1</v>
-      </c>
-      <c r="C3" s="122" t="s">
+      <c r="B3" s="102">
+        <v>1</v>
+      </c>
+      <c r="C3" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="122" t="s">
+      <c r="D3" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="104" t="s">
         <v>794</v>
       </c>
-      <c r="F3" s="120"/>
-      <c r="G3" s="120"/>
-      <c r="H3" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" s="120" t="s">
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="102" t="s">
         <v>43</v>
       </c>
-      <c r="J3" s="120"/>
-      <c r="K3" s="120"/>
-      <c r="L3" s="120"/>
-      <c r="M3" s="120"/>
-      <c r="N3" s="120" t="s">
+      <c r="J3" s="102"/>
+      <c r="K3" s="102"/>
+      <c r="L3" s="102"/>
+      <c r="M3" s="102"/>
+      <c r="N3" s="102" t="s">
         <v>928</v>
       </c>
-      <c r="O3" s="120" t="s">
+      <c r="O3" s="102" t="s">
         <v>929</v>
       </c>
-      <c r="P3" s="120" t="s">
+      <c r="P3" s="102" t="s">
         <v>42</v>
       </c>
-      <c r="Q3" s="120" t="s">
+      <c r="Q3" s="102" t="s">
         <v>929</v>
       </c>
-      <c r="R3" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="S3" s="120" t="s">
+      <c r="R3" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="S3" s="102" t="s">
         <v>43</v>
       </c>
-      <c r="T3" s="120"/>
-      <c r="U3" s="120"/>
-      <c r="V3" s="120"/>
+      <c r="T3" s="102"/>
+      <c r="U3" s="102"/>
+      <c r="V3" s="102"/>
     </row>
     <row r="4" spans="1:22">
-      <c r="A4" s="123" t="s">
+      <c r="A4" s="105" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="120">
+      <c r="B4" s="102">
         <v>0</v>
       </c>
-      <c r="C4" s="122" t="s">
+      <c r="C4" s="104" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="120"/>
-      <c r="F4" s="120"/>
-      <c r="G4" s="120"/>
-      <c r="H4" s="120"/>
-      <c r="I4" s="120"/>
-      <c r="J4" s="120"/>
-      <c r="K4" s="120"/>
-      <c r="L4" s="120"/>
-      <c r="M4" s="120"/>
-      <c r="N4" s="120"/>
-      <c r="O4" s="120"/>
-      <c r="P4" s="120"/>
-      <c r="Q4" s="120"/>
-      <c r="R4" s="120"/>
-      <c r="S4" s="120"/>
-      <c r="T4" s="120"/>
-      <c r="U4" s="120"/>
-      <c r="V4" s="120"/>
+      <c r="D4" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="102"/>
+      <c r="F4" s="102"/>
+      <c r="G4" s="102"/>
+      <c r="H4" s="102"/>
+      <c r="I4" s="102"/>
+      <c r="J4" s="102"/>
+      <c r="K4" s="102"/>
+      <c r="L4" s="102"/>
+      <c r="M4" s="102"/>
+      <c r="N4" s="102"/>
+      <c r="O4" s="102"/>
+      <c r="P4" s="102"/>
+      <c r="Q4" s="102"/>
+      <c r="R4" s="102"/>
+      <c r="S4" s="102"/>
+      <c r="T4" s="102"/>
+      <c r="U4" s="102"/>
+      <c r="V4" s="102"/>
     </row>
     <row r="5" spans="1:22">
-      <c r="A5" s="123" t="s">
+      <c r="A5" s="105" t="s">
         <v>89</v>
       </c>
-      <c r="B5" s="120">
-        <v>1</v>
-      </c>
-      <c r="C5" s="122" t="s">
+      <c r="B5" s="102">
+        <v>1</v>
+      </c>
+      <c r="C5" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="120" t="s">
+      <c r="D5" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="102" t="s">
         <v>252</v>
       </c>
-      <c r="F5" s="120" t="s">
+      <c r="F5" s="102" t="s">
         <v>930</v>
       </c>
-      <c r="G5" s="120"/>
-      <c r="H5" s="120"/>
-      <c r="I5" s="120"/>
-      <c r="J5" s="120"/>
-      <c r="K5" s="120"/>
-      <c r="L5" s="120"/>
-      <c r="M5" s="120"/>
-      <c r="N5" s="120"/>
-      <c r="O5" s="120"/>
-      <c r="P5" s="120"/>
-      <c r="Q5" s="120"/>
-      <c r="R5" s="120"/>
-      <c r="S5" s="120"/>
-      <c r="T5" s="120" t="s">
+      <c r="G5" s="102"/>
+      <c r="H5" s="102"/>
+      <c r="I5" s="102"/>
+      <c r="J5" s="102"/>
+      <c r="K5" s="102"/>
+      <c r="L5" s="102"/>
+      <c r="M5" s="102"/>
+      <c r="N5" s="102"/>
+      <c r="O5" s="102"/>
+      <c r="P5" s="102"/>
+      <c r="Q5" s="102"/>
+      <c r="R5" s="102"/>
+      <c r="S5" s="102"/>
+      <c r="T5" s="102" t="s">
         <v>14</v>
       </c>
-      <c r="U5" s="122" t="s">
+      <c r="U5" s="104" t="s">
         <v>19</v>
       </c>
-      <c r="V5" s="120"/>
+      <c r="V5" s="102"/>
     </row>
     <row r="6" spans="1:22">
-      <c r="A6" s="123" t="s">
+      <c r="A6" s="105" t="s">
         <v>90</v>
       </c>
-      <c r="B6" s="120">
-        <v>1</v>
-      </c>
-      <c r="C6" s="120" t="s">
+      <c r="B6" s="102">
+        <v>1</v>
+      </c>
+      <c r="C6" s="102" t="s">
         <v>304</v>
       </c>
-      <c r="D6" s="120" t="s">
+      <c r="D6" s="102" t="s">
         <v>197</v>
       </c>
-      <c r="E6" s="120"/>
-      <c r="F6" s="120"/>
-      <c r="G6" s="120"/>
-      <c r="H6" s="120"/>
-      <c r="I6" s="120"/>
-      <c r="J6" s="120"/>
-      <c r="K6" s="120"/>
-      <c r="L6" s="120"/>
-      <c r="M6" s="120"/>
-      <c r="N6" s="120"/>
-      <c r="O6" s="120"/>
-      <c r="P6" s="120"/>
-      <c r="Q6" s="120"/>
-      <c r="R6" s="120"/>
-      <c r="S6" s="120"/>
-      <c r="T6" s="120"/>
-      <c r="U6" s="120"/>
-      <c r="V6" s="120"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="102"/>
+      <c r="H6" s="102"/>
+      <c r="I6" s="102"/>
+      <c r="J6" s="102"/>
+      <c r="K6" s="102"/>
+      <c r="L6" s="102"/>
+      <c r="M6" s="102"/>
+      <c r="N6" s="102"/>
+      <c r="O6" s="102"/>
+      <c r="P6" s="102"/>
+      <c r="Q6" s="102"/>
+      <c r="R6" s="102"/>
+      <c r="S6" s="102"/>
+      <c r="T6" s="102"/>
+      <c r="U6" s="102"/>
+      <c r="V6" s="102"/>
     </row>
     <row r="7" spans="1:22">
-      <c r="A7" s="123" t="s">
+      <c r="A7" s="105" t="s">
         <v>91</v>
       </c>
-      <c r="B7" s="120">
-        <v>1</v>
-      </c>
-      <c r="C7" s="122" t="s">
+      <c r="B7" s="102">
+        <v>1</v>
+      </c>
+      <c r="C7" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="120" t="s">
+      <c r="D7" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="102" t="s">
         <v>252</v>
       </c>
-      <c r="F7" s="120" t="s">
+      <c r="F7" s="102" t="s">
         <v>930</v>
       </c>
-      <c r="G7" s="120"/>
-      <c r="H7" s="120"/>
-      <c r="I7" s="120"/>
-      <c r="J7" s="120"/>
-      <c r="K7" s="120"/>
-      <c r="L7" s="120"/>
-      <c r="M7" s="120"/>
-      <c r="N7" s="120"/>
-      <c r="O7" s="120"/>
-      <c r="P7" s="120"/>
-      <c r="Q7" s="120"/>
-      <c r="R7" s="120"/>
-      <c r="S7" s="120"/>
-      <c r="T7" s="120" t="s">
+      <c r="G7" s="102"/>
+      <c r="H7" s="102"/>
+      <c r="I7" s="102"/>
+      <c r="J7" s="102"/>
+      <c r="K7" s="102"/>
+      <c r="L7" s="102"/>
+      <c r="M7" s="102"/>
+      <c r="N7" s="102"/>
+      <c r="O7" s="102"/>
+      <c r="P7" s="102"/>
+      <c r="Q7" s="102"/>
+      <c r="R7" s="102"/>
+      <c r="S7" s="102"/>
+      <c r="T7" s="102" t="s">
         <v>14</v>
       </c>
-      <c r="U7" s="122" t="s">
+      <c r="U7" s="104" t="s">
         <v>19</v>
       </c>
-      <c r="V7" s="120"/>
+      <c r="V7" s="102"/>
     </row>
     <row r="8" spans="1:22">
-      <c r="A8" s="123" t="s">
+      <c r="A8" s="105" t="s">
         <v>92</v>
       </c>
-      <c r="B8" s="120">
-        <v>1</v>
-      </c>
-      <c r="C8" s="122" t="s">
+      <c r="B8" s="102">
+        <v>1</v>
+      </c>
+      <c r="C8" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="120" t="s">
+      <c r="D8" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="102" t="s">
         <v>252</v>
       </c>
-      <c r="F8" s="120" t="s">
+      <c r="F8" s="102" t="s">
         <v>795</v>
       </c>
-      <c r="G8" s="120"/>
-      <c r="H8" s="120"/>
-      <c r="I8" s="120"/>
-      <c r="J8" s="120"/>
-      <c r="K8" s="120"/>
-      <c r="L8" s="120"/>
-      <c r="M8" s="120"/>
-      <c r="N8" s="120"/>
-      <c r="O8" s="120"/>
-      <c r="P8" s="120"/>
-      <c r="Q8" s="120"/>
-      <c r="R8" s="120"/>
-      <c r="S8" s="120"/>
-      <c r="T8" s="120"/>
-      <c r="U8" s="120"/>
-      <c r="V8" s="120"/>
+      <c r="G8" s="102"/>
+      <c r="H8" s="102"/>
+      <c r="I8" s="102"/>
+      <c r="J8" s="102"/>
+      <c r="K8" s="102"/>
+      <c r="L8" s="102"/>
+      <c r="M8" s="102"/>
+      <c r="N8" s="102"/>
+      <c r="O8" s="102"/>
+      <c r="P8" s="102"/>
+      <c r="Q8" s="102"/>
+      <c r="R8" s="102"/>
+      <c r="S8" s="102"/>
+      <c r="T8" s="102"/>
+      <c r="U8" s="102"/>
+      <c r="V8" s="102"/>
     </row>
     <row r="9" spans="1:22">
-      <c r="A9" s="123" t="s">
+      <c r="A9" s="105" t="s">
         <v>93</v>
       </c>
-      <c r="B9" s="120">
-        <v>1</v>
-      </c>
-      <c r="C9" s="122" t="s">
+      <c r="B9" s="102">
+        <v>1</v>
+      </c>
+      <c r="C9" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="120" t="s">
+      <c r="D9" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="102" t="s">
         <v>252</v>
       </c>
-      <c r="F9" s="120" t="s">
+      <c r="F9" s="102" t="s">
         <v>795</v>
       </c>
-      <c r="G9" s="120"/>
-      <c r="H9" s="120"/>
-      <c r="I9" s="120"/>
-      <c r="J9" s="120"/>
-      <c r="K9" s="120"/>
-      <c r="L9" s="120"/>
-      <c r="M9" s="120"/>
-      <c r="N9" s="120"/>
-      <c r="O9" s="120"/>
-      <c r="P9" s="120"/>
-      <c r="Q9" s="120"/>
-      <c r="R9" s="120"/>
-      <c r="S9" s="120"/>
-      <c r="T9" s="120"/>
-      <c r="U9" s="120"/>
-      <c r="V9" s="120"/>
+      <c r="G9" s="102"/>
+      <c r="H9" s="102"/>
+      <c r="I9" s="102"/>
+      <c r="J9" s="102"/>
+      <c r="K9" s="102"/>
+      <c r="L9" s="102"/>
+      <c r="M9" s="102"/>
+      <c r="N9" s="102"/>
+      <c r="O9" s="102"/>
+      <c r="P9" s="102"/>
+      <c r="Q9" s="102"/>
+      <c r="R9" s="102"/>
+      <c r="S9" s="102"/>
+      <c r="T9" s="102"/>
+      <c r="U9" s="102"/>
+      <c r="V9" s="102"/>
     </row>
     <row r="10" spans="1:22">
-      <c r="A10" s="123" t="s">
+      <c r="A10" s="105" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="120">
-        <v>1</v>
-      </c>
-      <c r="C10" s="122"/>
-      <c r="D10" s="120"/>
-      <c r="E10" s="120" t="s">
+      <c r="B10" s="102">
+        <v>1</v>
+      </c>
+      <c r="C10" s="104"/>
+      <c r="D10" s="102"/>
+      <c r="E10" s="102" t="s">
         <v>252</v>
       </c>
-      <c r="F10" s="120" t="s">
+      <c r="F10" s="102" t="s">
         <v>252</v>
       </c>
-      <c r="G10" s="122" t="s">
+      <c r="G10" s="104" t="s">
         <v>28</v>
       </c>
-      <c r="H10" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="I10" s="120" t="s">
+      <c r="H10" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" s="102" t="s">
         <v>30</v>
       </c>
-      <c r="J10" s="120">
-        <v>1</v>
-      </c>
-      <c r="K10" s="122" t="s">
+      <c r="J10" s="102">
+        <v>1</v>
+      </c>
+      <c r="K10" s="104" t="s">
         <v>312</v>
       </c>
-      <c r="L10" s="120" t="s">
+      <c r="L10" s="102" t="s">
         <v>30</v>
       </c>
-      <c r="M10" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="N10" s="120" t="s">
+      <c r="M10" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="N10" s="102" t="s">
         <v>931</v>
       </c>
-      <c r="O10" s="120" t="s">
+      <c r="O10" s="102" t="s">
         <v>932</v>
       </c>
-      <c r="P10" s="120" t="s">
+      <c r="P10" s="102" t="s">
         <v>28</v>
       </c>
-      <c r="Q10" s="120" t="s">
+      <c r="Q10" s="102" t="s">
         <v>933</v>
       </c>
-      <c r="R10" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="S10" s="120" t="s">
+      <c r="R10" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="S10" s="102" t="s">
         <v>30</v>
       </c>
-      <c r="T10" s="120"/>
-      <c r="U10" s="120"/>
-      <c r="V10" s="120"/>
+      <c r="T10" s="102"/>
+      <c r="U10" s="102"/>
+      <c r="V10" s="102"/>
     </row>
     <row r="11" spans="1:22">
-      <c r="A11" s="123" t="s">
+      <c r="A11" s="105" t="s">
         <v>95</v>
       </c>
-      <c r="B11" s="120">
-        <v>1</v>
-      </c>
-      <c r="C11" s="122"/>
-      <c r="D11" s="120"/>
-      <c r="E11" s="120" t="s">
+      <c r="B11" s="102">
+        <v>1</v>
+      </c>
+      <c r="C11" s="104"/>
+      <c r="D11" s="102"/>
+      <c r="E11" s="102" t="s">
         <v>252</v>
       </c>
-      <c r="F11" s="120" t="s">
+      <c r="F11" s="102" t="s">
         <v>252</v>
       </c>
-      <c r="G11" s="122" t="s">
+      <c r="G11" s="104" t="s">
         <v>28</v>
       </c>
-      <c r="H11" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="I11" s="120" t="s">
+      <c r="H11" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="102" t="s">
         <v>30</v>
       </c>
-      <c r="J11" s="120">
-        <v>1</v>
-      </c>
-      <c r="K11" s="122" t="s">
+      <c r="J11" s="102">
+        <v>1</v>
+      </c>
+      <c r="K11" s="104" t="s">
         <v>312</v>
       </c>
-      <c r="L11" s="120" t="s">
+      <c r="L11" s="102" t="s">
         <v>30</v>
       </c>
-      <c r="M11" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="N11" s="120"/>
-      <c r="O11" s="120"/>
-      <c r="P11" s="120"/>
-      <c r="Q11" s="120"/>
-      <c r="R11" s="120"/>
-      <c r="S11" s="120"/>
-      <c r="T11" s="120"/>
-      <c r="U11" s="120"/>
-      <c r="V11" s="120"/>
+      <c r="M11" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="N11" s="102"/>
+      <c r="O11" s="102"/>
+      <c r="P11" s="102"/>
+      <c r="Q11" s="102"/>
+      <c r="R11" s="102"/>
+      <c r="S11" s="102"/>
+      <c r="T11" s="102"/>
+      <c r="U11" s="102"/>
+      <c r="V11" s="102"/>
     </row>
     <row r="12" spans="1:22">
-      <c r="A12" s="123" t="s">
+      <c r="A12" s="105" t="s">
         <v>96</v>
       </c>
-      <c r="B12" s="120">
-        <v>1</v>
-      </c>
-      <c r="C12" s="122" t="s">
+      <c r="B12" s="102">
+        <v>1</v>
+      </c>
+      <c r="C12" s="104" t="s">
         <v>305</v>
       </c>
-      <c r="D12" s="120" t="s">
+      <c r="D12" s="102" t="s">
         <v>197</v>
       </c>
-      <c r="E12" s="122" t="s">
+      <c r="E12" s="104" t="s">
         <v>794</v>
       </c>
-      <c r="F12" s="120"/>
-      <c r="G12" s="120"/>
-      <c r="H12" s="120"/>
-      <c r="I12" s="120"/>
-      <c r="J12" s="120"/>
-      <c r="K12" s="120"/>
-      <c r="L12" s="120"/>
-      <c r="M12" s="120"/>
-      <c r="N12" s="120"/>
-      <c r="O12" s="120"/>
-      <c r="P12" s="120"/>
-      <c r="Q12" s="120"/>
-      <c r="R12" s="120"/>
-      <c r="S12" s="120"/>
-      <c r="T12" s="120"/>
-      <c r="U12" s="120"/>
-      <c r="V12" s="120"/>
+      <c r="F12" s="102"/>
+      <c r="G12" s="102"/>
+      <c r="H12" s="102"/>
+      <c r="I12" s="102"/>
+      <c r="J12" s="102"/>
+      <c r="K12" s="102"/>
+      <c r="L12" s="102"/>
+      <c r="M12" s="102"/>
+      <c r="N12" s="102"/>
+      <c r="O12" s="102"/>
+      <c r="P12" s="102"/>
+      <c r="Q12" s="102"/>
+      <c r="R12" s="102"/>
+      <c r="S12" s="102"/>
+      <c r="T12" s="102"/>
+      <c r="U12" s="102"/>
+      <c r="V12" s="102"/>
     </row>
     <row r="13" spans="1:22">
-      <c r="A13" s="123" t="s">
+      <c r="A13" s="105" t="s">
         <v>97</v>
       </c>
-      <c r="B13" s="120">
+      <c r="B13" s="102">
         <v>0</v>
       </c>
-      <c r="C13" s="120" t="s">
+      <c r="C13" s="102" t="s">
         <v>252</v>
       </c>
-      <c r="D13" s="120" t="s">
+      <c r="D13" s="102" t="s">
         <v>252</v>
       </c>
-      <c r="E13" s="120"/>
-      <c r="F13" s="120"/>
-      <c r="G13" s="120"/>
-      <c r="H13" s="120"/>
-      <c r="I13" s="120"/>
-      <c r="J13" s="120"/>
-      <c r="K13" s="120"/>
-      <c r="L13" s="120"/>
-      <c r="M13" s="120"/>
-      <c r="N13" s="120"/>
-      <c r="O13" s="120"/>
-      <c r="P13" s="120"/>
-      <c r="Q13" s="120"/>
-      <c r="R13" s="120"/>
-      <c r="S13" s="120"/>
-      <c r="T13" s="120"/>
-      <c r="U13" s="120"/>
-      <c r="V13" s="120"/>
+      <c r="E13" s="102"/>
+      <c r="F13" s="102"/>
+      <c r="G13" s="102"/>
+      <c r="H13" s="102"/>
+      <c r="I13" s="102"/>
+      <c r="J13" s="102"/>
+      <c r="K13" s="102"/>
+      <c r="L13" s="102"/>
+      <c r="M13" s="102"/>
+      <c r="N13" s="102"/>
+      <c r="O13" s="102"/>
+      <c r="P13" s="102"/>
+      <c r="Q13" s="102"/>
+      <c r="R13" s="102"/>
+      <c r="S13" s="102"/>
+      <c r="T13" s="102"/>
+      <c r="U13" s="102"/>
+      <c r="V13" s="102"/>
     </row>
     <row r="14" spans="1:22">
-      <c r="A14" s="123" t="s">
+      <c r="A14" s="105" t="s">
         <v>98</v>
       </c>
-      <c r="B14" s="120">
-        <v>1</v>
-      </c>
-      <c r="C14" s="122" t="s">
+      <c r="B14" s="102">
+        <v>1</v>
+      </c>
+      <c r="C14" s="104" t="s">
         <v>934</v>
       </c>
-      <c r="D14" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="120"/>
-      <c r="F14" s="120"/>
-      <c r="G14" s="120"/>
-      <c r="H14" s="120"/>
-      <c r="I14" s="120"/>
-      <c r="J14" s="120"/>
-      <c r="K14" s="120"/>
-      <c r="L14" s="120"/>
-      <c r="M14" s="120"/>
-      <c r="N14" s="120"/>
-      <c r="O14" s="120"/>
-      <c r="P14" s="120"/>
-      <c r="Q14" s="120"/>
-      <c r="R14" s="120"/>
-      <c r="S14" s="120"/>
-      <c r="T14" s="120"/>
-      <c r="U14" s="120"/>
-      <c r="V14" s="120"/>
+      <c r="D14" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="102"/>
+      <c r="F14" s="102"/>
+      <c r="G14" s="102"/>
+      <c r="H14" s="102"/>
+      <c r="I14" s="102"/>
+      <c r="J14" s="102"/>
+      <c r="K14" s="102"/>
+      <c r="L14" s="102"/>
+      <c r="M14" s="102"/>
+      <c r="N14" s="102"/>
+      <c r="O14" s="102"/>
+      <c r="P14" s="102"/>
+      <c r="Q14" s="102"/>
+      <c r="R14" s="102"/>
+      <c r="S14" s="102"/>
+      <c r="T14" s="102"/>
+      <c r="U14" s="102"/>
+      <c r="V14" s="102"/>
     </row>
     <row r="15" spans="1:22">
-      <c r="A15" s="123" t="s">
+      <c r="A15" s="105" t="s">
         <v>99</v>
       </c>
-      <c r="B15" s="120">
-        <v>1</v>
-      </c>
-      <c r="C15" s="122" t="s">
+      <c r="B15" s="102">
+        <v>1</v>
+      </c>
+      <c r="C15" s="104" t="s">
         <v>178</v>
       </c>
-      <c r="D15" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="120"/>
-      <c r="F15" s="120"/>
-      <c r="G15" s="120"/>
-      <c r="H15" s="120"/>
-      <c r="I15" s="120"/>
-      <c r="J15" s="120"/>
-      <c r="K15" s="120"/>
-      <c r="L15" s="120"/>
-      <c r="M15" s="120"/>
-      <c r="N15" s="120"/>
-      <c r="O15" s="120"/>
-      <c r="P15" s="120"/>
-      <c r="Q15" s="120"/>
-      <c r="R15" s="120"/>
-      <c r="S15" s="120"/>
-      <c r="T15" s="120"/>
-      <c r="U15" s="120"/>
-      <c r="V15" s="120"/>
+      <c r="D15" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="102"/>
+      <c r="F15" s="102"/>
+      <c r="G15" s="102"/>
+      <c r="H15" s="102"/>
+      <c r="I15" s="102"/>
+      <c r="J15" s="102"/>
+      <c r="K15" s="102"/>
+      <c r="L15" s="102"/>
+      <c r="M15" s="102"/>
+      <c r="N15" s="102"/>
+      <c r="O15" s="102"/>
+      <c r="P15" s="102"/>
+      <c r="Q15" s="102"/>
+      <c r="R15" s="102"/>
+      <c r="S15" s="102"/>
+      <c r="T15" s="102"/>
+      <c r="U15" s="102"/>
+      <c r="V15" s="102"/>
     </row>
     <row r="16" spans="1:22">
-      <c r="A16" s="123" t="s">
+      <c r="A16" s="105" t="s">
         <v>100</v>
       </c>
-      <c r="B16" s="120">
-        <v>1</v>
-      </c>
-      <c r="C16" s="122" t="s">
+      <c r="B16" s="102">
+        <v>1</v>
+      </c>
+      <c r="C16" s="104" t="s">
         <v>305</v>
       </c>
-      <c r="D16" s="120" t="s">
+      <c r="D16" s="102" t="s">
         <v>197</v>
       </c>
-      <c r="E16" s="122" t="s">
+      <c r="E16" s="104" t="s">
         <v>794</v>
       </c>
-      <c r="F16" s="120"/>
-      <c r="G16" s="120"/>
-      <c r="H16" s="120"/>
-      <c r="I16" s="120"/>
-      <c r="J16" s="120"/>
-      <c r="K16" s="120"/>
-      <c r="L16" s="120"/>
-      <c r="M16" s="120"/>
-      <c r="N16" s="120"/>
-      <c r="O16" s="120"/>
-      <c r="P16" s="120"/>
-      <c r="Q16" s="120"/>
-      <c r="R16" s="120"/>
-      <c r="S16" s="120"/>
-      <c r="T16" s="120" t="s">
+      <c r="F16" s="102"/>
+      <c r="G16" s="102"/>
+      <c r="H16" s="102"/>
+      <c r="I16" s="102"/>
+      <c r="J16" s="102"/>
+      <c r="K16" s="102"/>
+      <c r="L16" s="102"/>
+      <c r="M16" s="102"/>
+      <c r="N16" s="102"/>
+      <c r="O16" s="102"/>
+      <c r="P16" s="102"/>
+      <c r="Q16" s="102"/>
+      <c r="R16" s="102"/>
+      <c r="S16" s="102"/>
+      <c r="T16" s="102" t="s">
         <v>14</v>
       </c>
-      <c r="U16" s="122" t="s">
+      <c r="U16" s="104" t="s">
         <v>708</v>
       </c>
-      <c r="V16" s="120"/>
+      <c r="V16" s="102"/>
     </row>
     <row r="17" spans="1:22">
-      <c r="A17" s="123" t="s">
+      <c r="A17" s="105" t="s">
         <v>101</v>
       </c>
-      <c r="B17" s="120">
-        <v>1</v>
-      </c>
-      <c r="C17" s="122" t="s">
+      <c r="B17" s="102">
+        <v>1</v>
+      </c>
+      <c r="C17" s="104" t="s">
         <v>305</v>
       </c>
-      <c r="D17" s="120" t="s">
+      <c r="D17" s="102" t="s">
         <v>197</v>
       </c>
-      <c r="E17" s="122" t="s">
+      <c r="E17" s="104" t="s">
         <v>794</v>
       </c>
-      <c r="F17" s="120"/>
-      <c r="G17" s="120"/>
-      <c r="H17" s="120"/>
-      <c r="I17" s="120"/>
-      <c r="J17" s="120"/>
-      <c r="K17" s="120"/>
-      <c r="L17" s="120"/>
-      <c r="M17" s="120"/>
-      <c r="N17" s="120"/>
-      <c r="O17" s="120"/>
-      <c r="P17" s="120"/>
-      <c r="Q17" s="120"/>
-      <c r="R17" s="120"/>
-      <c r="S17" s="120"/>
-      <c r="T17" s="120" t="s">
+      <c r="F17" s="102"/>
+      <c r="G17" s="102"/>
+      <c r="H17" s="102"/>
+      <c r="I17" s="102"/>
+      <c r="J17" s="102"/>
+      <c r="K17" s="102"/>
+      <c r="L17" s="102"/>
+      <c r="M17" s="102"/>
+      <c r="N17" s="102"/>
+      <c r="O17" s="102"/>
+      <c r="P17" s="102"/>
+      <c r="Q17" s="102"/>
+      <c r="R17" s="102"/>
+      <c r="S17" s="102"/>
+      <c r="T17" s="102" t="s">
         <v>14</v>
       </c>
-      <c r="U17" s="122" t="s">
+      <c r="U17" s="104" t="s">
         <v>721</v>
       </c>
-      <c r="V17" s="120"/>
+      <c r="V17" s="102"/>
     </row>
     <row r="18" spans="1:22">
-      <c r="A18" s="117" t="s">
+      <c r="A18" s="99" t="s">
         <v>1227</v>
       </c>
-      <c r="B18" s="124">
-        <v>1</v>
-      </c>
-      <c r="C18" s="125" t="s">
+      <c r="B18" s="106">
+        <v>1</v>
+      </c>
+      <c r="C18" s="107" t="s">
         <v>578</v>
       </c>
-      <c r="D18" s="124"/>
-      <c r="E18" s="122" t="s">
+      <c r="D18" s="106"/>
+      <c r="E18" s="104" t="s">
         <v>1228</v>
       </c>
-      <c r="F18" s="120"/>
-      <c r="G18" s="120"/>
-      <c r="H18" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="I18" s="120"/>
-      <c r="J18" s="120"/>
-      <c r="K18" s="120"/>
-      <c r="L18" s="120" t="s">
+      <c r="F18" s="102"/>
+      <c r="G18" s="102"/>
+      <c r="H18" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="I18" s="102"/>
+      <c r="J18" s="102"/>
+      <c r="K18" s="102"/>
+      <c r="L18" s="102" t="s">
         <v>318</v>
       </c>
-      <c r="M18" s="120"/>
-      <c r="N18" s="120"/>
-      <c r="O18" s="120"/>
-      <c r="P18" s="120"/>
-      <c r="Q18" s="120"/>
-      <c r="R18" s="120"/>
-      <c r="S18" s="120"/>
-      <c r="T18" s="120"/>
-      <c r="U18" s="120"/>
-      <c r="V18" s="122" t="s">
+      <c r="M18" s="102"/>
+      <c r="N18" s="102"/>
+      <c r="O18" s="102"/>
+      <c r="P18" s="102"/>
+      <c r="Q18" s="102"/>
+      <c r="R18" s="102"/>
+      <c r="S18" s="102"/>
+      <c r="T18" s="102"/>
+      <c r="U18" s="102"/>
+      <c r="V18" s="104" t="s">
         <v>1035</v>
       </c>
     </row>

</xml_diff>

<commit_message>
30 July 2024 - Updated request to remove the spaces
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4355" uniqueCount="1279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4383" uniqueCount="1299">
   <si>
     <t>Scenario</t>
   </si>
@@ -3911,6 +3911,66 @@
   </si>
   <si>
     <t>QGPXVV</t>
+  </si>
+  <si>
+    <t>QGUJQM</t>
+  </si>
+  <si>
+    <t>2302230000760</t>
+  </si>
+  <si>
+    <t>QGUKQR</t>
+  </si>
+  <si>
+    <t>2302230000762</t>
+  </si>
+  <si>
+    <t>QGUKXN</t>
+  </si>
+  <si>
+    <t>2302230000763</t>
+  </si>
+  <si>
+    <t>QGUK2L</t>
+  </si>
+  <si>
+    <t>2302230000764</t>
+  </si>
+  <si>
+    <t>QGULBV</t>
+  </si>
+  <si>
+    <t>2302230000765</t>
+  </si>
+  <si>
+    <t>QGULH2</t>
+  </si>
+  <si>
+    <t>2302230000766</t>
+  </si>
+  <si>
+    <t>QGULXJ</t>
+  </si>
+  <si>
+    <t>2302230000767</t>
+  </si>
+  <si>
+    <t>QGUMKK</t>
+  </si>
+  <si>
+    <t>2024-08-01T12:32:00</t>
+  </si>
+  <si>
+    <t>2024-08-01T13:19:00</t>
+  </si>
+  <si>
+    <t>QGUMOZ</t>
+  </si>
+  <si>
+    <t>2024-08-02T08:08:00</t>
+  </si>
+  <si>
+    <t>QGUMS0</t>
   </si>
 </sst>
 </file>
@@ -21015,7 +21075,7 @@
         <v>20</v>
       </c>
       <c r="J3" s="40" t="s">
-        <v>1269</v>
+        <v>1293</v>
       </c>
       <c r="K3" s="40"/>
       <c r="L3" s="40" t="s">
@@ -21025,7 +21085,7 @@
         <v>342</v>
       </c>
       <c r="N3" s="40" t="s">
-        <v>1270</v>
+        <v>1294</v>
       </c>
       <c r="O3" s="40" t="s">
         <v>204</v>
@@ -21040,7 +21100,7 @@
         <v>1</v>
       </c>
       <c r="S3" s="40" t="s">
-        <v>1271</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -21072,7 +21132,7 @@
         <v>740</v>
       </c>
       <c r="J4" s="40" t="s">
-        <v>1272</v>
+        <v>1296</v>
       </c>
       <c r="K4" s="40"/>
       <c r="L4" s="40" t="s">
@@ -21082,7 +21142,7 @@
         <v>407</v>
       </c>
       <c r="N4" s="40" t="s">
-        <v>1273</v>
+        <v>1297</v>
       </c>
       <c r="O4" s="40"/>
       <c r="P4" s="40"/>
@@ -21121,7 +21181,7 @@
         <v>968</v>
       </c>
       <c r="J5" s="40" t="s">
-        <v>1263</v>
+        <v>1298</v>
       </c>
       <c r="K5" s="40"/>
       <c r="L5" s="40" t="s">
@@ -21131,7 +21191,7 @@
         <v>342</v>
       </c>
       <c r="N5" s="40" t="s">
-        <v>1261</v>
+        <v>1294</v>
       </c>
       <c r="O5" s="40" t="s">
         <v>204</v>
@@ -21146,7 +21206,7 @@
         <v>1</v>
       </c>
       <c r="S5" s="40" t="s">
-        <v>1262</v>
+        <v>1295</v>
       </c>
     </row>
   </sheetData>
@@ -24261,10 +24321,10 @@
       <c r="P16" s="40"/>
       <c r="Q16" s="40"/>
       <c r="R16" s="40" t="s">
-        <v>809</v>
+        <v>1291</v>
       </c>
       <c r="S16" s="40" t="s">
-        <v>810</v>
+        <v>1292</v>
       </c>
       <c r="T16" s="40"/>
       <c r="U16" s="40"/>
@@ -24449,10 +24509,10 @@
         <v>30</v>
       </c>
       <c r="R19" s="40" t="s">
-        <v>1247</v>
+        <v>1279</v>
       </c>
       <c r="S19" s="40" t="s">
-        <v>827</v>
+        <v>1280</v>
       </c>
       <c r="T19" s="43">
         <v>0</v>
@@ -25099,10 +25159,10 @@
       <c r="P30" s="40"/>
       <c r="Q30" s="40"/>
       <c r="R30" s="40" t="s">
-        <v>1258</v>
+        <v>1289</v>
       </c>
       <c r="S30" s="40" t="s">
-        <v>1259</v>
+        <v>1290</v>
       </c>
       <c r="T30" s="40">
         <v>0</v>

</xml_diff>

<commit_message>
04 Aug 2024 - Updated extent reports
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ArunJK\Arun\Copa_SHDWebservices\src\test\java\TestData\"/>
     </mc:Choice>
@@ -55,7 +55,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4300" uniqueCount="1248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4321" uniqueCount="1269">
   <si>
     <t>Scenario</t>
   </si>
@@ -3818,12 +3818,76 @@
   </si>
   <si>
     <t>739</t>
+  </si>
+  <si>
+    <t>QG53BS</t>
+  </si>
+  <si>
+    <t>2024-08-02T01:55:00</t>
+  </si>
+  <si>
+    <t>2024-08-02T10:32:00</t>
+  </si>
+  <si>
+    <t>QG53OC</t>
+  </si>
+  <si>
+    <t>2024-08-02T09:24:00</t>
+  </si>
+  <si>
+    <t>2024-08-02T12:10:00</t>
+  </si>
+  <si>
+    <t>QHAFM3</t>
+  </si>
+  <si>
+    <t>2024-08-03T01:55:00</t>
+  </si>
+  <si>
+    <t>2024-08-03T10:32:00</t>
+  </si>
+  <si>
+    <t>QHAFZ1</t>
+  </si>
+  <si>
+    <t>2024-08-03T09:24:00</t>
+  </si>
+  <si>
+    <t>2024-08-03T12:10:00</t>
+  </si>
+  <si>
+    <t>2xjrinwzoxtuoovuiiozikkoy2</t>
+  </si>
+  <si>
+    <t>QHAG4H</t>
+  </si>
+  <si>
+    <t>2024-08-06T13:31:00</t>
+  </si>
+  <si>
+    <t>xsynkwmmojyjtovkjoo2ku2oio</t>
+  </si>
+  <si>
+    <t>kstrsvwxoiwjkovztnoioxzotn</t>
+  </si>
+  <si>
+    <t>QHAITO</t>
+  </si>
+  <si>
+    <t>xzizjnsioruzyovvjmoz2vkous</t>
+  </si>
+  <si>
+    <t>QHAL1O</t>
+  </si>
+  <si>
+    <t>2024-08-05T08:14:00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="20">
     <font>
       <sz val="11"/>
@@ -4825,24 +4889,24 @@
   <dimension ref="A1:AC25"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="52.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="52.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="8.21875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.21875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="11.6640625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="12.6640625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="12.6640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -6157,15 +6221,15 @@
   <dimension ref="A1:W36"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="54.77734375" customWidth="1"/>
-    <col min="10" max="10" width="8.77734375" style="25"/>
-    <col min="12" max="12" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="54.77734375"/>
+    <col min="10" max="10" style="25" width="8.77734375"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="11.44140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="12.6640625"/>
+    <col min="22" max="23" bestFit="true" customWidth="true" width="19.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -7699,16 +7763,16 @@
   <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="32.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5546875" style="27" customWidth="1"/>
-    <col min="4" max="4" width="29.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.77734375" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="11" width="14.33203125" style="27" customWidth="1"/>
-    <col min="12" max="12" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.88671875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="3" customWidth="true" style="27" width="17.5546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="29.77734375"/>
+    <col min="5" max="5" customWidth="true" width="13.77734375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="14.33203125"/>
+    <col min="7" max="11" customWidth="true" style="27" width="14.33203125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="13.77734375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.5546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -7763,13 +7827,13 @@
         <v>3</v>
       </c>
       <c r="C2" s="40" t="s">
-        <v>905</v>
+        <v>1262</v>
       </c>
       <c r="D2" s="43" t="s">
-        <v>906</v>
+        <v>1263</v>
       </c>
       <c r="E2" s="43" t="s">
-        <v>907</v>
+        <v>1261</v>
       </c>
       <c r="F2" s="40"/>
       <c r="G2" s="43" t="s">
@@ -7798,7 +7862,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="43" t="s">
-        <v>908</v>
+        <v>1264</v>
       </c>
       <c r="E3" s="43" t="s">
         <v>252</v>
@@ -7834,7 +7898,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="43" t="s">
-        <v>909</v>
+        <v>1260</v>
       </c>
       <c r="E4" s="40"/>
       <c r="F4" s="40" t="s">
@@ -7876,19 +7940,19 @@
   <dimension ref="A1:AL14"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="52.109375" style="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" style="27" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" style="27" customWidth="1"/>
-    <col min="4" max="4" width="18.77734375" style="27" customWidth="1"/>
-    <col min="5" max="6" width="12.88671875" style="27" customWidth="1"/>
-    <col min="7" max="7" width="15" style="27" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" style="27" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.77734375" style="27"/>
-    <col min="10" max="10" width="17.88671875" style="27" customWidth="1"/>
-    <col min="11" max="11" width="14.21875" style="27" customWidth="1"/>
-    <col min="12" max="37" width="8.77734375" style="27"/>
-    <col min="38" max="38" width="15.44140625" style="27" bestFit="1" customWidth="1"/>
-    <col min="39" max="16384" width="8.77734375" style="27"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="27" width="52.109375"/>
+    <col min="2" max="2" customWidth="true" style="27" width="16.5546875"/>
+    <col min="3" max="3" customWidth="true" style="27" width="19.88671875"/>
+    <col min="4" max="4" customWidth="true" style="27" width="18.77734375"/>
+    <col min="5" max="6" customWidth="true" style="27" width="12.88671875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="27" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="27" width="11.88671875"/>
+    <col min="9" max="9" style="27" width="8.77734375"/>
+    <col min="10" max="10" customWidth="true" style="27" width="17.88671875"/>
+    <col min="11" max="11" customWidth="true" style="27" width="14.21875"/>
+    <col min="12" max="37" style="27" width="8.77734375"/>
+    <col min="38" max="38" bestFit="true" customWidth="true" style="27" width="15.44140625"/>
+    <col min="39" max="16384" style="27" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -8762,15 +8826,15 @@
   <dimension ref="A1:M25"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="42.21875" style="27" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" style="27" customWidth="1"/>
-    <col min="3" max="3" width="17.77734375" style="27" customWidth="1"/>
-    <col min="4" max="4" width="16.77734375" style="27" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" style="27" customWidth="1"/>
-    <col min="6" max="11" width="8.77734375" style="27"/>
-    <col min="12" max="12" width="44.88671875" style="27" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.88671875" style="27" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.77734375" style="27"/>
+    <col min="1" max="1" customWidth="true" style="27" width="42.21875"/>
+    <col min="2" max="2" customWidth="true" style="27" width="15.77734375"/>
+    <col min="3" max="3" customWidth="true" style="27" width="17.77734375"/>
+    <col min="4" max="4" customWidth="true" style="27" width="16.77734375"/>
+    <col min="5" max="5" customWidth="true" style="27" width="15.6640625"/>
+    <col min="6" max="11" style="27" width="8.77734375"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="27" width="44.88671875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="27" width="11.88671875"/>
+    <col min="14" max="16384" style="27" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -9447,22 +9511,22 @@
   <dimension ref="A1:V11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="51.77734375" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.88671875" customWidth="1"/>
-    <col min="14" max="14" width="12.6640625" customWidth="1"/>
-    <col min="15" max="15" width="11.44140625" customWidth="1"/>
-    <col min="16" max="16" width="7.77734375" customWidth="1"/>
-    <col min="17" max="18" width="10.6640625" customWidth="1"/>
-    <col min="19" max="19" width="11.77734375" customWidth="1"/>
-    <col min="20" max="20" width="8.77734375" customWidth="1"/>
-    <col min="21" max="21" width="10.77734375" customWidth="1"/>
-    <col min="22" max="22" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="51.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="11" max="12" bestFit="true" customWidth="true" width="15.33203125"/>
+    <col min="13" max="13" customWidth="true" width="13.88671875"/>
+    <col min="14" max="14" customWidth="true" width="12.6640625"/>
+    <col min="15" max="15" customWidth="true" width="11.44140625"/>
+    <col min="16" max="16" customWidth="true" width="7.77734375"/>
+    <col min="17" max="18" customWidth="true" width="10.6640625"/>
+    <col min="19" max="19" customWidth="true" width="11.77734375"/>
+    <col min="20" max="20" customWidth="true" width="8.77734375"/>
+    <col min="21" max="21" customWidth="true" width="10.77734375"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="12.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -9718,16 +9782,16 @@
       <c r="H5" s="40"/>
       <c r="I5" s="40"/>
       <c r="J5" s="40" t="s">
-        <v>880</v>
+        <v>1257</v>
       </c>
       <c r="K5" s="40" t="s">
-        <v>882</v>
+        <v>1259</v>
       </c>
       <c r="L5" s="40" t="s">
         <v>632</v>
       </c>
       <c r="M5" s="40" t="s">
-        <v>881</v>
+        <v>1258</v>
       </c>
       <c r="N5" s="40" t="s">
         <v>632</v>
@@ -9770,16 +9834,16 @@
         <v>30</v>
       </c>
       <c r="J6" s="40" t="s">
-        <v>878</v>
+        <v>1254</v>
       </c>
       <c r="K6" s="40" t="s">
-        <v>876</v>
+        <v>1256</v>
       </c>
       <c r="L6" s="40" t="s">
         <v>632</v>
       </c>
       <c r="M6" s="40" t="s">
-        <v>877</v>
+        <v>1255</v>
       </c>
       <c r="N6" s="40" t="s">
         <v>632</v>
@@ -9871,12 +9935,12 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="76.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="76.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="13.44140625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="16.6640625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="19.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -10001,17 +10065,17 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="68.109375" style="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" style="27" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" style="27" customWidth="1"/>
-    <col min="4" max="4" width="9.6640625" style="27" customWidth="1"/>
-    <col min="5" max="5" width="17.21875" style="27" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" style="27" customWidth="1"/>
-    <col min="7" max="10" width="8.77734375" style="27"/>
-    <col min="11" max="11" width="10.6640625" style="27" customWidth="1"/>
-    <col min="12" max="12" width="12.21875" style="27" customWidth="1"/>
-    <col min="13" max="13" width="15.33203125" style="27" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.77734375" style="27"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="27" width="68.109375"/>
+    <col min="2" max="2" customWidth="true" style="27" width="12.5546875"/>
+    <col min="3" max="3" customWidth="true" style="27" width="12.33203125"/>
+    <col min="4" max="4" customWidth="true" style="27" width="9.6640625"/>
+    <col min="5" max="5" customWidth="true" style="27" width="17.21875"/>
+    <col min="6" max="6" customWidth="true" style="27" width="12.5546875"/>
+    <col min="7" max="10" style="27" width="8.77734375"/>
+    <col min="11" max="11" customWidth="true" style="27" width="10.6640625"/>
+    <col min="12" max="12" customWidth="true" style="27" width="12.21875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="27" width="15.33203125"/>
+    <col min="14" max="16384" style="27" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -10437,12 +10501,12 @@
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.5546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="11.77734375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="29.5546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="11.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -10518,7 +10582,7 @@
         <v>1181</v>
       </c>
       <c r="D5" s="40" t="s">
-        <v>1182</v>
+        <v>1266</v>
       </c>
       <c r="E5" s="40" t="s">
         <v>1183</v>
@@ -10543,12 +10607,12 @@
   <dimension ref="A1:AA9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="33.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.5546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.44140625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="21.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27">
@@ -11021,8 +11085,8 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="61.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="61.77734375"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="65" customFormat="1">
@@ -11418,31 +11482,31 @@
   <dimension ref="A1:AG14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="49.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="49.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="4.77734375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="9.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -12219,27 +12283,27 @@
   <dimension ref="A1:AH11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="10.44140625" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" customWidth="1"/>
-    <col min="12" max="12" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.77734375" customWidth="1"/>
-    <col min="20" max="20" width="9.44140625" customWidth="1"/>
-    <col min="21" max="21" width="11.109375" customWidth="1"/>
-    <col min="22" max="22" width="9.33203125" customWidth="1"/>
-    <col min="23" max="23" width="9.44140625" customWidth="1"/>
-    <col min="24" max="24" width="10.77734375" customWidth="1"/>
-    <col min="25" max="25" width="11.33203125" customWidth="1"/>
-    <col min="26" max="26" width="12" customWidth="1"/>
-    <col min="27" max="27" width="10.21875" customWidth="1"/>
-    <col min="30" max="30" width="9" customWidth="1"/>
-    <col min="34" max="34" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="33.0"/>
+    <col min="2" max="2" customWidth="true" width="10.44140625"/>
+    <col min="6" max="6" customWidth="true" width="10.88671875"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.33203125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.109375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.33203125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.33203125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="12.109375"/>
+    <col min="19" max="19" customWidth="true" width="8.77734375"/>
+    <col min="20" max="20" customWidth="true" width="9.44140625"/>
+    <col min="21" max="21" customWidth="true" width="11.109375"/>
+    <col min="22" max="22" customWidth="true" width="9.33203125"/>
+    <col min="23" max="23" customWidth="true" width="9.44140625"/>
+    <col min="24" max="24" customWidth="true" width="10.77734375"/>
+    <col min="25" max="25" customWidth="true" width="11.33203125"/>
+    <col min="26" max="26" customWidth="true" width="12.0"/>
+    <col min="27" max="27" customWidth="true" width="10.21875"/>
+    <col min="30" max="30" customWidth="true" width="9.0"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="17.5546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -12820,7 +12884,7 @@
       <c r="I9" s="40"/>
       <c r="J9" s="40"/>
       <c r="K9" s="40" t="s">
-        <v>673</v>
+        <v>1267</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>414</v>
@@ -12829,7 +12893,7 @@
         <v>303</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>672</v>
+        <v>1268</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>197</v>
@@ -12924,11 +12988,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="35.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="35.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.5546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.44140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -13012,10 +13076,10 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="33.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.5546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.44140625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.88671875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="14.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -13109,10 +13173,10 @@
   <dimension ref="A1:AH5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="46.6640625" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" customWidth="1"/>
-    <col min="29" max="29" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="46.6640625"/>
+    <col min="5" max="5" customWidth="true" width="6.21875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="13.33203125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -13489,16 +13553,16 @@
   <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="63.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="63.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="10.77734375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="19.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="15.5546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="8" max="9" bestFit="true" customWidth="true" width="19.44140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="10.88671875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="12.5546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -13827,24 +13891,24 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.6640625" customWidth="1"/>
-    <col min="18" max="18" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.77734375"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="7.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="17" max="17" customWidth="true" width="17.6640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="13.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -14145,28 +14209,28 @@
   <dimension ref="A1:W10"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="93.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.21875" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" customWidth="1"/>
-    <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="93.88671875"/>
+    <col min="2" max="2" customWidth="true" width="13.21875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.21875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.21875"/>
+    <col min="6" max="6" customWidth="true" width="11.6640625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="9.21875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="6.21875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="8.5546875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="18.6640625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="18.6640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.6640625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="18.6640625"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="14.109375"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="14.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -14525,8 +14589,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="32.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -14574,8 +14638,8 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="48.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="48.88671875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="11.44140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -14739,23 +14803,23 @@
   <dimension ref="A1:P75"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="24.88671875" style="27" customWidth="1"/>
-    <col min="2" max="2" width="14" style="27" customWidth="1"/>
-    <col min="3" max="3" width="11.77734375" style="27" customWidth="1"/>
-    <col min="4" max="4" width="9.5546875" style="27" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" style="27" customWidth="1"/>
-    <col min="6" max="6" width="9.33203125" style="27" customWidth="1"/>
-    <col min="7" max="7" width="9.77734375" style="27" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" style="27" customWidth="1"/>
-    <col min="9" max="9" width="8.77734375" style="27" customWidth="1"/>
-    <col min="10" max="10" width="8.109375" style="37" customWidth="1"/>
-    <col min="11" max="11" width="10" style="27" customWidth="1"/>
-    <col min="12" max="12" width="7.77734375" style="27" customWidth="1"/>
-    <col min="13" max="13" width="9" style="27" customWidth="1"/>
-    <col min="14" max="14" width="19.44140625" style="27" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.77734375" style="27"/>
-    <col min="16" max="16" width="14.77734375" style="27" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.77734375" style="27"/>
+    <col min="1" max="1" customWidth="true" style="27" width="24.88671875"/>
+    <col min="2" max="2" customWidth="true" style="27" width="14.0"/>
+    <col min="3" max="3" customWidth="true" style="27" width="11.77734375"/>
+    <col min="4" max="4" customWidth="true" style="27" width="9.5546875"/>
+    <col min="5" max="5" customWidth="true" style="27" width="10.33203125"/>
+    <col min="6" max="6" customWidth="true" style="27" width="9.33203125"/>
+    <col min="7" max="7" customWidth="true" style="27" width="9.77734375"/>
+    <col min="8" max="8" customWidth="true" style="27" width="10.44140625"/>
+    <col min="9" max="9" customWidth="true" style="27" width="8.77734375"/>
+    <col min="10" max="10" customWidth="true" style="37" width="8.109375"/>
+    <col min="11" max="11" customWidth="true" style="27" width="10.0"/>
+    <col min="12" max="12" customWidth="true" style="27" width="7.77734375"/>
+    <col min="13" max="13" customWidth="true" style="27" width="9.0"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="27" width="19.44140625"/>
+    <col min="15" max="15" style="27" width="8.77734375"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="27" width="14.77734375"/>
+    <col min="17" max="16384" style="27" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -18361,17 +18425,17 @@
   <dimension ref="A1:Q20"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="39.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.44140625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="21.77734375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="6.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="18.33203125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -19166,18 +19230,18 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="32.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" customWidth="1"/>
-    <col min="5" max="5" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.109375" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="4" max="4" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="17.33203125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="13" max="13" customWidth="true" width="15.109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -19350,7 +19414,7 @@
       <c r="H6" s="40"/>
       <c r="I6" s="40"/>
       <c r="J6" s="40" t="s">
-        <v>464</v>
+        <v>1265</v>
       </c>
       <c r="K6" s="40"/>
       <c r="L6" s="40"/>
@@ -19369,30 +19433,30 @@
   <dimension ref="A1:W5"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="19.88671875" style="27" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" style="37" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.77734375" style="37" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" style="37" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.77734375" style="37" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="27" customWidth="1"/>
-    <col min="9" max="9" width="16.5546875" style="27" customWidth="1"/>
-    <col min="10" max="10" width="14.109375" style="27" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.33203125" style="37" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.33203125" style="37" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" style="27"/>
-    <col min="14" max="14" width="12.5546875" style="27" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.77734375" style="27" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.21875" style="27" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5546875" style="37" customWidth="1"/>
-    <col min="18" max="18" width="8.77734375" style="37" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.88671875" style="27" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12" style="27" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.77734375" style="27"/>
-    <col min="22" max="22" width="10.6640625" style="27" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.88671875" style="27" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="8.77734375" style="27"/>
+    <col min="1" max="1" customWidth="true" style="27" width="19.88671875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="37" width="10.88671875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="37" width="9.44140625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="37" width="7.77734375"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="37" width="10.88671875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="37" width="9.44140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="37" width="7.77734375"/>
+    <col min="8" max="8" customWidth="true" style="27" width="13.0"/>
+    <col min="9" max="9" customWidth="true" style="27" width="16.5546875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="27" width="14.109375"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="37" width="10.33203125"/>
+    <col min="12" max="12" customWidth="true" style="37" width="10.33203125"/>
+    <col min="13" max="13" style="27" width="8.77734375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="27" width="12.5546875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="27" width="14.77734375"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="27" width="13.21875"/>
+    <col min="17" max="17" customWidth="true" style="37" width="11.5546875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="37" width="8.77734375"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="27" width="9.88671875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="27" width="12.0"/>
+    <col min="21" max="21" style="27" width="8.77734375"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="27" width="10.6640625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="27" width="13.88671875"/>
+    <col min="24" max="16384" style="27" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -19684,19 +19748,19 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="19.88671875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.33203125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.33203125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="17.33203125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -19799,20 +19863,20 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="25.77734375" style="37" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="37" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" style="37" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" style="37" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.33203125" style="37" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.44140625" style="37" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.33203125" style="37" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.21875" style="37" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="25.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="37" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="37" width="17.33203125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="37" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="37" width="17.33203125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="37" width="4.44140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="37" width="17.33203125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="37" width="14.21875"/>
+    <col min="14" max="16384" style="37" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -19938,21 +20002,21 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="20.21875" style="37" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="37" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" style="37" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="17.33203125" style="37" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" style="37" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.33203125" style="37" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.44140625" style="37" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.33203125" style="37" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.21875" style="37" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="20.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="37" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="37" width="17.33203125"/>
+    <col min="6" max="7" customWidth="true" style="37" width="17.33203125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="37" width="15.0"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="37" width="17.33203125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="37" width="4.44140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="37" width="17.33203125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="37" width="14.21875"/>
+    <col min="16" max="16384" style="37" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -20139,22 +20203,22 @@
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="28.33203125" style="37" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="37" customWidth="1"/>
-    <col min="4" max="4" width="11.21875" style="37" customWidth="1"/>
-    <col min="5" max="5" width="12.77734375" style="37" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" style="37" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" style="37" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" style="37" customWidth="1"/>
-    <col min="10" max="10" width="11.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5546875" style="37" customWidth="1"/>
-    <col min="12" max="12" width="10.77734375" style="37" customWidth="1"/>
-    <col min="13" max="13" width="12.21875" style="37" customWidth="1"/>
-    <col min="14" max="14" width="12.6640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.21875" style="37" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="28.33203125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="3" max="3" customWidth="true" style="37" width="10.33203125"/>
+    <col min="4" max="4" customWidth="true" style="37" width="11.21875"/>
+    <col min="5" max="5" customWidth="true" style="37" width="12.77734375"/>
+    <col min="6" max="6" customWidth="true" style="37" width="12.44140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="37" width="11.109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="9" max="9" customWidth="true" style="37" width="9.109375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="37" width="11.88671875"/>
+    <col min="11" max="11" customWidth="true" style="37" width="11.5546875"/>
+    <col min="12" max="12" customWidth="true" style="37" width="10.77734375"/>
+    <col min="13" max="13" customWidth="true" style="37" width="12.21875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="37" width="12.6640625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="37" width="14.21875"/>
+    <col min="16" max="16384" style="37" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -20485,11 +20549,11 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="24" style="37" customWidth="1"/>
-    <col min="2" max="2" width="11.44140625" style="37" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="37"/>
-    <col min="4" max="4" width="19.6640625" style="37" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="24.0"/>
+    <col min="2" max="2" customWidth="true" style="37" width="11.44140625"/>
+    <col min="3" max="3" style="37" width="8.88671875"/>
+    <col min="4" max="4" customWidth="true" style="37" width="19.6640625"/>
+    <col min="5" max="16384" style="37" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -20547,12 +20611,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="32.21875" style="37" customWidth="1"/>
-    <col min="2" max="2" width="14" style="37" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" style="37" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" style="37" customWidth="1"/>
-    <col min="5" max="5" width="11.77734375" style="37" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="32.21875"/>
+    <col min="2" max="2" customWidth="true" style="37" width="14.0"/>
+    <col min="3" max="3" customWidth="true" style="37" width="16.6640625"/>
+    <col min="4" max="4" customWidth="true" style="37" width="17.6640625"/>
+    <col min="5" max="5" customWidth="true" style="37" width="11.77734375"/>
+    <col min="6" max="16384" style="37" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -20636,11 +20700,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="38.21875" style="37" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="37" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" style="37" customWidth="1"/>
-    <col min="4" max="4" width="19" style="37" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="38.21875"/>
+    <col min="2" max="2" customWidth="true" style="37" width="13.5546875"/>
+    <col min="3" max="3" customWidth="true" style="37" width="15.5546875"/>
+    <col min="4" max="4" customWidth="true" style="37" width="19.0"/>
+    <col min="5" max="16384" style="37" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -20763,23 +20827,23 @@
   <dimension ref="A1:S5"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="30.88671875" style="37" customWidth="1"/>
-    <col min="2" max="2" width="17.77734375" style="37" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" style="37" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" style="37" customWidth="1"/>
-    <col min="5" max="5" width="12" style="37" customWidth="1"/>
-    <col min="6" max="6" width="18.109375" style="37" customWidth="1"/>
-    <col min="7" max="7" width="15.109375" style="37" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" style="37" customWidth="1"/>
-    <col min="9" max="9" width="10.77734375" style="37" customWidth="1"/>
-    <col min="10" max="10" width="8.88671875" style="37"/>
-    <col min="11" max="11" width="13.21875" style="37" customWidth="1"/>
-    <col min="12" max="12" width="12.6640625" style="37" customWidth="1"/>
-    <col min="13" max="13" width="14.109375" style="37" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" style="37" customWidth="1"/>
-    <col min="15" max="18" width="8.88671875" style="37"/>
-    <col min="19" max="19" width="18.33203125" style="37" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="8.88671875" style="37"/>
+    <col min="1" max="1" customWidth="true" style="37" width="30.88671875"/>
+    <col min="2" max="2" customWidth="true" style="37" width="17.77734375"/>
+    <col min="3" max="3" customWidth="true" style="37" width="16.44140625"/>
+    <col min="4" max="4" customWidth="true" style="37" width="16.109375"/>
+    <col min="5" max="5" customWidth="true" style="37" width="12.0"/>
+    <col min="6" max="6" customWidth="true" style="37" width="18.109375"/>
+    <col min="7" max="7" customWidth="true" style="37" width="15.109375"/>
+    <col min="8" max="8" customWidth="true" style="37" width="10.44140625"/>
+    <col min="9" max="9" customWidth="true" style="37" width="10.77734375"/>
+    <col min="10" max="10" style="37" width="8.88671875"/>
+    <col min="11" max="11" customWidth="true" style="37" width="13.21875"/>
+    <col min="12" max="12" customWidth="true" style="37" width="12.6640625"/>
+    <col min="13" max="13" customWidth="true" style="37" width="14.109375"/>
+    <col min="14" max="14" customWidth="true" style="37" width="14.33203125"/>
+    <col min="15" max="18" style="37" width="8.88671875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="37" width="18.33203125"/>
+    <col min="20" max="16384" style="37" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -21069,12 +21133,12 @@
   <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="39.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.44140625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.77734375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="16.109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -21764,11 +21828,11 @@
   <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="57.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="57.44140625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="15.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.77734375"/>
+    <col min="4" max="5" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="20.109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -22019,28 +22083,28 @@
   <dimension ref="A1:W15"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="50" style="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.33203125" style="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.109375" style="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" style="25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" style="25" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="8.77734375" style="25"/>
-    <col min="9" max="9" width="10.44140625" style="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.6640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" style="25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.21875" style="25" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.44140625" style="25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.21875" style="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13" style="25" customWidth="1"/>
-    <col min="16" max="16" width="10.21875" style="25" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.44140625" style="25" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.21875" style="25" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.6640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.6640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.21875" style="25" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="12.6640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="8.77734375" style="25"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="50.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="25" width="18.33203125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="25" width="12.109375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="25" width="15.33203125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="25" width="12.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="25" width="9.44140625"/>
+    <col min="7" max="8" style="25" width="8.77734375"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="25" width="10.44140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="25" width="12.6640625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="25" width="10.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="25" width="11.21875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="10.44140625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="8.21875"/>
+    <col min="15" max="15" customWidth="true" style="25" width="13.0"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="10.21875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="25" width="10.44140625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="25" width="9.21875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="25" width="11.6640625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="25" width="12.6640625"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="25" width="11.21875"/>
+    <col min="22" max="23" bestFit="true" customWidth="true" style="25" width="12.6640625"/>
+    <col min="24" max="16384" style="25" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -22760,29 +22824,29 @@
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="44.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="44.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.77734375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="8.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="13.5546875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.77734375"/>
+    <col min="11" max="12" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.21875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="7.77734375"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="8.21875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="14.21875"/>
+    <col min="27" max="28" bestFit="true" customWidth="true" width="12.77734375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="14.21875"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="12.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -23214,10 +23278,10 @@
   <dimension ref="A1:AJ40"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="54.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="54.33203125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="13.77734375"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="12.109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36">
@@ -25607,17 +25671,17 @@
   <dimension ref="A1:V18"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="53.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="12.21875" customWidth="1"/>
-    <col min="8" max="8" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="53.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="4" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="5" max="7" customWidth="true" width="12.21875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="11.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">

</xml_diff>

<commit_message>
05 Aug 2024 - Merged Sowmya and Harshitha code for Extent reports.
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4321" uniqueCount="1269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4327" uniqueCount="1272">
   <si>
     <t>Scenario</t>
   </si>
@@ -3881,6 +3881,15 @@
   </si>
   <si>
     <t>2024-08-05T08:14:00</t>
+  </si>
+  <si>
+    <t>QHBTLY</t>
+  </si>
+  <si>
+    <t>2024-08-06T18:24:00</t>
+  </si>
+  <si>
+    <t>2024-08-06T23:13:00</t>
   </si>
 </sst>
 </file>
@@ -14081,16 +14090,16 @@
       <c r="I4" s="40"/>
       <c r="J4" s="40"/>
       <c r="K4" s="40" t="s">
-        <v>860</v>
+        <v>1269</v>
       </c>
       <c r="L4" s="40" t="s">
-        <v>852</v>
+        <v>1270</v>
       </c>
       <c r="M4" s="40" t="s">
         <v>465</v>
       </c>
       <c r="N4" s="40" t="s">
-        <v>853</v>
+        <v>1271</v>
       </c>
       <c r="O4" s="40" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Extent Report added, AdvancedPassenger Module rectified for wrong extent loggers
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4327" uniqueCount="1272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4392" uniqueCount="1306">
   <si>
     <t>Scenario</t>
   </si>
@@ -3890,6 +3890,108 @@
   </si>
   <si>
     <t>2024-08-06T23:13:00</t>
+  </si>
+  <si>
+    <t>QHF2RD</t>
+  </si>
+  <si>
+    <t>QHF2YA</t>
+  </si>
+  <si>
+    <t>QHF20H</t>
+  </si>
+  <si>
+    <t>QHF24C</t>
+  </si>
+  <si>
+    <t>QHF3B1</t>
+  </si>
+  <si>
+    <t>QHF3FA</t>
+  </si>
+  <si>
+    <t>QHF3IR</t>
+  </si>
+  <si>
+    <t>QHF3O5</t>
+  </si>
+  <si>
+    <t>QHF3V2</t>
+  </si>
+  <si>
+    <t>QHF3ZU</t>
+  </si>
+  <si>
+    <t>QHF311</t>
+  </si>
+  <si>
+    <t>QHF4CD</t>
+  </si>
+  <si>
+    <t>QHF4II</t>
+  </si>
+  <si>
+    <t>QHF4MQ</t>
+  </si>
+  <si>
+    <t>QHF4R5</t>
+  </si>
+  <si>
+    <t>QHF4YG</t>
+  </si>
+  <si>
+    <t>QHF421</t>
+  </si>
+  <si>
+    <t>QHF5DM</t>
+  </si>
+  <si>
+    <t>QHF5HW</t>
+  </si>
+  <si>
+    <t>QHF5MI</t>
+  </si>
+  <si>
+    <t>QHGB0S</t>
+  </si>
+  <si>
+    <t>QHGB4P</t>
+  </si>
+  <si>
+    <t>QHGCCX</t>
+  </si>
+  <si>
+    <t>QHGCHF</t>
+  </si>
+  <si>
+    <t>2024-08-07T12:12:00</t>
+  </si>
+  <si>
+    <t>QHGCMH</t>
+  </si>
+  <si>
+    <t>QHGCR1</t>
+  </si>
+  <si>
+    <t>QHGDDD</t>
+  </si>
+  <si>
+    <t>QHGDJO</t>
+  </si>
+  <si>
+    <t>QHGDNQ</t>
+  </si>
+  <si>
+    <t>2024-08-05T17:19:05</t>
+  </si>
+  <si>
+    <t>QHGECO</t>
+  </si>
+  <si>
+    <t>QHGEFG</t>
+  </si>
+  <si>
+    <t>QHGEJS</t>
   </si>
 </sst>
 </file>
@@ -5030,7 +5132,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="108" t="s">
-        <v>1204</v>
+        <v>1281</v>
       </c>
       <c r="I2" s="108" t="s">
         <v>199</v>
@@ -5047,7 +5149,7 @@
       <c r="M2" s="108"/>
       <c r="N2" s="108"/>
       <c r="O2" s="108" t="s">
-        <v>822</v>
+        <v>1282</v>
       </c>
       <c r="P2" s="108"/>
       <c r="Q2" s="108"/>
@@ -5087,7 +5189,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="108" t="s">
-        <v>1205</v>
+        <v>1273</v>
       </c>
       <c r="I3" s="108" t="s">
         <v>200</v>
@@ -5146,7 +5248,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="35" t="s">
-        <v>1206</v>
+        <v>1284</v>
       </c>
       <c r="I4" s="35" t="s">
         <v>324</v>
@@ -5201,7 +5303,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="35" t="s">
-        <v>1207</v>
+        <v>1290</v>
       </c>
       <c r="I5" s="108" t="s">
         <v>200</v>
@@ -5258,7 +5360,7 @@
       </c>
       <c r="G6" s="108"/>
       <c r="H6" s="108" t="s">
-        <v>1208</v>
+        <v>1288</v>
       </c>
       <c r="I6" s="108" t="s">
         <v>590</v>
@@ -5311,7 +5413,7 @@
       </c>
       <c r="G7" s="108"/>
       <c r="H7" s="108" t="s">
-        <v>1209</v>
+        <v>1275</v>
       </c>
       <c r="I7" s="108" t="s">
         <v>593</v>
@@ -5360,7 +5462,7 @@
       </c>
       <c r="G8" s="108"/>
       <c r="H8" s="108" t="s">
-        <v>825</v>
+        <v>1291</v>
       </c>
       <c r="I8" s="108" t="s">
         <v>596</v>
@@ -5413,7 +5515,7 @@
       </c>
       <c r="G9" s="108"/>
       <c r="H9" s="108" t="s">
-        <v>1210</v>
+        <v>1287</v>
       </c>
       <c r="I9" s="108" t="s">
         <v>599</v>
@@ -5466,7 +5568,7 @@
       </c>
       <c r="G10" s="108"/>
       <c r="H10" s="108" t="s">
-        <v>1211</v>
+        <v>1286</v>
       </c>
       <c r="I10" s="108" t="s">
         <v>602</v>
@@ -5529,7 +5631,7 @@
       </c>
       <c r="G11" s="108"/>
       <c r="H11" s="108" t="s">
-        <v>824</v>
+        <v>1289</v>
       </c>
       <c r="I11" s="108" t="s">
         <v>330</v>
@@ -5637,7 +5739,7 @@
       </c>
       <c r="G13" s="108"/>
       <c r="H13" s="108" t="s">
-        <v>821</v>
+        <v>1277</v>
       </c>
       <c r="I13" s="108" t="s">
         <v>612</v>
@@ -5692,7 +5794,7 @@
       </c>
       <c r="G14" s="108"/>
       <c r="H14" s="108" t="s">
-        <v>1212</v>
+        <v>1278</v>
       </c>
       <c r="I14" s="108" t="s">
         <v>616</v>
@@ -5747,7 +5849,7 @@
       </c>
       <c r="G15" s="108"/>
       <c r="H15" s="108" t="s">
-        <v>839</v>
+        <v>1285</v>
       </c>
       <c r="I15" s="108" t="s">
         <v>620</v>
@@ -5800,7 +5902,7 @@
       </c>
       <c r="G16" s="108"/>
       <c r="H16" s="108" t="s">
-        <v>820</v>
+        <v>1276</v>
       </c>
       <c r="I16" s="108" t="s">
         <v>623</v>
@@ -5849,7 +5951,7 @@
       </c>
       <c r="G17" s="108"/>
       <c r="H17" s="108" t="s">
-        <v>819</v>
+        <v>1274</v>
       </c>
       <c r="I17" s="108"/>
       <c r="J17" s="108"/>
@@ -5894,7 +5996,7 @@
       </c>
       <c r="G18" s="108"/>
       <c r="H18" s="108" t="s">
-        <v>823</v>
+        <v>1283</v>
       </c>
       <c r="I18" s="108" t="s">
         <v>20</v>
@@ -5943,7 +6045,7 @@
       </c>
       <c r="G19" s="108"/>
       <c r="H19" s="108" t="s">
-        <v>1213</v>
+        <v>1279</v>
       </c>
       <c r="I19" s="108"/>
       <c r="J19" s="108"/>
@@ -6008,7 +6110,7 @@
       </c>
       <c r="G20" s="108"/>
       <c r="H20" s="108" t="s">
-        <v>1214</v>
+        <v>1280</v>
       </c>
       <c r="I20" s="108"/>
       <c r="J20" s="108"/>
@@ -18523,7 +18625,7 @@
         <v>46</v>
       </c>
       <c r="H2" s="40" t="s">
-        <v>868</v>
+        <v>1293</v>
       </c>
       <c r="I2" s="40" t="s">
         <v>354</v>
@@ -18560,7 +18662,7 @@
         <v>46</v>
       </c>
       <c r="H3" s="40" t="s">
-        <v>871</v>
+        <v>1297</v>
       </c>
       <c r="I3" s="40" t="s">
         <v>354</v>
@@ -18597,7 +18699,7 @@
         <v>15</v>
       </c>
       <c r="H4" s="40" t="s">
-        <v>969</v>
+        <v>1292</v>
       </c>
       <c r="I4" s="40"/>
       <c r="J4" s="43" t="s">
@@ -18735,7 +18837,7 @@
         <v>1</v>
       </c>
       <c r="H8" s="40" t="s">
-        <v>973</v>
+        <v>1295</v>
       </c>
       <c r="I8" s="40"/>
       <c r="J8" s="43" t="s">
@@ -18756,7 +18858,7 @@
       </c>
       <c r="P8" s="40"/>
       <c r="Q8" s="40" t="s">
-        <v>972</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -18780,14 +18882,14 @@
       </c>
       <c r="G9" s="40"/>
       <c r="H9" s="40" t="s">
-        <v>974</v>
+        <v>1303</v>
       </c>
       <c r="I9" s="40" t="s">
         <v>754</v>
       </c>
       <c r="J9" s="40"/>
       <c r="K9" s="40" t="s">
-        <v>975</v>
+        <v>752</v>
       </c>
       <c r="L9" s="40"/>
       <c r="M9" s="40"/>
@@ -18817,7 +18919,7 @@
       </c>
       <c r="G10" s="40"/>
       <c r="H10" s="40" t="s">
-        <v>976</v>
+        <v>1304</v>
       </c>
       <c r="I10" s="40" t="s">
         <v>845</v>
@@ -18854,7 +18956,7 @@
       </c>
       <c r="G11" s="40"/>
       <c r="H11" s="40" t="s">
-        <v>978</v>
+        <v>1305</v>
       </c>
       <c r="I11" s="40" t="s">
         <v>977</v>
@@ -19022,7 +19124,7 @@
       </c>
       <c r="G15" s="40"/>
       <c r="H15" s="40" t="s">
-        <v>983</v>
+        <v>1299</v>
       </c>
       <c r="I15" s="40" t="s">
         <v>843</v>
@@ -19059,7 +19161,7 @@
       </c>
       <c r="G16" s="40"/>
       <c r="H16" s="40" t="s">
-        <v>984</v>
+        <v>1300</v>
       </c>
       <c r="I16" s="40" t="s">
         <v>844</v>
@@ -19098,10 +19200,10 @@
       </c>
       <c r="G17" s="40"/>
       <c r="H17" s="40" t="s">
-        <v>985</v>
+        <v>1301</v>
       </c>
       <c r="I17" s="40" t="s">
-        <v>986</v>
+        <v>1302</v>
       </c>
       <c r="J17" s="43" t="s">
         <v>731</v>
@@ -19137,7 +19239,7 @@
         <v>46</v>
       </c>
       <c r="H18" s="40" t="s">
-        <v>869</v>
+        <v>1294</v>
       </c>
       <c r="I18" s="40" t="s">
         <v>870</v>
@@ -19174,7 +19276,7 @@
         <v>46</v>
       </c>
       <c r="H19" s="40" t="s">
-        <v>872</v>
+        <v>1298</v>
       </c>
       <c r="I19" s="40" t="s">
         <v>873</v>

</xml_diff>

<commit_message>
Assertions added for prerequisites for Checkin module (Issue and createbooking)
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4230" uniqueCount="1257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4239" uniqueCount="1260">
   <si>
     <t>Scenario</t>
   </si>
@@ -3844,6 +3844,15 @@
   </si>
   <si>
     <t>BJSOK3</t>
+  </si>
+  <si>
+    <t>BJVECV</t>
+  </si>
+  <si>
+    <t>BJVENA</t>
+  </si>
+  <si>
+    <t>BJVES0</t>
   </si>
 </sst>
 </file>
@@ -20616,7 +20625,7 @@
         <v>15</v>
       </c>
       <c r="H2" s="28" t="s">
-        <v>1226</v>
+        <v>1257</v>
       </c>
       <c r="I2" s="28" t="s">
         <v>197</v>
@@ -20782,7 +20791,7 @@
         <v>15</v>
       </c>
       <c r="H6" s="28" t="s">
-        <v>1228</v>
+        <v>1258</v>
       </c>
       <c r="I6" s="28" t="s">
         <v>730</v>
@@ -20917,7 +20926,7 @@
         <v>15</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>1229</v>
+        <v>1259</v>
       </c>
       <c r="I9" s="28" t="s">
         <v>1225</v>

</xml_diff>

<commit_message>
All wrong assertions for CreateBooking Module corrected. Missing Assertions in creatBooking module added
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4239" uniqueCount="1260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1264">
   <si>
     <t>Scenario</t>
   </si>
@@ -3853,6 +3853,18 @@
   </si>
   <si>
     <t>BJVES0</t>
+  </si>
+  <si>
+    <t>BKBWZG</t>
+  </si>
+  <si>
+    <t>2302187043589</t>
+  </si>
+  <si>
+    <t>BKBXTS</t>
+  </si>
+  <si>
+    <t>2302187043623</t>
   </si>
 </sst>
 </file>
@@ -21403,10 +21415,10 @@
       <c r="P2" s="38"/>
       <c r="Q2" s="38"/>
       <c r="R2" s="38" t="s">
-        <v>1236</v>
+        <v>1260</v>
       </c>
       <c r="S2" s="38" t="s">
-        <v>1237</v>
+        <v>1261</v>
       </c>
       <c r="T2" s="38"/>
       <c r="U2" s="38"/>
@@ -21781,10 +21793,10 @@
       <c r="P8" s="38"/>
       <c r="Q8" s="38"/>
       <c r="R8" s="38" t="s">
-        <v>800</v>
+        <v>1262</v>
       </c>
       <c r="S8" s="38" t="s">
-        <v>801</v>
+        <v>1263</v>
       </c>
       <c r="T8" s="38">
         <v>0</v>

</xml_diff>

<commit_message>
AirInventory Service Assertions modified based on excel
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{740D47A0-0523-449F-813A-70E278FE46D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D094E751-432F-4878-9FBE-E63B04A51B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4241" uniqueCount="1262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4273" uniqueCount="1274">
   <si>
     <t>Scenario</t>
   </si>
@@ -2838,9 +2838,6 @@
     <t>6-PR360/27SEPPTY.INIT#SEAT</t>
   </si>
   <si>
-    <t>BPVSYY</t>
-  </si>
-  <si>
     <t>ArrivalDate</t>
   </si>
   <si>
@@ -3585,9 +3582,6 @@
     <t>QHF20H</t>
   </si>
   <si>
-    <t>QHF24C</t>
-  </si>
-  <si>
     <t>QHF3B1</t>
   </si>
   <si>
@@ -3600,27 +3594,12 @@
     <t>QHF311</t>
   </si>
   <si>
-    <t>QHF4CD</t>
-  </si>
-  <si>
     <t>QHF4MQ</t>
   </si>
   <si>
     <t>QHF4R5</t>
   </si>
   <si>
-    <t>QHF4YG</t>
-  </si>
-  <si>
-    <t>QHF421</t>
-  </si>
-  <si>
-    <t>QHF5HW</t>
-  </si>
-  <si>
-    <t>QHF5MI</t>
-  </si>
-  <si>
     <t>QHGB0S</t>
   </si>
   <si>
@@ -3690,9 +3669,6 @@
     <t>QHIBXD</t>
   </si>
   <si>
-    <t>QHIEQF</t>
-  </si>
-  <si>
     <t>CA5093D8CMCMRPCT051C7DBC09</t>
   </si>
   <si>
@@ -3807,15 +3783,6 @@
     <t>BS1GVQ</t>
   </si>
   <si>
-    <t>AHPWO0</t>
-  </si>
-  <si>
-    <t>AHPWO3</t>
-  </si>
-  <si>
-    <t>AHPWP0</t>
-  </si>
-  <si>
     <t>QMTMPL</t>
   </si>
   <si>
@@ -3859,6 +3826,75 @@
   </si>
   <si>
     <t>QAY1L4</t>
+  </si>
+  <si>
+    <t>QBBYDY</t>
+  </si>
+  <si>
+    <t>QBBYQK</t>
+  </si>
+  <si>
+    <t>QBBYXF</t>
+  </si>
+  <si>
+    <t>QBBZ0N</t>
+  </si>
+  <si>
+    <t>QBB0I1</t>
+  </si>
+  <si>
+    <t>QBB0VQ</t>
+  </si>
+  <si>
+    <t>QBB05V</t>
+  </si>
+  <si>
+    <t>QBB1FK</t>
+  </si>
+  <si>
+    <t>QBB1OM</t>
+  </si>
+  <si>
+    <t>QBB1XW</t>
+  </si>
+  <si>
+    <t>QBCI3N</t>
+  </si>
+  <si>
+    <t>QBCJWU</t>
+  </si>
+  <si>
+    <t>QBCKAV</t>
+  </si>
+  <si>
+    <t>QBCKK4</t>
+  </si>
+  <si>
+    <t>QBCKY2</t>
+  </si>
+  <si>
+    <t>QBCK1C</t>
+  </si>
+  <si>
+    <t>QBCLVP</t>
+  </si>
+  <si>
+    <t>QBCL5I</t>
+  </si>
+  <si>
+    <t>QBCMFV</t>
+  </si>
+  <si>
+    <t>QBCMP3</t>
+  </si>
+  <si>
+    <t>QBCMYU</t>
+  </si>
+  <si>
+    <t>QBCM22</t>
+  </si>
+  <si>
+    <t>QBCNGW</t>
   </si>
 </sst>
 </file>
@@ -4867,7 +4903,7 @@
     <col min="4" max="4" bestFit="true" customWidth="true" width="15.453125"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="12.1796875"/>
     <col min="6" max="6" bestFit="true" customWidth="true" width="9.453125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="8.1796875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="8.453125"/>
     <col min="9" max="9" bestFit="true" customWidth="true" width="17.54296875"/>
     <col min="10" max="10" bestFit="true" customWidth="true" width="11.1796875"/>
     <col min="11" max="11" bestFit="true" customWidth="true" width="10.453125"/>
@@ -4975,16 +5011,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="107" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D2" s="106" t="s">
         <v>12</v>
       </c>
       <c r="E2" s="106" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="F2" s="106" t="s">
         <v>14</v>
@@ -4993,7 +5029,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="106" t="s">
-        <v>1247</v>
+        <v>1265</v>
       </c>
       <c r="I2" s="106" t="s">
         <v>197</v>
@@ -5010,7 +5046,7 @@
       <c r="M2" s="106"/>
       <c r="N2" s="106"/>
       <c r="O2" s="106" t="s">
-        <v>1174</v>
+        <v>1266</v>
       </c>
       <c r="P2" s="106"/>
       <c r="Q2" s="106"/>
@@ -5032,16 +5068,16 @@
         <v>17</v>
       </c>
       <c r="B3" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" s="107" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D3" s="106" t="s">
         <v>12</v>
       </c>
       <c r="E3" s="106" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="F3" s="106" t="s">
         <v>14</v>
@@ -5050,7 +5086,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="106" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="I3" s="106" t="s">
         <v>198</v>
@@ -5091,16 +5127,16 @@
         <v>320</v>
       </c>
       <c r="B4" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" s="107" t="s">
-        <v>725</v>
+        <v>28</v>
       </c>
       <c r="D4" s="106" t="s">
         <v>12</v>
       </c>
       <c r="E4" s="106" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="F4" s="106" t="s">
         <v>14</v>
@@ -5109,7 +5145,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="33" t="s">
-        <v>1205</v>
+        <v>1267</v>
       </c>
       <c r="I4" s="33" t="s">
         <v>321</v>
@@ -5146,16 +5182,16 @@
         <v>319</v>
       </c>
       <c r="B5" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="107" t="s">
-        <v>725</v>
+        <v>28</v>
       </c>
       <c r="D5" s="106" t="s">
         <v>12</v>
       </c>
       <c r="E5" s="106" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="F5" s="106" t="s">
         <v>14</v>
@@ -5164,7 +5200,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="33" t="s">
-        <v>1180</v>
+        <v>1272</v>
       </c>
       <c r="I5" s="106" t="s">
         <v>198</v>
@@ -5205,23 +5241,23 @@
         <v>578</v>
       </c>
       <c r="B6" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" s="107" t="s">
-        <v>725</v>
+        <v>28</v>
       </c>
       <c r="D6" s="106" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="106" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="F6" s="106" t="s">
         <v>14</v>
       </c>
       <c r="G6" s="106"/>
       <c r="H6" s="106" t="s">
-        <v>1179</v>
+        <v>1270</v>
       </c>
       <c r="I6" s="106" t="s">
         <v>579</v>
@@ -5258,23 +5294,23 @@
         <v>581</v>
       </c>
       <c r="B7" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="107" t="s">
-        <v>725</v>
+        <v>28</v>
       </c>
       <c r="D7" s="106" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="106" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="F7" s="106" t="s">
         <v>14</v>
       </c>
       <c r="G7" s="106"/>
       <c r="H7" s="106" t="s">
-        <v>1170</v>
+        <v>1262</v>
       </c>
       <c r="I7" s="106" t="s">
         <v>582</v>
@@ -5307,23 +5343,23 @@
         <v>584</v>
       </c>
       <c r="B8" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" s="107" t="s">
-        <v>725</v>
+        <v>28</v>
       </c>
       <c r="D8" s="106" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="106" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="F8" s="106" t="s">
         <v>14</v>
       </c>
       <c r="G8" s="106"/>
       <c r="H8" s="106" t="s">
-        <v>1181</v>
+        <v>1273</v>
       </c>
       <c r="I8" s="106" t="s">
         <v>585</v>
@@ -5360,23 +5396,23 @@
         <v>587</v>
       </c>
       <c r="B9" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" s="107" t="s">
-        <v>725</v>
+        <v>28</v>
       </c>
       <c r="D9" s="106" t="s">
         <v>12</v>
       </c>
       <c r="E9" s="106" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="F9" s="106" t="s">
         <v>14</v>
       </c>
       <c r="G9" s="106"/>
       <c r="H9" s="106" t="s">
-        <v>1178</v>
+        <v>1269</v>
       </c>
       <c r="I9" s="106" t="s">
         <v>588</v>
@@ -5413,23 +5449,23 @@
         <v>590</v>
       </c>
       <c r="B10" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C10" s="107" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D10" s="106" t="s">
         <v>12</v>
       </c>
       <c r="E10" s="106" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="F10" s="106" t="s">
         <v>14</v>
       </c>
       <c r="G10" s="106"/>
       <c r="H10" s="106" t="s">
-        <v>1177</v>
+        <v>1268</v>
       </c>
       <c r="I10" s="106" t="s">
         <v>591</v>
@@ -5476,10 +5512,10 @@
         <v>595</v>
       </c>
       <c r="B11" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" s="107" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="D11" s="106" t="s">
         <v>43</v>
@@ -5492,7 +5528,7 @@
       </c>
       <c r="G11" s="106"/>
       <c r="H11" s="106" t="s">
-        <v>1246</v>
+        <v>1271</v>
       </c>
       <c r="I11" s="106" t="s">
         <v>326</v>
@@ -5529,7 +5565,7 @@
         <v>597</v>
       </c>
       <c r="B12" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="107" t="s">
         <v>28</v>
@@ -5584,10 +5620,10 @@
         <v>600</v>
       </c>
       <c r="B13" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13" s="107" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="D13" s="106" t="s">
         <v>43</v>
@@ -5600,7 +5636,7 @@
       </c>
       <c r="G13" s="106"/>
       <c r="H13" s="106" t="s">
-        <v>1244</v>
+        <v>1263</v>
       </c>
       <c r="I13" s="106" t="s">
         <v>601</v>
@@ -5639,10 +5675,10 @@
         <v>603</v>
       </c>
       <c r="B14" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="107" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="D14" s="106" t="s">
         <v>12</v>
@@ -5655,7 +5691,7 @@
       </c>
       <c r="G14" s="106"/>
       <c r="H14" s="106" t="s">
-        <v>1245</v>
+        <v>1264</v>
       </c>
       <c r="I14" s="106" t="s">
         <v>605</v>
@@ -5694,7 +5730,7 @@
         <v>608</v>
       </c>
       <c r="B15" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" s="107" t="s">
         <v>42</v>
@@ -5710,7 +5746,7 @@
       </c>
       <c r="G15" s="106"/>
       <c r="H15" s="106" t="s">
-        <v>1176</v>
+        <v>1173</v>
       </c>
       <c r="I15" s="106" t="s">
         <v>609</v>
@@ -5747,7 +5783,7 @@
         <v>611</v>
       </c>
       <c r="B16" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" s="107" t="s">
         <v>59</v>
@@ -5763,7 +5799,7 @@
       </c>
       <c r="G16" s="106"/>
       <c r="H16" s="106" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="I16" s="106" t="s">
         <v>612</v>
@@ -5796,7 +5832,7 @@
         <v>614</v>
       </c>
       <c r="B17" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" s="107" t="s">
         <v>59</v>
@@ -5812,7 +5848,7 @@
       </c>
       <c r="G17" s="106"/>
       <c r="H17" s="106" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="I17" s="106"/>
       <c r="J17" s="106"/>
@@ -5841,7 +5877,7 @@
         <v>615</v>
       </c>
       <c r="B18" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" s="107" t="s">
         <v>28</v>
@@ -5857,7 +5893,7 @@
       </c>
       <c r="G18" s="106"/>
       <c r="H18" s="106" t="s">
-        <v>1175</v>
+        <v>1254</v>
       </c>
       <c r="I18" s="106" t="s">
         <v>20</v>
@@ -5890,7 +5926,7 @@
         <v>616</v>
       </c>
       <c r="B19" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" s="107" t="s">
         <v>564</v>
@@ -5906,7 +5942,7 @@
       </c>
       <c r="G19" s="106"/>
       <c r="H19" s="106" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
       <c r="I19" s="106"/>
       <c r="J19" s="106"/>
@@ -5921,7 +5957,7 @@
         <v>-10</v>
       </c>
       <c r="S19" s="107" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="T19" s="106" t="s">
         <v>314</v>
@@ -5955,10 +5991,10 @@
         <v>617</v>
       </c>
       <c r="B20" s="106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" s="107" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="D20" s="106" t="s">
         <v>12</v>
@@ -5971,7 +6007,7 @@
       </c>
       <c r="G20" s="106"/>
       <c r="H20" s="106" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
       <c r="I20" s="106"/>
       <c r="J20" s="106"/>
@@ -5986,7 +6022,7 @@
         <v>-8</v>
       </c>
       <c r="S20" s="107" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="T20" s="106" t="s">
         <v>618</v>
@@ -6001,7 +6037,7 @@
         <v>-8</v>
       </c>
       <c r="X20" s="107" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="Y20" s="106" t="s">
         <v>12</v>
@@ -6257,13 +6293,13 @@
         <v>3</v>
       </c>
       <c r="C2" s="38" t="s">
-        <v>1208</v>
+        <v>1200</v>
       </c>
       <c r="D2" s="41" t="s">
-        <v>1209</v>
+        <v>1201</v>
       </c>
       <c r="E2" s="41" t="s">
-        <v>1207</v>
+        <v>1199</v>
       </c>
       <c r="F2" s="38"/>
       <c r="G2" s="41" t="s">
@@ -6292,7 +6328,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="41" t="s">
-        <v>1210</v>
+        <v>1202</v>
       </c>
       <c r="E3" s="41" t="s">
         <v>249</v>
@@ -6328,7 +6364,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="41" t="s">
-        <v>1206</v>
+        <v>1198</v>
       </c>
       <c r="E4" s="38"/>
       <c r="F4" s="38" t="s">
@@ -6477,28 +6513,28 @@
         <v>4</v>
       </c>
       <c r="AE1" s="37" t="s">
+        <v>954</v>
+      </c>
+      <c r="AF1" s="37" t="s">
         <v>955</v>
       </c>
-      <c r="AF1" s="37" t="s">
+      <c r="AG1" s="37" t="s">
         <v>956</v>
       </c>
-      <c r="AG1" s="37" t="s">
+      <c r="AH1" s="37" t="s">
         <v>957</v>
       </c>
-      <c r="AH1" s="37" t="s">
+      <c r="AI1" s="37" t="s">
         <v>958</v>
       </c>
-      <c r="AI1" s="37" t="s">
+      <c r="AJ1" s="37" t="s">
         <v>959</v>
       </c>
-      <c r="AJ1" s="37" t="s">
+      <c r="AK1" s="37" t="s">
         <v>960</v>
       </c>
-      <c r="AK1" s="37" t="s">
+      <c r="AL1" s="37" t="s">
         <v>961</v>
-      </c>
-      <c r="AL1" s="37" t="s">
-        <v>962</v>
       </c>
     </row>
     <row r="2" spans="1:38">
@@ -6763,7 +6799,7 @@
     </row>
     <row r="7" spans="1:38">
       <c r="A7" s="48" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B7" s="38"/>
       <c r="C7" s="38">
@@ -6781,13 +6817,13 @@
         <v>12</v>
       </c>
       <c r="I7" s="38" t="s">
+        <v>963</v>
+      </c>
+      <c r="J7" s="38" t="s">
         <v>964</v>
       </c>
-      <c r="J7" s="38" t="s">
+      <c r="K7" s="38" t="s">
         <v>965</v>
-      </c>
-      <c r="K7" s="38" t="s">
-        <v>966</v>
       </c>
       <c r="L7" s="38"/>
       <c r="M7" s="38"/>
@@ -6819,7 +6855,7 @@
     </row>
     <row r="8" spans="1:38">
       <c r="A8" s="38" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B8" s="38"/>
       <c r="C8" s="38">
@@ -6837,10 +6873,10 @@
         <v>30</v>
       </c>
       <c r="I8" s="38" t="s">
+        <v>967</v>
+      </c>
+      <c r="J8" s="38" t="s">
         <v>968</v>
-      </c>
-      <c r="J8" s="38" t="s">
-        <v>969</v>
       </c>
       <c r="K8" s="38"/>
       <c r="L8" s="38"/>
@@ -6877,7 +6913,7 @@
     </row>
     <row r="9" spans="1:38">
       <c r="A9" s="38" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B9" s="38"/>
       <c r="C9" s="38">
@@ -6895,13 +6931,13 @@
         <v>30</v>
       </c>
       <c r="I9" s="38" t="s">
+        <v>970</v>
+      </c>
+      <c r="J9" s="38" t="s">
         <v>971</v>
       </c>
-      <c r="J9" s="38" t="s">
+      <c r="K9" s="38" t="s">
         <v>972</v>
-      </c>
-      <c r="K9" s="38" t="s">
-        <v>973</v>
       </c>
       <c r="L9" s="38"/>
       <c r="M9" s="38"/>
@@ -6934,7 +6970,7 @@
         <v>9</v>
       </c>
       <c r="X9" s="41" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="Y9" s="38" t="s">
         <v>314</v>
@@ -6965,7 +7001,7 @@
     </row>
     <row r="10" spans="1:38">
       <c r="A10" s="38" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B10" s="38"/>
       <c r="C10" s="38">
@@ -6983,13 +7019,13 @@
         <v>30</v>
       </c>
       <c r="I10" s="38" t="s">
+        <v>975</v>
+      </c>
+      <c r="J10" s="38" t="s">
         <v>976</v>
       </c>
-      <c r="J10" s="38" t="s">
+      <c r="K10" s="38" t="s">
         <v>977</v>
-      </c>
-      <c r="K10" s="38" t="s">
-        <v>978</v>
       </c>
       <c r="L10" s="38"/>
       <c r="M10" s="38"/>
@@ -7022,7 +7058,7 @@
         <v>9</v>
       </c>
       <c r="X10" s="41" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="Y10" s="38" t="s">
         <v>314</v>
@@ -7053,7 +7089,7 @@
     </row>
     <row r="11" spans="1:38">
       <c r="A11" s="48" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="B11" s="38"/>
       <c r="C11" s="38"/>
@@ -7095,7 +7131,7 @@
     </row>
     <row r="12" spans="1:38">
       <c r="A12" s="48" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="B12" s="38"/>
       <c r="C12" s="38"/>
@@ -7106,10 +7142,10 @@
       <c r="H12" s="38"/>
       <c r="I12" s="38"/>
       <c r="J12" s="93" t="s">
+        <v>980</v>
+      </c>
+      <c r="K12" s="41" t="s">
         <v>981</v>
-      </c>
-      <c r="K12" s="41" t="s">
-        <v>982</v>
       </c>
       <c r="L12" s="38"/>
       <c r="M12" s="38"/>
@@ -7131,33 +7167,33 @@
       <c r="AC12" s="38"/>
       <c r="AD12" s="38"/>
       <c r="AE12" s="41" t="s">
+        <v>982</v>
+      </c>
+      <c r="AF12" s="41" t="s">
         <v>983</v>
       </c>
-      <c r="AF12" s="41" t="s">
+      <c r="AG12" s="41" t="s">
         <v>984</v>
       </c>
-      <c r="AG12" s="41" t="s">
+      <c r="AH12" s="41" t="s">
         <v>985</v>
       </c>
-      <c r="AH12" s="41" t="s">
+      <c r="AI12" s="41" t="s">
         <v>986</v>
       </c>
-      <c r="AI12" s="41" t="s">
+      <c r="AJ12" s="41" t="s">
         <v>987</v>
       </c>
-      <c r="AJ12" s="41" t="s">
+      <c r="AK12" s="41" t="s">
         <v>988</v>
       </c>
-      <c r="AK12" s="41" t="s">
+      <c r="AL12" s="41" t="s">
         <v>989</v>
-      </c>
-      <c r="AL12" s="41" t="s">
-        <v>990</v>
       </c>
     </row>
     <row r="13" spans="1:38">
       <c r="A13" s="48" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="B13" s="38"/>
       <c r="C13" s="38"/>
@@ -7168,7 +7204,7 @@
       <c r="H13" s="38"/>
       <c r="I13" s="38"/>
       <c r="J13" s="41" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="K13" s="38"/>
       <c r="L13" s="38"/>
@@ -7201,7 +7237,7 @@
     </row>
     <row r="14" spans="1:38">
       <c r="A14" s="48" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="B14" s="38"/>
       <c r="C14" s="38"/>
@@ -7212,7 +7248,7 @@
       <c r="H14" s="38"/>
       <c r="I14" s="38"/>
       <c r="J14" s="41" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="K14" s="38"/>
       <c r="L14" s="38"/>
@@ -7478,7 +7514,7 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="48" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="B8" s="38"/>
       <c r="C8" s="38"/>
@@ -7499,7 +7535,7 @@
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="84" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="B9" s="38"/>
       <c r="C9" s="38"/>
@@ -7522,7 +7558,7 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="85" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="B10" s="38"/>
       <c r="C10" s="38" t="s">
@@ -7549,7 +7585,7 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="84" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="B11" s="38"/>
       <c r="C11" s="38" t="s">
@@ -7576,7 +7612,7 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="84" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="B12" s="38"/>
       <c r="C12" s="38" t="s">
@@ -7601,7 +7637,7 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="48" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="B13" s="38"/>
       <c r="C13" s="38" t="s">
@@ -7622,7 +7658,7 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="48" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="B14" s="38"/>
       <c r="C14" s="38" t="s">
@@ -7645,7 +7681,7 @@
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="86" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="B15" s="38"/>
       <c r="C15" s="38" t="s">
@@ -7656,7 +7692,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="41" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="G15" s="38" t="s">
         <v>12</v>
@@ -7667,12 +7703,12 @@
       <c r="K15" s="38"/>
       <c r="L15" s="38"/>
       <c r="M15" s="87" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="88" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="B16" s="38"/>
       <c r="C16" s="38" t="s">
@@ -7695,7 +7731,7 @@
     </row>
     <row r="17" spans="1:13">
       <c r="A17" s="84" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="B17" s="38"/>
       <c r="C17" s="38" t="s">
@@ -7718,13 +7754,13 @@
       <c r="J17" s="38"/>
       <c r="K17" s="38"/>
       <c r="L17" s="92" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="M17" s="38"/>
     </row>
     <row r="18" spans="1:13">
       <c r="A18" s="85" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="B18" s="38"/>
       <c r="C18" s="38" t="s">
@@ -7735,7 +7771,7 @@
         <v>2</v>
       </c>
       <c r="F18" s="89" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="G18" s="38" t="s">
         <v>487</v>
@@ -7747,13 +7783,13 @@
       <c r="J18" s="38"/>
       <c r="K18" s="38"/>
       <c r="L18" s="92" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="M18" s="38"/>
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="84" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="B19" s="38"/>
       <c r="C19" s="38" t="s">
@@ -7764,7 +7800,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="41" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="G19" s="38" t="s">
         <v>12</v>
@@ -7776,17 +7812,17 @@
       <c r="J19" s="38"/>
       <c r="K19" s="38"/>
       <c r="L19" s="92" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="M19" s="38"/>
     </row>
     <row r="20" spans="1:13">
       <c r="A20" s="88" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="B20" s="38"/>
       <c r="C20" s="38" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="D20" s="38"/>
       <c r="E20" s="38">
@@ -7805,7 +7841,7 @@
     </row>
     <row r="21" spans="1:13">
       <c r="A21" s="48" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="B21" s="38"/>
       <c r="C21" s="38" t="s">
@@ -7824,13 +7860,13 @@
       <c r="J21" s="38"/>
       <c r="K21" s="38"/>
       <c r="L21" s="90" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="M21" s="38"/>
     </row>
     <row r="22" spans="1:13">
       <c r="A22" s="86" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B22" s="38"/>
       <c r="C22" s="38" t="s">
@@ -7841,7 +7877,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="41" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="G22" s="38"/>
       <c r="H22" s="38"/>
@@ -7849,13 +7885,13 @@
       <c r="J22" s="38"/>
       <c r="K22" s="38"/>
       <c r="L22" s="90" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="M22" s="38"/>
     </row>
     <row r="23" spans="1:13">
       <c r="A23" s="48" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="B23" s="38"/>
       <c r="C23" s="38" t="s">
@@ -7874,13 +7910,13 @@
       <c r="J23" s="38"/>
       <c r="K23" s="38"/>
       <c r="L23" s="91" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="M23" s="38"/>
     </row>
     <row r="24" spans="1:13">
       <c r="A24" s="48" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B24" s="38"/>
       <c r="C24" s="38" t="s">
@@ -7905,7 +7941,7 @@
     </row>
     <row r="25" spans="1:13">
       <c r="A25" s="48" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="B25" s="38"/>
       <c r="C25" s="38" t="s">
@@ -8168,16 +8204,16 @@
       <c r="H4" s="38"/>
       <c r="I4" s="38"/>
       <c r="J4" s="38" t="s">
-        <v>1214</v>
+        <v>1206</v>
       </c>
       <c r="K4" s="38" t="s">
-        <v>1213</v>
+        <v>1205</v>
       </c>
       <c r="L4" s="38" t="s">
         <v>621</v>
       </c>
       <c r="M4" s="38" t="s">
-        <v>1212</v>
+        <v>1204</v>
       </c>
       <c r="N4" s="38" t="s">
         <v>621</v>
@@ -8212,16 +8248,16 @@
       <c r="H5" s="38"/>
       <c r="I5" s="38"/>
       <c r="J5" s="38" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="K5" s="38" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="L5" s="38" t="s">
         <v>621</v>
       </c>
       <c r="M5" s="38" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="N5" s="38" t="s">
         <v>621</v>
@@ -8264,16 +8300,16 @@
         <v>30</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>1211</v>
+        <v>1203</v>
       </c>
       <c r="K6" s="38" t="s">
-        <v>1213</v>
+        <v>1205</v>
       </c>
       <c r="L6" s="38" t="s">
         <v>621</v>
       </c>
       <c r="M6" s="38" t="s">
-        <v>1212</v>
+        <v>1204</v>
       </c>
       <c r="N6" s="38" t="s">
         <v>621</v>
@@ -8947,19 +8983,19 @@
         <v>100</v>
       </c>
       <c r="C1" s="36" t="s">
+        <v>1120</v>
+      </c>
+      <c r="D1" s="96" t="s">
         <v>1121</v>
       </c>
-      <c r="D1" s="96" t="s">
+      <c r="E1" s="36" t="s">
         <v>1122</v>
-      </c>
-      <c r="E1" s="36" t="s">
-        <v>1123</v>
       </c>
       <c r="F1" s="36" t="s">
         <v>251</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -8990,7 +9026,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="38" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="B4" s="38" t="s">
         <v>175</v>
@@ -9003,19 +9039,19 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="38" t="s">
+        <v>1116</v>
+      </c>
+      <c r="B5" s="38" t="s">
         <v>1117</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="C5" s="38" t="s">
         <v>1118</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="D5" s="38" t="s">
+        <v>1161</v>
+      </c>
+      <c r="E5" s="38" t="s">
         <v>1119</v>
-      </c>
-      <c r="D5" s="38" t="s">
-        <v>1162</v>
-      </c>
-      <c r="E5" s="38" t="s">
-        <v>1120</v>
       </c>
       <c r="F5" s="38" t="s">
         <v>139</v>
@@ -9169,7 +9205,7 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3" s="38" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="B3" s="38">
         <v>1</v>
@@ -9216,7 +9252,7 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4" s="38" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="B4" s="38">
         <v>2</v>
@@ -9251,15 +9287,15 @@
       <c r="X4" s="38"/>
       <c r="Y4" s="38"/>
       <c r="Z4" s="41" t="s">
+        <v>1107</v>
+      </c>
+      <c r="AA4" s="38" t="s">
         <v>1108</v>
-      </c>
-      <c r="AA4" s="38" t="s">
-        <v>1109</v>
       </c>
     </row>
     <row r="5" spans="1:27">
       <c r="A5" s="38" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B5" s="38">
         <v>1</v>
@@ -9306,7 +9342,7 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6" s="38" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B6" s="38">
         <v>1</v>
@@ -9345,7 +9381,7 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7" s="38" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="B7" s="38">
         <v>1</v>
@@ -9424,7 +9460,7 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8" s="38" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="B8" s="38">
         <v>1</v>
@@ -9463,7 +9499,7 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9" s="38" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="B9" s="38">
         <v>1</v>
@@ -9499,7 +9535,7 @@
       <c r="Y9" s="38"/>
       <c r="Z9" s="38"/>
       <c r="AA9" s="95" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
     </row>
   </sheetData>
@@ -10513,7 +10549,7 @@
       <c r="I9" s="38"/>
       <c r="J9" s="38"/>
       <c r="K9" s="38" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>407</v>
@@ -10522,7 +10558,7 @@
         <v>300</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>195</v>
@@ -10753,7 +10789,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="66" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="D2" s="66" t="s">
         <v>12</v>
@@ -10798,7 +10834,7 @@
         <v>-7</v>
       </c>
       <c r="C3" s="66" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="D3" s="66" t="s">
         <v>12</v>
@@ -11077,7 +11113,7 @@
         <v>3</v>
       </c>
       <c r="C8" s="66" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="D8" s="67" t="s">
         <v>487</v>
@@ -12027,7 +12063,7 @@
         <v>246</v>
       </c>
       <c r="K1" s="36" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -12131,12 +12167,12 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="62" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="B7" s="38"/>
       <c r="C7" s="38"/>
       <c r="D7" s="38" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="E7" s="38"/>
       <c r="F7" s="38"/>
@@ -12148,7 +12184,7 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="48" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B8" s="38"/>
       <c r="C8" s="38" t="s">
@@ -12165,11 +12201,11 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="48" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="B9" s="38"/>
       <c r="C9" s="90" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="D9" s="38"/>
       <c r="E9" s="38"/>
@@ -12182,7 +12218,7 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="48" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="B10" s="38"/>
       <c r="C10" s="38"/>
@@ -12197,12 +12233,12 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="48" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="B11" s="38"/>
       <c r="C11" s="38"/>
       <c r="D11" s="90" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="E11" s="90" t="s">
         <v>113</v>
@@ -12211,10 +12247,10 @@
         <v>109</v>
       </c>
       <c r="G11" s="90" t="s">
+        <v>1002</v>
+      </c>
+      <c r="H11" s="90" t="s">
         <v>1003</v>
-      </c>
-      <c r="H11" s="90" t="s">
-        <v>1004</v>
       </c>
       <c r="I11" s="38"/>
       <c r="J11" s="38"/>
@@ -12222,7 +12258,7 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="48" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="B12" s="38"/>
       <c r="C12" s="38"/>
@@ -12233,15 +12269,15 @@
       <c r="H12" s="38"/>
       <c r="I12" s="38"/>
       <c r="J12" s="38" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="K12" s="41" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="48" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="B13" s="38"/>
       <c r="C13" s="38"/>
@@ -12258,7 +12294,7 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="48" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="B14" s="38"/>
       <c r="C14" s="38"/>
@@ -12275,7 +12311,7 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="48" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B15" s="38"/>
       <c r="C15" s="38"/>
@@ -12292,7 +12328,7 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="86" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="B16" s="38"/>
       <c r="C16" s="38"/>
@@ -12511,16 +12547,16 @@
       <c r="I4" s="38"/>
       <c r="J4" s="38"/>
       <c r="K4" s="38" t="s">
+        <v>1164</v>
+      </c>
+      <c r="L4" s="38" t="s">
         <v>1165</v>
-      </c>
-      <c r="L4" s="38" t="s">
-        <v>1166</v>
       </c>
       <c r="M4" s="38" t="s">
         <v>457</v>
       </c>
       <c r="N4" s="38" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="O4" s="38" t="s">
         <v>12</v>
@@ -12870,13 +12906,13 @@
     </row>
     <row r="4" spans="1:23">
       <c r="A4" s="106" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="B4" s="106">
         <v>1</v>
       </c>
       <c r="C4" s="107" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="D4" s="106" t="s">
         <v>12</v>
@@ -12897,7 +12933,7 @@
         <v>153</v>
       </c>
       <c r="J4" s="106" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="K4" s="106"/>
       <c r="L4" s="106"/>
@@ -12919,7 +12955,7 @@
     </row>
     <row r="5" spans="1:23">
       <c r="A5" s="106" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="B5" s="106"/>
       <c r="C5" s="106"/>
@@ -12948,7 +12984,7 @@
     </row>
     <row r="6" spans="1:23">
       <c r="A6" s="106" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="B6" s="106">
         <v>1</v>
@@ -12967,7 +13003,7 @@
       <c r="H6" s="106"/>
       <c r="I6" s="106"/>
       <c r="J6" s="106" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="K6" s="106"/>
       <c r="L6" s="106"/>
@@ -12980,7 +13016,7 @@
       <c r="S6" s="106"/>
       <c r="T6" s="106"/>
       <c r="U6" s="87" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="V6" s="106"/>
       <c r="W6" s="106" t="s">
@@ -13126,13 +13162,13 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="106" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="B4" s="106" t="s">
         <v>139</v>
       </c>
       <c r="C4" s="106" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="D4" s="106"/>
       <c r="E4" s="106"/>
@@ -13140,13 +13176,13 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="108" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="B5" s="109" t="s">
         <v>139</v>
       </c>
       <c r="C5" s="109" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="D5" s="106" t="s">
         <v>142</v>
@@ -13156,13 +13192,13 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="108" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="B6" s="109" t="s">
         <v>139</v>
       </c>
       <c r="C6" s="109" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="D6" s="106"/>
       <c r="E6" s="106" t="s">
@@ -13172,25 +13208,25 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="108" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="B7" s="109" t="s">
         <v>139</v>
       </c>
       <c r="C7" s="109" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="D7" s="106" t="s">
         <v>142</v>
       </c>
       <c r="E7" s="107" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="F7" s="106"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="106" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="B8" s="109" t="s">
         <v>139</v>
@@ -13210,7 +13246,7 @@
         <v>139</v>
       </c>
       <c r="C9" s="106" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="D9" s="106" t="s">
         <v>142</v>
@@ -13299,7 +13335,7 @@
         <v>25</v>
       </c>
       <c r="P1" s="36" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -14040,7 +14076,7 @@
     </row>
     <row r="18" spans="1:16">
       <c r="A18" s="38" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="B18" s="38" t="s">
         <v>139</v>
@@ -14052,7 +14088,7 @@
         <v>111</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="F18" s="38" t="s">
         <v>429</v>
@@ -14070,7 +14106,7 @@
         <v>436</v>
       </c>
       <c r="K18" s="38" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="L18" s="38" t="s">
         <v>430</v>
@@ -14090,7 +14126,7 @@
     </row>
     <row r="19" spans="1:16">
       <c r="A19" s="38" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="B19" s="38" t="s">
         <v>139</v>
@@ -14102,7 +14138,7 @@
         <v>111</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="F19" s="38" t="s">
         <v>425</v>
@@ -14120,7 +14156,7 @@
         <v>436</v>
       </c>
       <c r="K19" s="38" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="L19" s="38" t="s">
         <v>425</v>
@@ -14140,7 +14176,7 @@
     </row>
     <row r="20" spans="1:16">
       <c r="A20" s="38" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="B20" s="38" t="s">
         <v>139</v>
@@ -14152,7 +14188,7 @@
         <v>111</v>
       </c>
       <c r="E20" s="38" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="F20" s="38" t="s">
         <v>429</v>
@@ -14170,7 +14206,7 @@
         <v>436</v>
       </c>
       <c r="K20" s="38" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="L20" s="38" t="s">
         <v>430</v>
@@ -14190,7 +14226,7 @@
     </row>
     <row r="21" spans="1:16">
       <c r="A21" s="38" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="B21" s="38" t="s">
         <v>139</v>
@@ -14202,16 +14238,16 @@
         <v>111</v>
       </c>
       <c r="E21" s="38" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F21" s="38" t="s">
         <v>1022</v>
-      </c>
-      <c r="F21" s="38" t="s">
-        <v>1023</v>
       </c>
       <c r="G21" s="38" t="s">
         <v>309</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="I21" s="38" t="s">
         <v>436</v>
@@ -14240,7 +14276,7 @@
     </row>
     <row r="22" spans="1:16">
       <c r="A22" s="38" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="B22" s="38" t="s">
         <v>139</v>
@@ -14252,7 +14288,7 @@
         <v>111</v>
       </c>
       <c r="E22" s="38" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="F22" s="38" t="s">
         <v>415</v>
@@ -14261,7 +14297,7 @@
         <v>309</v>
       </c>
       <c r="H22" s="38" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="I22" s="38" t="s">
         <v>436</v>
@@ -14290,7 +14326,7 @@
     </row>
     <row r="23" spans="1:16">
       <c r="A23" s="38" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="B23" s="38" t="s">
         <v>139</v>
@@ -14302,7 +14338,7 @@
         <v>111</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="F23" s="38" t="s">
         <v>415</v>
@@ -14311,7 +14347,7 @@
         <v>309</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="I23" s="38" t="s">
         <v>436</v>
@@ -14340,7 +14376,7 @@
     </row>
     <row r="24" spans="1:16">
       <c r="A24" s="38" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="B24" s="38" t="s">
         <v>139</v>
@@ -14361,16 +14397,16 @@
         <v>309</v>
       </c>
       <c r="H24" s="38" t="s">
+        <v>1031</v>
+      </c>
+      <c r="I24" s="38" t="s">
+        <v>436</v>
+      </c>
+      <c r="J24" s="38" t="s">
+        <v>436</v>
+      </c>
+      <c r="K24" s="38" t="s">
         <v>1032</v>
-      </c>
-      <c r="I24" s="38" t="s">
-        <v>436</v>
-      </c>
-      <c r="J24" s="38" t="s">
-        <v>436</v>
-      </c>
-      <c r="K24" s="38" t="s">
-        <v>1033</v>
       </c>
       <c r="L24" s="38" t="s">
         <v>429</v>
@@ -14390,7 +14426,7 @@
     </row>
     <row r="25" spans="1:16">
       <c r="A25" s="38" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="B25" s="38" t="s">
         <v>139</v>
@@ -14402,7 +14438,7 @@
         <v>111</v>
       </c>
       <c r="E25" s="38" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="F25" s="38" t="s">
         <v>425</v>
@@ -14440,7 +14476,7 @@
     </row>
     <row r="26" spans="1:16">
       <c r="A26" s="38" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="B26" s="38" t="s">
         <v>139</v>
@@ -14452,16 +14488,16 @@
         <v>111</v>
       </c>
       <c r="E26" s="38" t="s">
+        <v>1036</v>
+      </c>
+      <c r="F26" s="38" t="s">
         <v>1037</v>
-      </c>
-      <c r="F26" s="38" t="s">
-        <v>1038</v>
       </c>
       <c r="G26" s="38" t="s">
         <v>309</v>
       </c>
       <c r="H26" s="38" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="I26" s="38" t="s">
         <v>436</v>
@@ -14473,7 +14509,7 @@
         <v>430</v>
       </c>
       <c r="L26" s="38" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="M26" s="38" t="s">
         <v>436</v>
@@ -14490,7 +14526,7 @@
     </row>
     <row r="27" spans="1:16">
       <c r="A27" s="38" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="B27" s="38" t="s">
         <v>139</v>
@@ -14540,7 +14576,7 @@
     </row>
     <row r="28" spans="1:16">
       <c r="A28" s="38" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B28" s="38" t="s">
         <v>139</v>
@@ -14552,7 +14588,7 @@
         <v>111</v>
       </c>
       <c r="E28" s="38" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="F28" s="38" t="s">
         <v>415</v>
@@ -14561,7 +14597,7 @@
         <v>309</v>
       </c>
       <c r="H28" s="38" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="I28" s="38" t="s">
         <v>436</v>
@@ -14590,7 +14626,7 @@
     </row>
     <row r="29" spans="1:16">
       <c r="A29" s="38" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="B29" s="38" t="s">
         <v>139</v>
@@ -14602,7 +14638,7 @@
         <v>111</v>
       </c>
       <c r="E29" s="38" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="F29" s="38" t="s">
         <v>415</v>
@@ -14611,7 +14647,7 @@
         <v>309</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="I29" s="38" t="s">
         <v>436</v>
@@ -14640,7 +14676,7 @@
     </row>
     <row r="30" spans="1:16">
       <c r="A30" s="38" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B30" s="38" t="s">
         <v>139</v>
@@ -14652,7 +14688,7 @@
         <v>111</v>
       </c>
       <c r="E30" s="38" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="F30" s="38" t="s">
         <v>415</v>
@@ -14690,7 +14726,7 @@
     </row>
     <row r="31" spans="1:16">
       <c r="A31" s="38" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B31" s="38" t="s">
         <v>139</v>
@@ -14738,7 +14774,7 @@
     </row>
     <row r="32" spans="1:16">
       <c r="A32" s="38" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B32" s="38" t="s">
         <v>139</v>
@@ -14788,7 +14824,7 @@
     </row>
     <row r="33" spans="1:16">
       <c r="A33" s="38" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="B33" s="38" t="s">
         <v>139</v>
@@ -14838,7 +14874,7 @@
     </row>
     <row r="34" spans="1:16">
       <c r="A34" s="38" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B34" s="38" t="s">
         <v>139</v>
@@ -14888,7 +14924,7 @@
     </row>
     <row r="35" spans="1:16">
       <c r="A35" s="38" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="B35" s="38" t="s">
         <v>139</v>
@@ -14938,7 +14974,7 @@
     </row>
     <row r="36" spans="1:16">
       <c r="A36" s="38" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B36" s="38" t="s">
         <v>139</v>
@@ -14980,7 +15016,7 @@
         <v>436</v>
       </c>
       <c r="O36" s="38" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="P36" s="38" t="s">
         <v>436</v>
@@ -14988,7 +15024,7 @@
     </row>
     <row r="37" spans="1:16">
       <c r="A37" s="38" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="B37" s="38" t="s">
         <v>139</v>
@@ -15038,7 +15074,7 @@
     </row>
     <row r="38" spans="1:16">
       <c r="A38" s="38" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="B38" s="38" t="s">
         <v>139</v>
@@ -15083,12 +15119,12 @@
         <v>436</v>
       </c>
       <c r="P38" s="38" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="39" spans="1:16">
       <c r="A39" s="38" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="B39" s="38" t="s">
         <v>139</v>
@@ -15130,7 +15166,7 @@
         <v>436</v>
       </c>
       <c r="O39" s="38" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="P39" s="38" t="s">
         <v>436</v>
@@ -15138,7 +15174,7 @@
     </row>
     <row r="40" spans="1:16">
       <c r="A40" s="38" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B40" s="38" t="s">
         <v>139</v>
@@ -15183,12 +15219,12 @@
         <v>436</v>
       </c>
       <c r="P40" s="38" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="41" spans="1:16">
       <c r="A41" s="38" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="B41" s="38" t="s">
         <v>139</v>
@@ -15230,7 +15266,7 @@
         <v>436</v>
       </c>
       <c r="O41" s="38" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="P41" s="38" t="s">
         <v>436</v>
@@ -15238,7 +15274,7 @@
     </row>
     <row r="42" spans="1:16">
       <c r="A42" s="38" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="B42" s="38" t="s">
         <v>139</v>
@@ -15283,12 +15319,12 @@
         <v>436</v>
       </c>
       <c r="P42" s="38" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="43" spans="1:16">
       <c r="A43" s="38" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="B43" s="38" t="s">
         <v>139</v>
@@ -15330,7 +15366,7 @@
         <v>436</v>
       </c>
       <c r="O43" s="38" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="P43" s="38" t="s">
         <v>436</v>
@@ -15338,7 +15374,7 @@
     </row>
     <row r="44" spans="1:16">
       <c r="A44" s="38" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="B44" s="38" t="s">
         <v>139</v>
@@ -15388,7 +15424,7 @@
     </row>
     <row r="45" spans="1:16">
       <c r="A45" s="38" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="B45" s="38" t="s">
         <v>139</v>
@@ -15430,7 +15466,7 @@
         <v>436</v>
       </c>
       <c r="O45" s="38" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="P45" s="38" t="s">
         <v>436</v>
@@ -15438,7 +15474,7 @@
     </row>
     <row r="46" spans="1:16">
       <c r="A46" s="38" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="B46" s="38" t="s">
         <v>139</v>
@@ -15488,7 +15524,7 @@
     </row>
     <row r="47" spans="1:16">
       <c r="A47" s="38" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="B47" s="38" t="s">
         <v>139</v>
@@ -15538,7 +15574,7 @@
     </row>
     <row r="48" spans="1:16">
       <c r="A48" s="38" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="B48" s="38" t="s">
         <v>139</v>
@@ -15580,7 +15616,7 @@
         <v>436</v>
       </c>
       <c r="O48" s="38" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="P48" s="38" t="s">
         <v>436</v>
@@ -15588,7 +15624,7 @@
     </row>
     <row r="49" spans="1:16">
       <c r="A49" s="38" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B49" s="38" t="s">
         <v>139</v>
@@ -15638,7 +15674,7 @@
     </row>
     <row r="50" spans="1:16">
       <c r="A50" s="38" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="B50" s="38" t="s">
         <v>139</v>
@@ -15683,12 +15719,12 @@
         <v>436</v>
       </c>
       <c r="P50" s="38" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="51" spans="1:16">
       <c r="A51" s="94" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="B51" s="38" t="s">
         <v>139</v>
@@ -15738,7 +15774,7 @@
     </row>
     <row r="52" spans="1:16">
       <c r="A52" s="38" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="B52" s="38" t="s">
         <v>139</v>
@@ -15788,7 +15824,7 @@
     </row>
     <row r="53" spans="1:16">
       <c r="A53" s="38" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="B53" s="38" t="s">
         <v>139</v>
@@ -15833,12 +15869,12 @@
         <v>436</v>
       </c>
       <c r="P53" s="38" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="54" spans="1:16">
       <c r="A54" s="38" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="B54" s="38" t="s">
         <v>139</v>
@@ -15880,7 +15916,7 @@
         <v>436</v>
       </c>
       <c r="O54" s="38" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="P54" s="38" t="s">
         <v>436</v>
@@ -15888,7 +15924,7 @@
     </row>
     <row r="55" spans="1:16">
       <c r="A55" s="38" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="B55" s="38" t="s">
         <v>139</v>
@@ -15938,7 +15974,7 @@
     </row>
     <row r="56" spans="1:16">
       <c r="A56" s="38" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="B56" s="38" t="s">
         <v>139</v>
@@ -15983,12 +16019,12 @@
         <v>436</v>
       </c>
       <c r="P56" s="38" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="57" spans="1:16">
       <c r="A57" s="38" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="B57" s="38" t="s">
         <v>139</v>
@@ -16038,7 +16074,7 @@
     </row>
     <row r="58" spans="1:16">
       <c r="A58" s="38" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="B58" s="38" t="s">
         <v>139</v>
@@ -16088,7 +16124,7 @@
     </row>
     <row r="59" spans="1:16">
       <c r="A59" s="38" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="B59" s="38" t="s">
         <v>139</v>
@@ -16133,12 +16169,12 @@
         <v>436</v>
       </c>
       <c r="P59" s="38" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="60" spans="1:16">
       <c r="A60" s="38" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="B60" s="38" t="s">
         <v>139</v>
@@ -16188,7 +16224,7 @@
     </row>
     <row r="61" spans="1:16">
       <c r="A61" s="38" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="B61" s="38" t="s">
         <v>139</v>
@@ -16238,7 +16274,7 @@
     </row>
     <row r="62" spans="1:16">
       <c r="A62" s="38" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="B62" s="38" t="s">
         <v>139</v>
@@ -16288,7 +16324,7 @@
     </row>
     <row r="63" spans="1:16">
       <c r="A63" s="38" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="B63" s="38" t="s">
         <v>139</v>
@@ -16338,7 +16374,7 @@
     </row>
     <row r="64" spans="1:16">
       <c r="A64" s="38" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="B64" s="38" t="s">
         <v>139</v>
@@ -16380,7 +16416,7 @@
         <v>436</v>
       </c>
       <c r="O64" s="38" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="P64" s="38" t="s">
         <v>436</v>
@@ -16388,7 +16424,7 @@
     </row>
     <row r="65" spans="1:16">
       <c r="A65" s="38" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="B65" s="38" t="s">
         <v>139</v>
@@ -16433,12 +16469,12 @@
         <v>436</v>
       </c>
       <c r="P65" s="38" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="66" spans="1:16">
       <c r="A66" s="38" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="B66" s="38" t="s">
         <v>139</v>
@@ -16483,12 +16519,12 @@
         <v>436</v>
       </c>
       <c r="P66" s="38" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="67" spans="1:16">
       <c r="A67" s="38" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="B67" s="38" t="s">
         <v>139</v>
@@ -16538,7 +16574,7 @@
     </row>
     <row r="68" spans="1:16">
       <c r="A68" s="38" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="B68" s="38" t="s">
         <v>139</v>
@@ -16588,7 +16624,7 @@
     </row>
     <row r="69" spans="1:16">
       <c r="A69" s="38" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="B69" s="38" t="s">
         <v>139</v>
@@ -16638,7 +16674,7 @@
     </row>
     <row r="70" spans="1:16">
       <c r="A70" s="38" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="B70" s="38" t="s">
         <v>139</v>
@@ -16683,12 +16719,12 @@
         <v>436</v>
       </c>
       <c r="P70" s="38" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="71" spans="1:16">
       <c r="A71" s="38" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="B71" s="38" t="s">
         <v>139</v>
@@ -16738,7 +16774,7 @@
     </row>
     <row r="72" spans="1:16">
       <c r="A72" s="38" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="B72" s="38" t="s">
         <v>139</v>
@@ -16780,7 +16816,7 @@
         <v>436</v>
       </c>
       <c r="O72" s="38" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="P72" s="38" t="s">
         <v>436</v>
@@ -16788,7 +16824,7 @@
     </row>
     <row r="73" spans="1:16">
       <c r="A73" s="38" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="B73" s="38" t="s">
         <v>139</v>
@@ -17039,7 +17075,7 @@
       <c r="H6" s="38"/>
       <c r="I6" s="38"/>
       <c r="J6" s="38" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="K6" s="38"/>
       <c r="L6" s="38"/>
@@ -17123,10 +17159,10 @@
         <v>5</v>
       </c>
       <c r="Q1" s="82" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="R1" s="98" t="s">
-        <v>1257</v>
+        <v>1246</v>
       </c>
       <c r="S1" s="98" t="s">
         <v>8</v>
@@ -17158,7 +17194,7 @@
         <v>46</v>
       </c>
       <c r="H2" s="38" t="s">
-        <v>1221</v>
+        <v>1213</v>
       </c>
       <c r="I2" s="38" t="s">
         <v>347</v>
@@ -17198,7 +17234,7 @@
         <v>46</v>
       </c>
       <c r="H3" s="38" t="s">
-        <v>1183</v>
+        <v>1176</v>
       </c>
       <c r="I3" s="38" t="s">
         <v>347</v>
@@ -17238,7 +17274,7 @@
         <v>15</v>
       </c>
       <c r="H4" s="38" t="s">
-        <v>1182</v>
+        <v>1175</v>
       </c>
       <c r="I4" s="38"/>
       <c r="J4" s="41" t="s">
@@ -17318,7 +17354,7 @@
       </c>
       <c r="G6" s="38"/>
       <c r="H6" s="38" t="s">
-        <v>1261</v>
+        <v>1250</v>
       </c>
       <c r="I6" s="38"/>
       <c r="J6" s="41" t="s">
@@ -17332,13 +17368,13 @@
       <c r="P6" s="38"/>
       <c r="Q6" s="38"/>
       <c r="R6" s="107" t="s">
-        <v>1258</v>
+        <v>1247</v>
       </c>
       <c r="S6" s="107" t="s">
-        <v>1259</v>
+        <v>1248</v>
       </c>
       <c r="T6" s="106" t="s">
-        <v>1260</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -17394,7 +17430,7 @@
         <v>15</v>
       </c>
       <c r="H8" s="38" t="s">
-        <v>1248</v>
+        <v>1237</v>
       </c>
       <c r="I8" s="38"/>
       <c r="J8" s="41" t="s">
@@ -17415,7 +17451,7 @@
       </c>
       <c r="P8" s="38"/>
       <c r="Q8" s="38" t="s">
-        <v>1249</v>
+        <v>1238</v>
       </c>
       <c r="R8" s="106"/>
       <c r="S8" s="106"/>
@@ -17442,7 +17478,7 @@
       </c>
       <c r="G9" s="38"/>
       <c r="H9" s="38" t="s">
-        <v>1188</v>
+        <v>1181</v>
       </c>
       <c r="I9" s="38" t="s">
         <v>739</v>
@@ -17482,7 +17518,7 @@
       </c>
       <c r="G10" s="38"/>
       <c r="H10" s="38" t="s">
-        <v>1189</v>
+        <v>1182</v>
       </c>
       <c r="I10" s="38" t="s">
         <v>816</v>
@@ -17522,10 +17558,10 @@
       </c>
       <c r="G11" s="38"/>
       <c r="H11" s="38" t="s">
-        <v>1255</v>
+        <v>1244</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="J11" s="38"/>
       <c r="K11" s="41" t="s">
@@ -17562,7 +17598,7 @@
       </c>
       <c r="G12" s="38"/>
       <c r="H12" s="38" t="s">
-        <v>1251</v>
+        <v>1240</v>
       </c>
       <c r="I12" s="38" t="s">
         <v>740</v>
@@ -17612,10 +17648,10 @@
       </c>
       <c r="G13" s="38"/>
       <c r="H13" s="38" t="s">
-        <v>1252</v>
+        <v>1241</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>1253</v>
+        <v>1242</v>
       </c>
       <c r="J13" s="41" t="s">
         <v>712</v>
@@ -17652,7 +17688,7 @@
       </c>
       <c r="G14" s="38"/>
       <c r="H14" s="38" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="I14" s="38" t="s">
         <v>741</v>
@@ -17702,7 +17738,7 @@
       </c>
       <c r="G15" s="38"/>
       <c r="H15" s="38" t="s">
-        <v>1184</v>
+        <v>1177</v>
       </c>
       <c r="I15" s="38" t="s">
         <v>814</v>
@@ -17742,7 +17778,7 @@
       </c>
       <c r="G16" s="38"/>
       <c r="H16" s="38" t="s">
-        <v>1185</v>
+        <v>1178</v>
       </c>
       <c r="I16" s="38" t="s">
         <v>815</v>
@@ -17784,10 +17820,10 @@
       </c>
       <c r="G17" s="38"/>
       <c r="H17" s="38" t="s">
-        <v>1186</v>
+        <v>1179</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>1187</v>
+        <v>1180</v>
       </c>
       <c r="J17" s="41" t="s">
         <v>719</v>
@@ -17826,7 +17862,7 @@
         <v>46</v>
       </c>
       <c r="H18" s="38" t="s">
-        <v>1256</v>
+        <v>1245</v>
       </c>
       <c r="I18" s="38" t="s">
         <v>837</v>
@@ -17866,7 +17902,7 @@
         <v>46</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>1250</v>
+        <v>1239</v>
       </c>
       <c r="I19" s="38" t="s">
         <v>838</v>
@@ -17906,7 +17942,7 @@
         <v>15</v>
       </c>
       <c r="H20" s="38" t="s">
-        <v>1254</v>
+        <v>1243</v>
       </c>
       <c r="I20" s="38" t="s">
         <v>347</v>
@@ -18072,7 +18108,7 @@
         <v>14</v>
       </c>
       <c r="M2" s="28" t="s">
-        <v>1242</v>
+        <v>1234</v>
       </c>
       <c r="N2" s="28">
         <v>2</v>
@@ -18092,10 +18128,10 @@
       <c r="S2" s="28"/>
       <c r="T2" s="28"/>
       <c r="U2" s="38" t="s">
-        <v>1233</v>
+        <v>1225</v>
       </c>
       <c r="V2" s="38" t="s">
-        <v>1234</v>
+        <v>1226</v>
       </c>
       <c r="W2" s="38" t="s">
         <v>347</v>
@@ -18139,7 +18175,7 @@
         <v>14</v>
       </c>
       <c r="M3" s="28" t="s">
-        <v>1238</v>
+        <v>1230</v>
       </c>
       <c r="N3" s="28"/>
       <c r="O3" s="28"/>
@@ -18150,16 +18186,16 @@
         <v>865</v>
       </c>
       <c r="T3" s="28" t="s">
-        <v>1235</v>
+        <v>1227</v>
       </c>
       <c r="U3" s="38" t="s">
-        <v>1239</v>
+        <v>1231</v>
       </c>
       <c r="V3" s="38" t="s">
-        <v>1240</v>
+        <v>1232</v>
       </c>
       <c r="W3" s="38" t="s">
-        <v>1241</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -18200,7 +18236,7 @@
         <v>14</v>
       </c>
       <c r="M4" s="28" t="s">
-        <v>1243</v>
+        <v>1235</v>
       </c>
       <c r="N4" s="28"/>
       <c r="O4" s="28"/>
@@ -18214,10 +18250,10 @@
       <c r="S4" s="28"/>
       <c r="T4" s="28"/>
       <c r="U4" s="38" t="s">
-        <v>1233</v>
+        <v>1225</v>
       </c>
       <c r="V4" s="38" t="s">
-        <v>1234</v>
+        <v>1226</v>
       </c>
       <c r="W4" s="38" t="s">
         <v>347</v>
@@ -19438,7 +19474,7 @@
         <v>198</v>
       </c>
       <c r="J2" s="38" t="s">
-        <v>1193</v>
+        <v>1186</v>
       </c>
       <c r="K2" s="38">
         <f>B2</f>
@@ -19490,7 +19526,7 @@
         <v>20</v>
       </c>
       <c r="J3" s="38" t="s">
-        <v>1194</v>
+        <v>1187</v>
       </c>
       <c r="K3" s="38"/>
       <c r="L3" s="38" t="s">
@@ -19500,7 +19536,7 @@
         <v>335</v>
       </c>
       <c r="N3" s="38" t="s">
-        <v>1190</v>
+        <v>1183</v>
       </c>
       <c r="O3" s="38" t="s">
         <v>202</v>
@@ -19515,7 +19551,7 @@
         <v>1</v>
       </c>
       <c r="S3" s="38" t="s">
-        <v>1191</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -19547,7 +19583,7 @@
         <v>723</v>
       </c>
       <c r="J4" s="38" t="s">
-        <v>1195</v>
+        <v>1188</v>
       </c>
       <c r="K4" s="38"/>
       <c r="L4" s="38" t="s">
@@ -19557,7 +19593,7 @@
         <v>400</v>
       </c>
       <c r="N4" s="38" t="s">
-        <v>1192</v>
+        <v>1185</v>
       </c>
       <c r="O4" s="38"/>
       <c r="P4" s="38"/>
@@ -19596,7 +19632,7 @@
         <v>907</v>
       </c>
       <c r="J5" s="38" t="s">
-        <v>1196</v>
+        <v>1189</v>
       </c>
       <c r="K5" s="38"/>
       <c r="L5" s="38" t="s">
@@ -19606,7 +19642,7 @@
         <v>335</v>
       </c>
       <c r="N5" s="38" t="s">
-        <v>1190</v>
+        <v>1183</v>
       </c>
       <c r="O5" s="38" t="s">
         <v>202</v>
@@ -19621,7 +19657,7 @@
         <v>1</v>
       </c>
       <c r="S5" s="38" t="s">
-        <v>1191</v>
+        <v>1184</v>
       </c>
     </row>
   </sheetData>
@@ -19866,7 +19902,7 @@
         <v>30</v>
       </c>
       <c r="I9" s="107" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="J9" s="38"/>
     </row>
@@ -20100,7 +20136,7 @@
         <v>30</v>
       </c>
       <c r="E19" s="110" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="F19" s="38"/>
       <c r="G19" s="38"/>
@@ -20117,7 +20153,7 @@
       </c>
       <c r="C20" s="38"/>
       <c r="D20" s="110" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="E20" s="110" t="s">
         <v>497</v>
@@ -20705,7 +20741,7 @@
         <v>15</v>
       </c>
       <c r="H2" s="28" t="s">
-        <v>1236</v>
+        <v>1228</v>
       </c>
       <c r="I2" s="28" t="s">
         <v>197</v>
@@ -20732,7 +20768,7 @@
         <v>327</v>
       </c>
       <c r="S2" s="28" t="s">
-        <v>1237</v>
+        <v>1229</v>
       </c>
       <c r="T2" s="28" t="s">
         <v>411</v>
@@ -20875,7 +20911,7 @@
         <v>15</v>
       </c>
       <c r="H6" s="28" t="s">
-        <v>1222</v>
+        <v>1214</v>
       </c>
       <c r="I6" s="28" t="s">
         <v>723</v>
@@ -20924,7 +20960,7 @@
         <v>19</v>
       </c>
       <c r="H7" s="28" t="s">
-        <v>1198</v>
+        <v>1191</v>
       </c>
       <c r="I7" s="28" t="s">
         <v>329</v>
@@ -21010,10 +21046,10 @@
         <v>15</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>1223</v>
+        <v>1215</v>
       </c>
       <c r="I9" s="28" t="s">
-        <v>1197</v>
+        <v>1190</v>
       </c>
       <c r="J9" s="28" t="s">
         <v>197</v>
@@ -21053,7 +21089,7 @@
       </c>
       <c r="G10" s="50"/>
       <c r="H10" s="28" t="s">
-        <v>1199</v>
+        <v>1192</v>
       </c>
       <c r="I10" s="28"/>
       <c r="J10" s="28" t="s">
@@ -21102,13 +21138,13 @@
         <v>15</v>
       </c>
       <c r="H11" s="28" t="s">
-        <v>1200</v>
+        <v>1193</v>
       </c>
       <c r="I11" s="28" t="s">
         <v>197</v>
       </c>
       <c r="J11" s="28" t="s">
-        <v>1201</v>
+        <v>1194</v>
       </c>
       <c r="K11" s="28"/>
       <c r="L11" s="28"/>
@@ -21296,7 +21332,7 @@
         <v>15</v>
       </c>
       <c r="H15" s="28" t="s">
-        <v>1202</v>
+        <v>1195</v>
       </c>
       <c r="I15" s="28" t="s">
         <v>197</v>
@@ -21449,13 +21485,13 @@
         <v>257</v>
       </c>
       <c r="AK1" s="12" t="s">
-        <v>1216</v>
+        <v>1208</v>
       </c>
       <c r="AL1" s="12" t="s">
-        <v>1217</v>
+        <v>1209</v>
       </c>
       <c r="AM1" s="12" t="s">
-        <v>1215</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="2" spans="1:39">
@@ -21487,10 +21523,10 @@
       <c r="P2" s="38"/>
       <c r="Q2" s="38"/>
       <c r="R2" s="38" t="s">
-        <v>1224</v>
+        <v>1216</v>
       </c>
       <c r="S2" s="38" t="s">
-        <v>1225</v>
+        <v>1217</v>
       </c>
       <c r="T2" s="38"/>
       <c r="U2" s="38"/>
@@ -21865,10 +21901,10 @@
       <c r="P8" s="38"/>
       <c r="Q8" s="38"/>
       <c r="R8" s="38" t="s">
-        <v>1226</v>
+        <v>1218</v>
       </c>
       <c r="S8" s="38" t="s">
-        <v>1227</v>
+        <v>1219</v>
       </c>
       <c r="T8" s="38">
         <v>0</v>
@@ -22341,10 +22377,10 @@
       <c r="P16" s="38"/>
       <c r="Q16" s="38"/>
       <c r="R16" s="38" t="s">
+        <v>1154</v>
+      </c>
+      <c r="S16" s="38" t="s">
         <v>1155</v>
-      </c>
-      <c r="S16" s="38" t="s">
-        <v>1156</v>
       </c>
       <c r="T16" s="38"/>
       <c r="U16" s="38"/>
@@ -22482,13 +22518,13 @@
       <c r="AI18" s="38"/>
       <c r="AJ18" s="38"/>
       <c r="AK18" s="107" t="s">
-        <v>1218</v>
+        <v>1210</v>
       </c>
       <c r="AL18" s="106" t="s">
-        <v>1219</v>
+        <v>1211</v>
       </c>
       <c r="AM18" s="106" t="s">
-        <v>1220</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="19" spans="1:39">
@@ -22544,10 +22580,10 @@
         <v>30</v>
       </c>
       <c r="R19" s="38" t="s">
+        <v>1150</v>
+      </c>
+      <c r="S19" s="38" t="s">
         <v>1151</v>
-      </c>
-      <c r="S19" s="38" t="s">
-        <v>1152</v>
       </c>
       <c r="T19" s="41">
         <v>0</v>
@@ -22650,13 +22686,13 @@
       <c r="AI20" s="38"/>
       <c r="AJ20" s="38"/>
       <c r="AK20" s="107" t="s">
-        <v>1218</v>
+        <v>1210</v>
       </c>
       <c r="AL20" s="106" t="s">
-        <v>1219</v>
+        <v>1211</v>
       </c>
       <c r="AM20" s="106" t="s">
-        <v>1220</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="21" spans="1:39">
@@ -22731,13 +22767,13 @@
       <c r="AI21" s="38"/>
       <c r="AJ21" s="38"/>
       <c r="AK21" s="107" t="s">
-        <v>1218</v>
+        <v>1210</v>
       </c>
       <c r="AL21" s="106" t="s">
-        <v>1219</v>
+        <v>1211</v>
       </c>
       <c r="AM21" s="106" t="s">
-        <v>1220</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="22" spans="1:39">
@@ -22875,7 +22911,7 @@
       <c r="P24" s="38"/>
       <c r="Q24" s="38"/>
       <c r="R24" s="38" t="s">
-        <v>1203</v>
+        <v>1196</v>
       </c>
       <c r="S24" s="38"/>
       <c r="T24" s="41"/>
@@ -23089,7 +23125,7 @@
       <c r="P28" s="38"/>
       <c r="Q28" s="38"/>
       <c r="R28" s="38" t="s">
-        <v>1204</v>
+        <v>1197</v>
       </c>
       <c r="S28" s="38"/>
       <c r="T28" s="41">
@@ -23239,10 +23275,10 @@
       <c r="P30" s="38"/>
       <c r="Q30" s="38"/>
       <c r="R30" s="38" t="s">
+        <v>1152</v>
+      </c>
+      <c r="S30" s="38" t="s">
         <v>1153</v>
-      </c>
-      <c r="S30" s="38" t="s">
-        <v>1154</v>
       </c>
       <c r="T30" s="38">
         <v>0</v>
@@ -24563,7 +24599,7 @@
     </row>
     <row r="18" spans="1:22">
       <c r="A18" s="97" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="B18" s="104">
         <v>1</v>
@@ -24573,7 +24609,7 @@
       </c>
       <c r="D18" s="104"/>
       <c r="E18" s="102" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="F18" s="100"/>
       <c r="G18" s="100"/>
@@ -24596,7 +24632,7 @@
       <c r="T18" s="100"/>
       <c r="U18" s="100"/>
       <c r="V18" s="102" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
   </sheetData>
@@ -24724,7 +24760,7 @@
       </c>
       <c r="J2" s="38"/>
       <c r="K2" s="38" t="s">
-        <v>1232</v>
+        <v>1224</v>
       </c>
       <c r="L2" s="38"/>
       <c r="M2" s="38"/>
@@ -24802,11 +24838,11 @@
       <c r="I4" s="38"/>
       <c r="J4" s="38"/>
       <c r="K4" s="38" t="s">
-        <v>1229</v>
+        <v>1221</v>
       </c>
       <c r="L4" s="38"/>
       <c r="M4" s="38" t="s">
-        <v>1228</v>
+        <v>1220</v>
       </c>
       <c r="N4" s="38"/>
       <c r="O4" s="38"/>
@@ -25664,7 +25700,7 @@
       </c>
       <c r="L24" s="38"/>
       <c r="M24" s="106" t="s">
-        <v>1228</v>
+        <v>1220</v>
       </c>
       <c r="N24" s="38"/>
       <c r="O24" s="38"/>
@@ -26059,7 +26095,7 @@
         <v>1</v>
       </c>
       <c r="C35" s="107" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="D35" s="38" t="s">
         <v>12</v>
@@ -26071,7 +26107,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="107" t="s">
-        <v>1230</v>
+        <v>1222</v>
       </c>
       <c r="H35" s="38" t="s">
         <v>523</v>
@@ -26081,7 +26117,7 @@
       </c>
       <c r="J35" s="38"/>
       <c r="K35" s="38" t="s">
-        <v>1231</v>
+        <v>1223</v>
       </c>
       <c r="L35" s="38"/>
       <c r="M35" s="38"/>

</xml_diff>

<commit_message>
AirSchedule Service Assertions modified based on excel
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4273" uniqueCount="1274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4276" uniqueCount="1275">
   <si>
     <t>Scenario</t>
   </si>
@@ -3895,6 +3895,9 @@
   </si>
   <si>
     <t>QBCNGW</t>
+  </si>
+  <si>
+    <t>QBFLTO</t>
   </si>
 </sst>
 </file>
@@ -20741,7 +20744,7 @@
         <v>15</v>
       </c>
       <c r="H2" s="28" t="s">
-        <v>1228</v>
+        <v>1274</v>
       </c>
       <c r="I2" s="28" t="s">
         <v>197</v>

</xml_diff>

<commit_message>
APIS Service Assertions modified based on excel
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copa_SHD_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D094E751-432F-4878-9FBE-E63B04A51B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C93D54-E628-493F-8476-52B6FC9CAECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4276" uniqueCount="1275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4246" uniqueCount="1263">
   <si>
     <t>Scenario</t>
   </si>
@@ -2472,9 +2472,6 @@
     <t>AgencyName3</t>
   </si>
   <si>
-    <t>BKGOWT</t>
-  </si>
-  <si>
     <t>DepartureDate2</t>
   </si>
   <si>
@@ -3576,30 +3573,9 @@
     <t>2024-08-06T23:13:00</t>
   </si>
   <si>
-    <t>QHF2YA</t>
-  </si>
-  <si>
-    <t>QHF20H</t>
-  </si>
-  <si>
-    <t>QHF3B1</t>
-  </si>
-  <si>
     <t>QHF3O5</t>
   </si>
   <si>
-    <t>QHF3V2</t>
-  </si>
-  <si>
-    <t>QHF311</t>
-  </si>
-  <si>
-    <t>QHF4MQ</t>
-  </si>
-  <si>
-    <t>QHF4R5</t>
-  </si>
-  <si>
     <t>QHGB0S</t>
   </si>
   <si>
@@ -3759,9 +3735,6 @@
     <t>TODDLER</t>
   </si>
   <si>
-    <t>BR4JPJ</t>
-  </si>
-  <si>
     <t>GTOU</t>
   </si>
   <si>
@@ -3783,9 +3756,6 @@
     <t>BS1GVQ</t>
   </si>
   <si>
-    <t>QMTMPL</t>
-  </si>
-  <si>
     <t>QAYQQ3</t>
   </si>
   <si>
@@ -3828,76 +3798,70 @@
     <t>QAY1L4</t>
   </si>
   <si>
-    <t>QBBYDY</t>
-  </si>
-  <si>
-    <t>QBBYQK</t>
-  </si>
-  <si>
-    <t>QBBYXF</t>
-  </si>
-  <si>
-    <t>QBBZ0N</t>
-  </si>
-  <si>
-    <t>QBB0I1</t>
-  </si>
-  <si>
-    <t>QBB0VQ</t>
-  </si>
-  <si>
-    <t>QBB05V</t>
-  </si>
-  <si>
-    <t>QBB1FK</t>
-  </si>
-  <si>
-    <t>QBB1OM</t>
-  </si>
-  <si>
-    <t>QBB1XW</t>
-  </si>
-  <si>
-    <t>QBCI3N</t>
-  </si>
-  <si>
-    <t>QBCJWU</t>
-  </si>
-  <si>
-    <t>QBCKAV</t>
-  </si>
-  <si>
-    <t>QBCKK4</t>
-  </si>
-  <si>
-    <t>QBCKY2</t>
-  </si>
-  <si>
-    <t>QBCK1C</t>
-  </si>
-  <si>
-    <t>QBCLVP</t>
-  </si>
-  <si>
-    <t>QBCL5I</t>
-  </si>
-  <si>
-    <t>QBCMFV</t>
-  </si>
-  <si>
-    <t>QBCMP3</t>
-  </si>
-  <si>
-    <t>QBCMYU</t>
-  </si>
-  <si>
-    <t>QBCM22</t>
-  </si>
-  <si>
-    <t>QBCNGW</t>
-  </si>
-  <si>
     <t>QBFLTO</t>
+  </si>
+  <si>
+    <t>QBMFPR</t>
+  </si>
+  <si>
+    <t>AKRXMQ</t>
+  </si>
+  <si>
+    <t>AKRXMR</t>
+  </si>
+  <si>
+    <t>AKRXNB</t>
+  </si>
+  <si>
+    <t>AKRXNG</t>
+  </si>
+  <si>
+    <t>AKRXNP</t>
+  </si>
+  <si>
+    <t>AKRXNR</t>
+  </si>
+  <si>
+    <t>AKRXNV</t>
+  </si>
+  <si>
+    <t>AKRXNX</t>
+  </si>
+  <si>
+    <t>AKRXN0</t>
+  </si>
+  <si>
+    <t>AKRXN3</t>
+  </si>
+  <si>
+    <t>AKRXOE</t>
+  </si>
+  <si>
+    <t>AKRXPB</t>
+  </si>
+  <si>
+    <t>AKRXPH</t>
+  </si>
+  <si>
+    <t>AKRXPP</t>
+  </si>
+  <si>
+    <t>AKRXP2</t>
+  </si>
+  <si>
+    <t>AKR0K3</t>
+  </si>
+  <si>
+    <t>AKR0LS</t>
+  </si>
+  <si>
+    <t>AKR0NF</t>
+  </si>
+  <si>
+    <t>AKR0OY</t>
+  </si>
+  <si>
+    <t>AKR0UF</t>
   </si>
 </sst>
 </file>
@@ -5014,7 +4978,7 @@
         <v>11</v>
       </c>
       <c r="B2" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="107" t="s">
         <v>28</v>
@@ -5032,7 +4996,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="106" t="s">
-        <v>1265</v>
+        <v>1247</v>
       </c>
       <c r="I2" s="106" t="s">
         <v>197</v>
@@ -5049,7 +5013,7 @@
       <c r="M2" s="106"/>
       <c r="N2" s="106"/>
       <c r="O2" s="106" t="s">
-        <v>1266</v>
+        <v>1248</v>
       </c>
       <c r="P2" s="106"/>
       <c r="Q2" s="106"/>
@@ -5071,7 +5035,7 @@
         <v>17</v>
       </c>
       <c r="B3" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="107" t="s">
         <v>28</v>
@@ -5089,7 +5053,7 @@
         <v>3</v>
       </c>
       <c r="H3" s="106" t="s">
-        <v>1167</v>
+        <v>1243</v>
       </c>
       <c r="I3" s="106" t="s">
         <v>198</v>
@@ -5130,7 +5094,7 @@
         <v>320</v>
       </c>
       <c r="B4" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" s="107" t="s">
         <v>28</v>
@@ -5148,7 +5112,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="33" t="s">
-        <v>1267</v>
+        <v>1262</v>
       </c>
       <c r="I4" s="33" t="s">
         <v>321</v>
@@ -5162,10 +5126,10 @@
       <c r="N4" s="106"/>
       <c r="O4" s="106"/>
       <c r="P4" s="106" t="s">
+        <v>342</v>
+      </c>
+      <c r="Q4" s="106" t="s">
         <v>335</v>
-      </c>
-      <c r="Q4" s="106" t="s">
-        <v>724</v>
       </c>
       <c r="R4" s="106"/>
       <c r="S4" s="106"/>
@@ -5180,12 +5144,12 @@
       <c r="AB4" s="106"/>
       <c r="AC4" s="106"/>
     </row>
-    <row r="5" spans="1:29" ht="29">
+    <row r="5" spans="1:29">
       <c r="A5" s="33" t="s">
         <v>319</v>
       </c>
       <c r="B5" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" s="107" t="s">
         <v>28</v>
@@ -5203,7 +5167,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="33" t="s">
-        <v>1272</v>
+        <v>1256</v>
       </c>
       <c r="I5" s="106" t="s">
         <v>198</v>
@@ -5221,10 +5185,10 @@
       <c r="N5" s="106"/>
       <c r="O5" s="106"/>
       <c r="P5" s="106" t="s">
+        <v>342</v>
+      </c>
+      <c r="Q5" s="106" t="s">
         <v>335</v>
-      </c>
-      <c r="Q5" s="106" t="s">
-        <v>724</v>
       </c>
       <c r="R5" s="106"/>
       <c r="S5" s="106"/>
@@ -5244,7 +5208,7 @@
         <v>578</v>
       </c>
       <c r="B6" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" s="107" t="s">
         <v>28</v>
@@ -5260,7 +5224,7 @@
       </c>
       <c r="G6" s="106"/>
       <c r="H6" s="106" t="s">
-        <v>1270</v>
+        <v>1254</v>
       </c>
       <c r="I6" s="106" t="s">
         <v>579</v>
@@ -5274,10 +5238,10 @@
       <c r="N6" s="106"/>
       <c r="O6" s="106"/>
       <c r="P6" s="106" t="s">
+        <v>342</v>
+      </c>
+      <c r="Q6" s="106" t="s">
         <v>335</v>
-      </c>
-      <c r="Q6" s="106" t="s">
-        <v>724</v>
       </c>
       <c r="R6" s="106"/>
       <c r="S6" s="106"/>
@@ -5297,7 +5261,7 @@
         <v>581</v>
       </c>
       <c r="B7" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="107" t="s">
         <v>28</v>
@@ -5313,7 +5277,7 @@
       </c>
       <c r="G7" s="106"/>
       <c r="H7" s="106" t="s">
-        <v>1262</v>
+        <v>1244</v>
       </c>
       <c r="I7" s="106" t="s">
         <v>582</v>
@@ -5346,7 +5310,7 @@
         <v>584</v>
       </c>
       <c r="B8" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" s="107" t="s">
         <v>28</v>
@@ -5362,7 +5326,7 @@
       </c>
       <c r="G8" s="106"/>
       <c r="H8" s="106" t="s">
-        <v>1273</v>
+        <v>1257</v>
       </c>
       <c r="I8" s="106" t="s">
         <v>585</v>
@@ -5376,10 +5340,10 @@
       <c r="N8" s="106"/>
       <c r="O8" s="106"/>
       <c r="P8" s="106" t="s">
+        <v>342</v>
+      </c>
+      <c r="Q8" s="106" t="s">
         <v>335</v>
-      </c>
-      <c r="Q8" s="106" t="s">
-        <v>724</v>
       </c>
       <c r="R8" s="106"/>
       <c r="S8" s="106"/>
@@ -5399,7 +5363,7 @@
         <v>587</v>
       </c>
       <c r="B9" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="107" t="s">
         <v>28</v>
@@ -5415,7 +5379,7 @@
       </c>
       <c r="G9" s="106"/>
       <c r="H9" s="106" t="s">
-        <v>1269</v>
+        <v>1253</v>
       </c>
       <c r="I9" s="106" t="s">
         <v>588</v>
@@ -5429,10 +5393,10 @@
       <c r="N9" s="106"/>
       <c r="O9" s="106"/>
       <c r="P9" s="106" t="s">
+        <v>342</v>
+      </c>
+      <c r="Q9" s="106" t="s">
         <v>335</v>
-      </c>
-      <c r="Q9" s="106" t="s">
-        <v>724</v>
       </c>
       <c r="R9" s="106"/>
       <c r="S9" s="106"/>
@@ -5452,7 +5416,7 @@
         <v>590</v>
       </c>
       <c r="B10" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" s="107" t="s">
         <v>28</v>
@@ -5468,7 +5432,7 @@
       </c>
       <c r="G10" s="106"/>
       <c r="H10" s="106" t="s">
-        <v>1268</v>
+        <v>1251</v>
       </c>
       <c r="I10" s="106" t="s">
         <v>591</v>
@@ -5485,13 +5449,13 @@
       <c r="M10" s="106"/>
       <c r="N10" s="106"/>
       <c r="O10" s="106" t="s">
-        <v>799</v>
+        <v>1252</v>
       </c>
       <c r="P10" s="106" t="s">
+        <v>342</v>
+      </c>
+      <c r="Q10" s="106" t="s">
         <v>335</v>
-      </c>
-      <c r="Q10" s="106" t="s">
-        <v>724</v>
       </c>
       <c r="R10" s="106"/>
       <c r="S10" s="106"/>
@@ -5504,10 +5468,10 @@
       <c r="Z10" s="106"/>
       <c r="AA10" s="106"/>
       <c r="AB10" s="106" t="s">
+        <v>342</v>
+      </c>
+      <c r="AC10" s="106" t="s">
         <v>335</v>
-      </c>
-      <c r="AC10" s="106" t="s">
-        <v>724</v>
       </c>
     </row>
     <row r="11" spans="1:29">
@@ -5515,10 +5479,10 @@
         <v>595</v>
       </c>
       <c r="B11" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" s="107" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="D11" s="106" t="s">
         <v>43</v>
@@ -5531,7 +5495,7 @@
       </c>
       <c r="G11" s="106"/>
       <c r="H11" s="106" t="s">
-        <v>1271</v>
+        <v>1255</v>
       </c>
       <c r="I11" s="106" t="s">
         <v>326</v>
@@ -5568,7 +5532,7 @@
         <v>597</v>
       </c>
       <c r="B12" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" s="107" t="s">
         <v>28</v>
@@ -5623,10 +5587,10 @@
         <v>600</v>
       </c>
       <c r="B13" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C13" s="107" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="D13" s="106" t="s">
         <v>43</v>
@@ -5639,7 +5603,7 @@
       </c>
       <c r="G13" s="106"/>
       <c r="H13" s="106" t="s">
-        <v>1263</v>
+        <v>1245</v>
       </c>
       <c r="I13" s="106" t="s">
         <v>601</v>
@@ -5678,10 +5642,10 @@
         <v>603</v>
       </c>
       <c r="B14" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14" s="107" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="D14" s="106" t="s">
         <v>12</v>
@@ -5694,7 +5658,7 @@
       </c>
       <c r="G14" s="106"/>
       <c r="H14" s="106" t="s">
-        <v>1264</v>
+        <v>1246</v>
       </c>
       <c r="I14" s="106" t="s">
         <v>605</v>
@@ -5733,7 +5697,7 @@
         <v>608</v>
       </c>
       <c r="B15" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15" s="107" t="s">
         <v>42</v>
@@ -5749,7 +5713,7 @@
       </c>
       <c r="G15" s="106"/>
       <c r="H15" s="106" t="s">
-        <v>1173</v>
+        <v>1242</v>
       </c>
       <c r="I15" s="106" t="s">
         <v>609</v>
@@ -5786,23 +5750,23 @@
         <v>611</v>
       </c>
       <c r="B16" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" s="107" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="D16" s="106" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="E16" s="106" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F16" s="106" t="s">
         <v>14</v>
       </c>
       <c r="G16" s="106"/>
       <c r="H16" s="106" t="s">
-        <v>1169</v>
+        <v>1259</v>
       </c>
       <c r="I16" s="106" t="s">
         <v>612</v>
@@ -5835,23 +5799,23 @@
         <v>614</v>
       </c>
       <c r="B17" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" s="107" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="D17" s="106" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="E17" s="106" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F17" s="106" t="s">
         <v>14</v>
       </c>
       <c r="G17" s="106"/>
       <c r="H17" s="106" t="s">
-        <v>1168</v>
+        <v>1258</v>
       </c>
       <c r="I17" s="106"/>
       <c r="J17" s="106"/>
@@ -5880,7 +5844,7 @@
         <v>615</v>
       </c>
       <c r="B18" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" s="107" t="s">
         <v>28</v>
@@ -5896,7 +5860,7 @@
       </c>
       <c r="G18" s="106"/>
       <c r="H18" s="106" t="s">
-        <v>1254</v>
+        <v>1249</v>
       </c>
       <c r="I18" s="106" t="s">
         <v>20</v>
@@ -5929,7 +5893,7 @@
         <v>616</v>
       </c>
       <c r="B19" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" s="107" t="s">
         <v>564</v>
@@ -5945,7 +5909,7 @@
       </c>
       <c r="G19" s="106"/>
       <c r="H19" s="106" t="s">
-        <v>1170</v>
+        <v>1261</v>
       </c>
       <c r="I19" s="106"/>
       <c r="J19" s="106"/>
@@ -5957,10 +5921,10 @@
       <c r="P19" s="106"/>
       <c r="Q19" s="106"/>
       <c r="R19" s="106">
-        <v>-10</v>
+        <v>1</v>
       </c>
       <c r="S19" s="107" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="T19" s="106" t="s">
         <v>314</v>
@@ -5972,10 +5936,10 @@
         <v>14</v>
       </c>
       <c r="W19" s="106">
-        <v>-10</v>
+        <v>1</v>
       </c>
       <c r="X19" s="107" t="s">
-        <v>457</v>
+        <v>28</v>
       </c>
       <c r="Y19" s="106" t="s">
         <v>12</v>
@@ -5994,10 +5958,10 @@
         <v>617</v>
       </c>
       <c r="B20" s="106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" s="107" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="D20" s="106" t="s">
         <v>12</v>
@@ -6010,7 +5974,7 @@
       </c>
       <c r="G20" s="106"/>
       <c r="H20" s="106" t="s">
-        <v>1171</v>
+        <v>1260</v>
       </c>
       <c r="I20" s="106"/>
       <c r="J20" s="106"/>
@@ -6022,10 +5986,10 @@
       <c r="P20" s="106"/>
       <c r="Q20" s="106"/>
       <c r="R20" s="106">
-        <v>-8</v>
+        <v>1</v>
       </c>
       <c r="S20" s="107" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="T20" s="106" t="s">
         <v>618</v>
@@ -6037,10 +6001,10 @@
         <v>14</v>
       </c>
       <c r="W20" s="106">
-        <v>-8</v>
+        <v>1</v>
       </c>
       <c r="X20" s="107" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="Y20" s="106" t="s">
         <v>12</v>
@@ -6296,13 +6260,13 @@
         <v>3</v>
       </c>
       <c r="C2" s="38" t="s">
-        <v>1200</v>
+        <v>1192</v>
       </c>
       <c r="D2" s="41" t="s">
-        <v>1201</v>
+        <v>1193</v>
       </c>
       <c r="E2" s="41" t="s">
-        <v>1199</v>
+        <v>1191</v>
       </c>
       <c r="F2" s="38"/>
       <c r="G2" s="41" t="s">
@@ -6331,7 +6295,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="41" t="s">
-        <v>1202</v>
+        <v>1194</v>
       </c>
       <c r="E3" s="41" t="s">
         <v>249</v>
@@ -6367,7 +6331,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="41" t="s">
-        <v>1198</v>
+        <v>1190</v>
       </c>
       <c r="E4" s="38"/>
       <c r="F4" s="38" t="s">
@@ -6516,28 +6480,28 @@
         <v>4</v>
       </c>
       <c r="AE1" s="37" t="s">
+        <v>953</v>
+      </c>
+      <c r="AF1" s="37" t="s">
         <v>954</v>
       </c>
-      <c r="AF1" s="37" t="s">
+      <c r="AG1" s="37" t="s">
         <v>955</v>
       </c>
-      <c r="AG1" s="37" t="s">
+      <c r="AH1" s="37" t="s">
         <v>956</v>
       </c>
-      <c r="AH1" s="37" t="s">
+      <c r="AI1" s="37" t="s">
         <v>957</v>
       </c>
-      <c r="AI1" s="37" t="s">
+      <c r="AJ1" s="37" t="s">
         <v>958</v>
       </c>
-      <c r="AJ1" s="37" t="s">
+      <c r="AK1" s="37" t="s">
         <v>959</v>
       </c>
-      <c r="AK1" s="37" t="s">
+      <c r="AL1" s="37" t="s">
         <v>960</v>
-      </c>
-      <c r="AL1" s="37" t="s">
-        <v>961</v>
       </c>
     </row>
     <row r="2" spans="1:38">
@@ -6704,13 +6668,13 @@
         <v>12</v>
       </c>
       <c r="I5" s="38" t="s">
+        <v>816</v>
+      </c>
+      <c r="J5" s="38" t="s">
         <v>817</v>
       </c>
-      <c r="J5" s="38" t="s">
+      <c r="K5" s="38" t="s">
         <v>818</v>
-      </c>
-      <c r="K5" s="38" t="s">
-        <v>819</v>
       </c>
       <c r="L5" s="38"/>
       <c r="M5" s="38"/>
@@ -6766,10 +6730,10 @@
         <v>12</v>
       </c>
       <c r="I6" s="38" t="s">
+        <v>819</v>
+      </c>
+      <c r="J6" s="38" t="s">
         <v>820</v>
-      </c>
-      <c r="J6" s="38" t="s">
-        <v>821</v>
       </c>
       <c r="K6" s="38"/>
       <c r="L6" s="38"/>
@@ -6802,7 +6766,7 @@
     </row>
     <row r="7" spans="1:38">
       <c r="A7" s="48" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="B7" s="38"/>
       <c r="C7" s="38">
@@ -6820,13 +6784,13 @@
         <v>12</v>
       </c>
       <c r="I7" s="38" t="s">
+        <v>962</v>
+      </c>
+      <c r="J7" s="38" t="s">
         <v>963</v>
       </c>
-      <c r="J7" s="38" t="s">
+      <c r="K7" s="38" t="s">
         <v>964</v>
-      </c>
-      <c r="K7" s="38" t="s">
-        <v>965</v>
       </c>
       <c r="L7" s="38"/>
       <c r="M7" s="38"/>
@@ -6858,7 +6822,7 @@
     </row>
     <row r="8" spans="1:38">
       <c r="A8" s="38" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B8" s="38"/>
       <c r="C8" s="38">
@@ -6876,10 +6840,10 @@
         <v>30</v>
       </c>
       <c r="I8" s="38" t="s">
+        <v>966</v>
+      </c>
+      <c r="J8" s="38" t="s">
         <v>967</v>
-      </c>
-      <c r="J8" s="38" t="s">
-        <v>968</v>
       </c>
       <c r="K8" s="38"/>
       <c r="L8" s="38"/>
@@ -6916,7 +6880,7 @@
     </row>
     <row r="9" spans="1:38">
       <c r="A9" s="38" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B9" s="38"/>
       <c r="C9" s="38">
@@ -6934,13 +6898,13 @@
         <v>30</v>
       </c>
       <c r="I9" s="38" t="s">
+        <v>969</v>
+      </c>
+      <c r="J9" s="38" t="s">
         <v>970</v>
       </c>
-      <c r="J9" s="38" t="s">
+      <c r="K9" s="38" t="s">
         <v>971</v>
-      </c>
-      <c r="K9" s="38" t="s">
-        <v>972</v>
       </c>
       <c r="L9" s="38"/>
       <c r="M9" s="38"/>
@@ -6973,7 +6937,7 @@
         <v>9</v>
       </c>
       <c r="X9" s="41" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="Y9" s="38" t="s">
         <v>314</v>
@@ -7004,7 +6968,7 @@
     </row>
     <row r="10" spans="1:38">
       <c r="A10" s="38" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="B10" s="38"/>
       <c r="C10" s="38">
@@ -7022,13 +6986,13 @@
         <v>30</v>
       </c>
       <c r="I10" s="38" t="s">
+        <v>974</v>
+      </c>
+      <c r="J10" s="38" t="s">
         <v>975</v>
       </c>
-      <c r="J10" s="38" t="s">
+      <c r="K10" s="38" t="s">
         <v>976</v>
-      </c>
-      <c r="K10" s="38" t="s">
-        <v>977</v>
       </c>
       <c r="L10" s="38"/>
       <c r="M10" s="38"/>
@@ -7061,7 +7025,7 @@
         <v>9</v>
       </c>
       <c r="X10" s="41" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="Y10" s="38" t="s">
         <v>314</v>
@@ -7092,7 +7056,7 @@
     </row>
     <row r="11" spans="1:38">
       <c r="A11" s="48" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="B11" s="38"/>
       <c r="C11" s="38"/>
@@ -7134,7 +7098,7 @@
     </row>
     <row r="12" spans="1:38">
       <c r="A12" s="48" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="B12" s="38"/>
       <c r="C12" s="38"/>
@@ -7145,10 +7109,10 @@
       <c r="H12" s="38"/>
       <c r="I12" s="38"/>
       <c r="J12" s="93" t="s">
+        <v>979</v>
+      </c>
+      <c r="K12" s="41" t="s">
         <v>980</v>
-      </c>
-      <c r="K12" s="41" t="s">
-        <v>981</v>
       </c>
       <c r="L12" s="38"/>
       <c r="M12" s="38"/>
@@ -7170,33 +7134,33 @@
       <c r="AC12" s="38"/>
       <c r="AD12" s="38"/>
       <c r="AE12" s="41" t="s">
+        <v>981</v>
+      </c>
+      <c r="AF12" s="41" t="s">
         <v>982</v>
       </c>
-      <c r="AF12" s="41" t="s">
+      <c r="AG12" s="41" t="s">
         <v>983</v>
       </c>
-      <c r="AG12" s="41" t="s">
+      <c r="AH12" s="41" t="s">
         <v>984</v>
       </c>
-      <c r="AH12" s="41" t="s">
+      <c r="AI12" s="41" t="s">
         <v>985</v>
       </c>
-      <c r="AI12" s="41" t="s">
+      <c r="AJ12" s="41" t="s">
         <v>986</v>
       </c>
-      <c r="AJ12" s="41" t="s">
+      <c r="AK12" s="41" t="s">
         <v>987</v>
       </c>
-      <c r="AK12" s="41" t="s">
+      <c r="AL12" s="41" t="s">
         <v>988</v>
-      </c>
-      <c r="AL12" s="41" t="s">
-        <v>989</v>
       </c>
     </row>
     <row r="13" spans="1:38">
       <c r="A13" s="48" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B13" s="38"/>
       <c r="C13" s="38"/>
@@ -7207,7 +7171,7 @@
       <c r="H13" s="38"/>
       <c r="I13" s="38"/>
       <c r="J13" s="41" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="K13" s="38"/>
       <c r="L13" s="38"/>
@@ -7240,7 +7204,7 @@
     </row>
     <row r="14" spans="1:38">
       <c r="A14" s="48" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="B14" s="38"/>
       <c r="C14" s="38"/>
@@ -7251,7 +7215,7 @@
       <c r="H14" s="38"/>
       <c r="I14" s="38"/>
       <c r="J14" s="41" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="K14" s="38"/>
       <c r="L14" s="38"/>
@@ -7320,7 +7284,7 @@
         <v>252</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="F1" s="36" t="s">
         <v>24</v>
@@ -7455,7 +7419,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="G5" s="38"/>
       <c r="H5" s="38"/>
@@ -7463,7 +7427,7 @@
       <c r="J5" s="38"/>
       <c r="K5" s="38"/>
       <c r="L5" s="75" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="M5" s="38"/>
     </row>
@@ -7480,7 +7444,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="41" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="G6" s="38"/>
       <c r="H6" s="38"/>
@@ -7488,7 +7452,7 @@
       <c r="J6" s="38"/>
       <c r="K6" s="38"/>
       <c r="L6" s="38" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="M6" s="38"/>
     </row>
@@ -7505,7 +7469,7 @@
         <v>-1</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="G7" s="38"/>
       <c r="H7" s="38"/>
@@ -7517,7 +7481,7 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="48" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="B8" s="38"/>
       <c r="C8" s="38"/>
@@ -7538,7 +7502,7 @@
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="84" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="B9" s="38"/>
       <c r="C9" s="38"/>
@@ -7561,7 +7525,7 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="85" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="B10" s="38"/>
       <c r="C10" s="38" t="s">
@@ -7588,7 +7552,7 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="84" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="B11" s="38"/>
       <c r="C11" s="38" t="s">
@@ -7615,7 +7579,7 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="84" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="B12" s="38"/>
       <c r="C12" s="38" t="s">
@@ -7640,7 +7604,7 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="48" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="B13" s="38"/>
       <c r="C13" s="38" t="s">
@@ -7661,7 +7625,7 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="48" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="B14" s="38"/>
       <c r="C14" s="38" t="s">
@@ -7684,7 +7648,7 @@
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="86" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="B15" s="38"/>
       <c r="C15" s="38" t="s">
@@ -7695,7 +7659,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="41" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="G15" s="38" t="s">
         <v>12</v>
@@ -7706,12 +7670,12 @@
       <c r="K15" s="38"/>
       <c r="L15" s="38"/>
       <c r="M15" s="87" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="88" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="B16" s="38"/>
       <c r="C16" s="38" t="s">
@@ -7734,7 +7698,7 @@
     </row>
     <row r="17" spans="1:13">
       <c r="A17" s="84" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="B17" s="38"/>
       <c r="C17" s="38" t="s">
@@ -7757,13 +7721,13 @@
       <c r="J17" s="38"/>
       <c r="K17" s="38"/>
       <c r="L17" s="92" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="M17" s="38"/>
     </row>
     <row r="18" spans="1:13">
       <c r="A18" s="85" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="B18" s="38"/>
       <c r="C18" s="38" t="s">
@@ -7774,7 +7738,7 @@
         <v>2</v>
       </c>
       <c r="F18" s="89" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="G18" s="38" t="s">
         <v>487</v>
@@ -7786,13 +7750,13 @@
       <c r="J18" s="38"/>
       <c r="K18" s="38"/>
       <c r="L18" s="92" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="M18" s="38"/>
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="84" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="B19" s="38"/>
       <c r="C19" s="38" t="s">
@@ -7803,7 +7767,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="41" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="G19" s="38" t="s">
         <v>12</v>
@@ -7815,17 +7779,17 @@
       <c r="J19" s="38"/>
       <c r="K19" s="38"/>
       <c r="L19" s="92" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="M19" s="38"/>
     </row>
     <row r="20" spans="1:13">
       <c r="A20" s="88" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="B20" s="38"/>
       <c r="C20" s="38" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="D20" s="38"/>
       <c r="E20" s="38">
@@ -7844,7 +7808,7 @@
     </row>
     <row r="21" spans="1:13">
       <c r="A21" s="48" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="B21" s="38"/>
       <c r="C21" s="38" t="s">
@@ -7863,13 +7827,13 @@
       <c r="J21" s="38"/>
       <c r="K21" s="38"/>
       <c r="L21" s="90" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="M21" s="38"/>
     </row>
     <row r="22" spans="1:13">
       <c r="A22" s="86" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="B22" s="38"/>
       <c r="C22" s="38" t="s">
@@ -7880,7 +7844,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="41" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="G22" s="38"/>
       <c r="H22" s="38"/>
@@ -7888,13 +7852,13 @@
       <c r="J22" s="38"/>
       <c r="K22" s="38"/>
       <c r="L22" s="90" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="M22" s="38"/>
     </row>
     <row r="23" spans="1:13">
       <c r="A23" s="48" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="B23" s="38"/>
       <c r="C23" s="38" t="s">
@@ -7913,13 +7877,13 @@
       <c r="J23" s="38"/>
       <c r="K23" s="38"/>
       <c r="L23" s="91" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="M23" s="38"/>
     </row>
     <row r="24" spans="1:13">
       <c r="A24" s="48" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="B24" s="38"/>
       <c r="C24" s="38" t="s">
@@ -7944,7 +7908,7 @@
     </row>
     <row r="25" spans="1:13">
       <c r="A25" s="48" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B25" s="38"/>
       <c r="C25" s="38" t="s">
@@ -8095,13 +8059,13 @@
         <v>41</v>
       </c>
       <c r="J2" s="38" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="K2" s="38" t="s">
+        <v>838</v>
+      </c>
+      <c r="L2" s="38" t="s">
         <v>839</v>
-      </c>
-      <c r="L2" s="38" t="s">
-        <v>840</v>
       </c>
       <c r="M2" s="38" t="s">
         <v>621</v>
@@ -8147,19 +8111,19 @@
         <v>12</v>
       </c>
       <c r="J3" s="38" t="s">
+        <v>842</v>
+      </c>
+      <c r="K3" s="38" t="s">
+        <v>841</v>
+      </c>
+      <c r="L3" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="K3" s="38" t="s">
-        <v>842</v>
-      </c>
-      <c r="L3" s="38" t="s">
+      <c r="M3" s="38" t="s">
+        <v>840</v>
+      </c>
+      <c r="N3" s="38" t="s">
         <v>844</v>
-      </c>
-      <c r="M3" s="38" t="s">
-        <v>841</v>
-      </c>
-      <c r="N3" s="38" t="s">
-        <v>845</v>
       </c>
       <c r="O3" s="38">
         <v>30</v>
@@ -8207,16 +8171,16 @@
       <c r="H4" s="38"/>
       <c r="I4" s="38"/>
       <c r="J4" s="38" t="s">
-        <v>1206</v>
+        <v>1198</v>
       </c>
       <c r="K4" s="38" t="s">
-        <v>1205</v>
+        <v>1197</v>
       </c>
       <c r="L4" s="38" t="s">
         <v>621</v>
       </c>
       <c r="M4" s="38" t="s">
-        <v>1204</v>
+        <v>1196</v>
       </c>
       <c r="N4" s="38" t="s">
         <v>621</v>
@@ -8251,16 +8215,16 @@
       <c r="H5" s="38"/>
       <c r="I5" s="38"/>
       <c r="J5" s="38" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="K5" s="38" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="L5" s="38" t="s">
         <v>621</v>
       </c>
       <c r="M5" s="38" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="N5" s="38" t="s">
         <v>621</v>
@@ -8303,16 +8267,16 @@
         <v>30</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>1203</v>
+        <v>1195</v>
       </c>
       <c r="K6" s="38" t="s">
-        <v>1205</v>
+        <v>1197</v>
       </c>
       <c r="L6" s="38" t="s">
         <v>621</v>
       </c>
       <c r="M6" s="38" t="s">
-        <v>1204</v>
+        <v>1196</v>
       </c>
       <c r="N6" s="38" t="s">
         <v>621</v>
@@ -8628,7 +8592,7 @@
       </c>
       <c r="E3" s="38"/>
       <c r="F3" s="38" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="G3" s="38"/>
       <c r="H3" s="38"/>
@@ -8986,19 +8950,19 @@
         <v>100</v>
       </c>
       <c r="C1" s="36" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D1" s="96" t="s">
         <v>1120</v>
       </c>
-      <c r="D1" s="96" t="s">
+      <c r="E1" s="36" t="s">
         <v>1121</v>
-      </c>
-      <c r="E1" s="36" t="s">
-        <v>1122</v>
       </c>
       <c r="F1" s="36" t="s">
         <v>251</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -9029,7 +8993,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="38" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="B4" s="38" t="s">
         <v>175</v>
@@ -9042,19 +9006,19 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="38" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B5" s="38" t="s">
         <v>1116</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="C5" s="38" t="s">
         <v>1117</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="D5" s="38" t="s">
+        <v>1160</v>
+      </c>
+      <c r="E5" s="38" t="s">
         <v>1118</v>
-      </c>
-      <c r="D5" s="38" t="s">
-        <v>1161</v>
-      </c>
-      <c r="E5" s="38" t="s">
-        <v>1119</v>
       </c>
       <c r="F5" s="38" t="s">
         <v>139</v>
@@ -9208,7 +9172,7 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3" s="38" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="B3" s="38">
         <v>1</v>
@@ -9255,7 +9219,7 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4" s="38" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="B4" s="38">
         <v>2</v>
@@ -9290,15 +9254,15 @@
       <c r="X4" s="38"/>
       <c r="Y4" s="38"/>
       <c r="Z4" s="41" t="s">
+        <v>1106</v>
+      </c>
+      <c r="AA4" s="38" t="s">
         <v>1107</v>
-      </c>
-      <c r="AA4" s="38" t="s">
-        <v>1108</v>
       </c>
     </row>
     <row r="5" spans="1:27">
       <c r="A5" s="38" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="B5" s="38">
         <v>1</v>
@@ -9345,7 +9309,7 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6" s="38" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B6" s="38">
         <v>1</v>
@@ -9384,7 +9348,7 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7" s="38" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B7" s="38">
         <v>1</v>
@@ -9463,7 +9427,7 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8" s="38" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="B8" s="38">
         <v>1</v>
@@ -9502,13 +9466,13 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9" s="38" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="B9" s="38">
         <v>1</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="D9" s="38" t="s">
         <v>12</v>
@@ -9538,7 +9502,7 @@
       <c r="Y9" s="38"/>
       <c r="Z9" s="38"/>
       <c r="AA9" s="95" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
     </row>
   </sheetData>
@@ -10168,7 +10132,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="38" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
@@ -10552,7 +10516,7 @@
       <c r="I9" s="38"/>
       <c r="J9" s="38"/>
       <c r="K9" s="38" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>407</v>
@@ -10561,7 +10525,7 @@
         <v>300</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>195</v>
@@ -10792,7 +10756,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="66" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="D2" s="66" t="s">
         <v>12</v>
@@ -10837,7 +10801,7 @@
         <v>-7</v>
       </c>
       <c r="C3" s="66" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="D3" s="66" t="s">
         <v>12</v>
@@ -11116,7 +11080,7 @@
         <v>3</v>
       </c>
       <c r="C8" s="66" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="D8" s="67" t="s">
         <v>487</v>
@@ -11788,16 +11752,16 @@
       <c r="U2" s="38"/>
       <c r="V2" s="38"/>
       <c r="W2" s="38" t="s">
+        <v>802</v>
+      </c>
+      <c r="X2" s="38" t="s">
         <v>803</v>
-      </c>
-      <c r="X2" s="38" t="s">
-        <v>804</v>
       </c>
       <c r="Y2" s="38" t="s">
         <v>300</v>
       </c>
       <c r="Z2" s="38" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="AA2" s="38" t="s">
         <v>195</v>
@@ -11806,7 +11770,7 @@
         <v>12</v>
       </c>
       <c r="AC2" s="38" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="AD2" s="38"/>
       <c r="AE2" s="38"/>
@@ -11882,7 +11846,7 @@
         <v>5</v>
       </c>
       <c r="W3" s="38" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="X3" s="38"/>
       <c r="Y3" s="38"/>
@@ -11890,7 +11854,7 @@
       <c r="AA3" s="38"/>
       <c r="AB3" s="38"/>
       <c r="AC3" s="38" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="AD3" s="41" t="s">
         <v>784</v>
@@ -11905,7 +11869,7 @@
         <v>6</v>
       </c>
       <c r="AH3" s="41" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
     </row>
     <row r="4" spans="1:34">
@@ -11944,16 +11908,16 @@
       <c r="U4" s="38"/>
       <c r="V4" s="38"/>
       <c r="W4" s="38" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="X4" s="38" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="Y4" s="38" t="s">
         <v>300</v>
       </c>
       <c r="Z4" s="38" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="AA4" s="38" t="s">
         <v>195</v>
@@ -11962,7 +11926,7 @@
         <v>12</v>
       </c>
       <c r="AC4" s="38" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="AD4" s="38"/>
       <c r="AE4" s="38"/>
@@ -12066,7 +12030,7 @@
         <v>246</v>
       </c>
       <c r="K1" s="36" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -12076,7 +12040,7 @@
       <c r="B2" s="38"/>
       <c r="C2" s="38"/>
       <c r="D2" s="38" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="E2" s="38"/>
       <c r="F2" s="38"/>
@@ -12170,12 +12134,12 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="62" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="B7" s="38"/>
       <c r="C7" s="38"/>
       <c r="D7" s="38" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="E7" s="38"/>
       <c r="F7" s="38"/>
@@ -12187,7 +12151,7 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="48" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="B8" s="38"/>
       <c r="C8" s="38" t="s">
@@ -12204,11 +12168,11 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="48" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B9" s="38"/>
       <c r="C9" s="90" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="D9" s="38"/>
       <c r="E9" s="38"/>
@@ -12221,7 +12185,7 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="48" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="B10" s="38"/>
       <c r="C10" s="38"/>
@@ -12236,12 +12200,12 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="48" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="B11" s="38"/>
       <c r="C11" s="38"/>
       <c r="D11" s="90" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="E11" s="90" t="s">
         <v>113</v>
@@ -12250,10 +12214,10 @@
         <v>109</v>
       </c>
       <c r="G11" s="90" t="s">
+        <v>1001</v>
+      </c>
+      <c r="H11" s="90" t="s">
         <v>1002</v>
-      </c>
-      <c r="H11" s="90" t="s">
-        <v>1003</v>
       </c>
       <c r="I11" s="38"/>
       <c r="J11" s="38"/>
@@ -12261,7 +12225,7 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="48" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="B12" s="38"/>
       <c r="C12" s="38"/>
@@ -12272,20 +12236,20 @@
       <c r="H12" s="38"/>
       <c r="I12" s="38"/>
       <c r="J12" s="38" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="K12" s="41" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="48" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="B13" s="38"/>
       <c r="C13" s="38"/>
       <c r="D13" s="90" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="E13" s="38"/>
       <c r="F13" s="38"/>
@@ -12297,12 +12261,12 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="48" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="B14" s="38"/>
       <c r="C14" s="38"/>
       <c r="D14" s="38" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="E14" s="38"/>
       <c r="F14" s="38"/>
@@ -12314,12 +12278,12 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="48" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="B15" s="38"/>
       <c r="C15" s="38"/>
       <c r="D15" s="38" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="E15" s="38"/>
       <c r="F15" s="38"/>
@@ -12331,12 +12295,12 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="86" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B16" s="38"/>
       <c r="C16" s="38"/>
       <c r="D16" s="38" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="E16" s="38"/>
       <c r="F16" s="38"/>
@@ -12460,21 +12424,21 @@
       <c r="I2" s="38"/>
       <c r="J2" s="38"/>
       <c r="K2" s="38" t="s">
+        <v>821</v>
+      </c>
+      <c r="L2" s="38" t="s">
         <v>822</v>
-      </c>
-      <c r="L2" s="38" t="s">
-        <v>823</v>
       </c>
       <c r="M2" s="38" t="s">
         <v>457</v>
       </c>
       <c r="N2" s="38" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="O2" s="38"/>
       <c r="P2" s="38"/>
       <c r="Q2" s="38" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="R2" s="38"/>
     </row>
@@ -12502,16 +12466,16 @@
       <c r="I3" s="38"/>
       <c r="J3" s="38"/>
       <c r="K3" s="38" t="s">
+        <v>825</v>
+      </c>
+      <c r="L3" s="38" t="s">
         <v>826</v>
-      </c>
-      <c r="L3" s="38" t="s">
-        <v>827</v>
       </c>
       <c r="M3" s="38" t="s">
         <v>776</v>
       </c>
       <c r="N3" s="38" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="O3" s="38" t="s">
         <v>12</v>
@@ -12520,10 +12484,10 @@
         <v>13</v>
       </c>
       <c r="Q3" s="38" t="s">
+        <v>828</v>
+      </c>
+      <c r="R3" s="38" t="s">
         <v>829</v>
-      </c>
-      <c r="R3" s="38" t="s">
-        <v>830</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -12550,16 +12514,16 @@
       <c r="I4" s="38"/>
       <c r="J4" s="38"/>
       <c r="K4" s="38" t="s">
+        <v>1163</v>
+      </c>
+      <c r="L4" s="38" t="s">
         <v>1164</v>
-      </c>
-      <c r="L4" s="38" t="s">
-        <v>1165</v>
       </c>
       <c r="M4" s="38" t="s">
         <v>457</v>
       </c>
       <c r="N4" s="38" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="O4" s="38" t="s">
         <v>12</v>
@@ -12568,7 +12532,7 @@
         <v>30</v>
       </c>
       <c r="Q4" s="38" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="R4" s="38"/>
     </row>
@@ -12596,16 +12560,16 @@
       <c r="I5" s="38"/>
       <c r="J5" s="38"/>
       <c r="K5" s="38" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="L5" s="38" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="M5" s="38" t="s">
         <v>776</v>
       </c>
       <c r="N5" s="38" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="O5" s="38" t="s">
         <v>12</v>
@@ -12614,7 +12578,7 @@
         <v>13</v>
       </c>
       <c r="Q5" s="38" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="R5" s="38"/>
     </row>
@@ -12642,16 +12606,16 @@
       <c r="I6" s="38"/>
       <c r="J6" s="38"/>
       <c r="K6" s="38" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="L6" s="38" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="M6" s="38" t="s">
         <v>776</v>
       </c>
       <c r="N6" s="38" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="O6" s="38" t="s">
         <v>12</v>
@@ -12660,7 +12624,7 @@
         <v>13</v>
       </c>
       <c r="Q6" s="38" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="R6" s="38"/>
     </row>
@@ -12909,13 +12873,13 @@
     </row>
     <row r="4" spans="1:23">
       <c r="A4" s="106" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="B4" s="106">
         <v>1</v>
       </c>
       <c r="C4" s="107" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="D4" s="106" t="s">
         <v>12</v>
@@ -12936,7 +12900,7 @@
         <v>153</v>
       </c>
       <c r="J4" s="106" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="K4" s="106"/>
       <c r="L4" s="106"/>
@@ -12958,7 +12922,7 @@
     </row>
     <row r="5" spans="1:23">
       <c r="A5" s="106" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="B5" s="106"/>
       <c r="C5" s="106"/>
@@ -12987,7 +12951,7 @@
     </row>
     <row r="6" spans="1:23">
       <c r="A6" s="106" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="B6" s="106">
         <v>1</v>
@@ -13006,7 +12970,7 @@
       <c r="H6" s="106"/>
       <c r="I6" s="106"/>
       <c r="J6" s="106" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="K6" s="106"/>
       <c r="L6" s="106"/>
@@ -13019,7 +12983,7 @@
       <c r="S6" s="106"/>
       <c r="T6" s="106"/>
       <c r="U6" s="87" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="V6" s="106"/>
       <c r="W6" s="106" t="s">
@@ -13165,13 +13129,13 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="106" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="B4" s="106" t="s">
         <v>139</v>
       </c>
       <c r="C4" s="106" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="D4" s="106"/>
       <c r="E4" s="106"/>
@@ -13179,13 +13143,13 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="108" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="B5" s="109" t="s">
         <v>139</v>
       </c>
       <c r="C5" s="109" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="D5" s="106" t="s">
         <v>142</v>
@@ -13195,13 +13159,13 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="108" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="B6" s="109" t="s">
         <v>139</v>
       </c>
       <c r="C6" s="109" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="D6" s="106"/>
       <c r="E6" s="106" t="s">
@@ -13211,25 +13175,25 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="108" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="B7" s="109" t="s">
         <v>139</v>
       </c>
       <c r="C7" s="109" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="D7" s="106" t="s">
         <v>142</v>
       </c>
       <c r="E7" s="107" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="F7" s="106"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="106" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="B8" s="109" t="s">
         <v>139</v>
@@ -13249,7 +13213,7 @@
         <v>139</v>
       </c>
       <c r="C9" s="106" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="D9" s="106" t="s">
         <v>142</v>
@@ -13338,7 +13302,7 @@
         <v>25</v>
       </c>
       <c r="P1" s="36" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -14079,7 +14043,7 @@
     </row>
     <row r="18" spans="1:16">
       <c r="A18" s="38" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="B18" s="38" t="s">
         <v>139</v>
@@ -14091,7 +14055,7 @@
         <v>111</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="F18" s="38" t="s">
         <v>429</v>
@@ -14109,7 +14073,7 @@
         <v>436</v>
       </c>
       <c r="K18" s="38" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="L18" s="38" t="s">
         <v>430</v>
@@ -14129,7 +14093,7 @@
     </row>
     <row r="19" spans="1:16">
       <c r="A19" s="38" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="B19" s="38" t="s">
         <v>139</v>
@@ -14141,7 +14105,7 @@
         <v>111</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="F19" s="38" t="s">
         <v>425</v>
@@ -14159,7 +14123,7 @@
         <v>436</v>
       </c>
       <c r="K19" s="38" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="L19" s="38" t="s">
         <v>425</v>
@@ -14179,7 +14143,7 @@
     </row>
     <row r="20" spans="1:16">
       <c r="A20" s="38" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="B20" s="38" t="s">
         <v>139</v>
@@ -14191,7 +14155,7 @@
         <v>111</v>
       </c>
       <c r="E20" s="38" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="F20" s="38" t="s">
         <v>429</v>
@@ -14209,7 +14173,7 @@
         <v>436</v>
       </c>
       <c r="K20" s="38" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="L20" s="38" t="s">
         <v>430</v>
@@ -14229,7 +14193,7 @@
     </row>
     <row r="21" spans="1:16">
       <c r="A21" s="38" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="B21" s="38" t="s">
         <v>139</v>
@@ -14241,16 +14205,16 @@
         <v>111</v>
       </c>
       <c r="E21" s="38" t="s">
+        <v>1020</v>
+      </c>
+      <c r="F21" s="38" t="s">
         <v>1021</v>
-      </c>
-      <c r="F21" s="38" t="s">
-        <v>1022</v>
       </c>
       <c r="G21" s="38" t="s">
         <v>309</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="I21" s="38" t="s">
         <v>436</v>
@@ -14279,7 +14243,7 @@
     </row>
     <row r="22" spans="1:16">
       <c r="A22" s="38" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="B22" s="38" t="s">
         <v>139</v>
@@ -14291,7 +14255,7 @@
         <v>111</v>
       </c>
       <c r="E22" s="38" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="F22" s="38" t="s">
         <v>415</v>
@@ -14300,7 +14264,7 @@
         <v>309</v>
       </c>
       <c r="H22" s="38" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="I22" s="38" t="s">
         <v>436</v>
@@ -14329,7 +14293,7 @@
     </row>
     <row r="23" spans="1:16">
       <c r="A23" s="38" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B23" s="38" t="s">
         <v>139</v>
@@ -14341,7 +14305,7 @@
         <v>111</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="F23" s="38" t="s">
         <v>415</v>
@@ -14350,7 +14314,7 @@
         <v>309</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="I23" s="38" t="s">
         <v>436</v>
@@ -14379,7 +14343,7 @@
     </row>
     <row r="24" spans="1:16">
       <c r="A24" s="38" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B24" s="38" t="s">
         <v>139</v>
@@ -14400,16 +14364,16 @@
         <v>309</v>
       </c>
       <c r="H24" s="38" t="s">
+        <v>1030</v>
+      </c>
+      <c r="I24" s="38" t="s">
+        <v>436</v>
+      </c>
+      <c r="J24" s="38" t="s">
+        <v>436</v>
+      </c>
+      <c r="K24" s="38" t="s">
         <v>1031</v>
-      </c>
-      <c r="I24" s="38" t="s">
-        <v>436</v>
-      </c>
-      <c r="J24" s="38" t="s">
-        <v>436</v>
-      </c>
-      <c r="K24" s="38" t="s">
-        <v>1032</v>
       </c>
       <c r="L24" s="38" t="s">
         <v>429</v>
@@ -14429,7 +14393,7 @@
     </row>
     <row r="25" spans="1:16">
       <c r="A25" s="38" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="B25" s="38" t="s">
         <v>139</v>
@@ -14441,7 +14405,7 @@
         <v>111</v>
       </c>
       <c r="E25" s="38" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="F25" s="38" t="s">
         <v>425</v>
@@ -14479,7 +14443,7 @@
     </row>
     <row r="26" spans="1:16">
       <c r="A26" s="38" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="B26" s="38" t="s">
         <v>139</v>
@@ -14491,16 +14455,16 @@
         <v>111</v>
       </c>
       <c r="E26" s="38" t="s">
+        <v>1035</v>
+      </c>
+      <c r="F26" s="38" t="s">
         <v>1036</v>
-      </c>
-      <c r="F26" s="38" t="s">
-        <v>1037</v>
       </c>
       <c r="G26" s="38" t="s">
         <v>309</v>
       </c>
       <c r="H26" s="38" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="I26" s="38" t="s">
         <v>436</v>
@@ -14512,7 +14476,7 @@
         <v>430</v>
       </c>
       <c r="L26" s="38" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="M26" s="38" t="s">
         <v>436</v>
@@ -14529,7 +14493,7 @@
     </row>
     <row r="27" spans="1:16">
       <c r="A27" s="38" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="B27" s="38" t="s">
         <v>139</v>
@@ -14579,7 +14543,7 @@
     </row>
     <row r="28" spans="1:16">
       <c r="A28" s="38" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="B28" s="38" t="s">
         <v>139</v>
@@ -14591,7 +14555,7 @@
         <v>111</v>
       </c>
       <c r="E28" s="38" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="F28" s="38" t="s">
         <v>415</v>
@@ -14600,7 +14564,7 @@
         <v>309</v>
       </c>
       <c r="H28" s="38" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="I28" s="38" t="s">
         <v>436</v>
@@ -14629,7 +14593,7 @@
     </row>
     <row r="29" spans="1:16">
       <c r="A29" s="38" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="B29" s="38" t="s">
         <v>139</v>
@@ -14641,7 +14605,7 @@
         <v>111</v>
       </c>
       <c r="E29" s="38" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="F29" s="38" t="s">
         <v>415</v>
@@ -14650,7 +14614,7 @@
         <v>309</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="I29" s="38" t="s">
         <v>436</v>
@@ -14679,7 +14643,7 @@
     </row>
     <row r="30" spans="1:16">
       <c r="A30" s="38" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B30" s="38" t="s">
         <v>139</v>
@@ -14691,7 +14655,7 @@
         <v>111</v>
       </c>
       <c r="E30" s="38" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="F30" s="38" t="s">
         <v>415</v>
@@ -14729,7 +14693,7 @@
     </row>
     <row r="31" spans="1:16">
       <c r="A31" s="38" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B31" s="38" t="s">
         <v>139</v>
@@ -14777,7 +14741,7 @@
     </row>
     <row r="32" spans="1:16">
       <c r="A32" s="38" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B32" s="38" t="s">
         <v>139</v>
@@ -14827,7 +14791,7 @@
     </row>
     <row r="33" spans="1:16">
       <c r="A33" s="38" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B33" s="38" t="s">
         <v>139</v>
@@ -14877,7 +14841,7 @@
     </row>
     <row r="34" spans="1:16">
       <c r="A34" s="38" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="B34" s="38" t="s">
         <v>139</v>
@@ -14927,7 +14891,7 @@
     </row>
     <row r="35" spans="1:16">
       <c r="A35" s="38" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B35" s="38" t="s">
         <v>139</v>
@@ -14977,7 +14941,7 @@
     </row>
     <row r="36" spans="1:16">
       <c r="A36" s="38" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="B36" s="38" t="s">
         <v>139</v>
@@ -15019,7 +14983,7 @@
         <v>436</v>
       </c>
       <c r="O36" s="38" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="P36" s="38" t="s">
         <v>436</v>
@@ -15027,7 +14991,7 @@
     </row>
     <row r="37" spans="1:16">
       <c r="A37" s="38" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B37" s="38" t="s">
         <v>139</v>
@@ -15077,7 +15041,7 @@
     </row>
     <row r="38" spans="1:16">
       <c r="A38" s="38" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="B38" s="38" t="s">
         <v>139</v>
@@ -15122,12 +15086,12 @@
         <v>436</v>
       </c>
       <c r="P38" s="38" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="39" spans="1:16">
       <c r="A39" s="38" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="B39" s="38" t="s">
         <v>139</v>
@@ -15169,7 +15133,7 @@
         <v>436</v>
       </c>
       <c r="O39" s="38" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="P39" s="38" t="s">
         <v>436</v>
@@ -15177,7 +15141,7 @@
     </row>
     <row r="40" spans="1:16">
       <c r="A40" s="38" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B40" s="38" t="s">
         <v>139</v>
@@ -15222,12 +15186,12 @@
         <v>436</v>
       </c>
       <c r="P40" s="38" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="41" spans="1:16">
       <c r="A41" s="38" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="B41" s="38" t="s">
         <v>139</v>
@@ -15269,7 +15233,7 @@
         <v>436</v>
       </c>
       <c r="O41" s="38" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="P41" s="38" t="s">
         <v>436</v>
@@ -15277,7 +15241,7 @@
     </row>
     <row r="42" spans="1:16">
       <c r="A42" s="38" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="B42" s="38" t="s">
         <v>139</v>
@@ -15322,12 +15286,12 @@
         <v>436</v>
       </c>
       <c r="P42" s="38" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="43" spans="1:16">
       <c r="A43" s="38" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="B43" s="38" t="s">
         <v>139</v>
@@ -15369,7 +15333,7 @@
         <v>436</v>
       </c>
       <c r="O43" s="38" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="P43" s="38" t="s">
         <v>436</v>
@@ -15377,7 +15341,7 @@
     </row>
     <row r="44" spans="1:16">
       <c r="A44" s="38" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="B44" s="38" t="s">
         <v>139</v>
@@ -15427,7 +15391,7 @@
     </row>
     <row r="45" spans="1:16">
       <c r="A45" s="38" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="B45" s="38" t="s">
         <v>139</v>
@@ -15469,7 +15433,7 @@
         <v>436</v>
       </c>
       <c r="O45" s="38" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="P45" s="38" t="s">
         <v>436</v>
@@ -15477,7 +15441,7 @@
     </row>
     <row r="46" spans="1:16">
       <c r="A46" s="38" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="B46" s="38" t="s">
         <v>139</v>
@@ -15527,7 +15491,7 @@
     </row>
     <row r="47" spans="1:16">
       <c r="A47" s="38" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="B47" s="38" t="s">
         <v>139</v>
@@ -15577,7 +15541,7 @@
     </row>
     <row r="48" spans="1:16">
       <c r="A48" s="38" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="B48" s="38" t="s">
         <v>139</v>
@@ -15619,7 +15583,7 @@
         <v>436</v>
       </c>
       <c r="O48" s="38" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="P48" s="38" t="s">
         <v>436</v>
@@ -15627,7 +15591,7 @@
     </row>
     <row r="49" spans="1:16">
       <c r="A49" s="38" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="B49" s="38" t="s">
         <v>139</v>
@@ -15677,7 +15641,7 @@
     </row>
     <row r="50" spans="1:16">
       <c r="A50" s="38" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B50" s="38" t="s">
         <v>139</v>
@@ -15722,12 +15686,12 @@
         <v>436</v>
       </c>
       <c r="P50" s="38" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="51" spans="1:16">
       <c r="A51" s="94" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="B51" s="38" t="s">
         <v>139</v>
@@ -15777,7 +15741,7 @@
     </row>
     <row r="52" spans="1:16">
       <c r="A52" s="38" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="B52" s="38" t="s">
         <v>139</v>
@@ -15827,7 +15791,7 @@
     </row>
     <row r="53" spans="1:16">
       <c r="A53" s="38" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="B53" s="38" t="s">
         <v>139</v>
@@ -15872,12 +15836,12 @@
         <v>436</v>
       </c>
       <c r="P53" s="38" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="54" spans="1:16">
       <c r="A54" s="38" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="B54" s="38" t="s">
         <v>139</v>
@@ -15919,7 +15883,7 @@
         <v>436</v>
       </c>
       <c r="O54" s="38" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="P54" s="38" t="s">
         <v>436</v>
@@ -15927,7 +15891,7 @@
     </row>
     <row r="55" spans="1:16">
       <c r="A55" s="38" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="B55" s="38" t="s">
         <v>139</v>
@@ -15977,7 +15941,7 @@
     </row>
     <row r="56" spans="1:16">
       <c r="A56" s="38" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="B56" s="38" t="s">
         <v>139</v>
@@ -16022,12 +15986,12 @@
         <v>436</v>
       </c>
       <c r="P56" s="38" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="57" spans="1:16">
       <c r="A57" s="38" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="B57" s="38" t="s">
         <v>139</v>
@@ -16077,7 +16041,7 @@
     </row>
     <row r="58" spans="1:16">
       <c r="A58" s="38" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="B58" s="38" t="s">
         <v>139</v>
@@ -16127,7 +16091,7 @@
     </row>
     <row r="59" spans="1:16">
       <c r="A59" s="38" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="B59" s="38" t="s">
         <v>139</v>
@@ -16172,12 +16136,12 @@
         <v>436</v>
       </c>
       <c r="P59" s="38" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="60" spans="1:16">
       <c r="A60" s="38" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="B60" s="38" t="s">
         <v>139</v>
@@ -16227,7 +16191,7 @@
     </row>
     <row r="61" spans="1:16">
       <c r="A61" s="38" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="B61" s="38" t="s">
         <v>139</v>
@@ -16277,7 +16241,7 @@
     </row>
     <row r="62" spans="1:16">
       <c r="A62" s="38" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="B62" s="38" t="s">
         <v>139</v>
@@ -16327,7 +16291,7 @@
     </row>
     <row r="63" spans="1:16">
       <c r="A63" s="38" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="B63" s="38" t="s">
         <v>139</v>
@@ -16377,7 +16341,7 @@
     </row>
     <row r="64" spans="1:16">
       <c r="A64" s="38" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="B64" s="38" t="s">
         <v>139</v>
@@ -16419,7 +16383,7 @@
         <v>436</v>
       </c>
       <c r="O64" s="38" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="P64" s="38" t="s">
         <v>436</v>
@@ -16427,7 +16391,7 @@
     </row>
     <row r="65" spans="1:16">
       <c r="A65" s="38" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="B65" s="38" t="s">
         <v>139</v>
@@ -16472,12 +16436,12 @@
         <v>436</v>
       </c>
       <c r="P65" s="38" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="66" spans="1:16">
       <c r="A66" s="38" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="B66" s="38" t="s">
         <v>139</v>
@@ -16522,12 +16486,12 @@
         <v>436</v>
       </c>
       <c r="P66" s="38" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="67" spans="1:16">
       <c r="A67" s="38" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="B67" s="38" t="s">
         <v>139</v>
@@ -16577,7 +16541,7 @@
     </row>
     <row r="68" spans="1:16">
       <c r="A68" s="38" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="B68" s="38" t="s">
         <v>139</v>
@@ -16627,7 +16591,7 @@
     </row>
     <row r="69" spans="1:16">
       <c r="A69" s="38" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="B69" s="38" t="s">
         <v>139</v>
@@ -16677,7 +16641,7 @@
     </row>
     <row r="70" spans="1:16">
       <c r="A70" s="38" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="B70" s="38" t="s">
         <v>139</v>
@@ -16722,12 +16686,12 @@
         <v>436</v>
       </c>
       <c r="P70" s="38" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="71" spans="1:16">
       <c r="A71" s="38" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="B71" s="38" t="s">
         <v>139</v>
@@ -16777,7 +16741,7 @@
     </row>
     <row r="72" spans="1:16">
       <c r="A72" s="38" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="B72" s="38" t="s">
         <v>139</v>
@@ -16819,7 +16783,7 @@
         <v>436</v>
       </c>
       <c r="O72" s="38" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="P72" s="38" t="s">
         <v>436</v>
@@ -16827,7 +16791,7 @@
     </row>
     <row r="73" spans="1:16">
       <c r="A73" s="38" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="B73" s="38" t="s">
         <v>139</v>
@@ -17078,7 +17042,7 @@
       <c r="H6" s="38"/>
       <c r="I6" s="38"/>
       <c r="J6" s="38" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="K6" s="38"/>
       <c r="L6" s="38"/>
@@ -17162,10 +17126,10 @@
         <v>5</v>
       </c>
       <c r="Q1" s="82" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="R1" s="98" t="s">
-        <v>1246</v>
+        <v>1236</v>
       </c>
       <c r="S1" s="98" t="s">
         <v>8</v>
@@ -17197,7 +17161,7 @@
         <v>46</v>
       </c>
       <c r="H2" s="38" t="s">
-        <v>1213</v>
+        <v>1205</v>
       </c>
       <c r="I2" s="38" t="s">
         <v>347</v>
@@ -17237,7 +17201,7 @@
         <v>46</v>
       </c>
       <c r="H3" s="38" t="s">
-        <v>1176</v>
+        <v>1168</v>
       </c>
       <c r="I3" s="38" t="s">
         <v>347</v>
@@ -17277,7 +17241,7 @@
         <v>15</v>
       </c>
       <c r="H4" s="38" t="s">
-        <v>1175</v>
+        <v>1167</v>
       </c>
       <c r="I4" s="38"/>
       <c r="J4" s="41" t="s">
@@ -17357,7 +17321,7 @@
       </c>
       <c r="G6" s="38"/>
       <c r="H6" s="38" t="s">
-        <v>1250</v>
+        <v>1240</v>
       </c>
       <c r="I6" s="38"/>
       <c r="J6" s="41" t="s">
@@ -17371,13 +17335,13 @@
       <c r="P6" s="38"/>
       <c r="Q6" s="38"/>
       <c r="R6" s="107" t="s">
-        <v>1247</v>
+        <v>1237</v>
       </c>
       <c r="S6" s="107" t="s">
-        <v>1248</v>
+        <v>1238</v>
       </c>
       <c r="T6" s="106" t="s">
-        <v>1249</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -17433,7 +17397,7 @@
         <v>15</v>
       </c>
       <c r="H8" s="38" t="s">
-        <v>1237</v>
+        <v>1227</v>
       </c>
       <c r="I8" s="38"/>
       <c r="J8" s="41" t="s">
@@ -17454,7 +17418,7 @@
       </c>
       <c r="P8" s="38"/>
       <c r="Q8" s="38" t="s">
-        <v>1238</v>
+        <v>1228</v>
       </c>
       <c r="R8" s="106"/>
       <c r="S8" s="106"/>
@@ -17481,7 +17445,7 @@
       </c>
       <c r="G9" s="38"/>
       <c r="H9" s="38" t="s">
-        <v>1181</v>
+        <v>1173</v>
       </c>
       <c r="I9" s="38" t="s">
         <v>739</v>
@@ -17521,10 +17485,10 @@
       </c>
       <c r="G10" s="38"/>
       <c r="H10" s="38" t="s">
-        <v>1182</v>
+        <v>1174</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="J10" s="38"/>
       <c r="K10" s="38" t="s">
@@ -17561,10 +17525,10 @@
       </c>
       <c r="G11" s="38"/>
       <c r="H11" s="38" t="s">
-        <v>1244</v>
+        <v>1234</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="J11" s="38"/>
       <c r="K11" s="41" t="s">
@@ -17601,7 +17565,7 @@
       </c>
       <c r="G12" s="38"/>
       <c r="H12" s="38" t="s">
-        <v>1240</v>
+        <v>1230</v>
       </c>
       <c r="I12" s="38" t="s">
         <v>740</v>
@@ -17651,10 +17615,10 @@
       </c>
       <c r="G13" s="38"/>
       <c r="H13" s="38" t="s">
-        <v>1241</v>
+        <v>1231</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>1242</v>
+        <v>1232</v>
       </c>
       <c r="J13" s="41" t="s">
         <v>712</v>
@@ -17691,7 +17655,7 @@
       </c>
       <c r="G14" s="38"/>
       <c r="H14" s="38" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="I14" s="38" t="s">
         <v>741</v>
@@ -17741,10 +17705,10 @@
       </c>
       <c r="G15" s="38"/>
       <c r="H15" s="38" t="s">
-        <v>1177</v>
+        <v>1169</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="J15" s="41" t="s">
         <v>716</v>
@@ -17781,10 +17745,10 @@
       </c>
       <c r="G16" s="38"/>
       <c r="H16" s="38" t="s">
-        <v>1178</v>
+        <v>1170</v>
       </c>
       <c r="I16" s="38" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="J16" s="41" t="s">
         <v>683</v>
@@ -17823,10 +17787,10 @@
       </c>
       <c r="G17" s="38"/>
       <c r="H17" s="38" t="s">
-        <v>1179</v>
+        <v>1171</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>1180</v>
+        <v>1172</v>
       </c>
       <c r="J17" s="41" t="s">
         <v>719</v>
@@ -17865,10 +17829,10 @@
         <v>46</v>
       </c>
       <c r="H18" s="38" t="s">
-        <v>1245</v>
+        <v>1235</v>
       </c>
       <c r="I18" s="38" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="J18" s="38"/>
       <c r="K18" s="38"/>
@@ -17905,10 +17869,10 @@
         <v>46</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>1239</v>
+        <v>1229</v>
       </c>
       <c r="I19" s="38" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="J19" s="38"/>
       <c r="K19" s="38"/>
@@ -17924,7 +17888,7 @@
     </row>
     <row r="20" spans="1:20">
       <c r="A20" s="58" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="B20" s="38">
         <v>0</v>
@@ -17945,7 +17909,7 @@
         <v>15</v>
       </c>
       <c r="H20" s="38" t="s">
-        <v>1243</v>
+        <v>1233</v>
       </c>
       <c r="I20" s="38" t="s">
         <v>347</v>
@@ -18111,7 +18075,7 @@
         <v>14</v>
       </c>
       <c r="M2" s="28" t="s">
-        <v>1234</v>
+        <v>1225</v>
       </c>
       <c r="N2" s="28">
         <v>2</v>
@@ -18131,10 +18095,10 @@
       <c r="S2" s="28"/>
       <c r="T2" s="28"/>
       <c r="U2" s="38" t="s">
-        <v>1225</v>
+        <v>1217</v>
       </c>
       <c r="V2" s="38" t="s">
-        <v>1226</v>
+        <v>1218</v>
       </c>
       <c r="W2" s="38" t="s">
         <v>347</v>
@@ -18178,7 +18142,7 @@
         <v>14</v>
       </c>
       <c r="M3" s="28" t="s">
-        <v>1230</v>
+        <v>1221</v>
       </c>
       <c r="N3" s="28"/>
       <c r="O3" s="28"/>
@@ -18186,19 +18150,19 @@
       <c r="Q3" s="38"/>
       <c r="R3" s="38"/>
       <c r="S3" s="41" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="T3" s="28" t="s">
-        <v>1227</v>
+        <v>1219</v>
       </c>
       <c r="U3" s="38" t="s">
-        <v>1231</v>
+        <v>1222</v>
       </c>
       <c r="V3" s="38" t="s">
-        <v>1232</v>
+        <v>1223</v>
       </c>
       <c r="W3" s="38" t="s">
-        <v>1233</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -18239,7 +18203,7 @@
         <v>14</v>
       </c>
       <c r="M4" s="28" t="s">
-        <v>1235</v>
+        <v>1226</v>
       </c>
       <c r="N4" s="28"/>
       <c r="O4" s="28"/>
@@ -18253,10 +18217,10 @@
       <c r="S4" s="28"/>
       <c r="T4" s="28"/>
       <c r="U4" s="38" t="s">
-        <v>1225</v>
+        <v>1217</v>
       </c>
       <c r="V4" s="38" t="s">
-        <v>1226</v>
+        <v>1218</v>
       </c>
       <c r="W4" s="38" t="s">
         <v>347</v>
@@ -18880,7 +18844,7 @@
       </c>
       <c r="G4" s="38"/>
       <c r="H4" s="38" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="I4" s="38" t="s">
         <v>350</v>
@@ -18920,7 +18884,7 @@
       </c>
       <c r="G5" s="38"/>
       <c r="H5" s="38" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="I5" s="38" t="s">
         <v>350</v>
@@ -19036,7 +19000,7 @@
         <v>784</v>
       </c>
       <c r="H9" s="38" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="I9" s="38" t="s">
         <v>350</v>
@@ -19477,7 +19441,7 @@
         <v>198</v>
       </c>
       <c r="J2" s="38" t="s">
-        <v>1186</v>
+        <v>1178</v>
       </c>
       <c r="K2" s="38">
         <f>B2</f>
@@ -19523,13 +19487,13 @@
         <v>202</v>
       </c>
       <c r="H3" s="38" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="I3" s="38" t="s">
         <v>20</v>
       </c>
       <c r="J3" s="38" t="s">
-        <v>1187</v>
+        <v>1179</v>
       </c>
       <c r="K3" s="38"/>
       <c r="L3" s="38" t="s">
@@ -19539,7 +19503,7 @@
         <v>335</v>
       </c>
       <c r="N3" s="38" t="s">
-        <v>1183</v>
+        <v>1175</v>
       </c>
       <c r="O3" s="38" t="s">
         <v>202</v>
@@ -19554,7 +19518,7 @@
         <v>1</v>
       </c>
       <c r="S3" s="38" t="s">
-        <v>1184</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -19565,7 +19529,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="41" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="D4" s="38" t="s">
         <v>12</v>
@@ -19586,7 +19550,7 @@
         <v>723</v>
       </c>
       <c r="J4" s="38" t="s">
-        <v>1188</v>
+        <v>1180</v>
       </c>
       <c r="K4" s="38"/>
       <c r="L4" s="38" t="s">
@@ -19596,7 +19560,7 @@
         <v>400</v>
       </c>
       <c r="N4" s="38" t="s">
-        <v>1185</v>
+        <v>1177</v>
       </c>
       <c r="O4" s="38"/>
       <c r="P4" s="38"/>
@@ -19629,13 +19593,13 @@
         <v>202</v>
       </c>
       <c r="H5" s="38" t="s">
+        <v>905</v>
+      </c>
+      <c r="I5" s="38" t="s">
         <v>906</v>
       </c>
-      <c r="I5" s="38" t="s">
-        <v>907</v>
-      </c>
       <c r="J5" s="38" t="s">
-        <v>1189</v>
+        <v>1181</v>
       </c>
       <c r="K5" s="38"/>
       <c r="L5" s="38" t="s">
@@ -19645,7 +19609,7 @@
         <v>335</v>
       </c>
       <c r="N5" s="38" t="s">
-        <v>1183</v>
+        <v>1175</v>
       </c>
       <c r="O5" s="38" t="s">
         <v>202</v>
@@ -19660,7 +19624,7 @@
         <v>1</v>
       </c>
       <c r="S5" s="38" t="s">
-        <v>1184</v>
+        <v>1176</v>
       </c>
     </row>
   </sheetData>
@@ -19724,7 +19688,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="107" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="D2" s="38" t="s">
         <v>12</v>
@@ -19905,7 +19869,7 @@
         <v>30</v>
       </c>
       <c r="I9" s="107" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="J9" s="38"/>
     </row>
@@ -20139,7 +20103,7 @@
         <v>30</v>
       </c>
       <c r="E19" s="110" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="F19" s="38"/>
       <c r="G19" s="38"/>
@@ -20156,7 +20120,7 @@
       </c>
       <c r="C20" s="38"/>
       <c r="D20" s="110" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="E20" s="110" t="s">
         <v>497</v>
@@ -20398,7 +20362,7 @@
         <v>630</v>
       </c>
       <c r="G1" s="39" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -20515,7 +20479,7 @@
       <c r="E7" s="38"/>
       <c r="F7" s="38"/>
       <c r="G7" s="38" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -20586,7 +20550,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="35" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B13" s="35"/>
       <c r="C13" s="35"/>
@@ -20604,7 +20568,7 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="80" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="B15" s="35"/>
       <c r="C15" s="35"/>
@@ -20744,7 +20708,7 @@
         <v>15</v>
       </c>
       <c r="H2" s="28" t="s">
-        <v>1274</v>
+        <v>1241</v>
       </c>
       <c r="I2" s="28" t="s">
         <v>197</v>
@@ -20771,7 +20735,7 @@
         <v>327</v>
       </c>
       <c r="S2" s="28" t="s">
-        <v>1229</v>
+        <v>1220</v>
       </c>
       <c r="T2" s="28" t="s">
         <v>411</v>
@@ -20914,7 +20878,7 @@
         <v>15</v>
       </c>
       <c r="H6" s="28" t="s">
-        <v>1214</v>
+        <v>1206</v>
       </c>
       <c r="I6" s="28" t="s">
         <v>723</v>
@@ -20963,7 +20927,7 @@
         <v>19</v>
       </c>
       <c r="H7" s="28" t="s">
-        <v>1191</v>
+        <v>1183</v>
       </c>
       <c r="I7" s="28" t="s">
         <v>329</v>
@@ -21049,10 +21013,10 @@
         <v>15</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>1215</v>
+        <v>1207</v>
       </c>
       <c r="I9" s="28" t="s">
-        <v>1190</v>
+        <v>1182</v>
       </c>
       <c r="J9" s="28" t="s">
         <v>197</v>
@@ -21092,7 +21056,7 @@
       </c>
       <c r="G10" s="50"/>
       <c r="H10" s="28" t="s">
-        <v>1192</v>
+        <v>1184</v>
       </c>
       <c r="I10" s="28"/>
       <c r="J10" s="28" t="s">
@@ -21141,13 +21105,13 @@
         <v>15</v>
       </c>
       <c r="H11" s="28" t="s">
-        <v>1193</v>
+        <v>1185</v>
       </c>
       <c r="I11" s="28" t="s">
         <v>197</v>
       </c>
       <c r="J11" s="28" t="s">
-        <v>1194</v>
+        <v>1186</v>
       </c>
       <c r="K11" s="28"/>
       <c r="L11" s="28"/>
@@ -21335,13 +21299,13 @@
         <v>15</v>
       </c>
       <c r="H15" s="28" t="s">
-        <v>1195</v>
+        <v>1187</v>
       </c>
       <c r="I15" s="28" t="s">
         <v>197</v>
       </c>
       <c r="J15" s="28" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="K15" s="28"/>
       <c r="L15" s="28"/>
@@ -21488,13 +21452,13 @@
         <v>257</v>
       </c>
       <c r="AK1" s="12" t="s">
-        <v>1208</v>
+        <v>1200</v>
       </c>
       <c r="AL1" s="12" t="s">
-        <v>1209</v>
+        <v>1201</v>
       </c>
       <c r="AM1" s="12" t="s">
-        <v>1207</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="2" spans="1:39">
@@ -21526,10 +21490,10 @@
       <c r="P2" s="38"/>
       <c r="Q2" s="38"/>
       <c r="R2" s="38" t="s">
-        <v>1216</v>
+        <v>1208</v>
       </c>
       <c r="S2" s="38" t="s">
-        <v>1217</v>
+        <v>1209</v>
       </c>
       <c r="T2" s="38"/>
       <c r="U2" s="38"/>
@@ -21904,10 +21868,10 @@
       <c r="P8" s="38"/>
       <c r="Q8" s="38"/>
       <c r="R8" s="38" t="s">
-        <v>1218</v>
+        <v>1210</v>
       </c>
       <c r="S8" s="38" t="s">
-        <v>1219</v>
+        <v>1211</v>
       </c>
       <c r="T8" s="38">
         <v>0</v>
@@ -22380,10 +22344,10 @@
       <c r="P16" s="38"/>
       <c r="Q16" s="38"/>
       <c r="R16" s="38" t="s">
+        <v>1153</v>
+      </c>
+      <c r="S16" s="38" t="s">
         <v>1154</v>
-      </c>
-      <c r="S16" s="38" t="s">
-        <v>1155</v>
       </c>
       <c r="T16" s="38"/>
       <c r="U16" s="38"/>
@@ -22521,13 +22485,13 @@
       <c r="AI18" s="38"/>
       <c r="AJ18" s="38"/>
       <c r="AK18" s="107" t="s">
-        <v>1210</v>
+        <v>1202</v>
       </c>
       <c r="AL18" s="106" t="s">
-        <v>1211</v>
+        <v>1203</v>
       </c>
       <c r="AM18" s="106" t="s">
-        <v>1212</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="19" spans="1:39">
@@ -22583,10 +22547,10 @@
         <v>30</v>
       </c>
       <c r="R19" s="38" t="s">
+        <v>1149</v>
+      </c>
+      <c r="S19" s="38" t="s">
         <v>1150</v>
-      </c>
-      <c r="S19" s="38" t="s">
-        <v>1151</v>
       </c>
       <c r="T19" s="41">
         <v>0</v>
@@ -22689,13 +22653,13 @@
       <c r="AI20" s="38"/>
       <c r="AJ20" s="38"/>
       <c r="AK20" s="107" t="s">
-        <v>1210</v>
+        <v>1202</v>
       </c>
       <c r="AL20" s="106" t="s">
-        <v>1211</v>
+        <v>1203</v>
       </c>
       <c r="AM20" s="106" t="s">
-        <v>1212</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="21" spans="1:39">
@@ -22770,13 +22734,13 @@
       <c r="AI21" s="38"/>
       <c r="AJ21" s="38"/>
       <c r="AK21" s="107" t="s">
-        <v>1210</v>
+        <v>1202</v>
       </c>
       <c r="AL21" s="106" t="s">
-        <v>1211</v>
+        <v>1203</v>
       </c>
       <c r="AM21" s="106" t="s">
-        <v>1212</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="22" spans="1:39">
@@ -22914,7 +22878,7 @@
       <c r="P24" s="38"/>
       <c r="Q24" s="38"/>
       <c r="R24" s="38" t="s">
-        <v>1196</v>
+        <v>1188</v>
       </c>
       <c r="S24" s="38"/>
       <c r="T24" s="41"/>
@@ -23128,7 +23092,7 @@
       <c r="P28" s="38"/>
       <c r="Q28" s="38"/>
       <c r="R28" s="38" t="s">
-        <v>1197</v>
+        <v>1189</v>
       </c>
       <c r="S28" s="38"/>
       <c r="T28" s="41">
@@ -23278,10 +23242,10 @@
       <c r="P30" s="38"/>
       <c r="Q30" s="38"/>
       <c r="R30" s="38" t="s">
+        <v>1151</v>
+      </c>
+      <c r="S30" s="38" t="s">
         <v>1152</v>
-      </c>
-      <c r="S30" s="38" t="s">
-        <v>1153</v>
       </c>
       <c r="T30" s="38">
         <v>0</v>
@@ -23813,7 +23777,7 @@
       <c r="P39" s="38"/>
       <c r="Q39" s="38"/>
       <c r="R39" s="38" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="S39" s="38" t="s">
         <v>347</v>
@@ -23843,7 +23807,7 @@
     </row>
     <row r="40" spans="1:39">
       <c r="A40" s="58" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B40" s="60">
         <v>1</v>
@@ -23870,10 +23834,10 @@
       <c r="P40" s="38"/>
       <c r="Q40" s="38"/>
       <c r="R40" s="38" t="s">
+        <v>914</v>
+      </c>
+      <c r="S40" s="38" t="s">
         <v>915</v>
-      </c>
-      <c r="S40" s="38" t="s">
-        <v>916</v>
       </c>
       <c r="T40" s="38"/>
       <c r="U40" s="38"/>
@@ -24053,16 +24017,16 @@
       <c r="L3" s="100"/>
       <c r="M3" s="100"/>
       <c r="N3" s="100" t="s">
+        <v>852</v>
+      </c>
+      <c r="O3" s="100" t="s">
         <v>853</v>
-      </c>
-      <c r="O3" s="100" t="s">
-        <v>854</v>
       </c>
       <c r="P3" s="100" t="s">
         <v>42</v>
       </c>
       <c r="Q3" s="100" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="R3" s="100" t="s">
         <v>12</v>
@@ -24123,7 +24087,7 @@
         <v>249</v>
       </c>
       <c r="F5" s="100" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="G5" s="100"/>
       <c r="H5" s="100"/>
@@ -24195,7 +24159,7 @@
         <v>249</v>
       </c>
       <c r="F7" s="100" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="G7" s="100"/>
       <c r="H7" s="100"/>
@@ -24327,16 +24291,16 @@
         <v>12</v>
       </c>
       <c r="N10" s="100" t="s">
+        <v>855</v>
+      </c>
+      <c r="O10" s="100" t="s">
         <v>856</v>
-      </c>
-      <c r="O10" s="100" t="s">
-        <v>857</v>
       </c>
       <c r="P10" s="100" t="s">
         <v>28</v>
       </c>
       <c r="Q10" s="100" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="R10" s="100" t="s">
         <v>12</v>
@@ -24468,7 +24432,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="102" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="D14" s="100" t="s">
         <v>12</v>
@@ -24602,7 +24566,7 @@
     </row>
     <row r="18" spans="1:22">
       <c r="A18" s="97" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="B18" s="104">
         <v>1</v>
@@ -24612,7 +24576,7 @@
       </c>
       <c r="D18" s="104"/>
       <c r="E18" s="102" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="F18" s="100"/>
       <c r="G18" s="100"/>
@@ -24635,7 +24599,7 @@
       <c r="T18" s="100"/>
       <c r="U18" s="100"/>
       <c r="V18" s="102" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
   </sheetData>
@@ -24763,7 +24727,7 @@
       </c>
       <c r="J2" s="38"/>
       <c r="K2" s="38" t="s">
-        <v>1224</v>
+        <v>1216</v>
       </c>
       <c r="L2" s="38"/>
       <c r="M2" s="38"/>
@@ -24802,10 +24766,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="38" t="s">
+        <v>860</v>
+      </c>
+      <c r="L3" s="38" t="s">
         <v>861</v>
-      </c>
-      <c r="L3" s="38" t="s">
-        <v>862</v>
       </c>
       <c r="M3" s="38"/>
       <c r="N3" s="38"/>
@@ -24841,11 +24805,11 @@
       <c r="I4" s="38"/>
       <c r="J4" s="38"/>
       <c r="K4" s="38" t="s">
-        <v>1221</v>
+        <v>1213</v>
       </c>
       <c r="L4" s="38"/>
       <c r="M4" s="38" t="s">
-        <v>1220</v>
+        <v>1212</v>
       </c>
       <c r="N4" s="38"/>
       <c r="O4" s="38"/>
@@ -24880,10 +24844,10 @@
       <c r="I5" s="38"/>
       <c r="J5" s="38"/>
       <c r="K5" s="38" t="s">
+        <v>862</v>
+      </c>
+      <c r="L5" s="38" t="s">
         <v>863</v>
-      </c>
-      <c r="L5" s="38" t="s">
-        <v>864</v>
       </c>
       <c r="M5" s="38"/>
       <c r="N5" s="38" t="s">
@@ -24929,7 +24893,7 @@
       <c r="I6" s="38"/>
       <c r="J6" s="38"/>
       <c r="K6" s="38" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="L6" s="38"/>
       <c r="M6" s="38"/>
@@ -24940,7 +24904,7 @@
         <v>744</v>
       </c>
       <c r="P6" s="38" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="Q6" s="38"/>
       <c r="R6" s="38"/>
@@ -24976,26 +24940,26 @@
       <c r="I7" s="38"/>
       <c r="J7" s="38"/>
       <c r="K7" s="38" t="s">
+        <v>882</v>
+      </c>
+      <c r="L7" s="38" t="s">
         <v>883</v>
-      </c>
-      <c r="L7" s="38" t="s">
-        <v>884</v>
       </c>
       <c r="M7" s="38"/>
       <c r="N7" s="38" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="O7" s="38" t="s">
         <v>234</v>
       </c>
       <c r="P7" s="38" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="Q7" s="41" t="s">
         <v>80</v>
       </c>
       <c r="R7" s="38" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="S7" s="38"/>
       <c r="T7" s="38"/>
@@ -25033,10 +24997,10 @@
       </c>
       <c r="J8" s="38"/>
       <c r="K8" s="38" t="s">
+        <v>867</v>
+      </c>
+      <c r="L8" s="38" t="s">
         <v>868</v>
-      </c>
-      <c r="L8" s="38" t="s">
-        <v>869</v>
       </c>
       <c r="M8" s="38"/>
       <c r="N8" s="38" t="s">
@@ -25076,7 +25040,7 @@
       <c r="I9" s="38"/>
       <c r="J9" s="38"/>
       <c r="K9" s="38" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="L9" s="38"/>
       <c r="M9" s="38"/>
@@ -25093,7 +25057,7 @@
       <c r="T9" s="38"/>
       <c r="U9" s="38"/>
       <c r="V9" s="38" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="W9" s="38"/>
     </row>
@@ -25119,10 +25083,10 @@
       <c r="I10" s="38"/>
       <c r="J10" s="38"/>
       <c r="K10" s="38" t="s">
+        <v>870</v>
+      </c>
+      <c r="L10" s="38" t="s">
         <v>871</v>
-      </c>
-      <c r="L10" s="38" t="s">
-        <v>872</v>
       </c>
       <c r="M10" s="38"/>
       <c r="N10" s="38"/>
@@ -25160,10 +25124,10 @@
       <c r="I11" s="38"/>
       <c r="J11" s="38"/>
       <c r="K11" s="38" t="s">
+        <v>845</v>
+      </c>
+      <c r="L11" s="38" t="s">
         <v>846</v>
-      </c>
-      <c r="L11" s="38" t="s">
-        <v>847</v>
       </c>
       <c r="M11" s="38"/>
       <c r="N11" s="38"/>
@@ -25201,10 +25165,10 @@
       <c r="I12" s="38"/>
       <c r="J12" s="38"/>
       <c r="K12" s="38" t="s">
+        <v>872</v>
+      </c>
+      <c r="L12" s="38" t="s">
         <v>873</v>
-      </c>
-      <c r="L12" s="38" t="s">
-        <v>874</v>
       </c>
       <c r="M12" s="38"/>
       <c r="N12" s="38" t="s">
@@ -25246,10 +25210,10 @@
       <c r="I13" s="38"/>
       <c r="J13" s="38"/>
       <c r="K13" s="38" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="L13" s="38" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="M13" s="38"/>
       <c r="N13" s="38" t="s">
@@ -25328,10 +25292,10 @@
       <c r="I15" s="38"/>
       <c r="J15" s="38"/>
       <c r="K15" s="38" t="s">
+        <v>876</v>
+      </c>
+      <c r="L15" s="38" t="s">
         <v>877</v>
-      </c>
-      <c r="L15" s="38" t="s">
-        <v>878</v>
       </c>
       <c r="M15" s="38"/>
       <c r="N15" s="38" t="s">
@@ -25373,7 +25337,7 @@
       <c r="I16" s="38"/>
       <c r="J16" s="38"/>
       <c r="K16" s="38" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="L16" s="38"/>
       <c r="M16" s="38"/>
@@ -25414,7 +25378,7 @@
       <c r="I17" s="38"/>
       <c r="J17" s="38"/>
       <c r="K17" s="38" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="L17" s="38"/>
       <c r="M17" s="38"/>
@@ -25459,7 +25423,7 @@
       </c>
       <c r="J18" s="38"/>
       <c r="K18" s="38" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="L18" s="38"/>
       <c r="M18" s="38"/>
@@ -25476,10 +25440,10 @@
       <c r="T18" s="38"/>
       <c r="U18" s="38"/>
       <c r="V18" s="38" t="s">
+        <v>879</v>
+      </c>
+      <c r="W18" s="38" t="s">
         <v>880</v>
-      </c>
-      <c r="W18" s="38" t="s">
-        <v>881</v>
       </c>
     </row>
     <row r="19" spans="1:23">
@@ -25504,7 +25468,7 @@
       <c r="I19" s="38"/>
       <c r="J19" s="38"/>
       <c r="K19" s="38" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="L19" s="38"/>
       <c r="M19" s="38"/>
@@ -25521,7 +25485,7 @@
       <c r="T19" s="38"/>
       <c r="U19" s="38"/>
       <c r="V19" s="38" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="W19" s="38"/>
     </row>
@@ -25547,7 +25511,7 @@
       <c r="I20" s="38"/>
       <c r="J20" s="38"/>
       <c r="K20" s="38" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="L20" s="38"/>
       <c r="M20" s="38"/>
@@ -25588,7 +25552,7 @@
       <c r="I21" s="38"/>
       <c r="J21" s="38"/>
       <c r="K21" s="38" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="38"/>
@@ -25637,7 +25601,7 @@
       </c>
       <c r="J22" s="38"/>
       <c r="K22" s="38" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="38"/>
@@ -25703,7 +25667,7 @@
       </c>
       <c r="L24" s="38"/>
       <c r="M24" s="106" t="s">
-        <v>1220</v>
+        <v>1212</v>
       </c>
       <c r="N24" s="38"/>
       <c r="O24" s="38"/>
@@ -25738,10 +25702,10 @@
       <c r="I25" s="38"/>
       <c r="J25" s="38"/>
       <c r="K25" s="38" t="s">
+        <v>899</v>
+      </c>
+      <c r="L25" s="38" t="s">
         <v>900</v>
-      </c>
-      <c r="L25" s="38" t="s">
-        <v>901</v>
       </c>
       <c r="M25" s="38"/>
       <c r="N25" s="38" t="s">
@@ -25837,7 +25801,7 @@
       <c r="I28" s="38"/>
       <c r="J28" s="38"/>
       <c r="K28" s="38" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="L28" s="38"/>
       <c r="M28" s="38"/>
@@ -25874,7 +25838,7 @@
       <c r="I29" s="38"/>
       <c r="J29" s="38"/>
       <c r="K29" s="38" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="L29" s="38"/>
       <c r="M29" s="38"/>
@@ -25915,14 +25879,14 @@
       <c r="I30" s="38"/>
       <c r="J30" s="38"/>
       <c r="K30" s="38" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="L30" s="38"/>
       <c r="M30" s="38"/>
       <c r="N30" s="38"/>
       <c r="O30" s="38"/>
       <c r="P30" s="38" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="Q30" s="38"/>
       <c r="R30" s="38"/>
@@ -25997,14 +25961,14 @@
       </c>
       <c r="J32" s="38"/>
       <c r="K32" s="38" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="L32" s="38"/>
       <c r="M32" s="38"/>
       <c r="N32" s="38"/>
       <c r="O32" s="38"/>
       <c r="P32" s="38" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="Q32" s="38"/>
       <c r="R32" s="38"/>
@@ -26036,7 +26000,7 @@
       <c r="I33" s="38"/>
       <c r="J33" s="38"/>
       <c r="K33" s="38" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="L33" s="38"/>
       <c r="M33" s="38"/>
@@ -26098,7 +26062,7 @@
         <v>1</v>
       </c>
       <c r="C35" s="107" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="D35" s="38" t="s">
         <v>12</v>
@@ -26110,7 +26074,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="107" t="s">
-        <v>1222</v>
+        <v>1214</v>
       </c>
       <c r="H35" s="38" t="s">
         <v>523</v>
@@ -26120,7 +26084,7 @@
       </c>
       <c r="J35" s="38"/>
       <c r="K35" s="38" t="s">
-        <v>1223</v>
+        <v>1215</v>
       </c>
       <c r="L35" s="38"/>
       <c r="M35" s="38"/>
@@ -26143,7 +26107,7 @@
         <v>1</v>
       </c>
       <c r="C36" s="41" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="D36" s="38" t="s">
         <v>13</v>
@@ -26165,7 +26129,7 @@
       </c>
       <c r="J36" s="38"/>
       <c r="K36" s="38" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="L36" s="38"/>
       <c r="M36" s="38"/>
@@ -26174,7 +26138,7 @@
         <v>762</v>
       </c>
       <c r="P36" s="38" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="Q36" s="38"/>
       <c r="R36" s="38"/>

</xml_diff>

<commit_message>
SHD sanity suite getting flight numbers and BagTagDisplay changes- 17-11-2025
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Harshitha Rajesh\Copa_SHD_API_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E83739-1E8F-4695-8406-2A89B3C3A83B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B90428-8A08-4503-BC4C-60B5220BB06D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="6" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="32" activeTab="37" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4654" uniqueCount="1380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4652" uniqueCount="1377">
   <si>
     <t>Scenario</t>
   </si>
@@ -3936,9 +3936,6 @@
     <t>BRIN</t>
   </si>
   <si>
-    <t>2025-10-30T06:30:00</t>
-  </si>
-  <si>
     <t>2025-10-30T09:58:00</t>
   </si>
   <si>
@@ -3975,15 +3972,6 @@
     <t>2025-10-29T09:58:00</t>
   </si>
   <si>
-    <t>ARBEWD</t>
-  </si>
-  <si>
-    <t>HAYWOOD</t>
-  </si>
-  <si>
-    <t>HOPPE</t>
-  </si>
-  <si>
     <t>ARBL0L</t>
   </si>
   <si>
@@ -4029,197 +4017,199 @@
     <t>2025-11-19T06:37:00</t>
   </si>
   <si>
-    <t>BLRX1D</t>
-  </si>
-  <si>
-    <t>SHAVON</t>
-  </si>
-  <si>
-    <t>GAYLORD</t>
-  </si>
-  <si>
-    <t>BLRX3U</t>
-  </si>
-  <si>
-    <t>RENAY</t>
-  </si>
-  <si>
-    <t>OBERBRUNNER</t>
-  </si>
-  <si>
-    <t>BLRYG1</t>
-  </si>
-  <si>
-    <t>8DE80AD4CMCMRPCT029C62224E</t>
-  </si>
-  <si>
-    <t>BLRYXH</t>
-  </si>
-  <si>
     <t>2025-11-18T07:50:00</t>
   </si>
   <si>
-    <t>BLRYYL</t>
-  </si>
-  <si>
-    <t>2302152740340</t>
-  </si>
-  <si>
-    <t>2302152740341</t>
-  </si>
-  <si>
-    <t>BLRYZI</t>
-  </si>
-  <si>
-    <t>2302152740342</t>
-  </si>
-  <si>
-    <t>2302152740343</t>
-  </si>
-  <si>
-    <t>BLRY3S</t>
-  </si>
-  <si>
-    <t>BLRY5Z</t>
-  </si>
-  <si>
-    <t>BLRZBU</t>
-  </si>
-  <si>
-    <t>BLRZCU</t>
-  </si>
-  <si>
-    <t>BLRZDI</t>
-  </si>
-  <si>
     <t>2025-11-19T16:10:00</t>
   </si>
   <si>
     <t>2025-11-19T19:20:00</t>
   </si>
   <si>
-    <t>2302152740348</t>
-  </si>
-  <si>
-    <t>2302152740349</t>
-  </si>
-  <si>
-    <t>BLRZFT</t>
-  </si>
-  <si>
     <t>2025-11-23T10:47:00</t>
   </si>
   <si>
     <t>2025-11-23T13:58:00</t>
   </si>
   <si>
-    <t>2302152740351</t>
-  </si>
-  <si>
-    <t>BLRZI2</t>
-  </si>
-  <si>
-    <t>BLRZJ0</t>
-  </si>
-  <si>
-    <t>BLRZKD</t>
-  </si>
-  <si>
-    <t>2302152740354</t>
-  </si>
-  <si>
-    <t>BLRZLB</t>
-  </si>
-  <si>
-    <t>2302152740355</t>
-  </si>
-  <si>
-    <t>BLRZL5</t>
-  </si>
-  <si>
     <t>2025-11-18T10:06:00</t>
   </si>
   <si>
     <t>2025-11-18T16:18:00</t>
   </si>
   <si>
-    <t>BLRZSM</t>
-  </si>
-  <si>
-    <t>BLRZUO</t>
-  </si>
-  <si>
-    <t>BLRZVI</t>
-  </si>
-  <si>
-    <t>BLRZWI</t>
-  </si>
-  <si>
-    <t>BLRZXK</t>
-  </si>
-  <si>
-    <t>BLRZY4</t>
-  </si>
-  <si>
-    <t>BLRZ0M</t>
-  </si>
-  <si>
     <t>2025-11-19T07:15:00</t>
   </si>
   <si>
     <t>2025-11-19T10:41:00</t>
   </si>
   <si>
-    <t>2302152740360</t>
-  </si>
-  <si>
-    <t>BLRZ10</t>
-  </si>
-  <si>
-    <t>BLRZ4O</t>
-  </si>
-  <si>
-    <t>BLR0CJ</t>
-  </si>
-  <si>
-    <t>BLR0DH</t>
-  </si>
-  <si>
-    <t>BLR0EE</t>
-  </si>
-  <si>
     <t>2025-11-19T06:30:00</t>
   </si>
   <si>
     <t>2025-11-19T16:11:00</t>
   </si>
   <si>
-    <t>BLR0G5</t>
-  </si>
-  <si>
     <t>2025-11-19T00:10:00</t>
   </si>
   <si>
     <t>2025-11-19T08:11:00</t>
   </si>
   <si>
-    <t>BLVVEI</t>
-  </si>
-  <si>
-    <t>2302152740587</t>
-  </si>
-  <si>
-    <t>BLVYYM</t>
-  </si>
-  <si>
-    <t>2302152740603</t>
+    <t>BLV1OA</t>
+  </si>
+  <si>
+    <t>2302152740655</t>
+  </si>
+  <si>
+    <t>2302152740656</t>
+  </si>
+  <si>
+    <t>BLV1U0</t>
+  </si>
+  <si>
+    <t>BLV1U1</t>
+  </si>
+  <si>
+    <t>BLV1VZ</t>
+  </si>
+  <si>
+    <t>RVPRUM</t>
+  </si>
+  <si>
+    <t>2302282731720</t>
+  </si>
+  <si>
+    <t>RVPV2A</t>
+  </si>
+  <si>
+    <t>kmwnmzukom2xnovsjsozjs2orv</t>
+  </si>
+  <si>
+    <t>RVPZRO</t>
+  </si>
+  <si>
+    <t>RVP0JR</t>
+  </si>
+  <si>
+    <t>2302282731724</t>
+  </si>
+  <si>
+    <t>2302282731725</t>
+  </si>
+  <si>
+    <t>RVP1SH</t>
+  </si>
+  <si>
+    <t>RVP2LU</t>
+  </si>
+  <si>
+    <t>RVP21N</t>
+  </si>
+  <si>
+    <t>RVP3KF</t>
+  </si>
+  <si>
+    <t>RVP4BC</t>
+  </si>
+  <si>
+    <t>2302282731730</t>
+  </si>
+  <si>
+    <t>2302282731731</t>
+  </si>
+  <si>
+    <t>RVP50O</t>
+  </si>
+  <si>
+    <t>2302282731733</t>
+  </si>
+  <si>
+    <t>RVQAWC</t>
+  </si>
+  <si>
+    <t>RVQBCE</t>
+  </si>
+  <si>
+    <t>RVQBNL</t>
+  </si>
+  <si>
+    <t>2302282731734</t>
+  </si>
+  <si>
+    <t>RVQBZT</t>
+  </si>
+  <si>
+    <t>2302282731735</t>
+  </si>
+  <si>
+    <t>RVQCMT</t>
+  </si>
+  <si>
+    <t>RVQFGX</t>
+  </si>
+  <si>
+    <t>RVQGAI</t>
+  </si>
+  <si>
+    <t>RVQGO2</t>
+  </si>
+  <si>
+    <t>RVQG0V</t>
+  </si>
+  <si>
+    <t>RVQHUO</t>
+  </si>
+  <si>
+    <t>2302282731742</t>
+  </si>
+  <si>
+    <t>RVQISK</t>
+  </si>
+  <si>
+    <t>RVQKUM</t>
+  </si>
+  <si>
+    <t>RVQL3C</t>
+  </si>
+  <si>
+    <t>RVQMZC</t>
+  </si>
+  <si>
+    <t>RVQPWT</t>
+  </si>
+  <si>
+    <t>RVSXOT</t>
+  </si>
+  <si>
+    <t>ALDA</t>
+  </si>
+  <si>
+    <t>WAELCHI</t>
+  </si>
+  <si>
+    <t>RVSZQ4</t>
+  </si>
+  <si>
+    <t>BLAIR</t>
+  </si>
+  <si>
+    <t>GUTKOWSKI</t>
+  </si>
+  <si>
+    <t>RVS1JN</t>
+  </si>
+  <si>
+    <t>ERICH</t>
+  </si>
+  <si>
+    <t>STRACKE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="25">
     <font>
       <sz val="11"/>
@@ -5277,24 +5267,24 @@
   <dimension ref="A1:AC25"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="52.77734375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="18.44140625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.44140625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="8.21875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.5546875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="11.21875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="10.44140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.21875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="10.44140625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="11.21875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.21875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="11.6640625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="12.6640625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="9.44140625"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="12.6640625"/>
+    <col min="1" max="1" width="52.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -5525,7 +5515,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="32" t="s">
-        <v>1360</v>
+        <v>1330</v>
       </c>
       <c r="I4" s="32" t="s">
         <v>313</v>
@@ -5580,7 +5570,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="32" t="s">
-        <v>1361</v>
+        <v>1331</v>
       </c>
       <c r="I5" s="104" t="s">
         <v>194</v>
@@ -6179,7 +6169,7 @@
       </c>
       <c r="G16" s="104"/>
       <c r="H16" s="104" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="I16" s="104" t="s">
         <v>570</v>
@@ -6273,7 +6263,7 @@
       </c>
       <c r="G18" s="104"/>
       <c r="H18" s="104" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="I18" s="104" t="s">
         <v>20</v>
@@ -6609,16 +6599,16 @@
   <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.88671875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
-    <col min="3" max="3" customWidth="true" style="25" width="17.5546875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="29.77734375"/>
-    <col min="5" max="5" customWidth="true" width="14.33203125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="14.33203125"/>
-    <col min="7" max="11" customWidth="true" style="25" width="14.33203125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="13.77734375"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.5546875"/>
+    <col min="1" max="1" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" style="25" customWidth="1"/>
+    <col min="4" max="4" width="29.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="11" width="14.33203125" style="25" customWidth="1"/>
+    <col min="12" max="12" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -6673,13 +6663,13 @@
         <v>2</v>
       </c>
       <c r="C2" s="37" t="s">
-        <v>1312</v>
+        <v>1308</v>
       </c>
       <c r="D2" s="40" t="s">
-        <v>1313</v>
+        <v>1309</v>
       </c>
       <c r="E2" s="40" t="s">
-        <v>1311</v>
+        <v>1307</v>
       </c>
       <c r="F2" s="37"/>
       <c r="G2" s="105" t="s">
@@ -6786,19 +6776,19 @@
   <dimension ref="A1:AL15"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="52.109375"/>
-    <col min="2" max="2" customWidth="true" style="25" width="16.5546875"/>
-    <col min="3" max="3" customWidth="true" style="25" width="19.88671875"/>
-    <col min="4" max="4" customWidth="true" style="25" width="18.77734375"/>
-    <col min="5" max="6" customWidth="true" style="25" width="12.88671875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="25" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="25" width="11.88671875"/>
-    <col min="9" max="9" style="25" width="8.77734375"/>
-    <col min="10" max="10" customWidth="true" style="25" width="17.88671875"/>
-    <col min="11" max="11" customWidth="true" style="25" width="14.21875"/>
-    <col min="12" max="37" style="25" width="8.77734375"/>
-    <col min="38" max="38" bestFit="true" customWidth="true" style="25" width="15.44140625"/>
-    <col min="39" max="16384" style="25" width="8.77734375"/>
+    <col min="1" max="1" width="52.109375" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" style="25" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" style="25" customWidth="1"/>
+    <col min="4" max="4" width="18.77734375" style="25" customWidth="1"/>
+    <col min="5" max="6" width="12.88671875" style="25" customWidth="1"/>
+    <col min="7" max="7" width="15" style="25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" style="25" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.77734375" style="25"/>
+    <col min="10" max="10" width="17.88671875" style="25" customWidth="1"/>
+    <col min="11" max="11" width="14.21875" style="25" customWidth="1"/>
+    <col min="12" max="37" width="8.77734375" style="25"/>
+    <col min="38" max="38" width="15.44140625" style="25" bestFit="1" customWidth="1"/>
+    <col min="39" max="16384" width="8.77734375" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -7213,13 +7203,13 @@
         <v>43</v>
       </c>
       <c r="I7" s="37" t="s">
-        <v>1328</v>
+        <v>1338</v>
       </c>
       <c r="J7" s="37" t="s">
-        <v>1329</v>
+        <v>1339</v>
       </c>
       <c r="K7" s="37" t="s">
-        <v>1330</v>
+        <v>1340</v>
       </c>
       <c r="L7" s="37"/>
       <c r="M7" s="37"/>
@@ -7415,13 +7405,13 @@
         <v>43</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>1331</v>
+        <v>1327</v>
       </c>
       <c r="J10" s="37" t="s">
-        <v>1332</v>
+        <v>1328</v>
       </c>
       <c r="K10" s="37" t="s">
-        <v>1333</v>
+        <v>1329</v>
       </c>
       <c r="L10" s="37"/>
       <c r="M10" s="37"/>
@@ -7778,15 +7768,15 @@
   <dimension ref="A1:M26"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="25" width="43.21875"/>
-    <col min="2" max="2" customWidth="true" style="25" width="15.77734375"/>
-    <col min="3" max="3" customWidth="true" style="25" width="17.77734375"/>
-    <col min="4" max="4" customWidth="true" style="25" width="16.77734375"/>
-    <col min="5" max="5" customWidth="true" style="25" width="15.6640625"/>
-    <col min="6" max="11" style="25" width="8.77734375"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="25" width="44.88671875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="11.88671875"/>
-    <col min="14" max="16384" style="25" width="8.77734375"/>
+    <col min="1" max="1" width="43.21875" style="25" customWidth="1"/>
+    <col min="2" max="2" width="15.77734375" style="25" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" style="25" customWidth="1"/>
+    <col min="4" max="4" width="16.77734375" style="25" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" style="25" customWidth="1"/>
+    <col min="6" max="11" width="8.77734375" style="25"/>
+    <col min="12" max="12" width="44.88671875" style="25" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.88671875" style="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.77734375" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -8854,22 +8844,22 @@
   <dimension ref="A1:V11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="51.77734375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.44140625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="17.5546875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="11" max="12" bestFit="true" customWidth="true" width="15.33203125"/>
-    <col min="13" max="13" customWidth="true" width="13.88671875"/>
-    <col min="14" max="14" customWidth="true" width="12.6640625"/>
-    <col min="15" max="15" customWidth="true" width="11.44140625"/>
-    <col min="16" max="16" customWidth="true" width="7.77734375"/>
-    <col min="17" max="18" customWidth="true" width="10.6640625"/>
-    <col min="19" max="19" customWidth="true" width="11.77734375"/>
-    <col min="20" max="20" customWidth="true" width="8.77734375"/>
-    <col min="21" max="21" customWidth="true" width="10.77734375"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="1" max="1" width="51.77734375" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.88671875" customWidth="1"/>
+    <col min="14" max="14" width="12.6640625" customWidth="1"/>
+    <col min="15" max="15" width="11.44140625" customWidth="1"/>
+    <col min="16" max="16" width="7.77734375" customWidth="1"/>
+    <col min="17" max="18" width="10.6640625" customWidth="1"/>
+    <col min="19" max="19" width="11.77734375" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" customWidth="1"/>
+    <col min="21" max="21" width="10.77734375" customWidth="1"/>
+    <col min="22" max="22" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -9081,16 +9071,16 @@
       <c r="H4" s="37"/>
       <c r="I4" s="37"/>
       <c r="J4" s="37" t="s">
-        <v>1324</v>
+        <v>1335</v>
       </c>
       <c r="K4" s="37" t="s">
-        <v>1317</v>
+        <v>1313</v>
       </c>
       <c r="L4" s="37" t="s">
         <v>578</v>
       </c>
       <c r="M4" s="37" t="s">
-        <v>1316</v>
+        <v>1312</v>
       </c>
       <c r="N4" s="37" t="s">
         <v>578</v>
@@ -9177,16 +9167,16 @@
         <v>30</v>
       </c>
       <c r="J6" s="37" t="s">
-        <v>1308</v>
+        <v>1304</v>
       </c>
       <c r="K6" s="37" t="s">
-        <v>1310</v>
+        <v>1306</v>
       </c>
       <c r="L6" s="37" t="s">
         <v>578</v>
       </c>
       <c r="M6" s="37" t="s">
-        <v>1309</v>
+        <v>1305</v>
       </c>
       <c r="N6" s="37" t="s">
         <v>578</v>
@@ -9233,28 +9223,28 @@
       <c r="V8" s="136"/>
     </row>
     <row r="11" spans="1:22">
-      <c r="O11" s="0">
+      <c r="O11">
         <v>14</v>
       </c>
-      <c r="P11" s="0">
+      <c r="P11">
         <v>15</v>
       </c>
-      <c r="Q11" s="0">
+      <c r="Q11">
         <v>16</v>
       </c>
-      <c r="R11" s="0">
+      <c r="R11">
         <v>17</v>
       </c>
-      <c r="S11" s="0">
+      <c r="S11">
         <v>18</v>
       </c>
-      <c r="T11" s="0">
+      <c r="T11">
         <v>19</v>
       </c>
-      <c r="U11" s="0">
+      <c r="U11">
         <v>20</v>
       </c>
-      <c r="V11" s="0">
+      <c r="V11">
         <v>21</v>
       </c>
     </row>
@@ -9278,12 +9268,12 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="76.21875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="13.44140625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="16.6640625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="1" max="1" width="76.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -9408,17 +9398,17 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="68.109375"/>
-    <col min="2" max="2" customWidth="true" style="25" width="12.5546875"/>
-    <col min="3" max="3" customWidth="true" style="25" width="12.33203125"/>
-    <col min="4" max="4" customWidth="true" style="25" width="9.6640625"/>
-    <col min="5" max="5" customWidth="true" style="25" width="17.21875"/>
-    <col min="6" max="6" customWidth="true" style="25" width="12.5546875"/>
-    <col min="7" max="10" style="25" width="8.77734375"/>
-    <col min="11" max="11" customWidth="true" style="25" width="10.6640625"/>
-    <col min="12" max="12" customWidth="true" style="25" width="12.21875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="15.33203125"/>
-    <col min="14" max="16384" style="25" width="8.77734375"/>
+    <col min="1" max="1" width="68.109375" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" style="25" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" style="25" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" style="25" customWidth="1"/>
+    <col min="5" max="5" width="17.21875" style="25" customWidth="1"/>
+    <col min="6" max="6" width="12.5546875" style="25" customWidth="1"/>
+    <col min="7" max="10" width="8.77734375" style="25"/>
+    <col min="11" max="11" width="10.6640625" style="25" customWidth="1"/>
+    <col min="12" max="12" width="12.21875" style="25" customWidth="1"/>
+    <col min="13" max="13" width="15.33203125" style="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.77734375" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -9844,12 +9834,12 @@
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.5546875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="11.77734375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="29.5546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="11.0"/>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -9925,7 +9915,7 @@
         <v>910</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>1325</v>
+        <v>1336</v>
       </c>
       <c r="E5" s="37" t="s">
         <v>911</v>
@@ -9950,12 +9940,12 @@
   <dimension ref="A1:AA9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.5546875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.44140625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="21.88671875"/>
+    <col min="1" max="1" width="33.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="21.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27">
@@ -10428,8 +10418,8 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="61.77734375"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.109375"/>
+    <col min="1" max="1" width="61.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="62" customFormat="1">
@@ -10825,27 +10815,27 @@
   <dimension ref="A1:AH13"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="33.0"/>
-    <col min="2" max="2" customWidth="true" width="10.44140625"/>
-    <col min="6" max="6" customWidth="true" width="10.88671875"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.33203125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.109375"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.33203125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.33203125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="13.88671875"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="12.109375"/>
-    <col min="19" max="19" customWidth="true" width="8.77734375"/>
-    <col min="20" max="20" customWidth="true" width="9.44140625"/>
-    <col min="21" max="21" customWidth="true" width="11.109375"/>
-    <col min="22" max="22" customWidth="true" width="9.33203125"/>
-    <col min="23" max="23" customWidth="true" width="9.44140625"/>
-    <col min="24" max="24" customWidth="true" width="10.77734375"/>
-    <col min="25" max="25" customWidth="true" width="11.33203125"/>
-    <col min="26" max="26" customWidth="true" width="12.0"/>
-    <col min="27" max="27" customWidth="true" width="10.21875"/>
-    <col min="30" max="30" customWidth="true" width="9.0"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="1" max="1" width="33" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" customWidth="1"/>
+    <col min="6" max="6" width="10.88671875" customWidth="1"/>
+    <col min="12" max="12" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.77734375" customWidth="1"/>
+    <col min="20" max="20" width="9.44140625" customWidth="1"/>
+    <col min="21" max="21" width="11.109375" customWidth="1"/>
+    <col min="22" max="22" width="9.33203125" customWidth="1"/>
+    <col min="23" max="23" width="9.44140625" customWidth="1"/>
+    <col min="24" max="24" width="10.77734375" customWidth="1"/>
+    <col min="25" max="25" width="11.33203125" customWidth="1"/>
+    <col min="26" max="26" width="12" customWidth="1"/>
+    <col min="27" max="27" width="10.21875" customWidth="1"/>
+    <col min="30" max="30" width="9" customWidth="1"/>
+    <col min="34" max="34" width="17.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -11069,7 +11059,7 @@
       <c r="T3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="U3" s="0">
+      <c r="U3">
         <v>2</v>
       </c>
       <c r="V3" s="3"/>
@@ -11082,7 +11072,7 @@
       <c r="Y3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="Z3" s="0">
+      <c r="Z3">
         <v>3</v>
       </c>
       <c r="AA3" s="105" t="s">
@@ -11219,7 +11209,7 @@
       <c r="T5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="U5" s="0">
+      <c r="U5">
         <v>2</v>
       </c>
       <c r="V5" s="3">
@@ -11234,7 +11224,7 @@
       <c r="Y5" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="Z5" s="0">
+      <c r="Z5">
         <v>3</v>
       </c>
       <c r="AA5" s="105" t="s">
@@ -11428,7 +11418,7 @@
       <c r="I9" s="37"/>
       <c r="J9" s="37"/>
       <c r="K9" s="37" t="s">
-        <v>1326</v>
+        <v>1337</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>390</v>
@@ -11437,7 +11427,7 @@
         <v>294</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>1327</v>
+        <v>1314</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>191</v>
@@ -11628,31 +11618,31 @@
   <dimension ref="A1:AG14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="49.77734375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="4.77734375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.44140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.77734375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="4.44140625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="5.44140625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="9.77734375"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="4.44140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="5.44140625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="9.77734375"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="4.44140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="5.44140625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.77734375"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="4.44140625"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="5.44140625"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="9.77734375"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="4.44140625"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="5.44140625"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="9.77734375"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="4.44140625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="5.44140625"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="9.77734375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="4.44140625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="5.44140625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="1" max="1" width="49.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="9.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -12429,11 +12419,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="35.21875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.44140625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.5546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.44140625"/>
+    <col min="1" max="1" width="35.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -12517,10 +12507,10 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="33.5546875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.44140625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.88671875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="14.21875"/>
+    <col min="1" max="1" width="33.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -12614,10 +12604,10 @@
   <dimension ref="A1:AH5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="46.6640625"/>
-    <col min="5" max="5" customWidth="true" width="6.21875"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="13.88671875"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="13.33203125"/>
+    <col min="1" max="1" width="46.6640625" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" customWidth="1"/>
+    <col min="29" max="29" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -12916,16 +12906,16 @@
       <c r="U4" s="37"/>
       <c r="V4" s="37"/>
       <c r="W4" s="37" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="X4" s="37" t="s">
-        <v>1363</v>
+        <v>1321</v>
       </c>
       <c r="Y4" s="37" t="s">
         <v>295</v>
       </c>
       <c r="Z4" s="37" t="s">
-        <v>1364</v>
+        <v>1322</v>
       </c>
       <c r="AA4" s="37" t="s">
         <v>191</v>
@@ -12934,7 +12924,7 @@
         <v>12</v>
       </c>
       <c r="AC4" s="37" t="s">
-        <v>1365</v>
+        <v>1362</v>
       </c>
       <c r="AD4" s="37"/>
       <c r="AE4" s="37"/>
@@ -12994,16 +12984,16 @@
   <dimension ref="A1:K18"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="68.77734375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="10.77734375"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="19.44140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="15.5546875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="8" max="9" bestFit="true" customWidth="true" width="19.44140625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="10.88671875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="12.5546875"/>
+    <col min="1" max="1" width="68.77734375" customWidth="1"/>
+    <col min="2" max="2" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -13375,24 +13365,24 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.5546875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.44140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.21875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.77734375"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.44140625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.5546875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="7.44140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.44140625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="18.44140625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="15.44140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="17" max="17" customWidth="true" width="17.6640625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="1" max="1" width="20.5546875" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.6640625" customWidth="1"/>
+    <col min="18" max="18" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -13517,16 +13507,16 @@
       <c r="I3" s="37"/>
       <c r="J3" s="37"/>
       <c r="K3" s="37" t="s">
-        <v>1338</v>
+        <v>1345</v>
       </c>
       <c r="L3" s="37" t="s">
-        <v>1339</v>
+        <v>1315</v>
       </c>
       <c r="M3" s="37" t="s">
         <v>666</v>
       </c>
       <c r="N3" s="37" t="s">
-        <v>1340</v>
+        <v>1316</v>
       </c>
       <c r="O3" s="37" t="s">
         <v>12</v>
@@ -13535,10 +13525,10 @@
         <v>43</v>
       </c>
       <c r="Q3" s="37" t="s">
-        <v>1341</v>
+        <v>1346</v>
       </c>
       <c r="R3" s="37" t="s">
-        <v>1342</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -13657,16 +13647,16 @@
       <c r="I6" s="37"/>
       <c r="J6" s="37"/>
       <c r="K6" s="37" t="s">
-        <v>1343</v>
+        <v>1348</v>
       </c>
       <c r="L6" s="37" t="s">
-        <v>1344</v>
+        <v>1317</v>
       </c>
       <c r="M6" s="37" t="s">
         <v>172</v>
       </c>
       <c r="N6" s="37" t="s">
-        <v>1345</v>
+        <v>1318</v>
       </c>
       <c r="O6" s="37" t="s">
         <v>12</v>
@@ -13675,7 +13665,7 @@
         <v>13</v>
       </c>
       <c r="Q6" s="37" t="s">
-        <v>1346</v>
+        <v>1349</v>
       </c>
       <c r="R6" s="37"/>
     </row>
@@ -13693,37 +13683,37 @@
   <dimension ref="A1:AI16"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="93.88671875"/>
-    <col min="2" max="2" customWidth="true" width="13.21875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.21875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="6.21875"/>
-    <col min="6" max="6" customWidth="true" width="11.6640625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.21875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="6.21875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="8.5546875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="18.6640625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="18.6640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.6640625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="18.6640625"/>
-    <col min="19" max="19" customWidth="true" width="23.5546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="14.109375"/>
-    <col min="22" max="22" customWidth="true" width="13.44140625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="14.21875"/>
-    <col min="24" max="25" bestFit="true" customWidth="true" width="13.5546875"/>
-    <col min="26" max="26" customWidth="true" width="7.0"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="15.21875"/>
-    <col min="28" max="28" customWidth="true" width="16.33203125"/>
-    <col min="29" max="32" bestFit="true" customWidth="true" width="13.5546875"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="17.44140625"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="13.5546875"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="1" max="1" width="93.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.21875" customWidth="1"/>
+    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" customWidth="1"/>
+    <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.5546875" customWidth="1"/>
+    <col min="20" max="20" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.44140625" customWidth="1"/>
+    <col min="23" max="23" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="7" customWidth="1"/>
+    <col min="27" max="27" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="16.33203125" customWidth="1"/>
+    <col min="29" max="32" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:35">
@@ -14437,43 +14427,43 @@
         <v>150</v>
       </c>
       <c r="J11" s="104" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="K11" s="104"/>
       <c r="L11" s="104"/>
       <c r="M11" s="104" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="N11" s="104"/>
       <c r="O11" s="104"/>
       <c r="P11" s="104"/>
       <c r="Q11" s="104"/>
       <c r="R11" s="104" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="S11" s="104"/>
       <c r="T11" s="104"/>
       <c r="U11" s="104" t="s">
+        <v>1292</v>
+      </c>
+      <c r="V11" s="104" t="s">
         <v>1293</v>
-      </c>
-      <c r="V11" s="104" t="s">
-        <v>1294</v>
       </c>
       <c r="W11" s="104"/>
       <c r="X11" s="104" t="s">
+        <v>1295</v>
+      </c>
+      <c r="Y11" s="104" t="s">
         <v>1296</v>
       </c>
-      <c r="Y11" s="104" t="s">
-        <v>1297</v>
-      </c>
       <c r="Z11" s="104" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="AA11" s="104" t="s">
+        <v>1287</v>
+      </c>
+      <c r="AB11" s="104" t="s">
         <v>1288</v>
-      </c>
-      <c r="AB11" s="104" t="s">
-        <v>1289</v>
       </c>
       <c r="AC11" s="104"/>
       <c r="AD11" s="104"/>
@@ -14512,19 +14502,19 @@
         <v>150</v>
       </c>
       <c r="J12" s="104" t="s">
-        <v>1353</v>
+        <v>1356</v>
       </c>
       <c r="K12" s="104"/>
       <c r="L12" s="104"/>
       <c r="M12" s="104" t="s">
-        <v>1354</v>
+        <v>1319</v>
       </c>
       <c r="N12" s="104"/>
       <c r="O12" s="104"/>
       <c r="P12" s="104"/>
       <c r="Q12" s="104"/>
       <c r="R12" s="104" t="s">
-        <v>1355</v>
+        <v>1320</v>
       </c>
       <c r="S12" s="104"/>
       <c r="T12" s="104"/>
@@ -14677,8 +14667,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.21875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="1" max="1" width="32.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -14726,8 +14716,8 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="48.88671875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="11.44140625"/>
+    <col min="1" max="1" width="48.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -14891,24 +14881,24 @@
   <dimension ref="A1:Q81"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="25" width="28.77734375"/>
-    <col min="2" max="2" customWidth="true" style="25" width="16.21875"/>
-    <col min="3" max="3" customWidth="true" style="25" width="11.77734375"/>
-    <col min="4" max="4" customWidth="true" style="25" width="9.5546875"/>
-    <col min="5" max="5" customWidth="true" style="25" width="10.33203125"/>
-    <col min="6" max="6" customWidth="true" style="25" width="9.33203125"/>
-    <col min="7" max="7" customWidth="true" style="25" width="9.77734375"/>
-    <col min="8" max="8" customWidth="true" style="25" width="10.44140625"/>
-    <col min="9" max="9" customWidth="true" style="25" width="8.77734375"/>
-    <col min="10" max="10" customWidth="true" style="34" width="8.109375"/>
-    <col min="11" max="11" customWidth="true" style="25" width="10.0"/>
-    <col min="12" max="12" customWidth="true" style="25" width="7.77734375"/>
-    <col min="13" max="13" customWidth="true" style="25" width="9.0"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="19.44140625"/>
-    <col min="15" max="15" style="25" width="8.77734375"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="14.77734375"/>
-    <col min="17" max="17" customWidth="true" style="25" width="15.109375"/>
-    <col min="18" max="16384" style="25" width="8.77734375"/>
+    <col min="1" max="1" width="28.77734375" style="25" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" style="25" customWidth="1"/>
+    <col min="3" max="3" width="11.77734375" style="25" customWidth="1"/>
+    <col min="4" max="4" width="9.5546875" style="25" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" style="25" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" style="25" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" style="25" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" style="25" customWidth="1"/>
+    <col min="9" max="9" width="8.77734375" style="25" customWidth="1"/>
+    <col min="10" max="10" width="8.109375" style="34" customWidth="1"/>
+    <col min="11" max="11" width="10" style="25" customWidth="1"/>
+    <col min="12" max="12" width="7.77734375" style="25" customWidth="1"/>
+    <col min="13" max="13" width="9" style="25" customWidth="1"/>
+    <col min="14" max="14" width="19.44140625" style="25" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.77734375" style="25"/>
+    <col min="16" max="16" width="14.77734375" style="25" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.109375" style="25" customWidth="1"/>
+    <col min="18" max="16384" width="8.77734375" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -18656,18 +18646,18 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="32.21875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.44140625"/>
-    <col min="4" max="4" customWidth="true" width="15.44140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.5546875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.44140625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.5546875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="17.33203125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="13" max="13" customWidth="true" width="15.109375"/>
+    <col min="1" max="1" width="32.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" customWidth="1"/>
+    <col min="5" max="5" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -18867,17 +18857,17 @@
   <dimension ref="A1:Q21"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.44140625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="21.77734375"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.44140625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="6.44140625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="18.44140625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="10.44140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="9.44140625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="18.33203125"/>
+    <col min="1" max="1" width="39.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -18956,7 +18946,7 @@
         <v>46</v>
       </c>
       <c r="H2" s="37" t="s">
-        <v>1334</v>
+        <v>1341</v>
       </c>
       <c r="I2" s="37" t="s">
         <v>337</v>
@@ -19250,7 +19240,7 @@
       </c>
       <c r="G10" s="37"/>
       <c r="H10" s="37" t="s">
-        <v>1337</v>
+        <v>1344</v>
       </c>
       <c r="I10" s="37" t="s">
         <v>730</v>
@@ -19324,7 +19314,7 @@
       </c>
       <c r="G12" s="37"/>
       <c r="H12" s="37" t="s">
-        <v>1336</v>
+        <v>1343</v>
       </c>
       <c r="I12" s="37" t="s">
         <v>680</v>
@@ -19570,7 +19560,7 @@
         <v>46</v>
       </c>
       <c r="H18" s="37" t="s">
-        <v>1335</v>
+        <v>1342</v>
       </c>
       <c r="I18" s="37" t="s">
         <v>732</v>
@@ -19707,30 +19697,30 @@
   <dimension ref="A1:W22"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="25" width="19.88671875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="34" width="10.88671875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="34" width="9.44140625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="34" width="7.77734375"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="34" width="10.88671875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="34" width="9.44140625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="34" width="7.77734375"/>
-    <col min="8" max="8" customWidth="true" style="25" width="13.0"/>
-    <col min="9" max="9" customWidth="true" style="25" width="16.5546875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="25" width="14.109375"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="34" width="10.33203125"/>
-    <col min="12" max="12" customWidth="true" style="34" width="10.33203125"/>
-    <col min="13" max="13" style="25" width="8.77734375"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="12.5546875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="25" width="14.77734375"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="13.21875"/>
-    <col min="17" max="17" customWidth="true" style="34" width="11.5546875"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" style="34" width="8.77734375"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="25" width="9.88671875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="25" width="12.0"/>
-    <col min="21" max="21" style="25" width="8.77734375"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" style="25" width="10.6640625"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" style="25" width="13.88671875"/>
-    <col min="24" max="16384" style="25" width="8.77734375"/>
+    <col min="1" max="1" width="19.88671875" style="25" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.44140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.77734375" style="34" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.44140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.77734375" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" style="25" customWidth="1"/>
+    <col min="9" max="9" width="16.5546875" style="25" customWidth="1"/>
+    <col min="10" max="10" width="14.109375" style="25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.33203125" style="34" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.33203125" style="34" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="25"/>
+    <col min="14" max="14" width="12.5546875" style="25" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.77734375" style="25" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.21875" style="25" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5546875" style="34" customWidth="1"/>
+    <col min="18" max="18" width="8.77734375" style="34" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.88671875" style="25" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12" style="25" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="25"/>
+    <col min="22" max="22" width="10.6640625" style="25" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.88671875" style="25" bestFit="1" customWidth="1"/>
+    <col min="24" max="16384" width="8.77734375" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -19842,7 +19832,7 @@
         <v>14</v>
       </c>
       <c r="M2" s="28" t="s">
-        <v>1373</v>
+        <v>1367</v>
       </c>
       <c r="N2" s="28">
         <v>3</v>
@@ -19862,10 +19852,10 @@
       <c r="S2" s="28"/>
       <c r="T2" s="28"/>
       <c r="U2" s="37" t="s">
-        <v>1374</v>
+        <v>1325</v>
       </c>
       <c r="V2" s="37" t="s">
-        <v>1375</v>
+        <v>1326</v>
       </c>
       <c r="W2" s="37" t="s">
         <v>337</v>
@@ -19970,7 +19960,7 @@
         <v>14</v>
       </c>
       <c r="M4" s="28" t="s">
-        <v>1370</v>
+        <v>1366</v>
       </c>
       <c r="N4" s="28"/>
       <c r="O4" s="28"/>
@@ -19984,10 +19974,10 @@
       <c r="S4" s="28"/>
       <c r="T4" s="28"/>
       <c r="U4" s="37" t="s">
-        <v>1371</v>
+        <v>1323</v>
       </c>
       <c r="V4" s="37" t="s">
-        <v>1372</v>
+        <v>1324</v>
       </c>
       <c r="W4" s="37" t="s">
         <v>337</v>
@@ -20025,19 +20015,19 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="19.88671875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.33203125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="17.33203125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="4.44140625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="17.33203125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="11.88671875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="14.21875"/>
+    <col min="1" max="1" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -20140,20 +20130,20 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="34" width="25.77734375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="34" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="34" width="15.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="34" width="4.44140625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="34" width="14.21875"/>
-    <col min="14" max="16384" style="34" width="8.88671875"/>
+    <col min="1" max="1" width="25.77734375" style="34" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="34" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.44140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.21875" style="34" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.88671875" style="34"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -20279,21 +20269,21 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="34" width="20.21875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="34" width="15.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
-    <col min="6" max="7" customWidth="true" style="34" width="17.33203125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="34" width="15.0"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="34" width="4.44140625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="34" width="14.21875"/>
-    <col min="16" max="16384" style="34" width="8.88671875"/>
+    <col min="1" max="1" width="20.21875" style="34" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="34" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="17.33203125" style="34" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="34" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.44140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.21875" style="34" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="34"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -20481,22 +20471,22 @@
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="34" width="28.33203125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="3" max="3" customWidth="true" style="34" width="10.33203125"/>
-    <col min="4" max="4" customWidth="true" style="34" width="11.21875"/>
-    <col min="5" max="5" customWidth="true" style="34" width="12.77734375"/>
-    <col min="6" max="6" customWidth="true" style="34" width="12.44140625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="34" width="11.109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="9" max="9" customWidth="true" style="34" width="9.109375"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
-    <col min="11" max="11" customWidth="true" style="34" width="11.5546875"/>
-    <col min="12" max="12" customWidth="true" style="34" width="10.77734375"/>
-    <col min="13" max="13" customWidth="true" style="34" width="12.21875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="34" width="12.6640625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" style="34" width="14.21875"/>
-    <col min="16" max="16384" style="34" width="8.88671875"/>
+    <col min="1" max="1" width="28.33203125" style="34" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" style="34" customWidth="1"/>
+    <col min="4" max="4" width="11.21875" style="34" customWidth="1"/>
+    <col min="5" max="5" width="12.77734375" style="34" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" style="34" customWidth="1"/>
+    <col min="7" max="7" width="11.109375" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" style="34" customWidth="1"/>
+    <col min="10" max="10" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5546875" style="34" customWidth="1"/>
+    <col min="12" max="12" width="10.77734375" style="34" customWidth="1"/>
+    <col min="13" max="13" width="12.21875" style="34" customWidth="1"/>
+    <col min="14" max="14" width="12.6640625" style="34" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.21875" style="34" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="34"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -20615,7 +20605,7 @@
       </c>
       <c r="G4" s="37"/>
       <c r="H4" s="37" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="I4" s="37" t="s">
         <v>340</v>
@@ -20771,7 +20761,7 @@
         <v>734</v>
       </c>
       <c r="H9" s="37" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="I9" s="37" t="s">
         <v>340</v>
@@ -20827,11 +20817,11 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="34" width="24.0"/>
-    <col min="2" max="2" customWidth="true" style="34" width="11.44140625"/>
-    <col min="3" max="3" style="34" width="8.88671875"/>
-    <col min="4" max="4" customWidth="true" style="34" width="19.6640625"/>
-    <col min="5" max="16384" style="34" width="8.88671875"/>
+    <col min="1" max="1" width="24" style="34" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" style="34" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="34"/>
+    <col min="4" max="4" width="19.6640625" style="34" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="34"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -20889,12 +20879,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="34" width="32.21875"/>
-    <col min="2" max="2" customWidth="true" style="34" width="14.0"/>
-    <col min="3" max="3" customWidth="true" style="34" width="16.6640625"/>
-    <col min="4" max="4" customWidth="true" style="34" width="17.6640625"/>
-    <col min="5" max="5" customWidth="true" style="34" width="11.77734375"/>
-    <col min="6" max="16384" style="34" width="8.88671875"/>
+    <col min="1" max="1" width="32.21875" style="34" customWidth="1"/>
+    <col min="2" max="2" width="14" style="34" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" style="34" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" style="34" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" style="34" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="34"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -20978,11 +20968,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="34" width="38.21875"/>
-    <col min="2" max="2" customWidth="true" style="34" width="13.5546875"/>
-    <col min="3" max="3" customWidth="true" style="34" width="15.5546875"/>
-    <col min="4" max="4" customWidth="true" style="34" width="19.0"/>
-    <col min="5" max="16384" style="34" width="8.88671875"/>
+    <col min="1" max="1" width="38.21875" style="34" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="34" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" style="34" customWidth="1"/>
+    <col min="4" max="4" width="19" style="34" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="34"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -21105,23 +21095,23 @@
   <dimension ref="A1:S5"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="34" width="30.88671875"/>
-    <col min="2" max="2" customWidth="true" style="34" width="17.77734375"/>
-    <col min="3" max="3" customWidth="true" style="34" width="16.44140625"/>
-    <col min="4" max="4" customWidth="true" style="34" width="16.109375"/>
-    <col min="5" max="5" customWidth="true" style="34" width="12.0"/>
-    <col min="6" max="6" customWidth="true" style="34" width="18.109375"/>
-    <col min="7" max="7" customWidth="true" style="34" width="15.109375"/>
-    <col min="8" max="8" customWidth="true" style="34" width="10.44140625"/>
-    <col min="9" max="9" customWidth="true" style="34" width="10.77734375"/>
-    <col min="10" max="10" style="34" width="8.88671875"/>
-    <col min="11" max="11" customWidth="true" style="34" width="13.21875"/>
-    <col min="12" max="12" customWidth="true" style="34" width="12.6640625"/>
-    <col min="13" max="13" customWidth="true" style="34" width="14.109375"/>
-    <col min="14" max="14" customWidth="true" style="34" width="14.33203125"/>
-    <col min="15" max="18" style="34" width="8.88671875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="34" width="18.33203125"/>
-    <col min="20" max="16384" style="34" width="8.88671875"/>
+    <col min="1" max="1" width="30.88671875" style="34" customWidth="1"/>
+    <col min="2" max="2" width="17.77734375" style="34" customWidth="1"/>
+    <col min="3" max="3" width="16.44140625" style="34" customWidth="1"/>
+    <col min="4" max="4" width="16.109375" style="34" customWidth="1"/>
+    <col min="5" max="5" width="12" style="34" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" style="34" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" style="34" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" style="34" customWidth="1"/>
+    <col min="9" max="9" width="10.77734375" style="34" customWidth="1"/>
+    <col min="10" max="10" width="8.88671875" style="34"/>
+    <col min="11" max="11" width="13.21875" style="34" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" style="34" customWidth="1"/>
+    <col min="13" max="13" width="14.109375" style="34" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" style="34" customWidth="1"/>
+    <col min="15" max="18" width="8.88671875" style="34"/>
+    <col min="19" max="19" width="18.33203125" style="34" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="8.88671875" style="34"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -21206,13 +21196,13 @@
         <v>30</v>
       </c>
       <c r="H2" s="37" t="s">
-        <v>1319</v>
+        <v>1369</v>
       </c>
       <c r="I2" s="37" t="s">
-        <v>1320</v>
+        <v>1370</v>
       </c>
       <c r="J2" s="37" t="s">
-        <v>1318</v>
+        <v>1368</v>
       </c>
       <c r="K2" s="37">
         <f>B2</f>
@@ -21258,13 +21248,13 @@
         <v>962</v>
       </c>
       <c r="H3" s="37" t="s">
-        <v>1304</v>
+        <v>1300</v>
       </c>
       <c r="I3" s="37" t="s">
-        <v>1305</v>
+        <v>1301</v>
       </c>
       <c r="J3" s="37" t="s">
-        <v>1303</v>
+        <v>1299</v>
       </c>
       <c r="K3" s="37"/>
       <c r="L3" s="37" t="s">
@@ -21274,7 +21264,7 @@
         <v>665</v>
       </c>
       <c r="N3" s="37" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="O3" s="37" t="s">
         <v>962</v>
@@ -21289,7 +21279,7 @@
         <v>2</v>
       </c>
       <c r="S3" s="37" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -21315,13 +21305,13 @@
         <v>672</v>
       </c>
       <c r="H4" s="37" t="s">
-        <v>1301</v>
+        <v>1372</v>
       </c>
       <c r="I4" s="37" t="s">
-        <v>1302</v>
+        <v>1373</v>
       </c>
       <c r="J4" s="37" t="s">
-        <v>1300</v>
+        <v>1371</v>
       </c>
       <c r="K4" s="37"/>
       <c r="L4" s="37" t="s">
@@ -21331,7 +21321,7 @@
         <v>1286</v>
       </c>
       <c r="N4" s="37" t="s">
-        <v>1287</v>
+        <v>1310</v>
       </c>
       <c r="O4" s="37"/>
       <c r="P4" s="37"/>
@@ -21364,13 +21354,13 @@
         <v>672</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>1322</v>
+        <v>1375</v>
       </c>
       <c r="I5" s="37" t="s">
-        <v>1323</v>
+        <v>1376</v>
       </c>
       <c r="J5" s="37" t="s">
-        <v>1321</v>
+        <v>1374</v>
       </c>
       <c r="K5" s="37"/>
       <c r="L5" s="37" t="s">
@@ -21380,7 +21370,7 @@
         <v>1286</v>
       </c>
       <c r="N5" s="37" t="s">
-        <v>1314</v>
+        <v>1310</v>
       </c>
       <c r="O5" s="37" t="s">
         <v>306</v>
@@ -21395,7 +21385,7 @@
         <v>2</v>
       </c>
       <c r="S5" s="37" t="s">
-        <v>1315</v>
+        <v>1311</v>
       </c>
     </row>
   </sheetData>
@@ -21411,12 +21401,12 @@
   <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="39.44140625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.5546875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.77734375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.44140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.77734375"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="16.109375"/>
+    <col min="1" max="1" width="39.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -22106,13 +22096,13 @@
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="57.44140625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="15.5546875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.77734375"/>
-    <col min="4" max="5" bestFit="true" customWidth="true" width="11.21875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="20.109375"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="25.88671875"/>
-    <col min="8" max="8" customWidth="true" width="8.77734375"/>
+    <col min="1" max="1" width="57.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -22344,7 +22334,7 @@
       <c r="F15" s="34"/>
     </row>
     <row r="17" spans="8:8">
-      <c r="H17" t="s" s="0">
+      <c r="H17" t="s">
         <v>997</v>
       </c>
     </row>
@@ -22362,28 +22352,28 @@
   <dimension ref="A1:W15"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="23" width="50.0"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="23" width="18.33203125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="23" width="12.109375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="23" width="15.33203125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="23" width="12.21875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="23" width="9.44140625"/>
-    <col min="7" max="8" style="23" width="8.77734375"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="23" width="10.44140625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="23" width="12.6640625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="23" width="10.44140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="23" width="11.21875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" style="23" width="10.44140625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" style="23" width="8.21875"/>
-    <col min="15" max="15" customWidth="true" style="23" width="13.0"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" style="23" width="10.21875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="23" width="10.44140625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" style="23" width="9.21875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" style="23" width="11.6640625"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="23" width="12.6640625"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" style="23" width="11.21875"/>
-    <col min="22" max="23" bestFit="true" customWidth="true" style="23" width="12.6640625"/>
-    <col min="24" max="16384" style="23" width="8.77734375"/>
+    <col min="1" max="1" width="50" style="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" style="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" style="23" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" style="23" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" style="23" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.44140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="8.77734375" style="23"/>
+    <col min="9" max="9" width="10.44140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" style="23" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.21875" style="23" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.44140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" style="23" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13" style="23" customWidth="1"/>
+    <col min="16" max="16" width="10.21875" style="23" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.44140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.21875" style="23" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.6640625" style="23" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.6640625" style="23" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.21875" style="23" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="12.6640625" style="23" bestFit="1" customWidth="1"/>
+    <col min="24" max="16384" width="8.77734375" style="23"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -22609,7 +22599,7 @@
       </c>
       <c r="G5" s="49"/>
       <c r="H5" s="28" t="s">
-        <v>1368</v>
+        <v>1365</v>
       </c>
       <c r="I5" s="28"/>
       <c r="J5" s="28"/>
@@ -22705,7 +22695,7 @@
         <v>19</v>
       </c>
       <c r="H7" s="28" t="s">
-        <v>1366</v>
+        <v>1363</v>
       </c>
       <c r="I7" s="28" t="s">
         <v>320</v>
@@ -22950,7 +22940,7 @@
       </c>
       <c r="G12" s="49"/>
       <c r="H12" s="28" t="s">
-        <v>1367</v>
+        <v>1364</v>
       </c>
       <c r="I12" s="28" t="s">
         <v>330</v>
@@ -23091,7 +23081,7 @@
         <v>15</v>
       </c>
       <c r="H15" s="28" t="s">
-        <v>1369</v>
+        <v>1332</v>
       </c>
       <c r="I15" s="28" t="s">
         <v>193</v>
@@ -23127,14 +23117,14 @@
   <dimension ref="A1:AM45"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="77.109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="11.6640625"/>
-    <col min="18" max="18" customWidth="true" width="8.88671875"/>
-    <col min="19" max="19" customWidth="true" width="13.88671875"/>
-    <col min="20" max="20" customWidth="true" width="13.77734375"/>
-    <col min="21" max="26" customWidth="true" width="8.88671875"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="12.109375"/>
-    <col min="37" max="37" customWidth="true" width="11.0"/>
+    <col min="1" max="1" width="77.109375" customWidth="1"/>
+    <col min="17" max="17" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.88671875" customWidth="1"/>
+    <col min="19" max="19" width="13.88671875" customWidth="1"/>
+    <col min="20" max="20" width="13.77734375" customWidth="1"/>
+    <col min="21" max="26" width="8.88671875" customWidth="1"/>
+    <col min="36" max="36" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39">
@@ -23285,10 +23275,10 @@
       <c r="P2" s="37"/>
       <c r="Q2" s="37"/>
       <c r="R2" s="37" t="s">
-        <v>1306</v>
+        <v>1302</v>
       </c>
       <c r="S2" s="37" t="s">
-        <v>1307</v>
+        <v>1303</v>
       </c>
       <c r="T2" s="37">
         <v>1</v>
@@ -23665,10 +23655,10 @@
       <c r="P8" s="37"/>
       <c r="Q8" s="37"/>
       <c r="R8" s="37" t="s">
-        <v>1378</v>
+        <v>1333</v>
       </c>
       <c r="S8" s="37" t="s">
-        <v>1379</v>
+        <v>1334</v>
       </c>
       <c r="T8" s="37">
         <v>0</v>
@@ -24348,10 +24338,10 @@
         <v>41</v>
       </c>
       <c r="R19" s="37" t="s">
+        <v>1289</v>
+      </c>
+      <c r="S19" s="37" t="s">
         <v>1290</v>
-      </c>
-      <c r="S19" s="37" t="s">
-        <v>1291</v>
       </c>
       <c r="T19" s="40">
         <v>0</v>
@@ -25935,17 +25925,17 @@
   <dimension ref="A1:V19"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="53.77734375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
-    <col min="3" max="4" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="5" max="7" customWidth="true" width="12.21875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="15.44140625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.5546875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="15.44140625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="12.21875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="1" max="1" width="53.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="12.21875" customWidth="1"/>
+    <col min="8" max="8" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -26711,16 +26701,16 @@
   <dimension ref="A1:X38"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="64.5546875"/>
-    <col min="10" max="10" style="23" width="8.77734375"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="13.88671875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="11.44140625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="9.77734375"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="13.88671875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="12.6640625"/>
-    <col min="22" max="23" bestFit="true" customWidth="true" width="19.21875"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="15.5546875"/>
+    <col min="1" max="1" width="64.5546875" customWidth="1"/>
+    <col min="10" max="10" width="8.77734375" style="23"/>
+    <col min="12" max="12" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24">
@@ -26827,7 +26817,7 @@
       </c>
       <c r="J2" s="37"/>
       <c r="K2" s="37" t="s">
-        <v>1347</v>
+        <v>1350</v>
       </c>
       <c r="L2" s="37"/>
       <c r="M2" s="37"/>
@@ -26867,10 +26857,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="37" t="s">
-        <v>1351</v>
+        <v>1354</v>
       </c>
       <c r="L3" s="37" t="s">
-        <v>1352</v>
+        <v>1355</v>
       </c>
       <c r="M3" s="37"/>
       <c r="N3" s="37"/>
@@ -27835,10 +27825,10 @@
       <c r="I25" s="37"/>
       <c r="J25" s="37"/>
       <c r="K25" s="37" t="s">
-        <v>1349</v>
+        <v>1352</v>
       </c>
       <c r="L25" s="37" t="s">
-        <v>1350</v>
+        <v>1353</v>
       </c>
       <c r="M25" s="37"/>
       <c r="N25" s="37" t="s">
@@ -28227,7 +28217,7 @@
       </c>
       <c r="J35" s="37"/>
       <c r="K35" s="37" t="s">
-        <v>1348</v>
+        <v>1351</v>
       </c>
       <c r="L35" s="37"/>
       <c r="M35" s="37"/>

</xml_diff>

<commit_message>
SHD sanity suite getting flight numbers for multiple segments added - 18-11-2025
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Harshitha Rajesh\Copa_SHD_API_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B90428-8A08-4503-BC4C-60B5220BB06D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C6D7BFE-5D82-40FF-AC01-33156CBFF7A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="32" activeTab="37" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="6" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4652" uniqueCount="1377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4656" uniqueCount="1381">
   <si>
     <t>Scenario</t>
   </si>
@@ -3855,12 +3855,6 @@
     <t>GYE</t>
   </si>
   <si>
-    <t>RMV3KO</t>
-  </si>
-  <si>
-    <t>2302281562542</t>
-  </si>
-  <si>
     <t>807</t>
   </si>
   <si>
@@ -4074,120 +4068,12 @@
     <t>BLV1VZ</t>
   </si>
   <si>
-    <t>RVPRUM</t>
-  </si>
-  <si>
-    <t>2302282731720</t>
-  </si>
-  <si>
-    <t>RVPV2A</t>
-  </si>
-  <si>
-    <t>kmwnmzukom2xnovsjsozjs2orv</t>
-  </si>
-  <si>
-    <t>RVPZRO</t>
-  </si>
-  <si>
-    <t>RVP0JR</t>
-  </si>
-  <si>
-    <t>2302282731724</t>
-  </si>
-  <si>
-    <t>2302282731725</t>
-  </si>
-  <si>
-    <t>RVP1SH</t>
-  </si>
-  <si>
-    <t>RVP2LU</t>
-  </si>
-  <si>
-    <t>RVP21N</t>
-  </si>
-  <si>
-    <t>RVP3KF</t>
-  </si>
-  <si>
-    <t>RVP4BC</t>
-  </si>
-  <si>
-    <t>2302282731730</t>
-  </si>
-  <si>
-    <t>2302282731731</t>
-  </si>
-  <si>
-    <t>RVP50O</t>
-  </si>
-  <si>
-    <t>2302282731733</t>
-  </si>
-  <si>
-    <t>RVQAWC</t>
-  </si>
-  <si>
-    <t>RVQBCE</t>
-  </si>
-  <si>
-    <t>RVQBNL</t>
-  </si>
-  <si>
-    <t>2302282731734</t>
-  </si>
-  <si>
-    <t>RVQBZT</t>
-  </si>
-  <si>
-    <t>2302282731735</t>
-  </si>
-  <si>
     <t>RVQCMT</t>
   </si>
   <si>
-    <t>RVQFGX</t>
-  </si>
-  <si>
-    <t>RVQGAI</t>
-  </si>
-  <si>
-    <t>RVQGO2</t>
-  </si>
-  <si>
-    <t>RVQG0V</t>
-  </si>
-  <si>
-    <t>RVQHUO</t>
-  </si>
-  <si>
-    <t>2302282731742</t>
-  </si>
-  <si>
     <t>RVQISK</t>
   </si>
   <si>
-    <t>RVQKUM</t>
-  </si>
-  <si>
-    <t>RVQL3C</t>
-  </si>
-  <si>
-    <t>RVQMZC</t>
-  </si>
-  <si>
-    <t>RVQPWT</t>
-  </si>
-  <si>
-    <t>RVSXOT</t>
-  </si>
-  <si>
-    <t>ALDA</t>
-  </si>
-  <si>
-    <t>WAELCHI</t>
-  </si>
-  <si>
     <t>RVSZQ4</t>
   </si>
   <si>
@@ -4197,19 +4083,146 @@
     <t>GUTKOWSKI</t>
   </si>
   <si>
-    <t>RVS1JN</t>
-  </si>
-  <si>
-    <t>ERICH</t>
-  </si>
-  <si>
-    <t>STRACKE</t>
+    <t>RXZ0HZ</t>
+  </si>
+  <si>
+    <t>RYANN</t>
+  </si>
+  <si>
+    <t>JACOBS</t>
+  </si>
+  <si>
+    <t>RXZ1ZZ</t>
+  </si>
+  <si>
+    <t>CLARISA</t>
+  </si>
+  <si>
+    <t>GAYLORD</t>
+  </si>
+  <si>
+    <t>RX0A5S</t>
+  </si>
+  <si>
+    <t>2302282732213</t>
+  </si>
+  <si>
+    <t>RX0FOU</t>
+  </si>
+  <si>
+    <t>2302282732215</t>
+  </si>
+  <si>
+    <t>RX0V5T</t>
+  </si>
+  <si>
+    <t>ktwrxurvoyjirovyruojttwown</t>
+  </si>
+  <si>
+    <t>RX01FH</t>
+  </si>
+  <si>
+    <t>RX02DS</t>
+  </si>
+  <si>
+    <t>2302282732226</t>
+  </si>
+  <si>
+    <t>2302282732227</t>
+  </si>
+  <si>
+    <t>RX04I4</t>
+  </si>
+  <si>
+    <t>RX05ZF</t>
+  </si>
+  <si>
+    <t>RX1AYX</t>
+  </si>
+  <si>
+    <t>RX1DA0</t>
+  </si>
+  <si>
+    <t>RX1GQH</t>
+  </si>
+  <si>
+    <t>2302282732233</t>
+  </si>
+  <si>
+    <t>2302282732234</t>
+  </si>
+  <si>
+    <t>RX1QVA</t>
+  </si>
+  <si>
+    <t>2302282732239</t>
+  </si>
+  <si>
+    <t>RX1TRX</t>
+  </si>
+  <si>
+    <t>RX1VC2</t>
+  </si>
+  <si>
+    <t>RX1WVO</t>
+  </si>
+  <si>
+    <t>2302282732241</t>
+  </si>
+  <si>
+    <t>RX1YSX</t>
+  </si>
+  <si>
+    <t>2302282732242</t>
+  </si>
+  <si>
+    <t>RX15FV</t>
+  </si>
+  <si>
+    <t>RX2AXU</t>
+  </si>
+  <si>
+    <t>RX2CNT</t>
+  </si>
+  <si>
+    <t>RX2DRW</t>
+  </si>
+  <si>
+    <t>RX2FF2</t>
+  </si>
+  <si>
+    <t>2302282732247</t>
+  </si>
+  <si>
+    <t>RX2HUN</t>
+  </si>
+  <si>
+    <t>RX2MTC</t>
+  </si>
+  <si>
+    <t>RX2OVI</t>
+  </si>
+  <si>
+    <t>RX2UZ5</t>
+  </si>
+  <si>
+    <t>R3N45Z</t>
+  </si>
+  <si>
+    <t>2302282732964</t>
+  </si>
+  <si>
+    <t>R3OCHW</t>
+  </si>
+  <si>
+    <t>2302282732968</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="25">
     <font>
       <sz val="11"/>
@@ -5267,24 +5280,24 @@
   <dimension ref="A1:AC25"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="52.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="52.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="8.21875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.21875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="11.6640625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="12.6640625"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="12.6640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
@@ -5515,7 +5528,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="32" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
       <c r="I4" s="32" t="s">
         <v>313</v>
@@ -5570,7 +5583,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="32" t="s">
-        <v>1331</v>
+        <v>1329</v>
       </c>
       <c r="I5" s="104" t="s">
         <v>194</v>
@@ -6169,7 +6182,7 @@
       </c>
       <c r="G16" s="104"/>
       <c r="H16" s="104" t="s">
-        <v>1359</v>
+        <v>1369</v>
       </c>
       <c r="I16" s="104" t="s">
         <v>570</v>
@@ -6263,7 +6276,7 @@
       </c>
       <c r="G18" s="104"/>
       <c r="H18" s="104" t="s">
-        <v>1360</v>
+        <v>1370</v>
       </c>
       <c r="I18" s="104" t="s">
         <v>20</v>
@@ -6599,16 +6612,16 @@
   <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="32.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5546875" style="25" customWidth="1"/>
-    <col min="4" max="4" width="29.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.33203125" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="11" width="14.33203125" style="25" customWidth="1"/>
-    <col min="12" max="12" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.88671875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="3" customWidth="true" style="25" width="17.5546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="29.77734375"/>
+    <col min="5" max="5" customWidth="true" width="14.33203125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="14.33203125"/>
+    <col min="7" max="11" customWidth="true" style="25" width="14.33203125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="13.77734375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.5546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -6663,17 +6676,17 @@
         <v>2</v>
       </c>
       <c r="C2" s="37" t="s">
-        <v>1308</v>
+        <v>1306</v>
       </c>
       <c r="D2" s="40" t="s">
-        <v>1309</v>
+        <v>1307</v>
       </c>
       <c r="E2" s="40" t="s">
-        <v>1307</v>
+        <v>1305</v>
       </c>
       <c r="F2" s="37"/>
       <c r="G2" s="105" t="s">
-        <v>1273</v>
+        <v>1271</v>
       </c>
       <c r="H2" s="37" t="s">
         <v>12</v>
@@ -6776,19 +6789,19 @@
   <dimension ref="A1:AL15"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="52.109375" style="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" style="25" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" style="25" customWidth="1"/>
-    <col min="4" max="4" width="18.77734375" style="25" customWidth="1"/>
-    <col min="5" max="6" width="12.88671875" style="25" customWidth="1"/>
-    <col min="7" max="7" width="15" style="25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" style="25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.77734375" style="25"/>
-    <col min="10" max="10" width="17.88671875" style="25" customWidth="1"/>
-    <col min="11" max="11" width="14.21875" style="25" customWidth="1"/>
-    <col min="12" max="37" width="8.77734375" style="25"/>
-    <col min="38" max="38" width="15.44140625" style="25" bestFit="1" customWidth="1"/>
-    <col min="39" max="16384" width="8.77734375" style="25"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="52.109375"/>
+    <col min="2" max="2" customWidth="true" style="25" width="16.5546875"/>
+    <col min="3" max="3" customWidth="true" style="25" width="19.88671875"/>
+    <col min="4" max="4" customWidth="true" style="25" width="18.77734375"/>
+    <col min="5" max="6" customWidth="true" style="25" width="12.88671875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="25" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="25" width="11.88671875"/>
+    <col min="9" max="9" style="25" width="8.77734375"/>
+    <col min="10" max="10" customWidth="true" style="25" width="17.88671875"/>
+    <col min="11" max="11" customWidth="true" style="25" width="14.21875"/>
+    <col min="12" max="37" style="25" width="8.77734375"/>
+    <col min="38" max="38" bestFit="true" customWidth="true" style="25" width="15.44140625"/>
+    <col min="39" max="16384" style="25" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -7203,13 +7216,13 @@
         <v>43</v>
       </c>
       <c r="I7" s="37" t="s">
-        <v>1338</v>
+        <v>1349</v>
       </c>
       <c r="J7" s="37" t="s">
-        <v>1339</v>
+        <v>1350</v>
       </c>
       <c r="K7" s="37" t="s">
-        <v>1340</v>
+        <v>1351</v>
       </c>
       <c r="L7" s="37"/>
       <c r="M7" s="37"/>
@@ -7405,13 +7418,13 @@
         <v>43</v>
       </c>
       <c r="I10" s="37" t="s">
+        <v>1325</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>1326</v>
+      </c>
+      <c r="K10" s="37" t="s">
         <v>1327</v>
-      </c>
-      <c r="J10" s="37" t="s">
-        <v>1328</v>
-      </c>
-      <c r="K10" s="37" t="s">
-        <v>1329</v>
       </c>
       <c r="L10" s="37"/>
       <c r="M10" s="37"/>
@@ -7768,15 +7781,15 @@
   <dimension ref="A1:M26"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="43.21875" style="25" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" style="25" customWidth="1"/>
-    <col min="3" max="3" width="17.77734375" style="25" customWidth="1"/>
-    <col min="4" max="4" width="16.77734375" style="25" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" style="25" customWidth="1"/>
-    <col min="6" max="11" width="8.77734375" style="25"/>
-    <col min="12" max="12" width="44.88671875" style="25" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.88671875" style="25" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.77734375" style="25"/>
+    <col min="1" max="1" customWidth="true" style="25" width="43.21875"/>
+    <col min="2" max="2" customWidth="true" style="25" width="15.77734375"/>
+    <col min="3" max="3" customWidth="true" style="25" width="17.77734375"/>
+    <col min="4" max="4" customWidth="true" style="25" width="16.77734375"/>
+    <col min="5" max="5" customWidth="true" style="25" width="15.6640625"/>
+    <col min="6" max="11" style="25" width="8.77734375"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="25" width="44.88671875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="11.88671875"/>
+    <col min="14" max="16384" style="25" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -8391,7 +8404,7 @@
         <v>932</v>
       </c>
       <c r="M15" s="86" t="s">
-        <v>1263</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -8493,7 +8506,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="88" t="s">
-        <v>1262</v>
+        <v>1260</v>
       </c>
       <c r="G18" s="37" t="s">
         <v>467</v>
@@ -8511,7 +8524,7 @@
         <v>932</v>
       </c>
       <c r="L18" s="90" t="s">
-        <v>1274</v>
+        <v>1272</v>
       </c>
       <c r="M18" s="37" t="s">
         <v>932</v>
@@ -8844,22 +8857,22 @@
   <dimension ref="A1:V11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="51.77734375" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.88671875" customWidth="1"/>
-    <col min="14" max="14" width="12.6640625" customWidth="1"/>
-    <col min="15" max="15" width="11.44140625" customWidth="1"/>
-    <col min="16" max="16" width="7.77734375" customWidth="1"/>
-    <col min="17" max="18" width="10.6640625" customWidth="1"/>
-    <col min="19" max="19" width="11.77734375" customWidth="1"/>
-    <col min="20" max="20" width="8.77734375" customWidth="1"/>
-    <col min="21" max="21" width="10.77734375" customWidth="1"/>
-    <col min="22" max="22" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="51.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="11" max="12" bestFit="true" customWidth="true" width="15.33203125"/>
+    <col min="13" max="13" customWidth="true" width="13.88671875"/>
+    <col min="14" max="14" customWidth="true" width="12.6640625"/>
+    <col min="15" max="15" customWidth="true" width="11.44140625"/>
+    <col min="16" max="16" customWidth="true" width="7.77734375"/>
+    <col min="17" max="18" customWidth="true" width="10.6640625"/>
+    <col min="19" max="19" customWidth="true" width="11.77734375"/>
+    <col min="20" max="20" customWidth="true" width="8.77734375"/>
+    <col min="21" max="21" customWidth="true" width="10.77734375"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="12.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -9071,16 +9084,16 @@
       <c r="H4" s="37"/>
       <c r="I4" s="37"/>
       <c r="J4" s="37" t="s">
-        <v>1335</v>
+        <v>1346</v>
       </c>
       <c r="K4" s="37" t="s">
-        <v>1313</v>
+        <v>1311</v>
       </c>
       <c r="L4" s="37" t="s">
         <v>578</v>
       </c>
       <c r="M4" s="37" t="s">
-        <v>1312</v>
+        <v>1310</v>
       </c>
       <c r="N4" s="37" t="s">
         <v>578</v>
@@ -9167,16 +9180,16 @@
         <v>30</v>
       </c>
       <c r="J6" s="37" t="s">
+        <v>1302</v>
+      </c>
+      <c r="K6" s="37" t="s">
         <v>1304</v>
-      </c>
-      <c r="K6" s="37" t="s">
-        <v>1306</v>
       </c>
       <c r="L6" s="37" t="s">
         <v>578</v>
       </c>
       <c r="M6" s="37" t="s">
-        <v>1305</v>
+        <v>1303</v>
       </c>
       <c r="N6" s="37" t="s">
         <v>578</v>
@@ -9223,28 +9236,28 @@
       <c r="V8" s="136"/>
     </row>
     <row r="11" spans="1:22">
-      <c r="O11">
+      <c r="O11" s="0">
         <v>14</v>
       </c>
-      <c r="P11">
+      <c r="P11" s="0">
         <v>15</v>
       </c>
-      <c r="Q11">
+      <c r="Q11" s="0">
         <v>16</v>
       </c>
-      <c r="R11">
+      <c r="R11" s="0">
         <v>17</v>
       </c>
-      <c r="S11">
+      <c r="S11" s="0">
         <v>18</v>
       </c>
-      <c r="T11">
+      <c r="T11" s="0">
         <v>19</v>
       </c>
-      <c r="U11">
+      <c r="U11" s="0">
         <v>20</v>
       </c>
-      <c r="V11">
+      <c r="V11" s="0">
         <v>21</v>
       </c>
     </row>
@@ -9268,12 +9281,12 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="76.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="76.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="13.44140625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="16.6640625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="19.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -9398,17 +9411,17 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="68.109375" style="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" style="25" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" style="25" customWidth="1"/>
-    <col min="4" max="4" width="9.6640625" style="25" customWidth="1"/>
-    <col min="5" max="5" width="17.21875" style="25" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" style="25" customWidth="1"/>
-    <col min="7" max="10" width="8.77734375" style="25"/>
-    <col min="11" max="11" width="10.6640625" style="25" customWidth="1"/>
-    <col min="12" max="12" width="12.21875" style="25" customWidth="1"/>
-    <col min="13" max="13" width="15.33203125" style="25" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.77734375" style="25"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="25" width="68.109375"/>
+    <col min="2" max="2" customWidth="true" style="25" width="12.5546875"/>
+    <col min="3" max="3" customWidth="true" style="25" width="12.33203125"/>
+    <col min="4" max="4" customWidth="true" style="25" width="9.6640625"/>
+    <col min="5" max="5" customWidth="true" style="25" width="17.21875"/>
+    <col min="6" max="6" customWidth="true" style="25" width="12.5546875"/>
+    <col min="7" max="10" style="25" width="8.77734375"/>
+    <col min="11" max="11" customWidth="true" style="25" width="10.6640625"/>
+    <col min="12" max="12" customWidth="true" style="25" width="12.21875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="25" width="15.33203125"/>
+    <col min="14" max="16384" style="25" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -9653,10 +9666,10 @@
       <c r="I9" s="37"/>
       <c r="J9" s="37"/>
       <c r="K9" s="105" t="s">
-        <v>1266</v>
+        <v>1264</v>
       </c>
       <c r="L9" s="105" t="s">
-        <v>1267</v>
+        <v>1265</v>
       </c>
       <c r="M9" s="37"/>
     </row>
@@ -9834,12 +9847,12 @@
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.5546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="11.77734375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="29.5546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="11.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -9915,7 +9928,7 @@
         <v>910</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>1336</v>
+        <v>1347</v>
       </c>
       <c r="E5" s="37" t="s">
         <v>911</v>
@@ -9940,12 +9953,12 @@
   <dimension ref="A1:AA9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="33.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.5546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.44140625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="21.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27">
@@ -10215,7 +10228,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="105" t="s">
-        <v>1276</v>
+        <v>1274</v>
       </c>
       <c r="D6" s="37" t="s">
         <v>12</v>
@@ -10418,8 +10431,8 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="61.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="61.77734375"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="62" customFormat="1">
@@ -10815,27 +10828,27 @@
   <dimension ref="A1:AH13"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="10.44140625" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" customWidth="1"/>
-    <col min="12" max="12" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.77734375" customWidth="1"/>
-    <col min="20" max="20" width="9.44140625" customWidth="1"/>
-    <col min="21" max="21" width="11.109375" customWidth="1"/>
-    <col min="22" max="22" width="9.33203125" customWidth="1"/>
-    <col min="23" max="23" width="9.44140625" customWidth="1"/>
-    <col min="24" max="24" width="10.77734375" customWidth="1"/>
-    <col min="25" max="25" width="11.33203125" customWidth="1"/>
-    <col min="26" max="26" width="12" customWidth="1"/>
-    <col min="27" max="27" width="10.21875" customWidth="1"/>
-    <col min="30" max="30" width="9" customWidth="1"/>
-    <col min="34" max="34" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="33.0"/>
+    <col min="2" max="2" customWidth="true" width="10.44140625"/>
+    <col min="6" max="6" customWidth="true" width="10.88671875"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.33203125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.109375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.33203125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.33203125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="12.109375"/>
+    <col min="19" max="19" customWidth="true" width="8.77734375"/>
+    <col min="20" max="20" customWidth="true" width="9.44140625"/>
+    <col min="21" max="21" customWidth="true" width="11.109375"/>
+    <col min="22" max="22" customWidth="true" width="9.33203125"/>
+    <col min="23" max="23" customWidth="true" width="9.44140625"/>
+    <col min="24" max="24" customWidth="true" width="10.77734375"/>
+    <col min="25" max="25" customWidth="true" width="11.33203125"/>
+    <col min="26" max="26" customWidth="true" width="12.0"/>
+    <col min="27" max="27" customWidth="true" width="10.21875"/>
+    <col min="30" max="30" customWidth="true" width="9.0"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="17.5546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -11034,7 +11047,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="37" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
@@ -11059,7 +11072,7 @@
       <c r="T3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="U3">
+      <c r="U3" s="0">
         <v>2</v>
       </c>
       <c r="V3" s="3"/>
@@ -11072,7 +11085,7 @@
       <c r="Y3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="Z3">
+      <c r="Z3" s="0">
         <v>3</v>
       </c>
       <c r="AA3" s="105" t="s">
@@ -11209,7 +11222,7 @@
       <c r="T5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="U5">
+      <c r="U5" s="0">
         <v>2</v>
       </c>
       <c r="V5" s="3">
@@ -11224,7 +11237,7 @@
       <c r="Y5" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="Z5">
+      <c r="Z5" s="0">
         <v>3</v>
       </c>
       <c r="AA5" s="105" t="s">
@@ -11418,7 +11431,7 @@
       <c r="I9" s="37"/>
       <c r="J9" s="37"/>
       <c r="K9" s="37" t="s">
-        <v>1337</v>
+        <v>1348</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>390</v>
@@ -11427,7 +11440,7 @@
         <v>294</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>1314</v>
+        <v>1312</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>191</v>
@@ -11618,31 +11631,31 @@
   <dimension ref="A1:AG14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="49.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="49.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="4.77734375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="9.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33">
@@ -12419,11 +12432,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="35.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="35.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.5546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.44140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -12507,10 +12520,10 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="33.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="33.5546875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="13.44140625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.88671875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="14.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -12604,10 +12617,10 @@
   <dimension ref="A1:AH5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="46.6640625" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" customWidth="1"/>
-    <col min="29" max="29" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="46.6640625"/>
+    <col min="5" max="5" customWidth="true" width="6.21875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="13.33203125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34">
@@ -12844,7 +12857,7 @@
         <v>5</v>
       </c>
       <c r="W3" s="37" t="s">
-        <v>1270</v>
+        <v>1268</v>
       </c>
       <c r="X3" s="37"/>
       <c r="Y3" s="37"/>
@@ -12852,10 +12865,10 @@
       <c r="AA3" s="37"/>
       <c r="AB3" s="37"/>
       <c r="AC3" s="37" t="s">
-        <v>1271</v>
+        <v>1269</v>
       </c>
       <c r="AD3" s="105" t="s">
-        <v>1268</v>
+        <v>1266</v>
       </c>
       <c r="AE3" s="37" t="s">
         <v>12</v>
@@ -12867,7 +12880,7 @@
         <v>6</v>
       </c>
       <c r="AH3" s="40" t="s">
-        <v>1272</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="4" spans="1:34">
@@ -12906,16 +12919,16 @@
       <c r="U4" s="37"/>
       <c r="V4" s="37"/>
       <c r="W4" s="37" t="s">
-        <v>1361</v>
+        <v>1371</v>
       </c>
       <c r="X4" s="37" t="s">
-        <v>1321</v>
+        <v>1319</v>
       </c>
       <c r="Y4" s="37" t="s">
         <v>295</v>
       </c>
       <c r="Z4" s="37" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="AA4" s="37" t="s">
         <v>191</v>
@@ -12924,7 +12937,7 @@
         <v>12</v>
       </c>
       <c r="AC4" s="37" t="s">
-        <v>1362</v>
+        <v>1372</v>
       </c>
       <c r="AD4" s="37"/>
       <c r="AE4" s="37"/>
@@ -12984,16 +12997,16 @@
   <dimension ref="A1:K18"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="68.77734375" customWidth="1"/>
-    <col min="2" max="2" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="68.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="10.77734375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="19.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="15.5546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="8" max="9" bestFit="true" customWidth="true" width="19.44140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="10.88671875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="12.5546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -13365,24 +13378,24 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="20.5546875" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.6640625" customWidth="1"/>
-    <col min="18" max="18" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="20.5546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.77734375"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="7.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="17" max="17" customWidth="true" width="17.6640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="13.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -13507,16 +13520,16 @@
       <c r="I3" s="37"/>
       <c r="J3" s="37"/>
       <c r="K3" s="37" t="s">
-        <v>1345</v>
+        <v>1356</v>
       </c>
       <c r="L3" s="37" t="s">
-        <v>1315</v>
+        <v>1313</v>
       </c>
       <c r="M3" s="37" t="s">
         <v>666</v>
       </c>
       <c r="N3" s="37" t="s">
-        <v>1316</v>
+        <v>1314</v>
       </c>
       <c r="O3" s="37" t="s">
         <v>12</v>
@@ -13525,10 +13538,10 @@
         <v>43</v>
       </c>
       <c r="Q3" s="37" t="s">
-        <v>1346</v>
+        <v>1357</v>
       </c>
       <c r="R3" s="37" t="s">
-        <v>1347</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -13647,16 +13660,16 @@
       <c r="I6" s="37"/>
       <c r="J6" s="37"/>
       <c r="K6" s="37" t="s">
-        <v>1348</v>
+        <v>1359</v>
       </c>
       <c r="L6" s="37" t="s">
-        <v>1317</v>
+        <v>1315</v>
       </c>
       <c r="M6" s="37" t="s">
         <v>172</v>
       </c>
       <c r="N6" s="37" t="s">
-        <v>1318</v>
+        <v>1316</v>
       </c>
       <c r="O6" s="37" t="s">
         <v>12</v>
@@ -13665,7 +13678,7 @@
         <v>13</v>
       </c>
       <c r="Q6" s="37" t="s">
-        <v>1349</v>
+        <v>1360</v>
       </c>
       <c r="R6" s="37"/>
     </row>
@@ -13683,37 +13696,37 @@
   <dimension ref="A1:AI16"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="93.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.21875" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" customWidth="1"/>
-    <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="23.5546875" customWidth="1"/>
-    <col min="20" max="20" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.44140625" customWidth="1"/>
-    <col min="23" max="23" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="7" customWidth="1"/>
-    <col min="27" max="27" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="16.33203125" customWidth="1"/>
-    <col min="29" max="32" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="93.88671875"/>
+    <col min="2" max="2" customWidth="true" width="13.21875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.21875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="6.21875"/>
+    <col min="6" max="6" customWidth="true" width="11.6640625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="9.21875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="6.21875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="8.5546875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="18.6640625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="18.6640625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.6640625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="18.6640625"/>
+    <col min="19" max="19" customWidth="true" width="23.5546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="14.109375"/>
+    <col min="22" max="22" customWidth="true" width="13.44140625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="14.21875"/>
+    <col min="24" max="25" bestFit="true" customWidth="true" width="13.5546875"/>
+    <col min="26" max="26" customWidth="true" width="7.0"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="15.21875"/>
+    <col min="28" max="28" customWidth="true" width="16.33203125"/>
+    <col min="29" max="32" bestFit="true" customWidth="true" width="13.5546875"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="17.44140625"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="13.5546875"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" width="13.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:35">
@@ -14355,7 +14368,7 @@
         <v>4</v>
       </c>
       <c r="G10" s="105" t="s">
-        <v>1277</v>
+        <v>1275</v>
       </c>
       <c r="H10" s="104" t="s">
         <v>12</v>
@@ -14427,43 +14440,43 @@
         <v>150</v>
       </c>
       <c r="J11" s="104" t="s">
-        <v>1291</v>
+        <v>1289</v>
       </c>
       <c r="K11" s="104"/>
       <c r="L11" s="104"/>
       <c r="M11" s="104" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
       <c r="N11" s="104"/>
       <c r="O11" s="104"/>
       <c r="P11" s="104"/>
       <c r="Q11" s="104"/>
       <c r="R11" s="104" t="s">
-        <v>1288</v>
+        <v>1286</v>
       </c>
       <c r="S11" s="104"/>
       <c r="T11" s="104"/>
       <c r="U11" s="104" t="s">
-        <v>1292</v>
+        <v>1290</v>
       </c>
       <c r="V11" s="104" t="s">
-        <v>1293</v>
+        <v>1291</v>
       </c>
       <c r="W11" s="104"/>
       <c r="X11" s="104" t="s">
-        <v>1295</v>
+        <v>1293</v>
       </c>
       <c r="Y11" s="104" t="s">
-        <v>1296</v>
+        <v>1294</v>
       </c>
       <c r="Z11" s="104" t="s">
-        <v>1294</v>
+        <v>1292</v>
       </c>
       <c r="AA11" s="104" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
       <c r="AB11" s="104" t="s">
-        <v>1288</v>
+        <v>1286</v>
       </c>
       <c r="AC11" s="104"/>
       <c r="AD11" s="104"/>
@@ -14502,19 +14515,19 @@
         <v>150</v>
       </c>
       <c r="J12" s="104" t="s">
-        <v>1356</v>
+        <v>1331</v>
       </c>
       <c r="K12" s="104"/>
       <c r="L12" s="104"/>
       <c r="M12" s="104" t="s">
-        <v>1319</v>
+        <v>1317</v>
       </c>
       <c r="N12" s="104"/>
       <c r="O12" s="104"/>
       <c r="P12" s="104"/>
       <c r="Q12" s="104"/>
       <c r="R12" s="104" t="s">
-        <v>1320</v>
+        <v>1318</v>
       </c>
       <c r="S12" s="104"/>
       <c r="T12" s="104"/>
@@ -14667,8 +14680,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="32.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -14716,8 +14729,8 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="48.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="48.88671875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="11.44140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -14881,24 +14894,24 @@
   <dimension ref="A1:Q81"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="28.77734375" style="25" customWidth="1"/>
-    <col min="2" max="2" width="16.21875" style="25" customWidth="1"/>
-    <col min="3" max="3" width="11.77734375" style="25" customWidth="1"/>
-    <col min="4" max="4" width="9.5546875" style="25" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" style="25" customWidth="1"/>
-    <col min="6" max="6" width="9.33203125" style="25" customWidth="1"/>
-    <col min="7" max="7" width="9.77734375" style="25" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" style="25" customWidth="1"/>
-    <col min="9" max="9" width="8.77734375" style="25" customWidth="1"/>
-    <col min="10" max="10" width="8.109375" style="34" customWidth="1"/>
-    <col min="11" max="11" width="10" style="25" customWidth="1"/>
-    <col min="12" max="12" width="7.77734375" style="25" customWidth="1"/>
-    <col min="13" max="13" width="9" style="25" customWidth="1"/>
-    <col min="14" max="14" width="19.44140625" style="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.77734375" style="25"/>
-    <col min="16" max="16" width="14.77734375" style="25" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.109375" style="25" customWidth="1"/>
-    <col min="18" max="16384" width="8.77734375" style="25"/>
+    <col min="1" max="1" customWidth="true" style="25" width="28.77734375"/>
+    <col min="2" max="2" customWidth="true" style="25" width="16.21875"/>
+    <col min="3" max="3" customWidth="true" style="25" width="11.77734375"/>
+    <col min="4" max="4" customWidth="true" style="25" width="9.5546875"/>
+    <col min="5" max="5" customWidth="true" style="25" width="10.33203125"/>
+    <col min="6" max="6" customWidth="true" style="25" width="9.33203125"/>
+    <col min="7" max="7" customWidth="true" style="25" width="9.77734375"/>
+    <col min="8" max="8" customWidth="true" style="25" width="10.44140625"/>
+    <col min="9" max="9" customWidth="true" style="25" width="8.77734375"/>
+    <col min="10" max="10" customWidth="true" style="34" width="8.109375"/>
+    <col min="11" max="11" customWidth="true" style="25" width="10.0"/>
+    <col min="12" max="12" customWidth="true" style="25" width="7.77734375"/>
+    <col min="13" max="13" customWidth="true" style="25" width="9.0"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="19.44140625"/>
+    <col min="15" max="15" style="25" width="8.77734375"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="14.77734375"/>
+    <col min="17" max="17" customWidth="true" style="25" width="15.109375"/>
+    <col min="18" max="16384" style="25" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -18646,18 +18659,18 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="32.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" customWidth="1"/>
-    <col min="5" max="5" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.109375" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="32.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="4" max="4" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="17.33203125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="13" max="13" customWidth="true" width="15.109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -18857,17 +18870,17 @@
   <dimension ref="A1:Q21"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="39.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.44140625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="21.77734375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="6.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="18.44140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="9.44140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="18.33203125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -18946,7 +18959,7 @@
         <v>46</v>
       </c>
       <c r="H2" s="37" t="s">
-        <v>1341</v>
+        <v>1352</v>
       </c>
       <c r="I2" s="37" t="s">
         <v>337</v>
@@ -19240,7 +19253,7 @@
       </c>
       <c r="G10" s="37"/>
       <c r="H10" s="37" t="s">
-        <v>1344</v>
+        <v>1355</v>
       </c>
       <c r="I10" s="37" t="s">
         <v>730</v>
@@ -19314,7 +19327,7 @@
       </c>
       <c r="G12" s="37"/>
       <c r="H12" s="37" t="s">
-        <v>1343</v>
+        <v>1354</v>
       </c>
       <c r="I12" s="37" t="s">
         <v>680</v>
@@ -19560,7 +19573,7 @@
         <v>46</v>
       </c>
       <c r="H18" s="37" t="s">
-        <v>1342</v>
+        <v>1353</v>
       </c>
       <c r="I18" s="37" t="s">
         <v>732</v>
@@ -19697,30 +19710,30 @@
   <dimension ref="A1:W22"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="19.88671875" style="25" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" style="34" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.77734375" style="34" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" style="34" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.77734375" style="34" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="25" customWidth="1"/>
-    <col min="9" max="9" width="16.5546875" style="25" customWidth="1"/>
-    <col min="10" max="10" width="14.109375" style="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.33203125" style="34" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.33203125" style="34" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" style="25"/>
-    <col min="14" max="14" width="12.5546875" style="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.77734375" style="25" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.21875" style="25" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5546875" style="34" customWidth="1"/>
-    <col min="18" max="18" width="8.77734375" style="34" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.88671875" style="25" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12" style="25" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.77734375" style="25"/>
-    <col min="22" max="22" width="10.6640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.88671875" style="25" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="8.77734375" style="25"/>
+    <col min="1" max="1" customWidth="true" style="25" width="19.88671875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="34" width="10.88671875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="34" width="9.44140625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="34" width="7.77734375"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="34" width="10.88671875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="34" width="9.44140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="34" width="7.77734375"/>
+    <col min="8" max="8" customWidth="true" style="25" width="13.0"/>
+    <col min="9" max="9" customWidth="true" style="25" width="16.5546875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="25" width="14.109375"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="34" width="10.33203125"/>
+    <col min="12" max="12" customWidth="true" style="34" width="10.33203125"/>
+    <col min="13" max="13" style="25" width="8.77734375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="25" width="12.5546875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="25" width="14.77734375"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="25" width="13.21875"/>
+    <col min="17" max="17" customWidth="true" style="34" width="11.5546875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="34" width="8.77734375"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="25" width="9.88671875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="25" width="12.0"/>
+    <col min="21" max="21" style="25" width="8.77734375"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="25" width="10.6640625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="25" width="13.88671875"/>
+    <col min="24" max="16384" style="25" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -19805,7 +19818,7 @@
         <v>672</v>
       </c>
       <c r="D2" s="105" t="s">
-        <v>1284</v>
+        <v>1282</v>
       </c>
       <c r="E2" s="37" t="s">
         <v>672</v>
@@ -19832,7 +19845,7 @@
         <v>14</v>
       </c>
       <c r="M2" s="28" t="s">
-        <v>1367</v>
+        <v>1376</v>
       </c>
       <c r="N2" s="28">
         <v>3</v>
@@ -19844,7 +19857,7 @@
         <v>672</v>
       </c>
       <c r="Q2" s="105" t="s">
-        <v>1279</v>
+        <v>1277</v>
       </c>
       <c r="R2" s="40" t="s">
         <v>14</v>
@@ -19852,10 +19865,10 @@
       <c r="S2" s="28"/>
       <c r="T2" s="28"/>
       <c r="U2" s="37" t="s">
-        <v>1325</v>
+        <v>1323</v>
       </c>
       <c r="V2" s="37" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="W2" s="37" t="s">
         <v>337</v>
@@ -19933,7 +19946,7 @@
         <v>672</v>
       </c>
       <c r="D4" s="105" t="s">
-        <v>1281</v>
+        <v>1279</v>
       </c>
       <c r="E4" s="37" t="s">
         <v>672</v>
@@ -19942,7 +19955,7 @@
         <v>12</v>
       </c>
       <c r="G4" s="105" t="s">
-        <v>1282</v>
+        <v>1280</v>
       </c>
       <c r="H4" s="28">
         <v>1</v>
@@ -19960,13 +19973,13 @@
         <v>14</v>
       </c>
       <c r="M4" s="28" t="s">
-        <v>1366</v>
+        <v>1375</v>
       </c>
       <c r="N4" s="28"/>
       <c r="O4" s="28"/>
       <c r="P4" s="28"/>
       <c r="Q4" s="105" t="s">
-        <v>1283</v>
+        <v>1281</v>
       </c>
       <c r="R4" s="37" t="s">
         <v>662</v>
@@ -19974,10 +19987,10 @@
       <c r="S4" s="28"/>
       <c r="T4" s="28"/>
       <c r="U4" s="37" t="s">
-        <v>1323</v>
+        <v>1321</v>
       </c>
       <c r="V4" s="37" t="s">
-        <v>1324</v>
+        <v>1322</v>
       </c>
       <c r="W4" s="37" t="s">
         <v>337</v>
@@ -20015,19 +20028,19 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="19.88671875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.33203125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="17.33203125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="4.44140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="17.33203125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="11.88671875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -20130,20 +20143,20 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="25.77734375" style="34" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="34" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" style="34" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.44140625" style="34" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.21875" style="34" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="34"/>
+    <col min="1" max="1" customWidth="true" style="34" width="25.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="34" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="34" width="15.0"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="34" width="4.44140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="34" width="14.21875"/>
+    <col min="14" max="16384" style="34" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -20269,21 +20282,21 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="20.21875" style="34" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="34" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="17.33203125" style="34" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" style="34" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.44140625" style="34" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.33203125" style="34" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.21875" style="34" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="34"/>
+    <col min="1" max="1" customWidth="true" style="34" width="20.21875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="34" width="15.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
+    <col min="6" max="7" customWidth="true" style="34" width="17.33203125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="34" width="15.0"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="34" width="4.44140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="34" width="17.33203125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="34" width="14.21875"/>
+    <col min="16" max="16384" style="34" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -20471,22 +20484,22 @@
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="28.33203125" style="34" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="34" customWidth="1"/>
-    <col min="4" max="4" width="11.21875" style="34" customWidth="1"/>
-    <col min="5" max="5" width="12.77734375" style="34" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" style="34" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" style="34" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" style="34" customWidth="1"/>
-    <col min="10" max="10" width="11.88671875" style="34" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5546875" style="34" customWidth="1"/>
-    <col min="12" max="12" width="10.77734375" style="34" customWidth="1"/>
-    <col min="13" max="13" width="12.21875" style="34" customWidth="1"/>
-    <col min="14" max="14" width="12.6640625" style="34" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.21875" style="34" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="34"/>
+    <col min="1" max="1" customWidth="true" style="34" width="28.33203125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="3" max="3" customWidth="true" style="34" width="10.33203125"/>
+    <col min="4" max="4" customWidth="true" style="34" width="11.21875"/>
+    <col min="5" max="5" customWidth="true" style="34" width="12.77734375"/>
+    <col min="6" max="6" customWidth="true" style="34" width="12.44140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="34" width="11.109375"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="9" max="9" customWidth="true" style="34" width="9.109375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="34" width="11.88671875"/>
+    <col min="11" max="11" customWidth="true" style="34" width="11.5546875"/>
+    <col min="12" max="12" customWidth="true" style="34" width="10.77734375"/>
+    <col min="13" max="13" customWidth="true" style="34" width="12.21875"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="34" width="12.6640625"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" style="34" width="14.21875"/>
+    <col min="16" max="16384" style="34" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -20605,7 +20618,7 @@
       </c>
       <c r="G4" s="37"/>
       <c r="H4" s="37" t="s">
-        <v>1357</v>
+        <v>1367</v>
       </c>
       <c r="I4" s="37" t="s">
         <v>340</v>
@@ -20761,7 +20774,7 @@
         <v>734</v>
       </c>
       <c r="H9" s="37" t="s">
-        <v>1358</v>
+        <v>1368</v>
       </c>
       <c r="I9" s="37" t="s">
         <v>340</v>
@@ -20817,11 +20830,11 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="24" style="34" customWidth="1"/>
-    <col min="2" max="2" width="11.44140625" style="34" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="34"/>
-    <col min="4" max="4" width="19.6640625" style="34" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="34"/>
+    <col min="1" max="1" customWidth="true" style="34" width="24.0"/>
+    <col min="2" max="2" customWidth="true" style="34" width="11.44140625"/>
+    <col min="3" max="3" style="34" width="8.88671875"/>
+    <col min="4" max="4" customWidth="true" style="34" width="19.6640625"/>
+    <col min="5" max="16384" style="34" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -20879,12 +20892,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="32.21875" style="34" customWidth="1"/>
-    <col min="2" max="2" width="14" style="34" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" style="34" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" style="34" customWidth="1"/>
-    <col min="5" max="5" width="11.77734375" style="34" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="34"/>
+    <col min="1" max="1" customWidth="true" style="34" width="32.21875"/>
+    <col min="2" max="2" customWidth="true" style="34" width="14.0"/>
+    <col min="3" max="3" customWidth="true" style="34" width="16.6640625"/>
+    <col min="4" max="4" customWidth="true" style="34" width="17.6640625"/>
+    <col min="5" max="5" customWidth="true" style="34" width="11.77734375"/>
+    <col min="6" max="16384" style="34" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -20968,11 +20981,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="38.21875" style="34" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="34" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" style="34" customWidth="1"/>
-    <col min="4" max="4" width="19" style="34" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="34"/>
+    <col min="1" max="1" customWidth="true" style="34" width="38.21875"/>
+    <col min="2" max="2" customWidth="true" style="34" width="13.5546875"/>
+    <col min="3" max="3" customWidth="true" style="34" width="15.5546875"/>
+    <col min="4" max="4" customWidth="true" style="34" width="19.0"/>
+    <col min="5" max="16384" style="34" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -21095,23 +21108,23 @@
   <dimension ref="A1:S5"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="30.88671875" style="34" customWidth="1"/>
-    <col min="2" max="2" width="17.77734375" style="34" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" style="34" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" style="34" customWidth="1"/>
-    <col min="5" max="5" width="12" style="34" customWidth="1"/>
-    <col min="6" max="6" width="18.109375" style="34" customWidth="1"/>
-    <col min="7" max="7" width="15.109375" style="34" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" style="34" customWidth="1"/>
-    <col min="9" max="9" width="10.77734375" style="34" customWidth="1"/>
-    <col min="10" max="10" width="8.88671875" style="34"/>
-    <col min="11" max="11" width="13.21875" style="34" customWidth="1"/>
-    <col min="12" max="12" width="12.6640625" style="34" customWidth="1"/>
-    <col min="13" max="13" width="14.109375" style="34" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" style="34" customWidth="1"/>
-    <col min="15" max="18" width="8.88671875" style="34"/>
-    <col min="19" max="19" width="18.33203125" style="34" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="8.88671875" style="34"/>
+    <col min="1" max="1" customWidth="true" style="34" width="30.88671875"/>
+    <col min="2" max="2" customWidth="true" style="34" width="17.77734375"/>
+    <col min="3" max="3" customWidth="true" style="34" width="16.44140625"/>
+    <col min="4" max="4" customWidth="true" style="34" width="16.109375"/>
+    <col min="5" max="5" customWidth="true" style="34" width="12.0"/>
+    <col min="6" max="6" customWidth="true" style="34" width="18.109375"/>
+    <col min="7" max="7" customWidth="true" style="34" width="15.109375"/>
+    <col min="8" max="8" customWidth="true" style="34" width="10.44140625"/>
+    <col min="9" max="9" customWidth="true" style="34" width="10.77734375"/>
+    <col min="10" max="10" style="34" width="8.88671875"/>
+    <col min="11" max="11" customWidth="true" style="34" width="13.21875"/>
+    <col min="12" max="12" customWidth="true" style="34" width="12.6640625"/>
+    <col min="13" max="13" customWidth="true" style="34" width="14.109375"/>
+    <col min="14" max="14" customWidth="true" style="34" width="14.33203125"/>
+    <col min="15" max="18" style="34" width="8.88671875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="34" width="18.33203125"/>
+    <col min="20" max="16384" style="34" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -21196,13 +21209,13 @@
         <v>30</v>
       </c>
       <c r="H2" s="37" t="s">
-        <v>1369</v>
+        <v>1337</v>
       </c>
       <c r="I2" s="37" t="s">
-        <v>1370</v>
+        <v>1338</v>
       </c>
       <c r="J2" s="37" t="s">
-        <v>1368</v>
+        <v>1336</v>
       </c>
       <c r="K2" s="37">
         <f>B2</f>
@@ -21248,13 +21261,13 @@
         <v>962</v>
       </c>
       <c r="H3" s="37" t="s">
-        <v>1300</v>
+        <v>1298</v>
       </c>
       <c r="I3" s="37" t="s">
-        <v>1301</v>
+        <v>1299</v>
       </c>
       <c r="J3" s="37" t="s">
-        <v>1299</v>
+        <v>1297</v>
       </c>
       <c r="K3" s="37"/>
       <c r="L3" s="37" t="s">
@@ -21264,7 +21277,7 @@
         <v>665</v>
       </c>
       <c r="N3" s="37" t="s">
-        <v>1298</v>
+        <v>1296</v>
       </c>
       <c r="O3" s="37" t="s">
         <v>962</v>
@@ -21279,7 +21292,7 @@
         <v>2</v>
       </c>
       <c r="S3" s="37" t="s">
-        <v>1297</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -21290,7 +21303,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="105" t="s">
-        <v>1281</v>
+        <v>1279</v>
       </c>
       <c r="D4" s="37" t="s">
         <v>12</v>
@@ -21305,23 +21318,23 @@
         <v>672</v>
       </c>
       <c r="H4" s="37" t="s">
-        <v>1372</v>
+        <v>1334</v>
       </c>
       <c r="I4" s="37" t="s">
-        <v>1373</v>
+        <v>1335</v>
       </c>
       <c r="J4" s="37" t="s">
-        <v>1371</v>
+        <v>1333</v>
       </c>
       <c r="K4" s="37"/>
       <c r="L4" s="37" t="s">
         <v>326</v>
       </c>
       <c r="M4" s="37" t="s">
-        <v>1286</v>
+        <v>1284</v>
       </c>
       <c r="N4" s="37" t="s">
-        <v>1310</v>
+        <v>1308</v>
       </c>
       <c r="O4" s="37"/>
       <c r="P4" s="37"/>
@@ -21339,7 +21352,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="105" t="s">
-        <v>1281</v>
+        <v>1279</v>
       </c>
       <c r="D5" s="37" t="s">
         <v>12</v>
@@ -21354,23 +21367,23 @@
         <v>672</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>1375</v>
+        <v>1340</v>
       </c>
       <c r="I5" s="37" t="s">
-        <v>1376</v>
+        <v>1341</v>
       </c>
       <c r="J5" s="37" t="s">
-        <v>1374</v>
+        <v>1339</v>
       </c>
       <c r="K5" s="37"/>
       <c r="L5" s="37" t="s">
         <v>326</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>1286</v>
+        <v>1284</v>
       </c>
       <c r="N5" s="37" t="s">
-        <v>1310</v>
+        <v>1308</v>
       </c>
       <c r="O5" s="37" t="s">
         <v>306</v>
@@ -21385,7 +21398,7 @@
         <v>2</v>
       </c>
       <c r="S5" s="37" t="s">
-        <v>1311</v>
+        <v>1309</v>
       </c>
     </row>
   </sheetData>
@@ -21401,12 +21414,12 @@
   <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="39.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="39.44140625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.77734375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="5.44140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="16.109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -22096,13 +22109,13 @@
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="57.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.77734375" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="57.44140625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="15.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.77734375"/>
+    <col min="4" max="5" bestFit="true" customWidth="true" width="11.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="20.109375"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="25.88671875"/>
+    <col min="8" max="8" customWidth="true" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -22240,7 +22253,7 @@
       <c r="E7" s="37"/>
       <c r="F7" s="37"/>
       <c r="G7" s="105" t="s">
-        <v>1275</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -22334,7 +22347,7 @@
       <c r="F15" s="34"/>
     </row>
     <row r="17" spans="8:8">
-      <c r="H17" t="s">
+      <c r="H17" t="s" s="0">
         <v>997</v>
       </c>
     </row>
@@ -22352,28 +22365,28 @@
   <dimension ref="A1:W15"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="50" style="23" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.33203125" style="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.109375" style="23" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="23" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" style="23" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="8.77734375" style="23"/>
-    <col min="9" max="9" width="10.44140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.6640625" style="23" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.21875" style="23" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.44140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.21875" style="23" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13" style="23" customWidth="1"/>
-    <col min="16" max="16" width="10.21875" style="23" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.44140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.21875" style="23" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.6640625" style="23" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.6640625" style="23" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.21875" style="23" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="12.6640625" style="23" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="8.77734375" style="23"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="23" width="50.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="23" width="18.33203125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="23" width="12.109375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="23" width="15.33203125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="23" width="12.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="23" width="9.44140625"/>
+    <col min="7" max="8" style="23" width="8.77734375"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="23" width="10.44140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="23" width="12.6640625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" style="23" width="10.44140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" style="23" width="11.21875"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="23" width="10.44140625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="23" width="8.21875"/>
+    <col min="15" max="15" customWidth="true" style="23" width="13.0"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" style="23" width="10.21875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="23" width="10.44140625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="23" width="9.21875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="23" width="11.6640625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" style="23" width="12.6640625"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="23" width="11.21875"/>
+    <col min="22" max="23" bestFit="true" customWidth="true" style="23" width="12.6640625"/>
+    <col min="24" max="16384" style="23" width="8.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -22586,7 +22599,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="105" t="s">
-        <v>1280</v>
+        <v>1278</v>
       </c>
       <c r="D5" s="37" t="s">
         <v>672</v>
@@ -22599,7 +22612,7 @@
       </c>
       <c r="G5" s="49"/>
       <c r="H5" s="28" t="s">
-        <v>1365</v>
+        <v>1374</v>
       </c>
       <c r="I5" s="28"/>
       <c r="J5" s="28"/>
@@ -22695,7 +22708,7 @@
         <v>19</v>
       </c>
       <c r="H7" s="28" t="s">
-        <v>1363</v>
+        <v>1332</v>
       </c>
       <c r="I7" s="28" t="s">
         <v>320</v>
@@ -22715,14 +22728,14 @@
         <v>326</v>
       </c>
       <c r="T7" s="28" t="s">
-        <v>1285</v>
+        <v>1283</v>
       </c>
       <c r="U7" s="28"/>
       <c r="V7" s="28" t="s">
         <v>326</v>
       </c>
       <c r="W7" s="37" t="s">
-        <v>1285</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="8" spans="1:23" s="25" customFormat="1">
@@ -22927,7 +22940,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="105" t="s">
-        <v>1279</v>
+        <v>1277</v>
       </c>
       <c r="D12" s="37" t="s">
         <v>12</v>
@@ -22940,7 +22953,7 @@
       </c>
       <c r="G12" s="49"/>
       <c r="H12" s="28" t="s">
-        <v>1364</v>
+        <v>1373</v>
       </c>
       <c r="I12" s="28" t="s">
         <v>330</v>
@@ -22964,7 +22977,7 @@
         <v>326</v>
       </c>
       <c r="T12" s="28" t="s">
-        <v>1286</v>
+        <v>1284</v>
       </c>
       <c r="U12" s="28"/>
       <c r="V12" s="28" t="s">
@@ -23081,7 +23094,7 @@
         <v>15</v>
       </c>
       <c r="H15" s="28" t="s">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="I15" s="28" t="s">
         <v>193</v>
@@ -23117,14 +23130,14 @@
   <dimension ref="A1:AM45"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="77.109375" customWidth="1"/>
-    <col min="17" max="17" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.88671875" customWidth="1"/>
-    <col min="19" max="19" width="13.88671875" customWidth="1"/>
-    <col min="20" max="20" width="13.77734375" customWidth="1"/>
-    <col min="21" max="26" width="8.88671875" customWidth="1"/>
-    <col min="36" max="36" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="11" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="77.109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="11.6640625"/>
+    <col min="18" max="18" customWidth="true" width="8.88671875"/>
+    <col min="19" max="19" customWidth="true" width="13.88671875"/>
+    <col min="20" max="20" customWidth="true" width="13.77734375"/>
+    <col min="21" max="26" customWidth="true" width="8.88671875"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="12.109375"/>
+    <col min="37" max="37" customWidth="true" width="11.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39">
@@ -23138,7 +23151,7 @@
         <v>24</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>4</v>
@@ -23150,7 +23163,7 @@
         <v>24</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="I1" s="12" t="s">
         <v>4</v>
@@ -23162,7 +23175,7 @@
         <v>24</v>
       </c>
       <c r="L1" s="12" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="M1" s="12" t="s">
         <v>4</v>
@@ -23174,7 +23187,7 @@
         <v>24</v>
       </c>
       <c r="P1" s="12" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="Q1" s="12" t="s">
         <v>4</v>
@@ -23216,7 +23229,7 @@
         <v>24</v>
       </c>
       <c r="AD1" s="12" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="AE1" s="12" t="s">
         <v>4</v>
@@ -23228,7 +23241,7 @@
         <v>24</v>
       </c>
       <c r="AH1" s="12" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="AI1" s="12" t="s">
         <v>4</v>
@@ -23275,10 +23288,10 @@
       <c r="P2" s="37"/>
       <c r="Q2" s="37"/>
       <c r="R2" s="37" t="s">
-        <v>1302</v>
+        <v>1300</v>
       </c>
       <c r="S2" s="37" t="s">
-        <v>1303</v>
+        <v>1301</v>
       </c>
       <c r="T2" s="37">
         <v>1</v>
@@ -23655,10 +23668,10 @@
       <c r="P8" s="37"/>
       <c r="Q8" s="37"/>
       <c r="R8" s="37" t="s">
-        <v>1333</v>
+        <v>1379</v>
       </c>
       <c r="S8" s="37" t="s">
-        <v>1334</v>
+        <v>1380</v>
       </c>
       <c r="T8" s="37">
         <v>0</v>
@@ -24338,10 +24351,10 @@
         <v>41</v>
       </c>
       <c r="R19" s="37" t="s">
-        <v>1289</v>
+        <v>1377</v>
       </c>
       <c r="S19" s="37" t="s">
-        <v>1290</v>
+        <v>1378</v>
       </c>
       <c r="T19" s="40">
         <v>0</v>
@@ -24492,10 +24505,10 @@
       <c r="P21" s="37"/>
       <c r="Q21" s="37"/>
       <c r="R21" s="37" t="s">
-        <v>1260</v>
+        <v>1342</v>
       </c>
       <c r="S21" s="37" t="s">
-        <v>1261</v>
+        <v>1343</v>
       </c>
       <c r="T21" s="40">
         <v>0</v>
@@ -24507,7 +24520,7 @@
         <v>1162</v>
       </c>
       <c r="Y21" s="37" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="Z21" s="37" t="s">
         <v>1184</v>
@@ -25925,17 +25938,17 @@
   <dimension ref="A1:V19"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="53.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="12.21875" customWidth="1"/>
-    <col min="8" max="8" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="53.77734375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="3" max="4" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="5" max="7" customWidth="true" width="12.21875"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="17.5546875"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="15.44140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="12.21875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="11.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -26139,7 +26152,7 @@
         <v>243</v>
       </c>
       <c r="F5" s="98" t="s">
-        <v>1278</v>
+        <v>1276</v>
       </c>
       <c r="G5" s="98"/>
       <c r="H5" s="98"/>
@@ -26211,7 +26224,7 @@
         <v>243</v>
       </c>
       <c r="F7" s="98" t="s">
-        <v>1278</v>
+        <v>1276</v>
       </c>
       <c r="G7" s="98"/>
       <c r="H7" s="98"/>
@@ -26554,7 +26567,7 @@
         <v>12</v>
       </c>
       <c r="E16" s="105" t="s">
-        <v>1265</v>
+        <v>1263</v>
       </c>
       <c r="F16" s="98"/>
       <c r="G16" s="98"/>
@@ -26701,16 +26714,16 @@
   <dimension ref="A1:X38"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="64.5546875" customWidth="1"/>
-    <col min="10" max="10" width="8.77734375" style="23"/>
-    <col min="12" max="12" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="64.5546875"/>
+    <col min="10" max="10" style="23" width="8.77734375"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="11.44140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="13.88671875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="12.6640625"/>
+    <col min="22" max="23" bestFit="true" customWidth="true" width="19.21875"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="15.5546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24">
@@ -26817,7 +26830,7 @@
       </c>
       <c r="J2" s="37"/>
       <c r="K2" s="37" t="s">
-        <v>1350</v>
+        <v>1361</v>
       </c>
       <c r="L2" s="37"/>
       <c r="M2" s="37"/>
@@ -26857,10 +26870,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="37" t="s">
-        <v>1354</v>
+        <v>1365</v>
       </c>
       <c r="L3" s="37" t="s">
-        <v>1355</v>
+        <v>1366</v>
       </c>
       <c r="M3" s="37"/>
       <c r="N3" s="37"/>
@@ -27825,10 +27838,10 @@
       <c r="I25" s="37"/>
       <c r="J25" s="37"/>
       <c r="K25" s="37" t="s">
-        <v>1352</v>
+        <v>1363</v>
       </c>
       <c r="L25" s="37" t="s">
-        <v>1353</v>
+        <v>1364</v>
       </c>
       <c r="M25" s="37"/>
       <c r="N25" s="37" t="s">
@@ -28217,7 +28230,7 @@
       </c>
       <c r="J35" s="37"/>
       <c r="K35" s="37" t="s">
-        <v>1351</v>
+        <v>1362</v>
       </c>
       <c r="L35" s="37"/>
       <c r="M35" s="37"/>

</xml_diff>

<commit_message>
Padmashree and Shireena's code changes on 17/02/2026
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4691" uniqueCount="1372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4721" uniqueCount="1391">
   <si>
     <t>Scenario</t>
   </si>
@@ -4190,6 +4190,63 @@
   </si>
   <si>
     <t>SKFHCB</t>
+  </si>
+  <si>
+    <t>SKHCC3</t>
+  </si>
+  <si>
+    <t>2302283172127</t>
+  </si>
+  <si>
+    <t>SKHC0I</t>
+  </si>
+  <si>
+    <t>2302283172148</t>
+  </si>
+  <si>
+    <t>SKHC4K</t>
+  </si>
+  <si>
+    <t>SKHC5J</t>
+  </si>
+  <si>
+    <t>SKHDBZ</t>
+  </si>
+  <si>
+    <t>2302283172150</t>
+  </si>
+  <si>
+    <t>SKHDED</t>
+  </si>
+  <si>
+    <t>2302283172153</t>
+  </si>
+  <si>
+    <t>SKHDGY</t>
+  </si>
+  <si>
+    <t>SKHDKK</t>
+  </si>
+  <si>
+    <t>2026-02-17T19:51:00</t>
+  </si>
+  <si>
+    <t>SKHDNP</t>
+  </si>
+  <si>
+    <t>2302283172161</t>
+  </si>
+  <si>
+    <t>2302283172162</t>
+  </si>
+  <si>
+    <t>SKHDZ0</t>
+  </si>
+  <si>
+    <t>2302283172165</t>
+  </si>
+  <si>
+    <t>2302283172166</t>
   </si>
 </sst>
 </file>
@@ -7044,13 +7101,13 @@
         <v>18</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>1363</v>
+        <v>1385</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>1364</v>
+        <v>1386</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>1365</v>
+        <v>1387</v>
       </c>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
@@ -7246,13 +7303,13 @@
         <v>18</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>1366</v>
+        <v>1388</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>1367</v>
+        <v>1389</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>1368</v>
+        <v>1390</v>
       </c>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
@@ -10873,7 +10930,7 @@
         <v>10</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>1360</v>
+        <v>1382</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
@@ -11257,7 +11314,7 @@
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3" t="s">
-        <v>1361</v>
+        <v>1383</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>850</v>
@@ -11266,7 +11323,7 @@
         <v>277</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>1362</v>
+        <v>1384</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>114</v>
@@ -23457,10 +23514,10 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3" t="s">
-        <v>1352</v>
+        <v>1374</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>1353</v>
+        <v>1375</v>
       </c>
       <c r="T8" s="3">
         <v>0</v>
@@ -24140,10 +24197,10 @@
         <v>119</v>
       </c>
       <c r="R19" s="3" t="s">
-        <v>1350</v>
+        <v>1372</v>
       </c>
       <c r="S19" s="3" t="s">
-        <v>1351</v>
+        <v>1373</v>
       </c>
       <c r="T19" s="15">
         <v>0</v>
@@ -26647,7 +26704,7 @@
       </c>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
-        <v>1354</v>
+        <v>1376</v>
       </c>
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
@@ -26687,10 +26744,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>1358</v>
+        <v>1380</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1359</v>
+        <v>1381</v>
       </c>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
@@ -27655,10 +27712,10 @@
       <c r="I25" s="3"/>
       <c r="J25" s="3"/>
       <c r="K25" s="3" t="s">
-        <v>1356</v>
+        <v>1378</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1357</v>
+        <v>1379</v>
       </c>
       <c r="M25" s="3"/>
       <c r="N25" s="3" t="s">
@@ -28047,7 +28104,7 @@
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="3" t="s">
-        <v>1355</v>
+        <v>1377</v>
       </c>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>

</xml_diff>

<commit_message>
Test data and sanity suite update on 04/03/2026
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation\Copa_API_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0738717-DB99-4442-A763-036202531F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F05B48-8314-4BDB-BA3C-03DEBFA43390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="0" windowWidth="19180" windowHeight="10080" firstSheet="10" activeTab="11" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="6" xr2:uid="{5D5A4724-D560-4FC2-9708-4BBF1DBA0B11}"/>
   </bookViews>
   <sheets>
     <sheet name="AdvancePassengerInfo" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4721" uniqueCount="1391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4773" uniqueCount="1425">
   <si>
     <t>Scenario</t>
   </si>
@@ -3829,9 +3829,6 @@
     <t>STB_04_ClearAll_Standby</t>
   </si>
   <si>
-    <t>OG4XEU</t>
-  </si>
-  <si>
     <t>STB_05_Release_Held_Seats</t>
   </si>
   <si>
@@ -4126,63 +4123,6 @@
     <t>AGRJDE</t>
   </si>
   <si>
-    <t>OR3SVB</t>
-  </si>
-  <si>
-    <t>2302310031670</t>
-  </si>
-  <si>
-    <t>OR3TA2</t>
-  </si>
-  <si>
-    <t>2302310031682</t>
-  </si>
-  <si>
-    <t>OR3TD3</t>
-  </si>
-  <si>
-    <t>OR3TFE</t>
-  </si>
-  <si>
-    <t>OR3TGI</t>
-  </si>
-  <si>
-    <t>2302310031684</t>
-  </si>
-  <si>
-    <t>OR3TI2</t>
-  </si>
-  <si>
-    <t>2302310031685</t>
-  </si>
-  <si>
-    <t>OR3TLQ</t>
-  </si>
-  <si>
-    <t>OR3TOG</t>
-  </si>
-  <si>
-    <t>2026-02-07T19:51:00</t>
-  </si>
-  <si>
-    <t>OR3TRB</t>
-  </si>
-  <si>
-    <t>2302310031697</t>
-  </si>
-  <si>
-    <t>2302310031698</t>
-  </si>
-  <si>
-    <t>OR3TUK</t>
-  </si>
-  <si>
-    <t>2302310031699</t>
-  </si>
-  <si>
-    <t>2302310031700</t>
-  </si>
-  <si>
     <t>12</t>
   </si>
   <si>
@@ -4192,61 +4132,223 @@
     <t>SKFHCB</t>
   </si>
   <si>
-    <t>SKHCC3</t>
-  </si>
-  <si>
-    <t>2302283172127</t>
-  </si>
-  <si>
-    <t>SKHC0I</t>
-  </si>
-  <si>
-    <t>2302283172148</t>
-  </si>
-  <si>
-    <t>SKHC4K</t>
-  </si>
-  <si>
-    <t>SKHC5J</t>
-  </si>
-  <si>
-    <t>SKHDBZ</t>
-  </si>
-  <si>
-    <t>2302283172150</t>
-  </si>
-  <si>
-    <t>SKHDED</t>
-  </si>
-  <si>
-    <t>2302283172153</t>
-  </si>
-  <si>
-    <t>SKHDGY</t>
-  </si>
-  <si>
-    <t>SKHDKK</t>
-  </si>
-  <si>
-    <t>2026-02-17T19:51:00</t>
-  </si>
-  <si>
-    <t>SKHDNP</t>
-  </si>
-  <si>
-    <t>2302283172161</t>
-  </si>
-  <si>
-    <t>2302283172162</t>
-  </si>
-  <si>
-    <t>SKHDZ0</t>
-  </si>
-  <si>
-    <t>2302283172165</t>
-  </si>
-  <si>
-    <t>2302283172166</t>
+    <t>2026-02-21T19:51:00</t>
+  </si>
+  <si>
+    <t>AR3PY1</t>
+  </si>
+  <si>
+    <t>2302154010679</t>
+  </si>
+  <si>
+    <t>AR3PZT</t>
+  </si>
+  <si>
+    <t>AR3PZY</t>
+  </si>
+  <si>
+    <t>AR3PZZ</t>
+  </si>
+  <si>
+    <t>2302154010680</t>
+  </si>
+  <si>
+    <t>AR3P0F</t>
+  </si>
+  <si>
+    <t>2302154010681</t>
+  </si>
+  <si>
+    <t>AR3P15</t>
+  </si>
+  <si>
+    <t>AR3P2H</t>
+  </si>
+  <si>
+    <t>AR3P2V</t>
+  </si>
+  <si>
+    <t>2302154010687</t>
+  </si>
+  <si>
+    <t>2302154010688</t>
+  </si>
+  <si>
+    <t>AR3P3D</t>
+  </si>
+  <si>
+    <t>2302154010689</t>
+  </si>
+  <si>
+    <t>2302154010690</t>
+  </si>
+  <si>
+    <t>AR3QJZ</t>
+  </si>
+  <si>
+    <t>2302154010704</t>
+  </si>
+  <si>
+    <t>SOAL4Q</t>
+  </si>
+  <si>
+    <t>SOAN2S</t>
+  </si>
+  <si>
+    <t>SOAOAF</t>
+  </si>
+  <si>
+    <t>SOAOCF</t>
+  </si>
+  <si>
+    <t>SOAOGI</t>
+  </si>
+  <si>
+    <t>SOAOKC</t>
+  </si>
+  <si>
+    <t>SOAOLG</t>
+  </si>
+  <si>
+    <t>SOAORS</t>
+  </si>
+  <si>
+    <t>SOAOVE</t>
+  </si>
+  <si>
+    <t>2302283178748</t>
+  </si>
+  <si>
+    <t>2302283178749</t>
+  </si>
+  <si>
+    <t>SOAOYC</t>
+  </si>
+  <si>
+    <t>2302283178750</t>
+  </si>
+  <si>
+    <t>2302283178751</t>
+  </si>
+  <si>
+    <t>SOQ2S2</t>
+  </si>
+  <si>
+    <t>2302283181026</t>
+  </si>
+  <si>
+    <t>SORCT0</t>
+  </si>
+  <si>
+    <t>2302283181028</t>
+  </si>
+  <si>
+    <t>SORDOL</t>
+  </si>
+  <si>
+    <t>SOREEP</t>
+  </si>
+  <si>
+    <t>SORE5A</t>
+  </si>
+  <si>
+    <t>2302283181029</t>
+  </si>
+  <si>
+    <t>SORF3V</t>
+  </si>
+  <si>
+    <t>2302283181030</t>
+  </si>
+  <si>
+    <t>SORGOC</t>
+  </si>
+  <si>
+    <t>SORG1O</t>
+  </si>
+  <si>
+    <t>2026-02-22T19:51:00</t>
+  </si>
+  <si>
+    <t>SORHMM</t>
+  </si>
+  <si>
+    <t>2302283181036</t>
+  </si>
+  <si>
+    <t>2302283181037</t>
+  </si>
+  <si>
+    <t>SORILF</t>
+  </si>
+  <si>
+    <t>2302283181038</t>
+  </si>
+  <si>
+    <t>2302283181039</t>
+  </si>
+  <si>
+    <t>S0LRXO</t>
+  </si>
+  <si>
+    <t>2302283233945</t>
+  </si>
+  <si>
+    <t>S0LSQU</t>
+  </si>
+  <si>
+    <t>2302283233953</t>
+  </si>
+  <si>
+    <t>S0LS5P</t>
+  </si>
+  <si>
+    <t>2302283233959</t>
+  </si>
+  <si>
+    <t>S0LTSA</t>
+  </si>
+  <si>
+    <t>S0LTZU</t>
+  </si>
+  <si>
+    <t>S0LT5U</t>
+  </si>
+  <si>
+    <t>2302283233970</t>
+  </si>
+  <si>
+    <t>S0LUJF</t>
+  </si>
+  <si>
+    <t>2302283233975</t>
+  </si>
+  <si>
+    <t>S0LUWH</t>
+  </si>
+  <si>
+    <t>S0LU42</t>
+  </si>
+  <si>
+    <t>2026-03-05T19:50:00</t>
+  </si>
+  <si>
+    <t>S0LVJ3</t>
+  </si>
+  <si>
+    <t>2302283233988</t>
+  </si>
+  <si>
+    <t>2302283233989</t>
+  </si>
+  <si>
+    <t>S0LVTE</t>
+  </si>
+  <si>
+    <t>2302283233990</t>
+  </si>
+  <si>
+    <t>2302283233991</t>
   </si>
 </sst>
 </file>
@@ -5551,7 +5653,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="24" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="I4" s="24" t="s">
         <v>30</v>
@@ -5606,7 +5708,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="24" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>22</v>
@@ -6205,7 +6307,7 @@
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>93</v>
@@ -6286,7 +6388,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>98</v>
@@ -6299,7 +6401,7 @@
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>72</v>
@@ -6564,13 +6666,13 @@
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="15" t="s">
@@ -7101,13 +7203,13 @@
         <v>18</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>1385</v>
+        <v>1419</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>1386</v>
+        <v>1420</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>1387</v>
+        <v>1421</v>
       </c>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
@@ -7303,13 +7405,13 @@
         <v>18</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>1388</v>
+        <v>1422</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>1389</v>
+        <v>1423</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>1390</v>
+        <v>1424</v>
       </c>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
@@ -7915,7 +8017,7 @@
         <v>259</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>1370</v>
+        <v>1350</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>259</v>
@@ -8266,7 +8368,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>17</v>
@@ -8407,7 +8509,7 @@
         <v>259</v>
       </c>
       <c r="L18" s="68" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="M18" s="3" t="s">
         <v>259</v>
@@ -8571,7 +8673,7 @@
         <v>259</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>1342</v>
+        <v>1341</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>259</v>
@@ -8967,16 +9069,16 @@
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>580</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>580</v>
@@ -9063,16 +9165,16 @@
         <v>70</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>580</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>580</v>
@@ -9809,7 +9911,7 @@
         <v>801</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>802</v>
@@ -10930,7 +11032,7 @@
         <v>10</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>1382</v>
+        <v>1416</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
@@ -11314,7 +11416,7 @@
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3" t="s">
-        <v>1383</v>
+        <v>1417</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>850</v>
@@ -11323,7 +11425,7 @@
         <v>277</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>1384</v>
+        <v>1418</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>114</v>
@@ -11886,7 +11988,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="48" t="s">
-        <v>1369</v>
+        <v>1349</v>
       </c>
       <c r="D6" s="49" t="s">
         <v>17</v>
@@ -12815,16 +12917,16 @@
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="X4" s="3" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="Y4" s="3" t="s">
         <v>542</v>
       </c>
       <c r="Z4" s="3" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="AA4" s="3" t="s">
         <v>114</v>
@@ -12833,7 +12935,7 @@
         <v>17</v>
       </c>
       <c r="AC4" s="3" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
@@ -13402,16 +13504,16 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>240</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>17</v>
@@ -13420,10 +13522,10 @@
         <v>18</v>
       </c>
       <c r="Q3" s="3" t="s">
+        <v>1312</v>
+      </c>
+      <c r="R3" s="3" t="s">
         <v>1313</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>1314</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -13542,16 +13644,16 @@
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3" t="s">
+        <v>1332</v>
+      </c>
+      <c r="L6" s="3" t="s">
         <v>1333</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>1334</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>625</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="O6" s="3" t="s">
         <v>17</v>
@@ -13560,7 +13662,7 @@
         <v>121</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="R6" s="3"/>
     </row>
@@ -18827,7 +18929,7 @@
         <v>165</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>166</v>
@@ -18901,7 +19003,7 @@
         <v>171</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="15" t="s">
@@ -19121,7 +19223,7 @@
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>189</v>
@@ -19195,7 +19297,7 @@
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>196</v>
@@ -19441,7 +19543,7 @@
         <v>165</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>222</v>
@@ -19552,7 +19654,7 @@
         <v>165</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -19710,7 +19812,7 @@
         <v>19</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="N2" s="3">
         <v>3</v>
@@ -19730,10 +19832,10 @@
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="V2" s="3" t="s">
         <v>1294</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>1295</v>
       </c>
       <c r="W2" s="3" t="s">
         <v>166</v>
@@ -19838,7 +19940,7 @@
         <v>19</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
@@ -19852,10 +19954,10 @@
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
       <c r="U4" s="3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="V4" s="3" t="s">
         <v>1294</v>
-      </c>
-      <c r="V4" s="3" t="s">
-        <v>1295</v>
       </c>
       <c r="W4" s="3" t="s">
         <v>166</v>
@@ -20490,7 +20592,7 @@
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>1246</v>
@@ -20530,7 +20632,7 @@
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3" t="s">
-        <v>1371</v>
+        <v>1351</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>1246</v>
@@ -20551,7 +20653,7 @@
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="3" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>69</v>
@@ -20575,7 +20677,7 @@
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="3" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>69</v>
@@ -20599,7 +20701,7 @@
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="3" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>69</v>
@@ -20625,7 +20727,7 @@
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="3" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>173</v>
@@ -20646,7 +20748,7 @@
         <v>54</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>1246</v>
@@ -20667,7 +20769,7 @@
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="3" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>69</v>
@@ -20723,7 +20825,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>69</v>
@@ -20737,7 +20839,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>129</v>
@@ -20788,7 +20890,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>69</v>
@@ -20805,7 +20907,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>134</v>
@@ -20822,7 +20924,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>132</v>
@@ -20861,30 +20963,30 @@
         <v>0</v>
       </c>
       <c r="B1" s="27" t="s">
+        <v>1261</v>
+      </c>
+      <c r="C1" s="27" t="s">
         <v>1262</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="D1" s="27" t="s">
         <v>1263</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="E1" s="27" t="s">
         <v>1264</v>
-      </c>
-      <c r="E1" s="27" t="s">
-        <v>1265</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
+        <v>1265</v>
+      </c>
+      <c r="B2" s="15" t="s">
         <v>1266</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>1267</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>1080</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>17</v>
@@ -20892,16 +20994,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>1080</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>17</v>
@@ -20909,23 +21011,23 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>1270</v>
+        <v>1269</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E4" s="3"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="3" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>17</v>
@@ -20933,31 +21035,31 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="28" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>1080</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="29" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>1080</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>17</v>
@@ -21027,7 +21129,7 @@
         <v>4</v>
       </c>
       <c r="H1" s="31" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="I1" s="31" t="s">
         <v>9</v>
@@ -21065,7 +21167,7 @@
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="32" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="B2" s="3">
         <v>0</v>
@@ -21086,13 +21188,13 @@
         <v>70</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>1328</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>1329</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>1330</v>
-      </c>
       <c r="J2" s="3" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="K2" s="3">
         <f>B2</f>
@@ -21117,7 +21219,7 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="3" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="B3" s="3">
         <v>0</v>
@@ -21138,13 +21240,13 @@
         <v>92</v>
       </c>
       <c r="H3" s="3" t="s">
+        <v>1276</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>1277</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>1278</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>1279</v>
       </c>
       <c r="K3" s="3"/>
       <c r="L3" s="3" t="s">
@@ -21154,7 +21256,7 @@
         <v>33</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>92</v>
@@ -21169,12 +21271,12 @@
         <v>2</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="33" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
       <c r="B4" s="3">
         <v>0</v>
@@ -21195,13 +21297,13 @@
         <v>130</v>
       </c>
       <c r="H4" s="3" t="s">
+        <v>1282</v>
+      </c>
+      <c r="I4" s="3" t="s">
         <v>1283</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>1284</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>1285</v>
       </c>
       <c r="K4" s="3"/>
       <c r="L4" s="3" t="s">
@@ -21211,7 +21313,7 @@
         <v>328</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
@@ -21223,7 +21325,7 @@
     </row>
     <row r="5" spans="1:19">
       <c r="A5" s="3" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="B5" s="3">
         <v>0</v>
@@ -21244,13 +21346,13 @@
         <v>130</v>
       </c>
       <c r="H5" s="3" t="s">
+        <v>1287</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>1288</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>1289</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>1290</v>
       </c>
       <c r="K5" s="3"/>
       <c r="L5" s="3" t="s">
@@ -21260,7 +21362,7 @@
         <v>328</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>158</v>
@@ -21275,7 +21377,7 @@
         <v>2</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
     </row>
   </sheetData>
@@ -22043,7 +22145,7 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="J2" s="97" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -22091,7 +22193,7 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="J4" s="97" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -22459,7 +22561,7 @@
       </c>
       <c r="G5" s="34"/>
       <c r="H5" s="3" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
@@ -22555,7 +22657,7 @@
         <v>293</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>301</v>
@@ -22941,7 +23043,7 @@
         <v>171</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>21</v>
@@ -23134,10 +23236,10 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3" t="s">
+        <v>1343</v>
+      </c>
+      <c r="S2" s="3" t="s">
         <v>1344</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>1345</v>
       </c>
       <c r="T2" s="3">
         <v>1</v>
@@ -23215,7 +23317,7 @@
         <v>17</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>358</v>
@@ -23514,10 +23616,10 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3" t="s">
-        <v>1374</v>
+        <v>1408</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>1375</v>
+        <v>1409</v>
       </c>
       <c r="T8" s="3">
         <v>0</v>
@@ -24110,10 +24212,10 @@
       <c r="P18" s="3"/>
       <c r="Q18" s="3"/>
       <c r="R18" s="3" t="s">
+        <v>1345</v>
+      </c>
+      <c r="S18" s="3" t="s">
         <v>1346</v>
-      </c>
-      <c r="S18" s="3" t="s">
-        <v>1347</v>
       </c>
       <c r="T18" s="15">
         <v>0</v>
@@ -24197,10 +24299,10 @@
         <v>119</v>
       </c>
       <c r="R19" s="3" t="s">
-        <v>1372</v>
+        <v>1404</v>
       </c>
       <c r="S19" s="3" t="s">
-        <v>1373</v>
+        <v>1405</v>
       </c>
       <c r="T19" s="15">
         <v>0</v>
@@ -24351,10 +24453,10 @@
       <c r="P21" s="3"/>
       <c r="Q21" s="3"/>
       <c r="R21" s="3" t="s">
-        <v>1349</v>
+        <v>1406</v>
       </c>
       <c r="S21" s="3" t="s">
-        <v>1339</v>
+        <v>1407</v>
       </c>
       <c r="T21" s="15">
         <v>0</v>
@@ -25539,7 +25641,7 @@
       <c r="P41" s="3"/>
       <c r="Q41" s="3"/>
       <c r="R41" s="3" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
       <c r="S41" s="3"/>
       <c r="T41" s="3"/>
@@ -26704,7 +26806,7 @@
       </c>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
-        <v>1376</v>
+        <v>1410</v>
       </c>
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
@@ -26728,7 +26830,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>17</v>
@@ -26744,10 +26846,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>1380</v>
+        <v>1414</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1381</v>
+        <v>1415</v>
       </c>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
@@ -27712,10 +27814,10 @@
       <c r="I25" s="3"/>
       <c r="J25" s="3"/>
       <c r="K25" s="3" t="s">
-        <v>1378</v>
+        <v>1412</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1379</v>
+        <v>1413</v>
       </c>
       <c r="M25" s="3"/>
       <c r="N25" s="3" t="s">
@@ -28104,7 +28206,7 @@
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="3" t="s">
-        <v>1377</v>
+        <v>1411</v>
       </c>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>

</xml_diff>

<commit_message>
Excel report implemented for SHD Webservices 04-Mar-2026
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4773" uniqueCount="1425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4843" uniqueCount="1471">
   <si>
     <t>Scenario</t>
   </si>
@@ -4349,6 +4349,144 @@
   </si>
   <si>
     <t>2302283233991</t>
+  </si>
+  <si>
+    <t>S0LYNH</t>
+  </si>
+  <si>
+    <t>2302283234011</t>
+  </si>
+  <si>
+    <t>S0LYQK</t>
+  </si>
+  <si>
+    <t>2302283234013</t>
+  </si>
+  <si>
+    <t>S0LYUJ</t>
+  </si>
+  <si>
+    <t>S0LYVE</t>
+  </si>
+  <si>
+    <t>S0LYVZ</t>
+  </si>
+  <si>
+    <t>2302283234015</t>
+  </si>
+  <si>
+    <t>S0LYXI</t>
+  </si>
+  <si>
+    <t>2302283234016</t>
+  </si>
+  <si>
+    <t>S0LY0D</t>
+  </si>
+  <si>
+    <t>S0LY4J</t>
+  </si>
+  <si>
+    <t>S0LZCB</t>
+  </si>
+  <si>
+    <t>2302283234022</t>
+  </si>
+  <si>
+    <t>2302283234023</t>
+  </si>
+  <si>
+    <t>S0LZF5</t>
+  </si>
+  <si>
+    <t>2302283234025</t>
+  </si>
+  <si>
+    <t>2302283234026</t>
+  </si>
+  <si>
+    <t>S0OKM4</t>
+  </si>
+  <si>
+    <t>2302283235133</t>
+  </si>
+  <si>
+    <t>S0OKTM</t>
+  </si>
+  <si>
+    <t>2302283235135</t>
+  </si>
+  <si>
+    <t>S0OLPW</t>
+  </si>
+  <si>
+    <t>2302283235141</t>
+  </si>
+  <si>
+    <t>S0OLT4</t>
+  </si>
+  <si>
+    <t>2302283235144</t>
+  </si>
+  <si>
+    <t>S0OLZY</t>
+  </si>
+  <si>
+    <t>2302283235146</t>
+  </si>
+  <si>
+    <t>S0OMC5</t>
+  </si>
+  <si>
+    <t>2302283235149</t>
+  </si>
+  <si>
+    <t>S0ON2W</t>
+  </si>
+  <si>
+    <t>2302283235153</t>
+  </si>
+  <si>
+    <t>S0OOLJ</t>
+  </si>
+  <si>
+    <t>2302283235155</t>
+  </si>
+  <si>
+    <t>S0OOQJ</t>
+  </si>
+  <si>
+    <t>S0OORH</t>
+  </si>
+  <si>
+    <t>S0OOU0</t>
+  </si>
+  <si>
+    <t>2302283235158</t>
+  </si>
+  <si>
+    <t>S0OOWW</t>
+  </si>
+  <si>
+    <t>2302283235159</t>
+  </si>
+  <si>
+    <t>S0OO0G</t>
+  </si>
+  <si>
+    <t>S0OO3U</t>
+  </si>
+  <si>
+    <t>S0OPAW</t>
+  </si>
+  <si>
+    <t>S0OPIE</t>
+  </si>
+  <si>
+    <t>2302283235165</t>
+  </si>
+  <si>
+    <t>2302283235166</t>
   </si>
 </sst>
 </file>
@@ -7203,13 +7341,13 @@
         <v>18</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>1419</v>
+        <v>1467</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>1420</v>
+        <v>1438</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>1421</v>
+        <v>1439</v>
       </c>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
@@ -7405,13 +7543,13 @@
         <v>18</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>1422</v>
+        <v>1468</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>1423</v>
+        <v>1469</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>1424</v>
+        <v>1470</v>
       </c>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
@@ -11032,7 +11170,7 @@
         <v>10</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>1416</v>
+        <v>1465</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
@@ -11416,7 +11554,7 @@
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3" t="s">
-        <v>1417</v>
+        <v>1466</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>850</v>
@@ -23616,10 +23754,10 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3" t="s">
-        <v>1408</v>
+        <v>1457</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>1409</v>
+        <v>1458</v>
       </c>
       <c r="T8" s="3">
         <v>0</v>
@@ -24299,10 +24437,10 @@
         <v>119</v>
       </c>
       <c r="R19" s="3" t="s">
-        <v>1404</v>
+        <v>1455</v>
       </c>
       <c r="S19" s="3" t="s">
-        <v>1405</v>
+        <v>1456</v>
       </c>
       <c r="T19" s="15">
         <v>0</v>
@@ -24453,10 +24591,10 @@
       <c r="P21" s="3"/>
       <c r="Q21" s="3"/>
       <c r="R21" s="3" t="s">
-        <v>1406</v>
+        <v>1449</v>
       </c>
       <c r="S21" s="3" t="s">
-        <v>1407</v>
+        <v>1450</v>
       </c>
       <c r="T21" s="15">
         <v>0</v>
@@ -26806,7 +26944,7 @@
       </c>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
-        <v>1410</v>
+        <v>1459</v>
       </c>
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
@@ -26846,10 +26984,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>1414</v>
+        <v>1463</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1415</v>
+        <v>1464</v>
       </c>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
@@ -27814,10 +27952,10 @@
       <c r="I25" s="3"/>
       <c r="J25" s="3"/>
       <c r="K25" s="3" t="s">
-        <v>1412</v>
+        <v>1461</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1413</v>
+        <v>1462</v>
       </c>
       <c r="M25" s="3"/>
       <c r="N25" s="3" t="s">
@@ -28206,7 +28344,7 @@
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="3" t="s">
-        <v>1411</v>
+        <v>1460</v>
       </c>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>

</xml_diff>

<commit_message>
Dhivya and Supraja code changes on 09/04/2026
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4843" uniqueCount="1471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4849" uniqueCount="1475">
   <si>
     <t>Scenario</t>
   </si>
@@ -4487,6 +4487,18 @@
   </si>
   <si>
     <t>2302283235166</t>
+  </si>
+  <si>
+    <t>BAIFOD</t>
+  </si>
+  <si>
+    <t>2302154772865</t>
+  </si>
+  <si>
+    <t>QPN0BZ</t>
+  </si>
+  <si>
+    <t>2303084479066</t>
   </si>
 </sst>
 </file>
@@ -26984,10 +26996,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>1463</v>
+        <v>1473</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1464</v>
+        <v>1474</v>
       </c>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>

</xml_diff>

<commit_message>
Padmashree code changes on 15/04/2026
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/Scenario_TestData.xlsx
+++ b/src/test/java/TestData/Scenario_TestData.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4849" uniqueCount="1475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4852" uniqueCount="1477">
   <si>
     <t>Scenario</t>
   </si>
@@ -4499,6 +4499,12 @@
   </si>
   <si>
     <t>2303084479066</t>
+  </si>
+  <si>
+    <t>Q3A2V5</t>
+  </si>
+  <si>
+    <t>2303084495043</t>
   </si>
 </sst>
 </file>
@@ -26996,10 +27002,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>1473</v>
+        <v>1475</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1474</v>
+        <v>1476</v>
       </c>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>

</xml_diff>